<commit_message>
Renombra campaña a Día de los Muertos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111i7vn9WWo4QxCQbucWbrF
</commit_message>
<xml_diff>
--- a/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
+++ b/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
@@ -732,7 +732,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Campaña Día de los Difuntos 2026  ·  Precios sugeridos en dólares estadounidenses (USD)</t>
+          <t>Campaña Día de los Muertos 2026  ·  Precios sugeridos en dólares estadounidenses (USD)</t>
         </is>
       </c>
     </row>
@@ -784,7 +784,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>Observaciones del Lanzamiento (Difuntos)</t>
+          <t>Observaciones del Lanzamiento (Día de los Muertos)</t>
         </is>
       </c>
     </row>
@@ -897,7 +897,7 @@
       </c>
       <c r="J6" s="10" t="inlineStr">
         <is>
-          <t>• Ceremonia de aspersión con acompañamiento durante la temporada de Difuntos
+          <t>• Ceremonia de aspersión con acompañamiento durante la temporada del Día de los Muertos
 • Complemento natural para quienes contratan la Solución Modular</t>
         </is>
       </c>
@@ -1108,7 +1108,7 @@
     <row r="2">
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>Portafolio de Cremación — Campaña Día de los Difuntos 2026</t>
+          <t>Portafolio de Cremación — Campaña Día de los Muertos 2026</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1340,7 @@
     <row r="21" ht="20" customHeight="1">
       <c r="B21" s="20" t="inlineStr">
         <is>
-          <t>DIFERENCIALES DE LA CAMPAÑA DE DIFUNTOS</t>
+          <t>DIFERENCIALES DE LA CAMPAÑA DÍA DE LOS MUERTOS</t>
         </is>
       </c>
       <c r="C21" s="21" t="n"/>
@@ -1586,14 +1586,14 @@
     <row r="42" ht="20" customHeight="1">
       <c r="B42" s="20" t="inlineStr">
         <is>
-          <t>DIFERENCIALES DE LA CAMPAÑA DE DIFUNTOS</t>
+          <t>DIFERENCIALES DE LA CAMPAÑA DÍA DE LOS MUERTOS</t>
         </is>
       </c>
       <c r="C42" s="21" t="n"/>
       <c r="D42" s="21" t="n"/>
       <c r="E42" s="22" t="n"/>
     </row>
-    <row r="43" ht="35" customHeight="1">
+    <row r="43" ht="49.5" customHeight="1">
       <c r="B43" s="23" t="inlineStr">
         <is>
           <t>Campaña</t>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="C43" s="24" t="inlineStr">
         <is>
-          <t>• Ceremonia de aspersión con acompañamiento durante la temporada de Difuntos
+          <t>• Ceremonia de aspersión con acompañamiento durante la temporada del Día de los Muertos
 • Complemento natural para quienes contratan la Solución Modular</t>
         </is>
       </c>
@@ -1832,7 +1832,7 @@
     <row r="63" ht="20" customHeight="1">
       <c r="B63" s="20" t="inlineStr">
         <is>
-          <t>DIFERENCIALES DE LA CAMPAÑA DE DIFUNTOS</t>
+          <t>DIFERENCIALES DE LA CAMPAÑA DÍA DE LOS MUERTOS</t>
         </is>
       </c>
       <c r="C63" s="21" t="n"/>
@@ -2077,7 +2077,7 @@
     <row r="84" ht="20" customHeight="1">
       <c r="B84" s="20" t="inlineStr">
         <is>
-          <t>DIFERENCIALES DE LA CAMPAÑA DE DIFUNTOS</t>
+          <t>DIFERENCIALES DE LA CAMPAÑA DÍA DE LOS MUERTOS</t>
         </is>
       </c>
       <c r="C84" s="21" t="n"/>
@@ -2321,7 +2321,7 @@
     <row r="105" ht="20" customHeight="1">
       <c r="B105" s="20" t="inlineStr">
         <is>
-          <t>DIFERENCIALES DE LA CAMPAÑA DE DIFUNTOS</t>
+          <t>DIFERENCIALES DE LA CAMPAÑA DÍA DE LOS MUERTOS</t>
         </is>
       </c>
       <c r="C105" s="21" t="n"/>

</xml_diff>

<commit_message>
Actualiza fichas: columbario incluido, precios únicos, sin diferenciales de campaña
- Solución Modular: columbario 1 año pasa a servicio incluido; US$ 1.000
- Aspersión: sin mantenimiento; agrega placa memorial; US$ 250
- Jardín de Cenizas: versiones Individual (US$ 600) y Familiar (variable)
- PET: pago único US$ 500, sin recurrencia mensual
- Elimina columna/bloque de diferenciales de campaña

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111i7vn9WWo4QxCQbucWbrF
</commit_message>
<xml_diff>
--- a/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
+++ b/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
@@ -11,9 +11,9 @@
     <sheet name="Ficha Técnica Consolidada" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tabla Gral. - Visión Comercial'!$A$4:$J$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tabla Gral. - Visión Comercial'!$A$4:$I$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Tabla Gral. - Visión Comercial'!$4:$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Ficha Técnica Consolidada'!$A$1:$F$109</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Ficha Técnica Consolidada'!$A$1:$F$98</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -707,7 +707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -719,7 +719,6 @@
     <col width="36" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="34" customWidth="1" min="9" max="9"/>
-    <col width="44" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -782,13 +781,8 @@
           <t>Condiciones de Pago / Financiamiento</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>Observaciones del Lanzamiento (Día de los Muertos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="78.5" customHeight="1">
+    </row>
+    <row r="5" ht="93" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>VG-CRE-01</t>
@@ -819,6 +813,7 @@
           <t>• Proceso completo de cremación individual
 • Urna cineraria de línea modular
 • Trámites legales básicos
+• Alquiler temporal de columbario por 1 año
 • Integración al plan funerario base (actual o nuevo)</t>
         </is>
       </c>
@@ -829,23 +824,17 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>US$ 700 – US$ 1.000
-(Según el plan base)</t>
+          <t>US$ 1.000
+(Por módulo individual)</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>Hasta 120 cuotas mensuales (aprox. US$ 6,00 – US$ 8,50/mes).</t>
-        </is>
-      </c>
-      <c r="J5" s="6" t="inlineStr">
-        <is>
-          <t>• BONO ESPECIAL: Alquiler temporal de columbario por 1 año incluido
-• Producto ancla de la campaña: cuota de entrada más accesible del portafolio</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="78.5" customHeight="1">
+          <t>Hasta 120 cuotas mensuales (aprox. US$ 8,50/mes).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="93" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>VG-CRE-02</t>
@@ -876,7 +865,7 @@
           <t>• Acompañamiento ceremonial
 • Tiempo privado para la familia en entorno botánico
 • Asistencia protocolar
-• Mantenimiento del área</t>
+• Placa memorial que registra la aspersión realizada en el lugar</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
@@ -886,36 +875,30 @@
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>US$ 150 – US$ 250
+          <t>US$ 250
 (Pago único por servicio)</t>
         </is>
       </c>
       <c r="I6" s="10" t="inlineStr">
         <is>
           <t>Pago único; combinable con la Solución Modular de Cremación.</t>
-        </is>
-      </c>
-      <c r="J6" s="10" t="inlineStr">
-        <is>
-          <t>• Ceremonia de aspersión con acompañamiento durante la temporada del Día de los Muertos
-• Complemento natural para quienes contratan la Solución Modular</t>
         </is>
       </c>
     </row>
     <row r="7" ht="64" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>VG-CRE-03S</t>
+          <t>VG-CRE-03I</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Jardín de Cenizas · Standard</t>
+          <t>Jardín de Cenizas · Individual</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Destino final · Inhumación</t>
+          <t>Destino final · Inhumación individual</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -925,7 +908,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Individual (o paquete doble promocional).</t>
+          <t>Individual.</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -943,30 +926,25 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>US$ 400 – US$ 600
+          <t>US$ 600
 (Por espacio individual)</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
           <t>Pago único o financiado según política comercial vigente.</t>
-        </is>
-      </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>• Paquete doble promocional disponible durante la campaña</t>
         </is>
       </c>
     </row>
     <row r="8" ht="78.5" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>VG-CRE-03P</t>
+          <t>VG-CRE-03F</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Jardín de Cenizas · Premium</t>
+          <t>Jardín de Cenizas · Familiar</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
@@ -1000,17 +978,12 @@
       <c r="H8" s="11" t="inlineStr">
         <is>
           <t>US$ 1.490 – US$ 1.990
-(Por parcela familiar (hasta 4 espacios))</t>
+(Variable según la cantidad de personas · hasta 4 espacios)</t>
         </is>
       </c>
       <c r="I8" s="10" t="inlineStr">
         <is>
           <t>Pago único o financiado según política comercial vigente.</t>
-        </is>
-      </c>
-      <c r="J8" s="10" t="inlineStr">
-        <is>
-          <t>• Selección prioritaria de ubicación VIP durante la campaña</t>
         </is>
       </c>
     </row>
@@ -1054,26 +1027,21 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>US$ 5/mes
-(Adicional al plan)</t>
+          <t>US$ 500
+(Pago único por servicio)</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>US$ 5,00/mes adicional al plan, o tarifa única proporcional (add-on).</t>
-        </is>
-      </c>
-      <c r="J9" s="6" t="inlineStr">
-        <is>
-          <t>• Extensión del plan familiar a las mascotas con una cuota mínima</t>
+          <t>Pago único; puede contratarse como adicional al plan funerario.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J9"/>
+  <autoFilter ref="A4:I9"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -1087,7 +1055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:E108"/>
+  <dimension ref="B1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1243,18 +1211,18 @@
     <row r="14" ht="20.5" customHeight="1">
       <c r="B14" s="23" t="inlineStr">
         <is>
-          <t>Bono de lanzamiento</t>
+          <t>Columbario</t>
         </is>
       </c>
       <c r="C14" s="24" t="inlineStr">
         <is>
-          <t>Columbario temporal · 12 meses</t>
+          <t>Alquiler temporal · 12 meses incluido</t>
         </is>
       </c>
       <c r="D14" s="25" t="n"/>
       <c r="E14" s="26" t="n"/>
     </row>
-    <row r="15" ht="64" customHeight="1">
+    <row r="15" ht="78.5" customHeight="1">
       <c r="B15" s="27" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
@@ -1265,6 +1233,7 @@
           <t>• Proceso completo de cremación individual
 • Urna cineraria de línea modular
 • Trámites legales básicos
+• Alquiler temporal de columbario por 1 año
 • Integración al plan funerario base (actual o nuevo)</t>
         </is>
       </c>
@@ -1289,7 +1258,7 @@
       </c>
       <c r="C17" s="31" t="inlineStr">
         <is>
-          <t>US$ 700 – US$ 1.000</t>
+          <t>US$ 1.000</t>
         </is>
       </c>
       <c r="D17" s="25" t="n"/>
@@ -1303,7 +1272,7 @@
       </c>
       <c r="C18" s="28" t="inlineStr">
         <is>
-          <t>Según el plan base</t>
+          <t>Por módulo individual</t>
         </is>
       </c>
       <c r="D18" s="29" t="n"/>
@@ -1317,7 +1286,7 @@
       </c>
       <c r="C19" s="24" t="inlineStr">
         <is>
-          <t>Hasta 120 cuotas mensuales (aprox. US$ 6,00 – US$ 8,50/mes).</t>
+          <t>Hasta 120 cuotas mensuales (aprox. US$ 8,50/mes).</t>
         </is>
       </c>
       <c r="D19" s="25" t="n"/>
@@ -1331,7 +1300,7 @@
       </c>
       <c r="C20" s="28" t="inlineStr">
         <is>
-          <t>US$ 5,83 – US$ 8,33 sin intereses (120 cuotas)</t>
+          <t>US$ 8,33/mes sin intereses (120 cuotas)</t>
         </is>
       </c>
       <c r="D20" s="29" t="n"/>
@@ -1340,7 +1309,7 @@
     <row r="21" ht="20" customHeight="1">
       <c r="B21" s="20" t="inlineStr">
         <is>
-          <t>DIFERENCIALES DE LA CAMPAÑA DÍA DE LOS MUERTOS</t>
+          <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
       <c r="C21" s="21" t="n"/>
@@ -1348,125 +1317,128 @@
       <c r="E21" s="22" t="n"/>
     </row>
     <row r="22" ht="35" customHeight="1">
-      <c r="B22" s="23" t="inlineStr">
-        <is>
-          <t>Campaña</t>
-        </is>
-      </c>
-      <c r="C22" s="24" t="inlineStr">
-        <is>
-          <t>• BONO ESPECIAL: Alquiler temporal de columbario por 1 año incluido
-• Producto ancla de la campaña: cuota de entrada más accesible del portafolio</t>
-        </is>
-      </c>
-      <c r="D22" s="25" t="n"/>
-      <c r="E22" s="26" t="n"/>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="B23" s="20" t="inlineStr">
-        <is>
-          <t>PERFIL DEL COMPRADOR</t>
-        </is>
-      </c>
-      <c r="C23" s="21" t="n"/>
-      <c r="D23" s="21" t="n"/>
-      <c r="E23" s="22" t="n"/>
-    </row>
-    <row r="24" ht="35" customHeight="1">
-      <c r="B24" s="32" t="inlineStr">
+      <c r="B22" s="32" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C24" s="33" t="inlineStr">
+      <c r="C22" s="33" t="inlineStr">
         <is>
           <t>Afiliados actuales y nuevos que desean incorporar la cremación a su plan con una cuota mensual mínima.</t>
         </is>
       </c>
-      <c r="D24" s="34" t="n"/>
-      <c r="E24" s="35" t="n"/>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="B27" s="14" t="inlineStr">
+      <c r="D22" s="34" t="n"/>
+      <c r="E22" s="35" t="n"/>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="B25" s="14" t="inlineStr">
         <is>
           <t>JARDÍN DE ASPERSIÓN DE CENIZAS</t>
         </is>
       </c>
-      <c r="C27" s="15" t="n"/>
-      <c r="D27" s="15" t="n"/>
-      <c r="E27" s="16" t="inlineStr">
+      <c r="C25" s="15" t="n"/>
+      <c r="D25" s="15" t="n"/>
+      <c r="E25" s="16" t="inlineStr">
         <is>
           <t>VG-CRE-02</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="B28" s="17" t="inlineStr">
+    <row r="26" ht="20" customHeight="1">
+      <c r="B26" s="17" t="inlineStr">
         <is>
           <t>Jardines de la Memoria  ·  Destino final · Aspersión</t>
         </is>
       </c>
-      <c r="C28" s="18" t="n"/>
-      <c r="D28" s="18" t="n"/>
-      <c r="E28" s="19" t="n"/>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="B29" s="20" t="inlineStr">
+      <c r="C26" s="18" t="n"/>
+      <c r="D26" s="18" t="n"/>
+      <c r="E26" s="19" t="n"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="B27" s="20" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C29" s="21" t="n"/>
-      <c r="D29" s="21" t="n"/>
-      <c r="E29" s="22" t="n"/>
-    </row>
-    <row r="30" ht="35" customHeight="1">
-      <c r="B30" s="23" t="inlineStr">
+      <c r="C27" s="21" t="n"/>
+      <c r="D27" s="21" t="n"/>
+      <c r="E27" s="22" t="n"/>
+    </row>
+    <row r="28" ht="35" customHeight="1">
+      <c r="B28" s="23" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C30" s="24" t="inlineStr">
+      <c r="C28" s="24" t="inlineStr">
         <is>
           <t>Área reservada en jardín natural para la liberación ceremonial de cenizas, en armonía con la naturaleza.</t>
         </is>
       </c>
-      <c r="D30" s="25" t="n"/>
-      <c r="E30" s="26" t="n"/>
+      <c r="D28" s="25" t="n"/>
+      <c r="E28" s="26" t="n"/>
+    </row>
+    <row r="29" ht="20.5" customHeight="1">
+      <c r="B29" s="27" t="inlineStr">
+        <is>
+          <t>Capacidad / Cobertura</t>
+        </is>
+      </c>
+      <c r="C29" s="28" t="inlineStr">
+        <is>
+          <t>Servicio individual.</t>
+        </is>
+      </c>
+      <c r="D29" s="29" t="n"/>
+      <c r="E29" s="30" t="n"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="B30" s="20" t="inlineStr">
+        <is>
+          <t>ESPECIFICACIONES TÉCNICAS</t>
+        </is>
+      </c>
+      <c r="C30" s="21" t="n"/>
+      <c r="D30" s="21" t="n"/>
+      <c r="E30" s="22" t="n"/>
     </row>
     <row r="31" ht="20.5" customHeight="1">
-      <c r="B31" s="27" t="inlineStr">
-        <is>
-          <t>Capacidad / Cobertura</t>
-        </is>
-      </c>
-      <c r="C31" s="28" t="inlineStr">
-        <is>
-          <t>Servicio individual.</t>
-        </is>
-      </c>
-      <c r="D31" s="29" t="n"/>
-      <c r="E31" s="30" t="n"/>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="B32" s="20" t="inlineStr">
-        <is>
-          <t>ESPECIFICACIONES TÉCNICAS</t>
-        </is>
-      </c>
-      <c r="C32" s="21" t="n"/>
-      <c r="D32" s="21" t="n"/>
-      <c r="E32" s="22" t="n"/>
+      <c r="B31" s="23" t="inlineStr">
+        <is>
+          <t>Tipo de producto</t>
+        </is>
+      </c>
+      <c r="C31" s="24" t="inlineStr">
+        <is>
+          <t>Servicio ceremonial de destino final</t>
+        </is>
+      </c>
+      <c r="D31" s="25" t="n"/>
+      <c r="E31" s="26" t="n"/>
+    </row>
+    <row r="32" ht="20.5" customHeight="1">
+      <c r="B32" s="27" t="inlineStr">
+        <is>
+          <t>Capacidad</t>
+        </is>
+      </c>
+      <c r="C32" s="28" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="D32" s="29" t="n"/>
+      <c r="E32" s="30" t="n"/>
     </row>
     <row r="33" ht="20.5" customHeight="1">
       <c r="B33" s="23" t="inlineStr">
         <is>
-          <t>Tipo de producto</t>
+          <t>Espacio</t>
         </is>
       </c>
       <c r="C33" s="24" t="inlineStr">
         <is>
-          <t>Servicio ceremonial de destino final</t>
+          <t>Jardín natural reservado (sin espacio fijo asignado)</t>
         </is>
       </c>
       <c r="D33" s="25" t="n"/>
@@ -1475,298 +1447,245 @@
     <row r="34" ht="20.5" customHeight="1">
       <c r="B34" s="27" t="inlineStr">
         <is>
-          <t>Capacidad</t>
+          <t>Homenaje</t>
         </is>
       </c>
       <c r="C34" s="28" t="inlineStr">
         <is>
-          <t>Individual</t>
+          <t>Placa memorial de la aspersión</t>
         </is>
       </c>
       <c r="D34" s="29" t="n"/>
       <c r="E34" s="30" t="n"/>
     </row>
-    <row r="35" ht="20.5" customHeight="1">
+    <row r="35" ht="64" customHeight="1">
       <c r="B35" s="23" t="inlineStr">
         <is>
-          <t>Espacio</t>
+          <t>Servicios incluidos</t>
         </is>
       </c>
       <c r="C35" s="24" t="inlineStr">
-        <is>
-          <t>Jardín natural reservado (sin espacio fijo asignado)</t>
-        </is>
-      </c>
-      <c r="D35" s="25" t="n"/>
-      <c r="E35" s="26" t="n"/>
-    </row>
-    <row r="36" ht="20.5" customHeight="1">
-      <c r="B36" s="27" t="inlineStr">
-        <is>
-          <t>Mantenimiento</t>
-        </is>
-      </c>
-      <c r="C36" s="28" t="inlineStr">
-        <is>
-          <t>Incluido</t>
-        </is>
-      </c>
-      <c r="D36" s="29" t="n"/>
-      <c r="E36" s="30" t="n"/>
-    </row>
-    <row r="37" ht="64" customHeight="1">
-      <c r="B37" s="23" t="inlineStr">
-        <is>
-          <t>Servicios incluidos</t>
-        </is>
-      </c>
-      <c r="C37" s="24" t="inlineStr">
         <is>
           <t>• Acompañamiento ceremonial
 • Tiempo privado para la familia en entorno botánico
 • Asistencia protocolar
-• Mantenimiento del área</t>
+• Placa memorial que registra la aspersión realizada en el lugar</t>
+        </is>
+      </c>
+      <c r="D35" s="25" t="n"/>
+      <c r="E35" s="26" t="n"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="B36" s="20" t="inlineStr">
+        <is>
+          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
+        </is>
+      </c>
+      <c r="C36" s="21" t="n"/>
+      <c r="D36" s="21" t="n"/>
+      <c r="E36" s="22" t="n"/>
+    </row>
+    <row r="37" ht="26.5" customHeight="1">
+      <c r="B37" s="23" t="inlineStr">
+        <is>
+          <t>Precio sugerido</t>
+        </is>
+      </c>
+      <c r="C37" s="31" t="inlineStr">
+        <is>
+          <t>US$ 250</t>
         </is>
       </c>
       <c r="D37" s="25" t="n"/>
       <c r="E37" s="26" t="n"/>
     </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="B38" s="20" t="inlineStr">
-        <is>
-          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
-        </is>
-      </c>
-      <c r="C38" s="21" t="n"/>
-      <c r="D38" s="21" t="n"/>
-      <c r="E38" s="22" t="n"/>
-    </row>
-    <row r="39" ht="26.5" customHeight="1">
+    <row r="38" ht="20.5" customHeight="1">
+      <c r="B38" s="27" t="inlineStr">
+        <is>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C38" s="28" t="inlineStr">
+        <is>
+          <t>Pago único por servicio</t>
+        </is>
+      </c>
+      <c r="D38" s="29" t="n"/>
+      <c r="E38" s="30" t="n"/>
+    </row>
+    <row r="39" ht="20.5" customHeight="1">
       <c r="B39" s="23" t="inlineStr">
         <is>
-          <t>Precio sugerido</t>
-        </is>
-      </c>
-      <c r="C39" s="31" t="inlineStr">
-        <is>
-          <t>US$ 150 – US$ 250</t>
+          <t>Condiciones</t>
+        </is>
+      </c>
+      <c r="C39" s="24" t="inlineStr">
+        <is>
+          <t>Pago único; combinable con la Solución Modular de Cremación.</t>
         </is>
       </c>
       <c r="D39" s="25" t="n"/>
       <c r="E39" s="26" t="n"/>
     </row>
-    <row r="40" ht="20.5" customHeight="1">
-      <c r="B40" s="27" t="inlineStr">
-        <is>
-          <t>Base de precio</t>
-        </is>
-      </c>
-      <c r="C40" s="28" t="inlineStr">
-        <is>
-          <t>Pago único por servicio</t>
-        </is>
-      </c>
-      <c r="D40" s="29" t="n"/>
-      <c r="E40" s="30" t="n"/>
-    </row>
-    <row r="41" ht="20.5" customHeight="1">
-      <c r="B41" s="23" t="inlineStr">
-        <is>
-          <t>Condiciones</t>
-        </is>
-      </c>
-      <c r="C41" s="24" t="inlineStr">
-        <is>
-          <t>Pago único; combinable con la Solución Modular de Cremación.</t>
-        </is>
-      </c>
-      <c r="D41" s="25" t="n"/>
-      <c r="E41" s="26" t="n"/>
-    </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="B42" s="20" t="inlineStr">
-        <is>
-          <t>DIFERENCIALES DE LA CAMPAÑA DÍA DE LOS MUERTOS</t>
-        </is>
-      </c>
-      <c r="C42" s="21" t="n"/>
-      <c r="D42" s="21" t="n"/>
-      <c r="E42" s="22" t="n"/>
-    </row>
-    <row r="43" ht="49.5" customHeight="1">
-      <c r="B43" s="23" t="inlineStr">
-        <is>
-          <t>Campaña</t>
-        </is>
-      </c>
-      <c r="C43" s="24" t="inlineStr">
-        <is>
-          <t>• Ceremonia de aspersión con acompañamiento durante la temporada del Día de los Muertos
-• Complemento natural para quienes contratan la Solución Modular</t>
-        </is>
-      </c>
-      <c r="D43" s="25" t="n"/>
-      <c r="E43" s="26" t="n"/>
-    </row>
-    <row r="44" ht="20" customHeight="1">
-      <c r="B44" s="20" t="inlineStr">
+    <row r="40" ht="20" customHeight="1">
+      <c r="B40" s="20" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C44" s="21" t="n"/>
-      <c r="D44" s="21" t="n"/>
-      <c r="E44" s="22" t="n"/>
-    </row>
-    <row r="45" ht="35" customHeight="1">
-      <c r="B45" s="32" t="inlineStr">
+      <c r="C40" s="21" t="n"/>
+      <c r="D40" s="21" t="n"/>
+      <c r="E40" s="22" t="n"/>
+    </row>
+    <row r="41" ht="35" customHeight="1">
+      <c r="B41" s="32" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C45" s="33" t="inlineStr">
+      <c r="C41" s="33" t="inlineStr">
         <is>
           <t>Personas que buscan un concepto de libertad total, sin necesidad de un espacio físico fijo.</t>
         </is>
       </c>
-      <c r="D45" s="34" t="n"/>
-      <c r="E45" s="35" t="n"/>
-    </row>
-    <row r="48" ht="30" customHeight="1">
-      <c r="B48" s="14" t="inlineStr">
-        <is>
-          <t>JARDÍN DE CENIZAS · STANDARD</t>
-        </is>
-      </c>
-      <c r="C48" s="15" t="n"/>
-      <c r="D48" s="15" t="n"/>
-      <c r="E48" s="16" t="inlineStr">
-        <is>
-          <t>VG-CRE-03S</t>
-        </is>
-      </c>
+      <c r="D41" s="34" t="n"/>
+      <c r="E41" s="35" t="n"/>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>JARDÍN DE CENIZAS · INDIVIDUAL</t>
+        </is>
+      </c>
+      <c r="C44" s="15" t="n"/>
+      <c r="D44" s="15" t="n"/>
+      <c r="E44" s="16" t="inlineStr">
+        <is>
+          <t>VG-CRE-03I</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="B45" s="17" t="inlineStr">
+        <is>
+          <t>Jardines de la Memoria · Inhumación  ·  Destino final · Inhumación individual</t>
+        </is>
+      </c>
+      <c r="C45" s="18" t="n"/>
+      <c r="D45" s="18" t="n"/>
+      <c r="E45" s="19" t="n"/>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="B46" s="20" t="inlineStr">
+        <is>
+          <t>VISIÓN GENERAL</t>
+        </is>
+      </c>
+      <c r="C46" s="21" t="n"/>
+      <c r="D46" s="21" t="n"/>
+      <c r="E46" s="22" t="n"/>
+    </row>
+    <row r="47" ht="35" customHeight="1">
+      <c r="B47" s="23" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="C47" s="24" t="inlineStr">
+        <is>
+          <t>Inhumación de urnas en parcelas ajardinadas con demarcación personalizada: un lugar físico permanente de homenaje.</t>
+        </is>
+      </c>
+      <c r="D47" s="25" t="n"/>
+      <c r="E47" s="26" t="n"/>
+    </row>
+    <row r="48" ht="20.5" customHeight="1">
+      <c r="B48" s="27" t="inlineStr">
+        <is>
+          <t>Capacidad / Cobertura</t>
+        </is>
+      </c>
+      <c r="C48" s="28" t="inlineStr">
+        <is>
+          <t>Individual.</t>
+        </is>
+      </c>
+      <c r="D48" s="29" t="n"/>
+      <c r="E48" s="30" t="n"/>
     </row>
     <row r="49" ht="20" customHeight="1">
-      <c r="B49" s="17" t="inlineStr">
-        <is>
-          <t>Jardines de la Memoria · Inhumación  ·  Destino final · Inhumación</t>
-        </is>
-      </c>
-      <c r="C49" s="18" t="n"/>
-      <c r="D49" s="18" t="n"/>
-      <c r="E49" s="19" t="n"/>
-    </row>
-    <row r="50" ht="20" customHeight="1">
-      <c r="B50" s="20" t="inlineStr">
-        <is>
-          <t>VISIÓN GENERAL</t>
-        </is>
-      </c>
-      <c r="C50" s="21" t="n"/>
-      <c r="D50" s="21" t="n"/>
-      <c r="E50" s="22" t="n"/>
-    </row>
-    <row r="51" ht="35" customHeight="1">
-      <c r="B51" s="23" t="inlineStr">
-        <is>
-          <t>Concepto</t>
-        </is>
-      </c>
-      <c r="C51" s="24" t="inlineStr">
-        <is>
-          <t>Inhumación de urnas en parcelas ajardinadas con demarcación personalizada: un lugar físico permanente de homenaje.</t>
-        </is>
-      </c>
-      <c r="D51" s="25" t="n"/>
-      <c r="E51" s="26" t="n"/>
+      <c r="B49" s="20" t="inlineStr">
+        <is>
+          <t>ESPECIFICACIONES TÉCNICAS</t>
+        </is>
+      </c>
+      <c r="C49" s="21" t="n"/>
+      <c r="D49" s="21" t="n"/>
+      <c r="E49" s="22" t="n"/>
+    </row>
+    <row r="50" ht="20.5" customHeight="1">
+      <c r="B50" s="23" t="inlineStr">
+        <is>
+          <t>Versión</t>
+        </is>
+      </c>
+      <c r="C50" s="24" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="D50" s="25" t="n"/>
+      <c r="E50" s="26" t="n"/>
+    </row>
+    <row r="51" ht="20.5" customHeight="1">
+      <c r="B51" s="27" t="inlineStr">
+        <is>
+          <t>Capacidad</t>
+        </is>
+      </c>
+      <c r="C51" s="28" t="inlineStr">
+        <is>
+          <t>1 espacio</t>
+        </is>
+      </c>
+      <c r="D51" s="29" t="n"/>
+      <c r="E51" s="30" t="n"/>
     </row>
     <row r="52" ht="20.5" customHeight="1">
-      <c r="B52" s="27" t="inlineStr">
-        <is>
-          <t>Capacidad / Cobertura</t>
-        </is>
-      </c>
-      <c r="C52" s="28" t="inlineStr">
-        <is>
-          <t>Individual (o paquete doble promocional).</t>
-        </is>
-      </c>
-      <c r="D52" s="29" t="n"/>
-      <c r="E52" s="30" t="n"/>
-    </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="B53" s="20" t="inlineStr">
-        <is>
-          <t>ESPECIFICACIONES TÉCNICAS</t>
-        </is>
-      </c>
-      <c r="C53" s="21" t="n"/>
-      <c r="D53" s="21" t="n"/>
-      <c r="E53" s="22" t="n"/>
-    </row>
-    <row r="54" ht="20.5" customHeight="1">
+      <c r="B52" s="23" t="inlineStr">
+        <is>
+          <t>Ubicación</t>
+        </is>
+      </c>
+      <c r="C52" s="24" t="inlineStr">
+        <is>
+          <t>Sectores ajardinados generales</t>
+        </is>
+      </c>
+      <c r="D52" s="25" t="n"/>
+      <c r="E52" s="26" t="n"/>
+    </row>
+    <row r="53" ht="20.5" customHeight="1">
+      <c r="B53" s="27" t="inlineStr">
+        <is>
+          <t>Homenaje</t>
+        </is>
+      </c>
+      <c r="C53" s="28" t="inlineStr">
+        <is>
+          <t>Placa conmemorativa individual estándar</t>
+        </is>
+      </c>
+      <c r="D53" s="29" t="n"/>
+      <c r="E53" s="30" t="n"/>
+    </row>
+    <row r="54" ht="64" customHeight="1">
       <c r="B54" s="23" t="inlineStr">
         <is>
-          <t>Versión</t>
+          <t>Servicios incluidos</t>
         </is>
       </c>
       <c r="C54" s="24" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="D54" s="25" t="n"/>
-      <c r="E54" s="26" t="n"/>
-    </row>
-    <row r="55" ht="20.5" customHeight="1">
-      <c r="B55" s="27" t="inlineStr">
-        <is>
-          <t>Capacidad</t>
-        </is>
-      </c>
-      <c r="C55" s="28" t="inlineStr">
-        <is>
-          <t>Individual (o paquete doble promocional)</t>
-        </is>
-      </c>
-      <c r="D55" s="29" t="n"/>
-      <c r="E55" s="30" t="n"/>
-    </row>
-    <row r="56" ht="20.5" customHeight="1">
-      <c r="B56" s="23" t="inlineStr">
-        <is>
-          <t>Ubicación</t>
-        </is>
-      </c>
-      <c r="C56" s="24" t="inlineStr">
-        <is>
-          <t>Sectores ajardinados generales</t>
-        </is>
-      </c>
-      <c r="D56" s="25" t="n"/>
-      <c r="E56" s="26" t="n"/>
-    </row>
-    <row r="57" ht="20.5" customHeight="1">
-      <c r="B57" s="27" t="inlineStr">
-        <is>
-          <t>Homenaje</t>
-        </is>
-      </c>
-      <c r="C57" s="28" t="inlineStr">
-        <is>
-          <t>Placa conmemorativa individual estándar</t>
-        </is>
-      </c>
-      <c r="D57" s="29" t="n"/>
-      <c r="E57" s="30" t="n"/>
-    </row>
-    <row r="58" ht="64" customHeight="1">
-      <c r="B58" s="23" t="inlineStr">
-        <is>
-          <t>Servicios incluidos</t>
-        </is>
-      </c>
-      <c r="C58" s="24" t="inlineStr">
         <is>
           <t>• Inhumación de urna en parcela ajardinada
 • Ubicación en sectores ajardinados generales
@@ -1774,89 +1693,113 @@
 • Lugar físico permanente de homenaje</t>
         </is>
       </c>
+      <c r="D54" s="25" t="n"/>
+      <c r="E54" s="26" t="n"/>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="B55" s="20" t="inlineStr">
+        <is>
+          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
+        </is>
+      </c>
+      <c r="C55" s="21" t="n"/>
+      <c r="D55" s="21" t="n"/>
+      <c r="E55" s="22" t="n"/>
+    </row>
+    <row r="56" ht="26.5" customHeight="1">
+      <c r="B56" s="23" t="inlineStr">
+        <is>
+          <t>Precio sugerido</t>
+        </is>
+      </c>
+      <c r="C56" s="31" t="inlineStr">
+        <is>
+          <t>US$ 600</t>
+        </is>
+      </c>
+      <c r="D56" s="25" t="n"/>
+      <c r="E56" s="26" t="n"/>
+    </row>
+    <row r="57" ht="20.5" customHeight="1">
+      <c r="B57" s="27" t="inlineStr">
+        <is>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C57" s="28" t="inlineStr">
+        <is>
+          <t>Por espacio individual</t>
+        </is>
+      </c>
+      <c r="D57" s="29" t="n"/>
+      <c r="E57" s="30" t="n"/>
+    </row>
+    <row r="58" ht="20.5" customHeight="1">
+      <c r="B58" s="23" t="inlineStr">
+        <is>
+          <t>Condiciones</t>
+        </is>
+      </c>
+      <c r="C58" s="24" t="inlineStr">
+        <is>
+          <t>Pago único o financiado según política comercial vigente.</t>
+        </is>
+      </c>
       <c r="D58" s="25" t="n"/>
       <c r="E58" s="26" t="n"/>
     </row>
     <row r="59" ht="20" customHeight="1">
       <c r="B59" s="20" t="inlineStr">
         <is>
-          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
+          <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
       <c r="C59" s="21" t="n"/>
       <c r="D59" s="21" t="n"/>
       <c r="E59" s="22" t="n"/>
     </row>
-    <row r="60" ht="26.5" customHeight="1">
-      <c r="B60" s="23" t="inlineStr">
-        <is>
-          <t>Precio sugerido</t>
-        </is>
-      </c>
-      <c r="C60" s="31" t="inlineStr">
-        <is>
-          <t>US$ 400 – US$ 600</t>
-        </is>
-      </c>
-      <c r="D60" s="25" t="n"/>
-      <c r="E60" s="26" t="n"/>
-    </row>
-    <row r="61" ht="20.5" customHeight="1">
-      <c r="B61" s="27" t="inlineStr">
-        <is>
-          <t>Base de precio</t>
-        </is>
-      </c>
-      <c r="C61" s="28" t="inlineStr">
-        <is>
-          <t>Por espacio individual</t>
-        </is>
-      </c>
-      <c r="D61" s="29" t="n"/>
-      <c r="E61" s="30" t="n"/>
-    </row>
-    <row r="62" ht="20.5" customHeight="1">
-      <c r="B62" s="23" t="inlineStr">
-        <is>
-          <t>Condiciones</t>
-        </is>
-      </c>
-      <c r="C62" s="24" t="inlineStr">
-        <is>
-          <t>Pago único o financiado según política comercial vigente.</t>
-        </is>
-      </c>
-      <c r="D62" s="25" t="n"/>
-      <c r="E62" s="26" t="n"/>
-    </row>
-    <row r="63" ht="20" customHeight="1">
-      <c r="B63" s="20" t="inlineStr">
-        <is>
-          <t>DIFERENCIALES DE LA CAMPAÑA DÍA DE LOS MUERTOS</t>
-        </is>
-      </c>
-      <c r="C63" s="21" t="n"/>
-      <c r="D63" s="21" t="n"/>
-      <c r="E63" s="22" t="n"/>
-    </row>
-    <row r="64" ht="20.5" customHeight="1">
-      <c r="B64" s="23" t="inlineStr">
-        <is>
-          <t>Campaña</t>
-        </is>
-      </c>
-      <c r="C64" s="24" t="inlineStr">
-        <is>
-          <t>• Paquete doble promocional disponible durante la campaña</t>
-        </is>
-      </c>
-      <c r="D64" s="25" t="n"/>
-      <c r="E64" s="26" t="n"/>
+    <row r="60" ht="35" customHeight="1">
+      <c r="B60" s="32" t="inlineStr">
+        <is>
+          <t>Cliente objetivo</t>
+        </is>
+      </c>
+      <c r="C60" s="33" t="inlineStr">
+        <is>
+          <t>Familias que desean un lugar permanente para visitar y rendir homenaje, con una inversión moderada.</t>
+        </is>
+      </c>
+      <c r="D60" s="34" t="n"/>
+      <c r="E60" s="35" t="n"/>
+    </row>
+    <row r="63" ht="30" customHeight="1">
+      <c r="B63" s="14" t="inlineStr">
+        <is>
+          <t>JARDÍN DE CENIZAS · FAMILIAR</t>
+        </is>
+      </c>
+      <c r="C63" s="15" t="n"/>
+      <c r="D63" s="15" t="n"/>
+      <c r="E63" s="16" t="inlineStr">
+        <is>
+          <t>VG-CRE-03F</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="20" customHeight="1">
+      <c r="B64" s="17" t="inlineStr">
+        <is>
+          <t>Jardines de la Memoria · Inhumación  ·  Destino final · Inhumación familiar</t>
+        </is>
+      </c>
+      <c r="C64" s="18" t="n"/>
+      <c r="D64" s="18" t="n"/>
+      <c r="E64" s="19" t="n"/>
     </row>
     <row r="65" ht="20" customHeight="1">
       <c r="B65" s="20" t="inlineStr">
         <is>
-          <t>PERFIL DEL COMPRADOR</t>
+          <t>VISIÓN GENERAL</t>
         </is>
       </c>
       <c r="C65" s="21" t="n"/>
@@ -1864,154 +1807,106 @@
       <c r="E65" s="22" t="n"/>
     </row>
     <row r="66" ht="35" customHeight="1">
-      <c r="B66" s="32" t="inlineStr">
-        <is>
-          <t>Cliente objetivo</t>
-        </is>
-      </c>
-      <c r="C66" s="33" t="inlineStr">
-        <is>
-          <t>Familias que desean un lugar permanente para visitar y rendir homenaje, con una inversión moderada.</t>
-        </is>
-      </c>
-      <c r="D66" s="34" t="n"/>
-      <c r="E66" s="35" t="n"/>
-    </row>
-    <row r="69" ht="30" customHeight="1">
-      <c r="B69" s="14" t="inlineStr">
-        <is>
-          <t>JARDÍN DE CENIZAS · PREMIUM</t>
-        </is>
-      </c>
-      <c r="C69" s="15" t="n"/>
-      <c r="D69" s="15" t="n"/>
-      <c r="E69" s="16" t="inlineStr">
-        <is>
-          <t>VG-CRE-03P</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="20" customHeight="1">
-      <c r="B70" s="17" t="inlineStr">
-        <is>
-          <t>Jardines de la Memoria · Inhumación  ·  Destino final · Inhumación familiar</t>
-        </is>
-      </c>
-      <c r="C70" s="18" t="n"/>
-      <c r="D70" s="18" t="n"/>
-      <c r="E70" s="19" t="n"/>
-    </row>
-    <row r="71" ht="20" customHeight="1">
-      <c r="B71" s="20" t="inlineStr">
-        <is>
-          <t>VISIÓN GENERAL</t>
-        </is>
-      </c>
-      <c r="C71" s="21" t="n"/>
-      <c r="D71" s="21" t="n"/>
-      <c r="E71" s="22" t="n"/>
-    </row>
-    <row r="72" ht="35" customHeight="1">
-      <c r="B72" s="23" t="inlineStr">
+      <c r="B66" s="23" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C72" s="24" t="inlineStr">
+      <c r="C66" s="24" t="inlineStr">
         <is>
           <t>Inhumación familiar de urnas en sectores VIP del parque, con placa patrimonial de acabado superior.</t>
         </is>
       </c>
-      <c r="D72" s="25" t="n"/>
-      <c r="E72" s="26" t="n"/>
-    </row>
-    <row r="73" ht="20.5" customHeight="1">
-      <c r="B73" s="27" t="inlineStr">
+      <c r="D66" s="25" t="n"/>
+      <c r="E66" s="26" t="n"/>
+    </row>
+    <row r="67" ht="20.5" customHeight="1">
+      <c r="B67" s="27" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C73" s="28" t="inlineStr">
+      <c r="C67" s="28" t="inlineStr">
         <is>
           <t>Hasta 4 espacios (familiar).</t>
         </is>
       </c>
-      <c r="D73" s="29" t="n"/>
-      <c r="E73" s="30" t="n"/>
-    </row>
-    <row r="74" ht="20" customHeight="1">
-      <c r="B74" s="20" t="inlineStr">
+      <c r="D67" s="29" t="n"/>
+      <c r="E67" s="30" t="n"/>
+    </row>
+    <row r="68" ht="20" customHeight="1">
+      <c r="B68" s="20" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C74" s="21" t="n"/>
-      <c r="D74" s="21" t="n"/>
-      <c r="E74" s="22" t="n"/>
-    </row>
-    <row r="75" ht="20.5" customHeight="1">
-      <c r="B75" s="23" t="inlineStr">
+      <c r="C68" s="21" t="n"/>
+      <c r="D68" s="21" t="n"/>
+      <c r="E68" s="22" t="n"/>
+    </row>
+    <row r="69" ht="20.5" customHeight="1">
+      <c r="B69" s="23" t="inlineStr">
         <is>
           <t>Versión</t>
         </is>
       </c>
-      <c r="C75" s="24" t="inlineStr">
-        <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="D75" s="25" t="n"/>
-      <c r="E75" s="26" t="n"/>
-    </row>
-    <row r="76" ht="20.5" customHeight="1">
-      <c r="B76" s="27" t="inlineStr">
+      <c r="C69" s="24" t="inlineStr">
+        <is>
+          <t>Familiar</t>
+        </is>
+      </c>
+      <c r="D69" s="25" t="n"/>
+      <c r="E69" s="26" t="n"/>
+    </row>
+    <row r="70" ht="20.5" customHeight="1">
+      <c r="B70" s="27" t="inlineStr">
         <is>
           <t>Capacidad</t>
         </is>
       </c>
-      <c r="C76" s="28" t="inlineStr">
-        <is>
-          <t>Hasta 4 espacios (familiar)</t>
-        </is>
-      </c>
-      <c r="D76" s="29" t="n"/>
-      <c r="E76" s="30" t="n"/>
-    </row>
-    <row r="77" ht="20.5" customHeight="1">
-      <c r="B77" s="23" t="inlineStr">
+      <c r="C70" s="28" t="inlineStr">
+        <is>
+          <t>Hasta 4 espacios</t>
+        </is>
+      </c>
+      <c r="D70" s="29" t="n"/>
+      <c r="E70" s="30" t="n"/>
+    </row>
+    <row r="71" ht="20.5" customHeight="1">
+      <c r="B71" s="23" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C77" s="24" t="inlineStr">
+      <c r="C71" s="24" t="inlineStr">
         <is>
           <t>Sectores VIP / preferenciales del parque</t>
         </is>
       </c>
-      <c r="D77" s="25" t="n"/>
-      <c r="E77" s="26" t="n"/>
-    </row>
-    <row r="78" ht="20.5" customHeight="1">
-      <c r="B78" s="27" t="inlineStr">
+      <c r="D71" s="25" t="n"/>
+      <c r="E71" s="26" t="n"/>
+    </row>
+    <row r="72" ht="20.5" customHeight="1">
+      <c r="B72" s="27" t="inlineStr">
         <is>
           <t>Homenaje</t>
         </is>
       </c>
-      <c r="C78" s="28" t="inlineStr">
+      <c r="C72" s="28" t="inlineStr">
         <is>
           <t>Placa patrimonial con acabado superior</t>
         </is>
       </c>
-      <c r="D78" s="29" t="n"/>
-      <c r="E78" s="30" t="n"/>
-    </row>
-    <row r="79" ht="64" customHeight="1">
-      <c r="B79" s="23" t="inlineStr">
+      <c r="D72" s="29" t="n"/>
+      <c r="E72" s="30" t="n"/>
+    </row>
+    <row r="73" ht="64" customHeight="1">
+      <c r="B73" s="23" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C79" s="24" t="inlineStr">
+      <c r="C73" s="24" t="inlineStr">
         <is>
           <t>• Inhumación de hasta 4 urnas
 • Ubicación en sectores VIP / preferenciales del parque
@@ -2019,152 +1914,234 @@
 • Lugar físico permanente de homenaje familiar</t>
         </is>
       </c>
-      <c r="D79" s="25" t="n"/>
-      <c r="E79" s="26" t="n"/>
-    </row>
-    <row r="80" ht="20" customHeight="1">
-      <c r="B80" s="20" t="inlineStr">
+      <c r="D73" s="25" t="n"/>
+      <c r="E73" s="26" t="n"/>
+    </row>
+    <row r="74" ht="20" customHeight="1">
+      <c r="B74" s="20" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C80" s="21" t="n"/>
-      <c r="D80" s="21" t="n"/>
-      <c r="E80" s="22" t="n"/>
-    </row>
-    <row r="81" ht="26.5" customHeight="1">
-      <c r="B81" s="23" t="inlineStr">
+      <c r="C74" s="21" t="n"/>
+      <c r="D74" s="21" t="n"/>
+      <c r="E74" s="22" t="n"/>
+    </row>
+    <row r="75" ht="26.5" customHeight="1">
+      <c r="B75" s="23" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C81" s="31" t="inlineStr">
+      <c r="C75" s="31" t="inlineStr">
         <is>
           <t>US$ 1.490 – US$ 1.990</t>
         </is>
       </c>
-      <c r="D81" s="25" t="n"/>
-      <c r="E81" s="26" t="n"/>
-    </row>
-    <row r="82" ht="20.5" customHeight="1">
-      <c r="B82" s="27" t="inlineStr">
+      <c r="D75" s="25" t="n"/>
+      <c r="E75" s="26" t="n"/>
+    </row>
+    <row r="76" ht="20.5" customHeight="1">
+      <c r="B76" s="27" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C82" s="28" t="inlineStr">
-        <is>
-          <t>Por parcela familiar (hasta 4 espacios)</t>
-        </is>
-      </c>
-      <c r="D82" s="29" t="n"/>
-      <c r="E82" s="30" t="n"/>
-    </row>
-    <row r="83" ht="20.5" customHeight="1">
-      <c r="B83" s="23" t="inlineStr">
+      <c r="C76" s="28" t="inlineStr">
+        <is>
+          <t>Variable según la cantidad de personas · hasta 4 espacios</t>
+        </is>
+      </c>
+      <c r="D76" s="29" t="n"/>
+      <c r="E76" s="30" t="n"/>
+    </row>
+    <row r="77" ht="20.5" customHeight="1">
+      <c r="B77" s="23" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C83" s="24" t="inlineStr">
+      <c r="C77" s="24" t="inlineStr">
         <is>
           <t>Pago único o financiado según política comercial vigente.</t>
         </is>
       </c>
-      <c r="D83" s="25" t="n"/>
-      <c r="E83" s="26" t="n"/>
+      <c r="D77" s="25" t="n"/>
+      <c r="E77" s="26" t="n"/>
+    </row>
+    <row r="78" ht="20" customHeight="1">
+      <c r="B78" s="20" t="inlineStr">
+        <is>
+          <t>PERFIL DEL COMPRADOR</t>
+        </is>
+      </c>
+      <c r="C78" s="21" t="n"/>
+      <c r="D78" s="21" t="n"/>
+      <c r="E78" s="22" t="n"/>
+    </row>
+    <row r="79" ht="35" customHeight="1">
+      <c r="B79" s="32" t="inlineStr">
+        <is>
+          <t>Cliente objetivo</t>
+        </is>
+      </c>
+      <c r="C79" s="33" t="inlineStr">
+        <is>
+          <t>Familias que buscan un espacio patrimonial y exclusivo para varias generaciones.</t>
+        </is>
+      </c>
+      <c r="D79" s="34" t="n"/>
+      <c r="E79" s="35" t="n"/>
+    </row>
+    <row r="82" ht="30" customHeight="1">
+      <c r="B82" s="14" t="inlineStr">
+        <is>
+          <t>JARDÍN DE INHUMACIÓN DE CENIZAS PET</t>
+        </is>
+      </c>
+      <c r="C82" s="15" t="n"/>
+      <c r="D82" s="15" t="n"/>
+      <c r="E82" s="16" t="inlineStr">
+        <is>
+          <t>VG-CRE-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="20" customHeight="1">
+      <c r="B83" s="17" t="inlineStr">
+        <is>
+          <t>Jardines de la Memoria · Mascotas  ·  Mascotas · Cremación e inhumación</t>
+        </is>
+      </c>
+      <c r="C83" s="18" t="n"/>
+      <c r="D83" s="18" t="n"/>
+      <c r="E83" s="19" t="n"/>
     </row>
     <row r="84" ht="20" customHeight="1">
       <c r="B84" s="20" t="inlineStr">
         <is>
-          <t>DIFERENCIALES DE LA CAMPAÑA DÍA DE LOS MUERTOS</t>
+          <t>VISIÓN GENERAL</t>
         </is>
       </c>
       <c r="C84" s="21" t="n"/>
       <c r="D84" s="21" t="n"/>
       <c r="E84" s="22" t="n"/>
     </row>
-    <row r="85" ht="20.5" customHeight="1">
+    <row r="85" ht="35" customHeight="1">
       <c r="B85" s="23" t="inlineStr">
         <is>
-          <t>Campaña</t>
+          <t>Concepto</t>
         </is>
       </c>
       <c r="C85" s="24" t="inlineStr">
         <is>
-          <t>• Selección prioritaria de ubicación VIP durante la campaña</t>
+          <t>Servicio de cremación e inhumación de cenizas de mascotas en un área verde dedicada.</t>
         </is>
       </c>
       <c r="D85" s="25" t="n"/>
       <c r="E85" s="26" t="n"/>
     </row>
-    <row r="86" ht="20" customHeight="1">
-      <c r="B86" s="20" t="inlineStr">
-        <is>
-          <t>PERFIL DEL COMPRADOR</t>
-        </is>
-      </c>
-      <c r="C86" s="21" t="n"/>
-      <c r="D86" s="21" t="n"/>
-      <c r="E86" s="22" t="n"/>
-    </row>
-    <row r="87" ht="35" customHeight="1">
-      <c r="B87" s="32" t="inlineStr">
-        <is>
-          <t>Cliente objetivo</t>
-        </is>
-      </c>
-      <c r="C87" s="33" t="inlineStr">
-        <is>
-          <t>Familias que buscan un espacio patrimonial y exclusivo para varias generaciones.</t>
-        </is>
-      </c>
-      <c r="D87" s="34" t="n"/>
-      <c r="E87" s="35" t="n"/>
-    </row>
-    <row r="90" ht="30" customHeight="1">
-      <c r="B90" s="14" t="inlineStr">
-        <is>
-          <t>JARDÍN DE INHUMACIÓN DE CENIZAS PET</t>
-        </is>
-      </c>
-      <c r="C90" s="15" t="n"/>
-      <c r="D90" s="15" t="n"/>
-      <c r="E90" s="16" t="inlineStr">
-        <is>
-          <t>VG-CRE-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="20" customHeight="1">
-      <c r="B91" s="17" t="inlineStr">
-        <is>
-          <t>Jardines de la Memoria · Mascotas  ·  Mascotas · Cremación e inhumación</t>
-        </is>
-      </c>
-      <c r="C91" s="18" t="n"/>
-      <c r="D91" s="18" t="n"/>
-      <c r="E91" s="19" t="n"/>
+    <row r="86" ht="20.5" customHeight="1">
+      <c r="B86" s="27" t="inlineStr">
+        <is>
+          <t>Capacidad / Cobertura</t>
+        </is>
+      </c>
+      <c r="C86" s="28" t="inlineStr">
+        <is>
+          <t>Individual (una mascota por servicio).</t>
+        </is>
+      </c>
+      <c r="D86" s="29" t="n"/>
+      <c r="E86" s="30" t="n"/>
+    </row>
+    <row r="87" ht="20" customHeight="1">
+      <c r="B87" s="20" t="inlineStr">
+        <is>
+          <t>ESPECIFICACIONES TÉCNICAS</t>
+        </is>
+      </c>
+      <c r="C87" s="21" t="n"/>
+      <c r="D87" s="21" t="n"/>
+      <c r="E87" s="22" t="n"/>
+    </row>
+    <row r="88" ht="20.5" customHeight="1">
+      <c r="B88" s="23" t="inlineStr">
+        <is>
+          <t>Tipo de producto</t>
+        </is>
+      </c>
+      <c r="C88" s="24" t="inlineStr">
+        <is>
+          <t>Servicio de pago único</t>
+        </is>
+      </c>
+      <c r="D88" s="25" t="n"/>
+      <c r="E88" s="26" t="n"/>
+    </row>
+    <row r="89" ht="20.5" customHeight="1">
+      <c r="B89" s="27" t="inlineStr">
+        <is>
+          <t>Servicio</t>
+        </is>
+      </c>
+      <c r="C89" s="28" t="inlineStr">
+        <is>
+          <t>Cremación + inhumación de cenizas</t>
+        </is>
+      </c>
+      <c r="D89" s="29" t="n"/>
+      <c r="E89" s="30" t="n"/>
+    </row>
+    <row r="90" ht="20.5" customHeight="1">
+      <c r="B90" s="23" t="inlineStr">
+        <is>
+          <t>Espacio</t>
+        </is>
+      </c>
+      <c r="C90" s="24" t="inlineStr">
+        <is>
+          <t>Área verde dedicada a mascotas</t>
+        </is>
+      </c>
+      <c r="D90" s="25" t="n"/>
+      <c r="E90" s="26" t="n"/>
+    </row>
+    <row r="91" ht="49.5" customHeight="1">
+      <c r="B91" s="27" t="inlineStr">
+        <is>
+          <t>Servicios incluidos</t>
+        </is>
+      </c>
+      <c r="C91" s="28" t="inlineStr">
+        <is>
+          <t>• Cremación de la mascota
+• Inhumación de cenizas en área verde dedicada
+• Espacio de homenaje para la familia</t>
+        </is>
+      </c>
+      <c r="D91" s="29" t="n"/>
+      <c r="E91" s="30" t="n"/>
     </row>
     <row r="92" ht="20" customHeight="1">
       <c r="B92" s="20" t="inlineStr">
         <is>
-          <t>VISIÓN GENERAL</t>
+          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
       <c r="C92" s="21" t="n"/>
       <c r="D92" s="21" t="n"/>
       <c r="E92" s="22" t="n"/>
     </row>
-    <row r="93" ht="35" customHeight="1">
+    <row r="93" ht="26.5" customHeight="1">
       <c r="B93" s="23" t="inlineStr">
         <is>
-          <t>Concepto</t>
-        </is>
-      </c>
-      <c r="C93" s="24" t="inlineStr">
-        <is>
-          <t>Servicio de cremación e inhumación de cenizas de mascotas en un área verde dedicada.</t>
+          <t>Precio sugerido</t>
+        </is>
+      </c>
+      <c r="C93" s="31" t="inlineStr">
+        <is>
+          <t>US$ 500</t>
         </is>
       </c>
       <c r="D93" s="25" t="n"/>
@@ -2173,308 +2150,153 @@
     <row r="94" ht="20.5" customHeight="1">
       <c r="B94" s="27" t="inlineStr">
         <is>
-          <t>Capacidad / Cobertura</t>
+          <t>Base de precio</t>
         </is>
       </c>
       <c r="C94" s="28" t="inlineStr">
         <is>
-          <t>Individual (una mascota por servicio).</t>
+          <t>Pago único por servicio</t>
         </is>
       </c>
       <c r="D94" s="29" t="n"/>
       <c r="E94" s="30" t="n"/>
     </row>
-    <row r="95" ht="20" customHeight="1">
-      <c r="B95" s="20" t="inlineStr">
-        <is>
-          <t>ESPECIFICACIONES TÉCNICAS</t>
-        </is>
-      </c>
-      <c r="C95" s="21" t="n"/>
-      <c r="D95" s="21" t="n"/>
-      <c r="E95" s="22" t="n"/>
-    </row>
-    <row r="96" ht="20.5" customHeight="1">
-      <c r="B96" s="23" t="inlineStr">
-        <is>
-          <t>Tipo de producto</t>
-        </is>
-      </c>
-      <c r="C96" s="24" t="inlineStr">
-        <is>
-          <t>Add-on al plan funerario</t>
-        </is>
-      </c>
-      <c r="D96" s="25" t="n"/>
-      <c r="E96" s="26" t="n"/>
-    </row>
-    <row r="97" ht="20.5" customHeight="1">
-      <c r="B97" s="27" t="inlineStr">
-        <is>
-          <t>Servicio</t>
-        </is>
-      </c>
-      <c r="C97" s="28" t="inlineStr">
-        <is>
-          <t>Cremación + inhumación de cenizas</t>
-        </is>
-      </c>
-      <c r="D97" s="29" t="n"/>
-      <c r="E97" s="30" t="n"/>
-    </row>
-    <row r="98" ht="20.5" customHeight="1">
-      <c r="B98" s="23" t="inlineStr">
-        <is>
-          <t>Espacio</t>
-        </is>
-      </c>
-      <c r="C98" s="24" t="inlineStr">
-        <is>
-          <t>Área verde dedicada a mascotas</t>
-        </is>
-      </c>
-      <c r="D98" s="25" t="n"/>
-      <c r="E98" s="26" t="n"/>
-    </row>
-    <row r="99" ht="20.5" customHeight="1">
-      <c r="B99" s="27" t="inlineStr">
-        <is>
-          <t>Recurrencia</t>
-        </is>
-      </c>
-      <c r="C99" s="28" t="inlineStr">
-        <is>
-          <t>Mensual o tarifa única</t>
-        </is>
-      </c>
-      <c r="D99" s="29" t="n"/>
-      <c r="E99" s="30" t="n"/>
-    </row>
-    <row r="100" ht="49.5" customHeight="1">
-      <c r="B100" s="23" t="inlineStr">
-        <is>
-          <t>Servicios incluidos</t>
-        </is>
-      </c>
-      <c r="C100" s="24" t="inlineStr">
-        <is>
-          <t>• Cremación de la mascota
-• Inhumación de cenizas en área verde dedicada
-• Espacio de homenaje para la familia</t>
-        </is>
-      </c>
-      <c r="D100" s="25" t="n"/>
-      <c r="E100" s="26" t="n"/>
-    </row>
-    <row r="101" ht="20" customHeight="1">
-      <c r="B101" s="20" t="inlineStr">
-        <is>
-          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
-        </is>
-      </c>
-      <c r="C101" s="21" t="n"/>
-      <c r="D101" s="21" t="n"/>
-      <c r="E101" s="22" t="n"/>
-    </row>
-    <row r="102" ht="26.5" customHeight="1">
-      <c r="B102" s="23" t="inlineStr">
-        <is>
-          <t>Precio sugerido</t>
-        </is>
-      </c>
-      <c r="C102" s="31" t="inlineStr">
-        <is>
-          <t>US$ 5/mes</t>
-        </is>
-      </c>
-      <c r="D102" s="25" t="n"/>
-      <c r="E102" s="26" t="n"/>
-    </row>
-    <row r="103" ht="20.5" customHeight="1">
-      <c r="B103" s="27" t="inlineStr">
-        <is>
-          <t>Base de precio</t>
-        </is>
-      </c>
-      <c r="C103" s="28" t="inlineStr">
-        <is>
-          <t>Adicional al plan</t>
-        </is>
-      </c>
-      <c r="D103" s="29" t="n"/>
-      <c r="E103" s="30" t="n"/>
-    </row>
-    <row r="104" ht="20.5" customHeight="1">
-      <c r="B104" s="23" t="inlineStr">
+    <row r="95" ht="20.5" customHeight="1">
+      <c r="B95" s="23" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C104" s="24" t="inlineStr">
-        <is>
-          <t>US$ 5,00/mes adicional al plan, o tarifa única proporcional (add-on).</t>
-        </is>
-      </c>
-      <c r="D104" s="25" t="n"/>
-      <c r="E104" s="26" t="n"/>
-    </row>
-    <row r="105" ht="20" customHeight="1">
-      <c r="B105" s="20" t="inlineStr">
-        <is>
-          <t>DIFERENCIALES DE LA CAMPAÑA DÍA DE LOS MUERTOS</t>
-        </is>
-      </c>
-      <c r="C105" s="21" t="n"/>
-      <c r="D105" s="21" t="n"/>
-      <c r="E105" s="22" t="n"/>
-    </row>
-    <row r="106" ht="20.5" customHeight="1">
-      <c r="B106" s="23" t="inlineStr">
-        <is>
-          <t>Campaña</t>
-        </is>
-      </c>
-      <c r="C106" s="24" t="inlineStr">
-        <is>
-          <t>• Extensión del plan familiar a las mascotas con una cuota mínima</t>
-        </is>
-      </c>
-      <c r="D106" s="25" t="n"/>
-      <c r="E106" s="26" t="n"/>
-    </row>
-    <row r="107" ht="20" customHeight="1">
-      <c r="B107" s="20" t="inlineStr">
+      <c r="C95" s="24" t="inlineStr">
+        <is>
+          <t>Pago único; puede contratarse como adicional al plan funerario.</t>
+        </is>
+      </c>
+      <c r="D95" s="25" t="n"/>
+      <c r="E95" s="26" t="n"/>
+    </row>
+    <row r="96" ht="20" customHeight="1">
+      <c r="B96" s="20" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C107" s="21" t="n"/>
-      <c r="D107" s="21" t="n"/>
-      <c r="E107" s="22" t="n"/>
-    </row>
-    <row r="108" ht="35" customHeight="1">
-      <c r="B108" s="32" t="inlineStr">
+      <c r="C96" s="21" t="n"/>
+      <c r="D96" s="21" t="n"/>
+      <c r="E96" s="22" t="n"/>
+    </row>
+    <row r="97" ht="35" customHeight="1">
+      <c r="B97" s="32" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C108" s="33" t="inlineStr">
+      <c r="C97" s="33" t="inlineStr">
         <is>
           <t>Familias afiliadas que consideran a su mascota parte del hogar y desean un cierre digno.</t>
         </is>
       </c>
-      <c r="D108" s="34" t="n"/>
-      <c r="E108" s="35" t="n"/>
+      <c r="D97" s="34" t="n"/>
+      <c r="E97" s="35" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="99">
+  <mergeCells count="88">
     <mergeCell ref="B65:E65"/>
     <mergeCell ref="C31:E31"/>
     <mergeCell ref="B74:E74"/>
-    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="B68:E68"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="B36:E36"/>
     <mergeCell ref="C51:E51"/>
+    <mergeCell ref="C95:E95"/>
+    <mergeCell ref="B45:E45"/>
     <mergeCell ref="C60:E60"/>
-    <mergeCell ref="B91:E91"/>
+    <mergeCell ref="C71:E71"/>
     <mergeCell ref="C7:E7"/>
+    <mergeCell ref="C91:E91"/>
     <mergeCell ref="C57:E57"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="B21:E21"/>
     <mergeCell ref="C18:E18"/>
-    <mergeCell ref="B86:E86"/>
     <mergeCell ref="C77:E77"/>
     <mergeCell ref="C34:E34"/>
-    <mergeCell ref="B101:E101"/>
-    <mergeCell ref="B23:E23"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="B78:E78"/>
+    <mergeCell ref="B87:E87"/>
     <mergeCell ref="C20:E20"/>
-    <mergeCell ref="C103:E103"/>
     <mergeCell ref="C85:E85"/>
-    <mergeCell ref="C99:E99"/>
+    <mergeCell ref="B40:E40"/>
     <mergeCell ref="C94:E94"/>
     <mergeCell ref="B49:E49"/>
     <mergeCell ref="C75:E75"/>
     <mergeCell ref="C22:E22"/>
+    <mergeCell ref="B64:E64"/>
+    <mergeCell ref="B82:D82"/>
     <mergeCell ref="C12:E12"/>
-    <mergeCell ref="B32:E32"/>
-    <mergeCell ref="B63:E63"/>
-    <mergeCell ref="B50:E50"/>
+    <mergeCell ref="B26:E26"/>
     <mergeCell ref="C52:E52"/>
-    <mergeCell ref="C61:E61"/>
     <mergeCell ref="C39:E39"/>
     <mergeCell ref="B16:E16"/>
-    <mergeCell ref="C106:E106"/>
-    <mergeCell ref="C81:E81"/>
+    <mergeCell ref="C70:E70"/>
+    <mergeCell ref="C48:E48"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="B27:E27"/>
     <mergeCell ref="C13:E13"/>
-    <mergeCell ref="C87:E87"/>
     <mergeCell ref="C15:E15"/>
-    <mergeCell ref="C24:E24"/>
     <mergeCell ref="C33:E33"/>
-    <mergeCell ref="C104:E104"/>
-    <mergeCell ref="B53:E53"/>
+    <mergeCell ref="C89:E89"/>
     <mergeCell ref="C79:E79"/>
     <mergeCell ref="C73:E73"/>
-    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="C88:E88"/>
     <mergeCell ref="C35:E35"/>
-    <mergeCell ref="B48:D48"/>
     <mergeCell ref="B84:E84"/>
     <mergeCell ref="C10:E10"/>
-    <mergeCell ref="C55:E55"/>
+    <mergeCell ref="C50:E50"/>
     <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B80:E80"/>
-    <mergeCell ref="B95:E95"/>
-    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="B55:E55"/>
     <mergeCell ref="C11:E11"/>
+    <mergeCell ref="C67:E67"/>
     <mergeCell ref="C72:E72"/>
-    <mergeCell ref="B71:E71"/>
-    <mergeCell ref="B105:E105"/>
+    <mergeCell ref="C28:E28"/>
     <mergeCell ref="C37:E37"/>
-    <mergeCell ref="C96:E96"/>
-    <mergeCell ref="C78:E78"/>
+    <mergeCell ref="B63:D63"/>
+    <mergeCell ref="C69:E69"/>
     <mergeCell ref="B2:E2"/>
-    <mergeCell ref="C30:E30"/>
-    <mergeCell ref="B42:E42"/>
-    <mergeCell ref="B107:E107"/>
-    <mergeCell ref="C62:E62"/>
+    <mergeCell ref="B25:D25"/>
     <mergeCell ref="C14:E14"/>
-    <mergeCell ref="C98:E98"/>
-    <mergeCell ref="B44:E44"/>
-    <mergeCell ref="C64:E64"/>
-    <mergeCell ref="B28:E28"/>
     <mergeCell ref="C54:E54"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="C41:E41"/>
+    <mergeCell ref="B83:E83"/>
     <mergeCell ref="C93:E93"/>
     <mergeCell ref="B92:E92"/>
+    <mergeCell ref="B30:E30"/>
     <mergeCell ref="C56:E56"/>
     <mergeCell ref="B5:E5"/>
-    <mergeCell ref="C43:E43"/>
-    <mergeCell ref="B69:D69"/>
+    <mergeCell ref="C90:E90"/>
     <mergeCell ref="C76:E76"/>
     <mergeCell ref="C8:E8"/>
     <mergeCell ref="C17:E17"/>
     <mergeCell ref="B59:E59"/>
-    <mergeCell ref="C82:E82"/>
+    <mergeCell ref="B46:E46"/>
     <mergeCell ref="C66:E66"/>
     <mergeCell ref="C19:E19"/>
-    <mergeCell ref="C102:E102"/>
-    <mergeCell ref="B70:E70"/>
-    <mergeCell ref="C83:E83"/>
-    <mergeCell ref="C108:E108"/>
+    <mergeCell ref="C53:E53"/>
+    <mergeCell ref="B96:E96"/>
+    <mergeCell ref="C86:E86"/>
     <mergeCell ref="C58:E58"/>
-    <mergeCell ref="B90:D90"/>
-    <mergeCell ref="C45:E45"/>
     <mergeCell ref="C97:E97"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="C100:E100"/>
+    <mergeCell ref="C29:E29"/>
+    <mergeCell ref="C47:E47"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
   <rowBreaks count="4" manualBreakCount="4">
-    <brk id="25" min="0" max="16383" man="1"/>
-    <brk id="46" min="0" max="16383" man="1"/>
-    <brk id="67" min="0" max="16383" man="1"/>
-    <brk id="88" min="0" max="16383" man="1"/>
+    <brk id="23" min="0" max="16383" man="1"/>
+    <brk id="42" min="0" max="16383" man="1"/>
+    <brk id="61" min="0" max="16383" man="1"/>
+    <brk id="80" min="0" max="16383" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sincroniza jardines con el diseño de Canva "Jardines de Cenizas"
- Individual (Jardín 1): contenedor Ø32x40 cm, tapa de granito; US$ 600
- Familiar (Jardín 1): 4 espacios, sin plazo; US$ 2.000
- Nuevo Ecológico (Jardín 2 / Bosque de las Orquídeas); US$ 600
- Nuevo Ceremonial (Jardín 3), precio a definir
- Mascotas: US$ 350 solo jardín / US$ 500 con cremación
- Aspersión ubicada en el área de esparcimiento del Jardín 2

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111i7vn9WWo4QxCQbucWbrF
</commit_message>
<xml_diff>
--- a/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
+++ b/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
@@ -11,9 +11,9 @@
     <sheet name="Ficha Técnica Consolidada" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tabla Gral. - Visión Comercial'!$A$4:$I$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tabla Gral. - Visión Comercial'!$A$4:$I$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Tabla Gral. - Visión Comercial'!$4:$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Ficha Técnica Consolidada'!$A$1:$F$98</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Ficha Técnica Consolidada'!$A$1:$F$142</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -707,7 +707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -852,7 +852,7 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>Área reservada en jardín natural para la liberación ceremonial de cenizas, en armonía con la naturaleza.</t>
+          <t>Liberación ceremonial de cenizas en el área de esparcimiento del Jardín Ecológico, junto al agua corriente, en armonía con la naturaleza.</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
@@ -885,7 +885,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="64" customHeight="1">
+    <row r="7" ht="78.5" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>VG-CRE-03I</t>
@@ -903,20 +903,20 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Inhumación de urnas en parcelas ajardinadas con demarcación personalizada: un lugar físico permanente de homenaje.</t>
+          <t>Inhumación de la urna de cenizas en un contenedor enterrado con tapa de granito grabada, en un jardín de plantas de sombra: un lugar físico permanente de homenaje.</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Individual.</t>
+          <t>Individual (1 urna).</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>• Inhumación de urna en parcela ajardinada
-• Ubicación en sectores ajardinados generales
-• Placa conmemorativa individual estándar
-• Lugar físico permanente de homenaje</t>
+          <t>• Inhumación de la urna en contenedor individual
+• Tapa de granito con los datos del difunto
+• Ubicación en el Jardín 1, con paisajismo de plantas de sombra
+• Espacio de contemplación con banco</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -936,7 +936,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="78.5" customHeight="1">
+    <row r="8" ht="93" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>VG-CRE-03F</t>
@@ -954,7 +954,7 @@
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>Inhumación familiar de urnas en sectores VIP del parque, con placa patrimonial de acabado superior.</t>
+          <t>Parcela familiar en el Jardín 1 con cuatro contenedores agrupados, cada uno con tapa de granito grabada, sin plazo de permanencia.</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
@@ -965,20 +965,20 @@
       <c r="F8" s="10" t="inlineStr">
         <is>
           <t>• Inhumación de hasta 4 urnas
-• Ubicación en sectores VIP / preferenciales del parque
-• Placa patrimonial con acabado superior
-• Lugar físico permanente de homenaje familiar</t>
+• Tapa de granito grabada para cada espacio
+• Ubicación en el Jardín 1, con paisajismo de plantas de sombra
+• Lugar físico permanente de homenaje familiar, sin plazo</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
-          <t>Familias que buscan un espacio patrimonial y exclusivo para varias generaciones.</t>
+          <t>Familias que buscan un espacio propio y permanente para varias generaciones.</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>US$ 1.490 – US$ 1.990
-(Variable según la cantidad de personas · hasta 4 espacios)</t>
+          <t>US$ 2.000
+(Por parcela familiar · hasta 4 espacios)</t>
         </is>
       </c>
       <c r="I8" s="10" t="inlineStr">
@@ -987,58 +987,159 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="49.5" customHeight="1">
+    <row r="9" ht="93" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
+          <t>VG-CRE-03E</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Jardín de Cenizas · Ecológico</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Destino final · Inhumación ecológica</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>La urna biodegradable se entierra directamente en el suelo, se cubre con tierra y se descompone integrándose a la naturaleza. Jardín con agua corriente y área de esparcimiento de cenizas.</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Individual (1 urna).</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>• Inhumación ecológica de la urna directamente en el suelo
+• Placa de identificación
+• Ubicación en el Jardín 2 o en el Bosque de las Orquídeas
+• Entorno natural con agua corriente</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Personas con conciencia ambiental que desean que sus cenizas vuelvan a la tierra, con un lugar identificado para visitar.</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>US$ 600
+(Por espacio individual)</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>Pago único o financiado según política comercial vigente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="49.5" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>VG-CRE-03C</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Jardín de Cenizas · Ceremonial</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Destino final · Inhumación con ceremonia</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>Jardín para inhumación de urnas de cenizas con ceremonia de agua, con fuentes como elemento central del rito de despedida.</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>A definir.</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>• Inhumación de urnas de cenizas
+• Ceremonia con agua en fuente</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>Familias que valoran un rito de despedida simbólico y un entorno contemplativo.</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>A definir
+(Producto en definición)</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>A definir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="93" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
           <t>VG-CRE-04</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Jardín de Inhumación de Cenizas PET</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>Mascotas · Cremación e inhumación</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Servicio de cremación e inhumación de cenizas de mascotas en un área verde dedicada.</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Jardín de Mascotas</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Mascotas · Inhumación ecológica</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Jardín para inhumación ecológica de cenizas de mascotas: la urna biodegradable se entierra directamente en el suelo y se identifica con una placa de madera.</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>Individual (una mascota por servicio).</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>• Cremación de la mascota
-• Inhumación de cenizas en área verde dedicada
-• Espacio de homenaje para la familia</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>Familias afiliadas que consideran a su mascota parte del hogar y desean un cierre digno.</t>
-        </is>
-      </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>US$ 500
-(Pago único por servicio)</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>• Inhumación ecológica de la urna en el jardín
+• Placa de madera de 20 cm para identificación
+• Nombre de la mascota en la placa conmemorativa del jardín
+• Cremación de la mascota (opción Jardín + Cremación)</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Familias que consideran a su mascota parte del hogar y desean un cierre digno.</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>US$ 350 / US$ 500
+(US$ 350 solo jardín · US$ 500 jardín + cremación)</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>Pago único; puede contratarse como adicional al plan funerario.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I9"/>
+  <autoFilter ref="A4:I11"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
@@ -1055,7 +1156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:E97"/>
+  <dimension ref="B1:E141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1372,7 +1473,7 @@
       </c>
       <c r="C28" s="24" t="inlineStr">
         <is>
-          <t>Área reservada en jardín natural para la liberación ceremonial de cenizas, en armonía con la naturaleza.</t>
+          <t>Liberación ceremonial de cenizas en el área de esparcimiento del Jardín Ecológico, junto al agua corriente, en armonía con la naturaleza.</t>
         </is>
       </c>
       <c r="D28" s="25" t="n"/>
@@ -1433,12 +1534,12 @@
     <row r="33" ht="20.5" customHeight="1">
       <c r="B33" s="23" t="inlineStr">
         <is>
-          <t>Espacio</t>
+          <t>Ubicación</t>
         </is>
       </c>
       <c r="C33" s="24" t="inlineStr">
         <is>
-          <t>Jardín natural reservado (sin espacio fijo asignado)</t>
+          <t>Jardín 2 · Ecológico, área de esparcimiento de cenizas</t>
         </is>
       </c>
       <c r="D33" s="25" t="n"/>
@@ -1447,24 +1548,38 @@
     <row r="34" ht="20.5" customHeight="1">
       <c r="B34" s="27" t="inlineStr">
         <is>
-          <t>Homenaje</t>
+          <t>Entorno</t>
         </is>
       </c>
       <c r="C34" s="28" t="inlineStr">
         <is>
-          <t>Placa memorial de la aspersión</t>
+          <t>Agua corriente que se extiende hasta el jardín</t>
         </is>
       </c>
       <c r="D34" s="29" t="n"/>
       <c r="E34" s="30" t="n"/>
     </row>
-    <row r="35" ht="64" customHeight="1">
+    <row r="35" ht="20.5" customHeight="1">
       <c r="B35" s="23" t="inlineStr">
         <is>
+          <t>Homenaje</t>
+        </is>
+      </c>
+      <c r="C35" s="24" t="inlineStr">
+        <is>
+          <t>Placa memorial de la aspersión</t>
+        </is>
+      </c>
+      <c r="D35" s="25" t="n"/>
+      <c r="E35" s="26" t="n"/>
+    </row>
+    <row r="36" ht="64" customHeight="1">
+      <c r="B36" s="27" t="inlineStr">
+        <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C35" s="24" t="inlineStr">
+      <c r="C36" s="28" t="inlineStr">
         <is>
           <t>• Acompañamiento ceremonial
 • Tiempo privado para la familia en entorno botánico
@@ -1472,415 +1587,401 @@
 • Placa memorial que registra la aspersión realizada en el lugar</t>
         </is>
       </c>
-      <c r="D35" s="25" t="n"/>
-      <c r="E35" s="26" t="n"/>
-    </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="B36" s="20" t="inlineStr">
+      <c r="D36" s="29" t="n"/>
+      <c r="E36" s="30" t="n"/>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="B37" s="20" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C36" s="21" t="n"/>
-      <c r="D36" s="21" t="n"/>
-      <c r="E36" s="22" t="n"/>
-    </row>
-    <row r="37" ht="26.5" customHeight="1">
-      <c r="B37" s="23" t="inlineStr">
+      <c r="C37" s="21" t="n"/>
+      <c r="D37" s="21" t="n"/>
+      <c r="E37" s="22" t="n"/>
+    </row>
+    <row r="38" ht="26.5" customHeight="1">
+      <c r="B38" s="23" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C37" s="31" t="inlineStr">
+      <c r="C38" s="31" t="inlineStr">
         <is>
           <t>US$ 250</t>
         </is>
       </c>
-      <c r="D37" s="25" t="n"/>
-      <c r="E37" s="26" t="n"/>
-    </row>
-    <row r="38" ht="20.5" customHeight="1">
-      <c r="B38" s="27" t="inlineStr">
+      <c r="D38" s="25" t="n"/>
+      <c r="E38" s="26" t="n"/>
+    </row>
+    <row r="39" ht="20.5" customHeight="1">
+      <c r="B39" s="27" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C38" s="28" t="inlineStr">
+      <c r="C39" s="28" t="inlineStr">
         <is>
           <t>Pago único por servicio</t>
         </is>
       </c>
-      <c r="D38" s="29" t="n"/>
-      <c r="E38" s="30" t="n"/>
-    </row>
-    <row r="39" ht="20.5" customHeight="1">
-      <c r="B39" s="23" t="inlineStr">
+      <c r="D39" s="29" t="n"/>
+      <c r="E39" s="30" t="n"/>
+    </row>
+    <row r="40" ht="20.5" customHeight="1">
+      <c r="B40" s="23" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C39" s="24" t="inlineStr">
+      <c r="C40" s="24" t="inlineStr">
         <is>
           <t>Pago único; combinable con la Solución Modular de Cremación.</t>
         </is>
       </c>
-      <c r="D39" s="25" t="n"/>
-      <c r="E39" s="26" t="n"/>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="B40" s="20" t="inlineStr">
+      <c r="D40" s="25" t="n"/>
+      <c r="E40" s="26" t="n"/>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="B41" s="20" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C40" s="21" t="n"/>
-      <c r="D40" s="21" t="n"/>
-      <c r="E40" s="22" t="n"/>
-    </row>
-    <row r="41" ht="35" customHeight="1">
-      <c r="B41" s="32" t="inlineStr">
+      <c r="C41" s="21" t="n"/>
+      <c r="D41" s="21" t="n"/>
+      <c r="E41" s="22" t="n"/>
+    </row>
+    <row r="42" ht="35" customHeight="1">
+      <c r="B42" s="32" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C41" s="33" t="inlineStr">
+      <c r="C42" s="33" t="inlineStr">
         <is>
           <t>Personas que buscan un concepto de libertad total, sin necesidad de un espacio físico fijo.</t>
         </is>
       </c>
-      <c r="D41" s="34" t="n"/>
-      <c r="E41" s="35" t="n"/>
-    </row>
-    <row r="44" ht="30" customHeight="1">
-      <c r="B44" s="14" t="inlineStr">
+      <c r="D42" s="34" t="n"/>
+      <c r="E42" s="35" t="n"/>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="B45" s="14" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · INDIVIDUAL</t>
         </is>
       </c>
-      <c r="C44" s="15" t="n"/>
-      <c r="D44" s="15" t="n"/>
-      <c r="E44" s="16" t="inlineStr">
+      <c r="C45" s="15" t="n"/>
+      <c r="D45" s="15" t="n"/>
+      <c r="E45" s="16" t="inlineStr">
         <is>
           <t>VG-CRE-03I</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="20" customHeight="1">
-      <c r="B45" s="17" t="inlineStr">
-        <is>
-          <t>Jardines de la Memoria · Inhumación  ·  Destino final · Inhumación individual</t>
-        </is>
-      </c>
-      <c r="C45" s="18" t="n"/>
-      <c r="D45" s="18" t="n"/>
-      <c r="E45" s="19" t="n"/>
-    </row>
     <row r="46" ht="20" customHeight="1">
-      <c r="B46" s="20" t="inlineStr">
+      <c r="B46" s="17" t="inlineStr">
+        <is>
+          <t>Jardines de la Memoria · Jardín 1  ·  Destino final · Inhumación individual</t>
+        </is>
+      </c>
+      <c r="C46" s="18" t="n"/>
+      <c r="D46" s="18" t="n"/>
+      <c r="E46" s="19" t="n"/>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="B47" s="20" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C46" s="21" t="n"/>
-      <c r="D46" s="21" t="n"/>
-      <c r="E46" s="22" t="n"/>
-    </row>
-    <row r="47" ht="35" customHeight="1">
-      <c r="B47" s="23" t="inlineStr">
+      <c r="C47" s="21" t="n"/>
+      <c r="D47" s="21" t="n"/>
+      <c r="E47" s="22" t="n"/>
+    </row>
+    <row r="48" ht="49.5" customHeight="1">
+      <c r="B48" s="23" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C47" s="24" t="inlineStr">
-        <is>
-          <t>Inhumación de urnas en parcelas ajardinadas con demarcación personalizada: un lugar físico permanente de homenaje.</t>
-        </is>
-      </c>
-      <c r="D47" s="25" t="n"/>
-      <c r="E47" s="26" t="n"/>
-    </row>
-    <row r="48" ht="20.5" customHeight="1">
-      <c r="B48" s="27" t="inlineStr">
+      <c r="C48" s="24" t="inlineStr">
+        <is>
+          <t>Inhumación de la urna de cenizas en un contenedor enterrado con tapa de granito grabada, en un jardín de plantas de sombra: un lugar físico permanente de homenaje.</t>
+        </is>
+      </c>
+      <c r="D48" s="25" t="n"/>
+      <c r="E48" s="26" t="n"/>
+    </row>
+    <row r="49" ht="20.5" customHeight="1">
+      <c r="B49" s="27" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C48" s="28" t="inlineStr">
-        <is>
-          <t>Individual.</t>
-        </is>
-      </c>
-      <c r="D48" s="29" t="n"/>
-      <c r="E48" s="30" t="n"/>
-    </row>
-    <row r="49" ht="20" customHeight="1">
-      <c r="B49" s="20" t="inlineStr">
+      <c r="C49" s="28" t="inlineStr">
+        <is>
+          <t>Individual (1 urna).</t>
+        </is>
+      </c>
+      <c r="D49" s="29" t="n"/>
+      <c r="E49" s="30" t="n"/>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="B50" s="20" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C49" s="21" t="n"/>
-      <c r="D49" s="21" t="n"/>
-      <c r="E49" s="22" t="n"/>
-    </row>
-    <row r="50" ht="20.5" customHeight="1">
-      <c r="B50" s="23" t="inlineStr">
-        <is>
-          <t>Versión</t>
-        </is>
-      </c>
-      <c r="C50" s="24" t="inlineStr">
-        <is>
-          <t>Individual</t>
-        </is>
-      </c>
-      <c r="D50" s="25" t="n"/>
-      <c r="E50" s="26" t="n"/>
+      <c r="C50" s="21" t="n"/>
+      <c r="D50" s="21" t="n"/>
+      <c r="E50" s="22" t="n"/>
     </row>
     <row r="51" ht="20.5" customHeight="1">
-      <c r="B51" s="27" t="inlineStr">
-        <is>
-          <t>Capacidad</t>
-        </is>
-      </c>
-      <c r="C51" s="28" t="inlineStr">
-        <is>
-          <t>1 espacio</t>
-        </is>
-      </c>
-      <c r="D51" s="29" t="n"/>
-      <c r="E51" s="30" t="n"/>
+      <c r="B51" s="23" t="inlineStr">
+        <is>
+          <t>Ambiente</t>
+        </is>
+      </c>
+      <c r="C51" s="24" t="inlineStr">
+        <is>
+          <t>Jardín 1</t>
+        </is>
+      </c>
+      <c r="D51" s="25" t="n"/>
+      <c r="E51" s="26" t="n"/>
     </row>
     <row r="52" ht="20.5" customHeight="1">
-      <c r="B52" s="23" t="inlineStr">
-        <is>
-          <t>Ubicación</t>
-        </is>
-      </c>
-      <c r="C52" s="24" t="inlineStr">
-        <is>
-          <t>Sectores ajardinados generales</t>
-        </is>
-      </c>
-      <c r="D52" s="25" t="n"/>
-      <c r="E52" s="26" t="n"/>
+      <c r="B52" s="27" t="inlineStr">
+        <is>
+          <t>Contenedor</t>
+        </is>
+      </c>
+      <c r="C52" s="28" t="inlineStr">
+        <is>
+          <t>Ø 32 cm × 40 cm de altura; enterrado dejando 20 cm a la vista</t>
+        </is>
+      </c>
+      <c r="D52" s="29" t="n"/>
+      <c r="E52" s="30" t="n"/>
     </row>
     <row r="53" ht="20.5" customHeight="1">
-      <c r="B53" s="27" t="inlineStr">
-        <is>
-          <t>Homenaje</t>
-        </is>
-      </c>
-      <c r="C53" s="28" t="inlineStr">
-        <is>
-          <t>Placa conmemorativa individual estándar</t>
-        </is>
-      </c>
-      <c r="D53" s="29" t="n"/>
-      <c r="E53" s="30" t="n"/>
-    </row>
-    <row r="54" ht="64" customHeight="1">
-      <c r="B54" s="23" t="inlineStr">
+      <c r="B53" s="23" t="inlineStr">
+        <is>
+          <t>Identificación</t>
+        </is>
+      </c>
+      <c r="C53" s="24" t="inlineStr">
+        <is>
+          <t>Tapa de granito con la información del difunto</t>
+        </is>
+      </c>
+      <c r="D53" s="25" t="n"/>
+      <c r="E53" s="26" t="n"/>
+    </row>
+    <row r="54" ht="20.5" customHeight="1">
+      <c r="B54" s="27" t="inlineStr">
+        <is>
+          <t>Paisajismo</t>
+        </is>
+      </c>
+      <c r="C54" s="28" t="inlineStr">
+        <is>
+          <t>Plantas de sombra de diferentes alturas y texturas</t>
+        </is>
+      </c>
+      <c r="D54" s="29" t="n"/>
+      <c r="E54" s="30" t="n"/>
+    </row>
+    <row r="55" ht="20.5" customHeight="1">
+      <c r="B55" s="23" t="inlineStr">
+        <is>
+          <t>Acceso</t>
+        </is>
+      </c>
+      <c r="C55" s="24" t="inlineStr">
+        <is>
+          <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
+        </is>
+      </c>
+      <c r="D55" s="25" t="n"/>
+      <c r="E55" s="26" t="n"/>
+    </row>
+    <row r="56" ht="64" customHeight="1">
+      <c r="B56" s="27" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C54" s="24" t="inlineStr">
-        <is>
-          <t>• Inhumación de urna en parcela ajardinada
-• Ubicación en sectores ajardinados generales
-• Placa conmemorativa individual estándar
-• Lugar físico permanente de homenaje</t>
-        </is>
-      </c>
-      <c r="D54" s="25" t="n"/>
-      <c r="E54" s="26" t="n"/>
-    </row>
-    <row r="55" ht="20" customHeight="1">
-      <c r="B55" s="20" t="inlineStr">
+      <c r="C56" s="28" t="inlineStr">
+        <is>
+          <t>• Inhumación de la urna en contenedor individual
+• Tapa de granito con los datos del difunto
+• Ubicación en el Jardín 1, con paisajismo de plantas de sombra
+• Espacio de contemplación con banco</t>
+        </is>
+      </c>
+      <c r="D56" s="29" t="n"/>
+      <c r="E56" s="30" t="n"/>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="B57" s="20" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C55" s="21" t="n"/>
-      <c r="D55" s="21" t="n"/>
-      <c r="E55" s="22" t="n"/>
-    </row>
-    <row r="56" ht="26.5" customHeight="1">
-      <c r="B56" s="23" t="inlineStr">
+      <c r="C57" s="21" t="n"/>
+      <c r="D57" s="21" t="n"/>
+      <c r="E57" s="22" t="n"/>
+    </row>
+    <row r="58" ht="26.5" customHeight="1">
+      <c r="B58" s="23" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C56" s="31" t="inlineStr">
+      <c r="C58" s="31" t="inlineStr">
         <is>
           <t>US$ 600</t>
-        </is>
-      </c>
-      <c r="D56" s="25" t="n"/>
-      <c r="E56" s="26" t="n"/>
-    </row>
-    <row r="57" ht="20.5" customHeight="1">
-      <c r="B57" s="27" t="inlineStr">
-        <is>
-          <t>Base de precio</t>
-        </is>
-      </c>
-      <c r="C57" s="28" t="inlineStr">
-        <is>
-          <t>Por espacio individual</t>
-        </is>
-      </c>
-      <c r="D57" s="29" t="n"/>
-      <c r="E57" s="30" t="n"/>
-    </row>
-    <row r="58" ht="20.5" customHeight="1">
-      <c r="B58" s="23" t="inlineStr">
-        <is>
-          <t>Condiciones</t>
-        </is>
-      </c>
-      <c r="C58" s="24" t="inlineStr">
-        <is>
-          <t>Pago único o financiado según política comercial vigente.</t>
         </is>
       </c>
       <c r="D58" s="25" t="n"/>
       <c r="E58" s="26" t="n"/>
     </row>
-    <row r="59" ht="20" customHeight="1">
-      <c r="B59" s="20" t="inlineStr">
+    <row r="59" ht="20.5" customHeight="1">
+      <c r="B59" s="27" t="inlineStr">
+        <is>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C59" s="28" t="inlineStr">
+        <is>
+          <t>Por espacio individual</t>
+        </is>
+      </c>
+      <c r="D59" s="29" t="n"/>
+      <c r="E59" s="30" t="n"/>
+    </row>
+    <row r="60" ht="20.5" customHeight="1">
+      <c r="B60" s="23" t="inlineStr">
+        <is>
+          <t>Condiciones</t>
+        </is>
+      </c>
+      <c r="C60" s="24" t="inlineStr">
+        <is>
+          <t>Pago único o financiado según política comercial vigente.</t>
+        </is>
+      </c>
+      <c r="D60" s="25" t="n"/>
+      <c r="E60" s="26" t="n"/>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="B61" s="20" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C59" s="21" t="n"/>
-      <c r="D59" s="21" t="n"/>
-      <c r="E59" s="22" t="n"/>
-    </row>
-    <row r="60" ht="35" customHeight="1">
-      <c r="B60" s="32" t="inlineStr">
+      <c r="C61" s="21" t="n"/>
+      <c r="D61" s="21" t="n"/>
+      <c r="E61" s="22" t="n"/>
+    </row>
+    <row r="62" ht="35" customHeight="1">
+      <c r="B62" s="32" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C60" s="33" t="inlineStr">
+      <c r="C62" s="33" t="inlineStr">
         <is>
           <t>Familias que desean un lugar permanente para visitar y rendir homenaje, con una inversión moderada.</t>
         </is>
       </c>
-      <c r="D60" s="34" t="n"/>
-      <c r="E60" s="35" t="n"/>
-    </row>
-    <row r="63" ht="30" customHeight="1">
-      <c r="B63" s="14" t="inlineStr">
+      <c r="D62" s="34" t="n"/>
+      <c r="E62" s="35" t="n"/>
+    </row>
+    <row r="65" ht="30" customHeight="1">
+      <c r="B65" s="14" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · FAMILIAR</t>
         </is>
       </c>
-      <c r="C63" s="15" t="n"/>
-      <c r="D63" s="15" t="n"/>
-      <c r="E63" s="16" t="inlineStr">
+      <c r="C65" s="15" t="n"/>
+      <c r="D65" s="15" t="n"/>
+      <c r="E65" s="16" t="inlineStr">
         <is>
           <t>VG-CRE-03F</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="20" customHeight="1">
-      <c r="B64" s="17" t="inlineStr">
-        <is>
-          <t>Jardines de la Memoria · Inhumación  ·  Destino final · Inhumación familiar</t>
-        </is>
-      </c>
-      <c r="C64" s="18" t="n"/>
-      <c r="D64" s="18" t="n"/>
-      <c r="E64" s="19" t="n"/>
-    </row>
-    <row r="65" ht="20" customHeight="1">
-      <c r="B65" s="20" t="inlineStr">
+    <row r="66" ht="20" customHeight="1">
+      <c r="B66" s="17" t="inlineStr">
+        <is>
+          <t>Jardines de la Memoria · Jardín 1  ·  Destino final · Inhumación familiar</t>
+        </is>
+      </c>
+      <c r="C66" s="18" t="n"/>
+      <c r="D66" s="18" t="n"/>
+      <c r="E66" s="19" t="n"/>
+    </row>
+    <row r="67" ht="20" customHeight="1">
+      <c r="B67" s="20" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C65" s="21" t="n"/>
-      <c r="D65" s="21" t="n"/>
-      <c r="E65" s="22" t="n"/>
-    </row>
-    <row r="66" ht="35" customHeight="1">
-      <c r="B66" s="23" t="inlineStr">
+      <c r="C67" s="21" t="n"/>
+      <c r="D67" s="21" t="n"/>
+      <c r="E67" s="22" t="n"/>
+    </row>
+    <row r="68" ht="35" customHeight="1">
+      <c r="B68" s="23" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C66" s="24" t="inlineStr">
-        <is>
-          <t>Inhumación familiar de urnas en sectores VIP del parque, con placa patrimonial de acabado superior.</t>
-        </is>
-      </c>
-      <c r="D66" s="25" t="n"/>
-      <c r="E66" s="26" t="n"/>
-    </row>
-    <row r="67" ht="20.5" customHeight="1">
-      <c r="B67" s="27" t="inlineStr">
+      <c r="C68" s="24" t="inlineStr">
+        <is>
+          <t>Parcela familiar en el Jardín 1 con cuatro contenedores agrupados, cada uno con tapa de granito grabada, sin plazo de permanencia.</t>
+        </is>
+      </c>
+      <c r="D68" s="25" t="n"/>
+      <c r="E68" s="26" t="n"/>
+    </row>
+    <row r="69" ht="20.5" customHeight="1">
+      <c r="B69" s="27" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C67" s="28" t="inlineStr">
+      <c r="C69" s="28" t="inlineStr">
         <is>
           <t>Hasta 4 espacios (familiar).</t>
         </is>
       </c>
-      <c r="D67" s="29" t="n"/>
-      <c r="E67" s="30" t="n"/>
-    </row>
-    <row r="68" ht="20" customHeight="1">
-      <c r="B68" s="20" t="inlineStr">
+      <c r="D69" s="29" t="n"/>
+      <c r="E69" s="30" t="n"/>
+    </row>
+    <row r="70" ht="20" customHeight="1">
+      <c r="B70" s="20" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C68" s="21" t="n"/>
-      <c r="D68" s="21" t="n"/>
-      <c r="E68" s="22" t="n"/>
-    </row>
-    <row r="69" ht="20.5" customHeight="1">
-      <c r="B69" s="23" t="inlineStr">
-        <is>
-          <t>Versión</t>
-        </is>
-      </c>
-      <c r="C69" s="24" t="inlineStr">
-        <is>
-          <t>Familiar</t>
-        </is>
-      </c>
-      <c r="D69" s="25" t="n"/>
-      <c r="E69" s="26" t="n"/>
-    </row>
-    <row r="70" ht="20.5" customHeight="1">
-      <c r="B70" s="27" t="inlineStr">
-        <is>
-          <t>Capacidad</t>
-        </is>
-      </c>
-      <c r="C70" s="28" t="inlineStr">
-        <is>
-          <t>Hasta 4 espacios</t>
-        </is>
-      </c>
-      <c r="D70" s="29" t="n"/>
-      <c r="E70" s="30" t="n"/>
+      <c r="C70" s="21" t="n"/>
+      <c r="D70" s="21" t="n"/>
+      <c r="E70" s="22" t="n"/>
     </row>
     <row r="71" ht="20.5" customHeight="1">
       <c r="B71" s="23" t="inlineStr">
         <is>
-          <t>Ubicación</t>
+          <t>Ambiente</t>
         </is>
       </c>
       <c r="C71" s="24" t="inlineStr">
         <is>
-          <t>Sectores VIP / preferenciales del parque</t>
+          <t>Jardín 1</t>
         </is>
       </c>
       <c r="D71" s="25" t="n"/>
@@ -1889,191 +1990,195 @@
     <row r="72" ht="20.5" customHeight="1">
       <c r="B72" s="27" t="inlineStr">
         <is>
-          <t>Homenaje</t>
+          <t>Capacidad</t>
         </is>
       </c>
       <c r="C72" s="28" t="inlineStr">
         <is>
-          <t>Placa patrimonial con acabado superior</t>
+          <t>4 contenedores agrupados en losa</t>
         </is>
       </c>
       <c r="D72" s="29" t="n"/>
       <c r="E72" s="30" t="n"/>
     </row>
-    <row r="73" ht="64" customHeight="1">
+    <row r="73" ht="20.5" customHeight="1">
       <c r="B73" s="23" t="inlineStr">
         <is>
-          <t>Servicios incluidos</t>
+          <t>Identificación</t>
         </is>
       </c>
       <c r="C73" s="24" t="inlineStr">
         <is>
-          <t>• Inhumación de hasta 4 urnas
-• Ubicación en sectores VIP / preferenciales del parque
-• Placa patrimonial con acabado superior
-• Lugar físico permanente de homenaje familiar</t>
+          <t>Tapa de granito por espacio, con la información del difunto</t>
         </is>
       </c>
       <c r="D73" s="25" t="n"/>
       <c r="E73" s="26" t="n"/>
     </row>
-    <row r="74" ht="20" customHeight="1">
-      <c r="B74" s="20" t="inlineStr">
-        <is>
-          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
-        </is>
-      </c>
-      <c r="C74" s="21" t="n"/>
-      <c r="D74" s="21" t="n"/>
-      <c r="E74" s="22" t="n"/>
-    </row>
-    <row r="75" ht="26.5" customHeight="1">
+    <row r="74" ht="20.5" customHeight="1">
+      <c r="B74" s="27" t="inlineStr">
+        <is>
+          <t>Permanencia</t>
+        </is>
+      </c>
+      <c r="C74" s="28" t="inlineStr">
+        <is>
+          <t>Sin plazo</t>
+        </is>
+      </c>
+      <c r="D74" s="29" t="n"/>
+      <c r="E74" s="30" t="n"/>
+    </row>
+    <row r="75" ht="20.5" customHeight="1">
       <c r="B75" s="23" t="inlineStr">
         <is>
-          <t>Precio sugerido</t>
-        </is>
-      </c>
-      <c r="C75" s="31" t="inlineStr">
-        <is>
-          <t>US$ 1.490 – US$ 1.990</t>
+          <t>Acceso</t>
+        </is>
+      </c>
+      <c r="C75" s="24" t="inlineStr">
+        <is>
+          <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
         </is>
       </c>
       <c r="D75" s="25" t="n"/>
       <c r="E75" s="26" t="n"/>
     </row>
-    <row r="76" ht="20.5" customHeight="1">
+    <row r="76" ht="64" customHeight="1">
       <c r="B76" s="27" t="inlineStr">
         <is>
-          <t>Base de precio</t>
+          <t>Servicios incluidos</t>
         </is>
       </c>
       <c r="C76" s="28" t="inlineStr">
         <is>
-          <t>Variable según la cantidad de personas · hasta 4 espacios</t>
+          <t>• Inhumación de hasta 4 urnas
+• Tapa de granito grabada para cada espacio
+• Ubicación en el Jardín 1, con paisajismo de plantas de sombra
+• Lugar físico permanente de homenaje familiar, sin plazo</t>
         </is>
       </c>
       <c r="D76" s="29" t="n"/>
       <c r="E76" s="30" t="n"/>
     </row>
-    <row r="77" ht="20.5" customHeight="1">
-      <c r="B77" s="23" t="inlineStr">
+    <row r="77" ht="20" customHeight="1">
+      <c r="B77" s="20" t="inlineStr">
+        <is>
+          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
+        </is>
+      </c>
+      <c r="C77" s="21" t="n"/>
+      <c r="D77" s="21" t="n"/>
+      <c r="E77" s="22" t="n"/>
+    </row>
+    <row r="78" ht="26.5" customHeight="1">
+      <c r="B78" s="23" t="inlineStr">
+        <is>
+          <t>Precio sugerido</t>
+        </is>
+      </c>
+      <c r="C78" s="31" t="inlineStr">
+        <is>
+          <t>US$ 2.000</t>
+        </is>
+      </c>
+      <c r="D78" s="25" t="n"/>
+      <c r="E78" s="26" t="n"/>
+    </row>
+    <row r="79" ht="20.5" customHeight="1">
+      <c r="B79" s="27" t="inlineStr">
+        <is>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C79" s="28" t="inlineStr">
+        <is>
+          <t>Por parcela familiar · hasta 4 espacios</t>
+        </is>
+      </c>
+      <c r="D79" s="29" t="n"/>
+      <c r="E79" s="30" t="n"/>
+    </row>
+    <row r="80" ht="20.5" customHeight="1">
+      <c r="B80" s="23" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C77" s="24" t="inlineStr">
+      <c r="C80" s="24" t="inlineStr">
         <is>
           <t>Pago único o financiado según política comercial vigente.</t>
         </is>
       </c>
-      <c r="D77" s="25" t="n"/>
-      <c r="E77" s="26" t="n"/>
-    </row>
-    <row r="78" ht="20" customHeight="1">
-      <c r="B78" s="20" t="inlineStr">
+      <c r="D80" s="25" t="n"/>
+      <c r="E80" s="26" t="n"/>
+    </row>
+    <row r="81" ht="20" customHeight="1">
+      <c r="B81" s="20" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C78" s="21" t="n"/>
-      <c r="D78" s="21" t="n"/>
-      <c r="E78" s="22" t="n"/>
-    </row>
-    <row r="79" ht="35" customHeight="1">
-      <c r="B79" s="32" t="inlineStr">
+      <c r="C81" s="21" t="n"/>
+      <c r="D81" s="21" t="n"/>
+      <c r="E81" s="22" t="n"/>
+    </row>
+    <row r="82" ht="20.5" customHeight="1">
+      <c r="B82" s="32" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C79" s="33" t="inlineStr">
-        <is>
-          <t>Familias que buscan un espacio patrimonial y exclusivo para varias generaciones.</t>
-        </is>
-      </c>
-      <c r="D79" s="34" t="n"/>
-      <c r="E79" s="35" t="n"/>
-    </row>
-    <row r="82" ht="30" customHeight="1">
-      <c r="B82" s="14" t="inlineStr">
-        <is>
-          <t>JARDÍN DE INHUMACIÓN DE CENIZAS PET</t>
-        </is>
-      </c>
-      <c r="C82" s="15" t="n"/>
-      <c r="D82" s="15" t="n"/>
-      <c r="E82" s="16" t="inlineStr">
-        <is>
-          <t>VG-CRE-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="20" customHeight="1">
-      <c r="B83" s="17" t="inlineStr">
-        <is>
-          <t>Jardines de la Memoria · Mascotas  ·  Mascotas · Cremación e inhumación</t>
-        </is>
-      </c>
-      <c r="C83" s="18" t="n"/>
-      <c r="D83" s="18" t="n"/>
-      <c r="E83" s="19" t="n"/>
-    </row>
-    <row r="84" ht="20" customHeight="1">
-      <c r="B84" s="20" t="inlineStr">
-        <is>
-          <t>VISIÓN GENERAL</t>
-        </is>
-      </c>
-      <c r="C84" s="21" t="n"/>
-      <c r="D84" s="21" t="n"/>
-      <c r="E84" s="22" t="n"/>
-    </row>
-    <row r="85" ht="35" customHeight="1">
-      <c r="B85" s="23" t="inlineStr">
-        <is>
-          <t>Concepto</t>
-        </is>
-      </c>
-      <c r="C85" s="24" t="inlineStr">
-        <is>
-          <t>Servicio de cremación e inhumación de cenizas de mascotas en un área verde dedicada.</t>
-        </is>
-      </c>
-      <c r="D85" s="25" t="n"/>
-      <c r="E85" s="26" t="n"/>
-    </row>
-    <row r="86" ht="20.5" customHeight="1">
-      <c r="B86" s="27" t="inlineStr">
-        <is>
-          <t>Capacidad / Cobertura</t>
-        </is>
-      </c>
-      <c r="C86" s="28" t="inlineStr">
-        <is>
-          <t>Individual (una mascota por servicio).</t>
-        </is>
-      </c>
-      <c r="D86" s="29" t="n"/>
-      <c r="E86" s="30" t="n"/>
+      <c r="C82" s="33" t="inlineStr">
+        <is>
+          <t>Familias que buscan un espacio propio y permanente para varias generaciones.</t>
+        </is>
+      </c>
+      <c r="D82" s="34" t="n"/>
+      <c r="E82" s="35" t="n"/>
+    </row>
+    <row r="85" ht="30" customHeight="1">
+      <c r="B85" s="14" t="inlineStr">
+        <is>
+          <t>JARDÍN DE CENIZAS · ECOLÓGICO</t>
+        </is>
+      </c>
+      <c r="C85" s="15" t="n"/>
+      <c r="D85" s="15" t="n"/>
+      <c r="E85" s="16" t="inlineStr">
+        <is>
+          <t>VG-CRE-03E</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="20" customHeight="1">
+      <c r="B86" s="17" t="inlineStr">
+        <is>
+          <t>Jardines de la Memoria · Jardín 2  ·  Destino final · Inhumación ecológica</t>
+        </is>
+      </c>
+      <c r="C86" s="18" t="n"/>
+      <c r="D86" s="18" t="n"/>
+      <c r="E86" s="19" t="n"/>
     </row>
     <row r="87" ht="20" customHeight="1">
       <c r="B87" s="20" t="inlineStr">
         <is>
-          <t>ESPECIFICACIONES TÉCNICAS</t>
+          <t>VISIÓN GENERAL</t>
         </is>
       </c>
       <c r="C87" s="21" t="n"/>
       <c r="D87" s="21" t="n"/>
       <c r="E87" s="22" t="n"/>
     </row>
-    <row r="88" ht="20.5" customHeight="1">
+    <row r="88" ht="49.5" customHeight="1">
       <c r="B88" s="23" t="inlineStr">
         <is>
-          <t>Tipo de producto</t>
+          <t>Concepto</t>
         </is>
       </c>
       <c r="C88" s="24" t="inlineStr">
         <is>
-          <t>Servicio de pago único</t>
+          <t>La urna biodegradable se entierra directamente en el suelo, se cubre con tierra y se descompone integrándose a la naturaleza. Jardín con agua corriente y área de esparcimiento de cenizas.</t>
         </is>
       </c>
       <c r="D88" s="25" t="n"/>
@@ -2082,80 +2187,78 @@
     <row r="89" ht="20.5" customHeight="1">
       <c r="B89" s="27" t="inlineStr">
         <is>
-          <t>Servicio</t>
+          <t>Capacidad / Cobertura</t>
         </is>
       </c>
       <c r="C89" s="28" t="inlineStr">
         <is>
-          <t>Cremación + inhumación de cenizas</t>
+          <t>Individual (1 urna).</t>
         </is>
       </c>
       <c r="D89" s="29" t="n"/>
       <c r="E89" s="30" t="n"/>
     </row>
-    <row r="90" ht="20.5" customHeight="1">
-      <c r="B90" s="23" t="inlineStr">
-        <is>
-          <t>Espacio</t>
-        </is>
-      </c>
-      <c r="C90" s="24" t="inlineStr">
-        <is>
-          <t>Área verde dedicada a mascotas</t>
-        </is>
-      </c>
-      <c r="D90" s="25" t="n"/>
-      <c r="E90" s="26" t="n"/>
-    </row>
-    <row r="91" ht="49.5" customHeight="1">
-      <c r="B91" s="27" t="inlineStr">
-        <is>
-          <t>Servicios incluidos</t>
-        </is>
-      </c>
-      <c r="C91" s="28" t="inlineStr">
-        <is>
-          <t>• Cremación de la mascota
-• Inhumación de cenizas en área verde dedicada
-• Espacio de homenaje para la familia</t>
-        </is>
-      </c>
-      <c r="D91" s="29" t="n"/>
-      <c r="E91" s="30" t="n"/>
-    </row>
-    <row r="92" ht="20" customHeight="1">
-      <c r="B92" s="20" t="inlineStr">
-        <is>
-          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
-        </is>
-      </c>
-      <c r="C92" s="21" t="n"/>
-      <c r="D92" s="21" t="n"/>
-      <c r="E92" s="22" t="n"/>
-    </row>
-    <row r="93" ht="26.5" customHeight="1">
+    <row r="90" ht="20" customHeight="1">
+      <c r="B90" s="20" t="inlineStr">
+        <is>
+          <t>ESPECIFICACIONES TÉCNICAS</t>
+        </is>
+      </c>
+      <c r="C90" s="21" t="n"/>
+      <c r="D90" s="21" t="n"/>
+      <c r="E90" s="22" t="n"/>
+    </row>
+    <row r="91" ht="20.5" customHeight="1">
+      <c r="B91" s="23" t="inlineStr">
+        <is>
+          <t>Ambientes</t>
+        </is>
+      </c>
+      <c r="C91" s="24" t="inlineStr">
+        <is>
+          <t>Jardín 2 · Ecológico o Bosque de las Orquídeas</t>
+        </is>
+      </c>
+      <c r="D91" s="25" t="n"/>
+      <c r="E91" s="26" t="n"/>
+    </row>
+    <row r="92" ht="20.5" customHeight="1">
+      <c r="B92" s="27" t="inlineStr">
+        <is>
+          <t>Espacio por urna</t>
+        </is>
+      </c>
+      <c r="C92" s="28" t="inlineStr">
+        <is>
+          <t>30 × 30 cm, 40 cm de profundidad</t>
+        </is>
+      </c>
+      <c r="D92" s="29" t="n"/>
+      <c r="E92" s="30" t="n"/>
+    </row>
+    <row r="93" ht="20.5" customHeight="1">
       <c r="B93" s="23" t="inlineStr">
         <is>
-          <t>Precio sugerido</t>
-        </is>
-      </c>
-      <c r="C93" s="31" t="inlineStr">
-        <is>
-          <t>US$ 500</t>
+          <t>Urna</t>
+        </is>
+      </c>
+      <c r="C93" s="24" t="inlineStr">
+        <is>
+          <t>Biodegradable; se integra al suelo</t>
         </is>
       </c>
       <c r="D93" s="25" t="n"/>
       <c r="E93" s="26" t="n"/>
     </row>
-    <row r="94" ht="20.5" customHeight="1">
+    <row r="94" ht="35" customHeight="1">
       <c r="B94" s="27" t="inlineStr">
         <is>
-          <t>Base de precio</t>
+          <t>Identificación (Jardín 2)</t>
         </is>
       </c>
       <c r="C94" s="28" t="inlineStr">
         <is>
-          <t>Pago único por servicio</t>
+          <t>Placa de madera de 20 cm fijada a una varilla metálica, en posición vertical y sin contacto con el suelo</t>
         </is>
       </c>
       <c r="D94" s="29" t="n"/>
@@ -2164,139 +2267,704 @@
     <row r="95" ht="20.5" customHeight="1">
       <c r="B95" s="23" t="inlineStr">
         <is>
-          <t>Condiciones</t>
+          <t>Identificación (Bosque)</t>
         </is>
       </c>
       <c r="C95" s="24" t="inlineStr">
         <is>
-          <t>Pago único; puede contratarse como adicional al plan funerario.</t>
+          <t>Placa de mármol de 20 × 15 cm</t>
         </is>
       </c>
       <c r="D95" s="25" t="n"/>
       <c r="E95" s="26" t="n"/>
     </row>
-    <row r="96" ht="20" customHeight="1">
-      <c r="B96" s="20" t="inlineStr">
+    <row r="96" ht="20.5" customHeight="1">
+      <c r="B96" s="27" t="inlineStr">
+        <is>
+          <t>Acceso</t>
+        </is>
+      </c>
+      <c r="C96" s="28" t="inlineStr">
+        <is>
+          <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
+        </is>
+      </c>
+      <c r="D96" s="29" t="n"/>
+      <c r="E96" s="30" t="n"/>
+    </row>
+    <row r="97" ht="64" customHeight="1">
+      <c r="B97" s="23" t="inlineStr">
+        <is>
+          <t>Servicios incluidos</t>
+        </is>
+      </c>
+      <c r="C97" s="24" t="inlineStr">
+        <is>
+          <t>• Inhumación ecológica de la urna directamente en el suelo
+• Placa de identificación
+• Ubicación en el Jardín 2 o en el Bosque de las Orquídeas
+• Entorno natural con agua corriente</t>
+        </is>
+      </c>
+      <c r="D97" s="25" t="n"/>
+      <c r="E97" s="26" t="n"/>
+    </row>
+    <row r="98" ht="20" customHeight="1">
+      <c r="B98" s="20" t="inlineStr">
+        <is>
+          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
+        </is>
+      </c>
+      <c r="C98" s="21" t="n"/>
+      <c r="D98" s="21" t="n"/>
+      <c r="E98" s="22" t="n"/>
+    </row>
+    <row r="99" ht="26.5" customHeight="1">
+      <c r="B99" s="23" t="inlineStr">
+        <is>
+          <t>Precio sugerido</t>
+        </is>
+      </c>
+      <c r="C99" s="31" t="inlineStr">
+        <is>
+          <t>US$ 600</t>
+        </is>
+      </c>
+      <c r="D99" s="25" t="n"/>
+      <c r="E99" s="26" t="n"/>
+    </row>
+    <row r="100" ht="20.5" customHeight="1">
+      <c r="B100" s="27" t="inlineStr">
+        <is>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C100" s="28" t="inlineStr">
+        <is>
+          <t>Por espacio individual</t>
+        </is>
+      </c>
+      <c r="D100" s="29" t="n"/>
+      <c r="E100" s="30" t="n"/>
+    </row>
+    <row r="101" ht="20.5" customHeight="1">
+      <c r="B101" s="23" t="inlineStr">
+        <is>
+          <t>Condiciones</t>
+        </is>
+      </c>
+      <c r="C101" s="24" t="inlineStr">
+        <is>
+          <t>Pago único o financiado según política comercial vigente.</t>
+        </is>
+      </c>
+      <c r="D101" s="25" t="n"/>
+      <c r="E101" s="26" t="n"/>
+    </row>
+    <row r="102" ht="20" customHeight="1">
+      <c r="B102" s="20" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C96" s="21" t="n"/>
-      <c r="D96" s="21" t="n"/>
-      <c r="E96" s="22" t="n"/>
-    </row>
-    <row r="97" ht="35" customHeight="1">
-      <c r="B97" s="32" t="inlineStr">
+      <c r="C102" s="21" t="n"/>
+      <c r="D102" s="21" t="n"/>
+      <c r="E102" s="22" t="n"/>
+    </row>
+    <row r="103" ht="35" customHeight="1">
+      <c r="B103" s="32" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C97" s="33" t="inlineStr">
-        <is>
-          <t>Familias afiliadas que consideran a su mascota parte del hogar y desean un cierre digno.</t>
-        </is>
-      </c>
-      <c r="D97" s="34" t="n"/>
-      <c r="E97" s="35" t="n"/>
+      <c r="C103" s="33" t="inlineStr">
+        <is>
+          <t>Personas con conciencia ambiental que desean que sus cenizas vuelvan a la tierra, con un lugar identificado para visitar.</t>
+        </is>
+      </c>
+      <c r="D103" s="34" t="n"/>
+      <c r="E103" s="35" t="n"/>
+    </row>
+    <row r="106" ht="30" customHeight="1">
+      <c r="B106" s="14" t="inlineStr">
+        <is>
+          <t>JARDÍN DE CENIZAS · CEREMONIAL</t>
+        </is>
+      </c>
+      <c r="C106" s="15" t="n"/>
+      <c r="D106" s="15" t="n"/>
+      <c r="E106" s="16" t="inlineStr">
+        <is>
+          <t>VG-CRE-03C</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="20" customHeight="1">
+      <c r="B107" s="17" t="inlineStr">
+        <is>
+          <t>Jardines de la Memoria · Jardín 3  ·  Destino final · Inhumación con ceremonia</t>
+        </is>
+      </c>
+      <c r="C107" s="18" t="n"/>
+      <c r="D107" s="18" t="n"/>
+      <c r="E107" s="19" t="n"/>
+    </row>
+    <row r="108" ht="20" customHeight="1">
+      <c r="B108" s="20" t="inlineStr">
+        <is>
+          <t>VISIÓN GENERAL</t>
+        </is>
+      </c>
+      <c r="C108" s="21" t="n"/>
+      <c r="D108" s="21" t="n"/>
+      <c r="E108" s="22" t="n"/>
+    </row>
+    <row r="109" ht="35" customHeight="1">
+      <c r="B109" s="23" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="C109" s="24" t="inlineStr">
+        <is>
+          <t>Jardín para inhumación de urnas de cenizas con ceremonia de agua, con fuentes como elemento central del rito de despedida.</t>
+        </is>
+      </c>
+      <c r="D109" s="25" t="n"/>
+      <c r="E109" s="26" t="n"/>
+    </row>
+    <row r="110" ht="20.5" customHeight="1">
+      <c r="B110" s="27" t="inlineStr">
+        <is>
+          <t>Capacidad / Cobertura</t>
+        </is>
+      </c>
+      <c r="C110" s="28" t="inlineStr">
+        <is>
+          <t>A definir.</t>
+        </is>
+      </c>
+      <c r="D110" s="29" t="n"/>
+      <c r="E110" s="30" t="n"/>
+    </row>
+    <row r="111" ht="20" customHeight="1">
+      <c r="B111" s="20" t="inlineStr">
+        <is>
+          <t>ESPECIFICACIONES TÉCNICAS</t>
+        </is>
+      </c>
+      <c r="C111" s="21" t="n"/>
+      <c r="D111" s="21" t="n"/>
+      <c r="E111" s="22" t="n"/>
+    </row>
+    <row r="112" ht="20.5" customHeight="1">
+      <c r="B112" s="23" t="inlineStr">
+        <is>
+          <t>Ambiente</t>
+        </is>
+      </c>
+      <c r="C112" s="24" t="inlineStr">
+        <is>
+          <t>Jardín 3</t>
+        </is>
+      </c>
+      <c r="D112" s="25" t="n"/>
+      <c r="E112" s="26" t="n"/>
+    </row>
+    <row r="113" ht="20.5" customHeight="1">
+      <c r="B113" s="27" t="inlineStr">
+        <is>
+          <t>Elemento central</t>
+        </is>
+      </c>
+      <c r="C113" s="28" t="inlineStr">
+        <is>
+          <t>Fuente de agua para la ceremonia</t>
+        </is>
+      </c>
+      <c r="D113" s="29" t="n"/>
+      <c r="E113" s="30" t="n"/>
+    </row>
+    <row r="114" ht="20.5" customHeight="1">
+      <c r="B114" s="23" t="inlineStr">
+        <is>
+          <t>Entorno</t>
+        </is>
+      </c>
+      <c r="C114" s="24" t="inlineStr">
+        <is>
+          <t>Barrera visual que separa el jardín del crematorio</t>
+        </is>
+      </c>
+      <c r="D114" s="25" t="n"/>
+      <c r="E114" s="26" t="n"/>
+    </row>
+    <row r="115" ht="35" customHeight="1">
+      <c r="B115" s="27" t="inlineStr">
+        <is>
+          <t>Servicios incluidos</t>
+        </is>
+      </c>
+      <c r="C115" s="28" t="inlineStr">
+        <is>
+          <t>• Inhumación de urnas de cenizas
+• Ceremonia con agua en fuente</t>
+        </is>
+      </c>
+      <c r="D115" s="29" t="n"/>
+      <c r="E115" s="30" t="n"/>
+    </row>
+    <row r="116" ht="20" customHeight="1">
+      <c r="B116" s="20" t="inlineStr">
+        <is>
+          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
+        </is>
+      </c>
+      <c r="C116" s="21" t="n"/>
+      <c r="D116" s="21" t="n"/>
+      <c r="E116" s="22" t="n"/>
+    </row>
+    <row r="117" ht="26.5" customHeight="1">
+      <c r="B117" s="23" t="inlineStr">
+        <is>
+          <t>Precio sugerido</t>
+        </is>
+      </c>
+      <c r="C117" s="31" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="D117" s="25" t="n"/>
+      <c r="E117" s="26" t="n"/>
+    </row>
+    <row r="118" ht="20.5" customHeight="1">
+      <c r="B118" s="27" t="inlineStr">
+        <is>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C118" s="28" t="inlineStr">
+        <is>
+          <t>Producto en definición</t>
+        </is>
+      </c>
+      <c r="D118" s="29" t="n"/>
+      <c r="E118" s="30" t="n"/>
+    </row>
+    <row r="119" ht="20.5" customHeight="1">
+      <c r="B119" s="23" t="inlineStr">
+        <is>
+          <t>Condiciones</t>
+        </is>
+      </c>
+      <c r="C119" s="24" t="inlineStr">
+        <is>
+          <t>A definir.</t>
+        </is>
+      </c>
+      <c r="D119" s="25" t="n"/>
+      <c r="E119" s="26" t="n"/>
+    </row>
+    <row r="120" ht="20" customHeight="1">
+      <c r="B120" s="20" t="inlineStr">
+        <is>
+          <t>PERFIL DEL COMPRADOR</t>
+        </is>
+      </c>
+      <c r="C120" s="21" t="n"/>
+      <c r="D120" s="21" t="n"/>
+      <c r="E120" s="22" t="n"/>
+    </row>
+    <row r="121" ht="35" customHeight="1">
+      <c r="B121" s="32" t="inlineStr">
+        <is>
+          <t>Cliente objetivo</t>
+        </is>
+      </c>
+      <c r="C121" s="33" t="inlineStr">
+        <is>
+          <t>Familias que valoran un rito de despedida simbólico y un entorno contemplativo.</t>
+        </is>
+      </c>
+      <c r="D121" s="34" t="n"/>
+      <c r="E121" s="35" t="n"/>
+    </row>
+    <row r="124" ht="30" customHeight="1">
+      <c r="B124" s="14" t="inlineStr">
+        <is>
+          <t>JARDÍN DE MASCOTAS</t>
+        </is>
+      </c>
+      <c r="C124" s="15" t="n"/>
+      <c r="D124" s="15" t="n"/>
+      <c r="E124" s="16" t="inlineStr">
+        <is>
+          <t>VG-CRE-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="20" customHeight="1">
+      <c r="B125" s="17" t="inlineStr">
+        <is>
+          <t>Jardines de la Memoria · Mascotas  ·  Mascotas · Inhumación ecológica</t>
+        </is>
+      </c>
+      <c r="C125" s="18" t="n"/>
+      <c r="D125" s="18" t="n"/>
+      <c r="E125" s="19" t="n"/>
+    </row>
+    <row r="126" ht="20" customHeight="1">
+      <c r="B126" s="20" t="inlineStr">
+        <is>
+          <t>VISIÓN GENERAL</t>
+        </is>
+      </c>
+      <c r="C126" s="21" t="n"/>
+      <c r="D126" s="21" t="n"/>
+      <c r="E126" s="22" t="n"/>
+    </row>
+    <row r="127" ht="35" customHeight="1">
+      <c r="B127" s="23" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="C127" s="24" t="inlineStr">
+        <is>
+          <t>Jardín para inhumación ecológica de cenizas de mascotas: la urna biodegradable se entierra directamente en el suelo y se identifica con una placa de madera.</t>
+        </is>
+      </c>
+      <c r="D127" s="25" t="n"/>
+      <c r="E127" s="26" t="n"/>
+    </row>
+    <row r="128" ht="20.5" customHeight="1">
+      <c r="B128" s="27" t="inlineStr">
+        <is>
+          <t>Capacidad / Cobertura</t>
+        </is>
+      </c>
+      <c r="C128" s="28" t="inlineStr">
+        <is>
+          <t>Individual (una mascota por servicio).</t>
+        </is>
+      </c>
+      <c r="D128" s="29" t="n"/>
+      <c r="E128" s="30" t="n"/>
+    </row>
+    <row r="129" ht="20" customHeight="1">
+      <c r="B129" s="20" t="inlineStr">
+        <is>
+          <t>ESPECIFICACIONES TÉCNICAS</t>
+        </is>
+      </c>
+      <c r="C129" s="21" t="n"/>
+      <c r="D129" s="21" t="n"/>
+      <c r="E129" s="22" t="n"/>
+    </row>
+    <row r="130" ht="20.5" customHeight="1">
+      <c r="B130" s="23" t="inlineStr">
+        <is>
+          <t>Tipo de producto</t>
+        </is>
+      </c>
+      <c r="C130" s="24" t="inlineStr">
+        <is>
+          <t>Servicio de pago único</t>
+        </is>
+      </c>
+      <c r="D130" s="25" t="n"/>
+      <c r="E130" s="26" t="n"/>
+    </row>
+    <row r="131" ht="20.5" customHeight="1">
+      <c r="B131" s="27" t="inlineStr">
+        <is>
+          <t>Espacio por urna</t>
+        </is>
+      </c>
+      <c r="C131" s="28" t="inlineStr">
+        <is>
+          <t>15 × 20 cm o 15 × 30 cm, según el tamaño de la urna</t>
+        </is>
+      </c>
+      <c r="D131" s="29" t="n"/>
+      <c r="E131" s="30" t="n"/>
+    </row>
+    <row r="132" ht="20.5" customHeight="1">
+      <c r="B132" s="23" t="inlineStr">
+        <is>
+          <t>Urna</t>
+        </is>
+      </c>
+      <c r="C132" s="24" t="inlineStr">
+        <is>
+          <t>Biodegradable; se integra al suelo</t>
+        </is>
+      </c>
+      <c r="D132" s="25" t="n"/>
+      <c r="E132" s="26" t="n"/>
+    </row>
+    <row r="133" ht="20.5" customHeight="1">
+      <c r="B133" s="27" t="inlineStr">
+        <is>
+          <t>Identificación</t>
+        </is>
+      </c>
+      <c r="C133" s="28" t="inlineStr">
+        <is>
+          <t>Placa de madera de 20 cm</t>
+        </is>
+      </c>
+      <c r="D133" s="29" t="n"/>
+      <c r="E133" s="30" t="n"/>
+    </row>
+    <row r="134" ht="20.5" customHeight="1">
+      <c r="B134" s="23" t="inlineStr">
+        <is>
+          <t>Homenaje</t>
+        </is>
+      </c>
+      <c r="C134" s="24" t="inlineStr">
+        <is>
+          <t>Placa conmemorativa colectiva en el jardín</t>
+        </is>
+      </c>
+      <c r="D134" s="25" t="n"/>
+      <c r="E134" s="26" t="n"/>
+    </row>
+    <row r="135" ht="64" customHeight="1">
+      <c r="B135" s="27" t="inlineStr">
+        <is>
+          <t>Servicios incluidos</t>
+        </is>
+      </c>
+      <c r="C135" s="28" t="inlineStr">
+        <is>
+          <t>• Inhumación ecológica de la urna en el jardín
+• Placa de madera de 20 cm para identificación
+• Nombre de la mascota en la placa conmemorativa del jardín
+• Cremación de la mascota (opción Jardín + Cremación)</t>
+        </is>
+      </c>
+      <c r="D135" s="29" t="n"/>
+      <c r="E135" s="30" t="n"/>
+    </row>
+    <row r="136" ht="20" customHeight="1">
+      <c r="B136" s="20" t="inlineStr">
+        <is>
+          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
+        </is>
+      </c>
+      <c r="C136" s="21" t="n"/>
+      <c r="D136" s="21" t="n"/>
+      <c r="E136" s="22" t="n"/>
+    </row>
+    <row r="137" ht="26.5" customHeight="1">
+      <c r="B137" s="23" t="inlineStr">
+        <is>
+          <t>Precio sugerido</t>
+        </is>
+      </c>
+      <c r="C137" s="31" t="inlineStr">
+        <is>
+          <t>US$ 350 / US$ 500</t>
+        </is>
+      </c>
+      <c r="D137" s="25" t="n"/>
+      <c r="E137" s="26" t="n"/>
+    </row>
+    <row r="138" ht="20.5" customHeight="1">
+      <c r="B138" s="27" t="inlineStr">
+        <is>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C138" s="28" t="inlineStr">
+        <is>
+          <t>US$ 350 solo jardín · US$ 500 jardín + cremación</t>
+        </is>
+      </c>
+      <c r="D138" s="29" t="n"/>
+      <c r="E138" s="30" t="n"/>
+    </row>
+    <row r="139" ht="20.5" customHeight="1">
+      <c r="B139" s="23" t="inlineStr">
+        <is>
+          <t>Condiciones</t>
+        </is>
+      </c>
+      <c r="C139" s="24" t="inlineStr">
+        <is>
+          <t>Pago único; puede contratarse como adicional al plan funerario.</t>
+        </is>
+      </c>
+      <c r="D139" s="25" t="n"/>
+      <c r="E139" s="26" t="n"/>
+    </row>
+    <row r="140" ht="20" customHeight="1">
+      <c r="B140" s="20" t="inlineStr">
+        <is>
+          <t>PERFIL DEL COMPRADOR</t>
+        </is>
+      </c>
+      <c r="C140" s="21" t="n"/>
+      <c r="D140" s="21" t="n"/>
+      <c r="E140" s="22" t="n"/>
+    </row>
+    <row r="141" ht="20.5" customHeight="1">
+      <c r="B141" s="32" t="inlineStr">
+        <is>
+          <t>Cliente objetivo</t>
+        </is>
+      </c>
+      <c r="C141" s="33" t="inlineStr">
+        <is>
+          <t>Familias que consideran a su mascota parte del hogar y desean un cierre digno.</t>
+        </is>
+      </c>
+      <c r="D141" s="34" t="n"/>
+      <c r="E141" s="35" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="88">
-    <mergeCell ref="B65:E65"/>
+  <mergeCells count="128">
     <mergeCell ref="C31:E31"/>
-    <mergeCell ref="B74:E74"/>
-    <mergeCell ref="B68:E68"/>
-    <mergeCell ref="B44:D44"/>
-    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="C80:E80"/>
+    <mergeCell ref="C40:E40"/>
     <mergeCell ref="C51:E51"/>
     <mergeCell ref="C95:E95"/>
-    <mergeCell ref="B45:E45"/>
     <mergeCell ref="C60:E60"/>
     <mergeCell ref="C71:E71"/>
+    <mergeCell ref="B47:E47"/>
     <mergeCell ref="C7:E7"/>
     <mergeCell ref="C91:E91"/>
-    <mergeCell ref="C57:E57"/>
+    <mergeCell ref="B102:E102"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="B21:E21"/>
     <mergeCell ref="C18:E18"/>
-    <mergeCell ref="C77:E77"/>
+    <mergeCell ref="C49:E49"/>
+    <mergeCell ref="B86:E86"/>
+    <mergeCell ref="C101:E101"/>
     <mergeCell ref="C34:E34"/>
+    <mergeCell ref="B136:E136"/>
+    <mergeCell ref="C42:E42"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B78:E78"/>
+    <mergeCell ref="C74:E74"/>
+    <mergeCell ref="C141:E141"/>
     <mergeCell ref="B87:E87"/>
+    <mergeCell ref="C128:E128"/>
     <mergeCell ref="C20:E20"/>
-    <mergeCell ref="C85:E85"/>
-    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="C113:E113"/>
+    <mergeCell ref="C103:E103"/>
+    <mergeCell ref="C112:E112"/>
+    <mergeCell ref="C99:E99"/>
     <mergeCell ref="C94:E94"/>
-    <mergeCell ref="B49:E49"/>
+    <mergeCell ref="C118:E118"/>
     <mergeCell ref="C75:E75"/>
+    <mergeCell ref="C133:E133"/>
     <mergeCell ref="C22:E22"/>
-    <mergeCell ref="B64:E64"/>
-    <mergeCell ref="B82:D82"/>
+    <mergeCell ref="C127:E127"/>
+    <mergeCell ref="C114:E114"/>
+    <mergeCell ref="C59:E59"/>
+    <mergeCell ref="C130:E130"/>
     <mergeCell ref="C12:E12"/>
     <mergeCell ref="B26:E26"/>
+    <mergeCell ref="B41:E41"/>
+    <mergeCell ref="B50:E50"/>
     <mergeCell ref="C52:E52"/>
+    <mergeCell ref="B129:E129"/>
     <mergeCell ref="C39:E39"/>
     <mergeCell ref="B16:E16"/>
-    <mergeCell ref="C70:E70"/>
     <mergeCell ref="C48:E48"/>
+    <mergeCell ref="B90:E90"/>
     <mergeCell ref="C32:E32"/>
     <mergeCell ref="C38:E38"/>
+    <mergeCell ref="B66:E66"/>
+    <mergeCell ref="B124:D124"/>
     <mergeCell ref="B27:E27"/>
+    <mergeCell ref="B140:E140"/>
     <mergeCell ref="C13:E13"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="B85:D85"/>
+    <mergeCell ref="C131:E131"/>
+    <mergeCell ref="B77:E77"/>
     <mergeCell ref="C15:E15"/>
+    <mergeCell ref="B67:E67"/>
+    <mergeCell ref="B61:E61"/>
     <mergeCell ref="C33:E33"/>
     <mergeCell ref="C89:E89"/>
     <mergeCell ref="C79:E79"/>
     <mergeCell ref="C73:E73"/>
     <mergeCell ref="C88:E88"/>
+    <mergeCell ref="B116:E116"/>
+    <mergeCell ref="B37:E37"/>
     <mergeCell ref="C35:E35"/>
-    <mergeCell ref="B84:E84"/>
+    <mergeCell ref="C121:E121"/>
     <mergeCell ref="C10:E10"/>
-    <mergeCell ref="C50:E50"/>
+    <mergeCell ref="C117:E117"/>
+    <mergeCell ref="C55:E55"/>
     <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B55:E55"/>
+    <mergeCell ref="C115:E115"/>
+    <mergeCell ref="C36:E36"/>
     <mergeCell ref="C11:E11"/>
-    <mergeCell ref="C67:E67"/>
+    <mergeCell ref="C135:E135"/>
+    <mergeCell ref="B65:D65"/>
+    <mergeCell ref="B81:E81"/>
     <mergeCell ref="C72:E72"/>
     <mergeCell ref="C28:E28"/>
-    <mergeCell ref="C37:E37"/>
-    <mergeCell ref="B63:D63"/>
     <mergeCell ref="C69:E69"/>
+    <mergeCell ref="C96:E96"/>
+    <mergeCell ref="C78:E78"/>
+    <mergeCell ref="B120:E120"/>
     <mergeCell ref="B2:E2"/>
+    <mergeCell ref="C92:E92"/>
     <mergeCell ref="B25:D25"/>
+    <mergeCell ref="B107:E107"/>
+    <mergeCell ref="C62:E62"/>
     <mergeCell ref="C14:E14"/>
+    <mergeCell ref="B57:E57"/>
     <mergeCell ref="C54:E54"/>
+    <mergeCell ref="B108:E108"/>
     <mergeCell ref="B9:E9"/>
-    <mergeCell ref="C41:E41"/>
-    <mergeCell ref="B83:E83"/>
+    <mergeCell ref="C137:E137"/>
+    <mergeCell ref="C134:E134"/>
     <mergeCell ref="C93:E93"/>
-    <mergeCell ref="B92:E92"/>
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="C56:E56"/>
     <mergeCell ref="B5:E5"/>
-    <mergeCell ref="C90:E90"/>
+    <mergeCell ref="C139:E139"/>
+    <mergeCell ref="C138:E138"/>
     <mergeCell ref="C76:E76"/>
+    <mergeCell ref="B126:E126"/>
+    <mergeCell ref="C132:E132"/>
+    <mergeCell ref="C110:E110"/>
+    <mergeCell ref="C119:E119"/>
     <mergeCell ref="C8:E8"/>
     <mergeCell ref="C17:E17"/>
-    <mergeCell ref="B59:E59"/>
+    <mergeCell ref="C82:E82"/>
+    <mergeCell ref="B125:E125"/>
     <mergeCell ref="B46:E46"/>
-    <mergeCell ref="C66:E66"/>
     <mergeCell ref="C19:E19"/>
     <mergeCell ref="C53:E53"/>
-    <mergeCell ref="B96:E96"/>
-    <mergeCell ref="C86:E86"/>
+    <mergeCell ref="B70:E70"/>
+    <mergeCell ref="B106:D106"/>
+    <mergeCell ref="C68:E68"/>
+    <mergeCell ref="B111:E111"/>
+    <mergeCell ref="B98:E98"/>
     <mergeCell ref="C58:E58"/>
     <mergeCell ref="C97:E97"/>
     <mergeCell ref="C29:E29"/>
-    <mergeCell ref="C47:E47"/>
+    <mergeCell ref="C100:E100"/>
+    <mergeCell ref="C109:E109"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
-  <rowBreaks count="4" manualBreakCount="4">
+  <rowBreaks count="6" manualBreakCount="6">
     <brk id="23" min="0" max="16383" man="1"/>
-    <brk id="42" min="0" max="16383" man="1"/>
-    <brk id="61" min="0" max="16383" man="1"/>
-    <brk id="80" min="0" max="16383" man="1"/>
+    <brk id="43" min="0" max="16383" man="1"/>
+    <brk id="63" min="0" max="16383" man="1"/>
+    <brk id="83" min="0" max="16383" man="1"/>
+    <brk id="104" min="0" max="16383" man="1"/>
+    <brk id="122" min="0" max="16383" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Agrega mantenimiento anual y plazo de 3 años con placa memorial
- Individual: mantenimiento US$ 15/año; Familiar: US$ 25/año
- Ecológico y Mascotas: permanencia de 3 años; luego placa memorial en
  el monumento (US$ 150 humano / US$ 50 mascota) y reutilización del espacio

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111i7vn9WWo4QxCQbucWbrF
</commit_message>
<xml_diff>
--- a/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
+++ b/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
@@ -13,7 +13,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tabla Gral. - Visión Comercial'!$A$4:$I$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Tabla Gral. - Visión Comercial'!$4:$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Ficha Técnica Consolidada'!$A$1:$F$142</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Ficha Técnica Consolidada'!$A$1:$F$147</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -927,12 +927,12 @@
       <c r="H7" s="7" t="inlineStr">
         <is>
           <t>US$ 600
-(Por espacio individual)</t>
+(Por espacio individual · mantenimiento US$ 15/año)</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>Pago único o financiado según política comercial vigente.</t>
+          <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 15 anual.</t>
         </is>
       </c>
     </row>
@@ -978,16 +978,16 @@
       <c r="H8" s="11" t="inlineStr">
         <is>
           <t>US$ 2.000
-(Por parcela familiar · hasta 4 espacios)</t>
+(Por parcela familiar · hasta 4 espacios · mantenimiento US$ 25/año)</t>
         </is>
       </c>
       <c r="I8" s="10" t="inlineStr">
         <is>
-          <t>Pago único o financiado según política comercial vigente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="93" customHeight="1">
+          <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 25 anual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="122" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>VG-CRE-03E</t>
@@ -1018,7 +1018,8 @@
           <t>• Inhumación ecológica de la urna directamente en el suelo
 • Placa de identificación
 • Ubicación en el Jardín 2 o en el Bosque de las Orquídeas
-• Entorno natural con agua corriente</t>
+• Entorno natural con agua corriente
+• Permanencia de 3 años; luego, placa memorial en el monumento</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -1029,12 +1030,12 @@
       <c r="H9" s="7" t="inlineStr">
         <is>
           <t>US$ 600
-(Por espacio individual)</t>
+(Por espacio individual · placa memorial US$ 150)</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>Pago único o financiado según política comercial vigente.</t>
+          <t>Pago único o financiado según política comercial vigente. Placa memorial en el monumento al término del plazo: US$ 150.</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1118,7 @@
         <is>
           <t>• Inhumación ecológica de la urna en el jardín
 • Placa de madera de 20 cm para identificación
-• Nombre de la mascota en la placa conmemorativa del jardín
+• Permanencia de 3 años; luego, placa memorial en el monumento
 • Cremación de la mascota (opción Jardín + Cremación)</t>
         </is>
       </c>
@@ -1134,7 +1135,7 @@
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>Pago único; puede contratarse como adicional al plan funerario.</t>
+          <t>Pago único; puede contratarse como adicional al plan funerario. Placa memorial en el monumento al término del plazo: US$ 50.</t>
         </is>
       </c>
     </row>
@@ -1156,7 +1157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:E141"/>
+  <dimension ref="B1:E146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1808,13 +1809,27 @@
       <c r="D55" s="25" t="n"/>
       <c r="E55" s="26" t="n"/>
     </row>
-    <row r="56" ht="64" customHeight="1">
+    <row r="56" ht="20.5" customHeight="1">
       <c r="B56" s="27" t="inlineStr">
         <is>
+          <t>Mantenimiento</t>
+        </is>
+      </c>
+      <c r="C56" s="28" t="inlineStr">
+        <is>
+          <t>US$ 15 anual</t>
+        </is>
+      </c>
+      <c r="D56" s="29" t="n"/>
+      <c r="E56" s="30" t="n"/>
+    </row>
+    <row r="57" ht="64" customHeight="1">
+      <c r="B57" s="23" t="inlineStr">
+        <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C56" s="28" t="inlineStr">
+      <c r="C57" s="24" t="inlineStr">
         <is>
           <t>• Inhumación de la urna en contenedor individual
 • Tapa de granito con los datos del difunto
@@ -1822,234 +1837,248 @@
 • Espacio de contemplación con banco</t>
         </is>
       </c>
-      <c r="D56" s="29" t="n"/>
-      <c r="E56" s="30" t="n"/>
-    </row>
-    <row r="57" ht="20" customHeight="1">
-      <c r="B57" s="20" t="inlineStr">
+      <c r="D57" s="25" t="n"/>
+      <c r="E57" s="26" t="n"/>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="B58" s="20" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C57" s="21" t="n"/>
-      <c r="D57" s="21" t="n"/>
-      <c r="E57" s="22" t="n"/>
-    </row>
-    <row r="58" ht="26.5" customHeight="1">
-      <c r="B58" s="23" t="inlineStr">
+      <c r="C58" s="21" t="n"/>
+      <c r="D58" s="21" t="n"/>
+      <c r="E58" s="22" t="n"/>
+    </row>
+    <row r="59" ht="26.5" customHeight="1">
+      <c r="B59" s="23" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C58" s="31" t="inlineStr">
+      <c r="C59" s="31" t="inlineStr">
         <is>
           <t>US$ 600</t>
         </is>
       </c>
-      <c r="D58" s="25" t="n"/>
-      <c r="E58" s="26" t="n"/>
-    </row>
-    <row r="59" ht="20.5" customHeight="1">
-      <c r="B59" s="27" t="inlineStr">
+      <c r="D59" s="25" t="n"/>
+      <c r="E59" s="26" t="n"/>
+    </row>
+    <row r="60" ht="20.5" customHeight="1">
+      <c r="B60" s="27" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C59" s="28" t="inlineStr">
-        <is>
-          <t>Por espacio individual</t>
-        </is>
-      </c>
-      <c r="D59" s="29" t="n"/>
-      <c r="E59" s="30" t="n"/>
-    </row>
-    <row r="60" ht="20.5" customHeight="1">
-      <c r="B60" s="23" t="inlineStr">
+      <c r="C60" s="28" t="inlineStr">
+        <is>
+          <t>Por espacio individual · mantenimiento US$ 15/año</t>
+        </is>
+      </c>
+      <c r="D60" s="29" t="n"/>
+      <c r="E60" s="30" t="n"/>
+    </row>
+    <row r="61" ht="35" customHeight="1">
+      <c r="B61" s="23" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C60" s="24" t="inlineStr">
-        <is>
-          <t>Pago único o financiado según política comercial vigente.</t>
-        </is>
-      </c>
-      <c r="D60" s="25" t="n"/>
-      <c r="E60" s="26" t="n"/>
-    </row>
-    <row r="61" ht="20" customHeight="1">
-      <c r="B61" s="20" t="inlineStr">
+      <c r="C61" s="24" t="inlineStr">
+        <is>
+          <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 15 anual.</t>
+        </is>
+      </c>
+      <c r="D61" s="25" t="n"/>
+      <c r="E61" s="26" t="n"/>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="B62" s="20" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C61" s="21" t="n"/>
-      <c r="D61" s="21" t="n"/>
-      <c r="E61" s="22" t="n"/>
-    </row>
-    <row r="62" ht="35" customHeight="1">
-      <c r="B62" s="32" t="inlineStr">
+      <c r="C62" s="21" t="n"/>
+      <c r="D62" s="21" t="n"/>
+      <c r="E62" s="22" t="n"/>
+    </row>
+    <row r="63" ht="35" customHeight="1">
+      <c r="B63" s="32" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C62" s="33" t="inlineStr">
+      <c r="C63" s="33" t="inlineStr">
         <is>
           <t>Familias que desean un lugar permanente para visitar y rendir homenaje, con una inversión moderada.</t>
         </is>
       </c>
-      <c r="D62" s="34" t="n"/>
-      <c r="E62" s="35" t="n"/>
-    </row>
-    <row r="65" ht="30" customHeight="1">
-      <c r="B65" s="14" t="inlineStr">
+      <c r="D63" s="34" t="n"/>
+      <c r="E63" s="35" t="n"/>
+    </row>
+    <row r="66" ht="30" customHeight="1">
+      <c r="B66" s="14" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · FAMILIAR</t>
         </is>
       </c>
-      <c r="C65" s="15" t="n"/>
-      <c r="D65" s="15" t="n"/>
-      <c r="E65" s="16" t="inlineStr">
+      <c r="C66" s="15" t="n"/>
+      <c r="D66" s="15" t="n"/>
+      <c r="E66" s="16" t="inlineStr">
         <is>
           <t>VG-CRE-03F</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="20" customHeight="1">
-      <c r="B66" s="17" t="inlineStr">
+    <row r="67" ht="20" customHeight="1">
+      <c r="B67" s="17" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Jardín 1  ·  Destino final · Inhumación familiar</t>
         </is>
       </c>
-      <c r="C66" s="18" t="n"/>
-      <c r="D66" s="18" t="n"/>
-      <c r="E66" s="19" t="n"/>
-    </row>
-    <row r="67" ht="20" customHeight="1">
-      <c r="B67" s="20" t="inlineStr">
+      <c r="C67" s="18" t="n"/>
+      <c r="D67" s="18" t="n"/>
+      <c r="E67" s="19" t="n"/>
+    </row>
+    <row r="68" ht="20" customHeight="1">
+      <c r="B68" s="20" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C67" s="21" t="n"/>
-      <c r="D67" s="21" t="n"/>
-      <c r="E67" s="22" t="n"/>
-    </row>
-    <row r="68" ht="35" customHeight="1">
-      <c r="B68" s="23" t="inlineStr">
+      <c r="C68" s="21" t="n"/>
+      <c r="D68" s="21" t="n"/>
+      <c r="E68" s="22" t="n"/>
+    </row>
+    <row r="69" ht="35" customHeight="1">
+      <c r="B69" s="23" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C68" s="24" t="inlineStr">
+      <c r="C69" s="24" t="inlineStr">
         <is>
           <t>Parcela familiar en el Jardín 1 con cuatro contenedores agrupados, cada uno con tapa de granito grabada, sin plazo de permanencia.</t>
         </is>
       </c>
-      <c r="D68" s="25" t="n"/>
-      <c r="E68" s="26" t="n"/>
-    </row>
-    <row r="69" ht="20.5" customHeight="1">
-      <c r="B69" s="27" t="inlineStr">
+      <c r="D69" s="25" t="n"/>
+      <c r="E69" s="26" t="n"/>
+    </row>
+    <row r="70" ht="20.5" customHeight="1">
+      <c r="B70" s="27" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C69" s="28" t="inlineStr">
+      <c r="C70" s="28" t="inlineStr">
         <is>
           <t>Hasta 4 espacios (familiar).</t>
         </is>
       </c>
-      <c r="D69" s="29" t="n"/>
-      <c r="E69" s="30" t="n"/>
-    </row>
-    <row r="70" ht="20" customHeight="1">
-      <c r="B70" s="20" t="inlineStr">
+      <c r="D70" s="29" t="n"/>
+      <c r="E70" s="30" t="n"/>
+    </row>
+    <row r="71" ht="20" customHeight="1">
+      <c r="B71" s="20" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C70" s="21" t="n"/>
-      <c r="D70" s="21" t="n"/>
-      <c r="E70" s="22" t="n"/>
-    </row>
-    <row r="71" ht="20.5" customHeight="1">
-      <c r="B71" s="23" t="inlineStr">
+      <c r="C71" s="21" t="n"/>
+      <c r="D71" s="21" t="n"/>
+      <c r="E71" s="22" t="n"/>
+    </row>
+    <row r="72" ht="20.5" customHeight="1">
+      <c r="B72" s="23" t="inlineStr">
         <is>
           <t>Ambiente</t>
         </is>
       </c>
-      <c r="C71" s="24" t="inlineStr">
+      <c r="C72" s="24" t="inlineStr">
         <is>
           <t>Jardín 1</t>
         </is>
       </c>
-      <c r="D71" s="25" t="n"/>
-      <c r="E71" s="26" t="n"/>
-    </row>
-    <row r="72" ht="20.5" customHeight="1">
-      <c r="B72" s="27" t="inlineStr">
+      <c r="D72" s="25" t="n"/>
+      <c r="E72" s="26" t="n"/>
+    </row>
+    <row r="73" ht="20.5" customHeight="1">
+      <c r="B73" s="27" t="inlineStr">
         <is>
           <t>Capacidad</t>
         </is>
       </c>
-      <c r="C72" s="28" t="inlineStr">
+      <c r="C73" s="28" t="inlineStr">
         <is>
           <t>4 contenedores agrupados en losa</t>
         </is>
       </c>
-      <c r="D72" s="29" t="n"/>
-      <c r="E72" s="30" t="n"/>
-    </row>
-    <row r="73" ht="20.5" customHeight="1">
-      <c r="B73" s="23" t="inlineStr">
+      <c r="D73" s="29" t="n"/>
+      <c r="E73" s="30" t="n"/>
+    </row>
+    <row r="74" ht="20.5" customHeight="1">
+      <c r="B74" s="23" t="inlineStr">
         <is>
           <t>Identificación</t>
         </is>
       </c>
-      <c r="C73" s="24" t="inlineStr">
+      <c r="C74" s="24" t="inlineStr">
         <is>
           <t>Tapa de granito por espacio, con la información del difunto</t>
         </is>
       </c>
-      <c r="D73" s="25" t="n"/>
-      <c r="E73" s="26" t="n"/>
-    </row>
-    <row r="74" ht="20.5" customHeight="1">
-      <c r="B74" s="27" t="inlineStr">
+      <c r="D74" s="25" t="n"/>
+      <c r="E74" s="26" t="n"/>
+    </row>
+    <row r="75" ht="20.5" customHeight="1">
+      <c r="B75" s="27" t="inlineStr">
         <is>
           <t>Permanencia</t>
         </is>
       </c>
-      <c r="C74" s="28" t="inlineStr">
+      <c r="C75" s="28" t="inlineStr">
         <is>
           <t>Sin plazo</t>
         </is>
       </c>
-      <c r="D74" s="29" t="n"/>
-      <c r="E74" s="30" t="n"/>
-    </row>
-    <row r="75" ht="20.5" customHeight="1">
-      <c r="B75" s="23" t="inlineStr">
+      <c r="D75" s="29" t="n"/>
+      <c r="E75" s="30" t="n"/>
+    </row>
+    <row r="76" ht="20.5" customHeight="1">
+      <c r="B76" s="23" t="inlineStr">
         <is>
           <t>Acceso</t>
         </is>
       </c>
-      <c r="C75" s="24" t="inlineStr">
+      <c r="C76" s="24" t="inlineStr">
         <is>
           <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
         </is>
       </c>
-      <c r="D75" s="25" t="n"/>
-      <c r="E75" s="26" t="n"/>
-    </row>
-    <row r="76" ht="64" customHeight="1">
-      <c r="B76" s="27" t="inlineStr">
+      <c r="D76" s="25" t="n"/>
+      <c r="E76" s="26" t="n"/>
+    </row>
+    <row r="77" ht="20.5" customHeight="1">
+      <c r="B77" s="27" t="inlineStr">
+        <is>
+          <t>Mantenimiento</t>
+        </is>
+      </c>
+      <c r="C77" s="28" t="inlineStr">
+        <is>
+          <t>US$ 25 anual</t>
+        </is>
+      </c>
+      <c r="D77" s="29" t="n"/>
+      <c r="E77" s="30" t="n"/>
+    </row>
+    <row r="78" ht="64" customHeight="1">
+      <c r="B78" s="23" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C76" s="28" t="inlineStr">
+      <c r="C78" s="24" t="inlineStr">
         <is>
           <t>• Inhumación de hasta 4 urnas
 • Tapa de granito grabada para cada espacio
@@ -2057,208 +2086,180 @@
 • Lugar físico permanente de homenaje familiar, sin plazo</t>
         </is>
       </c>
-      <c r="D76" s="29" t="n"/>
-      <c r="E76" s="30" t="n"/>
-    </row>
-    <row r="77" ht="20" customHeight="1">
-      <c r="B77" s="20" t="inlineStr">
-        <is>
-          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
-        </is>
-      </c>
-      <c r="C77" s="21" t="n"/>
-      <c r="D77" s="21" t="n"/>
-      <c r="E77" s="22" t="n"/>
-    </row>
-    <row r="78" ht="26.5" customHeight="1">
-      <c r="B78" s="23" t="inlineStr">
-        <is>
-          <t>Precio sugerido</t>
-        </is>
-      </c>
-      <c r="C78" s="31" t="inlineStr">
-        <is>
-          <t>US$ 2.000</t>
-        </is>
-      </c>
       <c r="D78" s="25" t="n"/>
       <c r="E78" s="26" t="n"/>
     </row>
-    <row r="79" ht="20.5" customHeight="1">
-      <c r="B79" s="27" t="inlineStr">
-        <is>
-          <t>Base de precio</t>
-        </is>
-      </c>
-      <c r="C79" s="28" t="inlineStr">
-        <is>
-          <t>Por parcela familiar · hasta 4 espacios</t>
-        </is>
-      </c>
-      <c r="D79" s="29" t="n"/>
-      <c r="E79" s="30" t="n"/>
-    </row>
-    <row r="80" ht="20.5" customHeight="1">
+    <row r="79" ht="20" customHeight="1">
+      <c r="B79" s="20" t="inlineStr">
+        <is>
+          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
+        </is>
+      </c>
+      <c r="C79" s="21" t="n"/>
+      <c r="D79" s="21" t="n"/>
+      <c r="E79" s="22" t="n"/>
+    </row>
+    <row r="80" ht="26.5" customHeight="1">
       <c r="B80" s="23" t="inlineStr">
         <is>
-          <t>Condiciones</t>
-        </is>
-      </c>
-      <c r="C80" s="24" t="inlineStr">
-        <is>
-          <t>Pago único o financiado según política comercial vigente.</t>
+          <t>Precio sugerido</t>
+        </is>
+      </c>
+      <c r="C80" s="31" t="inlineStr">
+        <is>
+          <t>US$ 2.000</t>
         </is>
       </c>
       <c r="D80" s="25" t="n"/>
       <c r="E80" s="26" t="n"/>
     </row>
-    <row r="81" ht="20" customHeight="1">
-      <c r="B81" s="20" t="inlineStr">
+    <row r="81" ht="20.5" customHeight="1">
+      <c r="B81" s="27" t="inlineStr">
+        <is>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C81" s="28" t="inlineStr">
+        <is>
+          <t>Por parcela familiar · hasta 4 espacios · mantenimiento US$ 25/año</t>
+        </is>
+      </c>
+      <c r="D81" s="29" t="n"/>
+      <c r="E81" s="30" t="n"/>
+    </row>
+    <row r="82" ht="35" customHeight="1">
+      <c r="B82" s="23" t="inlineStr">
+        <is>
+          <t>Condiciones</t>
+        </is>
+      </c>
+      <c r="C82" s="24" t="inlineStr">
+        <is>
+          <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 25 anual.</t>
+        </is>
+      </c>
+      <c r="D82" s="25" t="n"/>
+      <c r="E82" s="26" t="n"/>
+    </row>
+    <row r="83" ht="20" customHeight="1">
+      <c r="B83" s="20" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C81" s="21" t="n"/>
-      <c r="D81" s="21" t="n"/>
-      <c r="E81" s="22" t="n"/>
-    </row>
-    <row r="82" ht="20.5" customHeight="1">
-      <c r="B82" s="32" t="inlineStr">
+      <c r="C83" s="21" t="n"/>
+      <c r="D83" s="21" t="n"/>
+      <c r="E83" s="22" t="n"/>
+    </row>
+    <row r="84" ht="20.5" customHeight="1">
+      <c r="B84" s="32" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C82" s="33" t="inlineStr">
+      <c r="C84" s="33" t="inlineStr">
         <is>
           <t>Familias que buscan un espacio propio y permanente para varias generaciones.</t>
         </is>
       </c>
-      <c r="D82" s="34" t="n"/>
-      <c r="E82" s="35" t="n"/>
-    </row>
-    <row r="85" ht="30" customHeight="1">
-      <c r="B85" s="14" t="inlineStr">
+      <c r="D84" s="34" t="n"/>
+      <c r="E84" s="35" t="n"/>
+    </row>
+    <row r="87" ht="30" customHeight="1">
+      <c r="B87" s="14" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · ECOLÓGICO</t>
         </is>
       </c>
-      <c r="C85" s="15" t="n"/>
-      <c r="D85" s="15" t="n"/>
-      <c r="E85" s="16" t="inlineStr">
+      <c r="C87" s="15" t="n"/>
+      <c r="D87" s="15" t="n"/>
+      <c r="E87" s="16" t="inlineStr">
         <is>
           <t>VG-CRE-03E</t>
         </is>
       </c>
     </row>
-    <row r="86" ht="20" customHeight="1">
-      <c r="B86" s="17" t="inlineStr">
+    <row r="88" ht="20" customHeight="1">
+      <c r="B88" s="17" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Jardín 2  ·  Destino final · Inhumación ecológica</t>
         </is>
       </c>
-      <c r="C86" s="18" t="n"/>
-      <c r="D86" s="18" t="n"/>
-      <c r="E86" s="19" t="n"/>
-    </row>
-    <row r="87" ht="20" customHeight="1">
-      <c r="B87" s="20" t="inlineStr">
+      <c r="C88" s="18" t="n"/>
+      <c r="D88" s="18" t="n"/>
+      <c r="E88" s="19" t="n"/>
+    </row>
+    <row r="89" ht="20" customHeight="1">
+      <c r="B89" s="20" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C87" s="21" t="n"/>
-      <c r="D87" s="21" t="n"/>
-      <c r="E87" s="22" t="n"/>
-    </row>
-    <row r="88" ht="49.5" customHeight="1">
-      <c r="B88" s="23" t="inlineStr">
+      <c r="C89" s="21" t="n"/>
+      <c r="D89" s="21" t="n"/>
+      <c r="E89" s="22" t="n"/>
+    </row>
+    <row r="90" ht="49.5" customHeight="1">
+      <c r="B90" s="23" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C88" s="24" t="inlineStr">
+      <c r="C90" s="24" t="inlineStr">
         <is>
           <t>La urna biodegradable se entierra directamente en el suelo, se cubre con tierra y se descompone integrándose a la naturaleza. Jardín con agua corriente y área de esparcimiento de cenizas.</t>
         </is>
       </c>
-      <c r="D88" s="25" t="n"/>
-      <c r="E88" s="26" t="n"/>
-    </row>
-    <row r="89" ht="20.5" customHeight="1">
-      <c r="B89" s="27" t="inlineStr">
+      <c r="D90" s="25" t="n"/>
+      <c r="E90" s="26" t="n"/>
+    </row>
+    <row r="91" ht="20.5" customHeight="1">
+      <c r="B91" s="27" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C89" s="28" t="inlineStr">
+      <c r="C91" s="28" t="inlineStr">
         <is>
           <t>Individual (1 urna).</t>
         </is>
       </c>
-      <c r="D89" s="29" t="n"/>
-      <c r="E89" s="30" t="n"/>
-    </row>
-    <row r="90" ht="20" customHeight="1">
-      <c r="B90" s="20" t="inlineStr">
+      <c r="D91" s="29" t="n"/>
+      <c r="E91" s="30" t="n"/>
+    </row>
+    <row r="92" ht="20" customHeight="1">
+      <c r="B92" s="20" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C90" s="21" t="n"/>
-      <c r="D90" s="21" t="n"/>
-      <c r="E90" s="22" t="n"/>
-    </row>
-    <row r="91" ht="20.5" customHeight="1">
-      <c r="B91" s="23" t="inlineStr">
-        <is>
-          <t>Ambientes</t>
-        </is>
-      </c>
-      <c r="C91" s="24" t="inlineStr">
-        <is>
-          <t>Jardín 2 · Ecológico o Bosque de las Orquídeas</t>
-        </is>
-      </c>
-      <c r="D91" s="25" t="n"/>
-      <c r="E91" s="26" t="n"/>
-    </row>
-    <row r="92" ht="20.5" customHeight="1">
-      <c r="B92" s="27" t="inlineStr">
-        <is>
-          <t>Espacio por urna</t>
-        </is>
-      </c>
-      <c r="C92" s="28" t="inlineStr">
-        <is>
-          <t>30 × 30 cm, 40 cm de profundidad</t>
-        </is>
-      </c>
-      <c r="D92" s="29" t="n"/>
-      <c r="E92" s="30" t="n"/>
+      <c r="C92" s="21" t="n"/>
+      <c r="D92" s="21" t="n"/>
+      <c r="E92" s="22" t="n"/>
     </row>
     <row r="93" ht="20.5" customHeight="1">
       <c r="B93" s="23" t="inlineStr">
         <is>
-          <t>Urna</t>
+          <t>Ambientes</t>
         </is>
       </c>
       <c r="C93" s="24" t="inlineStr">
         <is>
-          <t>Biodegradable; se integra al suelo</t>
+          <t>Jardín 2 · Ecológico o Bosque de las Orquídeas</t>
         </is>
       </c>
       <c r="D93" s="25" t="n"/>
       <c r="E93" s="26" t="n"/>
     </row>
-    <row r="94" ht="35" customHeight="1">
+    <row r="94" ht="20.5" customHeight="1">
       <c r="B94" s="27" t="inlineStr">
         <is>
-          <t>Identificación (Jardín 2)</t>
+          <t>Espacio por urna</t>
         </is>
       </c>
       <c r="C94" s="28" t="inlineStr">
         <is>
-          <t>Placa de madera de 20 cm fijada a una varilla metálica, en posición vertical y sin contacto con el suelo</t>
+          <t>30 × 30 cm, 40 cm de profundidad</t>
         </is>
       </c>
       <c r="D94" s="29" t="n"/>
@@ -2267,95 +2268,100 @@
     <row r="95" ht="20.5" customHeight="1">
       <c r="B95" s="23" t="inlineStr">
         <is>
-          <t>Identificación (Bosque)</t>
+          <t>Urna</t>
         </is>
       </c>
       <c r="C95" s="24" t="inlineStr">
         <is>
-          <t>Placa de mármol de 20 × 15 cm</t>
+          <t>Biodegradable; se integra al suelo</t>
         </is>
       </c>
       <c r="D95" s="25" t="n"/>
       <c r="E95" s="26" t="n"/>
     </row>
-    <row r="96" ht="20.5" customHeight="1">
+    <row r="96" ht="35" customHeight="1">
       <c r="B96" s="27" t="inlineStr">
         <is>
-          <t>Acceso</t>
+          <t>Identificación (Jardín 2)</t>
         </is>
       </c>
       <c r="C96" s="28" t="inlineStr">
         <is>
-          <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
+          <t>Placa de madera de 20 cm fijada a una varilla metálica, en posición vertical y sin contacto con el suelo</t>
         </is>
       </c>
       <c r="D96" s="29" t="n"/>
       <c r="E96" s="30" t="n"/>
     </row>
-    <row r="97" ht="64" customHeight="1">
+    <row r="97" ht="20.5" customHeight="1">
       <c r="B97" s="23" t="inlineStr">
         <is>
+          <t>Identificación (Bosque)</t>
+        </is>
+      </c>
+      <c r="C97" s="24" t="inlineStr">
+        <is>
+          <t>Placa de mármol de 20 × 15 cm</t>
+        </is>
+      </c>
+      <c r="D97" s="25" t="n"/>
+      <c r="E97" s="26" t="n"/>
+    </row>
+    <row r="98" ht="35" customHeight="1">
+      <c r="B98" s="27" t="inlineStr">
+        <is>
+          <t>Permanencia</t>
+        </is>
+      </c>
+      <c r="C98" s="28" t="inlineStr">
+        <is>
+          <t>3 años; luego el nombre pasa a una placa memorial en el monumento y el espacio se reutiliza</t>
+        </is>
+      </c>
+      <c r="D98" s="29" t="n"/>
+      <c r="E98" s="30" t="n"/>
+    </row>
+    <row r="99" ht="20.5" customHeight="1">
+      <c r="B99" s="23" t="inlineStr">
+        <is>
+          <t>Placa memorial</t>
+        </is>
+      </c>
+      <c r="C99" s="24" t="inlineStr">
+        <is>
+          <t>US$ 150</t>
+        </is>
+      </c>
+      <c r="D99" s="25" t="n"/>
+      <c r="E99" s="26" t="n"/>
+    </row>
+    <row r="100" ht="20.5" customHeight="1">
+      <c r="B100" s="27" t="inlineStr">
+        <is>
+          <t>Acceso</t>
+        </is>
+      </c>
+      <c r="C100" s="28" t="inlineStr">
+        <is>
+          <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
+        </is>
+      </c>
+      <c r="D100" s="29" t="n"/>
+      <c r="E100" s="30" t="n"/>
+    </row>
+    <row r="101" ht="78.5" customHeight="1">
+      <c r="B101" s="23" t="inlineStr">
+        <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C97" s="24" t="inlineStr">
+      <c r="C101" s="24" t="inlineStr">
         <is>
           <t>• Inhumación ecológica de la urna directamente en el suelo
 • Placa de identificación
 • Ubicación en el Jardín 2 o en el Bosque de las Orquídeas
-• Entorno natural con agua corriente</t>
-        </is>
-      </c>
-      <c r="D97" s="25" t="n"/>
-      <c r="E97" s="26" t="n"/>
-    </row>
-    <row r="98" ht="20" customHeight="1">
-      <c r="B98" s="20" t="inlineStr">
-        <is>
-          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
-        </is>
-      </c>
-      <c r="C98" s="21" t="n"/>
-      <c r="D98" s="21" t="n"/>
-      <c r="E98" s="22" t="n"/>
-    </row>
-    <row r="99" ht="26.5" customHeight="1">
-      <c r="B99" s="23" t="inlineStr">
-        <is>
-          <t>Precio sugerido</t>
-        </is>
-      </c>
-      <c r="C99" s="31" t="inlineStr">
-        <is>
-          <t>US$ 600</t>
-        </is>
-      </c>
-      <c r="D99" s="25" t="n"/>
-      <c r="E99" s="26" t="n"/>
-    </row>
-    <row r="100" ht="20.5" customHeight="1">
-      <c r="B100" s="27" t="inlineStr">
-        <is>
-          <t>Base de precio</t>
-        </is>
-      </c>
-      <c r="C100" s="28" t="inlineStr">
-        <is>
-          <t>Por espacio individual</t>
-        </is>
-      </c>
-      <c r="D100" s="29" t="n"/>
-      <c r="E100" s="30" t="n"/>
-    </row>
-    <row r="101" ht="20.5" customHeight="1">
-      <c r="B101" s="23" t="inlineStr">
-        <is>
-          <t>Condiciones</t>
-        </is>
-      </c>
-      <c r="C101" s="24" t="inlineStr">
-        <is>
-          <t>Pago único o financiado según política comercial vigente.</t>
+• Entorno natural con agua corriente
+• Permanencia de 3 años; luego, placa memorial en el monumento</t>
         </is>
       </c>
       <c r="D101" s="25" t="n"/>
@@ -2364,607 +2370,678 @@
     <row r="102" ht="20" customHeight="1">
       <c r="B102" s="20" t="inlineStr">
         <is>
-          <t>PERFIL DEL COMPRADOR</t>
+          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
       <c r="C102" s="21" t="n"/>
       <c r="D102" s="21" t="n"/>
       <c r="E102" s="22" t="n"/>
     </row>
-    <row r="103" ht="35" customHeight="1">
-      <c r="B103" s="32" t="inlineStr">
+    <row r="103" ht="26.5" customHeight="1">
+      <c r="B103" s="23" t="inlineStr">
+        <is>
+          <t>Precio sugerido</t>
+        </is>
+      </c>
+      <c r="C103" s="31" t="inlineStr">
+        <is>
+          <t>US$ 600</t>
+        </is>
+      </c>
+      <c r="D103" s="25" t="n"/>
+      <c r="E103" s="26" t="n"/>
+    </row>
+    <row r="104" ht="20.5" customHeight="1">
+      <c r="B104" s="27" t="inlineStr">
+        <is>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C104" s="28" t="inlineStr">
+        <is>
+          <t>Por espacio individual · placa memorial US$ 150</t>
+        </is>
+      </c>
+      <c r="D104" s="29" t="n"/>
+      <c r="E104" s="30" t="n"/>
+    </row>
+    <row r="105" ht="35" customHeight="1">
+      <c r="B105" s="23" t="inlineStr">
+        <is>
+          <t>Condiciones</t>
+        </is>
+      </c>
+      <c r="C105" s="24" t="inlineStr">
+        <is>
+          <t>Pago único o financiado según política comercial vigente. Placa memorial en el monumento al término del plazo: US$ 150.</t>
+        </is>
+      </c>
+      <c r="D105" s="25" t="n"/>
+      <c r="E105" s="26" t="n"/>
+    </row>
+    <row r="106" ht="20" customHeight="1">
+      <c r="B106" s="20" t="inlineStr">
+        <is>
+          <t>PERFIL DEL COMPRADOR</t>
+        </is>
+      </c>
+      <c r="C106" s="21" t="n"/>
+      <c r="D106" s="21" t="n"/>
+      <c r="E106" s="22" t="n"/>
+    </row>
+    <row r="107" ht="35" customHeight="1">
+      <c r="B107" s="32" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C103" s="33" t="inlineStr">
+      <c r="C107" s="33" t="inlineStr">
         <is>
           <t>Personas con conciencia ambiental que desean que sus cenizas vuelvan a la tierra, con un lugar identificado para visitar.</t>
         </is>
       </c>
-      <c r="D103" s="34" t="n"/>
-      <c r="E103" s="35" t="n"/>
-    </row>
-    <row r="106" ht="30" customHeight="1">
-      <c r="B106" s="14" t="inlineStr">
+      <c r="D107" s="34" t="n"/>
+      <c r="E107" s="35" t="n"/>
+    </row>
+    <row r="110" ht="30" customHeight="1">
+      <c r="B110" s="14" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · CEREMONIAL</t>
         </is>
       </c>
-      <c r="C106" s="15" t="n"/>
-      <c r="D106" s="15" t="n"/>
-      <c r="E106" s="16" t="inlineStr">
+      <c r="C110" s="15" t="n"/>
+      <c r="D110" s="15" t="n"/>
+      <c r="E110" s="16" t="inlineStr">
         <is>
           <t>VG-CRE-03C</t>
         </is>
       </c>
     </row>
-    <row r="107" ht="20" customHeight="1">
-      <c r="B107" s="17" t="inlineStr">
+    <row r="111" ht="20" customHeight="1">
+      <c r="B111" s="17" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Jardín 3  ·  Destino final · Inhumación con ceremonia</t>
         </is>
       </c>
-      <c r="C107" s="18" t="n"/>
-      <c r="D107" s="18" t="n"/>
-      <c r="E107" s="19" t="n"/>
-    </row>
-    <row r="108" ht="20" customHeight="1">
-      <c r="B108" s="20" t="inlineStr">
+      <c r="C111" s="18" t="n"/>
+      <c r="D111" s="18" t="n"/>
+      <c r="E111" s="19" t="n"/>
+    </row>
+    <row r="112" ht="20" customHeight="1">
+      <c r="B112" s="20" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C108" s="21" t="n"/>
-      <c r="D108" s="21" t="n"/>
-      <c r="E108" s="22" t="n"/>
-    </row>
-    <row r="109" ht="35" customHeight="1">
-      <c r="B109" s="23" t="inlineStr">
+      <c r="C112" s="21" t="n"/>
+      <c r="D112" s="21" t="n"/>
+      <c r="E112" s="22" t="n"/>
+    </row>
+    <row r="113" ht="35" customHeight="1">
+      <c r="B113" s="23" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C109" s="24" t="inlineStr">
+      <c r="C113" s="24" t="inlineStr">
         <is>
           <t>Jardín para inhumación de urnas de cenizas con ceremonia de agua, con fuentes como elemento central del rito de despedida.</t>
         </is>
       </c>
-      <c r="D109" s="25" t="n"/>
-      <c r="E109" s="26" t="n"/>
-    </row>
-    <row r="110" ht="20.5" customHeight="1">
-      <c r="B110" s="27" t="inlineStr">
+      <c r="D113" s="25" t="n"/>
+      <c r="E113" s="26" t="n"/>
+    </row>
+    <row r="114" ht="20.5" customHeight="1">
+      <c r="B114" s="27" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C110" s="28" t="inlineStr">
+      <c r="C114" s="28" t="inlineStr">
         <is>
           <t>A definir.</t>
         </is>
       </c>
-      <c r="D110" s="29" t="n"/>
-      <c r="E110" s="30" t="n"/>
-    </row>
-    <row r="111" ht="20" customHeight="1">
-      <c r="B111" s="20" t="inlineStr">
+      <c r="D114" s="29" t="n"/>
+      <c r="E114" s="30" t="n"/>
+    </row>
+    <row r="115" ht="20" customHeight="1">
+      <c r="B115" s="20" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C111" s="21" t="n"/>
-      <c r="D111" s="21" t="n"/>
-      <c r="E111" s="22" t="n"/>
-    </row>
-    <row r="112" ht="20.5" customHeight="1">
-      <c r="B112" s="23" t="inlineStr">
+      <c r="C115" s="21" t="n"/>
+      <c r="D115" s="21" t="n"/>
+      <c r="E115" s="22" t="n"/>
+    </row>
+    <row r="116" ht="20.5" customHeight="1">
+      <c r="B116" s="23" t="inlineStr">
         <is>
           <t>Ambiente</t>
         </is>
       </c>
-      <c r="C112" s="24" t="inlineStr">
+      <c r="C116" s="24" t="inlineStr">
         <is>
           <t>Jardín 3</t>
         </is>
       </c>
-      <c r="D112" s="25" t="n"/>
-      <c r="E112" s="26" t="n"/>
-    </row>
-    <row r="113" ht="20.5" customHeight="1">
-      <c r="B113" s="27" t="inlineStr">
+      <c r="D116" s="25" t="n"/>
+      <c r="E116" s="26" t="n"/>
+    </row>
+    <row r="117" ht="20.5" customHeight="1">
+      <c r="B117" s="27" t="inlineStr">
         <is>
           <t>Elemento central</t>
         </is>
       </c>
-      <c r="C113" s="28" t="inlineStr">
+      <c r="C117" s="28" t="inlineStr">
         <is>
           <t>Fuente de agua para la ceremonia</t>
         </is>
       </c>
-      <c r="D113" s="29" t="n"/>
-      <c r="E113" s="30" t="n"/>
-    </row>
-    <row r="114" ht="20.5" customHeight="1">
-      <c r="B114" s="23" t="inlineStr">
+      <c r="D117" s="29" t="n"/>
+      <c r="E117" s="30" t="n"/>
+    </row>
+    <row r="118" ht="20.5" customHeight="1">
+      <c r="B118" s="23" t="inlineStr">
         <is>
           <t>Entorno</t>
         </is>
       </c>
-      <c r="C114" s="24" t="inlineStr">
+      <c r="C118" s="24" t="inlineStr">
         <is>
           <t>Barrera visual que separa el jardín del crematorio</t>
         </is>
       </c>
-      <c r="D114" s="25" t="n"/>
-      <c r="E114" s="26" t="n"/>
-    </row>
-    <row r="115" ht="35" customHeight="1">
-      <c r="B115" s="27" t="inlineStr">
+      <c r="D118" s="25" t="n"/>
+      <c r="E118" s="26" t="n"/>
+    </row>
+    <row r="119" ht="35" customHeight="1">
+      <c r="B119" s="27" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C115" s="28" t="inlineStr">
+      <c r="C119" s="28" t="inlineStr">
         <is>
           <t>• Inhumación de urnas de cenizas
 • Ceremonia con agua en fuente</t>
         </is>
       </c>
-      <c r="D115" s="29" t="n"/>
-      <c r="E115" s="30" t="n"/>
-    </row>
-    <row r="116" ht="20" customHeight="1">
-      <c r="B116" s="20" t="inlineStr">
-        <is>
-          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
-        </is>
-      </c>
-      <c r="C116" s="21" t="n"/>
-      <c r="D116" s="21" t="n"/>
-      <c r="E116" s="22" t="n"/>
-    </row>
-    <row r="117" ht="26.5" customHeight="1">
-      <c r="B117" s="23" t="inlineStr">
-        <is>
-          <t>Precio sugerido</t>
-        </is>
-      </c>
-      <c r="C117" s="31" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-      <c r="D117" s="25" t="n"/>
-      <c r="E117" s="26" t="n"/>
-    </row>
-    <row r="118" ht="20.5" customHeight="1">
-      <c r="B118" s="27" t="inlineStr">
-        <is>
-          <t>Base de precio</t>
-        </is>
-      </c>
-      <c r="C118" s="28" t="inlineStr">
-        <is>
-          <t>Producto en definición</t>
-        </is>
-      </c>
-      <c r="D118" s="29" t="n"/>
-      <c r="E118" s="30" t="n"/>
-    </row>
-    <row r="119" ht="20.5" customHeight="1">
-      <c r="B119" s="23" t="inlineStr">
-        <is>
-          <t>Condiciones</t>
-        </is>
-      </c>
-      <c r="C119" s="24" t="inlineStr">
-        <is>
-          <t>A definir.</t>
-        </is>
-      </c>
-      <c r="D119" s="25" t="n"/>
-      <c r="E119" s="26" t="n"/>
+      <c r="D119" s="29" t="n"/>
+      <c r="E119" s="30" t="n"/>
     </row>
     <row r="120" ht="20" customHeight="1">
       <c r="B120" s="20" t="inlineStr">
         <is>
-          <t>PERFIL DEL COMPRADOR</t>
+          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
       <c r="C120" s="21" t="n"/>
       <c r="D120" s="21" t="n"/>
       <c r="E120" s="22" t="n"/>
     </row>
-    <row r="121" ht="35" customHeight="1">
-      <c r="B121" s="32" t="inlineStr">
+    <row r="121" ht="26.5" customHeight="1">
+      <c r="B121" s="23" t="inlineStr">
+        <is>
+          <t>Precio sugerido</t>
+        </is>
+      </c>
+      <c r="C121" s="31" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="D121" s="25" t="n"/>
+      <c r="E121" s="26" t="n"/>
+    </row>
+    <row r="122" ht="20.5" customHeight="1">
+      <c r="B122" s="27" t="inlineStr">
+        <is>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C122" s="28" t="inlineStr">
+        <is>
+          <t>Producto en definición</t>
+        </is>
+      </c>
+      <c r="D122" s="29" t="n"/>
+      <c r="E122" s="30" t="n"/>
+    </row>
+    <row r="123" ht="20.5" customHeight="1">
+      <c r="B123" s="23" t="inlineStr">
+        <is>
+          <t>Condiciones</t>
+        </is>
+      </c>
+      <c r="C123" s="24" t="inlineStr">
+        <is>
+          <t>A definir.</t>
+        </is>
+      </c>
+      <c r="D123" s="25" t="n"/>
+      <c r="E123" s="26" t="n"/>
+    </row>
+    <row r="124" ht="20" customHeight="1">
+      <c r="B124" s="20" t="inlineStr">
+        <is>
+          <t>PERFIL DEL COMPRADOR</t>
+        </is>
+      </c>
+      <c r="C124" s="21" t="n"/>
+      <c r="D124" s="21" t="n"/>
+      <c r="E124" s="22" t="n"/>
+    </row>
+    <row r="125" ht="35" customHeight="1">
+      <c r="B125" s="32" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C121" s="33" t="inlineStr">
+      <c r="C125" s="33" t="inlineStr">
         <is>
           <t>Familias que valoran un rito de despedida simbólico y un entorno contemplativo.</t>
         </is>
       </c>
-      <c r="D121" s="34" t="n"/>
-      <c r="E121" s="35" t="n"/>
-    </row>
-    <row r="124" ht="30" customHeight="1">
-      <c r="B124" s="14" t="inlineStr">
+      <c r="D125" s="34" t="n"/>
+      <c r="E125" s="35" t="n"/>
+    </row>
+    <row r="128" ht="30" customHeight="1">
+      <c r="B128" s="14" t="inlineStr">
         <is>
           <t>JARDÍN DE MASCOTAS</t>
         </is>
       </c>
-      <c r="C124" s="15" t="n"/>
-      <c r="D124" s="15" t="n"/>
-      <c r="E124" s="16" t="inlineStr">
+      <c r="C128" s="15" t="n"/>
+      <c r="D128" s="15" t="n"/>
+      <c r="E128" s="16" t="inlineStr">
         <is>
           <t>VG-CRE-04</t>
         </is>
       </c>
     </row>
-    <row r="125" ht="20" customHeight="1">
-      <c r="B125" s="17" t="inlineStr">
+    <row r="129" ht="20" customHeight="1">
+      <c r="B129" s="17" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Mascotas  ·  Mascotas · Inhumación ecológica</t>
         </is>
       </c>
-      <c r="C125" s="18" t="n"/>
-      <c r="D125" s="18" t="n"/>
-      <c r="E125" s="19" t="n"/>
-    </row>
-    <row r="126" ht="20" customHeight="1">
-      <c r="B126" s="20" t="inlineStr">
+      <c r="C129" s="18" t="n"/>
+      <c r="D129" s="18" t="n"/>
+      <c r="E129" s="19" t="n"/>
+    </row>
+    <row r="130" ht="20" customHeight="1">
+      <c r="B130" s="20" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C126" s="21" t="n"/>
-      <c r="D126" s="21" t="n"/>
-      <c r="E126" s="22" t="n"/>
-    </row>
-    <row r="127" ht="35" customHeight="1">
-      <c r="B127" s="23" t="inlineStr">
+      <c r="C130" s="21" t="n"/>
+      <c r="D130" s="21" t="n"/>
+      <c r="E130" s="22" t="n"/>
+    </row>
+    <row r="131" ht="35" customHeight="1">
+      <c r="B131" s="23" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C127" s="24" t="inlineStr">
+      <c r="C131" s="24" t="inlineStr">
         <is>
           <t>Jardín para inhumación ecológica de cenizas de mascotas: la urna biodegradable se entierra directamente en el suelo y se identifica con una placa de madera.</t>
         </is>
       </c>
-      <c r="D127" s="25" t="n"/>
-      <c r="E127" s="26" t="n"/>
-    </row>
-    <row r="128" ht="20.5" customHeight="1">
-      <c r="B128" s="27" t="inlineStr">
+      <c r="D131" s="25" t="n"/>
+      <c r="E131" s="26" t="n"/>
+    </row>
+    <row r="132" ht="20.5" customHeight="1">
+      <c r="B132" s="27" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C128" s="28" t="inlineStr">
+      <c r="C132" s="28" t="inlineStr">
         <is>
           <t>Individual (una mascota por servicio).</t>
         </is>
       </c>
-      <c r="D128" s="29" t="n"/>
-      <c r="E128" s="30" t="n"/>
-    </row>
-    <row r="129" ht="20" customHeight="1">
-      <c r="B129" s="20" t="inlineStr">
+      <c r="D132" s="29" t="n"/>
+      <c r="E132" s="30" t="n"/>
+    </row>
+    <row r="133" ht="20" customHeight="1">
+      <c r="B133" s="20" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C129" s="21" t="n"/>
-      <c r="D129" s="21" t="n"/>
-      <c r="E129" s="22" t="n"/>
-    </row>
-    <row r="130" ht="20.5" customHeight="1">
-      <c r="B130" s="23" t="inlineStr">
-        <is>
-          <t>Tipo de producto</t>
-        </is>
-      </c>
-      <c r="C130" s="24" t="inlineStr">
-        <is>
-          <t>Servicio de pago único</t>
-        </is>
-      </c>
-      <c r="D130" s="25" t="n"/>
-      <c r="E130" s="26" t="n"/>
-    </row>
-    <row r="131" ht="20.5" customHeight="1">
-      <c r="B131" s="27" t="inlineStr">
-        <is>
-          <t>Espacio por urna</t>
-        </is>
-      </c>
-      <c r="C131" s="28" t="inlineStr">
-        <is>
-          <t>15 × 20 cm o 15 × 30 cm, según el tamaño de la urna</t>
-        </is>
-      </c>
-      <c r="D131" s="29" t="n"/>
-      <c r="E131" s="30" t="n"/>
-    </row>
-    <row r="132" ht="20.5" customHeight="1">
-      <c r="B132" s="23" t="inlineStr">
-        <is>
-          <t>Urna</t>
-        </is>
-      </c>
-      <c r="C132" s="24" t="inlineStr">
-        <is>
-          <t>Biodegradable; se integra al suelo</t>
-        </is>
-      </c>
-      <c r="D132" s="25" t="n"/>
-      <c r="E132" s="26" t="n"/>
-    </row>
-    <row r="133" ht="20.5" customHeight="1">
-      <c r="B133" s="27" t="inlineStr">
-        <is>
-          <t>Identificación</t>
-        </is>
-      </c>
-      <c r="C133" s="28" t="inlineStr">
-        <is>
-          <t>Placa de madera de 20 cm</t>
-        </is>
-      </c>
-      <c r="D133" s="29" t="n"/>
-      <c r="E133" s="30" t="n"/>
+      <c r="C133" s="21" t="n"/>
+      <c r="D133" s="21" t="n"/>
+      <c r="E133" s="22" t="n"/>
     </row>
     <row r="134" ht="20.5" customHeight="1">
       <c r="B134" s="23" t="inlineStr">
         <is>
-          <t>Homenaje</t>
+          <t>Tipo de producto</t>
         </is>
       </c>
       <c r="C134" s="24" t="inlineStr">
         <is>
-          <t>Placa conmemorativa colectiva en el jardín</t>
+          <t>Servicio de pago único</t>
         </is>
       </c>
       <c r="D134" s="25" t="n"/>
       <c r="E134" s="26" t="n"/>
     </row>
-    <row r="135" ht="64" customHeight="1">
+    <row r="135" ht="20.5" customHeight="1">
       <c r="B135" s="27" t="inlineStr">
         <is>
+          <t>Espacio por urna</t>
+        </is>
+      </c>
+      <c r="C135" s="28" t="inlineStr">
+        <is>
+          <t>15 × 20 cm o 15 × 30 cm, según el tamaño de la urna</t>
+        </is>
+      </c>
+      <c r="D135" s="29" t="n"/>
+      <c r="E135" s="30" t="n"/>
+    </row>
+    <row r="136" ht="20.5" customHeight="1">
+      <c r="B136" s="23" t="inlineStr">
+        <is>
+          <t>Urna</t>
+        </is>
+      </c>
+      <c r="C136" s="24" t="inlineStr">
+        <is>
+          <t>Biodegradable; se integra al suelo</t>
+        </is>
+      </c>
+      <c r="D136" s="25" t="n"/>
+      <c r="E136" s="26" t="n"/>
+    </row>
+    <row r="137" ht="20.5" customHeight="1">
+      <c r="B137" s="27" t="inlineStr">
+        <is>
+          <t>Identificación</t>
+        </is>
+      </c>
+      <c r="C137" s="28" t="inlineStr">
+        <is>
+          <t>Placa de madera de 20 cm</t>
+        </is>
+      </c>
+      <c r="D137" s="29" t="n"/>
+      <c r="E137" s="30" t="n"/>
+    </row>
+    <row r="138" ht="35" customHeight="1">
+      <c r="B138" s="23" t="inlineStr">
+        <is>
+          <t>Permanencia</t>
+        </is>
+      </c>
+      <c r="C138" s="24" t="inlineStr">
+        <is>
+          <t>3 años; luego el nombre pasa a una placa memorial en el monumento y el espacio se reutiliza</t>
+        </is>
+      </c>
+      <c r="D138" s="25" t="n"/>
+      <c r="E138" s="26" t="n"/>
+    </row>
+    <row r="139" ht="20.5" customHeight="1">
+      <c r="B139" s="27" t="inlineStr">
+        <is>
+          <t>Placa memorial</t>
+        </is>
+      </c>
+      <c r="C139" s="28" t="inlineStr">
+        <is>
+          <t>US$ 50</t>
+        </is>
+      </c>
+      <c r="D139" s="29" t="n"/>
+      <c r="E139" s="30" t="n"/>
+    </row>
+    <row r="140" ht="64" customHeight="1">
+      <c r="B140" s="23" t="inlineStr">
+        <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C135" s="28" t="inlineStr">
+      <c r="C140" s="24" t="inlineStr">
         <is>
           <t>• Inhumación ecológica de la urna en el jardín
 • Placa de madera de 20 cm para identificación
-• Nombre de la mascota en la placa conmemorativa del jardín
+• Permanencia de 3 años; luego, placa memorial en el monumento
 • Cremación de la mascota (opción Jardín + Cremación)</t>
         </is>
       </c>
-      <c r="D135" s="29" t="n"/>
-      <c r="E135" s="30" t="n"/>
-    </row>
-    <row r="136" ht="20" customHeight="1">
-      <c r="B136" s="20" t="inlineStr">
+      <c r="D140" s="25" t="n"/>
+      <c r="E140" s="26" t="n"/>
+    </row>
+    <row r="141" ht="20" customHeight="1">
+      <c r="B141" s="20" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C136" s="21" t="n"/>
-      <c r="D136" s="21" t="n"/>
-      <c r="E136" s="22" t="n"/>
-    </row>
-    <row r="137" ht="26.5" customHeight="1">
-      <c r="B137" s="23" t="inlineStr">
+      <c r="C141" s="21" t="n"/>
+      <c r="D141" s="21" t="n"/>
+      <c r="E141" s="22" t="n"/>
+    </row>
+    <row r="142" ht="26.5" customHeight="1">
+      <c r="B142" s="23" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C137" s="31" t="inlineStr">
+      <c r="C142" s="31" t="inlineStr">
         <is>
           <t>US$ 350 / US$ 500</t>
         </is>
       </c>
-      <c r="D137" s="25" t="n"/>
-      <c r="E137" s="26" t="n"/>
-    </row>
-    <row r="138" ht="20.5" customHeight="1">
-      <c r="B138" s="27" t="inlineStr">
+      <c r="D142" s="25" t="n"/>
+      <c r="E142" s="26" t="n"/>
+    </row>
+    <row r="143" ht="20.5" customHeight="1">
+      <c r="B143" s="27" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C138" s="28" t="inlineStr">
+      <c r="C143" s="28" t="inlineStr">
         <is>
           <t>US$ 350 solo jardín · US$ 500 jardín + cremación</t>
         </is>
       </c>
-      <c r="D138" s="29" t="n"/>
-      <c r="E138" s="30" t="n"/>
-    </row>
-    <row r="139" ht="20.5" customHeight="1">
-      <c r="B139" s="23" t="inlineStr">
+      <c r="D143" s="29" t="n"/>
+      <c r="E143" s="30" t="n"/>
+    </row>
+    <row r="144" ht="35" customHeight="1">
+      <c r="B144" s="23" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C139" s="24" t="inlineStr">
-        <is>
-          <t>Pago único; puede contratarse como adicional al plan funerario.</t>
-        </is>
-      </c>
-      <c r="D139" s="25" t="n"/>
-      <c r="E139" s="26" t="n"/>
-    </row>
-    <row r="140" ht="20" customHeight="1">
-      <c r="B140" s="20" t="inlineStr">
+      <c r="C144" s="24" t="inlineStr">
+        <is>
+          <t>Pago único; puede contratarse como adicional al plan funerario. Placa memorial en el monumento al término del plazo: US$ 50.</t>
+        </is>
+      </c>
+      <c r="D144" s="25" t="n"/>
+      <c r="E144" s="26" t="n"/>
+    </row>
+    <row r="145" ht="20" customHeight="1">
+      <c r="B145" s="20" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C140" s="21" t="n"/>
-      <c r="D140" s="21" t="n"/>
-      <c r="E140" s="22" t="n"/>
-    </row>
-    <row r="141" ht="20.5" customHeight="1">
-      <c r="B141" s="32" t="inlineStr">
+      <c r="C145" s="21" t="n"/>
+      <c r="D145" s="21" t="n"/>
+      <c r="E145" s="22" t="n"/>
+    </row>
+    <row r="146" ht="20.5" customHeight="1">
+      <c r="B146" s="32" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C141" s="33" t="inlineStr">
+      <c r="C146" s="33" t="inlineStr">
         <is>
           <t>Familias que consideran a su mascota parte del hogar y desean un cierre digno.</t>
         </is>
       </c>
-      <c r="D141" s="34" t="n"/>
-      <c r="E141" s="35" t="n"/>
+      <c r="D146" s="34" t="n"/>
+      <c r="E146" s="35" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="128">
+  <mergeCells count="133">
+    <mergeCell ref="C142:E142"/>
     <mergeCell ref="C31:E31"/>
     <mergeCell ref="C80:E80"/>
+    <mergeCell ref="B68:E68"/>
     <mergeCell ref="C40:E40"/>
     <mergeCell ref="C51:E51"/>
     <mergeCell ref="C95:E95"/>
     <mergeCell ref="C60:E60"/>
-    <mergeCell ref="C71:E71"/>
+    <mergeCell ref="C123:E123"/>
     <mergeCell ref="B47:E47"/>
     <mergeCell ref="C7:E7"/>
     <mergeCell ref="C91:E91"/>
+    <mergeCell ref="B141:E141"/>
+    <mergeCell ref="B115:E115"/>
     <mergeCell ref="B102:E102"/>
+    <mergeCell ref="C57:E57"/>
+    <mergeCell ref="C140:E140"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="B21:E21"/>
     <mergeCell ref="C18:E18"/>
     <mergeCell ref="C49:E49"/>
-    <mergeCell ref="B86:E86"/>
     <mergeCell ref="C101:E101"/>
+    <mergeCell ref="C77:E77"/>
     <mergeCell ref="C34:E34"/>
-    <mergeCell ref="B136:E136"/>
     <mergeCell ref="C42:E42"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="C74:E74"/>
-    <mergeCell ref="C141:E141"/>
-    <mergeCell ref="B87:E87"/>
-    <mergeCell ref="C128:E128"/>
+    <mergeCell ref="B112:E112"/>
     <mergeCell ref="C20:E20"/>
     <mergeCell ref="C113:E113"/>
     <mergeCell ref="C103:E103"/>
-    <mergeCell ref="C112:E112"/>
+    <mergeCell ref="C143:E143"/>
     <mergeCell ref="C99:E99"/>
     <mergeCell ref="C94:E94"/>
     <mergeCell ref="C118:E118"/>
     <mergeCell ref="C75:E75"/>
-    <mergeCell ref="C133:E133"/>
+    <mergeCell ref="C84:E84"/>
     <mergeCell ref="C22:E22"/>
-    <mergeCell ref="C127:E127"/>
     <mergeCell ref="C114:E114"/>
     <mergeCell ref="C59:E59"/>
-    <mergeCell ref="C130:E130"/>
     <mergeCell ref="C12:E12"/>
     <mergeCell ref="B26:E26"/>
     <mergeCell ref="B41:E41"/>
     <mergeCell ref="B50:E50"/>
     <mergeCell ref="C52:E52"/>
+    <mergeCell ref="B106:E106"/>
     <mergeCell ref="B129:E129"/>
+    <mergeCell ref="C61:E61"/>
     <mergeCell ref="C39:E39"/>
     <mergeCell ref="B16:E16"/>
+    <mergeCell ref="C70:E70"/>
     <mergeCell ref="C48:E48"/>
-    <mergeCell ref="B90:E90"/>
     <mergeCell ref="C32:E32"/>
     <mergeCell ref="C38:E38"/>
-    <mergeCell ref="B66:E66"/>
-    <mergeCell ref="B124:D124"/>
+    <mergeCell ref="C81:E81"/>
+    <mergeCell ref="C125:E125"/>
     <mergeCell ref="B27:E27"/>
-    <mergeCell ref="B140:E140"/>
     <mergeCell ref="C13:E13"/>
     <mergeCell ref="B45:D45"/>
-    <mergeCell ref="B85:D85"/>
+    <mergeCell ref="B110:D110"/>
     <mergeCell ref="C131:E131"/>
-    <mergeCell ref="B77:E77"/>
+    <mergeCell ref="B130:E130"/>
     <mergeCell ref="C15:E15"/>
     <mergeCell ref="B67:E67"/>
-    <mergeCell ref="B61:E61"/>
     <mergeCell ref="C33:E33"/>
-    <mergeCell ref="C89:E89"/>
-    <mergeCell ref="C79:E79"/>
+    <mergeCell ref="C104:E104"/>
+    <mergeCell ref="C116:E116"/>
     <mergeCell ref="C73:E73"/>
-    <mergeCell ref="C88:E88"/>
-    <mergeCell ref="B116:E116"/>
     <mergeCell ref="B37:E37"/>
     <mergeCell ref="C35:E35"/>
+    <mergeCell ref="C63:E63"/>
     <mergeCell ref="C121:E121"/>
     <mergeCell ref="C10:E10"/>
     <mergeCell ref="C117:E117"/>
     <mergeCell ref="C55:E55"/>
     <mergeCell ref="B6:E6"/>
-    <mergeCell ref="C115:E115"/>
+    <mergeCell ref="B89:E89"/>
+    <mergeCell ref="B87:D87"/>
     <mergeCell ref="C36:E36"/>
     <mergeCell ref="C11:E11"/>
+    <mergeCell ref="B79:E79"/>
+    <mergeCell ref="B128:D128"/>
     <mergeCell ref="C135:E135"/>
-    <mergeCell ref="B65:D65"/>
-    <mergeCell ref="B81:E81"/>
+    <mergeCell ref="C144:E144"/>
+    <mergeCell ref="C122:E122"/>
     <mergeCell ref="C72:E72"/>
     <mergeCell ref="C28:E28"/>
+    <mergeCell ref="B71:E71"/>
+    <mergeCell ref="B58:E58"/>
     <mergeCell ref="C69:E69"/>
     <mergeCell ref="C96:E96"/>
     <mergeCell ref="C78:E78"/>
+    <mergeCell ref="C136:E136"/>
     <mergeCell ref="B120:E120"/>
     <mergeCell ref="B2:E2"/>
-    <mergeCell ref="C92:E92"/>
     <mergeCell ref="B25:D25"/>
-    <mergeCell ref="B107:E107"/>
-    <mergeCell ref="C62:E62"/>
     <mergeCell ref="C14:E14"/>
-    <mergeCell ref="B57:E57"/>
+    <mergeCell ref="B66:D66"/>
+    <mergeCell ref="C98:E98"/>
+    <mergeCell ref="C107:E107"/>
     <mergeCell ref="C54:E54"/>
-    <mergeCell ref="B108:E108"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="C137:E137"/>
     <mergeCell ref="C134:E134"/>
+    <mergeCell ref="C146:E146"/>
+    <mergeCell ref="B83:E83"/>
     <mergeCell ref="C93:E93"/>
+    <mergeCell ref="B92:E92"/>
     <mergeCell ref="B30:E30"/>
+    <mergeCell ref="B124:E124"/>
     <mergeCell ref="C56:E56"/>
     <mergeCell ref="B5:E5"/>
+    <mergeCell ref="C90:E90"/>
+    <mergeCell ref="C105:E105"/>
+    <mergeCell ref="B133:E133"/>
     <mergeCell ref="C139:E139"/>
     <mergeCell ref="C138:E138"/>
     <mergeCell ref="C76:E76"/>
-    <mergeCell ref="B126:E126"/>
     <mergeCell ref="C132:E132"/>
-    <mergeCell ref="C110:E110"/>
     <mergeCell ref="C119:E119"/>
     <mergeCell ref="C8:E8"/>
+    <mergeCell ref="B62:E62"/>
     <mergeCell ref="C17:E17"/>
     <mergeCell ref="C82:E82"/>
-    <mergeCell ref="B125:E125"/>
     <mergeCell ref="B46:E46"/>
     <mergeCell ref="C19:E19"/>
     <mergeCell ref="C53:E53"/>
-    <mergeCell ref="B70:E70"/>
-    <mergeCell ref="B106:D106"/>
-    <mergeCell ref="C68:E68"/>
     <mergeCell ref="B111:E111"/>
-    <mergeCell ref="B98:E98"/>
-    <mergeCell ref="C58:E58"/>
+    <mergeCell ref="B145:E145"/>
+    <mergeCell ref="B88:E88"/>
     <mergeCell ref="C97:E97"/>
     <mergeCell ref="C29:E29"/>
     <mergeCell ref="C100:E100"/>
-    <mergeCell ref="C109:E109"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
   <rowBreaks count="6" manualBreakCount="6">
     <brk id="23" min="0" max="16383" man="1"/>
     <brk id="43" min="0" max="16383" man="1"/>
-    <brk id="63" min="0" max="16383" man="1"/>
-    <brk id="83" min="0" max="16383" man="1"/>
-    <brk id="104" min="0" max="16383" man="1"/>
-    <brk id="122" min="0" max="16383" man="1"/>
+    <brk id="64" min="0" max="16383" man="1"/>
+    <brk id="85" min="0" max="16383" man="1"/>
+    <brk id="108" min="0" max="16383" man="1"/>
+    <brk id="126" min="0" max="16383" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Elimina Jardín de Aspersión: fichas basadas solo en los productos del Canva
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111i7vn9WWo4QxCQbucWbrF
</commit_message>
<xml_diff>
--- a/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
+++ b/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
@@ -11,9 +11,9 @@
     <sheet name="Ficha Técnica Consolidada" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tabla Gral. - Visión Comercial'!$A$4:$I$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tabla Gral. - Visión Comercial'!$A$4:$I$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Tabla Gral. - Visión Comercial'!$4:$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Ficha Técnica Consolidada'!$A$1:$F$147</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Ficha Técnica Consolidada'!$A$1:$F$127</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -707,7 +707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -834,84 +834,33 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="93" customHeight="1">
+    <row r="6" ht="78.5" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>VG-CRE-02</t>
+          <t>VG-CRE-03I</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Jardín de Aspersión de Cenizas</t>
+          <t>Jardín de Cenizas · Individual</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>Destino final · Aspersión</t>
+          <t>Destino final · Inhumación individual</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>Liberación ceremonial de cenizas en el área de esparcimiento del Jardín Ecológico, junto al agua corriente, en armonía con la naturaleza.</t>
+          <t>Inhumación de la urna de cenizas en un contenedor enterrado con tapa de granito grabada, en un jardín de plantas de sombra: un lugar físico permanente de homenaje.</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>Servicio individual.</t>
+          <t>Individual (1 urna).</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>• Acompañamiento ceremonial
-• Tiempo privado para la familia en entorno botánico
-• Asistencia protocolar
-• Placa memorial que registra la aspersión realizada en el lugar</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
-        <is>
-          <t>Personas que buscan un concepto de libertad total, sin necesidad de un espacio físico fijo.</t>
-        </is>
-      </c>
-      <c r="H6" s="11" t="inlineStr">
-        <is>
-          <t>US$ 250
-(Pago único por servicio)</t>
-        </is>
-      </c>
-      <c r="I6" s="10" t="inlineStr">
-        <is>
-          <t>Pago único; combinable con la Solución Modular de Cremación.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="78.5" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>VG-CRE-03I</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Jardín de Cenizas · Individual</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Destino final · Inhumación individual</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Inhumación de la urna de cenizas en un contenedor enterrado con tapa de granito grabada, en un jardín de plantas de sombra: un lugar físico permanente de homenaje.</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>Individual (1 urna).</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>• Inhumación de la urna en contenedor individual
 • Tapa de granito con los datos del difunto
@@ -919,50 +868,50 @@
 • Espacio de contemplación con banco</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="G6" s="10" t="inlineStr">
         <is>
           <t>Familias que desean un lugar permanente para visitar y rendir homenaje, con una inversión moderada.</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="H6" s="11" t="inlineStr">
         <is>
           <t>US$ 600
 (Por espacio individual · mantenimiento US$ 15/año)</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr">
+      <c r="I6" s="10" t="inlineStr">
         <is>
           <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 15 anual.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="93" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
+    <row r="7" ht="93" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>VG-CRE-03F</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Jardín de Cenizas · Familiar</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Destino final · Inhumación familiar</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>Parcela familiar en el Jardín 1 con cuatro contenedores agrupados, cada uno con tapa de granito grabada, sin plazo de permanencia.</t>
         </is>
       </c>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>Hasta 4 espacios (familiar).</t>
         </is>
       </c>
-      <c r="F8" s="10" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>• Inhumación de hasta 4 urnas
 • Tapa de granito grabada para cada espacio
@@ -970,50 +919,50 @@
 • Lugar físico permanente de homenaje familiar, sin plazo</t>
         </is>
       </c>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>Familias que buscan un espacio propio y permanente para varias generaciones.</t>
         </is>
       </c>
-      <c r="H8" s="11" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>US$ 2.000
 (Por parcela familiar · hasta 4 espacios · mantenimiento US$ 25/año)</t>
         </is>
       </c>
-      <c r="I8" s="10" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 25 anual.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="122" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="8" ht="122" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>VG-CRE-03E</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Jardín de Cenizas · Ecológico</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>Destino final · Inhumación ecológica</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>La urna biodegradable se entierra directamente en el suelo, se cubre con tierra y se descompone integrándose a la naturaleza. Jardín con agua corriente y área de esparcimiento de cenizas.</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>Individual (1 urna).</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F8" s="10" t="inlineStr">
         <is>
           <t>• Inhumación ecológica de la urna directamente en el suelo
 • Placa de identificación
@@ -1022,99 +971,99 @@
 • Permanencia de 3 años; luego, placa memorial en el monumento</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G8" s="10" t="inlineStr">
         <is>
           <t>Personas con conciencia ambiental que desean que sus cenizas vuelvan a la tierra, con un lugar identificado para visitar.</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="H8" s="11" t="inlineStr">
         <is>
           <t>US$ 600
 (Por espacio individual · placa memorial US$ 150)</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="I8" s="10" t="inlineStr">
         <is>
           <t>Pago único o financiado según política comercial vigente. Placa memorial en el monumento al término del plazo: US$ 150.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="49.5" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
+    <row r="9" ht="49.5" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>VG-CRE-03C</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Jardín de Cenizas · Ceremonial</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Destino final · Inhumación con ceremonia</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Jardín para inhumación de urnas de cenizas con ceremonia de agua, con fuentes como elemento central del rito de despedida.</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>A definir.</t>
         </is>
       </c>
-      <c r="F10" s="10" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>• Inhumación de urnas de cenizas
 • Ceremonia con agua en fuente</t>
         </is>
       </c>
-      <c r="G10" s="10" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>Familias que valoran un rito de despedida simbólico y un entorno contemplativo.</t>
         </is>
       </c>
-      <c r="H10" s="11" t="inlineStr">
+      <c r="H9" s="7" t="inlineStr">
         <is>
           <t>A definir
 (Producto en definición)</t>
         </is>
       </c>
-      <c r="I10" s="10" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>A definir.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="93" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="10" ht="93" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>VG-CRE-04</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Jardín de Mascotas</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>Mascotas · Inhumación ecológica</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>Jardín para inhumación ecológica de cenizas de mascotas: la urna biodegradable se entierra directamente en el suelo y se identifica con una placa de madera.</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>Individual (una mascota por servicio).</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F10" s="10" t="inlineStr">
         <is>
           <t>• Inhumación ecológica de la urna en el jardín
 • Placa de madera de 20 cm para identificación
@@ -1122,25 +1071,25 @@
 • Cremación de la mascota (opción Jardín + Cremación)</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G10" s="10" t="inlineStr">
         <is>
           <t>Familias que consideran a su mascota parte del hogar y desean un cierre digno.</t>
         </is>
       </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="H10" s="11" t="inlineStr">
         <is>
           <t>US$ 350 / US$ 500
 (US$ 350 solo jardín · US$ 500 jardín + cremación)</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="I10" s="10" t="inlineStr">
         <is>
           <t>Pago único; puede contratarse como adicional al plan funerario. Placa memorial en el monumento al término del plazo: US$ 50.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I11"/>
+  <autoFilter ref="A4:I10"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
@@ -1157,7 +1106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:E146"/>
+  <dimension ref="B1:E126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1435,21 +1384,21 @@
     <row r="25" ht="30" customHeight="1">
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>JARDÍN DE ASPERSIÓN DE CENIZAS</t>
+          <t>JARDÍN DE CENIZAS · INDIVIDUAL</t>
         </is>
       </c>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
       <c r="E25" s="16" t="inlineStr">
         <is>
-          <t>VG-CRE-02</t>
+          <t>VG-CRE-03I</t>
         </is>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="B26" s="17" t="inlineStr">
         <is>
-          <t>Jardines de la Memoria  ·  Destino final · Aspersión</t>
+          <t>Jardines de la Memoria · Jardín 1  ·  Destino final · Inhumación individual</t>
         </is>
       </c>
       <c r="C26" s="18" t="n"/>
@@ -1466,7 +1415,7 @@
       <c r="D27" s="21" t="n"/>
       <c r="E27" s="22" t="n"/>
     </row>
-    <row r="28" ht="35" customHeight="1">
+    <row r="28" ht="49.5" customHeight="1">
       <c r="B28" s="23" t="inlineStr">
         <is>
           <t>Concepto</t>
@@ -1474,7 +1423,7 @@
       </c>
       <c r="C28" s="24" t="inlineStr">
         <is>
-          <t>Liberación ceremonial de cenizas en el área de esparcimiento del Jardín Ecológico, junto al agua corriente, en armonía con la naturaleza.</t>
+          <t>Inhumación de la urna de cenizas en un contenedor enterrado con tapa de granito grabada, en un jardín de plantas de sombra: un lugar físico permanente de homenaje.</t>
         </is>
       </c>
       <c r="D28" s="25" t="n"/>
@@ -1488,7 +1437,7 @@
       </c>
       <c r="C29" s="28" t="inlineStr">
         <is>
-          <t>Servicio individual.</t>
+          <t>Individual (1 urna).</t>
         </is>
       </c>
       <c r="D29" s="29" t="n"/>
@@ -1507,12 +1456,12 @@
     <row r="31" ht="20.5" customHeight="1">
       <c r="B31" s="23" t="inlineStr">
         <is>
-          <t>Tipo de producto</t>
+          <t>Ambiente</t>
         </is>
       </c>
       <c r="C31" s="24" t="inlineStr">
         <is>
-          <t>Servicio ceremonial de destino final</t>
+          <t>Jardín 1</t>
         </is>
       </c>
       <c r="D31" s="25" t="n"/>
@@ -1521,12 +1470,12 @@
     <row r="32" ht="20.5" customHeight="1">
       <c r="B32" s="27" t="inlineStr">
         <is>
-          <t>Capacidad</t>
+          <t>Contenedor</t>
         </is>
       </c>
       <c r="C32" s="28" t="inlineStr">
         <is>
-          <t>Individual</t>
+          <t>Ø 32 cm × 40 cm de altura; enterrado dejando 20 cm a la vista</t>
         </is>
       </c>
       <c r="D32" s="29" t="n"/>
@@ -1535,12 +1484,12 @@
     <row r="33" ht="20.5" customHeight="1">
       <c r="B33" s="23" t="inlineStr">
         <is>
-          <t>Ubicación</t>
+          <t>Identificación</t>
         </is>
       </c>
       <c r="C33" s="24" t="inlineStr">
         <is>
-          <t>Jardín 2 · Ecológico, área de esparcimiento de cenizas</t>
+          <t>Tapa de granito con la información del difunto</t>
         </is>
       </c>
       <c r="D33" s="25" t="n"/>
@@ -1549,12 +1498,12 @@
     <row r="34" ht="20.5" customHeight="1">
       <c r="B34" s="27" t="inlineStr">
         <is>
-          <t>Entorno</t>
+          <t>Paisajismo</t>
         </is>
       </c>
       <c r="C34" s="28" t="inlineStr">
         <is>
-          <t>Agua corriente que se extiende hasta el jardín</t>
+          <t>Plantas de sombra de diferentes alturas y texturas</t>
         </is>
       </c>
       <c r="D34" s="29" t="n"/>
@@ -1563,273 +1512,38 @@
     <row r="35" ht="20.5" customHeight="1">
       <c r="B35" s="23" t="inlineStr">
         <is>
-          <t>Homenaje</t>
+          <t>Acceso</t>
         </is>
       </c>
       <c r="C35" s="24" t="inlineStr">
         <is>
-          <t>Placa memorial de la aspersión</t>
+          <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
         </is>
       </c>
       <c r="D35" s="25" t="n"/>
       <c r="E35" s="26" t="n"/>
     </row>
-    <row r="36" ht="64" customHeight="1">
+    <row r="36" ht="20.5" customHeight="1">
       <c r="B36" s="27" t="inlineStr">
         <is>
-          <t>Servicios incluidos</t>
+          <t>Mantenimiento</t>
         </is>
       </c>
       <c r="C36" s="28" t="inlineStr">
         <is>
-          <t>• Acompañamiento ceremonial
-• Tiempo privado para la familia en entorno botánico
-• Asistencia protocolar
-• Placa memorial que registra la aspersión realizada en el lugar</t>
+          <t>US$ 15 anual</t>
         </is>
       </c>
       <c r="D36" s="29" t="n"/>
       <c r="E36" s="30" t="n"/>
     </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="B37" s="20" t="inlineStr">
-        <is>
-          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
-        </is>
-      </c>
-      <c r="C37" s="21" t="n"/>
-      <c r="D37" s="21" t="n"/>
-      <c r="E37" s="22" t="n"/>
-    </row>
-    <row r="38" ht="26.5" customHeight="1">
-      <c r="B38" s="23" t="inlineStr">
-        <is>
-          <t>Precio sugerido</t>
-        </is>
-      </c>
-      <c r="C38" s="31" t="inlineStr">
-        <is>
-          <t>US$ 250</t>
-        </is>
-      </c>
-      <c r="D38" s="25" t="n"/>
-      <c r="E38" s="26" t="n"/>
-    </row>
-    <row r="39" ht="20.5" customHeight="1">
-      <c r="B39" s="27" t="inlineStr">
-        <is>
-          <t>Base de precio</t>
-        </is>
-      </c>
-      <c r="C39" s="28" t="inlineStr">
-        <is>
-          <t>Pago único por servicio</t>
-        </is>
-      </c>
-      <c r="D39" s="29" t="n"/>
-      <c r="E39" s="30" t="n"/>
-    </row>
-    <row r="40" ht="20.5" customHeight="1">
-      <c r="B40" s="23" t="inlineStr">
-        <is>
-          <t>Condiciones</t>
-        </is>
-      </c>
-      <c r="C40" s="24" t="inlineStr">
-        <is>
-          <t>Pago único; combinable con la Solución Modular de Cremación.</t>
-        </is>
-      </c>
-      <c r="D40" s="25" t="n"/>
-      <c r="E40" s="26" t="n"/>
-    </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="B41" s="20" t="inlineStr">
-        <is>
-          <t>PERFIL DEL COMPRADOR</t>
-        </is>
-      </c>
-      <c r="C41" s="21" t="n"/>
-      <c r="D41" s="21" t="n"/>
-      <c r="E41" s="22" t="n"/>
-    </row>
-    <row r="42" ht="35" customHeight="1">
-      <c r="B42" s="32" t="inlineStr">
-        <is>
-          <t>Cliente objetivo</t>
-        </is>
-      </c>
-      <c r="C42" s="33" t="inlineStr">
-        <is>
-          <t>Personas que buscan un concepto de libertad total, sin necesidad de un espacio físico fijo.</t>
-        </is>
-      </c>
-      <c r="D42" s="34" t="n"/>
-      <c r="E42" s="35" t="n"/>
-    </row>
-    <row r="45" ht="30" customHeight="1">
-      <c r="B45" s="14" t="inlineStr">
-        <is>
-          <t>JARDÍN DE CENIZAS · INDIVIDUAL</t>
-        </is>
-      </c>
-      <c r="C45" s="15" t="n"/>
-      <c r="D45" s="15" t="n"/>
-      <c r="E45" s="16" t="inlineStr">
-        <is>
-          <t>VG-CRE-03I</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="B46" s="17" t="inlineStr">
-        <is>
-          <t>Jardines de la Memoria · Jardín 1  ·  Destino final · Inhumación individual</t>
-        </is>
-      </c>
-      <c r="C46" s="18" t="n"/>
-      <c r="D46" s="18" t="n"/>
-      <c r="E46" s="19" t="n"/>
-    </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="B47" s="20" t="inlineStr">
-        <is>
-          <t>VISIÓN GENERAL</t>
-        </is>
-      </c>
-      <c r="C47" s="21" t="n"/>
-      <c r="D47" s="21" t="n"/>
-      <c r="E47" s="22" t="n"/>
-    </row>
-    <row r="48" ht="49.5" customHeight="1">
-      <c r="B48" s="23" t="inlineStr">
-        <is>
-          <t>Concepto</t>
-        </is>
-      </c>
-      <c r="C48" s="24" t="inlineStr">
-        <is>
-          <t>Inhumación de la urna de cenizas en un contenedor enterrado con tapa de granito grabada, en un jardín de plantas de sombra: un lugar físico permanente de homenaje.</t>
-        </is>
-      </c>
-      <c r="D48" s="25" t="n"/>
-      <c r="E48" s="26" t="n"/>
-    </row>
-    <row r="49" ht="20.5" customHeight="1">
-      <c r="B49" s="27" t="inlineStr">
-        <is>
-          <t>Capacidad / Cobertura</t>
-        </is>
-      </c>
-      <c r="C49" s="28" t="inlineStr">
-        <is>
-          <t>Individual (1 urna).</t>
-        </is>
-      </c>
-      <c r="D49" s="29" t="n"/>
-      <c r="E49" s="30" t="n"/>
-    </row>
-    <row r="50" ht="20" customHeight="1">
-      <c r="B50" s="20" t="inlineStr">
-        <is>
-          <t>ESPECIFICACIONES TÉCNICAS</t>
-        </is>
-      </c>
-      <c r="C50" s="21" t="n"/>
-      <c r="D50" s="21" t="n"/>
-      <c r="E50" s="22" t="n"/>
-    </row>
-    <row r="51" ht="20.5" customHeight="1">
-      <c r="B51" s="23" t="inlineStr">
-        <is>
-          <t>Ambiente</t>
-        </is>
-      </c>
-      <c r="C51" s="24" t="inlineStr">
-        <is>
-          <t>Jardín 1</t>
-        </is>
-      </c>
-      <c r="D51" s="25" t="n"/>
-      <c r="E51" s="26" t="n"/>
-    </row>
-    <row r="52" ht="20.5" customHeight="1">
-      <c r="B52" s="27" t="inlineStr">
-        <is>
-          <t>Contenedor</t>
-        </is>
-      </c>
-      <c r="C52" s="28" t="inlineStr">
-        <is>
-          <t>Ø 32 cm × 40 cm de altura; enterrado dejando 20 cm a la vista</t>
-        </is>
-      </c>
-      <c r="D52" s="29" t="n"/>
-      <c r="E52" s="30" t="n"/>
-    </row>
-    <row r="53" ht="20.5" customHeight="1">
-      <c r="B53" s="23" t="inlineStr">
-        <is>
-          <t>Identificación</t>
-        </is>
-      </c>
-      <c r="C53" s="24" t="inlineStr">
-        <is>
-          <t>Tapa de granito con la información del difunto</t>
-        </is>
-      </c>
-      <c r="D53" s="25" t="n"/>
-      <c r="E53" s="26" t="n"/>
-    </row>
-    <row r="54" ht="20.5" customHeight="1">
-      <c r="B54" s="27" t="inlineStr">
-        <is>
-          <t>Paisajismo</t>
-        </is>
-      </c>
-      <c r="C54" s="28" t="inlineStr">
-        <is>
-          <t>Plantas de sombra de diferentes alturas y texturas</t>
-        </is>
-      </c>
-      <c r="D54" s="29" t="n"/>
-      <c r="E54" s="30" t="n"/>
-    </row>
-    <row r="55" ht="20.5" customHeight="1">
-      <c r="B55" s="23" t="inlineStr">
-        <is>
-          <t>Acceso</t>
-        </is>
-      </c>
-      <c r="C55" s="24" t="inlineStr">
-        <is>
-          <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
-        </is>
-      </c>
-      <c r="D55" s="25" t="n"/>
-      <c r="E55" s="26" t="n"/>
-    </row>
-    <row r="56" ht="20.5" customHeight="1">
-      <c r="B56" s="27" t="inlineStr">
-        <is>
-          <t>Mantenimiento</t>
-        </is>
-      </c>
-      <c r="C56" s="28" t="inlineStr">
-        <is>
-          <t>US$ 15 anual</t>
-        </is>
-      </c>
-      <c r="D56" s="29" t="n"/>
-      <c r="E56" s="30" t="n"/>
-    </row>
-    <row r="57" ht="64" customHeight="1">
-      <c r="B57" s="23" t="inlineStr">
+    <row r="37" ht="64" customHeight="1">
+      <c r="B37" s="23" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C57" s="24" t="inlineStr">
+      <c r="C37" s="24" t="inlineStr">
         <is>
           <t>• Inhumación de la urna en contenedor individual
 • Tapa de granito con los datos del difunto
@@ -1837,248 +1551,248 @@
 • Espacio de contemplación con banco</t>
         </is>
       </c>
-      <c r="D57" s="25" t="n"/>
-      <c r="E57" s="26" t="n"/>
-    </row>
-    <row r="58" ht="20" customHeight="1">
-      <c r="B58" s="20" t="inlineStr">
+      <c r="D37" s="25" t="n"/>
+      <c r="E37" s="26" t="n"/>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="B38" s="20" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C58" s="21" t="n"/>
-      <c r="D58" s="21" t="n"/>
-      <c r="E58" s="22" t="n"/>
-    </row>
-    <row r="59" ht="26.5" customHeight="1">
-      <c r="B59" s="23" t="inlineStr">
+      <c r="C38" s="21" t="n"/>
+      <c r="D38" s="21" t="n"/>
+      <c r="E38" s="22" t="n"/>
+    </row>
+    <row r="39" ht="26.5" customHeight="1">
+      <c r="B39" s="23" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C59" s="31" t="inlineStr">
+      <c r="C39" s="31" t="inlineStr">
         <is>
           <t>US$ 600</t>
         </is>
       </c>
-      <c r="D59" s="25" t="n"/>
-      <c r="E59" s="26" t="n"/>
-    </row>
-    <row r="60" ht="20.5" customHeight="1">
-      <c r="B60" s="27" t="inlineStr">
+      <c r="D39" s="25" t="n"/>
+      <c r="E39" s="26" t="n"/>
+    </row>
+    <row r="40" ht="20.5" customHeight="1">
+      <c r="B40" s="27" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C60" s="28" t="inlineStr">
+      <c r="C40" s="28" t="inlineStr">
         <is>
           <t>Por espacio individual · mantenimiento US$ 15/año</t>
         </is>
       </c>
-      <c r="D60" s="29" t="n"/>
-      <c r="E60" s="30" t="n"/>
-    </row>
-    <row r="61" ht="35" customHeight="1">
-      <c r="B61" s="23" t="inlineStr">
+      <c r="D40" s="29" t="n"/>
+      <c r="E40" s="30" t="n"/>
+    </row>
+    <row r="41" ht="35" customHeight="1">
+      <c r="B41" s="23" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C61" s="24" t="inlineStr">
+      <c r="C41" s="24" t="inlineStr">
         <is>
           <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 15 anual.</t>
         </is>
       </c>
-      <c r="D61" s="25" t="n"/>
-      <c r="E61" s="26" t="n"/>
-    </row>
-    <row r="62" ht="20" customHeight="1">
-      <c r="B62" s="20" t="inlineStr">
+      <c r="D41" s="25" t="n"/>
+      <c r="E41" s="26" t="n"/>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="B42" s="20" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C62" s="21" t="n"/>
-      <c r="D62" s="21" t="n"/>
-      <c r="E62" s="22" t="n"/>
-    </row>
-    <row r="63" ht="35" customHeight="1">
-      <c r="B63" s="32" t="inlineStr">
+      <c r="C42" s="21" t="n"/>
+      <c r="D42" s="21" t="n"/>
+      <c r="E42" s="22" t="n"/>
+    </row>
+    <row r="43" ht="35" customHeight="1">
+      <c r="B43" s="32" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C63" s="33" t="inlineStr">
+      <c r="C43" s="33" t="inlineStr">
         <is>
           <t>Familias que desean un lugar permanente para visitar y rendir homenaje, con una inversión moderada.</t>
         </is>
       </c>
-      <c r="D63" s="34" t="n"/>
-      <c r="E63" s="35" t="n"/>
-    </row>
-    <row r="66" ht="30" customHeight="1">
-      <c r="B66" s="14" t="inlineStr">
+      <c r="D43" s="34" t="n"/>
+      <c r="E43" s="35" t="n"/>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="B46" s="14" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · FAMILIAR</t>
         </is>
       </c>
-      <c r="C66" s="15" t="n"/>
-      <c r="D66" s="15" t="n"/>
-      <c r="E66" s="16" t="inlineStr">
+      <c r="C46" s="15" t="n"/>
+      <c r="D46" s="15" t="n"/>
+      <c r="E46" s="16" t="inlineStr">
         <is>
           <t>VG-CRE-03F</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="20" customHeight="1">
-      <c r="B67" s="17" t="inlineStr">
+    <row r="47" ht="20" customHeight="1">
+      <c r="B47" s="17" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Jardín 1  ·  Destino final · Inhumación familiar</t>
         </is>
       </c>
-      <c r="C67" s="18" t="n"/>
-      <c r="D67" s="18" t="n"/>
-      <c r="E67" s="19" t="n"/>
-    </row>
-    <row r="68" ht="20" customHeight="1">
-      <c r="B68" s="20" t="inlineStr">
+      <c r="C47" s="18" t="n"/>
+      <c r="D47" s="18" t="n"/>
+      <c r="E47" s="19" t="n"/>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="B48" s="20" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C68" s="21" t="n"/>
-      <c r="D68" s="21" t="n"/>
-      <c r="E68" s="22" t="n"/>
-    </row>
-    <row r="69" ht="35" customHeight="1">
-      <c r="B69" s="23" t="inlineStr">
+      <c r="C48" s="21" t="n"/>
+      <c r="D48" s="21" t="n"/>
+      <c r="E48" s="22" t="n"/>
+    </row>
+    <row r="49" ht="35" customHeight="1">
+      <c r="B49" s="23" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C69" s="24" t="inlineStr">
+      <c r="C49" s="24" t="inlineStr">
         <is>
           <t>Parcela familiar en el Jardín 1 con cuatro contenedores agrupados, cada uno con tapa de granito grabada, sin plazo de permanencia.</t>
         </is>
       </c>
-      <c r="D69" s="25" t="n"/>
-      <c r="E69" s="26" t="n"/>
-    </row>
-    <row r="70" ht="20.5" customHeight="1">
-      <c r="B70" s="27" t="inlineStr">
+      <c r="D49" s="25" t="n"/>
+      <c r="E49" s="26" t="n"/>
+    </row>
+    <row r="50" ht="20.5" customHeight="1">
+      <c r="B50" s="27" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C70" s="28" t="inlineStr">
+      <c r="C50" s="28" t="inlineStr">
         <is>
           <t>Hasta 4 espacios (familiar).</t>
         </is>
       </c>
-      <c r="D70" s="29" t="n"/>
-      <c r="E70" s="30" t="n"/>
-    </row>
-    <row r="71" ht="20" customHeight="1">
-      <c r="B71" s="20" t="inlineStr">
+      <c r="D50" s="29" t="n"/>
+      <c r="E50" s="30" t="n"/>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="B51" s="20" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C71" s="21" t="n"/>
-      <c r="D71" s="21" t="n"/>
-      <c r="E71" s="22" t="n"/>
-    </row>
-    <row r="72" ht="20.5" customHeight="1">
-      <c r="B72" s="23" t="inlineStr">
+      <c r="C51" s="21" t="n"/>
+      <c r="D51" s="21" t="n"/>
+      <c r="E51" s="22" t="n"/>
+    </row>
+    <row r="52" ht="20.5" customHeight="1">
+      <c r="B52" s="23" t="inlineStr">
         <is>
           <t>Ambiente</t>
         </is>
       </c>
-      <c r="C72" s="24" t="inlineStr">
+      <c r="C52" s="24" t="inlineStr">
         <is>
           <t>Jardín 1</t>
         </is>
       </c>
-      <c r="D72" s="25" t="n"/>
-      <c r="E72" s="26" t="n"/>
-    </row>
-    <row r="73" ht="20.5" customHeight="1">
-      <c r="B73" s="27" t="inlineStr">
+      <c r="D52" s="25" t="n"/>
+      <c r="E52" s="26" t="n"/>
+    </row>
+    <row r="53" ht="20.5" customHeight="1">
+      <c r="B53" s="27" t="inlineStr">
         <is>
           <t>Capacidad</t>
         </is>
       </c>
-      <c r="C73" s="28" t="inlineStr">
+      <c r="C53" s="28" t="inlineStr">
         <is>
           <t>4 contenedores agrupados en losa</t>
         </is>
       </c>
-      <c r="D73" s="29" t="n"/>
-      <c r="E73" s="30" t="n"/>
-    </row>
-    <row r="74" ht="20.5" customHeight="1">
-      <c r="B74" s="23" t="inlineStr">
+      <c r="D53" s="29" t="n"/>
+      <c r="E53" s="30" t="n"/>
+    </row>
+    <row r="54" ht="20.5" customHeight="1">
+      <c r="B54" s="23" t="inlineStr">
         <is>
           <t>Identificación</t>
         </is>
       </c>
-      <c r="C74" s="24" t="inlineStr">
+      <c r="C54" s="24" t="inlineStr">
         <is>
           <t>Tapa de granito por espacio, con la información del difunto</t>
         </is>
       </c>
-      <c r="D74" s="25" t="n"/>
-      <c r="E74" s="26" t="n"/>
-    </row>
-    <row r="75" ht="20.5" customHeight="1">
-      <c r="B75" s="27" t="inlineStr">
+      <c r="D54" s="25" t="n"/>
+      <c r="E54" s="26" t="n"/>
+    </row>
+    <row r="55" ht="20.5" customHeight="1">
+      <c r="B55" s="27" t="inlineStr">
         <is>
           <t>Permanencia</t>
         </is>
       </c>
-      <c r="C75" s="28" t="inlineStr">
+      <c r="C55" s="28" t="inlineStr">
         <is>
           <t>Sin plazo</t>
         </is>
       </c>
-      <c r="D75" s="29" t="n"/>
-      <c r="E75" s="30" t="n"/>
-    </row>
-    <row r="76" ht="20.5" customHeight="1">
-      <c r="B76" s="23" t="inlineStr">
+      <c r="D55" s="29" t="n"/>
+      <c r="E55" s="30" t="n"/>
+    </row>
+    <row r="56" ht="20.5" customHeight="1">
+      <c r="B56" s="23" t="inlineStr">
         <is>
           <t>Acceso</t>
         </is>
       </c>
-      <c r="C76" s="24" t="inlineStr">
+      <c r="C56" s="24" t="inlineStr">
         <is>
           <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
         </is>
       </c>
-      <c r="D76" s="25" t="n"/>
-      <c r="E76" s="26" t="n"/>
-    </row>
-    <row r="77" ht="20.5" customHeight="1">
-      <c r="B77" s="27" t="inlineStr">
+      <c r="D56" s="25" t="n"/>
+      <c r="E56" s="26" t="n"/>
+    </row>
+    <row r="57" ht="20.5" customHeight="1">
+      <c r="B57" s="27" t="inlineStr">
         <is>
           <t>Mantenimiento</t>
         </is>
       </c>
-      <c r="C77" s="28" t="inlineStr">
+      <c r="C57" s="28" t="inlineStr">
         <is>
           <t>US$ 25 anual</t>
         </is>
       </c>
-      <c r="D77" s="29" t="n"/>
-      <c r="E77" s="30" t="n"/>
-    </row>
-    <row r="78" ht="64" customHeight="1">
-      <c r="B78" s="23" t="inlineStr">
+      <c r="D57" s="29" t="n"/>
+      <c r="E57" s="30" t="n"/>
+    </row>
+    <row r="58" ht="64" customHeight="1">
+      <c r="B58" s="23" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C78" s="24" t="inlineStr">
+      <c r="C58" s="24" t="inlineStr">
         <is>
           <t>• Inhumación de hasta 4 urnas
 • Tapa de granito grabada para cada espacio
@@ -2086,276 +1800,276 @@
 • Lugar físico permanente de homenaje familiar, sin plazo</t>
         </is>
       </c>
-      <c r="D78" s="25" t="n"/>
-      <c r="E78" s="26" t="n"/>
-    </row>
-    <row r="79" ht="20" customHeight="1">
-      <c r="B79" s="20" t="inlineStr">
+      <c r="D58" s="25" t="n"/>
+      <c r="E58" s="26" t="n"/>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="B59" s="20" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C79" s="21" t="n"/>
-      <c r="D79" s="21" t="n"/>
-      <c r="E79" s="22" t="n"/>
-    </row>
-    <row r="80" ht="26.5" customHeight="1">
-      <c r="B80" s="23" t="inlineStr">
+      <c r="C59" s="21" t="n"/>
+      <c r="D59" s="21" t="n"/>
+      <c r="E59" s="22" t="n"/>
+    </row>
+    <row r="60" ht="26.5" customHeight="1">
+      <c r="B60" s="23" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C80" s="31" t="inlineStr">
+      <c r="C60" s="31" t="inlineStr">
         <is>
           <t>US$ 2.000</t>
         </is>
       </c>
-      <c r="D80" s="25" t="n"/>
-      <c r="E80" s="26" t="n"/>
-    </row>
-    <row r="81" ht="20.5" customHeight="1">
-      <c r="B81" s="27" t="inlineStr">
+      <c r="D60" s="25" t="n"/>
+      <c r="E60" s="26" t="n"/>
+    </row>
+    <row r="61" ht="20.5" customHeight="1">
+      <c r="B61" s="27" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C81" s="28" t="inlineStr">
+      <c r="C61" s="28" t="inlineStr">
         <is>
           <t>Por parcela familiar · hasta 4 espacios · mantenimiento US$ 25/año</t>
         </is>
       </c>
-      <c r="D81" s="29" t="n"/>
-      <c r="E81" s="30" t="n"/>
-    </row>
-    <row r="82" ht="35" customHeight="1">
-      <c r="B82" s="23" t="inlineStr">
+      <c r="D61" s="29" t="n"/>
+      <c r="E61" s="30" t="n"/>
+    </row>
+    <row r="62" ht="35" customHeight="1">
+      <c r="B62" s="23" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C82" s="24" t="inlineStr">
+      <c r="C62" s="24" t="inlineStr">
         <is>
           <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 25 anual.</t>
         </is>
       </c>
-      <c r="D82" s="25" t="n"/>
-      <c r="E82" s="26" t="n"/>
-    </row>
-    <row r="83" ht="20" customHeight="1">
-      <c r="B83" s="20" t="inlineStr">
+      <c r="D62" s="25" t="n"/>
+      <c r="E62" s="26" t="n"/>
+    </row>
+    <row r="63" ht="20" customHeight="1">
+      <c r="B63" s="20" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C83" s="21" t="n"/>
-      <c r="D83" s="21" t="n"/>
-      <c r="E83" s="22" t="n"/>
-    </row>
-    <row r="84" ht="20.5" customHeight="1">
-      <c r="B84" s="32" t="inlineStr">
+      <c r="C63" s="21" t="n"/>
+      <c r="D63" s="21" t="n"/>
+      <c r="E63" s="22" t="n"/>
+    </row>
+    <row r="64" ht="20.5" customHeight="1">
+      <c r="B64" s="32" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C84" s="33" t="inlineStr">
+      <c r="C64" s="33" t="inlineStr">
         <is>
           <t>Familias que buscan un espacio propio y permanente para varias generaciones.</t>
         </is>
       </c>
-      <c r="D84" s="34" t="n"/>
-      <c r="E84" s="35" t="n"/>
-    </row>
-    <row r="87" ht="30" customHeight="1">
-      <c r="B87" s="14" t="inlineStr">
+      <c r="D64" s="34" t="n"/>
+      <c r="E64" s="35" t="n"/>
+    </row>
+    <row r="67" ht="30" customHeight="1">
+      <c r="B67" s="14" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · ECOLÓGICO</t>
         </is>
       </c>
-      <c r="C87" s="15" t="n"/>
-      <c r="D87" s="15" t="n"/>
-      <c r="E87" s="16" t="inlineStr">
+      <c r="C67" s="15" t="n"/>
+      <c r="D67" s="15" t="n"/>
+      <c r="E67" s="16" t="inlineStr">
         <is>
           <t>VG-CRE-03E</t>
         </is>
       </c>
     </row>
-    <row r="88" ht="20" customHeight="1">
-      <c r="B88" s="17" t="inlineStr">
+    <row r="68" ht="20" customHeight="1">
+      <c r="B68" s="17" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Jardín 2  ·  Destino final · Inhumación ecológica</t>
         </is>
       </c>
-      <c r="C88" s="18" t="n"/>
-      <c r="D88" s="18" t="n"/>
-      <c r="E88" s="19" t="n"/>
-    </row>
-    <row r="89" ht="20" customHeight="1">
-      <c r="B89" s="20" t="inlineStr">
+      <c r="C68" s="18" t="n"/>
+      <c r="D68" s="18" t="n"/>
+      <c r="E68" s="19" t="n"/>
+    </row>
+    <row r="69" ht="20" customHeight="1">
+      <c r="B69" s="20" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C89" s="21" t="n"/>
-      <c r="D89" s="21" t="n"/>
-      <c r="E89" s="22" t="n"/>
-    </row>
-    <row r="90" ht="49.5" customHeight="1">
-      <c r="B90" s="23" t="inlineStr">
+      <c r="C69" s="21" t="n"/>
+      <c r="D69" s="21" t="n"/>
+      <c r="E69" s="22" t="n"/>
+    </row>
+    <row r="70" ht="49.5" customHeight="1">
+      <c r="B70" s="23" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C90" s="24" t="inlineStr">
+      <c r="C70" s="24" t="inlineStr">
         <is>
           <t>La urna biodegradable se entierra directamente en el suelo, se cubre con tierra y se descompone integrándose a la naturaleza. Jardín con agua corriente y área de esparcimiento de cenizas.</t>
         </is>
       </c>
-      <c r="D90" s="25" t="n"/>
-      <c r="E90" s="26" t="n"/>
-    </row>
-    <row r="91" ht="20.5" customHeight="1">
-      <c r="B91" s="27" t="inlineStr">
+      <c r="D70" s="25" t="n"/>
+      <c r="E70" s="26" t="n"/>
+    </row>
+    <row r="71" ht="20.5" customHeight="1">
+      <c r="B71" s="27" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C91" s="28" t="inlineStr">
+      <c r="C71" s="28" t="inlineStr">
         <is>
           <t>Individual (1 urna).</t>
         </is>
       </c>
-      <c r="D91" s="29" t="n"/>
-      <c r="E91" s="30" t="n"/>
-    </row>
-    <row r="92" ht="20" customHeight="1">
-      <c r="B92" s="20" t="inlineStr">
+      <c r="D71" s="29" t="n"/>
+      <c r="E71" s="30" t="n"/>
+    </row>
+    <row r="72" ht="20" customHeight="1">
+      <c r="B72" s="20" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C92" s="21" t="n"/>
-      <c r="D92" s="21" t="n"/>
-      <c r="E92" s="22" t="n"/>
-    </row>
-    <row r="93" ht="20.5" customHeight="1">
-      <c r="B93" s="23" t="inlineStr">
+      <c r="C72" s="21" t="n"/>
+      <c r="D72" s="21" t="n"/>
+      <c r="E72" s="22" t="n"/>
+    </row>
+    <row r="73" ht="20.5" customHeight="1">
+      <c r="B73" s="23" t="inlineStr">
         <is>
           <t>Ambientes</t>
         </is>
       </c>
-      <c r="C93" s="24" t="inlineStr">
+      <c r="C73" s="24" t="inlineStr">
         <is>
           <t>Jardín 2 · Ecológico o Bosque de las Orquídeas</t>
         </is>
       </c>
-      <c r="D93" s="25" t="n"/>
-      <c r="E93" s="26" t="n"/>
-    </row>
-    <row r="94" ht="20.5" customHeight="1">
-      <c r="B94" s="27" t="inlineStr">
+      <c r="D73" s="25" t="n"/>
+      <c r="E73" s="26" t="n"/>
+    </row>
+    <row r="74" ht="20.5" customHeight="1">
+      <c r="B74" s="27" t="inlineStr">
         <is>
           <t>Espacio por urna</t>
         </is>
       </c>
-      <c r="C94" s="28" t="inlineStr">
+      <c r="C74" s="28" t="inlineStr">
         <is>
           <t>30 × 30 cm, 40 cm de profundidad</t>
         </is>
       </c>
-      <c r="D94" s="29" t="n"/>
-      <c r="E94" s="30" t="n"/>
-    </row>
-    <row r="95" ht="20.5" customHeight="1">
-      <c r="B95" s="23" t="inlineStr">
+      <c r="D74" s="29" t="n"/>
+      <c r="E74" s="30" t="n"/>
+    </row>
+    <row r="75" ht="20.5" customHeight="1">
+      <c r="B75" s="23" t="inlineStr">
         <is>
           <t>Urna</t>
         </is>
       </c>
-      <c r="C95" s="24" t="inlineStr">
+      <c r="C75" s="24" t="inlineStr">
         <is>
           <t>Biodegradable; se integra al suelo</t>
         </is>
       </c>
-      <c r="D95" s="25" t="n"/>
-      <c r="E95" s="26" t="n"/>
-    </row>
-    <row r="96" ht="35" customHeight="1">
-      <c r="B96" s="27" t="inlineStr">
+      <c r="D75" s="25" t="n"/>
+      <c r="E75" s="26" t="n"/>
+    </row>
+    <row r="76" ht="35" customHeight="1">
+      <c r="B76" s="27" t="inlineStr">
         <is>
           <t>Identificación (Jardín 2)</t>
         </is>
       </c>
-      <c r="C96" s="28" t="inlineStr">
+      <c r="C76" s="28" t="inlineStr">
         <is>
           <t>Placa de madera de 20 cm fijada a una varilla metálica, en posición vertical y sin contacto con el suelo</t>
         </is>
       </c>
-      <c r="D96" s="29" t="n"/>
-      <c r="E96" s="30" t="n"/>
-    </row>
-    <row r="97" ht="20.5" customHeight="1">
-      <c r="B97" s="23" t="inlineStr">
+      <c r="D76" s="29" t="n"/>
+      <c r="E76" s="30" t="n"/>
+    </row>
+    <row r="77" ht="20.5" customHeight="1">
+      <c r="B77" s="23" t="inlineStr">
         <is>
           <t>Identificación (Bosque)</t>
         </is>
       </c>
-      <c r="C97" s="24" t="inlineStr">
+      <c r="C77" s="24" t="inlineStr">
         <is>
           <t>Placa de mármol de 20 × 15 cm</t>
         </is>
       </c>
-      <c r="D97" s="25" t="n"/>
-      <c r="E97" s="26" t="n"/>
-    </row>
-    <row r="98" ht="35" customHeight="1">
-      <c r="B98" s="27" t="inlineStr">
+      <c r="D77" s="25" t="n"/>
+      <c r="E77" s="26" t="n"/>
+    </row>
+    <row r="78" ht="35" customHeight="1">
+      <c r="B78" s="27" t="inlineStr">
         <is>
           <t>Permanencia</t>
         </is>
       </c>
-      <c r="C98" s="28" t="inlineStr">
+      <c r="C78" s="28" t="inlineStr">
         <is>
           <t>3 años; luego el nombre pasa a una placa memorial en el monumento y el espacio se reutiliza</t>
         </is>
       </c>
-      <c r="D98" s="29" t="n"/>
-      <c r="E98" s="30" t="n"/>
-    </row>
-    <row r="99" ht="20.5" customHeight="1">
-      <c r="B99" s="23" t="inlineStr">
+      <c r="D78" s="29" t="n"/>
+      <c r="E78" s="30" t="n"/>
+    </row>
+    <row r="79" ht="20.5" customHeight="1">
+      <c r="B79" s="23" t="inlineStr">
         <is>
           <t>Placa memorial</t>
         </is>
       </c>
-      <c r="C99" s="24" t="inlineStr">
+      <c r="C79" s="24" t="inlineStr">
         <is>
           <t>US$ 150</t>
         </is>
       </c>
-      <c r="D99" s="25" t="n"/>
-      <c r="E99" s="26" t="n"/>
-    </row>
-    <row r="100" ht="20.5" customHeight="1">
-      <c r="B100" s="27" t="inlineStr">
+      <c r="D79" s="25" t="n"/>
+      <c r="E79" s="26" t="n"/>
+    </row>
+    <row r="80" ht="20.5" customHeight="1">
+      <c r="B80" s="27" t="inlineStr">
         <is>
           <t>Acceso</t>
         </is>
       </c>
-      <c r="C100" s="28" t="inlineStr">
+      <c r="C80" s="28" t="inlineStr">
         <is>
           <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
         </is>
       </c>
-      <c r="D100" s="29" t="n"/>
-      <c r="E100" s="30" t="n"/>
-    </row>
-    <row r="101" ht="78.5" customHeight="1">
-      <c r="B101" s="23" t="inlineStr">
+      <c r="D80" s="29" t="n"/>
+      <c r="E80" s="30" t="n"/>
+    </row>
+    <row r="81" ht="78.5" customHeight="1">
+      <c r="B81" s="23" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C101" s="24" t="inlineStr">
+      <c r="C81" s="24" t="inlineStr">
         <is>
           <t>• Inhumación ecológica de la urna directamente en el suelo
 • Placa de identificación
@@ -2364,166 +2078,399 @@
 • Permanencia de 3 años; luego, placa memorial en el monumento</t>
         </is>
       </c>
+      <c r="D81" s="25" t="n"/>
+      <c r="E81" s="26" t="n"/>
+    </row>
+    <row r="82" ht="20" customHeight="1">
+      <c r="B82" s="20" t="inlineStr">
+        <is>
+          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
+        </is>
+      </c>
+      <c r="C82" s="21" t="n"/>
+      <c r="D82" s="21" t="n"/>
+      <c r="E82" s="22" t="n"/>
+    </row>
+    <row r="83" ht="26.5" customHeight="1">
+      <c r="B83" s="23" t="inlineStr">
+        <is>
+          <t>Precio sugerido</t>
+        </is>
+      </c>
+      <c r="C83" s="31" t="inlineStr">
+        <is>
+          <t>US$ 600</t>
+        </is>
+      </c>
+      <c r="D83" s="25" t="n"/>
+      <c r="E83" s="26" t="n"/>
+    </row>
+    <row r="84" ht="20.5" customHeight="1">
+      <c r="B84" s="27" t="inlineStr">
+        <is>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C84" s="28" t="inlineStr">
+        <is>
+          <t>Por espacio individual · placa memorial US$ 150</t>
+        </is>
+      </c>
+      <c r="D84" s="29" t="n"/>
+      <c r="E84" s="30" t="n"/>
+    </row>
+    <row r="85" ht="35" customHeight="1">
+      <c r="B85" s="23" t="inlineStr">
+        <is>
+          <t>Condiciones</t>
+        </is>
+      </c>
+      <c r="C85" s="24" t="inlineStr">
+        <is>
+          <t>Pago único o financiado según política comercial vigente. Placa memorial en el monumento al término del plazo: US$ 150.</t>
+        </is>
+      </c>
+      <c r="D85" s="25" t="n"/>
+      <c r="E85" s="26" t="n"/>
+    </row>
+    <row r="86" ht="20" customHeight="1">
+      <c r="B86" s="20" t="inlineStr">
+        <is>
+          <t>PERFIL DEL COMPRADOR</t>
+        </is>
+      </c>
+      <c r="C86" s="21" t="n"/>
+      <c r="D86" s="21" t="n"/>
+      <c r="E86" s="22" t="n"/>
+    </row>
+    <row r="87" ht="35" customHeight="1">
+      <c r="B87" s="32" t="inlineStr">
+        <is>
+          <t>Cliente objetivo</t>
+        </is>
+      </c>
+      <c r="C87" s="33" t="inlineStr">
+        <is>
+          <t>Personas con conciencia ambiental que desean que sus cenizas vuelvan a la tierra, con un lugar identificado para visitar.</t>
+        </is>
+      </c>
+      <c r="D87" s="34" t="n"/>
+      <c r="E87" s="35" t="n"/>
+    </row>
+    <row r="90" ht="30" customHeight="1">
+      <c r="B90" s="14" t="inlineStr">
+        <is>
+          <t>JARDÍN DE CENIZAS · CEREMONIAL</t>
+        </is>
+      </c>
+      <c r="C90" s="15" t="n"/>
+      <c r="D90" s="15" t="n"/>
+      <c r="E90" s="16" t="inlineStr">
+        <is>
+          <t>VG-CRE-03C</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="20" customHeight="1">
+      <c r="B91" s="17" t="inlineStr">
+        <is>
+          <t>Jardines de la Memoria · Jardín 3  ·  Destino final · Inhumación con ceremonia</t>
+        </is>
+      </c>
+      <c r="C91" s="18" t="n"/>
+      <c r="D91" s="18" t="n"/>
+      <c r="E91" s="19" t="n"/>
+    </row>
+    <row r="92" ht="20" customHeight="1">
+      <c r="B92" s="20" t="inlineStr">
+        <is>
+          <t>VISIÓN GENERAL</t>
+        </is>
+      </c>
+      <c r="C92" s="21" t="n"/>
+      <c r="D92" s="21" t="n"/>
+      <c r="E92" s="22" t="n"/>
+    </row>
+    <row r="93" ht="35" customHeight="1">
+      <c r="B93" s="23" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="C93" s="24" t="inlineStr">
+        <is>
+          <t>Jardín para inhumación de urnas de cenizas con ceremonia de agua, con fuentes como elemento central del rito de despedida.</t>
+        </is>
+      </c>
+      <c r="D93" s="25" t="n"/>
+      <c r="E93" s="26" t="n"/>
+    </row>
+    <row r="94" ht="20.5" customHeight="1">
+      <c r="B94" s="27" t="inlineStr">
+        <is>
+          <t>Capacidad / Cobertura</t>
+        </is>
+      </c>
+      <c r="C94" s="28" t="inlineStr">
+        <is>
+          <t>A definir.</t>
+        </is>
+      </c>
+      <c r="D94" s="29" t="n"/>
+      <c r="E94" s="30" t="n"/>
+    </row>
+    <row r="95" ht="20" customHeight="1">
+      <c r="B95" s="20" t="inlineStr">
+        <is>
+          <t>ESPECIFICACIONES TÉCNICAS</t>
+        </is>
+      </c>
+      <c r="C95" s="21" t="n"/>
+      <c r="D95" s="21" t="n"/>
+      <c r="E95" s="22" t="n"/>
+    </row>
+    <row r="96" ht="20.5" customHeight="1">
+      <c r="B96" s="23" t="inlineStr">
+        <is>
+          <t>Ambiente</t>
+        </is>
+      </c>
+      <c r="C96" s="24" t="inlineStr">
+        <is>
+          <t>Jardín 3</t>
+        </is>
+      </c>
+      <c r="D96" s="25" t="n"/>
+      <c r="E96" s="26" t="n"/>
+    </row>
+    <row r="97" ht="20.5" customHeight="1">
+      <c r="B97" s="27" t="inlineStr">
+        <is>
+          <t>Elemento central</t>
+        </is>
+      </c>
+      <c r="C97" s="28" t="inlineStr">
+        <is>
+          <t>Fuente de agua para la ceremonia</t>
+        </is>
+      </c>
+      <c r="D97" s="29" t="n"/>
+      <c r="E97" s="30" t="n"/>
+    </row>
+    <row r="98" ht="20.5" customHeight="1">
+      <c r="B98" s="23" t="inlineStr">
+        <is>
+          <t>Entorno</t>
+        </is>
+      </c>
+      <c r="C98" s="24" t="inlineStr">
+        <is>
+          <t>Barrera visual que separa el jardín del crematorio</t>
+        </is>
+      </c>
+      <c r="D98" s="25" t="n"/>
+      <c r="E98" s="26" t="n"/>
+    </row>
+    <row r="99" ht="35" customHeight="1">
+      <c r="B99" s="27" t="inlineStr">
+        <is>
+          <t>Servicios incluidos</t>
+        </is>
+      </c>
+      <c r="C99" s="28" t="inlineStr">
+        <is>
+          <t>• Inhumación de urnas de cenizas
+• Ceremonia con agua en fuente</t>
+        </is>
+      </c>
+      <c r="D99" s="29" t="n"/>
+      <c r="E99" s="30" t="n"/>
+    </row>
+    <row r="100" ht="20" customHeight="1">
+      <c r="B100" s="20" t="inlineStr">
+        <is>
+          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
+        </is>
+      </c>
+      <c r="C100" s="21" t="n"/>
+      <c r="D100" s="21" t="n"/>
+      <c r="E100" s="22" t="n"/>
+    </row>
+    <row r="101" ht="26.5" customHeight="1">
+      <c r="B101" s="23" t="inlineStr">
+        <is>
+          <t>Precio sugerido</t>
+        </is>
+      </c>
+      <c r="C101" s="31" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
       <c r="D101" s="25" t="n"/>
       <c r="E101" s="26" t="n"/>
     </row>
-    <row r="102" ht="20" customHeight="1">
-      <c r="B102" s="20" t="inlineStr">
-        <is>
-          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
-        </is>
-      </c>
-      <c r="C102" s="21" t="n"/>
-      <c r="D102" s="21" t="n"/>
-      <c r="E102" s="22" t="n"/>
-    </row>
-    <row r="103" ht="26.5" customHeight="1">
+    <row r="102" ht="20.5" customHeight="1">
+      <c r="B102" s="27" t="inlineStr">
+        <is>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C102" s="28" t="inlineStr">
+        <is>
+          <t>Producto en definición</t>
+        </is>
+      </c>
+      <c r="D102" s="29" t="n"/>
+      <c r="E102" s="30" t="n"/>
+    </row>
+    <row r="103" ht="20.5" customHeight="1">
       <c r="B103" s="23" t="inlineStr">
         <is>
-          <t>Precio sugerido</t>
-        </is>
-      </c>
-      <c r="C103" s="31" t="inlineStr">
-        <is>
-          <t>US$ 600</t>
+          <t>Condiciones</t>
+        </is>
+      </c>
+      <c r="C103" s="24" t="inlineStr">
+        <is>
+          <t>A definir.</t>
         </is>
       </c>
       <c r="D103" s="25" t="n"/>
       <c r="E103" s="26" t="n"/>
     </row>
-    <row r="104" ht="20.5" customHeight="1">
-      <c r="B104" s="27" t="inlineStr">
-        <is>
-          <t>Base de precio</t>
-        </is>
-      </c>
-      <c r="C104" s="28" t="inlineStr">
-        <is>
-          <t>Por espacio individual · placa memorial US$ 150</t>
-        </is>
-      </c>
-      <c r="D104" s="29" t="n"/>
-      <c r="E104" s="30" t="n"/>
+    <row r="104" ht="20" customHeight="1">
+      <c r="B104" s="20" t="inlineStr">
+        <is>
+          <t>PERFIL DEL COMPRADOR</t>
+        </is>
+      </c>
+      <c r="C104" s="21" t="n"/>
+      <c r="D104" s="21" t="n"/>
+      <c r="E104" s="22" t="n"/>
     </row>
     <row r="105" ht="35" customHeight="1">
-      <c r="B105" s="23" t="inlineStr">
-        <is>
-          <t>Condiciones</t>
-        </is>
-      </c>
-      <c r="C105" s="24" t="inlineStr">
-        <is>
-          <t>Pago único o financiado según política comercial vigente. Placa memorial en el monumento al término del plazo: US$ 150.</t>
-        </is>
-      </c>
-      <c r="D105" s="25" t="n"/>
-      <c r="E105" s="26" t="n"/>
-    </row>
-    <row r="106" ht="20" customHeight="1">
-      <c r="B106" s="20" t="inlineStr">
-        <is>
-          <t>PERFIL DEL COMPRADOR</t>
-        </is>
-      </c>
-      <c r="C106" s="21" t="n"/>
-      <c r="D106" s="21" t="n"/>
-      <c r="E106" s="22" t="n"/>
-    </row>
-    <row r="107" ht="35" customHeight="1">
-      <c r="B107" s="32" t="inlineStr">
+      <c r="B105" s="32" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C107" s="33" t="inlineStr">
-        <is>
-          <t>Personas con conciencia ambiental que desean que sus cenizas vuelvan a la tierra, con un lugar identificado para visitar.</t>
-        </is>
-      </c>
-      <c r="D107" s="34" t="n"/>
-      <c r="E107" s="35" t="n"/>
-    </row>
-    <row r="110" ht="30" customHeight="1">
-      <c r="B110" s="14" t="inlineStr">
-        <is>
-          <t>JARDÍN DE CENIZAS · CEREMONIAL</t>
-        </is>
-      </c>
-      <c r="C110" s="15" t="n"/>
-      <c r="D110" s="15" t="n"/>
-      <c r="E110" s="16" t="inlineStr">
-        <is>
-          <t>VG-CRE-03C</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" ht="20" customHeight="1">
-      <c r="B111" s="17" t="inlineStr">
-        <is>
-          <t>Jardines de la Memoria · Jardín 3  ·  Destino final · Inhumación con ceremonia</t>
-        </is>
-      </c>
-      <c r="C111" s="18" t="n"/>
-      <c r="D111" s="18" t="n"/>
-      <c r="E111" s="19" t="n"/>
-    </row>
-    <row r="112" ht="20" customHeight="1">
-      <c r="B112" s="20" t="inlineStr">
+      <c r="C105" s="33" t="inlineStr">
+        <is>
+          <t>Familias que valoran un rito de despedida simbólico y un entorno contemplativo.</t>
+        </is>
+      </c>
+      <c r="D105" s="34" t="n"/>
+      <c r="E105" s="35" t="n"/>
+    </row>
+    <row r="108" ht="30" customHeight="1">
+      <c r="B108" s="14" t="inlineStr">
+        <is>
+          <t>JARDÍN DE MASCOTAS</t>
+        </is>
+      </c>
+      <c r="C108" s="15" t="n"/>
+      <c r="D108" s="15" t="n"/>
+      <c r="E108" s="16" t="inlineStr">
+        <is>
+          <t>VG-CRE-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="20" customHeight="1">
+      <c r="B109" s="17" t="inlineStr">
+        <is>
+          <t>Jardines de la Memoria · Mascotas  ·  Mascotas · Inhumación ecológica</t>
+        </is>
+      </c>
+      <c r="C109" s="18" t="n"/>
+      <c r="D109" s="18" t="n"/>
+      <c r="E109" s="19" t="n"/>
+    </row>
+    <row r="110" ht="20" customHeight="1">
+      <c r="B110" s="20" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C112" s="21" t="n"/>
-      <c r="D112" s="21" t="n"/>
-      <c r="E112" s="22" t="n"/>
-    </row>
-    <row r="113" ht="35" customHeight="1">
-      <c r="B113" s="23" t="inlineStr">
+      <c r="C110" s="21" t="n"/>
+      <c r="D110" s="21" t="n"/>
+      <c r="E110" s="22" t="n"/>
+    </row>
+    <row r="111" ht="35" customHeight="1">
+      <c r="B111" s="23" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C113" s="24" t="inlineStr">
-        <is>
-          <t>Jardín para inhumación de urnas de cenizas con ceremonia de agua, con fuentes como elemento central del rito de despedida.</t>
-        </is>
-      </c>
-      <c r="D113" s="25" t="n"/>
-      <c r="E113" s="26" t="n"/>
+      <c r="C111" s="24" t="inlineStr">
+        <is>
+          <t>Jardín para inhumación ecológica de cenizas de mascotas: la urna biodegradable se entierra directamente en el suelo y se identifica con una placa de madera.</t>
+        </is>
+      </c>
+      <c r="D111" s="25" t="n"/>
+      <c r="E111" s="26" t="n"/>
+    </row>
+    <row r="112" ht="20.5" customHeight="1">
+      <c r="B112" s="27" t="inlineStr">
+        <is>
+          <t>Capacidad / Cobertura</t>
+        </is>
+      </c>
+      <c r="C112" s="28" t="inlineStr">
+        <is>
+          <t>Individual (una mascota por servicio).</t>
+        </is>
+      </c>
+      <c r="D112" s="29" t="n"/>
+      <c r="E112" s="30" t="n"/>
+    </row>
+    <row r="113" ht="20" customHeight="1">
+      <c r="B113" s="20" t="inlineStr">
+        <is>
+          <t>ESPECIFICACIONES TÉCNICAS</t>
+        </is>
+      </c>
+      <c r="C113" s="21" t="n"/>
+      <c r="D113" s="21" t="n"/>
+      <c r="E113" s="22" t="n"/>
     </row>
     <row r="114" ht="20.5" customHeight="1">
-      <c r="B114" s="27" t="inlineStr">
-        <is>
-          <t>Capacidad / Cobertura</t>
-        </is>
-      </c>
-      <c r="C114" s="28" t="inlineStr">
-        <is>
-          <t>A definir.</t>
-        </is>
-      </c>
-      <c r="D114" s="29" t="n"/>
-      <c r="E114" s="30" t="n"/>
-    </row>
-    <row r="115" ht="20" customHeight="1">
-      <c r="B115" s="20" t="inlineStr">
-        <is>
-          <t>ESPECIFICACIONES TÉCNICAS</t>
-        </is>
-      </c>
-      <c r="C115" s="21" t="n"/>
-      <c r="D115" s="21" t="n"/>
-      <c r="E115" s="22" t="n"/>
+      <c r="B114" s="23" t="inlineStr">
+        <is>
+          <t>Tipo de producto</t>
+        </is>
+      </c>
+      <c r="C114" s="24" t="inlineStr">
+        <is>
+          <t>Servicio de pago único</t>
+        </is>
+      </c>
+      <c r="D114" s="25" t="n"/>
+      <c r="E114" s="26" t="n"/>
+    </row>
+    <row r="115" ht="20.5" customHeight="1">
+      <c r="B115" s="27" t="inlineStr">
+        <is>
+          <t>Espacio por urna</t>
+        </is>
+      </c>
+      <c r="C115" s="28" t="inlineStr">
+        <is>
+          <t>15 × 20 cm o 15 × 30 cm, según el tamaño de la urna</t>
+        </is>
+      </c>
+      <c r="D115" s="29" t="n"/>
+      <c r="E115" s="30" t="n"/>
     </row>
     <row r="116" ht="20.5" customHeight="1">
       <c r="B116" s="23" t="inlineStr">
         <is>
-          <t>Ambiente</t>
+          <t>Urna</t>
         </is>
       </c>
       <c r="C116" s="24" t="inlineStr">
         <is>
-          <t>Jardín 3</t>
+          <t>Biodegradable; se integra al suelo</t>
         </is>
       </c>
       <c r="D116" s="25" t="n"/>
@@ -2532,285 +2479,52 @@
     <row r="117" ht="20.5" customHeight="1">
       <c r="B117" s="27" t="inlineStr">
         <is>
-          <t>Elemento central</t>
+          <t>Identificación</t>
         </is>
       </c>
       <c r="C117" s="28" t="inlineStr">
         <is>
-          <t>Fuente de agua para la ceremonia</t>
+          <t>Placa de madera de 20 cm</t>
         </is>
       </c>
       <c r="D117" s="29" t="n"/>
       <c r="E117" s="30" t="n"/>
     </row>
-    <row r="118" ht="20.5" customHeight="1">
+    <row r="118" ht="35" customHeight="1">
       <c r="B118" s="23" t="inlineStr">
         <is>
-          <t>Entorno</t>
+          <t>Permanencia</t>
         </is>
       </c>
       <c r="C118" s="24" t="inlineStr">
         <is>
-          <t>Barrera visual que separa el jardín del crematorio</t>
+          <t>3 años; luego el nombre pasa a una placa memorial en el monumento y el espacio se reutiliza</t>
         </is>
       </c>
       <c r="D118" s="25" t="n"/>
       <c r="E118" s="26" t="n"/>
     </row>
-    <row r="119" ht="35" customHeight="1">
+    <row r="119" ht="20.5" customHeight="1">
       <c r="B119" s="27" t="inlineStr">
         <is>
-          <t>Servicios incluidos</t>
+          <t>Placa memorial</t>
         </is>
       </c>
       <c r="C119" s="28" t="inlineStr">
         <is>
-          <t>• Inhumación de urnas de cenizas
-• Ceremonia con agua en fuente</t>
+          <t>US$ 50</t>
         </is>
       </c>
       <c r="D119" s="29" t="n"/>
       <c r="E119" s="30" t="n"/>
     </row>
-    <row r="120" ht="20" customHeight="1">
-      <c r="B120" s="20" t="inlineStr">
-        <is>
-          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
-        </is>
-      </c>
-      <c r="C120" s="21" t="n"/>
-      <c r="D120" s="21" t="n"/>
-      <c r="E120" s="22" t="n"/>
-    </row>
-    <row r="121" ht="26.5" customHeight="1">
-      <c r="B121" s="23" t="inlineStr">
-        <is>
-          <t>Precio sugerido</t>
-        </is>
-      </c>
-      <c r="C121" s="31" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-      <c r="D121" s="25" t="n"/>
-      <c r="E121" s="26" t="n"/>
-    </row>
-    <row r="122" ht="20.5" customHeight="1">
-      <c r="B122" s="27" t="inlineStr">
-        <is>
-          <t>Base de precio</t>
-        </is>
-      </c>
-      <c r="C122" s="28" t="inlineStr">
-        <is>
-          <t>Producto en definición</t>
-        </is>
-      </c>
-      <c r="D122" s="29" t="n"/>
-      <c r="E122" s="30" t="n"/>
-    </row>
-    <row r="123" ht="20.5" customHeight="1">
-      <c r="B123" s="23" t="inlineStr">
-        <is>
-          <t>Condiciones</t>
-        </is>
-      </c>
-      <c r="C123" s="24" t="inlineStr">
-        <is>
-          <t>A definir.</t>
-        </is>
-      </c>
-      <c r="D123" s="25" t="n"/>
-      <c r="E123" s="26" t="n"/>
-    </row>
-    <row r="124" ht="20" customHeight="1">
-      <c r="B124" s="20" t="inlineStr">
-        <is>
-          <t>PERFIL DEL COMPRADOR</t>
-        </is>
-      </c>
-      <c r="C124" s="21" t="n"/>
-      <c r="D124" s="21" t="n"/>
-      <c r="E124" s="22" t="n"/>
-    </row>
-    <row r="125" ht="35" customHeight="1">
-      <c r="B125" s="32" t="inlineStr">
-        <is>
-          <t>Cliente objetivo</t>
-        </is>
-      </c>
-      <c r="C125" s="33" t="inlineStr">
-        <is>
-          <t>Familias que valoran un rito de despedida simbólico y un entorno contemplativo.</t>
-        </is>
-      </c>
-      <c r="D125" s="34" t="n"/>
-      <c r="E125" s="35" t="n"/>
-    </row>
-    <row r="128" ht="30" customHeight="1">
-      <c r="B128" s="14" t="inlineStr">
-        <is>
-          <t>JARDÍN DE MASCOTAS</t>
-        </is>
-      </c>
-      <c r="C128" s="15" t="n"/>
-      <c r="D128" s="15" t="n"/>
-      <c r="E128" s="16" t="inlineStr">
-        <is>
-          <t>VG-CRE-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="129" ht="20" customHeight="1">
-      <c r="B129" s="17" t="inlineStr">
-        <is>
-          <t>Jardines de la Memoria · Mascotas  ·  Mascotas · Inhumación ecológica</t>
-        </is>
-      </c>
-      <c r="C129" s="18" t="n"/>
-      <c r="D129" s="18" t="n"/>
-      <c r="E129" s="19" t="n"/>
-    </row>
-    <row r="130" ht="20" customHeight="1">
-      <c r="B130" s="20" t="inlineStr">
-        <is>
-          <t>VISIÓN GENERAL</t>
-        </is>
-      </c>
-      <c r="C130" s="21" t="n"/>
-      <c r="D130" s="21" t="n"/>
-      <c r="E130" s="22" t="n"/>
-    </row>
-    <row r="131" ht="35" customHeight="1">
-      <c r="B131" s="23" t="inlineStr">
-        <is>
-          <t>Concepto</t>
-        </is>
-      </c>
-      <c r="C131" s="24" t="inlineStr">
-        <is>
-          <t>Jardín para inhumación ecológica de cenizas de mascotas: la urna biodegradable se entierra directamente en el suelo y se identifica con una placa de madera.</t>
-        </is>
-      </c>
-      <c r="D131" s="25" t="n"/>
-      <c r="E131" s="26" t="n"/>
-    </row>
-    <row r="132" ht="20.5" customHeight="1">
-      <c r="B132" s="27" t="inlineStr">
-        <is>
-          <t>Capacidad / Cobertura</t>
-        </is>
-      </c>
-      <c r="C132" s="28" t="inlineStr">
-        <is>
-          <t>Individual (una mascota por servicio).</t>
-        </is>
-      </c>
-      <c r="D132" s="29" t="n"/>
-      <c r="E132" s="30" t="n"/>
-    </row>
-    <row r="133" ht="20" customHeight="1">
-      <c r="B133" s="20" t="inlineStr">
-        <is>
-          <t>ESPECIFICACIONES TÉCNICAS</t>
-        </is>
-      </c>
-      <c r="C133" s="21" t="n"/>
-      <c r="D133" s="21" t="n"/>
-      <c r="E133" s="22" t="n"/>
-    </row>
-    <row r="134" ht="20.5" customHeight="1">
-      <c r="B134" s="23" t="inlineStr">
-        <is>
-          <t>Tipo de producto</t>
-        </is>
-      </c>
-      <c r="C134" s="24" t="inlineStr">
-        <is>
-          <t>Servicio de pago único</t>
-        </is>
-      </c>
-      <c r="D134" s="25" t="n"/>
-      <c r="E134" s="26" t="n"/>
-    </row>
-    <row r="135" ht="20.5" customHeight="1">
-      <c r="B135" s="27" t="inlineStr">
-        <is>
-          <t>Espacio por urna</t>
-        </is>
-      </c>
-      <c r="C135" s="28" t="inlineStr">
-        <is>
-          <t>15 × 20 cm o 15 × 30 cm, según el tamaño de la urna</t>
-        </is>
-      </c>
-      <c r="D135" s="29" t="n"/>
-      <c r="E135" s="30" t="n"/>
-    </row>
-    <row r="136" ht="20.5" customHeight="1">
-      <c r="B136" s="23" t="inlineStr">
-        <is>
-          <t>Urna</t>
-        </is>
-      </c>
-      <c r="C136" s="24" t="inlineStr">
-        <is>
-          <t>Biodegradable; se integra al suelo</t>
-        </is>
-      </c>
-      <c r="D136" s="25" t="n"/>
-      <c r="E136" s="26" t="n"/>
-    </row>
-    <row r="137" ht="20.5" customHeight="1">
-      <c r="B137" s="27" t="inlineStr">
-        <is>
-          <t>Identificación</t>
-        </is>
-      </c>
-      <c r="C137" s="28" t="inlineStr">
-        <is>
-          <t>Placa de madera de 20 cm</t>
-        </is>
-      </c>
-      <c r="D137" s="29" t="n"/>
-      <c r="E137" s="30" t="n"/>
-    </row>
-    <row r="138" ht="35" customHeight="1">
-      <c r="B138" s="23" t="inlineStr">
-        <is>
-          <t>Permanencia</t>
-        </is>
-      </c>
-      <c r="C138" s="24" t="inlineStr">
-        <is>
-          <t>3 años; luego el nombre pasa a una placa memorial en el monumento y el espacio se reutiliza</t>
-        </is>
-      </c>
-      <c r="D138" s="25" t="n"/>
-      <c r="E138" s="26" t="n"/>
-    </row>
-    <row r="139" ht="20.5" customHeight="1">
-      <c r="B139" s="27" t="inlineStr">
-        <is>
-          <t>Placa memorial</t>
-        </is>
-      </c>
-      <c r="C139" s="28" t="inlineStr">
-        <is>
-          <t>US$ 50</t>
-        </is>
-      </c>
-      <c r="D139" s="29" t="n"/>
-      <c r="E139" s="30" t="n"/>
-    </row>
-    <row r="140" ht="64" customHeight="1">
-      <c r="B140" s="23" t="inlineStr">
+    <row r="120" ht="64" customHeight="1">
+      <c r="B120" s="23" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C140" s="24" t="inlineStr">
+      <c r="C120" s="24" t="inlineStr">
         <is>
           <t>• Inhumación ecológica de la urna en el jardín
 • Placa de madera de 20 cm para identificación
@@ -2818,230 +2532,211 @@
 • Cremación de la mascota (opción Jardín + Cremación)</t>
         </is>
       </c>
-      <c r="D140" s="25" t="n"/>
-      <c r="E140" s="26" t="n"/>
-    </row>
-    <row r="141" ht="20" customHeight="1">
-      <c r="B141" s="20" t="inlineStr">
+      <c r="D120" s="25" t="n"/>
+      <c r="E120" s="26" t="n"/>
+    </row>
+    <row r="121" ht="20" customHeight="1">
+      <c r="B121" s="20" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C141" s="21" t="n"/>
-      <c r="D141" s="21" t="n"/>
-      <c r="E141" s="22" t="n"/>
-    </row>
-    <row r="142" ht="26.5" customHeight="1">
-      <c r="B142" s="23" t="inlineStr">
+      <c r="C121" s="21" t="n"/>
+      <c r="D121" s="21" t="n"/>
+      <c r="E121" s="22" t="n"/>
+    </row>
+    <row r="122" ht="26.5" customHeight="1">
+      <c r="B122" s="23" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C142" s="31" t="inlineStr">
+      <c r="C122" s="31" t="inlineStr">
         <is>
           <t>US$ 350 / US$ 500</t>
         </is>
       </c>
-      <c r="D142" s="25" t="n"/>
-      <c r="E142" s="26" t="n"/>
-    </row>
-    <row r="143" ht="20.5" customHeight="1">
-      <c r="B143" s="27" t="inlineStr">
+      <c r="D122" s="25" t="n"/>
+      <c r="E122" s="26" t="n"/>
+    </row>
+    <row r="123" ht="20.5" customHeight="1">
+      <c r="B123" s="27" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C143" s="28" t="inlineStr">
+      <c r="C123" s="28" t="inlineStr">
         <is>
           <t>US$ 350 solo jardín · US$ 500 jardín + cremación</t>
         </is>
       </c>
-      <c r="D143" s="29" t="n"/>
-      <c r="E143" s="30" t="n"/>
-    </row>
-    <row r="144" ht="35" customHeight="1">
-      <c r="B144" s="23" t="inlineStr">
+      <c r="D123" s="29" t="n"/>
+      <c r="E123" s="30" t="n"/>
+    </row>
+    <row r="124" ht="35" customHeight="1">
+      <c r="B124" s="23" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C144" s="24" t="inlineStr">
+      <c r="C124" s="24" t="inlineStr">
         <is>
           <t>Pago único; puede contratarse como adicional al plan funerario. Placa memorial en el monumento al término del plazo: US$ 50.</t>
         </is>
       </c>
-      <c r="D144" s="25" t="n"/>
-      <c r="E144" s="26" t="n"/>
-    </row>
-    <row r="145" ht="20" customHeight="1">
-      <c r="B145" s="20" t="inlineStr">
+      <c r="D124" s="25" t="n"/>
+      <c r="E124" s="26" t="n"/>
+    </row>
+    <row r="125" ht="20" customHeight="1">
+      <c r="B125" s="20" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C145" s="21" t="n"/>
-      <c r="D145" s="21" t="n"/>
-      <c r="E145" s="22" t="n"/>
-    </row>
-    <row r="146" ht="20.5" customHeight="1">
-      <c r="B146" s="32" t="inlineStr">
+      <c r="C125" s="21" t="n"/>
+      <c r="D125" s="21" t="n"/>
+      <c r="E125" s="22" t="n"/>
+    </row>
+    <row r="126" ht="20.5" customHeight="1">
+      <c r="B126" s="32" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C146" s="33" t="inlineStr">
+      <c r="C126" s="33" t="inlineStr">
         <is>
           <t>Familias que consideran a su mascota parte del hogar y desean un cierre digno.</t>
         </is>
       </c>
-      <c r="D146" s="34" t="n"/>
-      <c r="E146" s="35" t="n"/>
+      <c r="D126" s="34" t="n"/>
+      <c r="E126" s="35" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="133">
-    <mergeCell ref="C142:E142"/>
+  <mergeCells count="115">
     <mergeCell ref="C31:E31"/>
     <mergeCell ref="C80:E80"/>
     <mergeCell ref="B68:E68"/>
     <mergeCell ref="C40:E40"/>
-    <mergeCell ref="C51:E51"/>
-    <mergeCell ref="C95:E95"/>
     <mergeCell ref="C60:E60"/>
+    <mergeCell ref="B110:E110"/>
+    <mergeCell ref="C71:E71"/>
+    <mergeCell ref="B108:D108"/>
+    <mergeCell ref="B113:E113"/>
     <mergeCell ref="C123:E123"/>
+    <mergeCell ref="B91:E91"/>
+    <mergeCell ref="B100:E100"/>
+    <mergeCell ref="B109:E109"/>
     <mergeCell ref="B47:E47"/>
     <mergeCell ref="C7:E7"/>
-    <mergeCell ref="C91:E91"/>
-    <mergeCell ref="B141:E141"/>
-    <mergeCell ref="B115:E115"/>
-    <mergeCell ref="B102:E102"/>
     <mergeCell ref="C57:E57"/>
-    <mergeCell ref="C140:E140"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="B21:E21"/>
     <mergeCell ref="C18:E18"/>
     <mergeCell ref="C49:E49"/>
+    <mergeCell ref="B86:E86"/>
     <mergeCell ref="C101:E101"/>
     <mergeCell ref="C77:E77"/>
     <mergeCell ref="C34:E34"/>
-    <mergeCell ref="C42:E42"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="C74:E74"/>
-    <mergeCell ref="B112:E112"/>
+    <mergeCell ref="C126:E126"/>
+    <mergeCell ref="B69:E69"/>
+    <mergeCell ref="B38:E38"/>
     <mergeCell ref="C20:E20"/>
-    <mergeCell ref="C113:E113"/>
     <mergeCell ref="C103:E103"/>
-    <mergeCell ref="C143:E143"/>
+    <mergeCell ref="C85:E85"/>
+    <mergeCell ref="C112:E112"/>
     <mergeCell ref="C99:E99"/>
     <mergeCell ref="C94:E94"/>
     <mergeCell ref="C118:E118"/>
     <mergeCell ref="C75:E75"/>
     <mergeCell ref="C84:E84"/>
     <mergeCell ref="C22:E22"/>
+    <mergeCell ref="B104:E104"/>
     <mergeCell ref="C114:E114"/>
-    <mergeCell ref="C59:E59"/>
+    <mergeCell ref="B51:E51"/>
     <mergeCell ref="C12:E12"/>
+    <mergeCell ref="B63:E63"/>
     <mergeCell ref="B26:E26"/>
-    <mergeCell ref="B41:E41"/>
-    <mergeCell ref="B50:E50"/>
     <mergeCell ref="C52:E52"/>
-    <mergeCell ref="B106:E106"/>
-    <mergeCell ref="B129:E129"/>
     <mergeCell ref="C61:E61"/>
     <mergeCell ref="C39:E39"/>
     <mergeCell ref="B16:E16"/>
     <mergeCell ref="C70:E70"/>
-    <mergeCell ref="C48:E48"/>
     <mergeCell ref="C32:E32"/>
-    <mergeCell ref="C38:E38"/>
     <mergeCell ref="C81:E81"/>
-    <mergeCell ref="C125:E125"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="C13:E13"/>
-    <mergeCell ref="B45:D45"/>
-    <mergeCell ref="B110:D110"/>
-    <mergeCell ref="C131:E131"/>
-    <mergeCell ref="B130:E130"/>
+    <mergeCell ref="C87:E87"/>
     <mergeCell ref="C15:E15"/>
-    <mergeCell ref="B67:E67"/>
     <mergeCell ref="C33:E33"/>
-    <mergeCell ref="C104:E104"/>
     <mergeCell ref="C116:E116"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="C79:E79"/>
     <mergeCell ref="C73:E73"/>
-    <mergeCell ref="B37:E37"/>
     <mergeCell ref="C35:E35"/>
-    <mergeCell ref="C63:E63"/>
-    <mergeCell ref="C121:E121"/>
     <mergeCell ref="C10:E10"/>
+    <mergeCell ref="C50:E50"/>
     <mergeCell ref="C117:E117"/>
     <mergeCell ref="C55:E55"/>
     <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B89:E89"/>
-    <mergeCell ref="B87:D87"/>
+    <mergeCell ref="B95:E95"/>
+    <mergeCell ref="C115:E115"/>
     <mergeCell ref="C36:E36"/>
     <mergeCell ref="C11:E11"/>
-    <mergeCell ref="B79:E79"/>
-    <mergeCell ref="B128:D128"/>
-    <mergeCell ref="C135:E135"/>
-    <mergeCell ref="C144:E144"/>
+    <mergeCell ref="B72:E72"/>
     <mergeCell ref="C122:E122"/>
-    <mergeCell ref="C72:E72"/>
+    <mergeCell ref="B121:E121"/>
     <mergeCell ref="C28:E28"/>
-    <mergeCell ref="B71:E71"/>
-    <mergeCell ref="B58:E58"/>
-    <mergeCell ref="C69:E69"/>
+    <mergeCell ref="C37:E37"/>
     <mergeCell ref="C96:E96"/>
     <mergeCell ref="C78:E78"/>
-    <mergeCell ref="C136:E136"/>
-    <mergeCell ref="B120:E120"/>
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="B25:D25"/>
+    <mergeCell ref="B42:E42"/>
+    <mergeCell ref="C62:E62"/>
     <mergeCell ref="C14:E14"/>
-    <mergeCell ref="B66:D66"/>
     <mergeCell ref="C98:E98"/>
-    <mergeCell ref="C107:E107"/>
+    <mergeCell ref="C64:E64"/>
     <mergeCell ref="C54:E54"/>
     <mergeCell ref="B9:E9"/>
-    <mergeCell ref="C137:E137"/>
-    <mergeCell ref="C134:E134"/>
-    <mergeCell ref="C146:E146"/>
-    <mergeCell ref="B83:E83"/>
+    <mergeCell ref="C41:E41"/>
+    <mergeCell ref="B67:D67"/>
     <mergeCell ref="C93:E93"/>
+    <mergeCell ref="C124:E124"/>
     <mergeCell ref="B92:E92"/>
     <mergeCell ref="B30:E30"/>
-    <mergeCell ref="B124:E124"/>
     <mergeCell ref="C56:E56"/>
     <mergeCell ref="B5:E5"/>
-    <mergeCell ref="C90:E90"/>
     <mergeCell ref="C105:E105"/>
-    <mergeCell ref="B133:E133"/>
-    <mergeCell ref="C139:E139"/>
-    <mergeCell ref="C138:E138"/>
+    <mergeCell ref="C43:E43"/>
     <mergeCell ref="C76:E76"/>
-    <mergeCell ref="C132:E132"/>
+    <mergeCell ref="C120:E120"/>
     <mergeCell ref="C119:E119"/>
     <mergeCell ref="C8:E8"/>
-    <mergeCell ref="B62:E62"/>
     <mergeCell ref="C17:E17"/>
-    <mergeCell ref="C82:E82"/>
-    <mergeCell ref="B46:E46"/>
+    <mergeCell ref="B59:E59"/>
+    <mergeCell ref="B125:E125"/>
     <mergeCell ref="C19:E19"/>
     <mergeCell ref="C53:E53"/>
-    <mergeCell ref="B111:E111"/>
-    <mergeCell ref="B145:E145"/>
-    <mergeCell ref="B88:E88"/>
+    <mergeCell ref="C102:E102"/>
+    <mergeCell ref="C111:E111"/>
+    <mergeCell ref="B48:E48"/>
+    <mergeCell ref="C83:E83"/>
+    <mergeCell ref="C58:E58"/>
+    <mergeCell ref="B90:D90"/>
+    <mergeCell ref="B82:E82"/>
     <mergeCell ref="C97:E97"/>
     <mergeCell ref="C29:E29"/>
-    <mergeCell ref="C100:E100"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
-  <rowBreaks count="6" manualBreakCount="6">
+  <rowBreaks count="5" manualBreakCount="5">
     <brk id="23" min="0" max="16383" man="1"/>
-    <brk id="43" min="0" max="16383" man="1"/>
-    <brk id="64" min="0" max="16383" man="1"/>
-    <brk id="85" min="0" max="16383" man="1"/>
-    <brk id="108" min="0" max="16383" man="1"/>
-    <brk id="126" min="0" max="16383" man="1"/>
+    <brk id="44" min="0" max="16383" man="1"/>
+    <brk id="65" min="0" max="16383" man="1"/>
+    <brk id="88" min="0" max="16383" man="1"/>
+    <brk id="106" min="0" max="16383" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Corrige subtítulo duplicado en Jardín de Mascotas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111i7vn9WWo4QxCQbucWbrF
</commit_message>
<xml_diff>
--- a/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
+++ b/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
@@ -1050,7 +1050,7 @@
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>Mascotas · Inhumación ecológica</t>
+          <t>Destino final · Inhumación ecológica</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
@@ -2379,7 +2379,7 @@
     <row r="109" ht="20" customHeight="1">
       <c r="B109" s="17" t="inlineStr">
         <is>
-          <t>Jardines de la Memoria · Mascotas  ·  Mascotas · Inhumación ecológica</t>
+          <t>Jardines de la Memoria · Mascotas  ·  Destino final · Inhumación ecológica</t>
         </is>
       </c>
       <c r="C109" s="18" t="n"/>

</xml_diff>

<commit_message>
Mueve Jardín Ceremonial al final y lo destaca como próximo lanzamiento
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111i7vn9WWo4QxCQbucWbrF
</commit_message>
<xml_diff>
--- a/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
+++ b/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
@@ -13,7 +13,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tabla Gral. - Visión Comercial'!$A$4:$I$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Tabla Gral. - Visión Comercial'!$4:$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Ficha Técnica Consolidada'!$A$1:$F$127</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Ficha Técnica Consolidada'!$A$1:$F$128</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -109,7 +109,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -146,8 +146,20 @@
         <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBF3E1"/>
+        <bgColor rgb="00FBF3E1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D4AF37"/>
+        <bgColor rgb="00D4AF37"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="12">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -178,6 +190,14 @@
       </top>
       <bottom style="thin">
         <color rgb="00D5DCE4"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="medium">
+        <color rgb="00C5A059"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00C5A059"/>
       </bottom>
     </border>
     <border>
@@ -256,7 +276,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -291,56 +311,73 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -988,82 +1025,33 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="49.5" customHeight="1">
+    <row r="9" ht="93" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>VG-CRE-03C</t>
+          <t>VG-CRE-04</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Jardín de Cenizas · Ceremonial</t>
+          <t>Jardín de Mascotas</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Destino final · Inhumación con ceremonia</t>
+          <t>Destino final · Inhumación ecológica</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Jardín para inhumación de urnas de cenizas con ceremonia de agua, con fuentes como elemento central del rito de despedida.</t>
+          <t>Jardín para inhumación ecológica de cenizas de mascotas: la urna biodegradable se entierra directamente en el suelo y se identifica con una placa de madera.</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>A definir.</t>
+          <t>Individual (una mascota por servicio).</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>• Inhumación de urnas de cenizas
-• Ceremonia con agua en fuente</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>Familias que valoran un rito de despedida simbólico y un entorno contemplativo.</t>
-        </is>
-      </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>A definir
-(Producto en definición)</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>A definir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="93" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>VG-CRE-04</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>Jardín de Mascotas</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>Destino final · Inhumación ecológica</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="inlineStr">
-        <is>
-          <t>Jardín para inhumación ecológica de cenizas de mascotas: la urna biodegradable se entierra directamente en el suelo y se identifica con una placa de madera.</t>
-        </is>
-      </c>
-      <c r="E10" s="10" t="inlineStr">
-        <is>
-          <t>Individual (una mascota por servicio).</t>
-        </is>
-      </c>
-      <c r="F10" s="10" t="inlineStr">
         <is>
           <t>• Inhumación ecológica de la urna en el jardín
 • Placa de madera de 20 cm para identificación
@@ -1071,20 +1059,70 @@
 • Cremación de la mascota (opción Jardín + Cremación)</t>
         </is>
       </c>
-      <c r="G10" s="10" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>Familias que consideran a su mascota parte del hogar y desean un cierre digno.</t>
         </is>
       </c>
-      <c r="H10" s="11" t="inlineStr">
+      <c r="H9" s="7" t="inlineStr">
         <is>
           <t>US$ 350 / US$ 500
 (US$ 350 solo jardín · US$ 500 jardín + cremación)</t>
         </is>
       </c>
-      <c r="I10" s="10" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>Pago único; puede contratarse como adicional al plan funerario. Placa memorial en el monumento al término del plazo: US$ 50.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="49.5" customHeight="1">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>VG-CRE-03C</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Jardín de Cenizas · Ceremonial
+★ PRÓXIMO LANZAMIENTO</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>Destino final · Inhumación con ceremonia</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Jardín para inhumación de urnas de cenizas con ceremonia de agua, con fuentes como elemento central del rito de despedida.</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>A definir.</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>• Inhumación de urnas de cenizas
+• Ceremonia con agua en fuente</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>Familias que valoran un rito de despedida simbólico y un entorno contemplativo.</t>
+        </is>
+      </c>
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>A definir
+(Producto en definición)</t>
+        </is>
+      </c>
+      <c r="I10" s="14" t="inlineStr">
+        <is>
+          <t>A definir.</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:E126"/>
+  <dimension ref="B1:E127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1118,168 +1156,168 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="16" t="inlineStr">
         <is>
           <t>FICHA TÉCNICA CONSOLIDADA  ·  LA AUXILIADORA · VANGRUPO</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="17" t="inlineStr">
         <is>
           <t>Portafolio de Cremación — Campaña Día de los Muertos 2026</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>SOLUCIÓN MODULAR DE CREMACIÓN</t>
         </is>
       </c>
-      <c r="C4" s="15" t="n"/>
-      <c r="D4" s="15" t="n"/>
-      <c r="E4" s="16" t="inlineStr">
+      <c r="C4" s="19" t="n"/>
+      <c r="D4" s="19" t="n"/>
+      <c r="E4" s="20" t="inlineStr">
         <is>
           <t>VG-CRE-01</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="B5" s="17" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>Línea Cremación Modular  ·  Cremación · Módulo add-on</t>
         </is>
       </c>
-      <c r="C5" s="18" t="n"/>
-      <c r="D5" s="18" t="n"/>
-      <c r="E5" s="19" t="n"/>
+      <c r="C5" s="22" t="n"/>
+      <c r="D5" s="22" t="n"/>
+      <c r="E5" s="23" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="B6" s="20" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C6" s="21" t="n"/>
-      <c r="D6" s="21" t="n"/>
-      <c r="E6" s="22" t="n"/>
+      <c r="C6" s="25" t="n"/>
+      <c r="D6" s="25" t="n"/>
+      <c r="E6" s="26" t="n"/>
     </row>
     <row r="7" ht="35" customHeight="1">
-      <c r="B7" s="23" t="inlineStr">
+      <c r="B7" s="27" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C7" s="24" t="inlineStr">
+      <c r="C7" s="28" t="inlineStr">
         <is>
           <t>Módulo de cremación integrable a cualquier plan funerario vigente o nuevo de Vangrupo, sin necesidad de cambiar de plan.</t>
         </is>
       </c>
-      <c r="D7" s="25" t="n"/>
-      <c r="E7" s="26" t="n"/>
+      <c r="D7" s="29" t="n"/>
+      <c r="E7" s="30" t="n"/>
     </row>
     <row r="8" ht="20.5" customHeight="1">
-      <c r="B8" s="27" t="inlineStr">
+      <c r="B8" s="31" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C8" s="28" t="inlineStr">
+      <c r="C8" s="32" t="inlineStr">
         <is>
           <t>Individual (1 titular / beneficiario por módulo).</t>
         </is>
       </c>
-      <c r="D8" s="29" t="n"/>
-      <c r="E8" s="30" t="n"/>
+      <c r="D8" s="33" t="n"/>
+      <c r="E8" s="34" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="B9" s="20" t="inlineStr">
+      <c r="B9" s="24" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C9" s="21" t="n"/>
-      <c r="D9" s="21" t="n"/>
-      <c r="E9" s="22" t="n"/>
+      <c r="C9" s="25" t="n"/>
+      <c r="D9" s="25" t="n"/>
+      <c r="E9" s="26" t="n"/>
     </row>
     <row r="10" ht="20.5" customHeight="1">
-      <c r="B10" s="23" t="inlineStr">
+      <c r="B10" s="27" t="inlineStr">
         <is>
           <t>Tipo de producto</t>
         </is>
       </c>
-      <c r="C10" s="24" t="inlineStr">
+      <c r="C10" s="28" t="inlineStr">
         <is>
           <t>Módulo adicional (add-on) a plan funerario</t>
         </is>
       </c>
-      <c r="D10" s="25" t="n"/>
-      <c r="E10" s="26" t="n"/>
+      <c r="D10" s="29" t="n"/>
+      <c r="E10" s="30" t="n"/>
     </row>
     <row r="11" ht="20.5" customHeight="1">
-      <c r="B11" s="27" t="inlineStr">
+      <c r="B11" s="31" t="inlineStr">
         <is>
           <t>Modalidad de cremación</t>
         </is>
       </c>
-      <c r="C11" s="28" t="inlineStr">
+      <c r="C11" s="32" t="inlineStr">
         <is>
           <t>Individual</t>
         </is>
       </c>
-      <c r="D11" s="29" t="n"/>
-      <c r="E11" s="30" t="n"/>
+      <c r="D11" s="33" t="n"/>
+      <c r="E11" s="34" t="n"/>
     </row>
     <row r="12" ht="20.5" customHeight="1">
-      <c r="B12" s="23" t="inlineStr">
+      <c r="B12" s="27" t="inlineStr">
         <is>
           <t>Urna</t>
         </is>
       </c>
-      <c r="C12" s="24" t="inlineStr">
+      <c r="C12" s="28" t="inlineStr">
         <is>
           <t>Cineraria, línea modular</t>
         </is>
       </c>
-      <c r="D12" s="25" t="n"/>
-      <c r="E12" s="26" t="n"/>
+      <c r="D12" s="29" t="n"/>
+      <c r="E12" s="30" t="n"/>
     </row>
     <row r="13" ht="20.5" customHeight="1">
-      <c r="B13" s="27" t="inlineStr">
+      <c r="B13" s="31" t="inlineStr">
         <is>
           <t>Gestión legal</t>
         </is>
       </c>
-      <c r="C13" s="28" t="inlineStr">
+      <c r="C13" s="32" t="inlineStr">
         <is>
           <t>Trámites básicos incluidos</t>
         </is>
       </c>
-      <c r="D13" s="29" t="n"/>
-      <c r="E13" s="30" t="n"/>
+      <c r="D13" s="33" t="n"/>
+      <c r="E13" s="34" t="n"/>
     </row>
     <row r="14" ht="20.5" customHeight="1">
-      <c r="B14" s="23" t="inlineStr">
+      <c r="B14" s="27" t="inlineStr">
         <is>
           <t>Columbario</t>
         </is>
       </c>
-      <c r="C14" s="24" t="inlineStr">
+      <c r="C14" s="28" t="inlineStr">
         <is>
           <t>Alquiler temporal · 12 meses incluido</t>
         </is>
       </c>
-      <c r="D14" s="25" t="n"/>
-      <c r="E14" s="26" t="n"/>
+      <c r="D14" s="29" t="n"/>
+      <c r="E14" s="30" t="n"/>
     </row>
     <row r="15" ht="78.5" customHeight="1">
-      <c r="B15" s="27" t="inlineStr">
+      <c r="B15" s="31" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C15" s="28" t="inlineStr">
+      <c r="C15" s="32" t="inlineStr">
         <is>
           <t>• Proceso completo de cremación individual
 • Urna cineraria de línea modular
@@ -1288,262 +1326,262 @@
 • Integración al plan funerario base (actual o nuevo)</t>
         </is>
       </c>
-      <c r="D15" s="29" t="n"/>
-      <c r="E15" s="30" t="n"/>
+      <c r="D15" s="33" t="n"/>
+      <c r="E15" s="34" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="B16" s="20" t="inlineStr">
+      <c r="B16" s="24" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C16" s="21" t="n"/>
-      <c r="D16" s="21" t="n"/>
-      <c r="E16" s="22" t="n"/>
+      <c r="C16" s="25" t="n"/>
+      <c r="D16" s="25" t="n"/>
+      <c r="E16" s="26" t="n"/>
     </row>
     <row r="17" ht="26.5" customHeight="1">
-      <c r="B17" s="23" t="inlineStr">
+      <c r="B17" s="27" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C17" s="31" t="inlineStr">
+      <c r="C17" s="35" t="inlineStr">
         <is>
           <t>US$ 1.000</t>
         </is>
       </c>
-      <c r="D17" s="25" t="n"/>
-      <c r="E17" s="26" t="n"/>
+      <c r="D17" s="29" t="n"/>
+      <c r="E17" s="30" t="n"/>
     </row>
     <row r="18" ht="20.5" customHeight="1">
-      <c r="B18" s="27" t="inlineStr">
+      <c r="B18" s="31" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C18" s="28" t="inlineStr">
+      <c r="C18" s="32" t="inlineStr">
         <is>
           <t>Por módulo individual</t>
         </is>
       </c>
-      <c r="D18" s="29" t="n"/>
-      <c r="E18" s="30" t="n"/>
+      <c r="D18" s="33" t="n"/>
+      <c r="E18" s="34" t="n"/>
     </row>
     <row r="19" ht="20.5" customHeight="1">
-      <c r="B19" s="23" t="inlineStr">
+      <c r="B19" s="27" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C19" s="24" t="inlineStr">
+      <c r="C19" s="28" t="inlineStr">
         <is>
           <t>Hasta 120 cuotas mensuales (aprox. US$ 8,50/mes).</t>
         </is>
       </c>
-      <c r="D19" s="25" t="n"/>
-      <c r="E19" s="26" t="n"/>
+      <c r="D19" s="29" t="n"/>
+      <c r="E19" s="30" t="n"/>
     </row>
     <row r="20" ht="20.5" customHeight="1">
-      <c r="B20" s="27" t="inlineStr">
+      <c r="B20" s="31" t="inlineStr">
         <is>
           <t>Cuota referencial</t>
         </is>
       </c>
-      <c r="C20" s="28" t="inlineStr">
+      <c r="C20" s="32" t="inlineStr">
         <is>
           <t>US$ 8,33/mes sin intereses (120 cuotas)</t>
         </is>
       </c>
-      <c r="D20" s="29" t="n"/>
-      <c r="E20" s="30" t="n"/>
+      <c r="D20" s="33" t="n"/>
+      <c r="E20" s="34" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="B21" s="20" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C21" s="21" t="n"/>
-      <c r="D21" s="21" t="n"/>
-      <c r="E21" s="22" t="n"/>
+      <c r="C21" s="25" t="n"/>
+      <c r="D21" s="25" t="n"/>
+      <c r="E21" s="26" t="n"/>
     </row>
     <row r="22" ht="35" customHeight="1">
-      <c r="B22" s="32" t="inlineStr">
+      <c r="B22" s="36" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C22" s="33" t="inlineStr">
+      <c r="C22" s="37" t="inlineStr">
         <is>
           <t>Afiliados actuales y nuevos que desean incorporar la cremación a su plan con una cuota mensual mínima.</t>
         </is>
       </c>
-      <c r="D22" s="34" t="n"/>
-      <c r="E22" s="35" t="n"/>
+      <c r="D22" s="38" t="n"/>
+      <c r="E22" s="39" t="n"/>
     </row>
     <row r="25" ht="30" customHeight="1">
-      <c r="B25" s="14" t="inlineStr">
+      <c r="B25" s="18" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · INDIVIDUAL</t>
         </is>
       </c>
-      <c r="C25" s="15" t="n"/>
-      <c r="D25" s="15" t="n"/>
-      <c r="E25" s="16" t="inlineStr">
+      <c r="C25" s="19" t="n"/>
+      <c r="D25" s="19" t="n"/>
+      <c r="E25" s="20" t="inlineStr">
         <is>
           <t>VG-CRE-03I</t>
         </is>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="B26" s="17" t="inlineStr">
+      <c r="B26" s="21" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Jardín 1  ·  Destino final · Inhumación individual</t>
         </is>
       </c>
-      <c r="C26" s="18" t="n"/>
-      <c r="D26" s="18" t="n"/>
-      <c r="E26" s="19" t="n"/>
+      <c r="C26" s="22" t="n"/>
+      <c r="D26" s="22" t="n"/>
+      <c r="E26" s="23" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="B27" s="20" t="inlineStr">
+      <c r="B27" s="24" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C27" s="21" t="n"/>
-      <c r="D27" s="21" t="n"/>
-      <c r="E27" s="22" t="n"/>
+      <c r="C27" s="25" t="n"/>
+      <c r="D27" s="25" t="n"/>
+      <c r="E27" s="26" t="n"/>
     </row>
     <row r="28" ht="49.5" customHeight="1">
-      <c r="B28" s="23" t="inlineStr">
+      <c r="B28" s="27" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C28" s="24" t="inlineStr">
+      <c r="C28" s="28" t="inlineStr">
         <is>
           <t>Inhumación de la urna de cenizas en un contenedor enterrado con tapa de granito grabada, en un jardín de plantas de sombra: un lugar físico permanente de homenaje.</t>
         </is>
       </c>
-      <c r="D28" s="25" t="n"/>
-      <c r="E28" s="26" t="n"/>
+      <c r="D28" s="29" t="n"/>
+      <c r="E28" s="30" t="n"/>
     </row>
     <row r="29" ht="20.5" customHeight="1">
-      <c r="B29" s="27" t="inlineStr">
+      <c r="B29" s="31" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C29" s="28" t="inlineStr">
+      <c r="C29" s="32" t="inlineStr">
         <is>
           <t>Individual (1 urna).</t>
         </is>
       </c>
-      <c r="D29" s="29" t="n"/>
-      <c r="E29" s="30" t="n"/>
+      <c r="D29" s="33" t="n"/>
+      <c r="E29" s="34" t="n"/>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="B30" s="20" t="inlineStr">
+      <c r="B30" s="24" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C30" s="21" t="n"/>
-      <c r="D30" s="21" t="n"/>
-      <c r="E30" s="22" t="n"/>
+      <c r="C30" s="25" t="n"/>
+      <c r="D30" s="25" t="n"/>
+      <c r="E30" s="26" t="n"/>
     </row>
     <row r="31" ht="20.5" customHeight="1">
-      <c r="B31" s="23" t="inlineStr">
+      <c r="B31" s="27" t="inlineStr">
         <is>
           <t>Ambiente</t>
         </is>
       </c>
-      <c r="C31" s="24" t="inlineStr">
+      <c r="C31" s="28" t="inlineStr">
         <is>
           <t>Jardín 1</t>
         </is>
       </c>
-      <c r="D31" s="25" t="n"/>
-      <c r="E31" s="26" t="n"/>
+      <c r="D31" s="29" t="n"/>
+      <c r="E31" s="30" t="n"/>
     </row>
     <row r="32" ht="20.5" customHeight="1">
-      <c r="B32" s="27" t="inlineStr">
+      <c r="B32" s="31" t="inlineStr">
         <is>
           <t>Contenedor</t>
         </is>
       </c>
-      <c r="C32" s="28" t="inlineStr">
+      <c r="C32" s="32" t="inlineStr">
         <is>
           <t>Ø 32 cm × 40 cm de altura; enterrado dejando 20 cm a la vista</t>
         </is>
       </c>
-      <c r="D32" s="29" t="n"/>
-      <c r="E32" s="30" t="n"/>
+      <c r="D32" s="33" t="n"/>
+      <c r="E32" s="34" t="n"/>
     </row>
     <row r="33" ht="20.5" customHeight="1">
-      <c r="B33" s="23" t="inlineStr">
+      <c r="B33" s="27" t="inlineStr">
         <is>
           <t>Identificación</t>
         </is>
       </c>
-      <c r="C33" s="24" t="inlineStr">
+      <c r="C33" s="28" t="inlineStr">
         <is>
           <t>Tapa de granito con la información del difunto</t>
         </is>
       </c>
-      <c r="D33" s="25" t="n"/>
-      <c r="E33" s="26" t="n"/>
+      <c r="D33" s="29" t="n"/>
+      <c r="E33" s="30" t="n"/>
     </row>
     <row r="34" ht="20.5" customHeight="1">
-      <c r="B34" s="27" t="inlineStr">
+      <c r="B34" s="31" t="inlineStr">
         <is>
           <t>Paisajismo</t>
         </is>
       </c>
-      <c r="C34" s="28" t="inlineStr">
+      <c r="C34" s="32" t="inlineStr">
         <is>
           <t>Plantas de sombra de diferentes alturas y texturas</t>
         </is>
       </c>
-      <c r="D34" s="29" t="n"/>
-      <c r="E34" s="30" t="n"/>
+      <c r="D34" s="33" t="n"/>
+      <c r="E34" s="34" t="n"/>
     </row>
     <row r="35" ht="20.5" customHeight="1">
-      <c r="B35" s="23" t="inlineStr">
+      <c r="B35" s="27" t="inlineStr">
         <is>
           <t>Acceso</t>
         </is>
       </c>
-      <c r="C35" s="24" t="inlineStr">
+      <c r="C35" s="28" t="inlineStr">
         <is>
           <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
         </is>
       </c>
-      <c r="D35" s="25" t="n"/>
-      <c r="E35" s="26" t="n"/>
+      <c r="D35" s="29" t="n"/>
+      <c r="E35" s="30" t="n"/>
     </row>
     <row r="36" ht="20.5" customHeight="1">
-      <c r="B36" s="27" t="inlineStr">
+      <c r="B36" s="31" t="inlineStr">
         <is>
           <t>Mantenimiento</t>
         </is>
       </c>
-      <c r="C36" s="28" t="inlineStr">
+      <c r="C36" s="32" t="inlineStr">
         <is>
           <t>US$ 15 anual</t>
         </is>
       </c>
-      <c r="D36" s="29" t="n"/>
-      <c r="E36" s="30" t="n"/>
+      <c r="D36" s="33" t="n"/>
+      <c r="E36" s="34" t="n"/>
     </row>
     <row r="37" ht="64" customHeight="1">
-      <c r="B37" s="23" t="inlineStr">
+      <c r="B37" s="27" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C37" s="24" t="inlineStr">
+      <c r="C37" s="28" t="inlineStr">
         <is>
           <t>• Inhumación de la urna en contenedor individual
 • Tapa de granito con los datos del difunto
@@ -1551,248 +1589,248 @@
 • Espacio de contemplación con banco</t>
         </is>
       </c>
-      <c r="D37" s="25" t="n"/>
-      <c r="E37" s="26" t="n"/>
+      <c r="D37" s="29" t="n"/>
+      <c r="E37" s="30" t="n"/>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="B38" s="20" t="inlineStr">
+      <c r="B38" s="24" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C38" s="21" t="n"/>
-      <c r="D38" s="21" t="n"/>
-      <c r="E38" s="22" t="n"/>
+      <c r="C38" s="25" t="n"/>
+      <c r="D38" s="25" t="n"/>
+      <c r="E38" s="26" t="n"/>
     </row>
     <row r="39" ht="26.5" customHeight="1">
-      <c r="B39" s="23" t="inlineStr">
+      <c r="B39" s="27" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C39" s="31" t="inlineStr">
+      <c r="C39" s="35" t="inlineStr">
         <is>
           <t>US$ 600</t>
         </is>
       </c>
-      <c r="D39" s="25" t="n"/>
-      <c r="E39" s="26" t="n"/>
+      <c r="D39" s="29" t="n"/>
+      <c r="E39" s="30" t="n"/>
     </row>
     <row r="40" ht="20.5" customHeight="1">
-      <c r="B40" s="27" t="inlineStr">
+      <c r="B40" s="31" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C40" s="28" t="inlineStr">
+      <c r="C40" s="32" t="inlineStr">
         <is>
           <t>Por espacio individual · mantenimiento US$ 15/año</t>
         </is>
       </c>
-      <c r="D40" s="29" t="n"/>
-      <c r="E40" s="30" t="n"/>
+      <c r="D40" s="33" t="n"/>
+      <c r="E40" s="34" t="n"/>
     </row>
     <row r="41" ht="35" customHeight="1">
-      <c r="B41" s="23" t="inlineStr">
+      <c r="B41" s="27" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C41" s="24" t="inlineStr">
+      <c r="C41" s="28" t="inlineStr">
         <is>
           <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 15 anual.</t>
         </is>
       </c>
-      <c r="D41" s="25" t="n"/>
-      <c r="E41" s="26" t="n"/>
+      <c r="D41" s="29" t="n"/>
+      <c r="E41" s="30" t="n"/>
     </row>
     <row r="42" ht="20" customHeight="1">
-      <c r="B42" s="20" t="inlineStr">
+      <c r="B42" s="24" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C42" s="21" t="n"/>
-      <c r="D42" s="21" t="n"/>
-      <c r="E42" s="22" t="n"/>
+      <c r="C42" s="25" t="n"/>
+      <c r="D42" s="25" t="n"/>
+      <c r="E42" s="26" t="n"/>
     </row>
     <row r="43" ht="35" customHeight="1">
-      <c r="B43" s="32" t="inlineStr">
+      <c r="B43" s="36" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C43" s="33" t="inlineStr">
+      <c r="C43" s="37" t="inlineStr">
         <is>
           <t>Familias que desean un lugar permanente para visitar y rendir homenaje, con una inversión moderada.</t>
         </is>
       </c>
-      <c r="D43" s="34" t="n"/>
-      <c r="E43" s="35" t="n"/>
+      <c r="D43" s="38" t="n"/>
+      <c r="E43" s="39" t="n"/>
     </row>
     <row r="46" ht="30" customHeight="1">
-      <c r="B46" s="14" t="inlineStr">
+      <c r="B46" s="18" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · FAMILIAR</t>
         </is>
       </c>
-      <c r="C46" s="15" t="n"/>
-      <c r="D46" s="15" t="n"/>
-      <c r="E46" s="16" t="inlineStr">
+      <c r="C46" s="19" t="n"/>
+      <c r="D46" s="19" t="n"/>
+      <c r="E46" s="20" t="inlineStr">
         <is>
           <t>VG-CRE-03F</t>
         </is>
       </c>
     </row>
     <row r="47" ht="20" customHeight="1">
-      <c r="B47" s="17" t="inlineStr">
+      <c r="B47" s="21" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Jardín 1  ·  Destino final · Inhumación familiar</t>
         </is>
       </c>
-      <c r="C47" s="18" t="n"/>
-      <c r="D47" s="18" t="n"/>
-      <c r="E47" s="19" t="n"/>
+      <c r="C47" s="22" t="n"/>
+      <c r="D47" s="22" t="n"/>
+      <c r="E47" s="23" t="n"/>
     </row>
     <row r="48" ht="20" customHeight="1">
-      <c r="B48" s="20" t="inlineStr">
+      <c r="B48" s="24" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C48" s="21" t="n"/>
-      <c r="D48" s="21" t="n"/>
-      <c r="E48" s="22" t="n"/>
+      <c r="C48" s="25" t="n"/>
+      <c r="D48" s="25" t="n"/>
+      <c r="E48" s="26" t="n"/>
     </row>
     <row r="49" ht="35" customHeight="1">
-      <c r="B49" s="23" t="inlineStr">
+      <c r="B49" s="27" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C49" s="24" t="inlineStr">
+      <c r="C49" s="28" t="inlineStr">
         <is>
           <t>Parcela familiar en el Jardín 1 con cuatro contenedores agrupados, cada uno con tapa de granito grabada, sin plazo de permanencia.</t>
         </is>
       </c>
-      <c r="D49" s="25" t="n"/>
-      <c r="E49" s="26" t="n"/>
+      <c r="D49" s="29" t="n"/>
+      <c r="E49" s="30" t="n"/>
     </row>
     <row r="50" ht="20.5" customHeight="1">
-      <c r="B50" s="27" t="inlineStr">
+      <c r="B50" s="31" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C50" s="28" t="inlineStr">
+      <c r="C50" s="32" t="inlineStr">
         <is>
           <t>Hasta 4 espacios (familiar).</t>
         </is>
       </c>
-      <c r="D50" s="29" t="n"/>
-      <c r="E50" s="30" t="n"/>
+      <c r="D50" s="33" t="n"/>
+      <c r="E50" s="34" t="n"/>
     </row>
     <row r="51" ht="20" customHeight="1">
-      <c r="B51" s="20" t="inlineStr">
+      <c r="B51" s="24" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C51" s="21" t="n"/>
-      <c r="D51" s="21" t="n"/>
-      <c r="E51" s="22" t="n"/>
+      <c r="C51" s="25" t="n"/>
+      <c r="D51" s="25" t="n"/>
+      <c r="E51" s="26" t="n"/>
     </row>
     <row r="52" ht="20.5" customHeight="1">
-      <c r="B52" s="23" t="inlineStr">
+      <c r="B52" s="27" t="inlineStr">
         <is>
           <t>Ambiente</t>
         </is>
       </c>
-      <c r="C52" s="24" t="inlineStr">
+      <c r="C52" s="28" t="inlineStr">
         <is>
           <t>Jardín 1</t>
         </is>
       </c>
-      <c r="D52" s="25" t="n"/>
-      <c r="E52" s="26" t="n"/>
+      <c r="D52" s="29" t="n"/>
+      <c r="E52" s="30" t="n"/>
     </row>
     <row r="53" ht="20.5" customHeight="1">
-      <c r="B53" s="27" t="inlineStr">
+      <c r="B53" s="31" t="inlineStr">
         <is>
           <t>Capacidad</t>
         </is>
       </c>
-      <c r="C53" s="28" t="inlineStr">
+      <c r="C53" s="32" t="inlineStr">
         <is>
           <t>4 contenedores agrupados en losa</t>
         </is>
       </c>
-      <c r="D53" s="29" t="n"/>
-      <c r="E53" s="30" t="n"/>
+      <c r="D53" s="33" t="n"/>
+      <c r="E53" s="34" t="n"/>
     </row>
     <row r="54" ht="20.5" customHeight="1">
-      <c r="B54" s="23" t="inlineStr">
+      <c r="B54" s="27" t="inlineStr">
         <is>
           <t>Identificación</t>
         </is>
       </c>
-      <c r="C54" s="24" t="inlineStr">
+      <c r="C54" s="28" t="inlineStr">
         <is>
           <t>Tapa de granito por espacio, con la información del difunto</t>
         </is>
       </c>
-      <c r="D54" s="25" t="n"/>
-      <c r="E54" s="26" t="n"/>
+      <c r="D54" s="29" t="n"/>
+      <c r="E54" s="30" t="n"/>
     </row>
     <row r="55" ht="20.5" customHeight="1">
-      <c r="B55" s="27" t="inlineStr">
+      <c r="B55" s="31" t="inlineStr">
         <is>
           <t>Permanencia</t>
         </is>
       </c>
-      <c r="C55" s="28" t="inlineStr">
+      <c r="C55" s="32" t="inlineStr">
         <is>
           <t>Sin plazo</t>
         </is>
       </c>
-      <c r="D55" s="29" t="n"/>
-      <c r="E55" s="30" t="n"/>
+      <c r="D55" s="33" t="n"/>
+      <c r="E55" s="34" t="n"/>
     </row>
     <row r="56" ht="20.5" customHeight="1">
-      <c r="B56" s="23" t="inlineStr">
+      <c r="B56" s="27" t="inlineStr">
         <is>
           <t>Acceso</t>
         </is>
       </c>
-      <c r="C56" s="24" t="inlineStr">
+      <c r="C56" s="28" t="inlineStr">
         <is>
           <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
         </is>
       </c>
-      <c r="D56" s="25" t="n"/>
-      <c r="E56" s="26" t="n"/>
+      <c r="D56" s="29" t="n"/>
+      <c r="E56" s="30" t="n"/>
     </row>
     <row r="57" ht="20.5" customHeight="1">
-      <c r="B57" s="27" t="inlineStr">
+      <c r="B57" s="31" t="inlineStr">
         <is>
           <t>Mantenimiento</t>
         </is>
       </c>
-      <c r="C57" s="28" t="inlineStr">
+      <c r="C57" s="32" t="inlineStr">
         <is>
           <t>US$ 25 anual</t>
         </is>
       </c>
-      <c r="D57" s="29" t="n"/>
-      <c r="E57" s="30" t="n"/>
+      <c r="D57" s="33" t="n"/>
+      <c r="E57" s="34" t="n"/>
     </row>
     <row r="58" ht="64" customHeight="1">
-      <c r="B58" s="23" t="inlineStr">
+      <c r="B58" s="27" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C58" s="24" t="inlineStr">
+      <c r="C58" s="28" t="inlineStr">
         <is>
           <t>• Inhumación de hasta 4 urnas
 • Tapa de granito grabada para cada espacio
@@ -1800,276 +1838,276 @@
 • Lugar físico permanente de homenaje familiar, sin plazo</t>
         </is>
       </c>
-      <c r="D58" s="25" t="n"/>
-      <c r="E58" s="26" t="n"/>
+      <c r="D58" s="29" t="n"/>
+      <c r="E58" s="30" t="n"/>
     </row>
     <row r="59" ht="20" customHeight="1">
-      <c r="B59" s="20" t="inlineStr">
+      <c r="B59" s="24" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C59" s="21" t="n"/>
-      <c r="D59" s="21" t="n"/>
-      <c r="E59" s="22" t="n"/>
+      <c r="C59" s="25" t="n"/>
+      <c r="D59" s="25" t="n"/>
+      <c r="E59" s="26" t="n"/>
     </row>
     <row r="60" ht="26.5" customHeight="1">
-      <c r="B60" s="23" t="inlineStr">
+      <c r="B60" s="27" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C60" s="31" t="inlineStr">
+      <c r="C60" s="35" t="inlineStr">
         <is>
           <t>US$ 2.000</t>
         </is>
       </c>
-      <c r="D60" s="25" t="n"/>
-      <c r="E60" s="26" t="n"/>
+      <c r="D60" s="29" t="n"/>
+      <c r="E60" s="30" t="n"/>
     </row>
     <row r="61" ht="20.5" customHeight="1">
-      <c r="B61" s="27" t="inlineStr">
+      <c r="B61" s="31" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C61" s="28" t="inlineStr">
+      <c r="C61" s="32" t="inlineStr">
         <is>
           <t>Por parcela familiar · hasta 4 espacios · mantenimiento US$ 25/año</t>
         </is>
       </c>
-      <c r="D61" s="29" t="n"/>
-      <c r="E61" s="30" t="n"/>
+      <c r="D61" s="33" t="n"/>
+      <c r="E61" s="34" t="n"/>
     </row>
     <row r="62" ht="35" customHeight="1">
-      <c r="B62" s="23" t="inlineStr">
+      <c r="B62" s="27" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C62" s="24" t="inlineStr">
+      <c r="C62" s="28" t="inlineStr">
         <is>
           <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 25 anual.</t>
         </is>
       </c>
-      <c r="D62" s="25" t="n"/>
-      <c r="E62" s="26" t="n"/>
+      <c r="D62" s="29" t="n"/>
+      <c r="E62" s="30" t="n"/>
     </row>
     <row r="63" ht="20" customHeight="1">
-      <c r="B63" s="20" t="inlineStr">
+      <c r="B63" s="24" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C63" s="21" t="n"/>
-      <c r="D63" s="21" t="n"/>
-      <c r="E63" s="22" t="n"/>
+      <c r="C63" s="25" t="n"/>
+      <c r="D63" s="25" t="n"/>
+      <c r="E63" s="26" t="n"/>
     </row>
     <row r="64" ht="20.5" customHeight="1">
-      <c r="B64" s="32" t="inlineStr">
+      <c r="B64" s="36" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C64" s="33" t="inlineStr">
+      <c r="C64" s="37" t="inlineStr">
         <is>
           <t>Familias que buscan un espacio propio y permanente para varias generaciones.</t>
         </is>
       </c>
-      <c r="D64" s="34" t="n"/>
-      <c r="E64" s="35" t="n"/>
+      <c r="D64" s="38" t="n"/>
+      <c r="E64" s="39" t="n"/>
     </row>
     <row r="67" ht="30" customHeight="1">
-      <c r="B67" s="14" t="inlineStr">
+      <c r="B67" s="18" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · ECOLÓGICO</t>
         </is>
       </c>
-      <c r="C67" s="15" t="n"/>
-      <c r="D67" s="15" t="n"/>
-      <c r="E67" s="16" t="inlineStr">
+      <c r="C67" s="19" t="n"/>
+      <c r="D67" s="19" t="n"/>
+      <c r="E67" s="20" t="inlineStr">
         <is>
           <t>VG-CRE-03E</t>
         </is>
       </c>
     </row>
     <row r="68" ht="20" customHeight="1">
-      <c r="B68" s="17" t="inlineStr">
+      <c r="B68" s="21" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Jardín 2  ·  Destino final · Inhumación ecológica</t>
         </is>
       </c>
-      <c r="C68" s="18" t="n"/>
-      <c r="D68" s="18" t="n"/>
-      <c r="E68" s="19" t="n"/>
+      <c r="C68" s="22" t="n"/>
+      <c r="D68" s="22" t="n"/>
+      <c r="E68" s="23" t="n"/>
     </row>
     <row r="69" ht="20" customHeight="1">
-      <c r="B69" s="20" t="inlineStr">
+      <c r="B69" s="24" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C69" s="21" t="n"/>
-      <c r="D69" s="21" t="n"/>
-      <c r="E69" s="22" t="n"/>
+      <c r="C69" s="25" t="n"/>
+      <c r="D69" s="25" t="n"/>
+      <c r="E69" s="26" t="n"/>
     </row>
     <row r="70" ht="49.5" customHeight="1">
-      <c r="B70" s="23" t="inlineStr">
+      <c r="B70" s="27" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C70" s="24" t="inlineStr">
+      <c r="C70" s="28" t="inlineStr">
         <is>
           <t>La urna biodegradable se entierra directamente en el suelo, se cubre con tierra y se descompone integrándose a la naturaleza. Jardín con agua corriente y área de esparcimiento de cenizas.</t>
         </is>
       </c>
-      <c r="D70" s="25" t="n"/>
-      <c r="E70" s="26" t="n"/>
+      <c r="D70" s="29" t="n"/>
+      <c r="E70" s="30" t="n"/>
     </row>
     <row r="71" ht="20.5" customHeight="1">
-      <c r="B71" s="27" t="inlineStr">
+      <c r="B71" s="31" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C71" s="28" t="inlineStr">
+      <c r="C71" s="32" t="inlineStr">
         <is>
           <t>Individual (1 urna).</t>
         </is>
       </c>
-      <c r="D71" s="29" t="n"/>
-      <c r="E71" s="30" t="n"/>
+      <c r="D71" s="33" t="n"/>
+      <c r="E71" s="34" t="n"/>
     </row>
     <row r="72" ht="20" customHeight="1">
-      <c r="B72" s="20" t="inlineStr">
+      <c r="B72" s="24" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C72" s="21" t="n"/>
-      <c r="D72" s="21" t="n"/>
-      <c r="E72" s="22" t="n"/>
+      <c r="C72" s="25" t="n"/>
+      <c r="D72" s="25" t="n"/>
+      <c r="E72" s="26" t="n"/>
     </row>
     <row r="73" ht="20.5" customHeight="1">
-      <c r="B73" s="23" t="inlineStr">
+      <c r="B73" s="27" t="inlineStr">
         <is>
           <t>Ambientes</t>
         </is>
       </c>
-      <c r="C73" s="24" t="inlineStr">
+      <c r="C73" s="28" t="inlineStr">
         <is>
           <t>Jardín 2 · Ecológico o Bosque de las Orquídeas</t>
         </is>
       </c>
-      <c r="D73" s="25" t="n"/>
-      <c r="E73" s="26" t="n"/>
+      <c r="D73" s="29" t="n"/>
+      <c r="E73" s="30" t="n"/>
     </row>
     <row r="74" ht="20.5" customHeight="1">
-      <c r="B74" s="27" t="inlineStr">
+      <c r="B74" s="31" t="inlineStr">
         <is>
           <t>Espacio por urna</t>
         </is>
       </c>
-      <c r="C74" s="28" t="inlineStr">
+      <c r="C74" s="32" t="inlineStr">
         <is>
           <t>30 × 30 cm, 40 cm de profundidad</t>
         </is>
       </c>
-      <c r="D74" s="29" t="n"/>
-      <c r="E74" s="30" t="n"/>
+      <c r="D74" s="33" t="n"/>
+      <c r="E74" s="34" t="n"/>
     </row>
     <row r="75" ht="20.5" customHeight="1">
-      <c r="B75" s="23" t="inlineStr">
+      <c r="B75" s="27" t="inlineStr">
         <is>
           <t>Urna</t>
         </is>
       </c>
-      <c r="C75" s="24" t="inlineStr">
+      <c r="C75" s="28" t="inlineStr">
         <is>
           <t>Biodegradable; se integra al suelo</t>
         </is>
       </c>
-      <c r="D75" s="25" t="n"/>
-      <c r="E75" s="26" t="n"/>
+      <c r="D75" s="29" t="n"/>
+      <c r="E75" s="30" t="n"/>
     </row>
     <row r="76" ht="35" customHeight="1">
-      <c r="B76" s="27" t="inlineStr">
+      <c r="B76" s="31" t="inlineStr">
         <is>
           <t>Identificación (Jardín 2)</t>
         </is>
       </c>
-      <c r="C76" s="28" t="inlineStr">
+      <c r="C76" s="32" t="inlineStr">
         <is>
           <t>Placa de madera de 20 cm fijada a una varilla metálica, en posición vertical y sin contacto con el suelo</t>
         </is>
       </c>
-      <c r="D76" s="29" t="n"/>
-      <c r="E76" s="30" t="n"/>
+      <c r="D76" s="33" t="n"/>
+      <c r="E76" s="34" t="n"/>
     </row>
     <row r="77" ht="20.5" customHeight="1">
-      <c r="B77" s="23" t="inlineStr">
+      <c r="B77" s="27" t="inlineStr">
         <is>
           <t>Identificación (Bosque)</t>
         </is>
       </c>
-      <c r="C77" s="24" t="inlineStr">
+      <c r="C77" s="28" t="inlineStr">
         <is>
           <t>Placa de mármol de 20 × 15 cm</t>
         </is>
       </c>
-      <c r="D77" s="25" t="n"/>
-      <c r="E77" s="26" t="n"/>
+      <c r="D77" s="29" t="n"/>
+      <c r="E77" s="30" t="n"/>
     </row>
     <row r="78" ht="35" customHeight="1">
-      <c r="B78" s="27" t="inlineStr">
+      <c r="B78" s="31" t="inlineStr">
         <is>
           <t>Permanencia</t>
         </is>
       </c>
-      <c r="C78" s="28" t="inlineStr">
+      <c r="C78" s="32" t="inlineStr">
         <is>
           <t>3 años; luego el nombre pasa a una placa memorial en el monumento y el espacio se reutiliza</t>
         </is>
       </c>
-      <c r="D78" s="29" t="n"/>
-      <c r="E78" s="30" t="n"/>
+      <c r="D78" s="33" t="n"/>
+      <c r="E78" s="34" t="n"/>
     </row>
     <row r="79" ht="20.5" customHeight="1">
-      <c r="B79" s="23" t="inlineStr">
+      <c r="B79" s="27" t="inlineStr">
         <is>
           <t>Placa memorial</t>
         </is>
       </c>
-      <c r="C79" s="24" t="inlineStr">
+      <c r="C79" s="28" t="inlineStr">
         <is>
           <t>US$ 150</t>
         </is>
       </c>
-      <c r="D79" s="25" t="n"/>
-      <c r="E79" s="26" t="n"/>
+      <c r="D79" s="29" t="n"/>
+      <c r="E79" s="30" t="n"/>
     </row>
     <row r="80" ht="20.5" customHeight="1">
-      <c r="B80" s="27" t="inlineStr">
+      <c r="B80" s="31" t="inlineStr">
         <is>
           <t>Acceso</t>
         </is>
       </c>
-      <c r="C80" s="28" t="inlineStr">
+      <c r="C80" s="32" t="inlineStr">
         <is>
           <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
         </is>
       </c>
-      <c r="D80" s="29" t="n"/>
-      <c r="E80" s="30" t="n"/>
+      <c r="D80" s="33" t="n"/>
+      <c r="E80" s="34" t="n"/>
     </row>
     <row r="81" ht="78.5" customHeight="1">
-      <c r="B81" s="23" t="inlineStr">
+      <c r="B81" s="27" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C81" s="24" t="inlineStr">
+      <c r="C81" s="28" t="inlineStr">
         <is>
           <t>• Inhumación ecológica de la urna directamente en el suelo
 • Placa de identificación
@@ -2078,453 +2116,248 @@
 • Permanencia de 3 años; luego, placa memorial en el monumento</t>
         </is>
       </c>
-      <c r="D81" s="25" t="n"/>
-      <c r="E81" s="26" t="n"/>
+      <c r="D81" s="29" t="n"/>
+      <c r="E81" s="30" t="n"/>
     </row>
     <row r="82" ht="20" customHeight="1">
-      <c r="B82" s="20" t="inlineStr">
+      <c r="B82" s="24" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C82" s="21" t="n"/>
-      <c r="D82" s="21" t="n"/>
-      <c r="E82" s="22" t="n"/>
+      <c r="C82" s="25" t="n"/>
+      <c r="D82" s="25" t="n"/>
+      <c r="E82" s="26" t="n"/>
     </row>
     <row r="83" ht="26.5" customHeight="1">
-      <c r="B83" s="23" t="inlineStr">
+      <c r="B83" s="27" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C83" s="31" t="inlineStr">
+      <c r="C83" s="35" t="inlineStr">
         <is>
           <t>US$ 600</t>
         </is>
       </c>
-      <c r="D83" s="25" t="n"/>
-      <c r="E83" s="26" t="n"/>
+      <c r="D83" s="29" t="n"/>
+      <c r="E83" s="30" t="n"/>
     </row>
     <row r="84" ht="20.5" customHeight="1">
-      <c r="B84" s="27" t="inlineStr">
+      <c r="B84" s="31" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C84" s="28" t="inlineStr">
+      <c r="C84" s="32" t="inlineStr">
         <is>
           <t>Por espacio individual · placa memorial US$ 150</t>
         </is>
       </c>
-      <c r="D84" s="29" t="n"/>
-      <c r="E84" s="30" t="n"/>
+      <c r="D84" s="33" t="n"/>
+      <c r="E84" s="34" t="n"/>
     </row>
     <row r="85" ht="35" customHeight="1">
-      <c r="B85" s="23" t="inlineStr">
+      <c r="B85" s="27" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C85" s="24" t="inlineStr">
+      <c r="C85" s="28" t="inlineStr">
         <is>
           <t>Pago único o financiado según política comercial vigente. Placa memorial en el monumento al término del plazo: US$ 150.</t>
         </is>
       </c>
-      <c r="D85" s="25" t="n"/>
-      <c r="E85" s="26" t="n"/>
+      <c r="D85" s="29" t="n"/>
+      <c r="E85" s="30" t="n"/>
     </row>
     <row r="86" ht="20" customHeight="1">
-      <c r="B86" s="20" t="inlineStr">
+      <c r="B86" s="24" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C86" s="21" t="n"/>
-      <c r="D86" s="21" t="n"/>
-      <c r="E86" s="22" t="n"/>
+      <c r="C86" s="25" t="n"/>
+      <c r="D86" s="25" t="n"/>
+      <c r="E86" s="26" t="n"/>
     </row>
     <row r="87" ht="35" customHeight="1">
-      <c r="B87" s="32" t="inlineStr">
+      <c r="B87" s="36" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C87" s="33" t="inlineStr">
+      <c r="C87" s="37" t="inlineStr">
         <is>
           <t>Personas con conciencia ambiental que desean que sus cenizas vuelvan a la tierra, con un lugar identificado para visitar.</t>
         </is>
       </c>
-      <c r="D87" s="34" t="n"/>
-      <c r="E87" s="35" t="n"/>
+      <c r="D87" s="38" t="n"/>
+      <c r="E87" s="39" t="n"/>
     </row>
     <row r="90" ht="30" customHeight="1">
-      <c r="B90" s="14" t="inlineStr">
-        <is>
-          <t>JARDÍN DE CENIZAS · CEREMONIAL</t>
-        </is>
-      </c>
-      <c r="C90" s="15" t="n"/>
-      <c r="D90" s="15" t="n"/>
-      <c r="E90" s="16" t="inlineStr">
-        <is>
-          <t>VG-CRE-03C</t>
+      <c r="B90" s="18" t="inlineStr">
+        <is>
+          <t>JARDÍN DE MASCOTAS</t>
+        </is>
+      </c>
+      <c r="C90" s="19" t="n"/>
+      <c r="D90" s="19" t="n"/>
+      <c r="E90" s="20" t="inlineStr">
+        <is>
+          <t>VG-CRE-04</t>
         </is>
       </c>
     </row>
     <row r="91" ht="20" customHeight="1">
-      <c r="B91" s="17" t="inlineStr">
-        <is>
-          <t>Jardines de la Memoria · Jardín 3  ·  Destino final · Inhumación con ceremonia</t>
-        </is>
-      </c>
-      <c r="C91" s="18" t="n"/>
-      <c r="D91" s="18" t="n"/>
-      <c r="E91" s="19" t="n"/>
+      <c r="B91" s="21" t="inlineStr">
+        <is>
+          <t>Jardines de la Memoria · Mascotas  ·  Destino final · Inhumación ecológica</t>
+        </is>
+      </c>
+      <c r="C91" s="22" t="n"/>
+      <c r="D91" s="22" t="n"/>
+      <c r="E91" s="23" t="n"/>
     </row>
     <row r="92" ht="20" customHeight="1">
-      <c r="B92" s="20" t="inlineStr">
+      <c r="B92" s="24" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C92" s="21" t="n"/>
-      <c r="D92" s="21" t="n"/>
-      <c r="E92" s="22" t="n"/>
+      <c r="C92" s="25" t="n"/>
+      <c r="D92" s="25" t="n"/>
+      <c r="E92" s="26" t="n"/>
     </row>
     <row r="93" ht="35" customHeight="1">
-      <c r="B93" s="23" t="inlineStr">
+      <c r="B93" s="27" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C93" s="24" t="inlineStr">
-        <is>
-          <t>Jardín para inhumación de urnas de cenizas con ceremonia de agua, con fuentes como elemento central del rito de despedida.</t>
-        </is>
-      </c>
-      <c r="D93" s="25" t="n"/>
-      <c r="E93" s="26" t="n"/>
+      <c r="C93" s="28" t="inlineStr">
+        <is>
+          <t>Jardín para inhumación ecológica de cenizas de mascotas: la urna biodegradable se entierra directamente en el suelo y se identifica con una placa de madera.</t>
+        </is>
+      </c>
+      <c r="D93" s="29" t="n"/>
+      <c r="E93" s="30" t="n"/>
     </row>
     <row r="94" ht="20.5" customHeight="1">
-      <c r="B94" s="27" t="inlineStr">
+      <c r="B94" s="31" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C94" s="28" t="inlineStr">
-        <is>
-          <t>A definir.</t>
-        </is>
-      </c>
-      <c r="D94" s="29" t="n"/>
-      <c r="E94" s="30" t="n"/>
+      <c r="C94" s="32" t="inlineStr">
+        <is>
+          <t>Individual (una mascota por servicio).</t>
+        </is>
+      </c>
+      <c r="D94" s="33" t="n"/>
+      <c r="E94" s="34" t="n"/>
     </row>
     <row r="95" ht="20" customHeight="1">
-      <c r="B95" s="20" t="inlineStr">
+      <c r="B95" s="24" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C95" s="21" t="n"/>
-      <c r="D95" s="21" t="n"/>
-      <c r="E95" s="22" t="n"/>
+      <c r="C95" s="25" t="n"/>
+      <c r="D95" s="25" t="n"/>
+      <c r="E95" s="26" t="n"/>
     </row>
     <row r="96" ht="20.5" customHeight="1">
-      <c r="B96" s="23" t="inlineStr">
-        <is>
-          <t>Ambiente</t>
-        </is>
-      </c>
-      <c r="C96" s="24" t="inlineStr">
-        <is>
-          <t>Jardín 3</t>
-        </is>
-      </c>
-      <c r="D96" s="25" t="n"/>
-      <c r="E96" s="26" t="n"/>
+      <c r="B96" s="27" t="inlineStr">
+        <is>
+          <t>Tipo de producto</t>
+        </is>
+      </c>
+      <c r="C96" s="28" t="inlineStr">
+        <is>
+          <t>Servicio de pago único</t>
+        </is>
+      </c>
+      <c r="D96" s="29" t="n"/>
+      <c r="E96" s="30" t="n"/>
     </row>
     <row r="97" ht="20.5" customHeight="1">
-      <c r="B97" s="27" t="inlineStr">
-        <is>
-          <t>Elemento central</t>
-        </is>
-      </c>
-      <c r="C97" s="28" t="inlineStr">
-        <is>
-          <t>Fuente de agua para la ceremonia</t>
-        </is>
-      </c>
-      <c r="D97" s="29" t="n"/>
-      <c r="E97" s="30" t="n"/>
+      <c r="B97" s="31" t="inlineStr">
+        <is>
+          <t>Espacio por urna</t>
+        </is>
+      </c>
+      <c r="C97" s="32" t="inlineStr">
+        <is>
+          <t>15 × 20 cm o 15 × 30 cm, según el tamaño de la urna</t>
+        </is>
+      </c>
+      <c r="D97" s="33" t="n"/>
+      <c r="E97" s="34" t="n"/>
     </row>
     <row r="98" ht="20.5" customHeight="1">
-      <c r="B98" s="23" t="inlineStr">
-        <is>
-          <t>Entorno</t>
-        </is>
-      </c>
-      <c r="C98" s="24" t="inlineStr">
-        <is>
-          <t>Barrera visual que separa el jardín del crematorio</t>
-        </is>
-      </c>
-      <c r="D98" s="25" t="n"/>
-      <c r="E98" s="26" t="n"/>
-    </row>
-    <row r="99" ht="35" customHeight="1">
-      <c r="B99" s="27" t="inlineStr">
+      <c r="B98" s="27" t="inlineStr">
+        <is>
+          <t>Urna</t>
+        </is>
+      </c>
+      <c r="C98" s="28" t="inlineStr">
+        <is>
+          <t>Biodegradable; se integra al suelo</t>
+        </is>
+      </c>
+      <c r="D98" s="29" t="n"/>
+      <c r="E98" s="30" t="n"/>
+    </row>
+    <row r="99" ht="20.5" customHeight="1">
+      <c r="B99" s="31" t="inlineStr">
+        <is>
+          <t>Identificación</t>
+        </is>
+      </c>
+      <c r="C99" s="32" t="inlineStr">
+        <is>
+          <t>Placa de madera de 20 cm</t>
+        </is>
+      </c>
+      <c r="D99" s="33" t="n"/>
+      <c r="E99" s="34" t="n"/>
+    </row>
+    <row r="100" ht="35" customHeight="1">
+      <c r="B100" s="27" t="inlineStr">
+        <is>
+          <t>Permanencia</t>
+        </is>
+      </c>
+      <c r="C100" s="28" t="inlineStr">
+        <is>
+          <t>3 años; luego el nombre pasa a una placa memorial en el monumento y el espacio se reutiliza</t>
+        </is>
+      </c>
+      <c r="D100" s="29" t="n"/>
+      <c r="E100" s="30" t="n"/>
+    </row>
+    <row r="101" ht="20.5" customHeight="1">
+      <c r="B101" s="31" t="inlineStr">
+        <is>
+          <t>Placa memorial</t>
+        </is>
+      </c>
+      <c r="C101" s="32" t="inlineStr">
+        <is>
+          <t>US$ 50</t>
+        </is>
+      </c>
+      <c r="D101" s="33" t="n"/>
+      <c r="E101" s="34" t="n"/>
+    </row>
+    <row r="102" ht="64" customHeight="1">
+      <c r="B102" s="27" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C99" s="28" t="inlineStr">
-        <is>
-          <t>• Inhumación de urnas de cenizas
-• Ceremonia con agua en fuente</t>
-        </is>
-      </c>
-      <c r="D99" s="29" t="n"/>
-      <c r="E99" s="30" t="n"/>
-    </row>
-    <row r="100" ht="20" customHeight="1">
-      <c r="B100" s="20" t="inlineStr">
-        <is>
-          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
-        </is>
-      </c>
-      <c r="C100" s="21" t="n"/>
-      <c r="D100" s="21" t="n"/>
-      <c r="E100" s="22" t="n"/>
-    </row>
-    <row r="101" ht="26.5" customHeight="1">
-      <c r="B101" s="23" t="inlineStr">
-        <is>
-          <t>Precio sugerido</t>
-        </is>
-      </c>
-      <c r="C101" s="31" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-      <c r="D101" s="25" t="n"/>
-      <c r="E101" s="26" t="n"/>
-    </row>
-    <row r="102" ht="20.5" customHeight="1">
-      <c r="B102" s="27" t="inlineStr">
-        <is>
-          <t>Base de precio</t>
-        </is>
-      </c>
       <c r="C102" s="28" t="inlineStr">
-        <is>
-          <t>Producto en definición</t>
-        </is>
-      </c>
-      <c r="D102" s="29" t="n"/>
-      <c r="E102" s="30" t="n"/>
-    </row>
-    <row r="103" ht="20.5" customHeight="1">
-      <c r="B103" s="23" t="inlineStr">
-        <is>
-          <t>Condiciones</t>
-        </is>
-      </c>
-      <c r="C103" s="24" t="inlineStr">
-        <is>
-          <t>A definir.</t>
-        </is>
-      </c>
-      <c r="D103" s="25" t="n"/>
-      <c r="E103" s="26" t="n"/>
-    </row>
-    <row r="104" ht="20" customHeight="1">
-      <c r="B104" s="20" t="inlineStr">
-        <is>
-          <t>PERFIL DEL COMPRADOR</t>
-        </is>
-      </c>
-      <c r="C104" s="21" t="n"/>
-      <c r="D104" s="21" t="n"/>
-      <c r="E104" s="22" t="n"/>
-    </row>
-    <row r="105" ht="35" customHeight="1">
-      <c r="B105" s="32" t="inlineStr">
-        <is>
-          <t>Cliente objetivo</t>
-        </is>
-      </c>
-      <c r="C105" s="33" t="inlineStr">
-        <is>
-          <t>Familias que valoran un rito de despedida simbólico y un entorno contemplativo.</t>
-        </is>
-      </c>
-      <c r="D105" s="34" t="n"/>
-      <c r="E105" s="35" t="n"/>
-    </row>
-    <row r="108" ht="30" customHeight="1">
-      <c r="B108" s="14" t="inlineStr">
-        <is>
-          <t>JARDÍN DE MASCOTAS</t>
-        </is>
-      </c>
-      <c r="C108" s="15" t="n"/>
-      <c r="D108" s="15" t="n"/>
-      <c r="E108" s="16" t="inlineStr">
-        <is>
-          <t>VG-CRE-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="109" ht="20" customHeight="1">
-      <c r="B109" s="17" t="inlineStr">
-        <is>
-          <t>Jardines de la Memoria · Mascotas  ·  Destino final · Inhumación ecológica</t>
-        </is>
-      </c>
-      <c r="C109" s="18" t="n"/>
-      <c r="D109" s="18" t="n"/>
-      <c r="E109" s="19" t="n"/>
-    </row>
-    <row r="110" ht="20" customHeight="1">
-      <c r="B110" s="20" t="inlineStr">
-        <is>
-          <t>VISIÓN GENERAL</t>
-        </is>
-      </c>
-      <c r="C110" s="21" t="n"/>
-      <c r="D110" s="21" t="n"/>
-      <c r="E110" s="22" t="n"/>
-    </row>
-    <row r="111" ht="35" customHeight="1">
-      <c r="B111" s="23" t="inlineStr">
-        <is>
-          <t>Concepto</t>
-        </is>
-      </c>
-      <c r="C111" s="24" t="inlineStr">
-        <is>
-          <t>Jardín para inhumación ecológica de cenizas de mascotas: la urna biodegradable se entierra directamente en el suelo y se identifica con una placa de madera.</t>
-        </is>
-      </c>
-      <c r="D111" s="25" t="n"/>
-      <c r="E111" s="26" t="n"/>
-    </row>
-    <row r="112" ht="20.5" customHeight="1">
-      <c r="B112" s="27" t="inlineStr">
-        <is>
-          <t>Capacidad / Cobertura</t>
-        </is>
-      </c>
-      <c r="C112" s="28" t="inlineStr">
-        <is>
-          <t>Individual (una mascota por servicio).</t>
-        </is>
-      </c>
-      <c r="D112" s="29" t="n"/>
-      <c r="E112" s="30" t="n"/>
-    </row>
-    <row r="113" ht="20" customHeight="1">
-      <c r="B113" s="20" t="inlineStr">
-        <is>
-          <t>ESPECIFICACIONES TÉCNICAS</t>
-        </is>
-      </c>
-      <c r="C113" s="21" t="n"/>
-      <c r="D113" s="21" t="n"/>
-      <c r="E113" s="22" t="n"/>
-    </row>
-    <row r="114" ht="20.5" customHeight="1">
-      <c r="B114" s="23" t="inlineStr">
-        <is>
-          <t>Tipo de producto</t>
-        </is>
-      </c>
-      <c r="C114" s="24" t="inlineStr">
-        <is>
-          <t>Servicio de pago único</t>
-        </is>
-      </c>
-      <c r="D114" s="25" t="n"/>
-      <c r="E114" s="26" t="n"/>
-    </row>
-    <row r="115" ht="20.5" customHeight="1">
-      <c r="B115" s="27" t="inlineStr">
-        <is>
-          <t>Espacio por urna</t>
-        </is>
-      </c>
-      <c r="C115" s="28" t="inlineStr">
-        <is>
-          <t>15 × 20 cm o 15 × 30 cm, según el tamaño de la urna</t>
-        </is>
-      </c>
-      <c r="D115" s="29" t="n"/>
-      <c r="E115" s="30" t="n"/>
-    </row>
-    <row r="116" ht="20.5" customHeight="1">
-      <c r="B116" s="23" t="inlineStr">
-        <is>
-          <t>Urna</t>
-        </is>
-      </c>
-      <c r="C116" s="24" t="inlineStr">
-        <is>
-          <t>Biodegradable; se integra al suelo</t>
-        </is>
-      </c>
-      <c r="D116" s="25" t="n"/>
-      <c r="E116" s="26" t="n"/>
-    </row>
-    <row r="117" ht="20.5" customHeight="1">
-      <c r="B117" s="27" t="inlineStr">
-        <is>
-          <t>Identificación</t>
-        </is>
-      </c>
-      <c r="C117" s="28" t="inlineStr">
-        <is>
-          <t>Placa de madera de 20 cm</t>
-        </is>
-      </c>
-      <c r="D117" s="29" t="n"/>
-      <c r="E117" s="30" t="n"/>
-    </row>
-    <row r="118" ht="35" customHeight="1">
-      <c r="B118" s="23" t="inlineStr">
-        <is>
-          <t>Permanencia</t>
-        </is>
-      </c>
-      <c r="C118" s="24" t="inlineStr">
-        <is>
-          <t>3 años; luego el nombre pasa a una placa memorial en el monumento y el espacio se reutiliza</t>
-        </is>
-      </c>
-      <c r="D118" s="25" t="n"/>
-      <c r="E118" s="26" t="n"/>
-    </row>
-    <row r="119" ht="20.5" customHeight="1">
-      <c r="B119" s="27" t="inlineStr">
-        <is>
-          <t>Placa memorial</t>
-        </is>
-      </c>
-      <c r="C119" s="28" t="inlineStr">
-        <is>
-          <t>US$ 50</t>
-        </is>
-      </c>
-      <c r="D119" s="29" t="n"/>
-      <c r="E119" s="30" t="n"/>
-    </row>
-    <row r="120" ht="64" customHeight="1">
-      <c r="B120" s="23" t="inlineStr">
-        <is>
-          <t>Servicios incluidos</t>
-        </is>
-      </c>
-      <c r="C120" s="24" t="inlineStr">
         <is>
           <t>• Inhumación ecológica de la urna en el jardín
 • Placa de madera de 20 cm para identificación
@@ -2532,100 +2365,311 @@
 • Cremación de la mascota (opción Jardín + Cremación)</t>
         </is>
       </c>
-      <c r="D120" s="25" t="n"/>
-      <c r="E120" s="26" t="n"/>
-    </row>
-    <row r="121" ht="20" customHeight="1">
-      <c r="B121" s="20" t="inlineStr">
+      <c r="D102" s="29" t="n"/>
+      <c r="E102" s="30" t="n"/>
+    </row>
+    <row r="103" ht="20" customHeight="1">
+      <c r="B103" s="24" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C121" s="21" t="n"/>
-      <c r="D121" s="21" t="n"/>
-      <c r="E121" s="22" t="n"/>
-    </row>
-    <row r="122" ht="26.5" customHeight="1">
-      <c r="B122" s="23" t="inlineStr">
+      <c r="C103" s="25" t="n"/>
+      <c r="D103" s="25" t="n"/>
+      <c r="E103" s="26" t="n"/>
+    </row>
+    <row r="104" ht="26.5" customHeight="1">
+      <c r="B104" s="27" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C122" s="31" t="inlineStr">
+      <c r="C104" s="35" t="inlineStr">
         <is>
           <t>US$ 350 / US$ 500</t>
         </is>
       </c>
+      <c r="D104" s="29" t="n"/>
+      <c r="E104" s="30" t="n"/>
+    </row>
+    <row r="105" ht="20.5" customHeight="1">
+      <c r="B105" s="31" t="inlineStr">
+        <is>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C105" s="32" t="inlineStr">
+        <is>
+          <t>US$ 350 solo jardín · US$ 500 jardín + cremación</t>
+        </is>
+      </c>
+      <c r="D105" s="33" t="n"/>
+      <c r="E105" s="34" t="n"/>
+    </row>
+    <row r="106" ht="35" customHeight="1">
+      <c r="B106" s="27" t="inlineStr">
+        <is>
+          <t>Condiciones</t>
+        </is>
+      </c>
+      <c r="C106" s="28" t="inlineStr">
+        <is>
+          <t>Pago único; puede contratarse como adicional al plan funerario. Placa memorial en el monumento al término del plazo: US$ 50.</t>
+        </is>
+      </c>
+      <c r="D106" s="29" t="n"/>
+      <c r="E106" s="30" t="n"/>
+    </row>
+    <row r="107" ht="20" customHeight="1">
+      <c r="B107" s="24" t="inlineStr">
+        <is>
+          <t>PERFIL DEL COMPRADOR</t>
+        </is>
+      </c>
+      <c r="C107" s="25" t="n"/>
+      <c r="D107" s="25" t="n"/>
+      <c r="E107" s="26" t="n"/>
+    </row>
+    <row r="108" ht="20.5" customHeight="1">
+      <c r="B108" s="36" t="inlineStr">
+        <is>
+          <t>Cliente objetivo</t>
+        </is>
+      </c>
+      <c r="C108" s="37" t="inlineStr">
+        <is>
+          <t>Familias que consideran a su mascota parte del hogar y desean un cierre digno.</t>
+        </is>
+      </c>
+      <c r="D108" s="38" t="n"/>
+      <c r="E108" s="39" t="n"/>
+    </row>
+    <row r="111" ht="30" customHeight="1">
+      <c r="B111" s="18" t="inlineStr">
+        <is>
+          <t>JARDÍN DE CENIZAS · CEREMONIAL</t>
+        </is>
+      </c>
+      <c r="C111" s="19" t="n"/>
+      <c r="D111" s="19" t="n"/>
+      <c r="E111" s="20" t="inlineStr">
+        <is>
+          <t>VG-CRE-03C</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="20" customHeight="1">
+      <c r="B112" s="21" t="inlineStr">
+        <is>
+          <t>Jardines de la Memoria · Jardín 3  ·  Destino final · Inhumación con ceremonia</t>
+        </is>
+      </c>
+      <c r="C112" s="22" t="n"/>
+      <c r="D112" s="22" t="n"/>
+      <c r="E112" s="23" t="n"/>
+    </row>
+    <row r="113" ht="24" customHeight="1">
+      <c r="B113" s="40" t="inlineStr">
+        <is>
+          <t>★  PRÓXIMO LANZAMIENTO · se lanzará en otro momento</t>
+        </is>
+      </c>
+      <c r="C113" s="41" t="n"/>
+      <c r="D113" s="41" t="n"/>
+      <c r="E113" s="42" t="n"/>
+    </row>
+    <row r="114" ht="20" customHeight="1">
+      <c r="B114" s="24" t="inlineStr">
+        <is>
+          <t>VISIÓN GENERAL</t>
+        </is>
+      </c>
+      <c r="C114" s="25" t="n"/>
+      <c r="D114" s="25" t="n"/>
+      <c r="E114" s="26" t="n"/>
+    </row>
+    <row r="115" ht="35" customHeight="1">
+      <c r="B115" s="27" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="C115" s="28" t="inlineStr">
+        <is>
+          <t>Jardín para inhumación de urnas de cenizas con ceremonia de agua, con fuentes como elemento central del rito de despedida.</t>
+        </is>
+      </c>
+      <c r="D115" s="29" t="n"/>
+      <c r="E115" s="30" t="n"/>
+    </row>
+    <row r="116" ht="20.5" customHeight="1">
+      <c r="B116" s="31" t="inlineStr">
+        <is>
+          <t>Capacidad / Cobertura</t>
+        </is>
+      </c>
+      <c r="C116" s="32" t="inlineStr">
+        <is>
+          <t>A definir.</t>
+        </is>
+      </c>
+      <c r="D116" s="33" t="n"/>
+      <c r="E116" s="34" t="n"/>
+    </row>
+    <row r="117" ht="20" customHeight="1">
+      <c r="B117" s="24" t="inlineStr">
+        <is>
+          <t>ESPECIFICACIONES TÉCNICAS</t>
+        </is>
+      </c>
+      <c r="C117" s="25" t="n"/>
+      <c r="D117" s="25" t="n"/>
+      <c r="E117" s="26" t="n"/>
+    </row>
+    <row r="118" ht="20.5" customHeight="1">
+      <c r="B118" s="27" t="inlineStr">
+        <is>
+          <t>Ambiente</t>
+        </is>
+      </c>
+      <c r="C118" s="28" t="inlineStr">
+        <is>
+          <t>Jardín 3</t>
+        </is>
+      </c>
+      <c r="D118" s="29" t="n"/>
+      <c r="E118" s="30" t="n"/>
+    </row>
+    <row r="119" ht="20.5" customHeight="1">
+      <c r="B119" s="31" t="inlineStr">
+        <is>
+          <t>Elemento central</t>
+        </is>
+      </c>
+      <c r="C119" s="32" t="inlineStr">
+        <is>
+          <t>Fuente de agua para la ceremonia</t>
+        </is>
+      </c>
+      <c r="D119" s="33" t="n"/>
+      <c r="E119" s="34" t="n"/>
+    </row>
+    <row r="120" ht="20.5" customHeight="1">
+      <c r="B120" s="27" t="inlineStr">
+        <is>
+          <t>Entorno</t>
+        </is>
+      </c>
+      <c r="C120" s="28" t="inlineStr">
+        <is>
+          <t>Barrera visual que separa el jardín del crematorio</t>
+        </is>
+      </c>
+      <c r="D120" s="29" t="n"/>
+      <c r="E120" s="30" t="n"/>
+    </row>
+    <row r="121" ht="35" customHeight="1">
+      <c r="B121" s="31" t="inlineStr">
+        <is>
+          <t>Servicios incluidos</t>
+        </is>
+      </c>
+      <c r="C121" s="32" t="inlineStr">
+        <is>
+          <t>• Inhumación de urnas de cenizas
+• Ceremonia con agua en fuente</t>
+        </is>
+      </c>
+      <c r="D121" s="33" t="n"/>
+      <c r="E121" s="34" t="n"/>
+    </row>
+    <row r="122" ht="20" customHeight="1">
+      <c r="B122" s="24" t="inlineStr">
+        <is>
+          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
+        </is>
+      </c>
+      <c r="C122" s="25" t="n"/>
       <c r="D122" s="25" t="n"/>
       <c r="E122" s="26" t="n"/>
     </row>
-    <row r="123" ht="20.5" customHeight="1">
+    <row r="123" ht="26.5" customHeight="1">
       <c r="B123" s="27" t="inlineStr">
         <is>
-          <t>Base de precio</t>
-        </is>
-      </c>
-      <c r="C123" s="28" t="inlineStr">
-        <is>
-          <t>US$ 350 solo jardín · US$ 500 jardín + cremación</t>
+          <t>Precio sugerido</t>
+        </is>
+      </c>
+      <c r="C123" s="35" t="inlineStr">
+        <is>
+          <t>A definir</t>
         </is>
       </c>
       <c r="D123" s="29" t="n"/>
       <c r="E123" s="30" t="n"/>
     </row>
-    <row r="124" ht="35" customHeight="1">
-      <c r="B124" s="23" t="inlineStr">
+    <row r="124" ht="20.5" customHeight="1">
+      <c r="B124" s="31" t="inlineStr">
+        <is>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C124" s="32" t="inlineStr">
+        <is>
+          <t>Producto en definición</t>
+        </is>
+      </c>
+      <c r="D124" s="33" t="n"/>
+      <c r="E124" s="34" t="n"/>
+    </row>
+    <row r="125" ht="20.5" customHeight="1">
+      <c r="B125" s="27" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C124" s="24" t="inlineStr">
-        <is>
-          <t>Pago único; puede contratarse como adicional al plan funerario. Placa memorial en el monumento al término del plazo: US$ 50.</t>
-        </is>
-      </c>
-      <c r="D124" s="25" t="n"/>
-      <c r="E124" s="26" t="n"/>
-    </row>
-    <row r="125" ht="20" customHeight="1">
-      <c r="B125" s="20" t="inlineStr">
+      <c r="C125" s="28" t="inlineStr">
+        <is>
+          <t>A definir.</t>
+        </is>
+      </c>
+      <c r="D125" s="29" t="n"/>
+      <c r="E125" s="30" t="n"/>
+    </row>
+    <row r="126" ht="20" customHeight="1">
+      <c r="B126" s="24" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C125" s="21" t="n"/>
-      <c r="D125" s="21" t="n"/>
-      <c r="E125" s="22" t="n"/>
-    </row>
-    <row r="126" ht="20.5" customHeight="1">
-      <c r="B126" s="32" t="inlineStr">
+      <c r="C126" s="25" t="n"/>
+      <c r="D126" s="25" t="n"/>
+      <c r="E126" s="26" t="n"/>
+    </row>
+    <row r="127" ht="35" customHeight="1">
+      <c r="B127" s="36" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C126" s="33" t="inlineStr">
-        <is>
-          <t>Familias que consideran a su mascota parte del hogar y desean un cierre digno.</t>
-        </is>
-      </c>
-      <c r="D126" s="34" t="n"/>
-      <c r="E126" s="35" t="n"/>
+      <c r="C127" s="37" t="inlineStr">
+        <is>
+          <t>Familias que valoran un rito de despedida simbólico y un entorno contemplativo.</t>
+        </is>
+      </c>
+      <c r="D127" s="38" t="n"/>
+      <c r="E127" s="39" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="115">
+  <mergeCells count="116">
     <mergeCell ref="C31:E31"/>
     <mergeCell ref="C80:E80"/>
     <mergeCell ref="B68:E68"/>
     <mergeCell ref="C40:E40"/>
     <mergeCell ref="C60:E60"/>
-    <mergeCell ref="B110:E110"/>
     <mergeCell ref="C71:E71"/>
-    <mergeCell ref="B108:D108"/>
     <mergeCell ref="B113:E113"/>
     <mergeCell ref="C123:E123"/>
     <mergeCell ref="B91:E91"/>
-    <mergeCell ref="B100:E100"/>
-    <mergeCell ref="B109:E109"/>
     <mergeCell ref="B47:E47"/>
     <mergeCell ref="C7:E7"/>
     <mergeCell ref="C57:E57"/>
@@ -2639,23 +2683,22 @@
     <mergeCell ref="C34:E34"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="C74:E74"/>
-    <mergeCell ref="C126:E126"/>
     <mergeCell ref="B69:E69"/>
     <mergeCell ref="B38:E38"/>
+    <mergeCell ref="B112:E112"/>
     <mergeCell ref="C20:E20"/>
-    <mergeCell ref="C103:E103"/>
     <mergeCell ref="C85:E85"/>
-    <mergeCell ref="C112:E112"/>
+    <mergeCell ref="B111:D111"/>
     <mergeCell ref="C99:E99"/>
     <mergeCell ref="C94:E94"/>
     <mergeCell ref="C118:E118"/>
     <mergeCell ref="C75:E75"/>
     <mergeCell ref="C84:E84"/>
     <mergeCell ref="C22:E22"/>
-    <mergeCell ref="B104:E104"/>
-    <mergeCell ref="C114:E114"/>
+    <mergeCell ref="C127:E127"/>
     <mergeCell ref="B51:E51"/>
     <mergeCell ref="C12:E12"/>
+    <mergeCell ref="B114:E114"/>
     <mergeCell ref="B63:E63"/>
     <mergeCell ref="B26:E26"/>
     <mergeCell ref="C52:E52"/>
@@ -2663,21 +2706,26 @@
     <mergeCell ref="C39:E39"/>
     <mergeCell ref="B16:E16"/>
     <mergeCell ref="C70:E70"/>
+    <mergeCell ref="C106:E106"/>
     <mergeCell ref="C32:E32"/>
     <mergeCell ref="C81:E81"/>
+    <mergeCell ref="C125:E125"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="C13:E13"/>
     <mergeCell ref="C87:E87"/>
+    <mergeCell ref="B117:E117"/>
     <mergeCell ref="C15:E15"/>
     <mergeCell ref="C33:E33"/>
+    <mergeCell ref="C104:E104"/>
     <mergeCell ref="C116:E116"/>
     <mergeCell ref="B46:D46"/>
     <mergeCell ref="C79:E79"/>
     <mergeCell ref="C73:E73"/>
+    <mergeCell ref="B103:E103"/>
     <mergeCell ref="C35:E35"/>
+    <mergeCell ref="C121:E121"/>
     <mergeCell ref="C10:E10"/>
     <mergeCell ref="C50:E50"/>
-    <mergeCell ref="C117:E117"/>
     <mergeCell ref="C55:E55"/>
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="B95:E95"/>
@@ -2685,8 +2733,7 @@
     <mergeCell ref="C36:E36"/>
     <mergeCell ref="C11:E11"/>
     <mergeCell ref="B72:E72"/>
-    <mergeCell ref="C122:E122"/>
-    <mergeCell ref="B121:E121"/>
+    <mergeCell ref="B122:E122"/>
     <mergeCell ref="C28:E28"/>
     <mergeCell ref="C37:E37"/>
     <mergeCell ref="C96:E96"/>
@@ -2694,6 +2741,7 @@
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="B25:D25"/>
     <mergeCell ref="B42:E42"/>
+    <mergeCell ref="B107:E107"/>
     <mergeCell ref="C62:E62"/>
     <mergeCell ref="C14:E14"/>
     <mergeCell ref="C98:E98"/>
@@ -2712,22 +2760,23 @@
     <mergeCell ref="C43:E43"/>
     <mergeCell ref="C76:E76"/>
     <mergeCell ref="C120:E120"/>
+    <mergeCell ref="B126:E126"/>
     <mergeCell ref="C119:E119"/>
     <mergeCell ref="C8:E8"/>
     <mergeCell ref="C17:E17"/>
     <mergeCell ref="B59:E59"/>
-    <mergeCell ref="B125:E125"/>
     <mergeCell ref="C19:E19"/>
     <mergeCell ref="C53:E53"/>
     <mergeCell ref="C102:E102"/>
-    <mergeCell ref="C111:E111"/>
     <mergeCell ref="B48:E48"/>
     <mergeCell ref="C83:E83"/>
+    <mergeCell ref="C108:E108"/>
     <mergeCell ref="C58:E58"/>
     <mergeCell ref="B90:D90"/>
     <mergeCell ref="B82:E82"/>
     <mergeCell ref="C97:E97"/>
     <mergeCell ref="C29:E29"/>
+    <mergeCell ref="C100:E100"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -2736,7 +2785,7 @@
     <brk id="44" min="0" max="16383" man="1"/>
     <brk id="65" min="0" max="16383" man="1"/>
     <brk id="88" min="0" max="16383" man="1"/>
-    <brk id="106" min="0" max="16383" man="1"/>
+    <brk id="109" min="0" max="16383" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Alinea Excel y HTML con la Planilha Google: sin ID de producto ni nota de USD
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111i7vn9WWo4QxCQbucWbrF
</commit_message>
<xml_diff>
--- a/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
+++ b/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Ficha Técnica Consolidada" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tabla Gral. - Visión Comercial'!$A$4:$I$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tabla Gral. - Visión Comercial'!$A$4:$H$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Tabla Gral. - Visión Comercial'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Ficha Técnica Consolidada'!$A$1:$F$128</definedName>
   </definedNames>
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,12 +58,6 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001B365D"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001B365D"/>
       <sz val="11"/>
     </font>
     <font>
@@ -86,12 +80,6 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00D4AF37"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
@@ -100,6 +88,12 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="000F2537"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001B365D"/>
       <sz val="10"/>
     </font>
     <font>
@@ -276,7 +270,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -288,65 +282,54 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -354,7 +337,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -362,10 +345,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -373,7 +356,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -744,18 +727,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="46" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -768,52 +750,47 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Campaña Día de los Muertos 2026  ·  Precios sugeridos en dólares estadounidenses (USD)</t>
+          <t>Campaña Día de los Muertos 2026</t>
         </is>
       </c>
     </row>
     <row r="4" ht="36" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>ID del Producto</t>
+          <t>Nombre Comercial</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Nombre Comercial</t>
+          <t>Categoría / Línea</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Categoría / Línea</t>
+          <t>Concepto / Descripción</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Concepto / Descripción</t>
+          <t>Capacidad / Cobertura</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Capacidad / Cobertura</t>
+          <t>Servicios Incluidos &amp; Diferenciales</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Servicios Incluidos &amp; Diferenciales</t>
+          <t>Perfil de Cliente</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Perfil de Cliente</t>
+          <t>Precio Sugerido (USD)</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Precio Sugerido (USD)</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Condiciones de Pago / Financiamiento</t>
         </is>
@@ -822,30 +799,25 @@
     <row r="5" ht="93" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>VG-CRE-01</t>
+          <t>Solución Modular de Cremación</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Solución Modular de Cremación</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
           <t>Cremación · Módulo add-on</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Módulo de cremación integrable a cualquier plan funerario vigente o nuevo de Vangrupo, sin necesidad de cambiar de plan.</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Individual (1 titular / beneficiario por módulo).</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>• Proceso completo de cremación individual
 • Urna cineraria de línea modular
@@ -854,50 +826,45 @@
 • Integración al plan funerario base (actual o nuevo)</t>
         </is>
       </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Afiliados actuales y nuevos que desean incorporar la cremación a su plan con una cuota mensual mínima.</t>
+        </is>
+      </c>
       <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>Afiliados actuales y nuevos que desean incorporar la cremación a su plan con una cuota mensual mínima.</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>US$ 1.000
 (Por módulo individual)</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>Hasta 120 cuotas mensuales (aprox. US$ 8,50/mes).</t>
         </is>
       </c>
     </row>
     <row r="6" ht="78.5" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>VG-CRE-03I</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Jardín de Cenizas · Individual</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Destino final · Inhumación individual</t>
         </is>
       </c>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>Inhumación de la urna de cenizas en un contenedor enterrado con tapa de granito grabada, en un jardín de plantas de sombra: un lugar físico permanente de homenaje.</t>
         </is>
       </c>
-      <c r="E6" s="10" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>Individual (1 urna).</t>
         </is>
       </c>
-      <c r="F6" s="10" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>• Inhumación de la urna en contenedor individual
 • Tapa de granito con los datos del difunto
@@ -905,18 +872,18 @@
 • Espacio de contemplación con banco</t>
         </is>
       </c>
-      <c r="G6" s="10" t="inlineStr">
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>Familias que desean un lugar permanente para visitar y rendir homenaje, con una inversión moderada.</t>
         </is>
       </c>
-      <c r="H6" s="11" t="inlineStr">
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>US$ 600
 (Por espacio individual · mantenimiento US$ 15/año)</t>
         </is>
       </c>
-      <c r="I6" s="10" t="inlineStr">
+      <c r="H6" s="8" t="inlineStr">
         <is>
           <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 15 anual.</t>
         </is>
@@ -925,30 +892,25 @@
     <row r="7" ht="93" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>VG-CRE-03F</t>
+          <t>Jardín de Cenizas · Familiar</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Jardín de Cenizas · Familiar</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
           <t>Destino final · Inhumación familiar</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Parcela familiar en el Jardín 1 con cuatro contenedores agrupados, cada uno con tapa de granito grabada, sin plazo de permanencia.</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Hasta 4 espacios (familiar).</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>• Inhumación de hasta 4 urnas
 • Tapa de granito grabada para cada espacio
@@ -956,50 +918,45 @@
 • Lugar físico permanente de homenaje familiar, sin plazo</t>
         </is>
       </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Familias que buscan un espacio propio y permanente para varias generaciones.</t>
+        </is>
+      </c>
       <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Familias que buscan un espacio propio y permanente para varias generaciones.</t>
-        </is>
-      </c>
-      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>US$ 2.000
 (Por parcela familiar · hasta 4 espacios · mantenimiento US$ 25/año)</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 25 anual.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="122" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>VG-CRE-03E</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Jardín de Cenizas · Ecológico</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Destino final · Inhumación ecológica</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>La urna biodegradable se entierra directamente en el suelo, se cubre con tierra y se descompone integrándose a la naturaleza. Jardín con agua corriente y área de esparcimiento de cenizas.</t>
         </is>
       </c>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>Individual (1 urna).</t>
         </is>
       </c>
-      <c r="F8" s="10" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>• Inhumación ecológica de la urna directamente en el suelo
 • Placa de identificación
@@ -1008,18 +965,18 @@
 • Permanencia de 3 años; luego, placa memorial en el monumento</t>
         </is>
       </c>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>Personas con conciencia ambiental que desean que sus cenizas vuelvan a la tierra, con un lugar identificado para visitar.</t>
         </is>
       </c>
-      <c r="H8" s="11" t="inlineStr">
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>US$ 600
 (Por espacio individual · placa memorial US$ 150)</t>
         </is>
       </c>
-      <c r="I8" s="10" t="inlineStr">
+      <c r="H8" s="8" t="inlineStr">
         <is>
           <t>Pago único o financiado según política comercial vigente. Placa memorial en el monumento al término del plazo: US$ 150.</t>
         </is>
@@ -1028,30 +985,25 @@
     <row r="9" ht="93" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>VG-CRE-04</t>
+          <t>Jardín de Mascotas</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Jardín de Mascotas</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
           <t>Destino final · Inhumación ecológica</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Jardín para inhumación ecológica de cenizas de mascotas: la urna biodegradable se entierra directamente en el suelo y se identifica con una placa de madera.</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>Individual (una mascota por servicio).</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>• Inhumación ecológica de la urna en el jardín
 • Placa de madera de 20 cm para identificación
@@ -1059,78 +1011,73 @@
 • Cremación de la mascota (opción Jardín + Cremación)</t>
         </is>
       </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Familias que consideran a su mascota parte del hogar y desean un cierre digno.</t>
+        </is>
+      </c>
       <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>Familias que consideran a su mascota parte del hogar y desean un cierre digno.</t>
-        </is>
-      </c>
-      <c r="H9" s="7" t="inlineStr">
         <is>
           <t>US$ 350 / US$ 500
 (US$ 350 solo jardín · US$ 500 jardín + cremación)</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>Pago único; puede contratarse como adicional al plan funerario. Placa memorial en el monumento al término del plazo: US$ 50.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="49.5" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>VG-CRE-03C</t>
-        </is>
-      </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Jardín de Cenizas · Ceremonial
 ★ PRÓXIMO LANZAMIENTO</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Destino final · Inhumación con ceremonia</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>Jardín para inhumación de urnas de cenizas con ceremonia de agua, con fuentes como elemento central del rito de despedida.</t>
         </is>
       </c>
-      <c r="E10" s="14" t="inlineStr">
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>A definir.</t>
         </is>
       </c>
-      <c r="F10" s="14" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>• Inhumación de urnas de cenizas
 • Ceremonia con agua en fuente</t>
         </is>
       </c>
-      <c r="G10" s="14" t="inlineStr">
+      <c r="F10" s="11" t="inlineStr">
         <is>
           <t>Familias que valoran un rito de despedida simbólico y un entorno contemplativo.</t>
         </is>
       </c>
-      <c r="H10" s="15" t="inlineStr">
+      <c r="G10" s="12" t="inlineStr">
         <is>
           <t>A definir
 (Producto en definición)</t>
         </is>
       </c>
-      <c r="I10" s="14" t="inlineStr">
+      <c r="H10" s="11" t="inlineStr">
         <is>
           <t>A definir.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I10"/>
+  <autoFilter ref="A4:H10"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -1156,168 +1103,164 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="B1" s="16" t="inlineStr">
+      <c r="B1" s="13" t="inlineStr">
         <is>
           <t>FICHA TÉCNICA CONSOLIDADA  ·  LA AUXILIADORA · VANGRUPO</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="17" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
         <is>
           <t>Portafolio de Cremación — Campaña Día de los Muertos 2026</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>SOLUCIÓN MODULAR DE CREMACIÓN</t>
         </is>
       </c>
-      <c r="C4" s="19" t="n"/>
-      <c r="D4" s="19" t="n"/>
-      <c r="E4" s="20" t="inlineStr">
-        <is>
-          <t>VG-CRE-01</t>
-        </is>
-      </c>
+      <c r="C4" s="16" t="n"/>
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="17" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="B5" s="21" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>Línea Cremación Modular  ·  Cremación · Módulo add-on</t>
         </is>
       </c>
-      <c r="C5" s="22" t="n"/>
-      <c r="D5" s="22" t="n"/>
-      <c r="E5" s="23" t="n"/>
+      <c r="C5" s="19" t="n"/>
+      <c r="D5" s="19" t="n"/>
+      <c r="E5" s="20" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="B6" s="24" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C6" s="25" t="n"/>
-      <c r="D6" s="25" t="n"/>
-      <c r="E6" s="26" t="n"/>
+      <c r="C6" s="22" t="n"/>
+      <c r="D6" s="22" t="n"/>
+      <c r="E6" s="23" t="n"/>
     </row>
     <row r="7" ht="35" customHeight="1">
-      <c r="B7" s="27" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C7" s="28" t="inlineStr">
+      <c r="C7" s="25" t="inlineStr">
         <is>
           <t>Módulo de cremación integrable a cualquier plan funerario vigente o nuevo de Vangrupo, sin necesidad de cambiar de plan.</t>
         </is>
       </c>
-      <c r="D7" s="29" t="n"/>
-      <c r="E7" s="30" t="n"/>
+      <c r="D7" s="26" t="n"/>
+      <c r="E7" s="27" t="n"/>
     </row>
     <row r="8" ht="20.5" customHeight="1">
-      <c r="B8" s="31" t="inlineStr">
+      <c r="B8" s="28" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C8" s="32" t="inlineStr">
+      <c r="C8" s="29" t="inlineStr">
         <is>
           <t>Individual (1 titular / beneficiario por módulo).</t>
         </is>
       </c>
-      <c r="D8" s="33" t="n"/>
-      <c r="E8" s="34" t="n"/>
+      <c r="D8" s="30" t="n"/>
+      <c r="E8" s="31" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="B9" s="24" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C9" s="25" t="n"/>
-      <c r="D9" s="25" t="n"/>
-      <c r="E9" s="26" t="n"/>
+      <c r="C9" s="22" t="n"/>
+      <c r="D9" s="22" t="n"/>
+      <c r="E9" s="23" t="n"/>
     </row>
     <row r="10" ht="20.5" customHeight="1">
-      <c r="B10" s="27" t="inlineStr">
+      <c r="B10" s="24" t="inlineStr">
         <is>
           <t>Tipo de producto</t>
         </is>
       </c>
-      <c r="C10" s="28" t="inlineStr">
+      <c r="C10" s="25" t="inlineStr">
         <is>
           <t>Módulo adicional (add-on) a plan funerario</t>
         </is>
       </c>
-      <c r="D10" s="29" t="n"/>
-      <c r="E10" s="30" t="n"/>
+      <c r="D10" s="26" t="n"/>
+      <c r="E10" s="27" t="n"/>
     </row>
     <row r="11" ht="20.5" customHeight="1">
-      <c r="B11" s="31" t="inlineStr">
+      <c r="B11" s="28" t="inlineStr">
         <is>
           <t>Modalidad de cremación</t>
         </is>
       </c>
-      <c r="C11" s="32" t="inlineStr">
+      <c r="C11" s="29" t="inlineStr">
         <is>
           <t>Individual</t>
         </is>
       </c>
-      <c r="D11" s="33" t="n"/>
-      <c r="E11" s="34" t="n"/>
+      <c r="D11" s="30" t="n"/>
+      <c r="E11" s="31" t="n"/>
     </row>
     <row r="12" ht="20.5" customHeight="1">
-      <c r="B12" s="27" t="inlineStr">
+      <c r="B12" s="24" t="inlineStr">
         <is>
           <t>Urna</t>
         </is>
       </c>
-      <c r="C12" s="28" t="inlineStr">
+      <c r="C12" s="25" t="inlineStr">
         <is>
           <t>Cineraria, línea modular</t>
         </is>
       </c>
-      <c r="D12" s="29" t="n"/>
-      <c r="E12" s="30" t="n"/>
+      <c r="D12" s="26" t="n"/>
+      <c r="E12" s="27" t="n"/>
     </row>
     <row r="13" ht="20.5" customHeight="1">
-      <c r="B13" s="31" t="inlineStr">
+      <c r="B13" s="28" t="inlineStr">
         <is>
           <t>Gestión legal</t>
         </is>
       </c>
-      <c r="C13" s="32" t="inlineStr">
+      <c r="C13" s="29" t="inlineStr">
         <is>
           <t>Trámites básicos incluidos</t>
         </is>
       </c>
-      <c r="D13" s="33" t="n"/>
-      <c r="E13" s="34" t="n"/>
+      <c r="D13" s="30" t="n"/>
+      <c r="E13" s="31" t="n"/>
     </row>
     <row r="14" ht="20.5" customHeight="1">
-      <c r="B14" s="27" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t>Columbario</t>
         </is>
       </c>
-      <c r="C14" s="28" t="inlineStr">
+      <c r="C14" s="25" t="inlineStr">
         <is>
           <t>Alquiler temporal · 12 meses incluido</t>
         </is>
       </c>
-      <c r="D14" s="29" t="n"/>
-      <c r="E14" s="30" t="n"/>
+      <c r="D14" s="26" t="n"/>
+      <c r="E14" s="27" t="n"/>
     </row>
     <row r="15" ht="78.5" customHeight="1">
-      <c r="B15" s="31" t="inlineStr">
+      <c r="B15" s="28" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C15" s="32" t="inlineStr">
+      <c r="C15" s="29" t="inlineStr">
         <is>
           <t>• Proceso completo de cremación individual
 • Urna cineraria de línea modular
@@ -1326,262 +1269,258 @@
 • Integración al plan funerario base (actual o nuevo)</t>
         </is>
       </c>
-      <c r="D15" s="33" t="n"/>
-      <c r="E15" s="34" t="n"/>
+      <c r="D15" s="30" t="n"/>
+      <c r="E15" s="31" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="B16" s="24" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C16" s="25" t="n"/>
-      <c r="D16" s="25" t="n"/>
-      <c r="E16" s="26" t="n"/>
+      <c r="C16" s="22" t="n"/>
+      <c r="D16" s="22" t="n"/>
+      <c r="E16" s="23" t="n"/>
     </row>
     <row r="17" ht="26.5" customHeight="1">
-      <c r="B17" s="27" t="inlineStr">
+      <c r="B17" s="24" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C17" s="35" t="inlineStr">
+      <c r="C17" s="32" t="inlineStr">
         <is>
           <t>US$ 1.000</t>
         </is>
       </c>
-      <c r="D17" s="29" t="n"/>
-      <c r="E17" s="30" t="n"/>
+      <c r="D17" s="26" t="n"/>
+      <c r="E17" s="27" t="n"/>
     </row>
     <row r="18" ht="20.5" customHeight="1">
-      <c r="B18" s="31" t="inlineStr">
+      <c r="B18" s="28" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C18" s="32" t="inlineStr">
+      <c r="C18" s="29" t="inlineStr">
         <is>
           <t>Por módulo individual</t>
         </is>
       </c>
-      <c r="D18" s="33" t="n"/>
-      <c r="E18" s="34" t="n"/>
+      <c r="D18" s="30" t="n"/>
+      <c r="E18" s="31" t="n"/>
     </row>
     <row r="19" ht="20.5" customHeight="1">
-      <c r="B19" s="27" t="inlineStr">
+      <c r="B19" s="24" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C19" s="28" t="inlineStr">
+      <c r="C19" s="25" t="inlineStr">
         <is>
           <t>Hasta 120 cuotas mensuales (aprox. US$ 8,50/mes).</t>
         </is>
       </c>
-      <c r="D19" s="29" t="n"/>
-      <c r="E19" s="30" t="n"/>
+      <c r="D19" s="26" t="n"/>
+      <c r="E19" s="27" t="n"/>
     </row>
     <row r="20" ht="20.5" customHeight="1">
-      <c r="B20" s="31" t="inlineStr">
+      <c r="B20" s="28" t="inlineStr">
         <is>
           <t>Cuota referencial</t>
         </is>
       </c>
-      <c r="C20" s="32" t="inlineStr">
+      <c r="C20" s="29" t="inlineStr">
         <is>
           <t>US$ 8,33/mes sin intereses (120 cuotas)</t>
         </is>
       </c>
-      <c r="D20" s="33" t="n"/>
-      <c r="E20" s="34" t="n"/>
+      <c r="D20" s="30" t="n"/>
+      <c r="E20" s="31" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="B21" s="24" t="inlineStr">
+      <c r="B21" s="21" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C21" s="25" t="n"/>
-      <c r="D21" s="25" t="n"/>
-      <c r="E21" s="26" t="n"/>
+      <c r="C21" s="22" t="n"/>
+      <c r="D21" s="22" t="n"/>
+      <c r="E21" s="23" t="n"/>
     </row>
     <row r="22" ht="35" customHeight="1">
-      <c r="B22" s="36" t="inlineStr">
+      <c r="B22" s="33" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C22" s="37" t="inlineStr">
+      <c r="C22" s="34" t="inlineStr">
         <is>
           <t>Afiliados actuales y nuevos que desean incorporar la cremación a su plan con una cuota mensual mínima.</t>
         </is>
       </c>
-      <c r="D22" s="38" t="n"/>
-      <c r="E22" s="39" t="n"/>
+      <c r="D22" s="35" t="n"/>
+      <c r="E22" s="36" t="n"/>
     </row>
     <row r="25" ht="30" customHeight="1">
-      <c r="B25" s="18" t="inlineStr">
+      <c r="B25" s="15" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · INDIVIDUAL</t>
         </is>
       </c>
-      <c r="C25" s="19" t="n"/>
-      <c r="D25" s="19" t="n"/>
-      <c r="E25" s="20" t="inlineStr">
-        <is>
-          <t>VG-CRE-03I</t>
-        </is>
-      </c>
+      <c r="C25" s="16" t="n"/>
+      <c r="D25" s="16" t="n"/>
+      <c r="E25" s="17" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="B26" s="21" t="inlineStr">
+      <c r="B26" s="18" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Jardín 1  ·  Destino final · Inhumación individual</t>
         </is>
       </c>
-      <c r="C26" s="22" t="n"/>
-      <c r="D26" s="22" t="n"/>
-      <c r="E26" s="23" t="n"/>
+      <c r="C26" s="19" t="n"/>
+      <c r="D26" s="19" t="n"/>
+      <c r="E26" s="20" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="B27" s="24" t="inlineStr">
+      <c r="B27" s="21" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C27" s="25" t="n"/>
-      <c r="D27" s="25" t="n"/>
-      <c r="E27" s="26" t="n"/>
+      <c r="C27" s="22" t="n"/>
+      <c r="D27" s="22" t="n"/>
+      <c r="E27" s="23" t="n"/>
     </row>
     <row r="28" ht="49.5" customHeight="1">
-      <c r="B28" s="27" t="inlineStr">
+      <c r="B28" s="24" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C28" s="28" t="inlineStr">
+      <c r="C28" s="25" t="inlineStr">
         <is>
           <t>Inhumación de la urna de cenizas en un contenedor enterrado con tapa de granito grabada, en un jardín de plantas de sombra: un lugar físico permanente de homenaje.</t>
         </is>
       </c>
-      <c r="D28" s="29" t="n"/>
-      <c r="E28" s="30" t="n"/>
+      <c r="D28" s="26" t="n"/>
+      <c r="E28" s="27" t="n"/>
     </row>
     <row r="29" ht="20.5" customHeight="1">
-      <c r="B29" s="31" t="inlineStr">
+      <c r="B29" s="28" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C29" s="32" t="inlineStr">
+      <c r="C29" s="29" t="inlineStr">
         <is>
           <t>Individual (1 urna).</t>
         </is>
       </c>
-      <c r="D29" s="33" t="n"/>
-      <c r="E29" s="34" t="n"/>
+      <c r="D29" s="30" t="n"/>
+      <c r="E29" s="31" t="n"/>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="B30" s="24" t="inlineStr">
+      <c r="B30" s="21" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C30" s="25" t="n"/>
-      <c r="D30" s="25" t="n"/>
-      <c r="E30" s="26" t="n"/>
+      <c r="C30" s="22" t="n"/>
+      <c r="D30" s="22" t="n"/>
+      <c r="E30" s="23" t="n"/>
     </row>
     <row r="31" ht="20.5" customHeight="1">
-      <c r="B31" s="27" t="inlineStr">
+      <c r="B31" s="24" t="inlineStr">
         <is>
           <t>Ambiente</t>
         </is>
       </c>
-      <c r="C31" s="28" t="inlineStr">
+      <c r="C31" s="25" t="inlineStr">
         <is>
           <t>Jardín 1</t>
         </is>
       </c>
-      <c r="D31" s="29" t="n"/>
-      <c r="E31" s="30" t="n"/>
+      <c r="D31" s="26" t="n"/>
+      <c r="E31" s="27" t="n"/>
     </row>
     <row r="32" ht="20.5" customHeight="1">
-      <c r="B32" s="31" t="inlineStr">
+      <c r="B32" s="28" t="inlineStr">
         <is>
           <t>Contenedor</t>
         </is>
       </c>
-      <c r="C32" s="32" t="inlineStr">
+      <c r="C32" s="29" t="inlineStr">
         <is>
           <t>Ø 32 cm × 40 cm de altura; enterrado dejando 20 cm a la vista</t>
         </is>
       </c>
-      <c r="D32" s="33" t="n"/>
-      <c r="E32" s="34" t="n"/>
+      <c r="D32" s="30" t="n"/>
+      <c r="E32" s="31" t="n"/>
     </row>
     <row r="33" ht="20.5" customHeight="1">
-      <c r="B33" s="27" t="inlineStr">
+      <c r="B33" s="24" t="inlineStr">
         <is>
           <t>Identificación</t>
         </is>
       </c>
-      <c r="C33" s="28" t="inlineStr">
+      <c r="C33" s="25" t="inlineStr">
         <is>
           <t>Tapa de granito con la información del difunto</t>
         </is>
       </c>
-      <c r="D33" s="29" t="n"/>
-      <c r="E33" s="30" t="n"/>
+      <c r="D33" s="26" t="n"/>
+      <c r="E33" s="27" t="n"/>
     </row>
     <row r="34" ht="20.5" customHeight="1">
-      <c r="B34" s="31" t="inlineStr">
+      <c r="B34" s="28" t="inlineStr">
         <is>
           <t>Paisajismo</t>
         </is>
       </c>
-      <c r="C34" s="32" t="inlineStr">
+      <c r="C34" s="29" t="inlineStr">
         <is>
           <t>Plantas de sombra de diferentes alturas y texturas</t>
         </is>
       </c>
-      <c r="D34" s="33" t="n"/>
-      <c r="E34" s="34" t="n"/>
+      <c r="D34" s="30" t="n"/>
+      <c r="E34" s="31" t="n"/>
     </row>
     <row r="35" ht="20.5" customHeight="1">
-      <c r="B35" s="27" t="inlineStr">
+      <c r="B35" s="24" t="inlineStr">
         <is>
           <t>Acceso</t>
         </is>
       </c>
-      <c r="C35" s="28" t="inlineStr">
+      <c r="C35" s="25" t="inlineStr">
         <is>
           <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
         </is>
       </c>
-      <c r="D35" s="29" t="n"/>
-      <c r="E35" s="30" t="n"/>
+      <c r="D35" s="26" t="n"/>
+      <c r="E35" s="27" t="n"/>
     </row>
     <row r="36" ht="20.5" customHeight="1">
-      <c r="B36" s="31" t="inlineStr">
+      <c r="B36" s="28" t="inlineStr">
         <is>
           <t>Mantenimiento</t>
         </is>
       </c>
-      <c r="C36" s="32" t="inlineStr">
+      <c r="C36" s="29" t="inlineStr">
         <is>
           <t>US$ 15 anual</t>
         </is>
       </c>
-      <c r="D36" s="33" t="n"/>
-      <c r="E36" s="34" t="n"/>
+      <c r="D36" s="30" t="n"/>
+      <c r="E36" s="31" t="n"/>
     </row>
     <row r="37" ht="64" customHeight="1">
-      <c r="B37" s="27" t="inlineStr">
+      <c r="B37" s="24" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C37" s="28" t="inlineStr">
+      <c r="C37" s="25" t="inlineStr">
         <is>
           <t>• Inhumación de la urna en contenedor individual
 • Tapa de granito con los datos del difunto
@@ -1589,248 +1528,244 @@
 • Espacio de contemplación con banco</t>
         </is>
       </c>
-      <c r="D37" s="29" t="n"/>
-      <c r="E37" s="30" t="n"/>
+      <c r="D37" s="26" t="n"/>
+      <c r="E37" s="27" t="n"/>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="B38" s="24" t="inlineStr">
+      <c r="B38" s="21" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C38" s="25" t="n"/>
-      <c r="D38" s="25" t="n"/>
-      <c r="E38" s="26" t="n"/>
+      <c r="C38" s="22" t="n"/>
+      <c r="D38" s="22" t="n"/>
+      <c r="E38" s="23" t="n"/>
     </row>
     <row r="39" ht="26.5" customHeight="1">
-      <c r="B39" s="27" t="inlineStr">
+      <c r="B39" s="24" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C39" s="35" t="inlineStr">
+      <c r="C39" s="32" t="inlineStr">
         <is>
           <t>US$ 600</t>
         </is>
       </c>
-      <c r="D39" s="29" t="n"/>
-      <c r="E39" s="30" t="n"/>
+      <c r="D39" s="26" t="n"/>
+      <c r="E39" s="27" t="n"/>
     </row>
     <row r="40" ht="20.5" customHeight="1">
-      <c r="B40" s="31" t="inlineStr">
+      <c r="B40" s="28" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C40" s="32" t="inlineStr">
+      <c r="C40" s="29" t="inlineStr">
         <is>
           <t>Por espacio individual · mantenimiento US$ 15/año</t>
         </is>
       </c>
-      <c r="D40" s="33" t="n"/>
-      <c r="E40" s="34" t="n"/>
+      <c r="D40" s="30" t="n"/>
+      <c r="E40" s="31" t="n"/>
     </row>
     <row r="41" ht="35" customHeight="1">
-      <c r="B41" s="27" t="inlineStr">
+      <c r="B41" s="24" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C41" s="28" t="inlineStr">
+      <c r="C41" s="25" t="inlineStr">
         <is>
           <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 15 anual.</t>
         </is>
       </c>
-      <c r="D41" s="29" t="n"/>
-      <c r="E41" s="30" t="n"/>
+      <c r="D41" s="26" t="n"/>
+      <c r="E41" s="27" t="n"/>
     </row>
     <row r="42" ht="20" customHeight="1">
-      <c r="B42" s="24" t="inlineStr">
+      <c r="B42" s="21" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C42" s="25" t="n"/>
-      <c r="D42" s="25" t="n"/>
-      <c r="E42" s="26" t="n"/>
+      <c r="C42" s="22" t="n"/>
+      <c r="D42" s="22" t="n"/>
+      <c r="E42" s="23" t="n"/>
     </row>
     <row r="43" ht="35" customHeight="1">
-      <c r="B43" s="36" t="inlineStr">
+      <c r="B43" s="33" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C43" s="37" t="inlineStr">
+      <c r="C43" s="34" t="inlineStr">
         <is>
           <t>Familias que desean un lugar permanente para visitar y rendir homenaje, con una inversión moderada.</t>
         </is>
       </c>
-      <c r="D43" s="38" t="n"/>
-      <c r="E43" s="39" t="n"/>
+      <c r="D43" s="35" t="n"/>
+      <c r="E43" s="36" t="n"/>
     </row>
     <row r="46" ht="30" customHeight="1">
-      <c r="B46" s="18" t="inlineStr">
+      <c r="B46" s="15" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · FAMILIAR</t>
         </is>
       </c>
-      <c r="C46" s="19" t="n"/>
-      <c r="D46" s="19" t="n"/>
-      <c r="E46" s="20" t="inlineStr">
-        <is>
-          <t>VG-CRE-03F</t>
-        </is>
-      </c>
+      <c r="C46" s="16" t="n"/>
+      <c r="D46" s="16" t="n"/>
+      <c r="E46" s="17" t="n"/>
     </row>
     <row r="47" ht="20" customHeight="1">
-      <c r="B47" s="21" t="inlineStr">
+      <c r="B47" s="18" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Jardín 1  ·  Destino final · Inhumación familiar</t>
         </is>
       </c>
-      <c r="C47" s="22" t="n"/>
-      <c r="D47" s="22" t="n"/>
-      <c r="E47" s="23" t="n"/>
+      <c r="C47" s="19" t="n"/>
+      <c r="D47" s="19" t="n"/>
+      <c r="E47" s="20" t="n"/>
     </row>
     <row r="48" ht="20" customHeight="1">
-      <c r="B48" s="24" t="inlineStr">
+      <c r="B48" s="21" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C48" s="25" t="n"/>
-      <c r="D48" s="25" t="n"/>
-      <c r="E48" s="26" t="n"/>
+      <c r="C48" s="22" t="n"/>
+      <c r="D48" s="22" t="n"/>
+      <c r="E48" s="23" t="n"/>
     </row>
     <row r="49" ht="35" customHeight="1">
-      <c r="B49" s="27" t="inlineStr">
+      <c r="B49" s="24" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C49" s="28" t="inlineStr">
+      <c r="C49" s="25" t="inlineStr">
         <is>
           <t>Parcela familiar en el Jardín 1 con cuatro contenedores agrupados, cada uno con tapa de granito grabada, sin plazo de permanencia.</t>
         </is>
       </c>
-      <c r="D49" s="29" t="n"/>
-      <c r="E49" s="30" t="n"/>
+      <c r="D49" s="26" t="n"/>
+      <c r="E49" s="27" t="n"/>
     </row>
     <row r="50" ht="20.5" customHeight="1">
-      <c r="B50" s="31" t="inlineStr">
+      <c r="B50" s="28" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C50" s="32" t="inlineStr">
+      <c r="C50" s="29" t="inlineStr">
         <is>
           <t>Hasta 4 espacios (familiar).</t>
         </is>
       </c>
-      <c r="D50" s="33" t="n"/>
-      <c r="E50" s="34" t="n"/>
+      <c r="D50" s="30" t="n"/>
+      <c r="E50" s="31" t="n"/>
     </row>
     <row r="51" ht="20" customHeight="1">
-      <c r="B51" s="24" t="inlineStr">
+      <c r="B51" s="21" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C51" s="25" t="n"/>
-      <c r="D51" s="25" t="n"/>
-      <c r="E51" s="26" t="n"/>
+      <c r="C51" s="22" t="n"/>
+      <c r="D51" s="22" t="n"/>
+      <c r="E51" s="23" t="n"/>
     </row>
     <row r="52" ht="20.5" customHeight="1">
-      <c r="B52" s="27" t="inlineStr">
+      <c r="B52" s="24" t="inlineStr">
         <is>
           <t>Ambiente</t>
         </is>
       </c>
-      <c r="C52" s="28" t="inlineStr">
+      <c r="C52" s="25" t="inlineStr">
         <is>
           <t>Jardín 1</t>
         </is>
       </c>
-      <c r="D52" s="29" t="n"/>
-      <c r="E52" s="30" t="n"/>
+      <c r="D52" s="26" t="n"/>
+      <c r="E52" s="27" t="n"/>
     </row>
     <row r="53" ht="20.5" customHeight="1">
-      <c r="B53" s="31" t="inlineStr">
+      <c r="B53" s="28" t="inlineStr">
         <is>
           <t>Capacidad</t>
         </is>
       </c>
-      <c r="C53" s="32" t="inlineStr">
+      <c r="C53" s="29" t="inlineStr">
         <is>
           <t>4 contenedores agrupados en losa</t>
         </is>
       </c>
-      <c r="D53" s="33" t="n"/>
-      <c r="E53" s="34" t="n"/>
+      <c r="D53" s="30" t="n"/>
+      <c r="E53" s="31" t="n"/>
     </row>
     <row r="54" ht="20.5" customHeight="1">
-      <c r="B54" s="27" t="inlineStr">
+      <c r="B54" s="24" t="inlineStr">
         <is>
           <t>Identificación</t>
         </is>
       </c>
-      <c r="C54" s="28" t="inlineStr">
+      <c r="C54" s="25" t="inlineStr">
         <is>
           <t>Tapa de granito por espacio, con la información del difunto</t>
         </is>
       </c>
-      <c r="D54" s="29" t="n"/>
-      <c r="E54" s="30" t="n"/>
+      <c r="D54" s="26" t="n"/>
+      <c r="E54" s="27" t="n"/>
     </row>
     <row r="55" ht="20.5" customHeight="1">
-      <c r="B55" s="31" t="inlineStr">
+      <c r="B55" s="28" t="inlineStr">
         <is>
           <t>Permanencia</t>
         </is>
       </c>
-      <c r="C55" s="32" t="inlineStr">
+      <c r="C55" s="29" t="inlineStr">
         <is>
           <t>Sin plazo</t>
         </is>
       </c>
-      <c r="D55" s="33" t="n"/>
-      <c r="E55" s="34" t="n"/>
+      <c r="D55" s="30" t="n"/>
+      <c r="E55" s="31" t="n"/>
     </row>
     <row r="56" ht="20.5" customHeight="1">
-      <c r="B56" s="27" t="inlineStr">
+      <c r="B56" s="24" t="inlineStr">
         <is>
           <t>Acceso</t>
         </is>
       </c>
-      <c r="C56" s="28" t="inlineStr">
+      <c r="C56" s="25" t="inlineStr">
         <is>
           <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
         </is>
       </c>
-      <c r="D56" s="29" t="n"/>
-      <c r="E56" s="30" t="n"/>
+      <c r="D56" s="26" t="n"/>
+      <c r="E56" s="27" t="n"/>
     </row>
     <row r="57" ht="20.5" customHeight="1">
-      <c r="B57" s="31" t="inlineStr">
+      <c r="B57" s="28" t="inlineStr">
         <is>
           <t>Mantenimiento</t>
         </is>
       </c>
-      <c r="C57" s="32" t="inlineStr">
+      <c r="C57" s="29" t="inlineStr">
         <is>
           <t>US$ 25 anual</t>
         </is>
       </c>
-      <c r="D57" s="33" t="n"/>
-      <c r="E57" s="34" t="n"/>
+      <c r="D57" s="30" t="n"/>
+      <c r="E57" s="31" t="n"/>
     </row>
     <row r="58" ht="64" customHeight="1">
-      <c r="B58" s="27" t="inlineStr">
+      <c r="B58" s="24" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C58" s="28" t="inlineStr">
+      <c r="C58" s="25" t="inlineStr">
         <is>
           <t>• Inhumación de hasta 4 urnas
 • Tapa de granito grabada para cada espacio
@@ -1838,276 +1773,272 @@
 • Lugar físico permanente de homenaje familiar, sin plazo</t>
         </is>
       </c>
-      <c r="D58" s="29" t="n"/>
-      <c r="E58" s="30" t="n"/>
+      <c r="D58" s="26" t="n"/>
+      <c r="E58" s="27" t="n"/>
     </row>
     <row r="59" ht="20" customHeight="1">
-      <c r="B59" s="24" t="inlineStr">
+      <c r="B59" s="21" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C59" s="25" t="n"/>
-      <c r="D59" s="25" t="n"/>
-      <c r="E59" s="26" t="n"/>
+      <c r="C59" s="22" t="n"/>
+      <c r="D59" s="22" t="n"/>
+      <c r="E59" s="23" t="n"/>
     </row>
     <row r="60" ht="26.5" customHeight="1">
-      <c r="B60" s="27" t="inlineStr">
+      <c r="B60" s="24" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C60" s="35" t="inlineStr">
+      <c r="C60" s="32" t="inlineStr">
         <is>
           <t>US$ 2.000</t>
         </is>
       </c>
-      <c r="D60" s="29" t="n"/>
-      <c r="E60" s="30" t="n"/>
+      <c r="D60" s="26" t="n"/>
+      <c r="E60" s="27" t="n"/>
     </row>
     <row r="61" ht="20.5" customHeight="1">
-      <c r="B61" s="31" t="inlineStr">
+      <c r="B61" s="28" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C61" s="32" t="inlineStr">
+      <c r="C61" s="29" t="inlineStr">
         <is>
           <t>Por parcela familiar · hasta 4 espacios · mantenimiento US$ 25/año</t>
         </is>
       </c>
-      <c r="D61" s="33" t="n"/>
-      <c r="E61" s="34" t="n"/>
+      <c r="D61" s="30" t="n"/>
+      <c r="E61" s="31" t="n"/>
     </row>
     <row r="62" ht="35" customHeight="1">
-      <c r="B62" s="27" t="inlineStr">
+      <c r="B62" s="24" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C62" s="28" t="inlineStr">
+      <c r="C62" s="25" t="inlineStr">
         <is>
           <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 25 anual.</t>
         </is>
       </c>
-      <c r="D62" s="29" t="n"/>
-      <c r="E62" s="30" t="n"/>
+      <c r="D62" s="26" t="n"/>
+      <c r="E62" s="27" t="n"/>
     </row>
     <row r="63" ht="20" customHeight="1">
-      <c r="B63" s="24" t="inlineStr">
+      <c r="B63" s="21" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C63" s="25" t="n"/>
-      <c r="D63" s="25" t="n"/>
-      <c r="E63" s="26" t="n"/>
+      <c r="C63" s="22" t="n"/>
+      <c r="D63" s="22" t="n"/>
+      <c r="E63" s="23" t="n"/>
     </row>
     <row r="64" ht="20.5" customHeight="1">
-      <c r="B64" s="36" t="inlineStr">
+      <c r="B64" s="33" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C64" s="37" t="inlineStr">
+      <c r="C64" s="34" t="inlineStr">
         <is>
           <t>Familias que buscan un espacio propio y permanente para varias generaciones.</t>
         </is>
       </c>
-      <c r="D64" s="38" t="n"/>
-      <c r="E64" s="39" t="n"/>
+      <c r="D64" s="35" t="n"/>
+      <c r="E64" s="36" t="n"/>
     </row>
     <row r="67" ht="30" customHeight="1">
-      <c r="B67" s="18" t="inlineStr">
+      <c r="B67" s="15" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · ECOLÓGICO</t>
         </is>
       </c>
-      <c r="C67" s="19" t="n"/>
-      <c r="D67" s="19" t="n"/>
-      <c r="E67" s="20" t="inlineStr">
-        <is>
-          <t>VG-CRE-03E</t>
-        </is>
-      </c>
+      <c r="C67" s="16" t="n"/>
+      <c r="D67" s="16" t="n"/>
+      <c r="E67" s="17" t="n"/>
     </row>
     <row r="68" ht="20" customHeight="1">
-      <c r="B68" s="21" t="inlineStr">
+      <c r="B68" s="18" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Jardín 2  ·  Destino final · Inhumación ecológica</t>
         </is>
       </c>
-      <c r="C68" s="22" t="n"/>
-      <c r="D68" s="22" t="n"/>
-      <c r="E68" s="23" t="n"/>
+      <c r="C68" s="19" t="n"/>
+      <c r="D68" s="19" t="n"/>
+      <c r="E68" s="20" t="n"/>
     </row>
     <row r="69" ht="20" customHeight="1">
-      <c r="B69" s="24" t="inlineStr">
+      <c r="B69" s="21" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C69" s="25" t="n"/>
-      <c r="D69" s="25" t="n"/>
-      <c r="E69" s="26" t="n"/>
+      <c r="C69" s="22" t="n"/>
+      <c r="D69" s="22" t="n"/>
+      <c r="E69" s="23" t="n"/>
     </row>
     <row r="70" ht="49.5" customHeight="1">
-      <c r="B70" s="27" t="inlineStr">
+      <c r="B70" s="24" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C70" s="28" t="inlineStr">
+      <c r="C70" s="25" t="inlineStr">
         <is>
           <t>La urna biodegradable se entierra directamente en el suelo, se cubre con tierra y se descompone integrándose a la naturaleza. Jardín con agua corriente y área de esparcimiento de cenizas.</t>
         </is>
       </c>
-      <c r="D70" s="29" t="n"/>
-      <c r="E70" s="30" t="n"/>
+      <c r="D70" s="26" t="n"/>
+      <c r="E70" s="27" t="n"/>
     </row>
     <row r="71" ht="20.5" customHeight="1">
-      <c r="B71" s="31" t="inlineStr">
+      <c r="B71" s="28" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C71" s="32" t="inlineStr">
+      <c r="C71" s="29" t="inlineStr">
         <is>
           <t>Individual (1 urna).</t>
         </is>
       </c>
-      <c r="D71" s="33" t="n"/>
-      <c r="E71" s="34" t="n"/>
+      <c r="D71" s="30" t="n"/>
+      <c r="E71" s="31" t="n"/>
     </row>
     <row r="72" ht="20" customHeight="1">
-      <c r="B72" s="24" t="inlineStr">
+      <c r="B72" s="21" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C72" s="25" t="n"/>
-      <c r="D72" s="25" t="n"/>
-      <c r="E72" s="26" t="n"/>
+      <c r="C72" s="22" t="n"/>
+      <c r="D72" s="22" t="n"/>
+      <c r="E72" s="23" t="n"/>
     </row>
     <row r="73" ht="20.5" customHeight="1">
-      <c r="B73" s="27" t="inlineStr">
+      <c r="B73" s="24" t="inlineStr">
         <is>
           <t>Ambientes</t>
         </is>
       </c>
-      <c r="C73" s="28" t="inlineStr">
+      <c r="C73" s="25" t="inlineStr">
         <is>
           <t>Jardín 2 · Ecológico o Bosque de las Orquídeas</t>
         </is>
       </c>
-      <c r="D73" s="29" t="n"/>
-      <c r="E73" s="30" t="n"/>
+      <c r="D73" s="26" t="n"/>
+      <c r="E73" s="27" t="n"/>
     </row>
     <row r="74" ht="20.5" customHeight="1">
-      <c r="B74" s="31" t="inlineStr">
+      <c r="B74" s="28" t="inlineStr">
         <is>
           <t>Espacio por urna</t>
         </is>
       </c>
-      <c r="C74" s="32" t="inlineStr">
+      <c r="C74" s="29" t="inlineStr">
         <is>
           <t>30 × 30 cm, 40 cm de profundidad</t>
         </is>
       </c>
-      <c r="D74" s="33" t="n"/>
-      <c r="E74" s="34" t="n"/>
+      <c r="D74" s="30" t="n"/>
+      <c r="E74" s="31" t="n"/>
     </row>
     <row r="75" ht="20.5" customHeight="1">
-      <c r="B75" s="27" t="inlineStr">
+      <c r="B75" s="24" t="inlineStr">
         <is>
           <t>Urna</t>
         </is>
       </c>
-      <c r="C75" s="28" t="inlineStr">
+      <c r="C75" s="25" t="inlineStr">
         <is>
           <t>Biodegradable; se integra al suelo</t>
         </is>
       </c>
-      <c r="D75" s="29" t="n"/>
-      <c r="E75" s="30" t="n"/>
+      <c r="D75" s="26" t="n"/>
+      <c r="E75" s="27" t="n"/>
     </row>
     <row r="76" ht="35" customHeight="1">
-      <c r="B76" s="31" t="inlineStr">
+      <c r="B76" s="28" t="inlineStr">
         <is>
           <t>Identificación (Jardín 2)</t>
         </is>
       </c>
-      <c r="C76" s="32" t="inlineStr">
+      <c r="C76" s="29" t="inlineStr">
         <is>
           <t>Placa de madera de 20 cm fijada a una varilla metálica, en posición vertical y sin contacto con el suelo</t>
         </is>
       </c>
-      <c r="D76" s="33" t="n"/>
-      <c r="E76" s="34" t="n"/>
+      <c r="D76" s="30" t="n"/>
+      <c r="E76" s="31" t="n"/>
     </row>
     <row r="77" ht="20.5" customHeight="1">
-      <c r="B77" s="27" t="inlineStr">
+      <c r="B77" s="24" t="inlineStr">
         <is>
           <t>Identificación (Bosque)</t>
         </is>
       </c>
-      <c r="C77" s="28" t="inlineStr">
+      <c r="C77" s="25" t="inlineStr">
         <is>
           <t>Placa de mármol de 20 × 15 cm</t>
         </is>
       </c>
-      <c r="D77" s="29" t="n"/>
-      <c r="E77" s="30" t="n"/>
+      <c r="D77" s="26" t="n"/>
+      <c r="E77" s="27" t="n"/>
     </row>
     <row r="78" ht="35" customHeight="1">
-      <c r="B78" s="31" t="inlineStr">
+      <c r="B78" s="28" t="inlineStr">
         <is>
           <t>Permanencia</t>
         </is>
       </c>
-      <c r="C78" s="32" t="inlineStr">
+      <c r="C78" s="29" t="inlineStr">
         <is>
           <t>3 años; luego el nombre pasa a una placa memorial en el monumento y el espacio se reutiliza</t>
         </is>
       </c>
-      <c r="D78" s="33" t="n"/>
-      <c r="E78" s="34" t="n"/>
+      <c r="D78" s="30" t="n"/>
+      <c r="E78" s="31" t="n"/>
     </row>
     <row r="79" ht="20.5" customHeight="1">
-      <c r="B79" s="27" t="inlineStr">
+      <c r="B79" s="24" t="inlineStr">
         <is>
           <t>Placa memorial</t>
         </is>
       </c>
-      <c r="C79" s="28" t="inlineStr">
+      <c r="C79" s="25" t="inlineStr">
         <is>
           <t>US$ 150</t>
         </is>
       </c>
-      <c r="D79" s="29" t="n"/>
-      <c r="E79" s="30" t="n"/>
+      <c r="D79" s="26" t="n"/>
+      <c r="E79" s="27" t="n"/>
     </row>
     <row r="80" ht="20.5" customHeight="1">
-      <c r="B80" s="31" t="inlineStr">
+      <c r="B80" s="28" t="inlineStr">
         <is>
           <t>Acceso</t>
         </is>
       </c>
-      <c r="C80" s="32" t="inlineStr">
+      <c r="C80" s="29" t="inlineStr">
         <is>
           <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
         </is>
       </c>
-      <c r="D80" s="33" t="n"/>
-      <c r="E80" s="34" t="n"/>
+      <c r="D80" s="30" t="n"/>
+      <c r="E80" s="31" t="n"/>
     </row>
     <row r="81" ht="78.5" customHeight="1">
-      <c r="B81" s="27" t="inlineStr">
+      <c r="B81" s="24" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C81" s="28" t="inlineStr">
+      <c r="C81" s="25" t="inlineStr">
         <is>
           <t>• Inhumación ecológica de la urna directamente en el suelo
 • Placa de identificación
@@ -2116,248 +2047,244 @@
 • Permanencia de 3 años; luego, placa memorial en el monumento</t>
         </is>
       </c>
-      <c r="D81" s="29" t="n"/>
-      <c r="E81" s="30" t="n"/>
+      <c r="D81" s="26" t="n"/>
+      <c r="E81" s="27" t="n"/>
     </row>
     <row r="82" ht="20" customHeight="1">
-      <c r="B82" s="24" t="inlineStr">
+      <c r="B82" s="21" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C82" s="25" t="n"/>
-      <c r="D82" s="25" t="n"/>
-      <c r="E82" s="26" t="n"/>
+      <c r="C82" s="22" t="n"/>
+      <c r="D82" s="22" t="n"/>
+      <c r="E82" s="23" t="n"/>
     </row>
     <row r="83" ht="26.5" customHeight="1">
-      <c r="B83" s="27" t="inlineStr">
+      <c r="B83" s="24" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C83" s="35" t="inlineStr">
+      <c r="C83" s="32" t="inlineStr">
         <is>
           <t>US$ 600</t>
         </is>
       </c>
-      <c r="D83" s="29" t="n"/>
-      <c r="E83" s="30" t="n"/>
+      <c r="D83" s="26" t="n"/>
+      <c r="E83" s="27" t="n"/>
     </row>
     <row r="84" ht="20.5" customHeight="1">
-      <c r="B84" s="31" t="inlineStr">
+      <c r="B84" s="28" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C84" s="32" t="inlineStr">
+      <c r="C84" s="29" t="inlineStr">
         <is>
           <t>Por espacio individual · placa memorial US$ 150</t>
         </is>
       </c>
-      <c r="D84" s="33" t="n"/>
-      <c r="E84" s="34" t="n"/>
+      <c r="D84" s="30" t="n"/>
+      <c r="E84" s="31" t="n"/>
     </row>
     <row r="85" ht="35" customHeight="1">
-      <c r="B85" s="27" t="inlineStr">
+      <c r="B85" s="24" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C85" s="28" t="inlineStr">
+      <c r="C85" s="25" t="inlineStr">
         <is>
           <t>Pago único o financiado según política comercial vigente. Placa memorial en el monumento al término del plazo: US$ 150.</t>
         </is>
       </c>
-      <c r="D85" s="29" t="n"/>
-      <c r="E85" s="30" t="n"/>
+      <c r="D85" s="26" t="n"/>
+      <c r="E85" s="27" t="n"/>
     </row>
     <row r="86" ht="20" customHeight="1">
-      <c r="B86" s="24" t="inlineStr">
+      <c r="B86" s="21" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C86" s="25" t="n"/>
-      <c r="D86" s="25" t="n"/>
-      <c r="E86" s="26" t="n"/>
+      <c r="C86" s="22" t="n"/>
+      <c r="D86" s="22" t="n"/>
+      <c r="E86" s="23" t="n"/>
     </row>
     <row r="87" ht="35" customHeight="1">
-      <c r="B87" s="36" t="inlineStr">
+      <c r="B87" s="33" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C87" s="37" t="inlineStr">
+      <c r="C87" s="34" t="inlineStr">
         <is>
           <t>Personas con conciencia ambiental que desean que sus cenizas vuelvan a la tierra, con un lugar identificado para visitar.</t>
         </is>
       </c>
-      <c r="D87" s="38" t="n"/>
-      <c r="E87" s="39" t="n"/>
+      <c r="D87" s="35" t="n"/>
+      <c r="E87" s="36" t="n"/>
     </row>
     <row r="90" ht="30" customHeight="1">
-      <c r="B90" s="18" t="inlineStr">
+      <c r="B90" s="15" t="inlineStr">
         <is>
           <t>JARDÍN DE MASCOTAS</t>
         </is>
       </c>
-      <c r="C90" s="19" t="n"/>
-      <c r="D90" s="19" t="n"/>
-      <c r="E90" s="20" t="inlineStr">
-        <is>
-          <t>VG-CRE-04</t>
-        </is>
-      </c>
+      <c r="C90" s="16" t="n"/>
+      <c r="D90" s="16" t="n"/>
+      <c r="E90" s="17" t="n"/>
     </row>
     <row r="91" ht="20" customHeight="1">
-      <c r="B91" s="21" t="inlineStr">
+      <c r="B91" s="18" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Mascotas  ·  Destino final · Inhumación ecológica</t>
         </is>
       </c>
-      <c r="C91" s="22" t="n"/>
-      <c r="D91" s="22" t="n"/>
-      <c r="E91" s="23" t="n"/>
+      <c r="C91" s="19" t="n"/>
+      <c r="D91" s="19" t="n"/>
+      <c r="E91" s="20" t="n"/>
     </row>
     <row r="92" ht="20" customHeight="1">
-      <c r="B92" s="24" t="inlineStr">
+      <c r="B92" s="21" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C92" s="25" t="n"/>
-      <c r="D92" s="25" t="n"/>
-      <c r="E92" s="26" t="n"/>
+      <c r="C92" s="22" t="n"/>
+      <c r="D92" s="22" t="n"/>
+      <c r="E92" s="23" t="n"/>
     </row>
     <row r="93" ht="35" customHeight="1">
-      <c r="B93" s="27" t="inlineStr">
+      <c r="B93" s="24" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C93" s="28" t="inlineStr">
+      <c r="C93" s="25" t="inlineStr">
         <is>
           <t>Jardín para inhumación ecológica de cenizas de mascotas: la urna biodegradable se entierra directamente en el suelo y se identifica con una placa de madera.</t>
         </is>
       </c>
-      <c r="D93" s="29" t="n"/>
-      <c r="E93" s="30" t="n"/>
+      <c r="D93" s="26" t="n"/>
+      <c r="E93" s="27" t="n"/>
     </row>
     <row r="94" ht="20.5" customHeight="1">
-      <c r="B94" s="31" t="inlineStr">
+      <c r="B94" s="28" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C94" s="32" t="inlineStr">
+      <c r="C94" s="29" t="inlineStr">
         <is>
           <t>Individual (una mascota por servicio).</t>
         </is>
       </c>
-      <c r="D94" s="33" t="n"/>
-      <c r="E94" s="34" t="n"/>
+      <c r="D94" s="30" t="n"/>
+      <c r="E94" s="31" t="n"/>
     </row>
     <row r="95" ht="20" customHeight="1">
-      <c r="B95" s="24" t="inlineStr">
+      <c r="B95" s="21" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C95" s="25" t="n"/>
-      <c r="D95" s="25" t="n"/>
-      <c r="E95" s="26" t="n"/>
+      <c r="C95" s="22" t="n"/>
+      <c r="D95" s="22" t="n"/>
+      <c r="E95" s="23" t="n"/>
     </row>
     <row r="96" ht="20.5" customHeight="1">
-      <c r="B96" s="27" t="inlineStr">
+      <c r="B96" s="24" t="inlineStr">
         <is>
           <t>Tipo de producto</t>
         </is>
       </c>
-      <c r="C96" s="28" t="inlineStr">
+      <c r="C96" s="25" t="inlineStr">
         <is>
           <t>Servicio de pago único</t>
         </is>
       </c>
-      <c r="D96" s="29" t="n"/>
-      <c r="E96" s="30" t="n"/>
+      <c r="D96" s="26" t="n"/>
+      <c r="E96" s="27" t="n"/>
     </row>
     <row r="97" ht="20.5" customHeight="1">
-      <c r="B97" s="31" t="inlineStr">
+      <c r="B97" s="28" t="inlineStr">
         <is>
           <t>Espacio por urna</t>
         </is>
       </c>
-      <c r="C97" s="32" t="inlineStr">
+      <c r="C97" s="29" t="inlineStr">
         <is>
           <t>15 × 20 cm o 15 × 30 cm, según el tamaño de la urna</t>
         </is>
       </c>
-      <c r="D97" s="33" t="n"/>
-      <c r="E97" s="34" t="n"/>
+      <c r="D97" s="30" t="n"/>
+      <c r="E97" s="31" t="n"/>
     </row>
     <row r="98" ht="20.5" customHeight="1">
-      <c r="B98" s="27" t="inlineStr">
+      <c r="B98" s="24" t="inlineStr">
         <is>
           <t>Urna</t>
         </is>
       </c>
-      <c r="C98" s="28" t="inlineStr">
+      <c r="C98" s="25" t="inlineStr">
         <is>
           <t>Biodegradable; se integra al suelo</t>
         </is>
       </c>
-      <c r="D98" s="29" t="n"/>
-      <c r="E98" s="30" t="n"/>
+      <c r="D98" s="26" t="n"/>
+      <c r="E98" s="27" t="n"/>
     </row>
     <row r="99" ht="20.5" customHeight="1">
-      <c r="B99" s="31" t="inlineStr">
+      <c r="B99" s="28" t="inlineStr">
         <is>
           <t>Identificación</t>
         </is>
       </c>
-      <c r="C99" s="32" t="inlineStr">
+      <c r="C99" s="29" t="inlineStr">
         <is>
           <t>Placa de madera de 20 cm</t>
         </is>
       </c>
-      <c r="D99" s="33" t="n"/>
-      <c r="E99" s="34" t="n"/>
+      <c r="D99" s="30" t="n"/>
+      <c r="E99" s="31" t="n"/>
     </row>
     <row r="100" ht="35" customHeight="1">
-      <c r="B100" s="27" t="inlineStr">
+      <c r="B100" s="24" t="inlineStr">
         <is>
           <t>Permanencia</t>
         </is>
       </c>
-      <c r="C100" s="28" t="inlineStr">
+      <c r="C100" s="25" t="inlineStr">
         <is>
           <t>3 años; luego el nombre pasa a una placa memorial en el monumento y el espacio se reutiliza</t>
         </is>
       </c>
-      <c r="D100" s="29" t="n"/>
-      <c r="E100" s="30" t="n"/>
+      <c r="D100" s="26" t="n"/>
+      <c r="E100" s="27" t="n"/>
     </row>
     <row r="101" ht="20.5" customHeight="1">
-      <c r="B101" s="31" t="inlineStr">
+      <c r="B101" s="28" t="inlineStr">
         <is>
           <t>Placa memorial</t>
         </is>
       </c>
-      <c r="C101" s="32" t="inlineStr">
+      <c r="C101" s="29" t="inlineStr">
         <is>
           <t>US$ 50</t>
         </is>
       </c>
-      <c r="D101" s="33" t="n"/>
-      <c r="E101" s="34" t="n"/>
+      <c r="D101" s="30" t="n"/>
+      <c r="E101" s="31" t="n"/>
     </row>
     <row r="102" ht="64" customHeight="1">
-      <c r="B102" s="27" t="inlineStr">
+      <c r="B102" s="24" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C102" s="28" t="inlineStr">
+      <c r="C102" s="25" t="inlineStr">
         <is>
           <t>• Inhumación ecológica de la urna en el jardín
 • Placa de madera de 20 cm para identificación
@@ -2365,299 +2292,295 @@
 • Cremación de la mascota (opción Jardín + Cremación)</t>
         </is>
       </c>
-      <c r="D102" s="29" t="n"/>
-      <c r="E102" s="30" t="n"/>
+      <c r="D102" s="26" t="n"/>
+      <c r="E102" s="27" t="n"/>
     </row>
     <row r="103" ht="20" customHeight="1">
-      <c r="B103" s="24" t="inlineStr">
+      <c r="B103" s="21" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C103" s="25" t="n"/>
-      <c r="D103" s="25" t="n"/>
-      <c r="E103" s="26" t="n"/>
+      <c r="C103" s="22" t="n"/>
+      <c r="D103" s="22" t="n"/>
+      <c r="E103" s="23" t="n"/>
     </row>
     <row r="104" ht="26.5" customHeight="1">
-      <c r="B104" s="27" t="inlineStr">
+      <c r="B104" s="24" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C104" s="35" t="inlineStr">
+      <c r="C104" s="32" t="inlineStr">
         <is>
           <t>US$ 350 / US$ 500</t>
         </is>
       </c>
-      <c r="D104" s="29" t="n"/>
-      <c r="E104" s="30" t="n"/>
+      <c r="D104" s="26" t="n"/>
+      <c r="E104" s="27" t="n"/>
     </row>
     <row r="105" ht="20.5" customHeight="1">
-      <c r="B105" s="31" t="inlineStr">
+      <c r="B105" s="28" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C105" s="32" t="inlineStr">
+      <c r="C105" s="29" t="inlineStr">
         <is>
           <t>US$ 350 solo jardín · US$ 500 jardín + cremación</t>
         </is>
       </c>
-      <c r="D105" s="33" t="n"/>
-      <c r="E105" s="34" t="n"/>
+      <c r="D105" s="30" t="n"/>
+      <c r="E105" s="31" t="n"/>
     </row>
     <row r="106" ht="35" customHeight="1">
-      <c r="B106" s="27" t="inlineStr">
+      <c r="B106" s="24" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C106" s="28" t="inlineStr">
+      <c r="C106" s="25" t="inlineStr">
         <is>
           <t>Pago único; puede contratarse como adicional al plan funerario. Placa memorial en el monumento al término del plazo: US$ 50.</t>
         </is>
       </c>
-      <c r="D106" s="29" t="n"/>
-      <c r="E106" s="30" t="n"/>
+      <c r="D106" s="26" t="n"/>
+      <c r="E106" s="27" t="n"/>
     </row>
     <row r="107" ht="20" customHeight="1">
-      <c r="B107" s="24" t="inlineStr">
+      <c r="B107" s="21" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C107" s="25" t="n"/>
-      <c r="D107" s="25" t="n"/>
-      <c r="E107" s="26" t="n"/>
+      <c r="C107" s="22" t="n"/>
+      <c r="D107" s="22" t="n"/>
+      <c r="E107" s="23" t="n"/>
     </row>
     <row r="108" ht="20.5" customHeight="1">
-      <c r="B108" s="36" t="inlineStr">
+      <c r="B108" s="33" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C108" s="37" t="inlineStr">
+      <c r="C108" s="34" t="inlineStr">
         <is>
           <t>Familias que consideran a su mascota parte del hogar y desean un cierre digno.</t>
         </is>
       </c>
-      <c r="D108" s="38" t="n"/>
-      <c r="E108" s="39" t="n"/>
+      <c r="D108" s="35" t="n"/>
+      <c r="E108" s="36" t="n"/>
     </row>
     <row r="111" ht="30" customHeight="1">
-      <c r="B111" s="18" t="inlineStr">
+      <c r="B111" s="15" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · CEREMONIAL</t>
         </is>
       </c>
-      <c r="C111" s="19" t="n"/>
-      <c r="D111" s="19" t="n"/>
-      <c r="E111" s="20" t="inlineStr">
-        <is>
-          <t>VG-CRE-03C</t>
-        </is>
-      </c>
+      <c r="C111" s="16" t="n"/>
+      <c r="D111" s="16" t="n"/>
+      <c r="E111" s="17" t="n"/>
     </row>
     <row r="112" ht="20" customHeight="1">
-      <c r="B112" s="21" t="inlineStr">
+      <c r="B112" s="18" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Jardín 3  ·  Destino final · Inhumación con ceremonia</t>
         </is>
       </c>
-      <c r="C112" s="22" t="n"/>
-      <c r="D112" s="22" t="n"/>
-      <c r="E112" s="23" t="n"/>
+      <c r="C112" s="19" t="n"/>
+      <c r="D112" s="19" t="n"/>
+      <c r="E112" s="20" t="n"/>
     </row>
     <row r="113" ht="24" customHeight="1">
-      <c r="B113" s="40" t="inlineStr">
+      <c r="B113" s="37" t="inlineStr">
         <is>
           <t>★  PRÓXIMO LANZAMIENTO · se lanzará en otro momento</t>
         </is>
       </c>
-      <c r="C113" s="41" t="n"/>
-      <c r="D113" s="41" t="n"/>
-      <c r="E113" s="42" t="n"/>
+      <c r="C113" s="38" t="n"/>
+      <c r="D113" s="38" t="n"/>
+      <c r="E113" s="39" t="n"/>
     </row>
     <row r="114" ht="20" customHeight="1">
-      <c r="B114" s="24" t="inlineStr">
+      <c r="B114" s="21" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C114" s="25" t="n"/>
-      <c r="D114" s="25" t="n"/>
-      <c r="E114" s="26" t="n"/>
+      <c r="C114" s="22" t="n"/>
+      <c r="D114" s="22" t="n"/>
+      <c r="E114" s="23" t="n"/>
     </row>
     <row r="115" ht="35" customHeight="1">
-      <c r="B115" s="27" t="inlineStr">
+      <c r="B115" s="24" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C115" s="28" t="inlineStr">
+      <c r="C115" s="25" t="inlineStr">
         <is>
           <t>Jardín para inhumación de urnas de cenizas con ceremonia de agua, con fuentes como elemento central del rito de despedida.</t>
         </is>
       </c>
-      <c r="D115" s="29" t="n"/>
-      <c r="E115" s="30" t="n"/>
+      <c r="D115" s="26" t="n"/>
+      <c r="E115" s="27" t="n"/>
     </row>
     <row r="116" ht="20.5" customHeight="1">
-      <c r="B116" s="31" t="inlineStr">
+      <c r="B116" s="28" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C116" s="32" t="inlineStr">
+      <c r="C116" s="29" t="inlineStr">
         <is>
           <t>A definir.</t>
         </is>
       </c>
-      <c r="D116" s="33" t="n"/>
-      <c r="E116" s="34" t="n"/>
+      <c r="D116" s="30" t="n"/>
+      <c r="E116" s="31" t="n"/>
     </row>
     <row r="117" ht="20" customHeight="1">
-      <c r="B117" s="24" t="inlineStr">
+      <c r="B117" s="21" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C117" s="25" t="n"/>
-      <c r="D117" s="25" t="n"/>
-      <c r="E117" s="26" t="n"/>
+      <c r="C117" s="22" t="n"/>
+      <c r="D117" s="22" t="n"/>
+      <c r="E117" s="23" t="n"/>
     </row>
     <row r="118" ht="20.5" customHeight="1">
-      <c r="B118" s="27" t="inlineStr">
+      <c r="B118" s="24" t="inlineStr">
         <is>
           <t>Ambiente</t>
         </is>
       </c>
-      <c r="C118" s="28" t="inlineStr">
+      <c r="C118" s="25" t="inlineStr">
         <is>
           <t>Jardín 3</t>
         </is>
       </c>
-      <c r="D118" s="29" t="n"/>
-      <c r="E118" s="30" t="n"/>
+      <c r="D118" s="26" t="n"/>
+      <c r="E118" s="27" t="n"/>
     </row>
     <row r="119" ht="20.5" customHeight="1">
-      <c r="B119" s="31" t="inlineStr">
+      <c r="B119" s="28" t="inlineStr">
         <is>
           <t>Elemento central</t>
         </is>
       </c>
-      <c r="C119" s="32" t="inlineStr">
+      <c r="C119" s="29" t="inlineStr">
         <is>
           <t>Fuente de agua para la ceremonia</t>
         </is>
       </c>
-      <c r="D119" s="33" t="n"/>
-      <c r="E119" s="34" t="n"/>
+      <c r="D119" s="30" t="n"/>
+      <c r="E119" s="31" t="n"/>
     </row>
     <row r="120" ht="20.5" customHeight="1">
-      <c r="B120" s="27" t="inlineStr">
+      <c r="B120" s="24" t="inlineStr">
         <is>
           <t>Entorno</t>
         </is>
       </c>
-      <c r="C120" s="28" t="inlineStr">
+      <c r="C120" s="25" t="inlineStr">
         <is>
           <t>Barrera visual que separa el jardín del crematorio</t>
         </is>
       </c>
-      <c r="D120" s="29" t="n"/>
-      <c r="E120" s="30" t="n"/>
+      <c r="D120" s="26" t="n"/>
+      <c r="E120" s="27" t="n"/>
     </row>
     <row r="121" ht="35" customHeight="1">
-      <c r="B121" s="31" t="inlineStr">
+      <c r="B121" s="28" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C121" s="32" t="inlineStr">
+      <c r="C121" s="29" t="inlineStr">
         <is>
           <t>• Inhumación de urnas de cenizas
 • Ceremonia con agua en fuente</t>
         </is>
       </c>
-      <c r="D121" s="33" t="n"/>
-      <c r="E121" s="34" t="n"/>
+      <c r="D121" s="30" t="n"/>
+      <c r="E121" s="31" t="n"/>
     </row>
     <row r="122" ht="20" customHeight="1">
-      <c r="B122" s="24" t="inlineStr">
+      <c r="B122" s="21" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C122" s="25" t="n"/>
-      <c r="D122" s="25" t="n"/>
-      <c r="E122" s="26" t="n"/>
+      <c r="C122" s="22" t="n"/>
+      <c r="D122" s="22" t="n"/>
+      <c r="E122" s="23" t="n"/>
     </row>
     <row r="123" ht="26.5" customHeight="1">
-      <c r="B123" s="27" t="inlineStr">
+      <c r="B123" s="24" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C123" s="35" t="inlineStr">
+      <c r="C123" s="32" t="inlineStr">
         <is>
           <t>A definir</t>
         </is>
       </c>
-      <c r="D123" s="29" t="n"/>
-      <c r="E123" s="30" t="n"/>
+      <c r="D123" s="26" t="n"/>
+      <c r="E123" s="27" t="n"/>
     </row>
     <row r="124" ht="20.5" customHeight="1">
-      <c r="B124" s="31" t="inlineStr">
+      <c r="B124" s="28" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C124" s="32" t="inlineStr">
+      <c r="C124" s="29" t="inlineStr">
         <is>
           <t>Producto en definición</t>
         </is>
       </c>
-      <c r="D124" s="33" t="n"/>
-      <c r="E124" s="34" t="n"/>
+      <c r="D124" s="30" t="n"/>
+      <c r="E124" s="31" t="n"/>
     </row>
     <row r="125" ht="20.5" customHeight="1">
-      <c r="B125" s="27" t="inlineStr">
+      <c r="B125" s="24" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C125" s="28" t="inlineStr">
+      <c r="C125" s="25" t="inlineStr">
         <is>
           <t>A definir.</t>
         </is>
       </c>
-      <c r="D125" s="29" t="n"/>
-      <c r="E125" s="30" t="n"/>
+      <c r="D125" s="26" t="n"/>
+      <c r="E125" s="27" t="n"/>
     </row>
     <row r="126" ht="20" customHeight="1">
-      <c r="B126" s="24" t="inlineStr">
+      <c r="B126" s="21" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C126" s="25" t="n"/>
-      <c r="D126" s="25" t="n"/>
-      <c r="E126" s="26" t="n"/>
+      <c r="C126" s="22" t="n"/>
+      <c r="D126" s="22" t="n"/>
+      <c r="E126" s="23" t="n"/>
     </row>
     <row r="127" ht="35" customHeight="1">
-      <c r="B127" s="36" t="inlineStr">
+      <c r="B127" s="33" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C127" s="37" t="inlineStr">
+      <c r="C127" s="34" t="inlineStr">
         <is>
           <t>Familias que valoran un rito de despedida simbólico y un entorno contemplativo.</t>
         </is>
       </c>
-      <c r="D127" s="38" t="n"/>
-      <c r="E127" s="39" t="n"/>
+      <c r="D127" s="35" t="n"/>
+      <c r="E127" s="36" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="116">
@@ -2673,11 +2596,10 @@
     <mergeCell ref="B47:E47"/>
     <mergeCell ref="C7:E7"/>
     <mergeCell ref="C57:E57"/>
-    <mergeCell ref="B4:D4"/>
     <mergeCell ref="B21:E21"/>
+    <mergeCell ref="B86:E86"/>
     <mergeCell ref="C18:E18"/>
     <mergeCell ref="C49:E49"/>
-    <mergeCell ref="B86:E86"/>
     <mergeCell ref="C101:E101"/>
     <mergeCell ref="C77:E77"/>
     <mergeCell ref="C34:E34"/>
@@ -2688,7 +2610,6 @@
     <mergeCell ref="B112:E112"/>
     <mergeCell ref="C20:E20"/>
     <mergeCell ref="C85:E85"/>
-    <mergeCell ref="B111:D111"/>
     <mergeCell ref="C99:E99"/>
     <mergeCell ref="C94:E94"/>
     <mergeCell ref="C118:E118"/>
@@ -2706,6 +2627,8 @@
     <mergeCell ref="C39:E39"/>
     <mergeCell ref="B16:E16"/>
     <mergeCell ref="C70:E70"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B90:E90"/>
     <mergeCell ref="C106:E106"/>
     <mergeCell ref="C32:E32"/>
     <mergeCell ref="C81:E81"/>
@@ -2715,10 +2638,10 @@
     <mergeCell ref="C87:E87"/>
     <mergeCell ref="B117:E117"/>
     <mergeCell ref="C15:E15"/>
+    <mergeCell ref="B67:E67"/>
     <mergeCell ref="C33:E33"/>
     <mergeCell ref="C104:E104"/>
     <mergeCell ref="C116:E116"/>
-    <mergeCell ref="B46:D46"/>
     <mergeCell ref="C79:E79"/>
     <mergeCell ref="C73:E73"/>
     <mergeCell ref="B103:E103"/>
@@ -2739,7 +2662,6 @@
     <mergeCell ref="C96:E96"/>
     <mergeCell ref="C78:E78"/>
     <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B25:D25"/>
     <mergeCell ref="B42:E42"/>
     <mergeCell ref="B107:E107"/>
     <mergeCell ref="C62:E62"/>
@@ -2749,7 +2671,6 @@
     <mergeCell ref="C54:E54"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="C41:E41"/>
-    <mergeCell ref="B67:D67"/>
     <mergeCell ref="C93:E93"/>
     <mergeCell ref="C124:E124"/>
     <mergeCell ref="B92:E92"/>
@@ -2759,20 +2680,22 @@
     <mergeCell ref="C105:E105"/>
     <mergeCell ref="C43:E43"/>
     <mergeCell ref="C76:E76"/>
+    <mergeCell ref="B4:E4"/>
     <mergeCell ref="C120:E120"/>
     <mergeCell ref="B126:E126"/>
     <mergeCell ref="C119:E119"/>
     <mergeCell ref="C8:E8"/>
     <mergeCell ref="C17:E17"/>
     <mergeCell ref="B59:E59"/>
+    <mergeCell ref="B46:E46"/>
     <mergeCell ref="C19:E19"/>
     <mergeCell ref="C53:E53"/>
     <mergeCell ref="C102:E102"/>
     <mergeCell ref="B48:E48"/>
+    <mergeCell ref="B111:E111"/>
     <mergeCell ref="C83:E83"/>
     <mergeCell ref="C108:E108"/>
     <mergeCell ref="C58:E58"/>
-    <mergeCell ref="B90:D90"/>
     <mergeCell ref="B82:E82"/>
     <mergeCell ref="C97:E97"/>
     <mergeCell ref="C29:E29"/>

</xml_diff>

<commit_message>
Agrega aba interna de comisiones (propuesta pendiente de validación)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111i7vn9WWo4QxCQbucWbrF
</commit_message>
<xml_diff>
--- a/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
+++ b/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Tabla Gral. - Visión Comercial" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Ficha Técnica Consolidada" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Comisiones - uso interno" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tabla Gral. - Visión Comercial'!$A$4:$H$10</definedName>
@@ -21,7 +22,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="&quot;US$&quot; #,##0.00"/>
+  </numFmts>
   <fonts count="13">
     <font>
       <name val="Calibri"/>
@@ -270,7 +273,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -361,6 +364,36 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2711,4 +2744,388 @@
     <brk id="109" min="0" max="16383" man="1"/>
   </rowBreaks>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="000F2537"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>LA AUXILIADORA · VANGRUPO  |  POLÍTICA DE COMISIONES — USO INTERNO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="40" t="inlineStr">
+        <is>
+          <t>PROPUESTA · pendiente de validación con el Gerente Comercial</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="41" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="B4" s="41" t="inlineStr">
+        <is>
+          <t>Precio (c/ IVA)</t>
+        </is>
+      </c>
+      <c r="C4" s="41" t="inlineStr">
+        <is>
+          <t>Precio sin IVA</t>
+        </is>
+      </c>
+      <c r="D4" s="41" t="inlineStr">
+        <is>
+          <t>% Comisión</t>
+        </is>
+      </c>
+      <c r="E4" s="41" t="inlineStr">
+        <is>
+          <t>Comisión por venta (sin IVA)</t>
+        </is>
+      </c>
+      <c r="F4" s="41" t="inlineStr">
+        <is>
+          <t>Momento de pago</t>
+        </is>
+      </c>
+      <c r="G4" s="41" t="inlineStr">
+        <is>
+          <t>Estorno</t>
+        </is>
+      </c>
+      <c r="H4" s="41" t="inlineStr">
+        <is>
+          <t>Observaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Solución Modular de Cremación</t>
+        </is>
+      </c>
+      <c r="B5" s="42" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C5" s="42">
+        <f>B5/1.13</f>
+        <v/>
+      </c>
+      <c r="D5" s="43" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E5" s="44">
+        <f>C5*D5</f>
+        <v/>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Pago único cuando el cliente paga la 3ª cuota</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Si el cliente cancela antes de la 12ª cuota</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Alternativa: comisión = 10 primeras cuotas del cliente (≈ US$ 83), pagadas mes a mes, sin estorno.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Jardín de Cenizas · Individual</t>
+        </is>
+      </c>
+      <c r="B6" s="45" t="n">
+        <v>600</v>
+      </c>
+      <c r="C6" s="45">
+        <f>B6/1.13</f>
+        <v/>
+      </c>
+      <c r="D6" s="46" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E6" s="47">
+        <f>C6*D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Contado: mes siguiente al pago. Financiado: proporcional a lo cobrado</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>Cancelación en los primeros 90 días</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>Acelerador de campaña opcional: +2 pp hasta 30/11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="44" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Jardín de Cenizas · Familiar</t>
+        </is>
+      </c>
+      <c r="B7" s="42" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C7" s="42">
+        <f>B7/1.13</f>
+        <v/>
+      </c>
+      <c r="D7" s="43" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E7" s="44">
+        <f>C7*D7</f>
+        <v/>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Contado: mes siguiente al pago. Financiado: proporcional a lo cobrado</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Cancelación en los primeros 90 días</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Margen ajustada (≈ 26%): revisar precio o costo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="44" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Jardín de Cenizas · Ecológico</t>
+        </is>
+      </c>
+      <c r="B8" s="45" t="n">
+        <v>600</v>
+      </c>
+      <c r="C8" s="45">
+        <f>B8/1.13</f>
+        <v/>
+      </c>
+      <c r="D8" s="46" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E8" s="47">
+        <f>C8*D8</f>
+        <v/>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Contado: mes siguiente al pago. Financiado: proporcional a lo cobrado</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>Cancelación en los primeros 90 días</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>Acelerador de campaña opcional: +2 pp hasta 30/11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="44" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Jardín de Mascotas · solo jardín</t>
+        </is>
+      </c>
+      <c r="B9" s="42" t="n">
+        <v>350</v>
+      </c>
+      <c r="C9" s="42">
+        <f>B9/1.13</f>
+        <v/>
+      </c>
+      <c r="D9" s="43" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E9" s="44">
+        <f>C9*D9</f>
+        <v/>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Mes siguiente al pago (pago único)</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Cancelación en los primeros 90 días</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Margen ajustada (≈ 20%): revisar precio o costo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="44" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Jardín de Mascotas · jardín + cremación</t>
+        </is>
+      </c>
+      <c r="B10" s="45" t="n">
+        <v>500</v>
+      </c>
+      <c r="C10" s="45">
+        <f>B10/1.13</f>
+        <v/>
+      </c>
+      <c r="D10" s="46" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E10" s="47">
+        <f>C10*D10</f>
+        <v/>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Mes siguiente al pago (pago único)</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Cancelación en los primeros 90 días</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>Margen ajustada (≈ 26%): revisar precio o costo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="44" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Jardín de Cenizas · Ceremonial</t>
+        </is>
+      </c>
+      <c r="B11" s="42" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="C11" s="42" t="inlineStr"/>
+      <c r="D11" s="43" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="E11" s="44" t="inlineStr"/>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Próximo lanzamiento; precio a definir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="48" t="inlineStr">
+        <is>
+          <t>REGLAS GENERALES</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="49" t="inlineStr">
+        <is>
+          <t>1. Base de cálculo: valor efectivamente cobrado al cliente, sin IVA (13%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="49" t="inlineStr">
+        <is>
+          <t>2. No generan comisión: cuotas de mantenimiento anual (US$ 15 / US$ 25) ni placas memoriales (US$ 150 / US$ 50).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="49" t="inlineStr">
+        <is>
+          <t>3. Bono de venta combinada: US$ 15 al vender la Solución Modular junto con cualquier jardín.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="49" t="inlineStr">
+        <is>
+          <t>4. Acelerador de campaña Día de los Muertos (opcional): +2 pp en Individual y Ecológico para ventas cerradas hasta el 30/11/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="49" t="inlineStr">
+        <is>
+          <t>5. Estorno: la comisión se descuenta de los pagos siguientes al vendedor.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A17:H17"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fórmula de precio sin IVA independiente de la configuración regional
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111i7vn9WWo4QxCQbucWbrF
</commit_message>
<xml_diff>
--- a/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
+++ b/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
@@ -2832,7 +2832,7 @@
         <v>1000</v>
       </c>
       <c r="C5" s="42">
-        <f>B5/1.13</f>
+        <f>B5*100/113</f>
         <v/>
       </c>
       <c r="D5" s="43" t="n">
@@ -2868,7 +2868,7 @@
         <v>600</v>
       </c>
       <c r="C6" s="45">
-        <f>B6/1.13</f>
+        <f>B6*100/113</f>
         <v/>
       </c>
       <c r="D6" s="46" t="n">
@@ -2904,7 +2904,7 @@
         <v>2000</v>
       </c>
       <c r="C7" s="42">
-        <f>B7/1.13</f>
+        <f>B7*100/113</f>
         <v/>
       </c>
       <c r="D7" s="43" t="n">
@@ -2940,7 +2940,7 @@
         <v>600</v>
       </c>
       <c r="C8" s="45">
-        <f>B8/1.13</f>
+        <f>B8*100/113</f>
         <v/>
       </c>
       <c r="D8" s="46" t="n">
@@ -2976,7 +2976,7 @@
         <v>350</v>
       </c>
       <c r="C9" s="42">
-        <f>B9/1.13</f>
+        <f>B9*100/113</f>
         <v/>
       </c>
       <c r="D9" s="43" t="n">
@@ -3012,7 +3012,7 @@
         <v>500</v>
       </c>
       <c r="C10" s="45">
-        <f>B10/1.13</f>
+        <f>B10*100/113</f>
         <v/>
       </c>
       <c r="D10" s="46" t="n">

</xml_diff>

<commit_message>
Precios Ecológico US$ 750 y Mascotas US$ 400/550 con placa; comisión única de 8%
Ficha técnica, comisiones y playbook alineados con la planilla Google.
Agrega el generador PPTX del playbook (versión Canva) y los entregables
DOCX y PPTX.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111i7vn9WWo4QxCQbucWbrF
</commit_message>
<xml_diff>
--- a/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
+++ b/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Tabla Gral. - Visión Comercial" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Ficha Técnica Consolidada" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Comisiones - uso interno" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabla Gral. - Visión Comercial" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ficha Técnica Consolidada" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comisiones - uso interno" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tabla Gral. - Visión Comercial'!$A$4:$H$10</definedName>
@@ -829,7 +829,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="93" customHeight="1">
+    <row r="5" ht="107.5" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Solución Modular de Cremación</t>
@@ -855,7 +855,7 @@
           <t>• Proceso completo de cremación individual
 • Urna cineraria de línea modular
 • Trámites legales básicos
-• Alquiler temporal de columbario por 1 año
+• Alquiler temporal de columbario por 1 año en nivel 1 HDLM
 • Integración al plan funerario base (actual o nuevo)</t>
         </is>
       </c>
@@ -872,7 +872,8 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Hasta 120 cuotas mensuales (aprox. US$ 8,50/mes).</t>
+          <t>Hasta 120 cuotas mensuales (aprox. US$ 8,50/mes).
+Debe estar pagado en su totalidad para el uso de la cremación y el columbario</t>
         </is>
       </c>
     </row>
@@ -995,7 +996,7 @@
 • Placa de identificación
 • Ubicación en el Jardín 2 o en el Bosque de las Orquídeas
 • Entorno natural con agua corriente
-• Permanencia de 3 años; luego, placa memorial en el monumento</t>
+• Permanencia de 3 años; luego, placa memorial en el monumento (incluida)</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -1005,17 +1006,17 @@
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>US$ 600
-(Por espacio individual · placa memorial US$ 150)</t>
+          <t>US$ 750
+(Por espacio individual · placa memorial incluida)</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>Pago único o financiado según política comercial vigente. Placa memorial en el monumento al término del plazo: US$ 150.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="93" customHeight="1">
+          <t>Pago único o financiado según política comercial vigente. Incluye la placa memorial en el monumento al término del plazo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="78.5" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Jardín de Mascotas</t>
@@ -1040,8 +1041,8 @@
         <is>
           <t>• Inhumación ecológica de la urna en el jardín
 • Placa de madera de 20 cm para identificación
-• Permanencia de 3 años; luego, placa memorial en el monumento
-• Cremación de la mascota (opción Jardín + Cremación)</t>
+• Permanencia de 3 años
+• Placa memorial en el monumento al término del plazo (opción US$ 550)</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -1051,13 +1052,13 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>US$ 350 / US$ 500
-(US$ 350 solo jardín · US$ 500 jardín + cremación)</t>
+          <t>US$ 400 / US$ 550
+(US$ 400 solo espacio · US$ 550 con placa memorial)</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Pago único; puede contratarse como adicional al plan funerario. Placa memorial en el monumento al término del plazo: US$ 50.</t>
+          <t>Pago único; puede contratarse como adicional al plan funerario. La opción de US$ 550 incluye la placa memorial en el monumento al término del plazo.</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1282,7 @@
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
-          <t>Alquiler temporal · 12 meses incluido</t>
+          <t>Alquiler temporal · 12 meses incluido (Hogar de Las Memorias)</t>
         </is>
       </c>
       <c r="D14" s="26" t="n"/>
@@ -1298,7 +1299,7 @@
           <t>• Proceso completo de cremación individual
 • Urna cineraria de línea modular
 • Trámites legales básicos
-• Alquiler temporal de columbario por 1 año
+• Alquiler temporal de columbario por 1 año en nivel 1 HDLM
 • Integración al plan funerario base (actual o nuevo)</t>
         </is>
       </c>
@@ -1343,7 +1344,7 @@
       <c r="D18" s="30" t="n"/>
       <c r="E18" s="31" t="n"/>
     </row>
-    <row r="19" ht="20.5" customHeight="1">
+    <row r="19" ht="35" customHeight="1">
       <c r="B19" s="24" t="inlineStr">
         <is>
           <t>Condiciones</t>
@@ -1351,7 +1352,8 @@
       </c>
       <c r="C19" s="25" t="inlineStr">
         <is>
-          <t>Hasta 120 cuotas mensuales (aprox. US$ 8,50/mes).</t>
+          <t>Hasta 120 cuotas mensuales (aprox. US$ 8,50/mes).
+Debe estar pagado en su totalidad para el uso de la cremación y el columbario</t>
         </is>
       </c>
       <c r="D19" s="26" t="n"/>
@@ -2045,7 +2047,7 @@
       </c>
       <c r="C79" s="25" t="inlineStr">
         <is>
-          <t>US$ 150</t>
+          <t>Incluida en el precio</t>
         </is>
       </c>
       <c r="D79" s="26" t="n"/>
@@ -2077,7 +2079,7 @@
 • Placa de identificación
 • Ubicación en el Jardín 2 o en el Bosque de las Orquídeas
 • Entorno natural con agua corriente
-• Permanencia de 3 años; luego, placa memorial en el monumento</t>
+• Permanencia de 3 años; luego, placa memorial en el monumento (incluida)</t>
         </is>
       </c>
       <c r="D81" s="26" t="n"/>
@@ -2101,7 +2103,7 @@
       </c>
       <c r="C83" s="32" t="inlineStr">
         <is>
-          <t>US$ 600</t>
+          <t>US$ 750</t>
         </is>
       </c>
       <c r="D83" s="26" t="n"/>
@@ -2115,7 +2117,7 @@
       </c>
       <c r="C84" s="29" t="inlineStr">
         <is>
-          <t>Por espacio individual · placa memorial US$ 150</t>
+          <t>Por espacio individual · placa memorial incluida</t>
         </is>
       </c>
       <c r="D84" s="30" t="n"/>
@@ -2129,7 +2131,7 @@
       </c>
       <c r="C85" s="25" t="inlineStr">
         <is>
-          <t>Pago único o financiado según política comercial vigente. Placa memorial en el monumento al término del plazo: US$ 150.</t>
+          <t>Pago único o financiado según política comercial vigente. Incluye la placa memorial en el monumento al término del plazo.</t>
         </is>
       </c>
       <c r="D85" s="26" t="n"/>
@@ -2283,7 +2285,7 @@
       <c r="D99" s="30" t="n"/>
       <c r="E99" s="31" t="n"/>
     </row>
-    <row r="100" ht="35" customHeight="1">
+    <row r="100" ht="20.5" customHeight="1">
       <c r="B100" s="24" t="inlineStr">
         <is>
           <t>Permanencia</t>
@@ -2291,7 +2293,7 @@
       </c>
       <c r="C100" s="25" t="inlineStr">
         <is>
-          <t>3 años; luego el nombre pasa a una placa memorial en el monumento y el espacio se reutiliza</t>
+          <t>3 años; luego el espacio se reutiliza</t>
         </is>
       </c>
       <c r="D100" s="26" t="n"/>
@@ -2305,7 +2307,7 @@
       </c>
       <c r="C101" s="29" t="inlineStr">
         <is>
-          <t>US$ 50</t>
+          <t>En el monumento al término del plazo; incluida en la opción de US$ 550</t>
         </is>
       </c>
       <c r="D101" s="30" t="n"/>
@@ -2321,8 +2323,8 @@
         <is>
           <t>• Inhumación ecológica de la urna en el jardín
 • Placa de madera de 20 cm para identificación
-• Permanencia de 3 años; luego, placa memorial en el monumento
-• Cremación de la mascota (opción Jardín + Cremación)</t>
+• Permanencia de 3 años
+• Placa memorial en el monumento al término del plazo (opción US$ 550)</t>
         </is>
       </c>
       <c r="D102" s="26" t="n"/>
@@ -2346,7 +2348,7 @@
       </c>
       <c r="C104" s="32" t="inlineStr">
         <is>
-          <t>US$ 350 / US$ 500</t>
+          <t>US$ 400 / US$ 550</t>
         </is>
       </c>
       <c r="D104" s="26" t="n"/>
@@ -2360,7 +2362,7 @@
       </c>
       <c r="C105" s="29" t="inlineStr">
         <is>
-          <t>US$ 350 solo jardín · US$ 500 jardín + cremación</t>
+          <t>US$ 400 solo espacio · US$ 550 con placa memorial</t>
         </is>
       </c>
       <c r="D105" s="30" t="n"/>
@@ -2374,7 +2376,7 @@
       </c>
       <c r="C106" s="25" t="inlineStr">
         <is>
-          <t>Pago único; puede contratarse como adicional al plan funerario. Placa memorial en el monumento al término del plazo: US$ 50.</t>
+          <t>Pago único; puede contratarse como adicional al plan funerario. La opción de US$ 550 incluye la placa memorial en el monumento al término del plazo.</t>
         </is>
       </c>
       <c r="D106" s="26" t="n"/>
@@ -2836,7 +2838,7 @@
         <v/>
       </c>
       <c r="D5" s="43" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="E5" s="44">
         <f>C5*D5</f>
@@ -2872,7 +2874,7 @@
         <v/>
       </c>
       <c r="D6" s="46" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="E6" s="47">
         <f>C6*D6</f>
@@ -2888,11 +2890,7 @@
           <t>Cancelación en los primeros 90 días</t>
         </is>
       </c>
-      <c r="H6" s="8" t="inlineStr">
-        <is>
-          <t>Acelerador de campaña opcional: +2 pp hasta 30/11.</t>
-        </is>
-      </c>
+      <c r="H6" s="8" t="inlineStr"/>
     </row>
     <row r="7" ht="44" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -2924,11 +2922,7 @@
           <t>Cancelación en los primeros 90 días</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>Margen ajustada (≈ 26%): revisar precio o costo.</t>
-        </is>
-      </c>
+      <c r="H7" s="5" t="inlineStr"/>
     </row>
     <row r="8" ht="44" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
@@ -2937,14 +2931,14 @@
         </is>
       </c>
       <c r="B8" s="45" t="n">
-        <v>600</v>
+        <v>750</v>
       </c>
       <c r="C8" s="45">
         <f>B8*100/113</f>
         <v/>
       </c>
       <c r="D8" s="46" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="E8" s="47">
         <f>C8*D8</f>
@@ -2960,20 +2954,16 @@
           <t>Cancelación en los primeros 90 días</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr">
-        <is>
-          <t>Acelerador de campaña opcional: +2 pp hasta 30/11.</t>
-        </is>
-      </c>
+      <c r="H8" s="8" t="inlineStr"/>
     </row>
     <row r="9" ht="44" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Jardín de Mascotas · solo jardín</t>
+          <t>Jardín de Mascotas · solo espacio</t>
         </is>
       </c>
       <c r="B9" s="42" t="n">
-        <v>350</v>
+        <v>400</v>
       </c>
       <c r="C9" s="42">
         <f>B9*100/113</f>
@@ -2996,20 +2986,16 @@
           <t>Cancelación en los primeros 90 días</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>Margen ajustada (≈ 20%): revisar precio o costo.</t>
-        </is>
-      </c>
+      <c r="H9" s="5" t="inlineStr"/>
     </row>
     <row r="10" ht="44" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Jardín de Mascotas · jardín + cremación</t>
+          <t>Jardín de Mascotas · con placa memorial</t>
         </is>
       </c>
       <c r="B10" s="45" t="n">
-        <v>500</v>
+        <v>550</v>
       </c>
       <c r="C10" s="45">
         <f>B10*100/113</f>
@@ -3032,11 +3018,7 @@
           <t>Cancelación en los primeros 90 días</t>
         </is>
       </c>
-      <c r="H10" s="8" t="inlineStr">
-        <is>
-          <t>Margen ajustada (≈ 26%): revisar precio o costo.</t>
-        </is>
-      </c>
+      <c r="H10" s="8" t="inlineStr"/>
     </row>
     <row r="11" ht="44" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -3089,7 +3071,7 @@
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="49" t="inlineStr">
         <is>
-          <t>2. No generan comisión: cuotas de mantenimiento anual (US$ 15 / US$ 25) ni placas memoriales (US$ 150 / US$ 50).</t>
+          <t>2. No generan comisión: cuotas de mantenimiento anual (US$ 15 / US$ 25).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ficha técnica: precio de lanzamiento -20%, permanencia de 30 años renovable y mantenimiento Familiar US$ 24
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111i7vn9WWo4QxCQbucWbrF
</commit_message>
<xml_diff>
--- a/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
+++ b/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
@@ -12,9 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comisiones - uso interno" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tabla Gral. - Visión Comercial'!$A$4:$H$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tabla Gral. - Visión Comercial'!$A$4:$I$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Tabla Gral. - Visión Comercial'!$4:$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Ficha Técnica Consolidada'!$A$1:$F$128</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Ficha Técnica Consolidada'!$A$1:$F$135</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -273,7 +273,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -349,6 +349,9 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -760,7 +763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -770,7 +773,8 @@
     <col width="46" customWidth="1" min="5" max="5"/>
     <col width="36" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -824,6 +828,11 @@
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Precio lanzamiento (−20%)</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Condiciones de Pago / Financiamiento</t>
         </is>
@@ -872,12 +881,18 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
+          <t>US$ 800 · 120 cuotas de aprox. US$ 6,80/mes
+(descuento especial de lanzamiento)</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
           <t>Hasta 120 cuotas mensuales (aprox. US$ 8,50/mes).
 Debe estar pagado en su totalidad para el uso de la cremación y el columbario</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="78.5" customHeight="1">
+    <row r="6" ht="107.5" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Jardín de Cenizas · Individual</t>
@@ -890,7 +905,7 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Inhumación de la urna de cenizas en un contenedor enterrado con tapa de granito grabada, en un jardín de plantas de sombra: un lugar físico permanente de homenaje.</t>
+          <t>Inhumación de la urna de cenizas en un contenedor enterrado con tapa de granito grabada, en un jardín de plantas de sombra: un lugar físico de homenaje por 30 años desde la primera inhumación, renovable.</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
@@ -903,12 +918,13 @@
           <t>• Inhumación de la urna en contenedor individual
 • Tapa de granito con los datos del difunto
 • Ubicación en el Jardín 1, con paisajismo de plantas de sombra
-• Espacio de contemplación con banco</t>
+• Espacio de contemplación con banco
+• Permanencia de 30 años desde la primera inhumación, renovable por igual período</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>Familias que desean un lugar permanente para visitar y rendir homenaje, con una inversión moderada.</t>
+          <t>Familias que desean un lugar propio para visitar y rendir homenaje, con una inversión moderada.</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
@@ -919,6 +935,12 @@
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
+          <t>US$ 480
+(descuento especial de lanzamiento)</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
           <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 15 anual.</t>
         </is>
       </c>
@@ -936,7 +958,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Parcela familiar en el Jardín 1 con cuatro contenedores agrupados, cada uno con tapa de granito grabada, sin plazo de permanencia.</t>
+          <t>Parcela familiar en el Jardín 1 con cuatro contenedores agrupados, cada uno con tapa de granito grabada, con permanencia de 30 años desde la primera inhumación, renovable por igual período.</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -949,23 +971,29 @@
           <t>• Inhumación de hasta 4 urnas
 • Tapa de granito grabada para cada espacio
 • Ubicación en el Jardín 1, con paisajismo de plantas de sombra
-• Lugar físico permanente de homenaje familiar, sin plazo</t>
+• Lugar de homenaje familiar por 30 años, renovable por igual período</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Familias que buscan un espacio propio y permanente para varias generaciones.</t>
+          <t>Familias que buscan un espacio propio para varias generaciones.</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
           <t>US$ 2.000
-(Por parcela familiar · hasta 4 espacios · mantenimiento US$ 25/año)</t>
+(Por parcela familiar · hasta 4 espacios · mantenimiento US$ 24/año)</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 25 anual.</t>
+          <t>US$ 1.600
+(descuento especial de lanzamiento)</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 24 anual.</t>
         </is>
       </c>
     </row>
@@ -1012,6 +1040,12 @@
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
+          <t>US$ 600
+(descuento especial de lanzamiento)</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
           <t>Pago único o financiado según política comercial vigente. Incluye la placa memorial en el monumento al término del plazo.</t>
         </is>
       </c>
@@ -1058,6 +1092,12 @@
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
+          <t>US$ 320 / US$ 440
+(descuento especial de lanzamiento)</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
           <t>Pago único; puede contratarse como adicional al plan funerario. La opción de US$ 550 incluye la placa memorial en el monumento al término del plazo.</t>
         </is>
       </c>
@@ -1103,15 +1143,20 @@
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
           <t>A definir.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H10"/>
+  <autoFilter ref="A4:I10"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -1125,7 +1170,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:E127"/>
+  <dimension ref="B1:E134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1330,395 +1375,400 @@
       <c r="D17" s="26" t="n"/>
       <c r="E17" s="27" t="n"/>
     </row>
-    <row r="18" ht="20.5" customHeight="1">
+    <row r="18" ht="26.5" customHeight="1">
       <c r="B18" s="28" t="inlineStr">
         <is>
-          <t>Base de precio</t>
-        </is>
-      </c>
-      <c r="C18" s="29" t="inlineStr">
-        <is>
-          <t>Por módulo individual</t>
+          <t>Precio lanzamiento (−20%)</t>
+        </is>
+      </c>
+      <c r="C18" s="33" t="inlineStr">
+        <is>
+          <t>US$ 800 · 120 cuotas de aprox. US$ 6,80/mes</t>
         </is>
       </c>
       <c r="D18" s="30" t="n"/>
       <c r="E18" s="31" t="n"/>
     </row>
-    <row r="19" ht="35" customHeight="1">
-      <c r="B19" s="24" t="inlineStr">
+    <row r="19" ht="20.5" customHeight="1">
+      <c r="B19" s="28" t="inlineStr">
+        <is>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C19" s="29" t="inlineStr">
+        <is>
+          <t>Por módulo individual</t>
+        </is>
+      </c>
+      <c r="D19" s="30" t="n"/>
+      <c r="E19" s="31" t="n"/>
+    </row>
+    <row r="20" ht="35" customHeight="1">
+      <c r="B20" s="24" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C19" s="25" t="inlineStr">
+      <c r="C20" s="25" t="inlineStr">
         <is>
           <t>Hasta 120 cuotas mensuales (aprox. US$ 8,50/mes).
 Debe estar pagado en su totalidad para el uso de la cremación y el columbario</t>
         </is>
       </c>
-      <c r="D19" s="26" t="n"/>
-      <c r="E19" s="27" t="n"/>
-    </row>
-    <row r="20" ht="20.5" customHeight="1">
-      <c r="B20" s="28" t="inlineStr">
+      <c r="D20" s="26" t="n"/>
+      <c r="E20" s="27" t="n"/>
+    </row>
+    <row r="21" ht="20.5" customHeight="1">
+      <c r="B21" s="28" t="inlineStr">
         <is>
           <t>Cuota referencial</t>
         </is>
       </c>
-      <c r="C20" s="29" t="inlineStr">
+      <c r="C21" s="29" t="inlineStr">
         <is>
           <t>US$ 8,33/mes sin intereses (120 cuotas)</t>
         </is>
       </c>
-      <c r="D20" s="30" t="n"/>
-      <c r="E20" s="31" t="n"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="B21" s="21" t="inlineStr">
+      <c r="D21" s="30" t="n"/>
+      <c r="E21" s="31" t="n"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="B22" s="21" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C21" s="22" t="n"/>
-      <c r="D21" s="22" t="n"/>
-      <c r="E21" s="23" t="n"/>
-    </row>
-    <row r="22" ht="35" customHeight="1">
-      <c r="B22" s="33" t="inlineStr">
+      <c r="C22" s="22" t="n"/>
+      <c r="D22" s="22" t="n"/>
+      <c r="E22" s="23" t="n"/>
+    </row>
+    <row r="23" ht="35" customHeight="1">
+      <c r="B23" s="34" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C22" s="34" t="inlineStr">
+      <c r="C23" s="35" t="inlineStr">
         <is>
           <t>Afiliados actuales y nuevos que desean incorporar la cremación a su plan con una cuota mensual mínima.</t>
         </is>
       </c>
-      <c r="D22" s="35" t="n"/>
-      <c r="E22" s="36" t="n"/>
-    </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="B25" s="15" t="inlineStr">
+      <c r="D23" s="36" t="n"/>
+      <c r="E23" s="37" t="n"/>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="B26" s="15" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · INDIVIDUAL</t>
         </is>
       </c>
-      <c r="C25" s="16" t="n"/>
-      <c r="D25" s="16" t="n"/>
-      <c r="E25" s="17" t="n"/>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="B26" s="18" t="inlineStr">
+      <c r="C26" s="16" t="n"/>
+      <c r="D26" s="16" t="n"/>
+      <c r="E26" s="17" t="n"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="B27" s="18" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Jardín 1  ·  Destino final · Inhumación individual</t>
         </is>
       </c>
-      <c r="C26" s="19" t="n"/>
-      <c r="D26" s="19" t="n"/>
-      <c r="E26" s="20" t="n"/>
-    </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="B27" s="21" t="inlineStr">
+      <c r="C27" s="19" t="n"/>
+      <c r="D27" s="19" t="n"/>
+      <c r="E27" s="20" t="n"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="B28" s="21" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C27" s="22" t="n"/>
-      <c r="D27" s="22" t="n"/>
-      <c r="E27" s="23" t="n"/>
-    </row>
-    <row r="28" ht="49.5" customHeight="1">
-      <c r="B28" s="24" t="inlineStr">
+      <c r="C28" s="22" t="n"/>
+      <c r="D28" s="22" t="n"/>
+      <c r="E28" s="23" t="n"/>
+    </row>
+    <row r="29" ht="49.5" customHeight="1">
+      <c r="B29" s="24" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C28" s="25" t="inlineStr">
-        <is>
-          <t>Inhumación de la urna de cenizas en un contenedor enterrado con tapa de granito grabada, en un jardín de plantas de sombra: un lugar físico permanente de homenaje.</t>
-        </is>
-      </c>
-      <c r="D28" s="26" t="n"/>
-      <c r="E28" s="27" t="n"/>
-    </row>
-    <row r="29" ht="20.5" customHeight="1">
-      <c r="B29" s="28" t="inlineStr">
+      <c r="C29" s="25" t="inlineStr">
+        <is>
+          <t>Inhumación de la urna de cenizas en un contenedor enterrado con tapa de granito grabada, en un jardín de plantas de sombra: un lugar físico de homenaje por 30 años desde la primera inhumación, renovable.</t>
+        </is>
+      </c>
+      <c r="D29" s="26" t="n"/>
+      <c r="E29" s="27" t="n"/>
+    </row>
+    <row r="30" ht="20.5" customHeight="1">
+      <c r="B30" s="28" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C29" s="29" t="inlineStr">
+      <c r="C30" s="29" t="inlineStr">
         <is>
           <t>Individual (1 urna).</t>
         </is>
       </c>
-      <c r="D29" s="30" t="n"/>
-      <c r="E29" s="31" t="n"/>
-    </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="B30" s="21" t="inlineStr">
+      <c r="D30" s="30" t="n"/>
+      <c r="E30" s="31" t="n"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="B31" s="21" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C30" s="22" t="n"/>
-      <c r="D30" s="22" t="n"/>
-      <c r="E30" s="23" t="n"/>
-    </row>
-    <row r="31" ht="20.5" customHeight="1">
-      <c r="B31" s="24" t="inlineStr">
+      <c r="C31" s="22" t="n"/>
+      <c r="D31" s="22" t="n"/>
+      <c r="E31" s="23" t="n"/>
+    </row>
+    <row r="32" ht="20.5" customHeight="1">
+      <c r="B32" s="24" t="inlineStr">
         <is>
           <t>Ambiente</t>
         </is>
       </c>
-      <c r="C31" s="25" t="inlineStr">
+      <c r="C32" s="25" t="inlineStr">
         <is>
           <t>Jardín 1</t>
         </is>
       </c>
-      <c r="D31" s="26" t="n"/>
-      <c r="E31" s="27" t="n"/>
-    </row>
-    <row r="32" ht="20.5" customHeight="1">
-      <c r="B32" s="28" t="inlineStr">
+      <c r="D32" s="26" t="n"/>
+      <c r="E32" s="27" t="n"/>
+    </row>
+    <row r="33" ht="20.5" customHeight="1">
+      <c r="B33" s="28" t="inlineStr">
         <is>
           <t>Contenedor</t>
         </is>
       </c>
-      <c r="C32" s="29" t="inlineStr">
+      <c r="C33" s="29" t="inlineStr">
         <is>
           <t>Ø 32 cm × 40 cm de altura; enterrado dejando 20 cm a la vista</t>
         </is>
       </c>
-      <c r="D32" s="30" t="n"/>
-      <c r="E32" s="31" t="n"/>
-    </row>
-    <row r="33" ht="20.5" customHeight="1">
-      <c r="B33" s="24" t="inlineStr">
+      <c r="D33" s="30" t="n"/>
+      <c r="E33" s="31" t="n"/>
+    </row>
+    <row r="34" ht="20.5" customHeight="1">
+      <c r="B34" s="24" t="inlineStr">
         <is>
           <t>Identificación</t>
         </is>
       </c>
-      <c r="C33" s="25" t="inlineStr">
+      <c r="C34" s="25" t="inlineStr">
         <is>
           <t>Tapa de granito con la información del difunto</t>
         </is>
       </c>
-      <c r="D33" s="26" t="n"/>
-      <c r="E33" s="27" t="n"/>
-    </row>
-    <row r="34" ht="20.5" customHeight="1">
-      <c r="B34" s="28" t="inlineStr">
+      <c r="D34" s="26" t="n"/>
+      <c r="E34" s="27" t="n"/>
+    </row>
+    <row r="35" ht="20.5" customHeight="1">
+      <c r="B35" s="28" t="inlineStr">
         <is>
           <t>Paisajismo</t>
         </is>
       </c>
-      <c r="C34" s="29" t="inlineStr">
+      <c r="C35" s="29" t="inlineStr">
         <is>
           <t>Plantas de sombra de diferentes alturas y texturas</t>
         </is>
       </c>
-      <c r="D34" s="30" t="n"/>
-      <c r="E34" s="31" t="n"/>
-    </row>
-    <row r="35" ht="20.5" customHeight="1">
-      <c r="B35" s="24" t="inlineStr">
+      <c r="D35" s="30" t="n"/>
+      <c r="E35" s="31" t="n"/>
+    </row>
+    <row r="36" ht="20.5" customHeight="1">
+      <c r="B36" s="24" t="inlineStr">
         <is>
           <t>Acceso</t>
         </is>
       </c>
-      <c r="C35" s="25" t="inlineStr">
+      <c r="C36" s="25" t="inlineStr">
         <is>
           <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
         </is>
       </c>
-      <c r="D35" s="26" t="n"/>
-      <c r="E35" s="27" t="n"/>
-    </row>
-    <row r="36" ht="20.5" customHeight="1">
-      <c r="B36" s="28" t="inlineStr">
+      <c r="D36" s="26" t="n"/>
+      <c r="E36" s="27" t="n"/>
+    </row>
+    <row r="37" ht="20.5" customHeight="1">
+      <c r="B37" s="28" t="inlineStr">
+        <is>
+          <t>Permanencia</t>
+        </is>
+      </c>
+      <c r="C37" s="29" t="inlineStr">
+        <is>
+          <t>30 años desde la primera inhumación, renovable por igual período</t>
+        </is>
+      </c>
+      <c r="D37" s="30" t="n"/>
+      <c r="E37" s="31" t="n"/>
+    </row>
+    <row r="38" ht="20.5" customHeight="1">
+      <c r="B38" s="24" t="inlineStr">
         <is>
           <t>Mantenimiento</t>
         </is>
       </c>
-      <c r="C36" s="29" t="inlineStr">
+      <c r="C38" s="25" t="inlineStr">
         <is>
           <t>US$ 15 anual</t>
         </is>
       </c>
-      <c r="D36" s="30" t="n"/>
-      <c r="E36" s="31" t="n"/>
-    </row>
-    <row r="37" ht="64" customHeight="1">
-      <c r="B37" s="24" t="inlineStr">
+      <c r="D38" s="26" t="n"/>
+      <c r="E38" s="27" t="n"/>
+    </row>
+    <row r="39" ht="93" customHeight="1">
+      <c r="B39" s="28" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C37" s="25" t="inlineStr">
+      <c r="C39" s="29" t="inlineStr">
         <is>
           <t>• Inhumación de la urna en contenedor individual
 • Tapa de granito con los datos del difunto
 • Ubicación en el Jardín 1, con paisajismo de plantas de sombra
-• Espacio de contemplación con banco</t>
-        </is>
-      </c>
-      <c r="D37" s="26" t="n"/>
-      <c r="E37" s="27" t="n"/>
-    </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="B38" s="21" t="inlineStr">
+• Espacio de contemplación con banco
+• Permanencia de 30 años desde la primera inhumación, renovable por igual período</t>
+        </is>
+      </c>
+      <c r="D39" s="30" t="n"/>
+      <c r="E39" s="31" t="n"/>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="B40" s="21" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C38" s="22" t="n"/>
-      <c r="D38" s="22" t="n"/>
-      <c r="E38" s="23" t="n"/>
-    </row>
-    <row r="39" ht="26.5" customHeight="1">
-      <c r="B39" s="24" t="inlineStr">
+      <c r="C40" s="22" t="n"/>
+      <c r="D40" s="22" t="n"/>
+      <c r="E40" s="23" t="n"/>
+    </row>
+    <row r="41" ht="26.5" customHeight="1">
+      <c r="B41" s="24" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C39" s="32" t="inlineStr">
+      <c r="C41" s="32" t="inlineStr">
         <is>
           <t>US$ 600</t>
-        </is>
-      </c>
-      <c r="D39" s="26" t="n"/>
-      <c r="E39" s="27" t="n"/>
-    </row>
-    <row r="40" ht="20.5" customHeight="1">
-      <c r="B40" s="28" t="inlineStr">
-        <is>
-          <t>Base de precio</t>
-        </is>
-      </c>
-      <c r="C40" s="29" t="inlineStr">
-        <is>
-          <t>Por espacio individual · mantenimiento US$ 15/año</t>
-        </is>
-      </c>
-      <c r="D40" s="30" t="n"/>
-      <c r="E40" s="31" t="n"/>
-    </row>
-    <row r="41" ht="35" customHeight="1">
-      <c r="B41" s="24" t="inlineStr">
-        <is>
-          <t>Condiciones</t>
-        </is>
-      </c>
-      <c r="C41" s="25" t="inlineStr">
-        <is>
-          <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 15 anual.</t>
         </is>
       </c>
       <c r="D41" s="26" t="n"/>
       <c r="E41" s="27" t="n"/>
     </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="B42" s="21" t="inlineStr">
+    <row r="42" ht="26.5" customHeight="1">
+      <c r="B42" s="28" t="inlineStr">
+        <is>
+          <t>Precio lanzamiento (−20%)</t>
+        </is>
+      </c>
+      <c r="C42" s="33" t="inlineStr">
+        <is>
+          <t>US$ 480</t>
+        </is>
+      </c>
+      <c r="D42" s="30" t="n"/>
+      <c r="E42" s="31" t="n"/>
+    </row>
+    <row r="43" ht="20.5" customHeight="1">
+      <c r="B43" s="28" t="inlineStr">
+        <is>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C43" s="29" t="inlineStr">
+        <is>
+          <t>Por espacio individual · mantenimiento US$ 15/año</t>
+        </is>
+      </c>
+      <c r="D43" s="30" t="n"/>
+      <c r="E43" s="31" t="n"/>
+    </row>
+    <row r="44" ht="35" customHeight="1">
+      <c r="B44" s="24" t="inlineStr">
+        <is>
+          <t>Condiciones</t>
+        </is>
+      </c>
+      <c r="C44" s="25" t="inlineStr">
+        <is>
+          <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 15 anual.</t>
+        </is>
+      </c>
+      <c r="D44" s="26" t="n"/>
+      <c r="E44" s="27" t="n"/>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="B45" s="21" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C42" s="22" t="n"/>
-      <c r="D42" s="22" t="n"/>
-      <c r="E42" s="23" t="n"/>
-    </row>
-    <row r="43" ht="35" customHeight="1">
-      <c r="B43" s="33" t="inlineStr">
+      <c r="C45" s="22" t="n"/>
+      <c r="D45" s="22" t="n"/>
+      <c r="E45" s="23" t="n"/>
+    </row>
+    <row r="46" ht="35" customHeight="1">
+      <c r="B46" s="34" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C43" s="34" t="inlineStr">
-        <is>
-          <t>Familias que desean un lugar permanente para visitar y rendir homenaje, con una inversión moderada.</t>
-        </is>
-      </c>
-      <c r="D43" s="35" t="n"/>
-      <c r="E43" s="36" t="n"/>
-    </row>
-    <row r="46" ht="30" customHeight="1">
-      <c r="B46" s="15" t="inlineStr">
+      <c r="C46" s="35" t="inlineStr">
+        <is>
+          <t>Familias que desean un lugar propio para visitar y rendir homenaje, con una inversión moderada.</t>
+        </is>
+      </c>
+      <c r="D46" s="36" t="n"/>
+      <c r="E46" s="37" t="n"/>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="B49" s="15" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · FAMILIAR</t>
         </is>
       </c>
-      <c r="C46" s="16" t="n"/>
-      <c r="D46" s="16" t="n"/>
-      <c r="E46" s="17" t="n"/>
-    </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="B47" s="18" t="inlineStr">
+      <c r="C49" s="16" t="n"/>
+      <c r="D49" s="16" t="n"/>
+      <c r="E49" s="17" t="n"/>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="B50" s="18" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Jardín 1  ·  Destino final · Inhumación familiar</t>
         </is>
       </c>
-      <c r="C47" s="19" t="n"/>
-      <c r="D47" s="19" t="n"/>
-      <c r="E47" s="20" t="n"/>
-    </row>
-    <row r="48" ht="20" customHeight="1">
-      <c r="B48" s="21" t="inlineStr">
-        <is>
-          <t>VISIÓN GENERAL</t>
-        </is>
-      </c>
-      <c r="C48" s="22" t="n"/>
-      <c r="D48" s="22" t="n"/>
-      <c r="E48" s="23" t="n"/>
-    </row>
-    <row r="49" ht="35" customHeight="1">
-      <c r="B49" s="24" t="inlineStr">
-        <is>
-          <t>Concepto</t>
-        </is>
-      </c>
-      <c r="C49" s="25" t="inlineStr">
-        <is>
-          <t>Parcela familiar en el Jardín 1 con cuatro contenedores agrupados, cada uno con tapa de granito grabada, sin plazo de permanencia.</t>
-        </is>
-      </c>
-      <c r="D49" s="26" t="n"/>
-      <c r="E49" s="27" t="n"/>
-    </row>
-    <row r="50" ht="20.5" customHeight="1">
-      <c r="B50" s="28" t="inlineStr">
-        <is>
-          <t>Capacidad / Cobertura</t>
-        </is>
-      </c>
-      <c r="C50" s="29" t="inlineStr">
-        <is>
-          <t>Hasta 4 espacios (familiar).</t>
-        </is>
-      </c>
-      <c r="D50" s="30" t="n"/>
-      <c r="E50" s="31" t="n"/>
+      <c r="C50" s="19" t="n"/>
+      <c r="D50" s="19" t="n"/>
+      <c r="E50" s="20" t="n"/>
     </row>
     <row r="51" ht="20" customHeight="1">
       <c r="B51" s="21" t="inlineStr">
         <is>
-          <t>ESPECIFICACIONES TÉCNICAS</t>
+          <t>VISIÓN GENERAL</t>
         </is>
       </c>
       <c r="C51" s="22" t="n"/>
       <c r="D51" s="22" t="n"/>
       <c r="E51" s="23" t="n"/>
     </row>
-    <row r="52" ht="20.5" customHeight="1">
+    <row r="52" ht="49.5" customHeight="1">
       <c r="B52" s="24" t="inlineStr">
         <is>
-          <t>Ambiente</t>
+          <t>Concepto</t>
         </is>
       </c>
       <c r="C52" s="25" t="inlineStr">
         <is>
-          <t>Jardín 1</t>
+          <t>Parcela familiar en el Jardín 1 con cuatro contenedores agrupados, cada uno con tapa de granito grabada, con permanencia de 30 años desde la primera inhumación, renovable por igual período.</t>
         </is>
       </c>
       <c r="D52" s="26" t="n"/>
@@ -1727,313 +1777,309 @@
     <row r="53" ht="20.5" customHeight="1">
       <c r="B53" s="28" t="inlineStr">
         <is>
-          <t>Capacidad</t>
+          <t>Capacidad / Cobertura</t>
         </is>
       </c>
       <c r="C53" s="29" t="inlineStr">
         <is>
-          <t>4 contenedores agrupados en losa</t>
+          <t>Hasta 4 espacios (familiar).</t>
         </is>
       </c>
       <c r="D53" s="30" t="n"/>
       <c r="E53" s="31" t="n"/>
     </row>
-    <row r="54" ht="20.5" customHeight="1">
-      <c r="B54" s="24" t="inlineStr">
+    <row r="54" ht="20" customHeight="1">
+      <c r="B54" s="21" t="inlineStr">
+        <is>
+          <t>ESPECIFICACIONES TÉCNICAS</t>
+        </is>
+      </c>
+      <c r="C54" s="22" t="n"/>
+      <c r="D54" s="22" t="n"/>
+      <c r="E54" s="23" t="n"/>
+    </row>
+    <row r="55" ht="20.5" customHeight="1">
+      <c r="B55" s="24" t="inlineStr">
+        <is>
+          <t>Ambiente</t>
+        </is>
+      </c>
+      <c r="C55" s="25" t="inlineStr">
+        <is>
+          <t>Jardín 1</t>
+        </is>
+      </c>
+      <c r="D55" s="26" t="n"/>
+      <c r="E55" s="27" t="n"/>
+    </row>
+    <row r="56" ht="20.5" customHeight="1">
+      <c r="B56" s="28" t="inlineStr">
+        <is>
+          <t>Capacidad</t>
+        </is>
+      </c>
+      <c r="C56" s="29" t="inlineStr">
+        <is>
+          <t>4 contenedores agrupados en losa</t>
+        </is>
+      </c>
+      <c r="D56" s="30" t="n"/>
+      <c r="E56" s="31" t="n"/>
+    </row>
+    <row r="57" ht="20.5" customHeight="1">
+      <c r="B57" s="24" t="inlineStr">
         <is>
           <t>Identificación</t>
         </is>
       </c>
-      <c r="C54" s="25" t="inlineStr">
+      <c r="C57" s="25" t="inlineStr">
         <is>
           <t>Tapa de granito por espacio, con la información del difunto</t>
         </is>
       </c>
-      <c r="D54" s="26" t="n"/>
-      <c r="E54" s="27" t="n"/>
-    </row>
-    <row r="55" ht="20.5" customHeight="1">
-      <c r="B55" s="28" t="inlineStr">
+      <c r="D57" s="26" t="n"/>
+      <c r="E57" s="27" t="n"/>
+    </row>
+    <row r="58" ht="20.5" customHeight="1">
+      <c r="B58" s="28" t="inlineStr">
         <is>
           <t>Permanencia</t>
         </is>
       </c>
-      <c r="C55" s="29" t="inlineStr">
-        <is>
-          <t>Sin plazo</t>
-        </is>
-      </c>
-      <c r="D55" s="30" t="n"/>
-      <c r="E55" s="31" t="n"/>
-    </row>
-    <row r="56" ht="20.5" customHeight="1">
-      <c r="B56" s="24" t="inlineStr">
+      <c r="C58" s="29" t="inlineStr">
+        <is>
+          <t>30 años desde la primera inhumación, renovable por igual período</t>
+        </is>
+      </c>
+      <c r="D58" s="30" t="n"/>
+      <c r="E58" s="31" t="n"/>
+    </row>
+    <row r="59" ht="20.5" customHeight="1">
+      <c r="B59" s="24" t="inlineStr">
         <is>
           <t>Acceso</t>
         </is>
       </c>
-      <c r="C56" s="25" t="inlineStr">
+      <c r="C59" s="25" t="inlineStr">
         <is>
           <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
         </is>
       </c>
-      <c r="D56" s="26" t="n"/>
-      <c r="E56" s="27" t="n"/>
-    </row>
-    <row r="57" ht="20.5" customHeight="1">
-      <c r="B57" s="28" t="inlineStr">
+      <c r="D59" s="26" t="n"/>
+      <c r="E59" s="27" t="n"/>
+    </row>
+    <row r="60" ht="20.5" customHeight="1">
+      <c r="B60" s="28" t="inlineStr">
         <is>
           <t>Mantenimiento</t>
         </is>
       </c>
-      <c r="C57" s="29" t="inlineStr">
-        <is>
-          <t>US$ 25 anual</t>
-        </is>
-      </c>
-      <c r="D57" s="30" t="n"/>
-      <c r="E57" s="31" t="n"/>
-    </row>
-    <row r="58" ht="64" customHeight="1">
-      <c r="B58" s="24" t="inlineStr">
+      <c r="C60" s="29" t="inlineStr">
+        <is>
+          <t>US$ 24 anual</t>
+        </is>
+      </c>
+      <c r="D60" s="30" t="n"/>
+      <c r="E60" s="31" t="n"/>
+    </row>
+    <row r="61" ht="64" customHeight="1">
+      <c r="B61" s="24" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C58" s="25" t="inlineStr">
+      <c r="C61" s="25" t="inlineStr">
         <is>
           <t>• Inhumación de hasta 4 urnas
 • Tapa de granito grabada para cada espacio
 • Ubicación en el Jardín 1, con paisajismo de plantas de sombra
-• Lugar físico permanente de homenaje familiar, sin plazo</t>
-        </is>
-      </c>
-      <c r="D58" s="26" t="n"/>
-      <c r="E58" s="27" t="n"/>
-    </row>
-    <row r="59" ht="20" customHeight="1">
-      <c r="B59" s="21" t="inlineStr">
+• Lugar de homenaje familiar por 30 años, renovable por igual período</t>
+        </is>
+      </c>
+      <c r="D61" s="26" t="n"/>
+      <c r="E61" s="27" t="n"/>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="B62" s="21" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C59" s="22" t="n"/>
-      <c r="D59" s="22" t="n"/>
-      <c r="E59" s="23" t="n"/>
-    </row>
-    <row r="60" ht="26.5" customHeight="1">
-      <c r="B60" s="24" t="inlineStr">
+      <c r="C62" s="22" t="n"/>
+      <c r="D62" s="22" t="n"/>
+      <c r="E62" s="23" t="n"/>
+    </row>
+    <row r="63" ht="26.5" customHeight="1">
+      <c r="B63" s="24" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C60" s="32" t="inlineStr">
+      <c r="C63" s="32" t="inlineStr">
         <is>
           <t>US$ 2.000</t>
         </is>
       </c>
-      <c r="D60" s="26" t="n"/>
-      <c r="E60" s="27" t="n"/>
-    </row>
-    <row r="61" ht="20.5" customHeight="1">
-      <c r="B61" s="28" t="inlineStr">
+      <c r="D63" s="26" t="n"/>
+      <c r="E63" s="27" t="n"/>
+    </row>
+    <row r="64" ht="26.5" customHeight="1">
+      <c r="B64" s="28" t="inlineStr">
+        <is>
+          <t>Precio lanzamiento (−20%)</t>
+        </is>
+      </c>
+      <c r="C64" s="33" t="inlineStr">
+        <is>
+          <t>US$ 1.600</t>
+        </is>
+      </c>
+      <c r="D64" s="30" t="n"/>
+      <c r="E64" s="31" t="n"/>
+    </row>
+    <row r="65" ht="20.5" customHeight="1">
+      <c r="B65" s="28" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C61" s="29" t="inlineStr">
-        <is>
-          <t>Por parcela familiar · hasta 4 espacios · mantenimiento US$ 25/año</t>
-        </is>
-      </c>
-      <c r="D61" s="30" t="n"/>
-      <c r="E61" s="31" t="n"/>
-    </row>
-    <row r="62" ht="35" customHeight="1">
-      <c r="B62" s="24" t="inlineStr">
+      <c r="C65" s="29" t="inlineStr">
+        <is>
+          <t>Por parcela familiar · hasta 4 espacios · mantenimiento US$ 24/año</t>
+        </is>
+      </c>
+      <c r="D65" s="30" t="n"/>
+      <c r="E65" s="31" t="n"/>
+    </row>
+    <row r="66" ht="35" customHeight="1">
+      <c r="B66" s="24" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C62" s="25" t="inlineStr">
-        <is>
-          <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 25 anual.</t>
-        </is>
-      </c>
-      <c r="D62" s="26" t="n"/>
-      <c r="E62" s="27" t="n"/>
-    </row>
-    <row r="63" ht="20" customHeight="1">
-      <c r="B63" s="21" t="inlineStr">
+      <c r="C66" s="25" t="inlineStr">
+        <is>
+          <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 24 anual.</t>
+        </is>
+      </c>
+      <c r="D66" s="26" t="n"/>
+      <c r="E66" s="27" t="n"/>
+    </row>
+    <row r="67" ht="20" customHeight="1">
+      <c r="B67" s="21" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C63" s="22" t="n"/>
-      <c r="D63" s="22" t="n"/>
-      <c r="E63" s="23" t="n"/>
-    </row>
-    <row r="64" ht="20.5" customHeight="1">
-      <c r="B64" s="33" t="inlineStr">
+      <c r="C67" s="22" t="n"/>
+      <c r="D67" s="22" t="n"/>
+      <c r="E67" s="23" t="n"/>
+    </row>
+    <row r="68" ht="20.5" customHeight="1">
+      <c r="B68" s="34" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C64" s="34" t="inlineStr">
-        <is>
-          <t>Familias que buscan un espacio propio y permanente para varias generaciones.</t>
-        </is>
-      </c>
-      <c r="D64" s="35" t="n"/>
-      <c r="E64" s="36" t="n"/>
-    </row>
-    <row r="67" ht="30" customHeight="1">
-      <c r="B67" s="15" t="inlineStr">
+      <c r="C68" s="35" t="inlineStr">
+        <is>
+          <t>Familias que buscan un espacio propio para varias generaciones.</t>
+        </is>
+      </c>
+      <c r="D68" s="36" t="n"/>
+      <c r="E68" s="37" t="n"/>
+    </row>
+    <row r="71" ht="30" customHeight="1">
+      <c r="B71" s="15" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · ECOLÓGICO</t>
         </is>
       </c>
-      <c r="C67" s="16" t="n"/>
-      <c r="D67" s="16" t="n"/>
-      <c r="E67" s="17" t="n"/>
-    </row>
-    <row r="68" ht="20" customHeight="1">
-      <c r="B68" s="18" t="inlineStr">
+      <c r="C71" s="16" t="n"/>
+      <c r="D71" s="16" t="n"/>
+      <c r="E71" s="17" t="n"/>
+    </row>
+    <row r="72" ht="20" customHeight="1">
+      <c r="B72" s="18" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Jardín 2  ·  Destino final · Inhumación ecológica</t>
         </is>
       </c>
-      <c r="C68" s="19" t="n"/>
-      <c r="D68" s="19" t="n"/>
-      <c r="E68" s="20" t="n"/>
-    </row>
-    <row r="69" ht="20" customHeight="1">
-      <c r="B69" s="21" t="inlineStr">
+      <c r="C72" s="19" t="n"/>
+      <c r="D72" s="19" t="n"/>
+      <c r="E72" s="20" t="n"/>
+    </row>
+    <row r="73" ht="20" customHeight="1">
+      <c r="B73" s="21" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C69" s="22" t="n"/>
-      <c r="D69" s="22" t="n"/>
-      <c r="E69" s="23" t="n"/>
-    </row>
-    <row r="70" ht="49.5" customHeight="1">
-      <c r="B70" s="24" t="inlineStr">
+      <c r="C73" s="22" t="n"/>
+      <c r="D73" s="22" t="n"/>
+      <c r="E73" s="23" t="n"/>
+    </row>
+    <row r="74" ht="49.5" customHeight="1">
+      <c r="B74" s="24" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C70" s="25" t="inlineStr">
+      <c r="C74" s="25" t="inlineStr">
         <is>
           <t>La urna biodegradable se entierra directamente en el suelo, se cubre con tierra y se descompone integrándose a la naturaleza. Jardín con agua corriente y área de esparcimiento de cenizas.</t>
         </is>
       </c>
-      <c r="D70" s="26" t="n"/>
-      <c r="E70" s="27" t="n"/>
-    </row>
-    <row r="71" ht="20.5" customHeight="1">
-      <c r="B71" s="28" t="inlineStr">
+      <c r="D74" s="26" t="n"/>
+      <c r="E74" s="27" t="n"/>
+    </row>
+    <row r="75" ht="20.5" customHeight="1">
+      <c r="B75" s="28" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C71" s="29" t="inlineStr">
+      <c r="C75" s="29" t="inlineStr">
         <is>
           <t>Individual (1 urna).</t>
         </is>
       </c>
-      <c r="D71" s="30" t="n"/>
-      <c r="E71" s="31" t="n"/>
-    </row>
-    <row r="72" ht="20" customHeight="1">
-      <c r="B72" s="21" t="inlineStr">
+      <c r="D75" s="30" t="n"/>
+      <c r="E75" s="31" t="n"/>
+    </row>
+    <row r="76" ht="20" customHeight="1">
+      <c r="B76" s="21" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C72" s="22" t="n"/>
-      <c r="D72" s="22" t="n"/>
-      <c r="E72" s="23" t="n"/>
-    </row>
-    <row r="73" ht="20.5" customHeight="1">
-      <c r="B73" s="24" t="inlineStr">
-        <is>
-          <t>Ambientes</t>
-        </is>
-      </c>
-      <c r="C73" s="25" t="inlineStr">
-        <is>
-          <t>Jardín 2 · Ecológico o Bosque de las Orquídeas</t>
-        </is>
-      </c>
-      <c r="D73" s="26" t="n"/>
-      <c r="E73" s="27" t="n"/>
-    </row>
-    <row r="74" ht="20.5" customHeight="1">
-      <c r="B74" s="28" t="inlineStr">
-        <is>
-          <t>Espacio por urna</t>
-        </is>
-      </c>
-      <c r="C74" s="29" t="inlineStr">
-        <is>
-          <t>30 × 30 cm, 40 cm de profundidad</t>
-        </is>
-      </c>
-      <c r="D74" s="30" t="n"/>
-      <c r="E74" s="31" t="n"/>
-    </row>
-    <row r="75" ht="20.5" customHeight="1">
-      <c r="B75" s="24" t="inlineStr">
-        <is>
-          <t>Urna</t>
-        </is>
-      </c>
-      <c r="C75" s="25" t="inlineStr">
-        <is>
-          <t>Biodegradable; se integra al suelo</t>
-        </is>
-      </c>
-      <c r="D75" s="26" t="n"/>
-      <c r="E75" s="27" t="n"/>
-    </row>
-    <row r="76" ht="35" customHeight="1">
-      <c r="B76" s="28" t="inlineStr">
-        <is>
-          <t>Identificación (Jardín 2)</t>
-        </is>
-      </c>
-      <c r="C76" s="29" t="inlineStr">
-        <is>
-          <t>Placa de madera de 20 cm fijada a una varilla metálica, en posición vertical y sin contacto con el suelo</t>
-        </is>
-      </c>
-      <c r="D76" s="30" t="n"/>
-      <c r="E76" s="31" t="n"/>
+      <c r="C76" s="22" t="n"/>
+      <c r="D76" s="22" t="n"/>
+      <c r="E76" s="23" t="n"/>
     </row>
     <row r="77" ht="20.5" customHeight="1">
       <c r="B77" s="24" t="inlineStr">
         <is>
-          <t>Identificación (Bosque)</t>
+          <t>Ambientes</t>
         </is>
       </c>
       <c r="C77" s="25" t="inlineStr">
         <is>
-          <t>Placa de mármol de 20 × 15 cm</t>
+          <t>Jardín 2 · Ecológico o Bosque de las Orquídeas</t>
         </is>
       </c>
       <c r="D77" s="26" t="n"/>
       <c r="E77" s="27" t="n"/>
     </row>
-    <row r="78" ht="35" customHeight="1">
+    <row r="78" ht="20.5" customHeight="1">
       <c r="B78" s="28" t="inlineStr">
         <is>
-          <t>Permanencia</t>
+          <t>Espacio por urna</t>
         </is>
       </c>
       <c r="C78" s="29" t="inlineStr">
         <is>
-          <t>3 años; luego el nombre pasa a una placa memorial en el monumento y el espacio se reutiliza</t>
+          <t>30 × 30 cm, 40 cm de profundidad</t>
         </is>
       </c>
       <c r="D78" s="30" t="n"/>
@@ -2042,38 +2088,94 @@
     <row r="79" ht="20.5" customHeight="1">
       <c r="B79" s="24" t="inlineStr">
         <is>
-          <t>Placa memorial</t>
+          <t>Urna</t>
         </is>
       </c>
       <c r="C79" s="25" t="inlineStr">
         <is>
-          <t>Incluida en el precio</t>
+          <t>Biodegradable; se integra al suelo</t>
         </is>
       </c>
       <c r="D79" s="26" t="n"/>
       <c r="E79" s="27" t="n"/>
     </row>
-    <row r="80" ht="20.5" customHeight="1">
+    <row r="80" ht="35" customHeight="1">
       <c r="B80" s="28" t="inlineStr">
         <is>
-          <t>Acceso</t>
+          <t>Identificación (Jardín 2)</t>
         </is>
       </c>
       <c r="C80" s="29" t="inlineStr">
         <is>
-          <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
+          <t>Placa de madera de 20 cm fijada a una varilla metálica, en posición vertical y sin contacto con el suelo</t>
         </is>
       </c>
       <c r="D80" s="30" t="n"/>
       <c r="E80" s="31" t="n"/>
     </row>
-    <row r="81" ht="78.5" customHeight="1">
+    <row r="81" ht="20.5" customHeight="1">
       <c r="B81" s="24" t="inlineStr">
         <is>
+          <t>Identificación (Bosque)</t>
+        </is>
+      </c>
+      <c r="C81" s="25" t="inlineStr">
+        <is>
+          <t>Placa de mármol de 20 × 15 cm</t>
+        </is>
+      </c>
+      <c r="D81" s="26" t="n"/>
+      <c r="E81" s="27" t="n"/>
+    </row>
+    <row r="82" ht="35" customHeight="1">
+      <c r="B82" s="28" t="inlineStr">
+        <is>
+          <t>Permanencia</t>
+        </is>
+      </c>
+      <c r="C82" s="29" t="inlineStr">
+        <is>
+          <t>3 años; luego el nombre pasa a una placa memorial en el monumento y el espacio se reutiliza</t>
+        </is>
+      </c>
+      <c r="D82" s="30" t="n"/>
+      <c r="E82" s="31" t="n"/>
+    </row>
+    <row r="83" ht="20.5" customHeight="1">
+      <c r="B83" s="24" t="inlineStr">
+        <is>
+          <t>Placa memorial</t>
+        </is>
+      </c>
+      <c r="C83" s="25" t="inlineStr">
+        <is>
+          <t>Incluida en el precio</t>
+        </is>
+      </c>
+      <c r="D83" s="26" t="n"/>
+      <c r="E83" s="27" t="n"/>
+    </row>
+    <row r="84" ht="20.5" customHeight="1">
+      <c r="B84" s="28" t="inlineStr">
+        <is>
+          <t>Acceso</t>
+        </is>
+      </c>
+      <c r="C84" s="29" t="inlineStr">
+        <is>
+          <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
+        </is>
+      </c>
+      <c r="D84" s="30" t="n"/>
+      <c r="E84" s="31" t="n"/>
+    </row>
+    <row r="85" ht="78.5" customHeight="1">
+      <c r="B85" s="24" t="inlineStr">
+        <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C81" s="25" t="inlineStr">
+      <c r="C85" s="25" t="inlineStr">
         <is>
           <t>• Inhumación ecológica de la urna directamente en el suelo
 • Placa de identificación
@@ -2082,190 +2184,138 @@
 • Permanencia de 3 años; luego, placa memorial en el monumento (incluida)</t>
         </is>
       </c>
-      <c r="D81" s="26" t="n"/>
-      <c r="E81" s="27" t="n"/>
-    </row>
-    <row r="82" ht="20" customHeight="1">
-      <c r="B82" s="21" t="inlineStr">
-        <is>
-          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
-        </is>
-      </c>
-      <c r="C82" s="22" t="n"/>
-      <c r="D82" s="22" t="n"/>
-      <c r="E82" s="23" t="n"/>
-    </row>
-    <row r="83" ht="26.5" customHeight="1">
-      <c r="B83" s="24" t="inlineStr">
-        <is>
-          <t>Precio sugerido</t>
-        </is>
-      </c>
-      <c r="C83" s="32" t="inlineStr">
-        <is>
-          <t>US$ 750</t>
-        </is>
-      </c>
-      <c r="D83" s="26" t="n"/>
-      <c r="E83" s="27" t="n"/>
-    </row>
-    <row r="84" ht="20.5" customHeight="1">
-      <c r="B84" s="28" t="inlineStr">
-        <is>
-          <t>Base de precio</t>
-        </is>
-      </c>
-      <c r="C84" s="29" t="inlineStr">
-        <is>
-          <t>Por espacio individual · placa memorial incluida</t>
-        </is>
-      </c>
-      <c r="D84" s="30" t="n"/>
-      <c r="E84" s="31" t="n"/>
-    </row>
-    <row r="85" ht="35" customHeight="1">
-      <c r="B85" s="24" t="inlineStr">
-        <is>
-          <t>Condiciones</t>
-        </is>
-      </c>
-      <c r="C85" s="25" t="inlineStr">
-        <is>
-          <t>Pago único o financiado según política comercial vigente. Incluye la placa memorial en el monumento al término del plazo.</t>
-        </is>
-      </c>
       <c r="D85" s="26" t="n"/>
       <c r="E85" s="27" t="n"/>
     </row>
     <row r="86" ht="20" customHeight="1">
       <c r="B86" s="21" t="inlineStr">
         <is>
-          <t>PERFIL DEL COMPRADOR</t>
+          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
       <c r="C86" s="22" t="n"/>
       <c r="D86" s="22" t="n"/>
       <c r="E86" s="23" t="n"/>
     </row>
-    <row r="87" ht="35" customHeight="1">
-      <c r="B87" s="33" t="inlineStr">
+    <row r="87" ht="26.5" customHeight="1">
+      <c r="B87" s="24" t="inlineStr">
+        <is>
+          <t>Precio sugerido</t>
+        </is>
+      </c>
+      <c r="C87" s="32" t="inlineStr">
+        <is>
+          <t>US$ 750</t>
+        </is>
+      </c>
+      <c r="D87" s="26" t="n"/>
+      <c r="E87" s="27" t="n"/>
+    </row>
+    <row r="88" ht="26.5" customHeight="1">
+      <c r="B88" s="28" t="inlineStr">
+        <is>
+          <t>Precio lanzamiento (−20%)</t>
+        </is>
+      </c>
+      <c r="C88" s="33" t="inlineStr">
+        <is>
+          <t>US$ 600</t>
+        </is>
+      </c>
+      <c r="D88" s="30" t="n"/>
+      <c r="E88" s="31" t="n"/>
+    </row>
+    <row r="89" ht="20.5" customHeight="1">
+      <c r="B89" s="28" t="inlineStr">
+        <is>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C89" s="29" t="inlineStr">
+        <is>
+          <t>Por espacio individual · placa memorial incluida</t>
+        </is>
+      </c>
+      <c r="D89" s="30" t="n"/>
+      <c r="E89" s="31" t="n"/>
+    </row>
+    <row r="90" ht="35" customHeight="1">
+      <c r="B90" s="24" t="inlineStr">
+        <is>
+          <t>Condiciones</t>
+        </is>
+      </c>
+      <c r="C90" s="25" t="inlineStr">
+        <is>
+          <t>Pago único o financiado según política comercial vigente. Incluye la placa memorial en el monumento al término del plazo.</t>
+        </is>
+      </c>
+      <c r="D90" s="26" t="n"/>
+      <c r="E90" s="27" t="n"/>
+    </row>
+    <row r="91" ht="20" customHeight="1">
+      <c r="B91" s="21" t="inlineStr">
+        <is>
+          <t>PERFIL DEL COMPRADOR</t>
+        </is>
+      </c>
+      <c r="C91" s="22" t="n"/>
+      <c r="D91" s="22" t="n"/>
+      <c r="E91" s="23" t="n"/>
+    </row>
+    <row r="92" ht="35" customHeight="1">
+      <c r="B92" s="34" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C87" s="34" t="inlineStr">
+      <c r="C92" s="35" t="inlineStr">
         <is>
           <t>Personas con conciencia ambiental que desean que sus cenizas vuelvan a la tierra, con un lugar identificado para visitar.</t>
         </is>
       </c>
-      <c r="D87" s="35" t="n"/>
-      <c r="E87" s="36" t="n"/>
-    </row>
-    <row r="90" ht="30" customHeight="1">
-      <c r="B90" s="15" t="inlineStr">
+      <c r="D92" s="36" t="n"/>
+      <c r="E92" s="37" t="n"/>
+    </row>
+    <row r="95" ht="30" customHeight="1">
+      <c r="B95" s="15" t="inlineStr">
         <is>
           <t>JARDÍN DE MASCOTAS</t>
         </is>
       </c>
-      <c r="C90" s="16" t="n"/>
-      <c r="D90" s="16" t="n"/>
-      <c r="E90" s="17" t="n"/>
-    </row>
-    <row r="91" ht="20" customHeight="1">
-      <c r="B91" s="18" t="inlineStr">
+      <c r="C95" s="16" t="n"/>
+      <c r="D95" s="16" t="n"/>
+      <c r="E95" s="17" t="n"/>
+    </row>
+    <row r="96" ht="20" customHeight="1">
+      <c r="B96" s="18" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Mascotas  ·  Destino final · Inhumación ecológica</t>
         </is>
       </c>
-      <c r="C91" s="19" t="n"/>
-      <c r="D91" s="19" t="n"/>
-      <c r="E91" s="20" t="n"/>
-    </row>
-    <row r="92" ht="20" customHeight="1">
-      <c r="B92" s="21" t="inlineStr">
+      <c r="C96" s="19" t="n"/>
+      <c r="D96" s="19" t="n"/>
+      <c r="E96" s="20" t="n"/>
+    </row>
+    <row r="97" ht="20" customHeight="1">
+      <c r="B97" s="21" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C92" s="22" t="n"/>
-      <c r="D92" s="22" t="n"/>
-      <c r="E92" s="23" t="n"/>
-    </row>
-    <row r="93" ht="35" customHeight="1">
-      <c r="B93" s="24" t="inlineStr">
+      <c r="C97" s="22" t="n"/>
+      <c r="D97" s="22" t="n"/>
+      <c r="E97" s="23" t="n"/>
+    </row>
+    <row r="98" ht="35" customHeight="1">
+      <c r="B98" s="24" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C93" s="25" t="inlineStr">
+      <c r="C98" s="25" t="inlineStr">
         <is>
           <t>Jardín para inhumación ecológica de cenizas de mascotas: la urna biodegradable se entierra directamente en el suelo y se identifica con una placa de madera.</t>
-        </is>
-      </c>
-      <c r="D93" s="26" t="n"/>
-      <c r="E93" s="27" t="n"/>
-    </row>
-    <row r="94" ht="20.5" customHeight="1">
-      <c r="B94" s="28" t="inlineStr">
-        <is>
-          <t>Capacidad / Cobertura</t>
-        </is>
-      </c>
-      <c r="C94" s="29" t="inlineStr">
-        <is>
-          <t>Individual (una mascota por servicio).</t>
-        </is>
-      </c>
-      <c r="D94" s="30" t="n"/>
-      <c r="E94" s="31" t="n"/>
-    </row>
-    <row r="95" ht="20" customHeight="1">
-      <c r="B95" s="21" t="inlineStr">
-        <is>
-          <t>ESPECIFICACIONES TÉCNICAS</t>
-        </is>
-      </c>
-      <c r="C95" s="22" t="n"/>
-      <c r="D95" s="22" t="n"/>
-      <c r="E95" s="23" t="n"/>
-    </row>
-    <row r="96" ht="20.5" customHeight="1">
-      <c r="B96" s="24" t="inlineStr">
-        <is>
-          <t>Tipo de producto</t>
-        </is>
-      </c>
-      <c r="C96" s="25" t="inlineStr">
-        <is>
-          <t>Servicio de pago único</t>
-        </is>
-      </c>
-      <c r="D96" s="26" t="n"/>
-      <c r="E96" s="27" t="n"/>
-    </row>
-    <row r="97" ht="20.5" customHeight="1">
-      <c r="B97" s="28" t="inlineStr">
-        <is>
-          <t>Espacio por urna</t>
-        </is>
-      </c>
-      <c r="C97" s="29" t="inlineStr">
-        <is>
-          <t>15 × 20 cm o 15 × 30 cm, según el tamaño de la urna</t>
-        </is>
-      </c>
-      <c r="D97" s="30" t="n"/>
-      <c r="E97" s="31" t="n"/>
-    </row>
-    <row r="98" ht="20.5" customHeight="1">
-      <c r="B98" s="24" t="inlineStr">
-        <is>
-          <t>Urna</t>
-        </is>
-      </c>
-      <c r="C98" s="25" t="inlineStr">
-        <is>
-          <t>Biodegradable; se integra al suelo</t>
         </is>
       </c>
       <c r="D98" s="26" t="n"/>
@@ -2274,52 +2324,118 @@
     <row r="99" ht="20.5" customHeight="1">
       <c r="B99" s="28" t="inlineStr">
         <is>
-          <t>Identificación</t>
+          <t>Capacidad / Cobertura</t>
         </is>
       </c>
       <c r="C99" s="29" t="inlineStr">
         <is>
-          <t>Placa de madera de 20 cm</t>
+          <t>Individual (una mascota por servicio).</t>
         </is>
       </c>
       <c r="D99" s="30" t="n"/>
       <c r="E99" s="31" t="n"/>
     </row>
-    <row r="100" ht="20.5" customHeight="1">
-      <c r="B100" s="24" t="inlineStr">
+    <row r="100" ht="20" customHeight="1">
+      <c r="B100" s="21" t="inlineStr">
+        <is>
+          <t>ESPECIFICACIONES TÉCNICAS</t>
+        </is>
+      </c>
+      <c r="C100" s="22" t="n"/>
+      <c r="D100" s="22" t="n"/>
+      <c r="E100" s="23" t="n"/>
+    </row>
+    <row r="101" ht="20.5" customHeight="1">
+      <c r="B101" s="24" t="inlineStr">
+        <is>
+          <t>Tipo de producto</t>
+        </is>
+      </c>
+      <c r="C101" s="25" t="inlineStr">
+        <is>
+          <t>Servicio de pago único</t>
+        </is>
+      </c>
+      <c r="D101" s="26" t="n"/>
+      <c r="E101" s="27" t="n"/>
+    </row>
+    <row r="102" ht="20.5" customHeight="1">
+      <c r="B102" s="28" t="inlineStr">
+        <is>
+          <t>Espacio por urna</t>
+        </is>
+      </c>
+      <c r="C102" s="29" t="inlineStr">
+        <is>
+          <t>15 × 20 cm o 15 × 30 cm, según el tamaño de la urna</t>
+        </is>
+      </c>
+      <c r="D102" s="30" t="n"/>
+      <c r="E102" s="31" t="n"/>
+    </row>
+    <row r="103" ht="20.5" customHeight="1">
+      <c r="B103" s="24" t="inlineStr">
+        <is>
+          <t>Urna</t>
+        </is>
+      </c>
+      <c r="C103" s="25" t="inlineStr">
+        <is>
+          <t>Biodegradable; se integra al suelo</t>
+        </is>
+      </c>
+      <c r="D103" s="26" t="n"/>
+      <c r="E103" s="27" t="n"/>
+    </row>
+    <row r="104" ht="20.5" customHeight="1">
+      <c r="B104" s="28" t="inlineStr">
+        <is>
+          <t>Identificación</t>
+        </is>
+      </c>
+      <c r="C104" s="29" t="inlineStr">
+        <is>
+          <t>Placa de madera de 20 cm</t>
+        </is>
+      </c>
+      <c r="D104" s="30" t="n"/>
+      <c r="E104" s="31" t="n"/>
+    </row>
+    <row r="105" ht="20.5" customHeight="1">
+      <c r="B105" s="24" t="inlineStr">
         <is>
           <t>Permanencia</t>
         </is>
       </c>
-      <c r="C100" s="25" t="inlineStr">
+      <c r="C105" s="25" t="inlineStr">
         <is>
           <t>3 años; luego el espacio se reutiliza</t>
         </is>
       </c>
-      <c r="D100" s="26" t="n"/>
-      <c r="E100" s="27" t="n"/>
-    </row>
-    <row r="101" ht="20.5" customHeight="1">
-      <c r="B101" s="28" t="inlineStr">
+      <c r="D105" s="26" t="n"/>
+      <c r="E105" s="27" t="n"/>
+    </row>
+    <row r="106" ht="20.5" customHeight="1">
+      <c r="B106" s="28" t="inlineStr">
         <is>
           <t>Placa memorial</t>
         </is>
       </c>
-      <c r="C101" s="29" t="inlineStr">
+      <c r="C106" s="29" t="inlineStr">
         <is>
           <t>En el monumento al término del plazo; incluida en la opción de US$ 550</t>
         </is>
       </c>
-      <c r="D101" s="30" t="n"/>
-      <c r="E101" s="31" t="n"/>
-    </row>
-    <row r="102" ht="64" customHeight="1">
-      <c r="B102" s="24" t="inlineStr">
+      <c r="D106" s="30" t="n"/>
+      <c r="E106" s="31" t="n"/>
+    </row>
+    <row r="107" ht="64" customHeight="1">
+      <c r="B107" s="24" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C102" s="25" t="inlineStr">
+      <c r="C107" s="25" t="inlineStr">
         <is>
           <t>• Inhumación ecológica de la urna en el jardín
 • Placa de madera de 20 cm para identificación
@@ -2327,423 +2443,458 @@
 • Placa memorial en el monumento al término del plazo (opción US$ 550)</t>
         </is>
       </c>
-      <c r="D102" s="26" t="n"/>
-      <c r="E102" s="27" t="n"/>
-    </row>
-    <row r="103" ht="20" customHeight="1">
-      <c r="B103" s="21" t="inlineStr">
+      <c r="D107" s="26" t="n"/>
+      <c r="E107" s="27" t="n"/>
+    </row>
+    <row r="108" ht="20" customHeight="1">
+      <c r="B108" s="21" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C103" s="22" t="n"/>
-      <c r="D103" s="22" t="n"/>
-      <c r="E103" s="23" t="n"/>
-    </row>
-    <row r="104" ht="26.5" customHeight="1">
-      <c r="B104" s="24" t="inlineStr">
+      <c r="C108" s="22" t="n"/>
+      <c r="D108" s="22" t="n"/>
+      <c r="E108" s="23" t="n"/>
+    </row>
+    <row r="109" ht="26.5" customHeight="1">
+      <c r="B109" s="24" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C104" s="32" t="inlineStr">
+      <c r="C109" s="32" t="inlineStr">
         <is>
           <t>US$ 400 / US$ 550</t>
         </is>
       </c>
-      <c r="D104" s="26" t="n"/>
-      <c r="E104" s="27" t="n"/>
-    </row>
-    <row r="105" ht="20.5" customHeight="1">
-      <c r="B105" s="28" t="inlineStr">
+      <c r="D109" s="26" t="n"/>
+      <c r="E109" s="27" t="n"/>
+    </row>
+    <row r="110" ht="26.5" customHeight="1">
+      <c r="B110" s="28" t="inlineStr">
+        <is>
+          <t>Precio lanzamiento (−20%)</t>
+        </is>
+      </c>
+      <c r="C110" s="33" t="inlineStr">
+        <is>
+          <t>US$ 320 / US$ 440</t>
+        </is>
+      </c>
+      <c r="D110" s="30" t="n"/>
+      <c r="E110" s="31" t="n"/>
+    </row>
+    <row r="111" ht="20.5" customHeight="1">
+      <c r="B111" s="28" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C105" s="29" t="inlineStr">
+      <c r="C111" s="29" t="inlineStr">
         <is>
           <t>US$ 400 solo espacio · US$ 550 con placa memorial</t>
         </is>
       </c>
-      <c r="D105" s="30" t="n"/>
-      <c r="E105" s="31" t="n"/>
-    </row>
-    <row r="106" ht="35" customHeight="1">
-      <c r="B106" s="24" t="inlineStr">
+      <c r="D111" s="30" t="n"/>
+      <c r="E111" s="31" t="n"/>
+    </row>
+    <row r="112" ht="35" customHeight="1">
+      <c r="B112" s="24" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C106" s="25" t="inlineStr">
+      <c r="C112" s="25" t="inlineStr">
         <is>
           <t>Pago único; puede contratarse como adicional al plan funerario. La opción de US$ 550 incluye la placa memorial en el monumento al término del plazo.</t>
         </is>
       </c>
-      <c r="D106" s="26" t="n"/>
-      <c r="E106" s="27" t="n"/>
-    </row>
-    <row r="107" ht="20" customHeight="1">
-      <c r="B107" s="21" t="inlineStr">
+      <c r="D112" s="26" t="n"/>
+      <c r="E112" s="27" t="n"/>
+    </row>
+    <row r="113" ht="20" customHeight="1">
+      <c r="B113" s="21" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C107" s="22" t="n"/>
-      <c r="D107" s="22" t="n"/>
-      <c r="E107" s="23" t="n"/>
-    </row>
-    <row r="108" ht="20.5" customHeight="1">
-      <c r="B108" s="33" t="inlineStr">
+      <c r="C113" s="22" t="n"/>
+      <c r="D113" s="22" t="n"/>
+      <c r="E113" s="23" t="n"/>
+    </row>
+    <row r="114" ht="20.5" customHeight="1">
+      <c r="B114" s="34" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C108" s="34" t="inlineStr">
+      <c r="C114" s="35" t="inlineStr">
         <is>
           <t>Familias que consideran a su mascota parte del hogar y desean un cierre digno.</t>
         </is>
       </c>
-      <c r="D108" s="35" t="n"/>
-      <c r="E108" s="36" t="n"/>
-    </row>
-    <row r="111" ht="30" customHeight="1">
-      <c r="B111" s="15" t="inlineStr">
+      <c r="D114" s="36" t="n"/>
+      <c r="E114" s="37" t="n"/>
+    </row>
+    <row r="117" ht="30" customHeight="1">
+      <c r="B117" s="15" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · CEREMONIAL</t>
         </is>
       </c>
-      <c r="C111" s="16" t="n"/>
-      <c r="D111" s="16" t="n"/>
-      <c r="E111" s="17" t="n"/>
-    </row>
-    <row r="112" ht="20" customHeight="1">
-      <c r="B112" s="18" t="inlineStr">
+      <c r="C117" s="16" t="n"/>
+      <c r="D117" s="16" t="n"/>
+      <c r="E117" s="17" t="n"/>
+    </row>
+    <row r="118" ht="20" customHeight="1">
+      <c r="B118" s="18" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Jardín 3  ·  Destino final · Inhumación con ceremonia</t>
         </is>
       </c>
-      <c r="C112" s="19" t="n"/>
-      <c r="D112" s="19" t="n"/>
-      <c r="E112" s="20" t="n"/>
-    </row>
-    <row r="113" ht="24" customHeight="1">
-      <c r="B113" s="37" t="inlineStr">
+      <c r="C118" s="19" t="n"/>
+      <c r="D118" s="19" t="n"/>
+      <c r="E118" s="20" t="n"/>
+    </row>
+    <row r="119" ht="24" customHeight="1">
+      <c r="B119" s="38" t="inlineStr">
         <is>
           <t>★  PRÓXIMO LANZAMIENTO · se lanzará en otro momento</t>
         </is>
       </c>
-      <c r="C113" s="38" t="n"/>
-      <c r="D113" s="38" t="n"/>
-      <c r="E113" s="39" t="n"/>
-    </row>
-    <row r="114" ht="20" customHeight="1">
-      <c r="B114" s="21" t="inlineStr">
+      <c r="C119" s="39" t="n"/>
+      <c r="D119" s="39" t="n"/>
+      <c r="E119" s="40" t="n"/>
+    </row>
+    <row r="120" ht="20" customHeight="1">
+      <c r="B120" s="21" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C114" s="22" t="n"/>
-      <c r="D114" s="22" t="n"/>
-      <c r="E114" s="23" t="n"/>
-    </row>
-    <row r="115" ht="35" customHeight="1">
-      <c r="B115" s="24" t="inlineStr">
+      <c r="C120" s="22" t="n"/>
+      <c r="D120" s="22" t="n"/>
+      <c r="E120" s="23" t="n"/>
+    </row>
+    <row r="121" ht="35" customHeight="1">
+      <c r="B121" s="24" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C115" s="25" t="inlineStr">
+      <c r="C121" s="25" t="inlineStr">
         <is>
           <t>Jardín para inhumación de urnas de cenizas con ceremonia de agua, con fuentes como elemento central del rito de despedida.</t>
         </is>
       </c>
-      <c r="D115" s="26" t="n"/>
-      <c r="E115" s="27" t="n"/>
-    </row>
-    <row r="116" ht="20.5" customHeight="1">
-      <c r="B116" s="28" t="inlineStr">
+      <c r="D121" s="26" t="n"/>
+      <c r="E121" s="27" t="n"/>
+    </row>
+    <row r="122" ht="20.5" customHeight="1">
+      <c r="B122" s="28" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C116" s="29" t="inlineStr">
+      <c r="C122" s="29" t="inlineStr">
         <is>
           <t>A definir.</t>
         </is>
       </c>
-      <c r="D116" s="30" t="n"/>
-      <c r="E116" s="31" t="n"/>
-    </row>
-    <row r="117" ht="20" customHeight="1">
-      <c r="B117" s="21" t="inlineStr">
+      <c r="D122" s="30" t="n"/>
+      <c r="E122" s="31" t="n"/>
+    </row>
+    <row r="123" ht="20" customHeight="1">
+      <c r="B123" s="21" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C117" s="22" t="n"/>
-      <c r="D117" s="22" t="n"/>
-      <c r="E117" s="23" t="n"/>
-    </row>
-    <row r="118" ht="20.5" customHeight="1">
-      <c r="B118" s="24" t="inlineStr">
+      <c r="C123" s="22" t="n"/>
+      <c r="D123" s="22" t="n"/>
+      <c r="E123" s="23" t="n"/>
+    </row>
+    <row r="124" ht="20.5" customHeight="1">
+      <c r="B124" s="24" t="inlineStr">
         <is>
           <t>Ambiente</t>
         </is>
       </c>
-      <c r="C118" s="25" t="inlineStr">
+      <c r="C124" s="25" t="inlineStr">
         <is>
           <t>Jardín 3</t>
         </is>
       </c>
-      <c r="D118" s="26" t="n"/>
-      <c r="E118" s="27" t="n"/>
-    </row>
-    <row r="119" ht="20.5" customHeight="1">
-      <c r="B119" s="28" t="inlineStr">
+      <c r="D124" s="26" t="n"/>
+      <c r="E124" s="27" t="n"/>
+    </row>
+    <row r="125" ht="20.5" customHeight="1">
+      <c r="B125" s="28" t="inlineStr">
         <is>
           <t>Elemento central</t>
         </is>
       </c>
-      <c r="C119" s="29" t="inlineStr">
+      <c r="C125" s="29" t="inlineStr">
         <is>
           <t>Fuente de agua para la ceremonia</t>
         </is>
       </c>
-      <c r="D119" s="30" t="n"/>
-      <c r="E119" s="31" t="n"/>
-    </row>
-    <row r="120" ht="20.5" customHeight="1">
-      <c r="B120" s="24" t="inlineStr">
+      <c r="D125" s="30" t="n"/>
+      <c r="E125" s="31" t="n"/>
+    </row>
+    <row r="126" ht="20.5" customHeight="1">
+      <c r="B126" s="24" t="inlineStr">
         <is>
           <t>Entorno</t>
         </is>
       </c>
-      <c r="C120" s="25" t="inlineStr">
+      <c r="C126" s="25" t="inlineStr">
         <is>
           <t>Barrera visual que separa el jardín del crematorio</t>
         </is>
       </c>
-      <c r="D120" s="26" t="n"/>
-      <c r="E120" s="27" t="n"/>
-    </row>
-    <row r="121" ht="35" customHeight="1">
-      <c r="B121" s="28" t="inlineStr">
+      <c r="D126" s="26" t="n"/>
+      <c r="E126" s="27" t="n"/>
+    </row>
+    <row r="127" ht="35" customHeight="1">
+      <c r="B127" s="28" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C121" s="29" t="inlineStr">
+      <c r="C127" s="29" t="inlineStr">
         <is>
           <t>• Inhumación de urnas de cenizas
 • Ceremonia con agua en fuente</t>
         </is>
       </c>
-      <c r="D121" s="30" t="n"/>
-      <c r="E121" s="31" t="n"/>
-    </row>
-    <row r="122" ht="20" customHeight="1">
-      <c r="B122" s="21" t="inlineStr">
+      <c r="D127" s="30" t="n"/>
+      <c r="E127" s="31" t="n"/>
+    </row>
+    <row r="128" ht="20" customHeight="1">
+      <c r="B128" s="21" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C122" s="22" t="n"/>
-      <c r="D122" s="22" t="n"/>
-      <c r="E122" s="23" t="n"/>
-    </row>
-    <row r="123" ht="26.5" customHeight="1">
-      <c r="B123" s="24" t="inlineStr">
+      <c r="C128" s="22" t="n"/>
+      <c r="D128" s="22" t="n"/>
+      <c r="E128" s="23" t="n"/>
+    </row>
+    <row r="129" ht="26.5" customHeight="1">
+      <c r="B129" s="24" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C123" s="32" t="inlineStr">
+      <c r="C129" s="32" t="inlineStr">
         <is>
           <t>A definir</t>
         </is>
       </c>
-      <c r="D123" s="26" t="n"/>
-      <c r="E123" s="27" t="n"/>
-    </row>
-    <row r="124" ht="20.5" customHeight="1">
-      <c r="B124" s="28" t="inlineStr">
+      <c r="D129" s="26" t="n"/>
+      <c r="E129" s="27" t="n"/>
+    </row>
+    <row r="130" ht="26.5" customHeight="1">
+      <c r="B130" s="28" t="inlineStr">
+        <is>
+          <t>Precio lanzamiento (−20%)</t>
+        </is>
+      </c>
+      <c r="C130" s="33" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="D130" s="30" t="n"/>
+      <c r="E130" s="31" t="n"/>
+    </row>
+    <row r="131" ht="20.5" customHeight="1">
+      <c r="B131" s="28" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C124" s="29" t="inlineStr">
+      <c r="C131" s="29" t="inlineStr">
         <is>
           <t>Producto en definición</t>
         </is>
       </c>
-      <c r="D124" s="30" t="n"/>
-      <c r="E124" s="31" t="n"/>
-    </row>
-    <row r="125" ht="20.5" customHeight="1">
-      <c r="B125" s="24" t="inlineStr">
+      <c r="D131" s="30" t="n"/>
+      <c r="E131" s="31" t="n"/>
+    </row>
+    <row r="132" ht="20.5" customHeight="1">
+      <c r="B132" s="24" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C125" s="25" t="inlineStr">
+      <c r="C132" s="25" t="inlineStr">
         <is>
           <t>A definir.</t>
         </is>
       </c>
-      <c r="D125" s="26" t="n"/>
-      <c r="E125" s="27" t="n"/>
-    </row>
-    <row r="126" ht="20" customHeight="1">
-      <c r="B126" s="21" t="inlineStr">
+      <c r="D132" s="26" t="n"/>
+      <c r="E132" s="27" t="n"/>
+    </row>
+    <row r="133" ht="20" customHeight="1">
+      <c r="B133" s="21" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C126" s="22" t="n"/>
-      <c r="D126" s="22" t="n"/>
-      <c r="E126" s="23" t="n"/>
-    </row>
-    <row r="127" ht="35" customHeight="1">
-      <c r="B127" s="33" t="inlineStr">
+      <c r="C133" s="22" t="n"/>
+      <c r="D133" s="22" t="n"/>
+      <c r="E133" s="23" t="n"/>
+    </row>
+    <row r="134" ht="35" customHeight="1">
+      <c r="B134" s="34" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C127" s="34" t="inlineStr">
+      <c r="C134" s="35" t="inlineStr">
         <is>
           <t>Familias que valoran un rito de despedida simbólico y un entorno contemplativo.</t>
         </is>
       </c>
-      <c r="D127" s="35" t="n"/>
-      <c r="E127" s="36" t="n"/>
+      <c r="D134" s="36" t="n"/>
+      <c r="E134" s="37" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="116">
-    <mergeCell ref="C31:E31"/>
+  <mergeCells count="123">
+    <mergeCell ref="C44:E44"/>
     <mergeCell ref="C80:E80"/>
-    <mergeCell ref="B68:E68"/>
-    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="C129:E129"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="B123:E123"/>
+    <mergeCell ref="B76:E76"/>
+    <mergeCell ref="B45:E45"/>
     <mergeCell ref="C60:E60"/>
-    <mergeCell ref="C71:E71"/>
     <mergeCell ref="B113:E113"/>
-    <mergeCell ref="C123:E123"/>
     <mergeCell ref="B91:E91"/>
-    <mergeCell ref="B47:E47"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="B100:E100"/>
     <mergeCell ref="C7:E7"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B31:E31"/>
     <mergeCell ref="C57:E57"/>
-    <mergeCell ref="B21:E21"/>
     <mergeCell ref="B86:E86"/>
     <mergeCell ref="C18:E18"/>
-    <mergeCell ref="C49:E49"/>
     <mergeCell ref="C101:E101"/>
     <mergeCell ref="C77:E77"/>
     <mergeCell ref="C34:E34"/>
+    <mergeCell ref="C42:E42"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="C74:E74"/>
-    <mergeCell ref="B69:E69"/>
-    <mergeCell ref="B38:E38"/>
-    <mergeCell ref="B112:E112"/>
+    <mergeCell ref="C126:E126"/>
     <mergeCell ref="C20:E20"/>
+    <mergeCell ref="C103:E103"/>
     <mergeCell ref="C85:E85"/>
+    <mergeCell ref="C112:E112"/>
+    <mergeCell ref="B40:E40"/>
     <mergeCell ref="C99:E99"/>
-    <mergeCell ref="C94:E94"/>
-    <mergeCell ref="C118:E118"/>
+    <mergeCell ref="B49:E49"/>
     <mergeCell ref="C75:E75"/>
     <mergeCell ref="C84:E84"/>
-    <mergeCell ref="C22:E22"/>
     <mergeCell ref="C127:E127"/>
+    <mergeCell ref="C114:E114"/>
     <mergeCell ref="B51:E51"/>
+    <mergeCell ref="C59:E59"/>
+    <mergeCell ref="C130:E130"/>
     <mergeCell ref="C12:E12"/>
-    <mergeCell ref="B114:E114"/>
-    <mergeCell ref="B63:E63"/>
+    <mergeCell ref="C46:E46"/>
     <mergeCell ref="B26:E26"/>
+    <mergeCell ref="B50:E50"/>
     <mergeCell ref="C52:E52"/>
     <mergeCell ref="C61:E61"/>
     <mergeCell ref="C39:E39"/>
     <mergeCell ref="B16:E16"/>
-    <mergeCell ref="C70:E70"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="B90:E90"/>
     <mergeCell ref="C106:E106"/>
     <mergeCell ref="C32:E32"/>
+    <mergeCell ref="C38:E38"/>
     <mergeCell ref="C81:E81"/>
     <mergeCell ref="C125:E125"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="C13:E13"/>
+    <mergeCell ref="C131:E131"/>
     <mergeCell ref="C87:E87"/>
     <mergeCell ref="B117:E117"/>
     <mergeCell ref="C15:E15"/>
     <mergeCell ref="B67:E67"/>
     <mergeCell ref="C33:E33"/>
+    <mergeCell ref="C89:E89"/>
     <mergeCell ref="C104:E104"/>
-    <mergeCell ref="C116:E116"/>
+    <mergeCell ref="B119:E119"/>
     <mergeCell ref="C79:E79"/>
-    <mergeCell ref="C73:E73"/>
-    <mergeCell ref="B103:E103"/>
+    <mergeCell ref="C88:E88"/>
     <mergeCell ref="C35:E35"/>
+    <mergeCell ref="C63:E63"/>
     <mergeCell ref="C121:E121"/>
     <mergeCell ref="C10:E10"/>
-    <mergeCell ref="C50:E50"/>
+    <mergeCell ref="B118:E118"/>
     <mergeCell ref="C55:E55"/>
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="B95:E95"/>
-    <mergeCell ref="C115:E115"/>
     <mergeCell ref="C36:E36"/>
     <mergeCell ref="C11:E11"/>
+    <mergeCell ref="B97:E97"/>
+    <mergeCell ref="B54:E54"/>
     <mergeCell ref="B72:E72"/>
-    <mergeCell ref="B122:E122"/>
-    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="C122:E122"/>
+    <mergeCell ref="C109:E109"/>
+    <mergeCell ref="B71:E71"/>
     <mergeCell ref="C37:E37"/>
-    <mergeCell ref="C96:E96"/>
     <mergeCell ref="C78:E78"/>
+    <mergeCell ref="B120:E120"/>
     <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B42:E42"/>
-    <mergeCell ref="B107:E107"/>
-    <mergeCell ref="C62:E62"/>
+    <mergeCell ref="C92:E92"/>
+    <mergeCell ref="C30:E30"/>
     <mergeCell ref="C14:E14"/>
     <mergeCell ref="C98:E98"/>
+    <mergeCell ref="C107:E107"/>
     <mergeCell ref="C64:E64"/>
-    <mergeCell ref="C54:E54"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="B108:E108"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="C41:E41"/>
-    <mergeCell ref="C93:E93"/>
+    <mergeCell ref="C134:E134"/>
     <mergeCell ref="C124:E124"/>
-    <mergeCell ref="B92:E92"/>
-    <mergeCell ref="B30:E30"/>
     <mergeCell ref="C56:E56"/>
     <mergeCell ref="B5:E5"/>
+    <mergeCell ref="C90:E90"/>
     <mergeCell ref="C105:E105"/>
+    <mergeCell ref="B133:E133"/>
     <mergeCell ref="C43:E43"/>
-    <mergeCell ref="C76:E76"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="C120:E120"/>
-    <mergeCell ref="B126:E126"/>
-    <mergeCell ref="C119:E119"/>
+    <mergeCell ref="C132:E132"/>
+    <mergeCell ref="C110:E110"/>
     <mergeCell ref="C8:E8"/>
+    <mergeCell ref="B62:E62"/>
     <mergeCell ref="C17:E17"/>
-    <mergeCell ref="B59:E59"/>
-    <mergeCell ref="B46:E46"/>
+    <mergeCell ref="C82:E82"/>
+    <mergeCell ref="C66:E66"/>
     <mergeCell ref="C19:E19"/>
     <mergeCell ref="C53:E53"/>
+    <mergeCell ref="B96:E96"/>
     <mergeCell ref="C102:E102"/>
-    <mergeCell ref="B48:E48"/>
-    <mergeCell ref="B111:E111"/>
+    <mergeCell ref="C111:E111"/>
+    <mergeCell ref="C68:E68"/>
     <mergeCell ref="C83:E83"/>
-    <mergeCell ref="C108:E108"/>
     <mergeCell ref="C58:E58"/>
-    <mergeCell ref="B82:E82"/>
-    <mergeCell ref="C97:E97"/>
+    <mergeCell ref="B73:E73"/>
     <mergeCell ref="C29:E29"/>
-    <mergeCell ref="C100:E100"/>
+    <mergeCell ref="B128:E128"/>
+    <mergeCell ref="C65:E65"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
   <rowBreaks count="5" manualBreakCount="5">
-    <brk id="23" min="0" max="16383" man="1"/>
-    <brk id="44" min="0" max="16383" man="1"/>
-    <brk id="65" min="0" max="16383" man="1"/>
-    <brk id="88" min="0" max="16383" man="1"/>
-    <brk id="109" min="0" max="16383" man="1"/>
+    <brk id="24" min="0" max="16383" man="1"/>
+    <brk id="47" min="0" max="16383" man="1"/>
+    <brk id="69" min="0" max="16383" man="1"/>
+    <brk id="93" min="0" max="16383" man="1"/>
+    <brk id="115" min="0" max="16383" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
@@ -2776,49 +2927,49 @@
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="40" t="inlineStr">
+      <c r="A2" s="41" t="inlineStr">
         <is>
           <t>PROPUESTA · pendiente de validación con el Gerente Comercial</t>
         </is>
       </c>
     </row>
     <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="41" t="inlineStr">
+      <c r="A4" s="42" t="inlineStr">
         <is>
           <t>Producto</t>
         </is>
       </c>
-      <c r="B4" s="41" t="inlineStr">
+      <c r="B4" s="42" t="inlineStr">
         <is>
           <t>Precio (c/ IVA)</t>
         </is>
       </c>
-      <c r="C4" s="41" t="inlineStr">
+      <c r="C4" s="42" t="inlineStr">
         <is>
           <t>Precio sin IVA</t>
         </is>
       </c>
-      <c r="D4" s="41" t="inlineStr">
+      <c r="D4" s="42" t="inlineStr">
         <is>
           <t>% Comisión</t>
         </is>
       </c>
-      <c r="E4" s="41" t="inlineStr">
+      <c r="E4" s="42" t="inlineStr">
         <is>
           <t>Comisión por venta (sin IVA)</t>
         </is>
       </c>
-      <c r="F4" s="41" t="inlineStr">
+      <c r="F4" s="42" t="inlineStr">
         <is>
           <t>Momento de pago</t>
         </is>
       </c>
-      <c r="G4" s="41" t="inlineStr">
+      <c r="G4" s="42" t="inlineStr">
         <is>
           <t>Estorno</t>
         </is>
       </c>
-      <c r="H4" s="41" t="inlineStr">
+      <c r="H4" s="42" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -2830,17 +2981,17 @@
           <t>Solución Modular de Cremación</t>
         </is>
       </c>
-      <c r="B5" s="42" t="n">
+      <c r="B5" s="43" t="n">
         <v>1000</v>
       </c>
-      <c r="C5" s="42">
+      <c r="C5" s="43">
         <f>B5*100/113</f>
         <v/>
       </c>
-      <c r="D5" s="43" t="n">
+      <c r="D5" s="44" t="n">
         <v>0.08</v>
       </c>
-      <c r="E5" s="44">
+      <c r="E5" s="45">
         <f>C5*D5</f>
         <v/>
       </c>
@@ -2866,17 +3017,17 @@
           <t>Jardín de Cenizas · Individual</t>
         </is>
       </c>
-      <c r="B6" s="45" t="n">
+      <c r="B6" s="46" t="n">
         <v>600</v>
       </c>
-      <c r="C6" s="45">
+      <c r="C6" s="46">
         <f>B6*100/113</f>
         <v/>
       </c>
-      <c r="D6" s="46" t="n">
+      <c r="D6" s="47" t="n">
         <v>0.08</v>
       </c>
-      <c r="E6" s="47">
+      <c r="E6" s="48">
         <f>C6*D6</f>
         <v/>
       </c>
@@ -2898,17 +3049,17 @@
           <t>Jardín de Cenizas · Familiar</t>
         </is>
       </c>
-      <c r="B7" s="42" t="n">
+      <c r="B7" s="43" t="n">
         <v>2000</v>
       </c>
-      <c r="C7" s="42">
+      <c r="C7" s="43">
         <f>B7*100/113</f>
         <v/>
       </c>
-      <c r="D7" s="43" t="n">
+      <c r="D7" s="44" t="n">
         <v>0.08</v>
       </c>
-      <c r="E7" s="44">
+      <c r="E7" s="45">
         <f>C7*D7</f>
         <v/>
       </c>
@@ -2930,17 +3081,17 @@
           <t>Jardín de Cenizas · Ecológico</t>
         </is>
       </c>
-      <c r="B8" s="45" t="n">
+      <c r="B8" s="46" t="n">
         <v>750</v>
       </c>
-      <c r="C8" s="45">
+      <c r="C8" s="46">
         <f>B8*100/113</f>
         <v/>
       </c>
-      <c r="D8" s="46" t="n">
+      <c r="D8" s="47" t="n">
         <v>0.08</v>
       </c>
-      <c r="E8" s="47">
+      <c r="E8" s="48">
         <f>C8*D8</f>
         <v/>
       </c>
@@ -2962,17 +3113,17 @@
           <t>Jardín de Mascotas · solo espacio</t>
         </is>
       </c>
-      <c r="B9" s="42" t="n">
+      <c r="B9" s="43" t="n">
         <v>400</v>
       </c>
-      <c r="C9" s="42">
+      <c r="C9" s="43">
         <f>B9*100/113</f>
         <v/>
       </c>
-      <c r="D9" s="43" t="n">
+      <c r="D9" s="44" t="n">
         <v>0.08</v>
       </c>
-      <c r="E9" s="44">
+      <c r="E9" s="45">
         <f>C9*D9</f>
         <v/>
       </c>
@@ -2994,17 +3145,17 @@
           <t>Jardín de Mascotas · con placa memorial</t>
         </is>
       </c>
-      <c r="B10" s="45" t="n">
+      <c r="B10" s="46" t="n">
         <v>550</v>
       </c>
-      <c r="C10" s="45">
+      <c r="C10" s="46">
         <f>B10*100/113</f>
         <v/>
       </c>
-      <c r="D10" s="46" t="n">
+      <c r="D10" s="47" t="n">
         <v>0.08</v>
       </c>
-      <c r="E10" s="47">
+      <c r="E10" s="48">
         <f>C10*D10</f>
         <v/>
       </c>
@@ -3026,18 +3177,18 @@
           <t>Jardín de Cenizas · Ceremonial</t>
         </is>
       </c>
-      <c r="B11" s="42" t="inlineStr">
+      <c r="B11" s="43" t="inlineStr">
         <is>
           <t>A definir</t>
         </is>
       </c>
-      <c r="C11" s="42" t="inlineStr"/>
-      <c r="D11" s="43" t="inlineStr">
+      <c r="C11" s="43" t="inlineStr"/>
+      <c r="D11" s="44" t="inlineStr">
         <is>
           <t>A definir</t>
         </is>
       </c>
-      <c r="E11" s="44" t="inlineStr"/>
+      <c r="E11" s="45" t="inlineStr"/>
       <c r="F11" s="5" t="inlineStr">
         <is>
           <t>A definir</t>
@@ -3055,42 +3206,42 @@
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="48" t="inlineStr">
+      <c r="A13" s="49" t="inlineStr">
         <is>
           <t>REGLAS GENERALES</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="49" t="inlineStr">
+      <c r="A14" s="50" t="inlineStr">
         <is>
           <t>1. Base de cálculo: valor efectivamente cobrado al cliente, sin IVA (13%).</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="49" t="inlineStr">
-        <is>
-          <t>2. No generan comisión: cuotas de mantenimiento anual (US$ 15 / US$ 25).</t>
+      <c r="A15" s="50" t="inlineStr">
+        <is>
+          <t>2. No generan comisión: cuotas de mantenimiento anual (US$ 15 / US$ 24).</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="49" t="inlineStr">
+      <c r="A16" s="50" t="inlineStr">
         <is>
           <t>3. Bono de venta combinada: US$ 15 al vender la Solución Modular junto con cualquier jardín.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="49" t="inlineStr">
+      <c r="A17" s="50" t="inlineStr">
         <is>
           <t>4. Acelerador de campaña Día de los Muertos (opcional): +2 pp en Individual y Ecológico para ventas cerradas hasta el 30/11/2026.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="49" t="inlineStr">
+      <c r="A18" s="50" t="inlineStr">
         <is>
           <t>5. Estorno: la comisión se descuenta de los pagos siguientes al vendedor.</t>
         </is>

</xml_diff>

<commit_message>
Ficha técnica: Mascotas US$ 550 con cremación, cuota con intereses, sin referencia a nivel 1 HDLM
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111i7vn9WWo4QxCQbucWbrF
</commit_message>
<xml_diff>
--- a/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
+++ b/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
@@ -838,7 +838,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="107.5" customHeight="1">
+    <row r="5" ht="93" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Solución Modular de Cremación</t>
@@ -864,7 +864,7 @@
           <t>• Proceso completo de cremación individual
 • Urna cineraria de línea modular
 • Trámites legales básicos
-• Alquiler temporal de columbario por 1 año en nivel 1 HDLM
+• Alquiler temporal de columbario por 1 año
 • Integración al plan funerario base (actual o nuevo)</t>
         </is>
       </c>
@@ -887,7 +887,7 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Hasta 120 cuotas mensuales (aprox. US$ 8,50/mes).
+          <t>Hasta 120 cuotas mensuales con intereses (aprox. US$ 8,50/mes).
 Debe estar pagado en su totalidad para el uso de la cremación y el columbario</t>
         </is>
       </c>
@@ -1050,7 +1050,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="78.5" customHeight="1">
+    <row r="9" ht="64" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Jardín de Mascotas</t>
@@ -1076,7 +1076,7 @@
           <t>• Inhumación ecológica de la urna en el jardín
 • Placa de madera de 20 cm para identificación
 • Permanencia de 3 años
-• Placa memorial en el monumento al término del plazo (opción US$ 550)</t>
+• Cremación de la mascota (opción US$ 550)</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -1087,7 +1087,7 @@
       <c r="G9" s="6" t="inlineStr">
         <is>
           <t>US$ 400 / US$ 550
-(US$ 400 solo espacio · US$ 550 con placa memorial)</t>
+(US$ 400 solo espacio · US$ 550 con cremación)</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Pago único; puede contratarse como adicional al plan funerario. La opción de US$ 550 incluye la placa memorial en el monumento al término del plazo.</t>
+          <t>Pago único; puede contratarse como adicional al plan funerario. La opción de US$ 550 incluye la cremación de la mascota.</t>
         </is>
       </c>
     </row>
@@ -1344,7 +1344,7 @@
           <t>• Proceso completo de cremación individual
 • Urna cineraria de línea modular
 • Trámites legales básicos
-• Alquiler temporal de columbario por 1 año en nivel 1 HDLM
+• Alquiler temporal de columbario por 1 año
 • Integración al plan funerario base (actual o nuevo)</t>
         </is>
       </c>
@@ -1411,7 +1411,7 @@
       </c>
       <c r="C20" s="25" t="inlineStr">
         <is>
-          <t>Hasta 120 cuotas mensuales (aprox. US$ 8,50/mes).
+          <t>Hasta 120 cuotas mensuales con intereses (aprox. US$ 8,50/mes).
 Debe estar pagado en su totalidad para el uso de la cremación y el columbario</t>
         </is>
       </c>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="C21" s="29" t="inlineStr">
         <is>
-          <t>US$ 8,33/mes sin intereses (120 cuotas)</t>
+          <t>US$ 8,50/mes con intereses (120 cuotas)</t>
         </is>
       </c>
       <c r="D21" s="30" t="n"/>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="C106" s="29" t="inlineStr">
         <is>
-          <t>En el monumento al término del plazo; incluida en la opción de US$ 550</t>
+          <t>En el monumento al término del plazo (valor a confirmar)</t>
         </is>
       </c>
       <c r="D106" s="30" t="n"/>
@@ -2440,7 +2440,7 @@
           <t>• Inhumación ecológica de la urna en el jardín
 • Placa de madera de 20 cm para identificación
 • Permanencia de 3 años
-• Placa memorial en el monumento al término del plazo (opción US$ 550)</t>
+• Cremación de la mascota (opción US$ 550)</t>
         </is>
       </c>
       <c r="D107" s="26" t="n"/>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="C111" s="29" t="inlineStr">
         <is>
-          <t>US$ 400 solo espacio · US$ 550 con placa memorial</t>
+          <t>US$ 400 solo espacio · US$ 550 con cremación</t>
         </is>
       </c>
       <c r="D111" s="30" t="n"/>
@@ -2506,7 +2506,7 @@
       </c>
       <c r="C112" s="25" t="inlineStr">
         <is>
-          <t>Pago único; puede contratarse como adicional al plan funerario. La opción de US$ 550 incluye la placa memorial en el monumento al término del plazo.</t>
+          <t>Pago único; puede contratarse como adicional al plan funerario. La opción de US$ 550 incluye la cremación de la mascota.</t>
         </is>
       </c>
       <c r="D112" s="26" t="n"/>
@@ -3142,7 +3142,7 @@
     <row r="10" ht="44" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Jardín de Mascotas · con placa memorial</t>
+          <t>Jardín de Mascotas · jardín + cremación</t>
         </is>
       </c>
       <c r="B10" s="46" t="n">

</xml_diff>

<commit_message>
Ficha técnica: urna de mascotas solo con cremación, sin HDLM en columbario y PDF para cliente
- Mascotas: urna biodegradable incluida solo en la opción US$ 550; con solo espacio se adquiere aparte
- Modular: quita la referencia a Hogar de Las Memorias en Columbario
- CSS de impresión ajustado para una ficha por página A4
- Agrega salida/Ficha_Tecnica_Cremacion_Vangrupo.pdf

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111i7vn9WWo4QxCQbucWbrF
</commit_message>
<xml_diff>
--- a/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
+++ b/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
@@ -1050,7 +1050,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="64" customHeight="1">
+    <row r="9" ht="107.5" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Jardín de Mascotas</t>
@@ -1076,7 +1076,7 @@
           <t>• Inhumación ecológica de la urna en el jardín
 • Placa de madera de 20 cm para identificación
 • Permanencia de 3 años
-• Cremación de la mascota (opción US$ 550)</t>
+• Cremación de la mascota y urna biodegradable (opción US$ 550)</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -1087,7 +1087,7 @@
       <c r="G9" s="6" t="inlineStr">
         <is>
           <t>US$ 400 / US$ 550
-(US$ 400 solo espacio · US$ 550 con cremación)</t>
+(US$ 400 solo espacio (urna aparte) · US$ 550 con cremación y urna)</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Pago único; puede contratarse como adicional al plan funerario. La opción de US$ 550 incluye la cremación de la mascota.</t>
+          <t>Pago único; puede contratarse como adicional al plan funerario. La opción de US$ 550 incluye la cremación de la mascota y la urna biodegradable; en la opción de US$ 400 (solo espacio) la urna biodegradable se adquiere por separado.</t>
         </is>
       </c>
     </row>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
-          <t>Alquiler temporal · 12 meses incluido (Hogar de Las Memorias)</t>
+          <t>Alquiler temporal · 12 meses incluido</t>
         </is>
       </c>
       <c r="D14" s="26" t="n"/>
@@ -2373,7 +2373,7 @@
       <c r="D102" s="30" t="n"/>
       <c r="E102" s="31" t="n"/>
     </row>
-    <row r="103" ht="20.5" customHeight="1">
+    <row r="103" ht="35" customHeight="1">
       <c r="B103" s="24" t="inlineStr">
         <is>
           <t>Urna</t>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="C103" s="25" t="inlineStr">
         <is>
-          <t>Biodegradable; se integra al suelo</t>
+          <t>Biodegradable; se integra al suelo. Incluida solo en la opción con cremación (US$ 550); con solo espacio (US$ 400) se adquiere por separado</t>
         </is>
       </c>
       <c r="D103" s="26" t="n"/>
@@ -2440,7 +2440,7 @@
           <t>• Inhumación ecológica de la urna en el jardín
 • Placa de madera de 20 cm para identificación
 • Permanencia de 3 años
-• Cremación de la mascota (opción US$ 550)</t>
+• Cremación de la mascota y urna biodegradable (opción US$ 550)</t>
         </is>
       </c>
       <c r="D107" s="26" t="n"/>
@@ -2492,13 +2492,13 @@
       </c>
       <c r="C111" s="29" t="inlineStr">
         <is>
-          <t>US$ 400 solo espacio · US$ 550 con cremación</t>
+          <t>US$ 400 solo espacio (urna aparte) · US$ 550 con cremación y urna</t>
         </is>
       </c>
       <c r="D111" s="30" t="n"/>
       <c r="E111" s="31" t="n"/>
     </row>
-    <row r="112" ht="35" customHeight="1">
+    <row r="112" ht="49.5" customHeight="1">
       <c r="B112" s="24" t="inlineStr">
         <is>
           <t>Condiciones</t>
@@ -2506,7 +2506,7 @@
       </c>
       <c r="C112" s="25" t="inlineStr">
         <is>
-          <t>Pago único; puede contratarse como adicional al plan funerario. La opción de US$ 550 incluye la cremación de la mascota.</t>
+          <t>Pago único; puede contratarse como adicional al plan funerario. La opción de US$ 550 incluye la cremación de la mascota y la urna biodegradable; en la opción de US$ 400 (solo espacio) la urna biodegradable se adquiere por separado.</t>
         </is>
       </c>
       <c r="D112" s="26" t="n"/>

</xml_diff>

<commit_message>
Ficha técnica: placa memorial de mascotas incluida en el precio
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111i7vn9WWo4QxCQbucWbrF
</commit_message>
<xml_diff>
--- a/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
+++ b/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
@@ -1075,7 +1075,7 @@
         <is>
           <t>• Inhumación ecológica de la urna en el jardín
 • Placa de madera de 20 cm para identificación
-• Permanencia de 3 años
+• Permanencia de 3 años; luego, placa memorial en el monumento (incluida)
 • Cremación de la mascota y urna biodegradable (opción US$ 550)</t>
         </is>
       </c>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="C106" s="29" t="inlineStr">
         <is>
-          <t>En el monumento al término del plazo (valor a confirmar)</t>
+          <t>Incluida en el precio; en el monumento al término del plazo</t>
         </is>
       </c>
       <c r="D106" s="30" t="n"/>
@@ -2439,7 +2439,7 @@
         <is>
           <t>• Inhumación ecológica de la urna en el jardín
 • Placa de madera de 20 cm para identificación
-• Permanencia de 3 años
+• Permanencia de 3 años; luego, placa memorial en el monumento (incluida)
 • Cremación de la mascota y urna biodegradable (opción US$ 550)</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Ficha técnica: columbario de la Solución Modular en Hogar de las Memorias
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111i7vn9WWo4QxCQbucWbrF
</commit_message>
<xml_diff>
--- a/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
+++ b/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
@@ -838,7 +838,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="93" customHeight="1">
+    <row r="5" ht="107.5" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Solución Modular de Cremación</t>
@@ -864,7 +864,7 @@
           <t>• Proceso completo de cremación individual
 • Urna cineraria de línea modular
 • Trámites legales básicos
-• Alquiler temporal de columbario por 1 año
+• Alquiler temporal de columbario por 1 año en Hogar de las Memorias
 • Integración al plan funerario base (actual o nuevo)</t>
         </is>
       </c>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
-          <t>Alquiler temporal · 12 meses incluido</t>
+          <t>Alquiler temporal · 12 meses incluido en Hogar de las Memorias</t>
         </is>
       </c>
       <c r="D14" s="26" t="n"/>
@@ -1344,7 +1344,7 @@
           <t>• Proceso completo de cremación individual
 • Urna cineraria de línea modular
 • Trámites legales básicos
-• Alquiler temporal de columbario por 1 año
+• Alquiler temporal de columbario por 1 año en Hogar de las Memorias
 • Integración al plan funerario base (actual o nuevo)</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Quita los valores de cuota mensual: pago en hasta 120 meses con intereses
- Ficha técnica: sin cuota aprox. en condiciones, precio de lanzamiento ni cuota referencial
- Comisiones: quita el valor estimado de las 10 primeras cuotas
- Playbook: speech, objeción, tabla de precios y herramientas sin valor de cuota

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111i7vn9WWo4QxCQbucWbrF
</commit_message>
<xml_diff>
--- a/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
+++ b/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
@@ -14,7 +14,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tabla Gral. - Visión Comercial'!$A$4:$I$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Tabla Gral. - Visión Comercial'!$4:$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Ficha Técnica Consolidada'!$A$1:$F$135</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Ficha Técnica Consolidada'!$A$1:$F$134</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -881,13 +881,13 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>US$ 800 · 120 cuotas de aprox. US$ 6,80/mes
+          <t>US$ 800
 (descuento especial de lanzamiento)</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Hasta 120 cuotas mensuales con intereses (aprox. US$ 8,50/mes).
+          <t>Pago en hasta 120 meses, con intereses.
 Debe estar pagado en su totalidad para el uso de la cremación y el columbario</t>
         </is>
       </c>
@@ -1170,7 +1170,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:E134"/>
+  <dimension ref="B1:E133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C18" s="33" t="inlineStr">
         <is>
-          <t>US$ 800 · 120 cuotas de aprox. US$ 6,80/mes</t>
+          <t>US$ 800</t>
         </is>
       </c>
       <c r="D18" s="30" t="n"/>
@@ -1411,224 +1411,210 @@
       </c>
       <c r="C20" s="25" t="inlineStr">
         <is>
-          <t>Hasta 120 cuotas mensuales con intereses (aprox. US$ 8,50/mes).
+          <t>Pago en hasta 120 meses, con intereses.
 Debe estar pagado en su totalidad para el uso de la cremación y el columbario</t>
         </is>
       </c>
       <c r="D20" s="26" t="n"/>
       <c r="E20" s="27" t="n"/>
     </row>
-    <row r="21" ht="20.5" customHeight="1">
-      <c r="B21" s="28" t="inlineStr">
-        <is>
-          <t>Cuota referencial</t>
-        </is>
-      </c>
-      <c r="C21" s="29" t="inlineStr">
-        <is>
-          <t>US$ 8,50/mes con intereses (120 cuotas)</t>
-        </is>
-      </c>
-      <c r="D21" s="30" t="n"/>
-      <c r="E21" s="31" t="n"/>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="B22" s="21" t="inlineStr">
+    <row r="21" ht="20" customHeight="1">
+      <c r="B21" s="21" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C22" s="22" t="n"/>
-      <c r="D22" s="22" t="n"/>
-      <c r="E22" s="23" t="n"/>
-    </row>
-    <row r="23" ht="35" customHeight="1">
-      <c r="B23" s="34" t="inlineStr">
+      <c r="C21" s="22" t="n"/>
+      <c r="D21" s="22" t="n"/>
+      <c r="E21" s="23" t="n"/>
+    </row>
+    <row r="22" ht="35" customHeight="1">
+      <c r="B22" s="34" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C23" s="35" t="inlineStr">
+      <c r="C22" s="35" t="inlineStr">
         <is>
           <t>Afiliados actuales y nuevos que desean incorporar la cremación a su plan con una cuota mensual mínima.</t>
         </is>
       </c>
-      <c r="D23" s="36" t="n"/>
-      <c r="E23" s="37" t="n"/>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="B26" s="15" t="inlineStr">
+      <c r="D22" s="36" t="n"/>
+      <c r="E22" s="37" t="n"/>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="B25" s="15" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · INDIVIDUAL</t>
         </is>
       </c>
-      <c r="C26" s="16" t="n"/>
-      <c r="D26" s="16" t="n"/>
-      <c r="E26" s="17" t="n"/>
+      <c r="C25" s="16" t="n"/>
+      <c r="D25" s="16" t="n"/>
+      <c r="E25" s="17" t="n"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>Jardines de la Memoria · Jardín 1  ·  Destino final · Inhumación individual</t>
+        </is>
+      </c>
+      <c r="C26" s="19" t="n"/>
+      <c r="D26" s="19" t="n"/>
+      <c r="E26" s="20" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="B27" s="18" t="inlineStr">
-        <is>
-          <t>Jardines de la Memoria · Jardín 1  ·  Destino final · Inhumación individual</t>
-        </is>
-      </c>
-      <c r="C27" s="19" t="n"/>
-      <c r="D27" s="19" t="n"/>
-      <c r="E27" s="20" t="n"/>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="B28" s="21" t="inlineStr">
+      <c r="B27" s="21" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C28" s="22" t="n"/>
-      <c r="D28" s="22" t="n"/>
-      <c r="E28" s="23" t="n"/>
-    </row>
-    <row r="29" ht="49.5" customHeight="1">
-      <c r="B29" s="24" t="inlineStr">
+      <c r="C27" s="22" t="n"/>
+      <c r="D27" s="22" t="n"/>
+      <c r="E27" s="23" t="n"/>
+    </row>
+    <row r="28" ht="49.5" customHeight="1">
+      <c r="B28" s="24" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C29" s="25" t="inlineStr">
+      <c r="C28" s="25" t="inlineStr">
         <is>
           <t>Inhumación de la urna de cenizas en un contenedor enterrado con tapa de granito grabada, en un jardín de plantas de sombra: un lugar físico de homenaje por 30 años desde la primera inhumación, renovable.</t>
         </is>
       </c>
-      <c r="D29" s="26" t="n"/>
-      <c r="E29" s="27" t="n"/>
-    </row>
-    <row r="30" ht="20.5" customHeight="1">
-      <c r="B30" s="28" t="inlineStr">
+      <c r="D28" s="26" t="n"/>
+      <c r="E28" s="27" t="n"/>
+    </row>
+    <row r="29" ht="20.5" customHeight="1">
+      <c r="B29" s="28" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C30" s="29" t="inlineStr">
+      <c r="C29" s="29" t="inlineStr">
         <is>
           <t>Individual (1 urna).</t>
         </is>
       </c>
-      <c r="D30" s="30" t="n"/>
-      <c r="E30" s="31" t="n"/>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="B31" s="21" t="inlineStr">
+      <c r="D29" s="30" t="n"/>
+      <c r="E29" s="31" t="n"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="B30" s="21" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C31" s="22" t="n"/>
-      <c r="D31" s="22" t="n"/>
-      <c r="E31" s="23" t="n"/>
+      <c r="C30" s="22" t="n"/>
+      <c r="D30" s="22" t="n"/>
+      <c r="E30" s="23" t="n"/>
+    </row>
+    <row r="31" ht="20.5" customHeight="1">
+      <c r="B31" s="24" t="inlineStr">
+        <is>
+          <t>Ambiente</t>
+        </is>
+      </c>
+      <c r="C31" s="25" t="inlineStr">
+        <is>
+          <t>Jardín 1</t>
+        </is>
+      </c>
+      <c r="D31" s="26" t="n"/>
+      <c r="E31" s="27" t="n"/>
     </row>
     <row r="32" ht="20.5" customHeight="1">
-      <c r="B32" s="24" t="inlineStr">
-        <is>
-          <t>Ambiente</t>
-        </is>
-      </c>
-      <c r="C32" s="25" t="inlineStr">
-        <is>
-          <t>Jardín 1</t>
-        </is>
-      </c>
-      <c r="D32" s="26" t="n"/>
-      <c r="E32" s="27" t="n"/>
+      <c r="B32" s="28" t="inlineStr">
+        <is>
+          <t>Contenedor</t>
+        </is>
+      </c>
+      <c r="C32" s="29" t="inlineStr">
+        <is>
+          <t>Ø 32 cm × 40 cm de altura; enterrado dejando 20 cm a la vista</t>
+        </is>
+      </c>
+      <c r="D32" s="30" t="n"/>
+      <c r="E32" s="31" t="n"/>
     </row>
     <row r="33" ht="20.5" customHeight="1">
-      <c r="B33" s="28" t="inlineStr">
-        <is>
-          <t>Contenedor</t>
-        </is>
-      </c>
-      <c r="C33" s="29" t="inlineStr">
-        <is>
-          <t>Ø 32 cm × 40 cm de altura; enterrado dejando 20 cm a la vista</t>
-        </is>
-      </c>
-      <c r="D33" s="30" t="n"/>
-      <c r="E33" s="31" t="n"/>
+      <c r="B33" s="24" t="inlineStr">
+        <is>
+          <t>Identificación</t>
+        </is>
+      </c>
+      <c r="C33" s="25" t="inlineStr">
+        <is>
+          <t>Tapa de granito con la información del difunto</t>
+        </is>
+      </c>
+      <c r="D33" s="26" t="n"/>
+      <c r="E33" s="27" t="n"/>
     </row>
     <row r="34" ht="20.5" customHeight="1">
-      <c r="B34" s="24" t="inlineStr">
-        <is>
-          <t>Identificación</t>
-        </is>
-      </c>
-      <c r="C34" s="25" t="inlineStr">
-        <is>
-          <t>Tapa de granito con la información del difunto</t>
-        </is>
-      </c>
-      <c r="D34" s="26" t="n"/>
-      <c r="E34" s="27" t="n"/>
+      <c r="B34" s="28" t="inlineStr">
+        <is>
+          <t>Paisajismo</t>
+        </is>
+      </c>
+      <c r="C34" s="29" t="inlineStr">
+        <is>
+          <t>Plantas de sombra de diferentes alturas y texturas</t>
+        </is>
+      </c>
+      <c r="D34" s="30" t="n"/>
+      <c r="E34" s="31" t="n"/>
     </row>
     <row r="35" ht="20.5" customHeight="1">
-      <c r="B35" s="28" t="inlineStr">
-        <is>
-          <t>Paisajismo</t>
-        </is>
-      </c>
-      <c r="C35" s="29" t="inlineStr">
-        <is>
-          <t>Plantas de sombra de diferentes alturas y texturas</t>
-        </is>
-      </c>
-      <c r="D35" s="30" t="n"/>
-      <c r="E35" s="31" t="n"/>
+      <c r="B35" s="24" t="inlineStr">
+        <is>
+          <t>Acceso</t>
+        </is>
+      </c>
+      <c r="C35" s="25" t="inlineStr">
+        <is>
+          <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
+        </is>
+      </c>
+      <c r="D35" s="26" t="n"/>
+      <c r="E35" s="27" t="n"/>
     </row>
     <row r="36" ht="20.5" customHeight="1">
-      <c r="B36" s="24" t="inlineStr">
-        <is>
-          <t>Acceso</t>
-        </is>
-      </c>
-      <c r="C36" s="25" t="inlineStr">
-        <is>
-          <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
-        </is>
-      </c>
-      <c r="D36" s="26" t="n"/>
-      <c r="E36" s="27" t="n"/>
+      <c r="B36" s="28" t="inlineStr">
+        <is>
+          <t>Permanencia</t>
+        </is>
+      </c>
+      <c r="C36" s="29" t="inlineStr">
+        <is>
+          <t>30 años desde la primera inhumación, renovable por igual período</t>
+        </is>
+      </c>
+      <c r="D36" s="30" t="n"/>
+      <c r="E36" s="31" t="n"/>
     </row>
     <row r="37" ht="20.5" customHeight="1">
-      <c r="B37" s="28" t="inlineStr">
-        <is>
-          <t>Permanencia</t>
-        </is>
-      </c>
-      <c r="C37" s="29" t="inlineStr">
-        <is>
-          <t>30 años desde la primera inhumación, renovable por igual período</t>
-        </is>
-      </c>
-      <c r="D37" s="30" t="n"/>
-      <c r="E37" s="31" t="n"/>
-    </row>
-    <row r="38" ht="20.5" customHeight="1">
-      <c r="B38" s="24" t="inlineStr">
+      <c r="B37" s="24" t="inlineStr">
         <is>
           <t>Mantenimiento</t>
         </is>
       </c>
-      <c r="C38" s="25" t="inlineStr">
+      <c r="C37" s="25" t="inlineStr">
         <is>
           <t>US$ 15 anual</t>
         </is>
       </c>
-      <c r="D38" s="26" t="n"/>
-      <c r="E38" s="27" t="n"/>
-    </row>
-    <row r="39" ht="93" customHeight="1">
-      <c r="B39" s="28" t="inlineStr">
+      <c r="D37" s="26" t="n"/>
+      <c r="E37" s="27" t="n"/>
+    </row>
+    <row r="38" ht="93" customHeight="1">
+      <c r="B38" s="28" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C39" s="29" t="inlineStr">
+      <c r="C38" s="29" t="inlineStr">
         <is>
           <t>• Inhumación de la urna en contenedor individual
 • Tapa de granito con los datos del difunto
@@ -1637,258 +1623,258 @@
 • Permanencia de 30 años desde la primera inhumación, renovable por igual período</t>
         </is>
       </c>
-      <c r="D39" s="30" t="n"/>
-      <c r="E39" s="31" t="n"/>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="B40" s="21" t="inlineStr">
+      <c r="D38" s="30" t="n"/>
+      <c r="E38" s="31" t="n"/>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="B39" s="21" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C40" s="22" t="n"/>
-      <c r="D40" s="22" t="n"/>
-      <c r="E40" s="23" t="n"/>
+      <c r="C39" s="22" t="n"/>
+      <c r="D39" s="22" t="n"/>
+      <c r="E39" s="23" t="n"/>
+    </row>
+    <row r="40" ht="26.5" customHeight="1">
+      <c r="B40" s="24" t="inlineStr">
+        <is>
+          <t>Precio sugerido</t>
+        </is>
+      </c>
+      <c r="C40" s="32" t="inlineStr">
+        <is>
+          <t>US$ 600</t>
+        </is>
+      </c>
+      <c r="D40" s="26" t="n"/>
+      <c r="E40" s="27" t="n"/>
     </row>
     <row r="41" ht="26.5" customHeight="1">
-      <c r="B41" s="24" t="inlineStr">
-        <is>
-          <t>Precio sugerido</t>
-        </is>
-      </c>
-      <c r="C41" s="32" t="inlineStr">
-        <is>
-          <t>US$ 600</t>
-        </is>
-      </c>
-      <c r="D41" s="26" t="n"/>
-      <c r="E41" s="27" t="n"/>
-    </row>
-    <row r="42" ht="26.5" customHeight="1">
+      <c r="B41" s="28" t="inlineStr">
+        <is>
+          <t>Precio lanzamiento (−20%)</t>
+        </is>
+      </c>
+      <c r="C41" s="33" t="inlineStr">
+        <is>
+          <t>US$ 480</t>
+        </is>
+      </c>
+      <c r="D41" s="30" t="n"/>
+      <c r="E41" s="31" t="n"/>
+    </row>
+    <row r="42" ht="20.5" customHeight="1">
       <c r="B42" s="28" t="inlineStr">
         <is>
-          <t>Precio lanzamiento (−20%)</t>
-        </is>
-      </c>
-      <c r="C42" s="33" t="inlineStr">
-        <is>
-          <t>US$ 480</t>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C42" s="29" t="inlineStr">
+        <is>
+          <t>Por espacio individual · mantenimiento US$ 15/año</t>
         </is>
       </c>
       <c r="D42" s="30" t="n"/>
       <c r="E42" s="31" t="n"/>
     </row>
-    <row r="43" ht="20.5" customHeight="1">
-      <c r="B43" s="28" t="inlineStr">
-        <is>
-          <t>Base de precio</t>
-        </is>
-      </c>
-      <c r="C43" s="29" t="inlineStr">
-        <is>
-          <t>Por espacio individual · mantenimiento US$ 15/año</t>
-        </is>
-      </c>
-      <c r="D43" s="30" t="n"/>
-      <c r="E43" s="31" t="n"/>
-    </row>
-    <row r="44" ht="35" customHeight="1">
-      <c r="B44" s="24" t="inlineStr">
+    <row r="43" ht="35" customHeight="1">
+      <c r="B43" s="24" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C44" s="25" t="inlineStr">
+      <c r="C43" s="25" t="inlineStr">
         <is>
           <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 15 anual.</t>
         </is>
       </c>
-      <c r="D44" s="26" t="n"/>
-      <c r="E44" s="27" t="n"/>
-    </row>
-    <row r="45" ht="20" customHeight="1">
-      <c r="B45" s="21" t="inlineStr">
+      <c r="D43" s="26" t="n"/>
+      <c r="E43" s="27" t="n"/>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="B44" s="21" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C45" s="22" t="n"/>
-      <c r="D45" s="22" t="n"/>
-      <c r="E45" s="23" t="n"/>
-    </row>
-    <row r="46" ht="35" customHeight="1">
-      <c r="B46" s="34" t="inlineStr">
+      <c r="C44" s="22" t="n"/>
+      <c r="D44" s="22" t="n"/>
+      <c r="E44" s="23" t="n"/>
+    </row>
+    <row r="45" ht="35" customHeight="1">
+      <c r="B45" s="34" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C46" s="35" t="inlineStr">
+      <c r="C45" s="35" t="inlineStr">
         <is>
           <t>Familias que desean un lugar propio para visitar y rendir homenaje, con una inversión moderada.</t>
         </is>
       </c>
-      <c r="D46" s="36" t="n"/>
-      <c r="E46" s="37" t="n"/>
-    </row>
-    <row r="49" ht="30" customHeight="1">
-      <c r="B49" s="15" t="inlineStr">
+      <c r="D45" s="36" t="n"/>
+      <c r="E45" s="37" t="n"/>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="B48" s="15" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · FAMILIAR</t>
         </is>
       </c>
-      <c r="C49" s="16" t="n"/>
-      <c r="D49" s="16" t="n"/>
-      <c r="E49" s="17" t="n"/>
+      <c r="C48" s="16" t="n"/>
+      <c r="D48" s="16" t="n"/>
+      <c r="E48" s="17" t="n"/>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="B49" s="18" t="inlineStr">
+        <is>
+          <t>Jardines de la Memoria · Jardín 1  ·  Destino final · Inhumación familiar</t>
+        </is>
+      </c>
+      <c r="C49" s="19" t="n"/>
+      <c r="D49" s="19" t="n"/>
+      <c r="E49" s="20" t="n"/>
     </row>
     <row r="50" ht="20" customHeight="1">
-      <c r="B50" s="18" t="inlineStr">
-        <is>
-          <t>Jardines de la Memoria · Jardín 1  ·  Destino final · Inhumación familiar</t>
-        </is>
-      </c>
-      <c r="C50" s="19" t="n"/>
-      <c r="D50" s="19" t="n"/>
-      <c r="E50" s="20" t="n"/>
-    </row>
-    <row r="51" ht="20" customHeight="1">
-      <c r="B51" s="21" t="inlineStr">
+      <c r="B50" s="21" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C51" s="22" t="n"/>
-      <c r="D51" s="22" t="n"/>
-      <c r="E51" s="23" t="n"/>
-    </row>
-    <row r="52" ht="49.5" customHeight="1">
-      <c r="B52" s="24" t="inlineStr">
+      <c r="C50" s="22" t="n"/>
+      <c r="D50" s="22" t="n"/>
+      <c r="E50" s="23" t="n"/>
+    </row>
+    <row r="51" ht="49.5" customHeight="1">
+      <c r="B51" s="24" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C52" s="25" t="inlineStr">
+      <c r="C51" s="25" t="inlineStr">
         <is>
           <t>Parcela familiar en el Jardín 1 con cuatro contenedores agrupados, cada uno con tapa de granito grabada, con permanencia de 30 años desde la primera inhumación, renovable por igual período.</t>
         </is>
       </c>
-      <c r="D52" s="26" t="n"/>
-      <c r="E52" s="27" t="n"/>
-    </row>
-    <row r="53" ht="20.5" customHeight="1">
-      <c r="B53" s="28" t="inlineStr">
+      <c r="D51" s="26" t="n"/>
+      <c r="E51" s="27" t="n"/>
+    </row>
+    <row r="52" ht="20.5" customHeight="1">
+      <c r="B52" s="28" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C53" s="29" t="inlineStr">
+      <c r="C52" s="29" t="inlineStr">
         <is>
           <t>Hasta 4 espacios (familiar).</t>
         </is>
       </c>
-      <c r="D53" s="30" t="n"/>
-      <c r="E53" s="31" t="n"/>
-    </row>
-    <row r="54" ht="20" customHeight="1">
-      <c r="B54" s="21" t="inlineStr">
+      <c r="D52" s="30" t="n"/>
+      <c r="E52" s="31" t="n"/>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="B53" s="21" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C54" s="22" t="n"/>
-      <c r="D54" s="22" t="n"/>
-      <c r="E54" s="23" t="n"/>
+      <c r="C53" s="22" t="n"/>
+      <c r="D53" s="22" t="n"/>
+      <c r="E53" s="23" t="n"/>
+    </row>
+    <row r="54" ht="20.5" customHeight="1">
+      <c r="B54" s="24" t="inlineStr">
+        <is>
+          <t>Ambiente</t>
+        </is>
+      </c>
+      <c r="C54" s="25" t="inlineStr">
+        <is>
+          <t>Jardín 1</t>
+        </is>
+      </c>
+      <c r="D54" s="26" t="n"/>
+      <c r="E54" s="27" t="n"/>
     </row>
     <row r="55" ht="20.5" customHeight="1">
-      <c r="B55" s="24" t="inlineStr">
-        <is>
-          <t>Ambiente</t>
-        </is>
-      </c>
-      <c r="C55" s="25" t="inlineStr">
-        <is>
-          <t>Jardín 1</t>
-        </is>
-      </c>
-      <c r="D55" s="26" t="n"/>
-      <c r="E55" s="27" t="n"/>
+      <c r="B55" s="28" t="inlineStr">
+        <is>
+          <t>Capacidad</t>
+        </is>
+      </c>
+      <c r="C55" s="29" t="inlineStr">
+        <is>
+          <t>4 contenedores agrupados en losa</t>
+        </is>
+      </c>
+      <c r="D55" s="30" t="n"/>
+      <c r="E55" s="31" t="n"/>
     </row>
     <row r="56" ht="20.5" customHeight="1">
-      <c r="B56" s="28" t="inlineStr">
-        <is>
-          <t>Capacidad</t>
-        </is>
-      </c>
-      <c r="C56" s="29" t="inlineStr">
-        <is>
-          <t>4 contenedores agrupados en losa</t>
-        </is>
-      </c>
-      <c r="D56" s="30" t="n"/>
-      <c r="E56" s="31" t="n"/>
+      <c r="B56" s="24" t="inlineStr">
+        <is>
+          <t>Identificación</t>
+        </is>
+      </c>
+      <c r="C56" s="25" t="inlineStr">
+        <is>
+          <t>Tapa de granito por espacio, con la información del difunto</t>
+        </is>
+      </c>
+      <c r="D56" s="26" t="n"/>
+      <c r="E56" s="27" t="n"/>
     </row>
     <row r="57" ht="20.5" customHeight="1">
-      <c r="B57" s="24" t="inlineStr">
-        <is>
-          <t>Identificación</t>
-        </is>
-      </c>
-      <c r="C57" s="25" t="inlineStr">
-        <is>
-          <t>Tapa de granito por espacio, con la información del difunto</t>
-        </is>
-      </c>
-      <c r="D57" s="26" t="n"/>
-      <c r="E57" s="27" t="n"/>
+      <c r="B57" s="28" t="inlineStr">
+        <is>
+          <t>Permanencia</t>
+        </is>
+      </c>
+      <c r="C57" s="29" t="inlineStr">
+        <is>
+          <t>30 años desde la primera inhumación, renovable por igual período</t>
+        </is>
+      </c>
+      <c r="D57" s="30" t="n"/>
+      <c r="E57" s="31" t="n"/>
     </row>
     <row r="58" ht="20.5" customHeight="1">
-      <c r="B58" s="28" t="inlineStr">
-        <is>
-          <t>Permanencia</t>
-        </is>
-      </c>
-      <c r="C58" s="29" t="inlineStr">
-        <is>
-          <t>30 años desde la primera inhumación, renovable por igual período</t>
-        </is>
-      </c>
-      <c r="D58" s="30" t="n"/>
-      <c r="E58" s="31" t="n"/>
+      <c r="B58" s="24" t="inlineStr">
+        <is>
+          <t>Acceso</t>
+        </is>
+      </c>
+      <c r="C58" s="25" t="inlineStr">
+        <is>
+          <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
+        </is>
+      </c>
+      <c r="D58" s="26" t="n"/>
+      <c r="E58" s="27" t="n"/>
     </row>
     <row r="59" ht="20.5" customHeight="1">
-      <c r="B59" s="24" t="inlineStr">
-        <is>
-          <t>Acceso</t>
-        </is>
-      </c>
-      <c r="C59" s="25" t="inlineStr">
-        <is>
-          <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
-        </is>
-      </c>
-      <c r="D59" s="26" t="n"/>
-      <c r="E59" s="27" t="n"/>
-    </row>
-    <row r="60" ht="20.5" customHeight="1">
-      <c r="B60" s="28" t="inlineStr">
+      <c r="B59" s="28" t="inlineStr">
         <is>
           <t>Mantenimiento</t>
         </is>
       </c>
-      <c r="C60" s="29" t="inlineStr">
+      <c r="C59" s="29" t="inlineStr">
         <is>
           <t>US$ 24 anual</t>
         </is>
       </c>
-      <c r="D60" s="30" t="n"/>
-      <c r="E60" s="31" t="n"/>
-    </row>
-    <row r="61" ht="64" customHeight="1">
-      <c r="B61" s="24" t="inlineStr">
+      <c r="D59" s="30" t="n"/>
+      <c r="E59" s="31" t="n"/>
+    </row>
+    <row r="60" ht="64" customHeight="1">
+      <c r="B60" s="24" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C61" s="25" t="inlineStr">
+      <c r="C60" s="25" t="inlineStr">
         <is>
           <t>• Inhumación de hasta 4 urnas
 • Tapa de granito grabada para cada espacio
@@ -1896,286 +1882,286 @@
 • Lugar de homenaje familiar por 30 años, renovable por igual período</t>
         </is>
       </c>
-      <c r="D61" s="26" t="n"/>
-      <c r="E61" s="27" t="n"/>
-    </row>
-    <row r="62" ht="20" customHeight="1">
-      <c r="B62" s="21" t="inlineStr">
+      <c r="D60" s="26" t="n"/>
+      <c r="E60" s="27" t="n"/>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="B61" s="21" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C62" s="22" t="n"/>
-      <c r="D62" s="22" t="n"/>
-      <c r="E62" s="23" t="n"/>
+      <c r="C61" s="22" t="n"/>
+      <c r="D61" s="22" t="n"/>
+      <c r="E61" s="23" t="n"/>
+    </row>
+    <row r="62" ht="26.5" customHeight="1">
+      <c r="B62" s="24" t="inlineStr">
+        <is>
+          <t>Precio sugerido</t>
+        </is>
+      </c>
+      <c r="C62" s="32" t="inlineStr">
+        <is>
+          <t>US$ 2.000</t>
+        </is>
+      </c>
+      <c r="D62" s="26" t="n"/>
+      <c r="E62" s="27" t="n"/>
     </row>
     <row r="63" ht="26.5" customHeight="1">
-      <c r="B63" s="24" t="inlineStr">
-        <is>
-          <t>Precio sugerido</t>
-        </is>
-      </c>
-      <c r="C63" s="32" t="inlineStr">
-        <is>
-          <t>US$ 2.000</t>
-        </is>
-      </c>
-      <c r="D63" s="26" t="n"/>
-      <c r="E63" s="27" t="n"/>
-    </row>
-    <row r="64" ht="26.5" customHeight="1">
+      <c r="B63" s="28" t="inlineStr">
+        <is>
+          <t>Precio lanzamiento (−20%)</t>
+        </is>
+      </c>
+      <c r="C63" s="33" t="inlineStr">
+        <is>
+          <t>US$ 1.600</t>
+        </is>
+      </c>
+      <c r="D63" s="30" t="n"/>
+      <c r="E63" s="31" t="n"/>
+    </row>
+    <row r="64" ht="20.5" customHeight="1">
       <c r="B64" s="28" t="inlineStr">
         <is>
-          <t>Precio lanzamiento (−20%)</t>
-        </is>
-      </c>
-      <c r="C64" s="33" t="inlineStr">
-        <is>
-          <t>US$ 1.600</t>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C64" s="29" t="inlineStr">
+        <is>
+          <t>Por parcela familiar · hasta 4 espacios · mantenimiento US$ 24/año</t>
         </is>
       </c>
       <c r="D64" s="30" t="n"/>
       <c r="E64" s="31" t="n"/>
     </row>
-    <row r="65" ht="20.5" customHeight="1">
-      <c r="B65" s="28" t="inlineStr">
-        <is>
-          <t>Base de precio</t>
-        </is>
-      </c>
-      <c r="C65" s="29" t="inlineStr">
-        <is>
-          <t>Por parcela familiar · hasta 4 espacios · mantenimiento US$ 24/año</t>
-        </is>
-      </c>
-      <c r="D65" s="30" t="n"/>
-      <c r="E65" s="31" t="n"/>
-    </row>
-    <row r="66" ht="35" customHeight="1">
-      <c r="B66" s="24" t="inlineStr">
+    <row r="65" ht="35" customHeight="1">
+      <c r="B65" s="24" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C66" s="25" t="inlineStr">
+      <c r="C65" s="25" t="inlineStr">
         <is>
           <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 24 anual.</t>
         </is>
       </c>
-      <c r="D66" s="26" t="n"/>
-      <c r="E66" s="27" t="n"/>
-    </row>
-    <row r="67" ht="20" customHeight="1">
-      <c r="B67" s="21" t="inlineStr">
+      <c r="D65" s="26" t="n"/>
+      <c r="E65" s="27" t="n"/>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="B66" s="21" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C67" s="22" t="n"/>
-      <c r="D67" s="22" t="n"/>
-      <c r="E67" s="23" t="n"/>
-    </row>
-    <row r="68" ht="20.5" customHeight="1">
-      <c r="B68" s="34" t="inlineStr">
+      <c r="C66" s="22" t="n"/>
+      <c r="D66" s="22" t="n"/>
+      <c r="E66" s="23" t="n"/>
+    </row>
+    <row r="67" ht="20.5" customHeight="1">
+      <c r="B67" s="34" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C68" s="35" t="inlineStr">
+      <c r="C67" s="35" t="inlineStr">
         <is>
           <t>Familias que buscan un espacio propio para varias generaciones.</t>
         </is>
       </c>
-      <c r="D68" s="36" t="n"/>
-      <c r="E68" s="37" t="n"/>
-    </row>
-    <row r="71" ht="30" customHeight="1">
-      <c r="B71" s="15" t="inlineStr">
+      <c r="D67" s="36" t="n"/>
+      <c r="E67" s="37" t="n"/>
+    </row>
+    <row r="70" ht="30" customHeight="1">
+      <c r="B70" s="15" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · ECOLÓGICO</t>
         </is>
       </c>
-      <c r="C71" s="16" t="n"/>
-      <c r="D71" s="16" t="n"/>
-      <c r="E71" s="17" t="n"/>
+      <c r="C70" s="16" t="n"/>
+      <c r="D70" s="16" t="n"/>
+      <c r="E70" s="17" t="n"/>
+    </row>
+    <row r="71" ht="20" customHeight="1">
+      <c r="B71" s="18" t="inlineStr">
+        <is>
+          <t>Jardines de la Memoria · Jardín 2  ·  Destino final · Inhumación ecológica</t>
+        </is>
+      </c>
+      <c r="C71" s="19" t="n"/>
+      <c r="D71" s="19" t="n"/>
+      <c r="E71" s="20" t="n"/>
     </row>
     <row r="72" ht="20" customHeight="1">
-      <c r="B72" s="18" t="inlineStr">
-        <is>
-          <t>Jardines de la Memoria · Jardín 2  ·  Destino final · Inhumación ecológica</t>
-        </is>
-      </c>
-      <c r="C72" s="19" t="n"/>
-      <c r="D72" s="19" t="n"/>
-      <c r="E72" s="20" t="n"/>
-    </row>
-    <row r="73" ht="20" customHeight="1">
-      <c r="B73" s="21" t="inlineStr">
+      <c r="B72" s="21" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C73" s="22" t="n"/>
-      <c r="D73" s="22" t="n"/>
-      <c r="E73" s="23" t="n"/>
-    </row>
-    <row r="74" ht="49.5" customHeight="1">
-      <c r="B74" s="24" t="inlineStr">
+      <c r="C72" s="22" t="n"/>
+      <c r="D72" s="22" t="n"/>
+      <c r="E72" s="23" t="n"/>
+    </row>
+    <row r="73" ht="49.5" customHeight="1">
+      <c r="B73" s="24" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C74" s="25" t="inlineStr">
+      <c r="C73" s="25" t="inlineStr">
         <is>
           <t>La urna biodegradable se entierra directamente en el suelo, se cubre con tierra y se descompone integrándose a la naturaleza. Jardín con agua corriente y área de esparcimiento de cenizas.</t>
         </is>
       </c>
-      <c r="D74" s="26" t="n"/>
-      <c r="E74" s="27" t="n"/>
-    </row>
-    <row r="75" ht="20.5" customHeight="1">
-      <c r="B75" s="28" t="inlineStr">
+      <c r="D73" s="26" t="n"/>
+      <c r="E73" s="27" t="n"/>
+    </row>
+    <row r="74" ht="20.5" customHeight="1">
+      <c r="B74" s="28" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C75" s="29" t="inlineStr">
+      <c r="C74" s="29" t="inlineStr">
         <is>
           <t>Individual (1 urna).</t>
         </is>
       </c>
-      <c r="D75" s="30" t="n"/>
-      <c r="E75" s="31" t="n"/>
-    </row>
-    <row r="76" ht="20" customHeight="1">
-      <c r="B76" s="21" t="inlineStr">
+      <c r="D74" s="30" t="n"/>
+      <c r="E74" s="31" t="n"/>
+    </row>
+    <row r="75" ht="20" customHeight="1">
+      <c r="B75" s="21" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C76" s="22" t="n"/>
-      <c r="D76" s="22" t="n"/>
-      <c r="E76" s="23" t="n"/>
+      <c r="C75" s="22" t="n"/>
+      <c r="D75" s="22" t="n"/>
+      <c r="E75" s="23" t="n"/>
+    </row>
+    <row r="76" ht="20.5" customHeight="1">
+      <c r="B76" s="24" t="inlineStr">
+        <is>
+          <t>Ambientes</t>
+        </is>
+      </c>
+      <c r="C76" s="25" t="inlineStr">
+        <is>
+          <t>Jardín 2 · Ecológico o Bosque de las Orquídeas</t>
+        </is>
+      </c>
+      <c r="D76" s="26" t="n"/>
+      <c r="E76" s="27" t="n"/>
     </row>
     <row r="77" ht="20.5" customHeight="1">
-      <c r="B77" s="24" t="inlineStr">
-        <is>
-          <t>Ambientes</t>
-        </is>
-      </c>
-      <c r="C77" s="25" t="inlineStr">
-        <is>
-          <t>Jardín 2 · Ecológico o Bosque de las Orquídeas</t>
-        </is>
-      </c>
-      <c r="D77" s="26" t="n"/>
-      <c r="E77" s="27" t="n"/>
+      <c r="B77" s="28" t="inlineStr">
+        <is>
+          <t>Espacio por urna</t>
+        </is>
+      </c>
+      <c r="C77" s="29" t="inlineStr">
+        <is>
+          <t>30 × 30 cm, 40 cm de profundidad</t>
+        </is>
+      </c>
+      <c r="D77" s="30" t="n"/>
+      <c r="E77" s="31" t="n"/>
     </row>
     <row r="78" ht="20.5" customHeight="1">
-      <c r="B78" s="28" t="inlineStr">
-        <is>
-          <t>Espacio por urna</t>
-        </is>
-      </c>
-      <c r="C78" s="29" t="inlineStr">
-        <is>
-          <t>30 × 30 cm, 40 cm de profundidad</t>
-        </is>
-      </c>
-      <c r="D78" s="30" t="n"/>
-      <c r="E78" s="31" t="n"/>
-    </row>
-    <row r="79" ht="20.5" customHeight="1">
-      <c r="B79" s="24" t="inlineStr">
+      <c r="B78" s="24" t="inlineStr">
         <is>
           <t>Urna</t>
         </is>
       </c>
-      <c r="C79" s="25" t="inlineStr">
+      <c r="C78" s="25" t="inlineStr">
         <is>
           <t>Biodegradable; se integra al suelo</t>
         </is>
       </c>
-      <c r="D79" s="26" t="n"/>
-      <c r="E79" s="27" t="n"/>
-    </row>
-    <row r="80" ht="35" customHeight="1">
-      <c r="B80" s="28" t="inlineStr">
+      <c r="D78" s="26" t="n"/>
+      <c r="E78" s="27" t="n"/>
+    </row>
+    <row r="79" ht="35" customHeight="1">
+      <c r="B79" s="28" t="inlineStr">
         <is>
           <t>Identificación (Jardín 2)</t>
         </is>
       </c>
-      <c r="C80" s="29" t="inlineStr">
+      <c r="C79" s="29" t="inlineStr">
         <is>
           <t>Placa de madera de 20 cm fijada a una varilla metálica, en posición vertical y sin contacto con el suelo</t>
         </is>
       </c>
-      <c r="D80" s="30" t="n"/>
-      <c r="E80" s="31" t="n"/>
-    </row>
-    <row r="81" ht="20.5" customHeight="1">
-      <c r="B81" s="24" t="inlineStr">
+      <c r="D79" s="30" t="n"/>
+      <c r="E79" s="31" t="n"/>
+    </row>
+    <row r="80" ht="20.5" customHeight="1">
+      <c r="B80" s="24" t="inlineStr">
         <is>
           <t>Identificación (Bosque)</t>
         </is>
       </c>
-      <c r="C81" s="25" t="inlineStr">
+      <c r="C80" s="25" t="inlineStr">
         <is>
           <t>Placa de mármol de 20 × 15 cm</t>
         </is>
       </c>
-      <c r="D81" s="26" t="n"/>
-      <c r="E81" s="27" t="n"/>
-    </row>
-    <row r="82" ht="35" customHeight="1">
-      <c r="B82" s="28" t="inlineStr">
+      <c r="D80" s="26" t="n"/>
+      <c r="E80" s="27" t="n"/>
+    </row>
+    <row r="81" ht="35" customHeight="1">
+      <c r="B81" s="28" t="inlineStr">
         <is>
           <t>Permanencia</t>
         </is>
       </c>
-      <c r="C82" s="29" t="inlineStr">
+      <c r="C81" s="29" t="inlineStr">
         <is>
           <t>3 años; luego el nombre pasa a una placa memorial en el monumento y el espacio se reutiliza</t>
         </is>
       </c>
-      <c r="D82" s="30" t="n"/>
-      <c r="E82" s="31" t="n"/>
+      <c r="D81" s="30" t="n"/>
+      <c r="E81" s="31" t="n"/>
+    </row>
+    <row r="82" ht="20.5" customHeight="1">
+      <c r="B82" s="24" t="inlineStr">
+        <is>
+          <t>Placa memorial</t>
+        </is>
+      </c>
+      <c r="C82" s="25" t="inlineStr">
+        <is>
+          <t>Incluida en el precio</t>
+        </is>
+      </c>
+      <c r="D82" s="26" t="n"/>
+      <c r="E82" s="27" t="n"/>
     </row>
     <row r="83" ht="20.5" customHeight="1">
-      <c r="B83" s="24" t="inlineStr">
-        <is>
-          <t>Placa memorial</t>
-        </is>
-      </c>
-      <c r="C83" s="25" t="inlineStr">
-        <is>
-          <t>Incluida en el precio</t>
-        </is>
-      </c>
-      <c r="D83" s="26" t="n"/>
-      <c r="E83" s="27" t="n"/>
-    </row>
-    <row r="84" ht="20.5" customHeight="1">
-      <c r="B84" s="28" t="inlineStr">
+      <c r="B83" s="28" t="inlineStr">
         <is>
           <t>Acceso</t>
         </is>
       </c>
-      <c r="C84" s="29" t="inlineStr">
+      <c r="C83" s="29" t="inlineStr">
         <is>
           <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
         </is>
       </c>
-      <c r="D84" s="30" t="n"/>
-      <c r="E84" s="31" t="n"/>
-    </row>
-    <row r="85" ht="78.5" customHeight="1">
-      <c r="B85" s="24" t="inlineStr">
+      <c r="D83" s="30" t="n"/>
+      <c r="E83" s="31" t="n"/>
+    </row>
+    <row r="84" ht="78.5" customHeight="1">
+      <c r="B84" s="24" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C85" s="25" t="inlineStr">
+      <c r="C84" s="25" t="inlineStr">
         <is>
           <t>• Inhumación ecológica de la urna directamente en el suelo
 • Placa de identificación
@@ -2184,258 +2170,258 @@
 • Permanencia de 3 años; luego, placa memorial en el monumento (incluida)</t>
         </is>
       </c>
-      <c r="D85" s="26" t="n"/>
-      <c r="E85" s="27" t="n"/>
-    </row>
-    <row r="86" ht="20" customHeight="1">
-      <c r="B86" s="21" t="inlineStr">
+      <c r="D84" s="26" t="n"/>
+      <c r="E84" s="27" t="n"/>
+    </row>
+    <row r="85" ht="20" customHeight="1">
+      <c r="B85" s="21" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C86" s="22" t="n"/>
-      <c r="D86" s="22" t="n"/>
-      <c r="E86" s="23" t="n"/>
+      <c r="C85" s="22" t="n"/>
+      <c r="D85" s="22" t="n"/>
+      <c r="E85" s="23" t="n"/>
+    </row>
+    <row r="86" ht="26.5" customHeight="1">
+      <c r="B86" s="24" t="inlineStr">
+        <is>
+          <t>Precio sugerido</t>
+        </is>
+      </c>
+      <c r="C86" s="32" t="inlineStr">
+        <is>
+          <t>US$ 750</t>
+        </is>
+      </c>
+      <c r="D86" s="26" t="n"/>
+      <c r="E86" s="27" t="n"/>
     </row>
     <row r="87" ht="26.5" customHeight="1">
-      <c r="B87" s="24" t="inlineStr">
-        <is>
-          <t>Precio sugerido</t>
-        </is>
-      </c>
-      <c r="C87" s="32" t="inlineStr">
-        <is>
-          <t>US$ 750</t>
-        </is>
-      </c>
-      <c r="D87" s="26" t="n"/>
-      <c r="E87" s="27" t="n"/>
-    </row>
-    <row r="88" ht="26.5" customHeight="1">
+      <c r="B87" s="28" t="inlineStr">
+        <is>
+          <t>Precio lanzamiento (−20%)</t>
+        </is>
+      </c>
+      <c r="C87" s="33" t="inlineStr">
+        <is>
+          <t>US$ 600</t>
+        </is>
+      </c>
+      <c r="D87" s="30" t="n"/>
+      <c r="E87" s="31" t="n"/>
+    </row>
+    <row r="88" ht="20.5" customHeight="1">
       <c r="B88" s="28" t="inlineStr">
         <is>
-          <t>Precio lanzamiento (−20%)</t>
-        </is>
-      </c>
-      <c r="C88" s="33" t="inlineStr">
-        <is>
-          <t>US$ 600</t>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C88" s="29" t="inlineStr">
+        <is>
+          <t>Por espacio individual · placa memorial incluida</t>
         </is>
       </c>
       <c r="D88" s="30" t="n"/>
       <c r="E88" s="31" t="n"/>
     </row>
-    <row r="89" ht="20.5" customHeight="1">
-      <c r="B89" s="28" t="inlineStr">
-        <is>
-          <t>Base de precio</t>
-        </is>
-      </c>
-      <c r="C89" s="29" t="inlineStr">
-        <is>
-          <t>Por espacio individual · placa memorial incluida</t>
-        </is>
-      </c>
-      <c r="D89" s="30" t="n"/>
-      <c r="E89" s="31" t="n"/>
-    </row>
-    <row r="90" ht="35" customHeight="1">
-      <c r="B90" s="24" t="inlineStr">
+    <row r="89" ht="35" customHeight="1">
+      <c r="B89" s="24" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C90" s="25" t="inlineStr">
+      <c r="C89" s="25" t="inlineStr">
         <is>
           <t>Pago único o financiado según política comercial vigente. Incluye la placa memorial en el monumento al término del plazo.</t>
         </is>
       </c>
-      <c r="D90" s="26" t="n"/>
-      <c r="E90" s="27" t="n"/>
-    </row>
-    <row r="91" ht="20" customHeight="1">
-      <c r="B91" s="21" t="inlineStr">
+      <c r="D89" s="26" t="n"/>
+      <c r="E89" s="27" t="n"/>
+    </row>
+    <row r="90" ht="20" customHeight="1">
+      <c r="B90" s="21" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C91" s="22" t="n"/>
-      <c r="D91" s="22" t="n"/>
-      <c r="E91" s="23" t="n"/>
-    </row>
-    <row r="92" ht="35" customHeight="1">
-      <c r="B92" s="34" t="inlineStr">
+      <c r="C90" s="22" t="n"/>
+      <c r="D90" s="22" t="n"/>
+      <c r="E90" s="23" t="n"/>
+    </row>
+    <row r="91" ht="35" customHeight="1">
+      <c r="B91" s="34" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C92" s="35" t="inlineStr">
+      <c r="C91" s="35" t="inlineStr">
         <is>
           <t>Personas con conciencia ambiental que desean que sus cenizas vuelvan a la tierra, con un lugar identificado para visitar.</t>
         </is>
       </c>
-      <c r="D92" s="36" t="n"/>
-      <c r="E92" s="37" t="n"/>
-    </row>
-    <row r="95" ht="30" customHeight="1">
-      <c r="B95" s="15" t="inlineStr">
+      <c r="D91" s="36" t="n"/>
+      <c r="E91" s="37" t="n"/>
+    </row>
+    <row r="94" ht="30" customHeight="1">
+      <c r="B94" s="15" t="inlineStr">
         <is>
           <t>JARDÍN DE MASCOTAS</t>
         </is>
       </c>
-      <c r="C95" s="16" t="n"/>
-      <c r="D95" s="16" t="n"/>
-      <c r="E95" s="17" t="n"/>
+      <c r="C94" s="16" t="n"/>
+      <c r="D94" s="16" t="n"/>
+      <c r="E94" s="17" t="n"/>
+    </row>
+    <row r="95" ht="20" customHeight="1">
+      <c r="B95" s="18" t="inlineStr">
+        <is>
+          <t>Jardines de la Memoria · Mascotas  ·  Destino final · Inhumación ecológica</t>
+        </is>
+      </c>
+      <c r="C95" s="19" t="n"/>
+      <c r="D95" s="19" t="n"/>
+      <c r="E95" s="20" t="n"/>
     </row>
     <row r="96" ht="20" customHeight="1">
-      <c r="B96" s="18" t="inlineStr">
-        <is>
-          <t>Jardines de la Memoria · Mascotas  ·  Destino final · Inhumación ecológica</t>
-        </is>
-      </c>
-      <c r="C96" s="19" t="n"/>
-      <c r="D96" s="19" t="n"/>
-      <c r="E96" s="20" t="n"/>
-    </row>
-    <row r="97" ht="20" customHeight="1">
-      <c r="B97" s="21" t="inlineStr">
+      <c r="B96" s="21" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C97" s="22" t="n"/>
-      <c r="D97" s="22" t="n"/>
-      <c r="E97" s="23" t="n"/>
-    </row>
-    <row r="98" ht="35" customHeight="1">
-      <c r="B98" s="24" t="inlineStr">
+      <c r="C96" s="22" t="n"/>
+      <c r="D96" s="22" t="n"/>
+      <c r="E96" s="23" t="n"/>
+    </row>
+    <row r="97" ht="35" customHeight="1">
+      <c r="B97" s="24" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C98" s="25" t="inlineStr">
+      <c r="C97" s="25" t="inlineStr">
         <is>
           <t>Jardín para inhumación ecológica de cenizas de mascotas: la urna biodegradable se entierra directamente en el suelo y se identifica con una placa de madera.</t>
         </is>
       </c>
-      <c r="D98" s="26" t="n"/>
-      <c r="E98" s="27" t="n"/>
-    </row>
-    <row r="99" ht="20.5" customHeight="1">
-      <c r="B99" s="28" t="inlineStr">
+      <c r="D97" s="26" t="n"/>
+      <c r="E97" s="27" t="n"/>
+    </row>
+    <row r="98" ht="20.5" customHeight="1">
+      <c r="B98" s="28" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C99" s="29" t="inlineStr">
+      <c r="C98" s="29" t="inlineStr">
         <is>
           <t>Individual (una mascota por servicio).</t>
         </is>
       </c>
-      <c r="D99" s="30" t="n"/>
-      <c r="E99" s="31" t="n"/>
-    </row>
-    <row r="100" ht="20" customHeight="1">
-      <c r="B100" s="21" t="inlineStr">
+      <c r="D98" s="30" t="n"/>
+      <c r="E98" s="31" t="n"/>
+    </row>
+    <row r="99" ht="20" customHeight="1">
+      <c r="B99" s="21" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C100" s="22" t="n"/>
-      <c r="D100" s="22" t="n"/>
-      <c r="E100" s="23" t="n"/>
+      <c r="C99" s="22" t="n"/>
+      <c r="D99" s="22" t="n"/>
+      <c r="E99" s="23" t="n"/>
+    </row>
+    <row r="100" ht="20.5" customHeight="1">
+      <c r="B100" s="24" t="inlineStr">
+        <is>
+          <t>Tipo de producto</t>
+        </is>
+      </c>
+      <c r="C100" s="25" t="inlineStr">
+        <is>
+          <t>Servicio de pago único</t>
+        </is>
+      </c>
+      <c r="D100" s="26" t="n"/>
+      <c r="E100" s="27" t="n"/>
     </row>
     <row r="101" ht="20.5" customHeight="1">
-      <c r="B101" s="24" t="inlineStr">
-        <is>
-          <t>Tipo de producto</t>
-        </is>
-      </c>
-      <c r="C101" s="25" t="inlineStr">
-        <is>
-          <t>Servicio de pago único</t>
-        </is>
-      </c>
-      <c r="D101" s="26" t="n"/>
-      <c r="E101" s="27" t="n"/>
-    </row>
-    <row r="102" ht="20.5" customHeight="1">
-      <c r="B102" s="28" t="inlineStr">
+      <c r="B101" s="28" t="inlineStr">
         <is>
           <t>Espacio por urna</t>
         </is>
       </c>
-      <c r="C102" s="29" t="inlineStr">
+      <c r="C101" s="29" t="inlineStr">
         <is>
           <t>15 × 20 cm o 15 × 30 cm, según el tamaño de la urna</t>
         </is>
       </c>
-      <c r="D102" s="30" t="n"/>
-      <c r="E102" s="31" t="n"/>
-    </row>
-    <row r="103" ht="35" customHeight="1">
-      <c r="B103" s="24" t="inlineStr">
+      <c r="D101" s="30" t="n"/>
+      <c r="E101" s="31" t="n"/>
+    </row>
+    <row r="102" ht="35" customHeight="1">
+      <c r="B102" s="24" t="inlineStr">
         <is>
           <t>Urna</t>
         </is>
       </c>
-      <c r="C103" s="25" t="inlineStr">
+      <c r="C102" s="25" t="inlineStr">
         <is>
           <t>Biodegradable; se integra al suelo. Incluida solo en la opción con cremación (US$ 550); con solo espacio (US$ 400) se adquiere por separado</t>
         </is>
       </c>
-      <c r="D103" s="26" t="n"/>
-      <c r="E103" s="27" t="n"/>
+      <c r="D102" s="26" t="n"/>
+      <c r="E102" s="27" t="n"/>
+    </row>
+    <row r="103" ht="20.5" customHeight="1">
+      <c r="B103" s="28" t="inlineStr">
+        <is>
+          <t>Identificación</t>
+        </is>
+      </c>
+      <c r="C103" s="29" t="inlineStr">
+        <is>
+          <t>Placa de madera de 20 cm</t>
+        </is>
+      </c>
+      <c r="D103" s="30" t="n"/>
+      <c r="E103" s="31" t="n"/>
     </row>
     <row r="104" ht="20.5" customHeight="1">
-      <c r="B104" s="28" t="inlineStr">
-        <is>
-          <t>Identificación</t>
-        </is>
-      </c>
-      <c r="C104" s="29" t="inlineStr">
-        <is>
-          <t>Placa de madera de 20 cm</t>
-        </is>
-      </c>
-      <c r="D104" s="30" t="n"/>
-      <c r="E104" s="31" t="n"/>
+      <c r="B104" s="24" t="inlineStr">
+        <is>
+          <t>Permanencia</t>
+        </is>
+      </c>
+      <c r="C104" s="25" t="inlineStr">
+        <is>
+          <t>3 años; luego el espacio se reutiliza</t>
+        </is>
+      </c>
+      <c r="D104" s="26" t="n"/>
+      <c r="E104" s="27" t="n"/>
     </row>
     <row r="105" ht="20.5" customHeight="1">
-      <c r="B105" s="24" t="inlineStr">
-        <is>
-          <t>Permanencia</t>
-        </is>
-      </c>
-      <c r="C105" s="25" t="inlineStr">
-        <is>
-          <t>3 años; luego el espacio se reutiliza</t>
-        </is>
-      </c>
-      <c r="D105" s="26" t="n"/>
-      <c r="E105" s="27" t="n"/>
-    </row>
-    <row r="106" ht="20.5" customHeight="1">
-      <c r="B106" s="28" t="inlineStr">
+      <c r="B105" s="28" t="inlineStr">
         <is>
           <t>Placa memorial</t>
         </is>
       </c>
-      <c r="C106" s="29" t="inlineStr">
+      <c r="C105" s="29" t="inlineStr">
         <is>
           <t>Incluida en el precio; en el monumento al término del plazo</t>
         </is>
       </c>
-      <c r="D106" s="30" t="n"/>
-      <c r="E106" s="31" t="n"/>
-    </row>
-    <row r="107" ht="64" customHeight="1">
-      <c r="B107" s="24" t="inlineStr">
+      <c r="D105" s="30" t="n"/>
+      <c r="E105" s="31" t="n"/>
+    </row>
+    <row r="106" ht="64" customHeight="1">
+      <c r="B106" s="24" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C107" s="25" t="inlineStr">
+      <c r="C106" s="25" t="inlineStr">
         <is>
           <t>• Inhumación ecológica de la urna en el jardín
 • Placa de madera de 20 cm para identificación
@@ -2443,344 +2429,339 @@
 • Cremación de la mascota y urna biodegradable (opción US$ 550)</t>
         </is>
       </c>
-      <c r="D107" s="26" t="n"/>
-      <c r="E107" s="27" t="n"/>
-    </row>
-    <row r="108" ht="20" customHeight="1">
-      <c r="B108" s="21" t="inlineStr">
+      <c r="D106" s="26" t="n"/>
+      <c r="E106" s="27" t="n"/>
+    </row>
+    <row r="107" ht="20" customHeight="1">
+      <c r="B107" s="21" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C108" s="22" t="n"/>
-      <c r="D108" s="22" t="n"/>
-      <c r="E108" s="23" t="n"/>
+      <c r="C107" s="22" t="n"/>
+      <c r="D107" s="22" t="n"/>
+      <c r="E107" s="23" t="n"/>
+    </row>
+    <row r="108" ht="26.5" customHeight="1">
+      <c r="B108" s="24" t="inlineStr">
+        <is>
+          <t>Precio sugerido</t>
+        </is>
+      </c>
+      <c r="C108" s="32" t="inlineStr">
+        <is>
+          <t>US$ 400 / US$ 550</t>
+        </is>
+      </c>
+      <c r="D108" s="26" t="n"/>
+      <c r="E108" s="27" t="n"/>
     </row>
     <row r="109" ht="26.5" customHeight="1">
-      <c r="B109" s="24" t="inlineStr">
-        <is>
-          <t>Precio sugerido</t>
-        </is>
-      </c>
-      <c r="C109" s="32" t="inlineStr">
-        <is>
-          <t>US$ 400 / US$ 550</t>
-        </is>
-      </c>
-      <c r="D109" s="26" t="n"/>
-      <c r="E109" s="27" t="n"/>
-    </row>
-    <row r="110" ht="26.5" customHeight="1">
+      <c r="B109" s="28" t="inlineStr">
+        <is>
+          <t>Precio lanzamiento (−20%)</t>
+        </is>
+      </c>
+      <c r="C109" s="33" t="inlineStr">
+        <is>
+          <t>US$ 320 / US$ 440</t>
+        </is>
+      </c>
+      <c r="D109" s="30" t="n"/>
+      <c r="E109" s="31" t="n"/>
+    </row>
+    <row r="110" ht="20.5" customHeight="1">
       <c r="B110" s="28" t="inlineStr">
         <is>
-          <t>Precio lanzamiento (−20%)</t>
-        </is>
-      </c>
-      <c r="C110" s="33" t="inlineStr">
-        <is>
-          <t>US$ 320 / US$ 440</t>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C110" s="29" t="inlineStr">
+        <is>
+          <t>US$ 400 solo espacio (urna aparte) · US$ 550 con cremación y urna</t>
         </is>
       </c>
       <c r="D110" s="30" t="n"/>
       <c r="E110" s="31" t="n"/>
     </row>
-    <row r="111" ht="20.5" customHeight="1">
-      <c r="B111" s="28" t="inlineStr">
-        <is>
-          <t>Base de precio</t>
-        </is>
-      </c>
-      <c r="C111" s="29" t="inlineStr">
-        <is>
-          <t>US$ 400 solo espacio (urna aparte) · US$ 550 con cremación y urna</t>
-        </is>
-      </c>
-      <c r="D111" s="30" t="n"/>
-      <c r="E111" s="31" t="n"/>
-    </row>
-    <row r="112" ht="49.5" customHeight="1">
-      <c r="B112" s="24" t="inlineStr">
+    <row r="111" ht="49.5" customHeight="1">
+      <c r="B111" s="24" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C112" s="25" t="inlineStr">
+      <c r="C111" s="25" t="inlineStr">
         <is>
           <t>Pago único; puede contratarse como adicional al plan funerario. La opción de US$ 550 incluye la cremación de la mascota y la urna biodegradable; en la opción de US$ 400 (solo espacio) la urna biodegradable se adquiere por separado.</t>
         </is>
       </c>
-      <c r="D112" s="26" t="n"/>
-      <c r="E112" s="27" t="n"/>
-    </row>
-    <row r="113" ht="20" customHeight="1">
-      <c r="B113" s="21" t="inlineStr">
+      <c r="D111" s="26" t="n"/>
+      <c r="E111" s="27" t="n"/>
+    </row>
+    <row r="112" ht="20" customHeight="1">
+      <c r="B112" s="21" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C113" s="22" t="n"/>
-      <c r="D113" s="22" t="n"/>
-      <c r="E113" s="23" t="n"/>
-    </row>
-    <row r="114" ht="20.5" customHeight="1">
-      <c r="B114" s="34" t="inlineStr">
+      <c r="C112" s="22" t="n"/>
+      <c r="D112" s="22" t="n"/>
+      <c r="E112" s="23" t="n"/>
+    </row>
+    <row r="113" ht="20.5" customHeight="1">
+      <c r="B113" s="34" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C114" s="35" t="inlineStr">
+      <c r="C113" s="35" t="inlineStr">
         <is>
           <t>Familias que consideran a su mascota parte del hogar y desean un cierre digno.</t>
         </is>
       </c>
-      <c r="D114" s="36" t="n"/>
-      <c r="E114" s="37" t="n"/>
-    </row>
-    <row r="117" ht="30" customHeight="1">
-      <c r="B117" s="15" t="inlineStr">
+      <c r="D113" s="36" t="n"/>
+      <c r="E113" s="37" t="n"/>
+    </row>
+    <row r="116" ht="30" customHeight="1">
+      <c r="B116" s="15" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · CEREMONIAL</t>
         </is>
       </c>
-      <c r="C117" s="16" t="n"/>
-      <c r="D117" s="16" t="n"/>
-      <c r="E117" s="17" t="n"/>
-    </row>
-    <row r="118" ht="20" customHeight="1">
-      <c r="B118" s="18" t="inlineStr">
+      <c r="C116" s="16" t="n"/>
+      <c r="D116" s="16" t="n"/>
+      <c r="E116" s="17" t="n"/>
+    </row>
+    <row r="117" ht="20" customHeight="1">
+      <c r="B117" s="18" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Jardín 3  ·  Destino final · Inhumación con ceremonia</t>
         </is>
       </c>
-      <c r="C118" s="19" t="n"/>
-      <c r="D118" s="19" t="n"/>
-      <c r="E118" s="20" t="n"/>
-    </row>
-    <row r="119" ht="24" customHeight="1">
-      <c r="B119" s="38" t="inlineStr">
+      <c r="C117" s="19" t="n"/>
+      <c r="D117" s="19" t="n"/>
+      <c r="E117" s="20" t="n"/>
+    </row>
+    <row r="118" ht="24" customHeight="1">
+      <c r="B118" s="38" t="inlineStr">
         <is>
           <t>★  PRÓXIMO LANZAMIENTO · se lanzará en otro momento</t>
         </is>
       </c>
-      <c r="C119" s="39" t="n"/>
-      <c r="D119" s="39" t="n"/>
-      <c r="E119" s="40" t="n"/>
-    </row>
-    <row r="120" ht="20" customHeight="1">
-      <c r="B120" s="21" t="inlineStr">
+      <c r="C118" s="39" t="n"/>
+      <c r="D118" s="39" t="n"/>
+      <c r="E118" s="40" t="n"/>
+    </row>
+    <row r="119" ht="20" customHeight="1">
+      <c r="B119" s="21" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C120" s="22" t="n"/>
-      <c r="D120" s="22" t="n"/>
-      <c r="E120" s="23" t="n"/>
-    </row>
-    <row r="121" ht="35" customHeight="1">
-      <c r="B121" s="24" t="inlineStr">
+      <c r="C119" s="22" t="n"/>
+      <c r="D119" s="22" t="n"/>
+      <c r="E119" s="23" t="n"/>
+    </row>
+    <row r="120" ht="35" customHeight="1">
+      <c r="B120" s="24" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C121" s="25" t="inlineStr">
+      <c r="C120" s="25" t="inlineStr">
         <is>
           <t>Jardín para inhumación de urnas de cenizas con ceremonia de agua, con fuentes como elemento central del rito de despedida.</t>
         </is>
       </c>
-      <c r="D121" s="26" t="n"/>
-      <c r="E121" s="27" t="n"/>
-    </row>
-    <row r="122" ht="20.5" customHeight="1">
-      <c r="B122" s="28" t="inlineStr">
+      <c r="D120" s="26" t="n"/>
+      <c r="E120" s="27" t="n"/>
+    </row>
+    <row r="121" ht="20.5" customHeight="1">
+      <c r="B121" s="28" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C122" s="29" t="inlineStr">
+      <c r="C121" s="29" t="inlineStr">
         <is>
           <t>A definir.</t>
         </is>
       </c>
-      <c r="D122" s="30" t="n"/>
-      <c r="E122" s="31" t="n"/>
-    </row>
-    <row r="123" ht="20" customHeight="1">
-      <c r="B123" s="21" t="inlineStr">
+      <c r="D121" s="30" t="n"/>
+      <c r="E121" s="31" t="n"/>
+    </row>
+    <row r="122" ht="20" customHeight="1">
+      <c r="B122" s="21" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C123" s="22" t="n"/>
-      <c r="D123" s="22" t="n"/>
-      <c r="E123" s="23" t="n"/>
+      <c r="C122" s="22" t="n"/>
+      <c r="D122" s="22" t="n"/>
+      <c r="E122" s="23" t="n"/>
+    </row>
+    <row r="123" ht="20.5" customHeight="1">
+      <c r="B123" s="24" t="inlineStr">
+        <is>
+          <t>Ambiente</t>
+        </is>
+      </c>
+      <c r="C123" s="25" t="inlineStr">
+        <is>
+          <t>Jardín 3</t>
+        </is>
+      </c>
+      <c r="D123" s="26" t="n"/>
+      <c r="E123" s="27" t="n"/>
     </row>
     <row r="124" ht="20.5" customHeight="1">
-      <c r="B124" s="24" t="inlineStr">
-        <is>
-          <t>Ambiente</t>
-        </is>
-      </c>
-      <c r="C124" s="25" t="inlineStr">
-        <is>
-          <t>Jardín 3</t>
-        </is>
-      </c>
-      <c r="D124" s="26" t="n"/>
-      <c r="E124" s="27" t="n"/>
+      <c r="B124" s="28" t="inlineStr">
+        <is>
+          <t>Elemento central</t>
+        </is>
+      </c>
+      <c r="C124" s="29" t="inlineStr">
+        <is>
+          <t>Fuente de agua para la ceremonia</t>
+        </is>
+      </c>
+      <c r="D124" s="30" t="n"/>
+      <c r="E124" s="31" t="n"/>
     </row>
     <row r="125" ht="20.5" customHeight="1">
-      <c r="B125" s="28" t="inlineStr">
-        <is>
-          <t>Elemento central</t>
-        </is>
-      </c>
-      <c r="C125" s="29" t="inlineStr">
-        <is>
-          <t>Fuente de agua para la ceremonia</t>
-        </is>
-      </c>
-      <c r="D125" s="30" t="n"/>
-      <c r="E125" s="31" t="n"/>
-    </row>
-    <row r="126" ht="20.5" customHeight="1">
-      <c r="B126" s="24" t="inlineStr">
+      <c r="B125" s="24" t="inlineStr">
         <is>
           <t>Entorno</t>
         </is>
       </c>
-      <c r="C126" s="25" t="inlineStr">
+      <c r="C125" s="25" t="inlineStr">
         <is>
           <t>Barrera visual que separa el jardín del crematorio</t>
         </is>
       </c>
-      <c r="D126" s="26" t="n"/>
-      <c r="E126" s="27" t="n"/>
-    </row>
-    <row r="127" ht="35" customHeight="1">
-      <c r="B127" s="28" t="inlineStr">
+      <c r="D125" s="26" t="n"/>
+      <c r="E125" s="27" t="n"/>
+    </row>
+    <row r="126" ht="35" customHeight="1">
+      <c r="B126" s="28" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C127" s="29" t="inlineStr">
+      <c r="C126" s="29" t="inlineStr">
         <is>
           <t>• Inhumación de urnas de cenizas
 • Ceremonia con agua en fuente</t>
         </is>
       </c>
-      <c r="D127" s="30" t="n"/>
-      <c r="E127" s="31" t="n"/>
-    </row>
-    <row r="128" ht="20" customHeight="1">
-      <c r="B128" s="21" t="inlineStr">
+      <c r="D126" s="30" t="n"/>
+      <c r="E126" s="31" t="n"/>
+    </row>
+    <row r="127" ht="20" customHeight="1">
+      <c r="B127" s="21" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C128" s="22" t="n"/>
-      <c r="D128" s="22" t="n"/>
-      <c r="E128" s="23" t="n"/>
+      <c r="C127" s="22" t="n"/>
+      <c r="D127" s="22" t="n"/>
+      <c r="E127" s="23" t="n"/>
+    </row>
+    <row r="128" ht="26.5" customHeight="1">
+      <c r="B128" s="24" t="inlineStr">
+        <is>
+          <t>Precio sugerido</t>
+        </is>
+      </c>
+      <c r="C128" s="32" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="D128" s="26" t="n"/>
+      <c r="E128" s="27" t="n"/>
     </row>
     <row r="129" ht="26.5" customHeight="1">
-      <c r="B129" s="24" t="inlineStr">
-        <is>
-          <t>Precio sugerido</t>
-        </is>
-      </c>
-      <c r="C129" s="32" t="inlineStr">
+      <c r="B129" s="28" t="inlineStr">
+        <is>
+          <t>Precio lanzamiento (−20%)</t>
+        </is>
+      </c>
+      <c r="C129" s="33" t="inlineStr">
         <is>
           <t>A definir</t>
         </is>
       </c>
-      <c r="D129" s="26" t="n"/>
-      <c r="E129" s="27" t="n"/>
-    </row>
-    <row r="130" ht="26.5" customHeight="1">
+      <c r="D129" s="30" t="n"/>
+      <c r="E129" s="31" t="n"/>
+    </row>
+    <row r="130" ht="20.5" customHeight="1">
       <c r="B130" s="28" t="inlineStr">
         <is>
-          <t>Precio lanzamiento (−20%)</t>
-        </is>
-      </c>
-      <c r="C130" s="33" t="inlineStr">
-        <is>
-          <t>A definir</t>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C130" s="29" t="inlineStr">
+        <is>
+          <t>Producto en definición</t>
         </is>
       </c>
       <c r="D130" s="30" t="n"/>
       <c r="E130" s="31" t="n"/>
     </row>
     <row r="131" ht="20.5" customHeight="1">
-      <c r="B131" s="28" t="inlineStr">
-        <is>
-          <t>Base de precio</t>
-        </is>
-      </c>
-      <c r="C131" s="29" t="inlineStr">
-        <is>
-          <t>Producto en definición</t>
-        </is>
-      </c>
-      <c r="D131" s="30" t="n"/>
-      <c r="E131" s="31" t="n"/>
-    </row>
-    <row r="132" ht="20.5" customHeight="1">
-      <c r="B132" s="24" t="inlineStr">
+      <c r="B131" s="24" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C132" s="25" t="inlineStr">
+      <c r="C131" s="25" t="inlineStr">
         <is>
           <t>A definir.</t>
         </is>
       </c>
-      <c r="D132" s="26" t="n"/>
-      <c r="E132" s="27" t="n"/>
-    </row>
-    <row r="133" ht="20" customHeight="1">
-      <c r="B133" s="21" t="inlineStr">
+      <c r="D131" s="26" t="n"/>
+      <c r="E131" s="27" t="n"/>
+    </row>
+    <row r="132" ht="20" customHeight="1">
+      <c r="B132" s="21" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C133" s="22" t="n"/>
-      <c r="D133" s="22" t="n"/>
-      <c r="E133" s="23" t="n"/>
-    </row>
-    <row r="134" ht="35" customHeight="1">
-      <c r="B134" s="34" t="inlineStr">
+      <c r="C132" s="22" t="n"/>
+      <c r="D132" s="22" t="n"/>
+      <c r="E132" s="23" t="n"/>
+    </row>
+    <row r="133" ht="35" customHeight="1">
+      <c r="B133" s="34" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C134" s="35" t="inlineStr">
+      <c r="C133" s="35" t="inlineStr">
         <is>
           <t>Familias que valoran un rito de despedida simbólico y un entorno contemplativo.</t>
         </is>
       </c>
-      <c r="D134" s="36" t="n"/>
-      <c r="E134" s="37" t="n"/>
+      <c r="D133" s="36" t="n"/>
+      <c r="E133" s="37" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="123">
-    <mergeCell ref="C44:E44"/>
+  <mergeCells count="122">
+    <mergeCell ref="C31:E31"/>
     <mergeCell ref="C80:E80"/>
+    <mergeCell ref="C40:E40"/>
     <mergeCell ref="C129:E129"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="B123:E123"/>
-    <mergeCell ref="B76:E76"/>
-    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="C51:E51"/>
     <mergeCell ref="C60:E60"/>
-    <mergeCell ref="B113:E113"/>
-    <mergeCell ref="B91:E91"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="B100:E100"/>
+    <mergeCell ref="C123:E123"/>
     <mergeCell ref="C7:E7"/>
-    <mergeCell ref="B22:E22"/>
-    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="C91:E91"/>
     <mergeCell ref="C57:E57"/>
-    <mergeCell ref="B86:E86"/>
+    <mergeCell ref="B21:E21"/>
     <mergeCell ref="C18:E18"/>
+    <mergeCell ref="B39:E39"/>
     <mergeCell ref="C101:E101"/>
     <mergeCell ref="C77:E77"/>
     <mergeCell ref="C34:E34"/>
@@ -2788,31 +2769,28 @@
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="C74:E74"/>
     <mergeCell ref="C126:E126"/>
+    <mergeCell ref="B112:E112"/>
+    <mergeCell ref="C128:E128"/>
     <mergeCell ref="C20:E20"/>
+    <mergeCell ref="C113:E113"/>
     <mergeCell ref="C103:E103"/>
-    <mergeCell ref="C85:E85"/>
-    <mergeCell ref="C112:E112"/>
-    <mergeCell ref="B40:E40"/>
-    <mergeCell ref="C99:E99"/>
     <mergeCell ref="B49:E49"/>
-    <mergeCell ref="C75:E75"/>
     <mergeCell ref="C84:E84"/>
-    <mergeCell ref="C127:E127"/>
-    <mergeCell ref="C114:E114"/>
-    <mergeCell ref="B51:E51"/>
+    <mergeCell ref="C133:E133"/>
+    <mergeCell ref="C22:E22"/>
     <mergeCell ref="C59:E59"/>
     <mergeCell ref="C130:E130"/>
     <mergeCell ref="C12:E12"/>
-    <mergeCell ref="C46:E46"/>
     <mergeCell ref="B26:E26"/>
     <mergeCell ref="B50:E50"/>
     <mergeCell ref="C52:E52"/>
-    <mergeCell ref="C61:E61"/>
-    <mergeCell ref="C39:E39"/>
     <mergeCell ref="B16:E16"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B90:E90"/>
     <mergeCell ref="C106:E106"/>
     <mergeCell ref="C32:E32"/>
     <mergeCell ref="C38:E38"/>
+    <mergeCell ref="B66:E66"/>
     <mergeCell ref="C81:E81"/>
     <mergeCell ref="C125:E125"/>
     <mergeCell ref="B27:E27"/>
@@ -2821,80 +2799,87 @@
     <mergeCell ref="C87:E87"/>
     <mergeCell ref="B117:E117"/>
     <mergeCell ref="C15:E15"/>
-    <mergeCell ref="B67:E67"/>
+    <mergeCell ref="B61:E61"/>
     <mergeCell ref="C33:E33"/>
     <mergeCell ref="C89:E89"/>
     <mergeCell ref="C104:E104"/>
+    <mergeCell ref="B132:E132"/>
+    <mergeCell ref="B53:E53"/>
     <mergeCell ref="B119:E119"/>
     <mergeCell ref="C79:E79"/>
+    <mergeCell ref="C73:E73"/>
     <mergeCell ref="C88:E88"/>
+    <mergeCell ref="B116:E116"/>
     <mergeCell ref="C35:E35"/>
     <mergeCell ref="C63:E63"/>
     <mergeCell ref="C121:E121"/>
     <mergeCell ref="C10:E10"/>
     <mergeCell ref="B118:E118"/>
+    <mergeCell ref="B127:E127"/>
     <mergeCell ref="C55:E55"/>
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="B95:E95"/>
     <mergeCell ref="C36:E36"/>
     <mergeCell ref="C11:E11"/>
-    <mergeCell ref="B97:E97"/>
-    <mergeCell ref="B54:E54"/>
     <mergeCell ref="B72:E72"/>
-    <mergeCell ref="C122:E122"/>
+    <mergeCell ref="C67:E67"/>
     <mergeCell ref="C109:E109"/>
+    <mergeCell ref="B122:E122"/>
+    <mergeCell ref="C28:E28"/>
     <mergeCell ref="B71:E71"/>
     <mergeCell ref="C37:E37"/>
     <mergeCell ref="C78:E78"/>
-    <mergeCell ref="B120:E120"/>
     <mergeCell ref="B2:E2"/>
-    <mergeCell ref="C92:E92"/>
-    <mergeCell ref="C30:E30"/>
+    <mergeCell ref="B107:E107"/>
+    <mergeCell ref="C62:E62"/>
     <mergeCell ref="C14:E14"/>
     <mergeCell ref="C98:E98"/>
-    <mergeCell ref="C107:E107"/>
+    <mergeCell ref="B44:E44"/>
     <mergeCell ref="C64:E64"/>
-    <mergeCell ref="B28:E28"/>
-    <mergeCell ref="B108:E108"/>
+    <mergeCell ref="B99:E99"/>
+    <mergeCell ref="C54:E54"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="C41:E41"/>
-    <mergeCell ref="C134:E134"/>
     <mergeCell ref="C124:E124"/>
+    <mergeCell ref="B30:E30"/>
     <mergeCell ref="C56:E56"/>
     <mergeCell ref="B5:E5"/>
-    <mergeCell ref="C90:E90"/>
     <mergeCell ref="C105:E105"/>
-    <mergeCell ref="B133:E133"/>
     <mergeCell ref="C43:E43"/>
+    <mergeCell ref="B85:E85"/>
+    <mergeCell ref="B94:E94"/>
+    <mergeCell ref="C76:E76"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="C132:E132"/>
+    <mergeCell ref="C120:E120"/>
+    <mergeCell ref="B75:E75"/>
     <mergeCell ref="C110:E110"/>
     <mergeCell ref="C8:E8"/>
-    <mergeCell ref="B62:E62"/>
     <mergeCell ref="C17:E17"/>
     <mergeCell ref="C82:E82"/>
-    <mergeCell ref="C66:E66"/>
     <mergeCell ref="C19:E19"/>
-    <mergeCell ref="C53:E53"/>
     <mergeCell ref="B96:E96"/>
     <mergeCell ref="C102:E102"/>
+    <mergeCell ref="B70:E70"/>
     <mergeCell ref="C111:E111"/>
-    <mergeCell ref="C68:E68"/>
+    <mergeCell ref="B48:E48"/>
+    <mergeCell ref="C86:E86"/>
     <mergeCell ref="C83:E83"/>
+    <mergeCell ref="C108:E108"/>
     <mergeCell ref="C58:E58"/>
-    <mergeCell ref="B73:E73"/>
+    <mergeCell ref="C45:E45"/>
+    <mergeCell ref="C97:E97"/>
     <mergeCell ref="C29:E29"/>
-    <mergeCell ref="B128:E128"/>
+    <mergeCell ref="C100:E100"/>
     <mergeCell ref="C65:E65"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
   <rowBreaks count="5" manualBreakCount="5">
-    <brk id="24" min="0" max="16383" man="1"/>
-    <brk id="47" min="0" max="16383" man="1"/>
-    <brk id="69" min="0" max="16383" man="1"/>
-    <brk id="93" min="0" max="16383" man="1"/>
-    <brk id="115" min="0" max="16383" man="1"/>
+    <brk id="23" min="0" max="16383" man="1"/>
+    <brk id="46" min="0" max="16383" man="1"/>
+    <brk id="68" min="0" max="16383" man="1"/>
+    <brk id="92" min="0" max="16383" man="1"/>
+    <brk id="114" min="0" max="16383" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
@@ -3007,7 +2992,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Alternativa: comisión = 10 primeras cuotas del cliente (≈ US$ 83), pagadas mes a mes, sin estorno.</t>
+          <t>Alternativa: comisión = 10 primeras cuotas del cliente, pagadas mes a mes, sin estorno.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agrega pestaña Portafolio existente (columbarios, −15% Finados y noviembre)
Los cinco productos existentes del portafolio de cremación quedan en una
pestaña aparte del Excel; la tabla general y el HTML no los incluyen.
El descuento de lanzamiento aclara que vale en Finados y noviembre.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111i7vn9WWo4QxCQbucWbrF
</commit_message>
<xml_diff>
--- a/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
+++ b/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
@@ -9,12 +9,14 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabla Gral. - Visión Comercial" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ficha Técnica Consolidada" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comisiones - uso interno" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portafolio existente" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comisiones - uso interno" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tabla Gral. - Visión Comercial'!$A$4:$I$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Tabla Gral. - Visión Comercial'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Ficha Técnica Consolidada'!$A$1:$F$134</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Portafolio existente'!$A$1:$F$103</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -882,7 +884,7 @@
       <c r="H5" s="5" t="inlineStr">
         <is>
           <t>US$ 800
-(descuento especial de lanzamiento)</t>
+(descuento de lanzamiento · Finados y noviembre)</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -936,7 +938,7 @@
       <c r="H6" s="8" t="inlineStr">
         <is>
           <t>US$ 480
-(descuento especial de lanzamiento)</t>
+(descuento de lanzamiento · Finados y noviembre)</t>
         </is>
       </c>
       <c r="I6" s="8" t="inlineStr">
@@ -988,7 +990,7 @@
       <c r="H7" s="5" t="inlineStr">
         <is>
           <t>US$ 1.600
-(descuento especial de lanzamiento)</t>
+(descuento de lanzamiento · Finados y noviembre)</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -1041,7 +1043,7 @@
       <c r="H8" s="8" t="inlineStr">
         <is>
           <t>US$ 600
-(descuento especial de lanzamiento)</t>
+(descuento de lanzamiento · Finados y noviembre)</t>
         </is>
       </c>
       <c r="I8" s="8" t="inlineStr">
@@ -1093,7 +1095,7 @@
       <c r="H9" s="5" t="inlineStr">
         <is>
           <t>US$ 320 / US$ 440
-(descuento especial de lanzamiento)</t>
+(descuento de lanzamiento · Finados y noviembre)</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
@@ -2887,6 +2889,1325 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00C5A059"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B1:E102"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="3" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="B1" s="13" t="inlineStr">
+        <is>
+          <t>PORTAFOLIO EXISTENTE DE CREMACIÓN  ·  LA AUXILIADORA · VANGRUPO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="14" t="inlineStr">
+        <is>
+          <t>Columbarios y cremación · descuento −15% en Finados y noviembre</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>COLUMBARIO SUPREMO PLUS</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="n"/>
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="17" t="n"/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>El Hogar de las Memorias  ·  Servicio funerario + cremación + columbario</t>
+        </is>
+      </c>
+      <c r="C5" s="19" t="n"/>
+      <c r="D5" s="19" t="n"/>
+      <c r="E5" s="20" t="n"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>VISIÓN GENERAL</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="n"/>
+      <c r="D6" s="22" t="n"/>
+      <c r="E6" s="23" t="n"/>
+    </row>
+    <row r="7" ht="49.5" customHeight="1">
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="C7" s="25" t="inlineStr">
+        <is>
+          <t>Experiencia integral que combina servicio funerario y cremación, con un espacio conmemorativo para resguardar hasta dos urnas cinerarias en un entorno de respeto, acompañamiento y serenidad.</t>
+        </is>
+      </c>
+      <c r="D7" s="26" t="n"/>
+      <c r="E7" s="27" t="n"/>
+    </row>
+    <row r="8" ht="20.5" customHeight="1">
+      <c r="B8" s="28" t="inlineStr">
+        <is>
+          <t>Capacidad / Cobertura</t>
+        </is>
+      </c>
+      <c r="C8" s="29" t="inlineStr">
+        <is>
+          <t>Hasta 2 urnas cinerarias (incluye 2 cremaciones).</t>
+        </is>
+      </c>
+      <c r="D8" s="30" t="n"/>
+      <c r="E8" s="31" t="n"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>ESPECIFICACIONES TÉCNICAS</t>
+        </is>
+      </c>
+      <c r="C9" s="22" t="n"/>
+      <c r="D9" s="22" t="n"/>
+      <c r="E9" s="23" t="n"/>
+    </row>
+    <row r="10" ht="20.5" customHeight="1">
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C10" s="25" t="inlineStr">
+        <is>
+          <t>Cristal o mármol</t>
+        </is>
+      </c>
+      <c r="D10" s="26" t="n"/>
+      <c r="E10" s="27" t="n"/>
+    </row>
+    <row r="11" ht="20.5" customHeight="1">
+      <c r="B11" s="28" t="inlineStr">
+        <is>
+          <t>Columbario</t>
+        </is>
+      </c>
+      <c r="C11" s="29" t="inlineStr">
+        <is>
+          <t>Estándar, espacio permanente para hasta 2 urnas</t>
+        </is>
+      </c>
+      <c r="D11" s="30" t="n"/>
+      <c r="E11" s="31" t="n"/>
+    </row>
+    <row r="12" ht="20.5" customHeight="1">
+      <c r="B12" s="24" t="inlineStr">
+        <is>
+          <t>Cremación</t>
+        </is>
+      </c>
+      <c r="C12" s="25" t="inlineStr">
+        <is>
+          <t>2 cremaciones en crematorio propio, con certificado</t>
+        </is>
+      </c>
+      <c r="D12" s="26" t="n"/>
+      <c r="E12" s="27" t="n"/>
+    </row>
+    <row r="13" ht="20.5" customHeight="1">
+      <c r="B13" s="28" t="inlineStr">
+        <is>
+          <t>Preparación y resguardo</t>
+        </is>
+      </c>
+      <c r="C13" s="29" t="inlineStr">
+        <is>
+          <t>Preparación química y custodia en laboratorio hasta por 5 días</t>
+        </is>
+      </c>
+      <c r="D13" s="30" t="n"/>
+      <c r="E13" s="31" t="n"/>
+    </row>
+    <row r="14" ht="35" customHeight="1">
+      <c r="B14" s="24" t="inlineStr">
+        <is>
+          <t>Velación</t>
+        </is>
+      </c>
+      <c r="C14" s="25" t="inlineStr">
+        <is>
+          <t>Sala de velación 24 horas · La Auxiliadora: Capilla Maquilishuat o Básica · Capillas Memoriales: Capilla Las Camelias o Básica</t>
+        </is>
+      </c>
+      <c r="D14" s="26" t="n"/>
+      <c r="E14" s="27" t="n"/>
+    </row>
+    <row r="15" ht="35" customHeight="1">
+      <c r="B15" s="28" t="inlineStr">
+        <is>
+          <t>Ubicación</t>
+        </is>
+      </c>
+      <c r="C15" s="29" t="inlineStr">
+        <is>
+          <t>Definida: se elige el nicho al contratar · A futuro: el nicho se asigna más adelante. El precio varía según fila y nivel.</t>
+        </is>
+      </c>
+      <c r="D15" s="30" t="n"/>
+      <c r="E15" s="31" t="n"/>
+    </row>
+    <row r="16" ht="122" customHeight="1">
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t>Servicios incluidos</t>
+        </is>
+      </c>
+      <c r="C16" s="25" t="inlineStr">
+        <is>
+          <t>• Columbario estándar de cristal o mármol para hasta 2 urnas
+• Traslados durante todo el proceso funerario
+• Preparación química y resguardo hasta por 5 días
+• 2 cremaciones y 2 urnas cinerarias básicas
+• Certificado de cremación y ceremonias privadas de colocación
+• Sala de velación 24 h, ataúd ceremonial y carroza tradicional
+• Asesoría en trámites, libro de condolencias y 50 tarjetas de agradecimiento
+• Programa Vive (acompañamiento en el duelo) y café y agua ilimitados</t>
+        </is>
+      </c>
+      <c r="D16" s="26" t="n"/>
+      <c r="E16" s="27" t="n"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="B17" s="21" t="inlineStr">
+        <is>
+          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
+        </is>
+      </c>
+      <c r="C17" s="22" t="n"/>
+      <c r="D17" s="22" t="n"/>
+      <c r="E17" s="23" t="n"/>
+    </row>
+    <row r="18" ht="41" customHeight="1">
+      <c r="B18" s="24" t="inlineStr">
+        <is>
+          <t>Precio</t>
+        </is>
+      </c>
+      <c r="C18" s="32" t="inlineStr">
+        <is>
+          <t>Ubicación definida: US$ 3.400 – US$ 3.900
+Ubicación a futuro: US$ 2.700 – US$ 3.200</t>
+        </is>
+      </c>
+      <c r="D18" s="26" t="n"/>
+      <c r="E18" s="27" t="n"/>
+    </row>
+    <row r="19" ht="41" customHeight="1">
+      <c r="B19" s="28" t="inlineStr">
+        <is>
+          <t>Precio Finados y noviembre (−15%)</t>
+        </is>
+      </c>
+      <c r="C19" s="33" t="inlineStr">
+        <is>
+          <t>Ubicación definida: US$ 2.890 – US$ 3.315
+Ubicación a futuro: US$ 2.295 – US$ 2.720</t>
+        </is>
+      </c>
+      <c r="D19" s="30" t="n"/>
+      <c r="E19" s="31" t="n"/>
+    </row>
+    <row r="20" ht="20.5" customHeight="1">
+      <c r="B20" s="28" t="inlineStr">
+        <is>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C20" s="29" t="inlineStr">
+        <is>
+          <t>Precio según fila y nivel del columbario</t>
+        </is>
+      </c>
+      <c r="D20" s="30" t="n"/>
+      <c r="E20" s="31" t="n"/>
+    </row>
+    <row r="21" ht="20.5" customHeight="1">
+      <c r="B21" s="24" t="inlineStr">
+        <is>
+          <t>Condiciones</t>
+        </is>
+      </c>
+      <c r="C21" s="25" t="inlineStr">
+        <is>
+          <t>Pago único o financiado hasta 120 meses, con intereses.</t>
+        </is>
+      </c>
+      <c r="D21" s="26" t="n"/>
+      <c r="E21" s="27" t="n"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="B22" s="21" t="inlineStr">
+        <is>
+          <t>PERFIL DEL COMPRADOR</t>
+        </is>
+      </c>
+      <c r="C22" s="22" t="n"/>
+      <c r="D22" s="22" t="n"/>
+      <c r="E22" s="23" t="n"/>
+    </row>
+    <row r="23" ht="35" customHeight="1">
+      <c r="B23" s="34" t="inlineStr">
+        <is>
+          <t>Cliente objetivo</t>
+        </is>
+      </c>
+      <c r="C23" s="35" t="inlineStr">
+        <is>
+          <t>Familias que quieren resolver en una sola compra el servicio funerario, la cremación y un lugar permanente para dos seres queridos.</t>
+        </is>
+      </c>
+      <c r="D23" s="36" t="n"/>
+      <c r="E23" s="37" t="n"/>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>COLUMBARIO MÁRMOL O CRISTAL</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="n"/>
+      <c r="D26" s="16" t="n"/>
+      <c r="E26" s="17" t="n"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>El Hogar de las Memorias  ·  Destino final · Columbario</t>
+        </is>
+      </c>
+      <c r="C27" s="19" t="n"/>
+      <c r="D27" s="19" t="n"/>
+      <c r="E27" s="20" t="n"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="B28" s="21" t="inlineStr">
+        <is>
+          <t>VISIÓN GENERAL</t>
+        </is>
+      </c>
+      <c r="C28" s="22" t="n"/>
+      <c r="D28" s="22" t="n"/>
+      <c r="E28" s="23" t="n"/>
+    </row>
+    <row r="29" ht="35" customHeight="1">
+      <c r="B29" s="24" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="C29" s="25" t="inlineStr">
+        <is>
+          <t>Espacio permanente, elegante y sereno en mármol o cristal para preservar el legado de quienes más ama la familia, con un diseño atemporal.</t>
+        </is>
+      </c>
+      <c r="D29" s="26" t="n"/>
+      <c r="E29" s="27" t="n"/>
+    </row>
+    <row r="30" ht="20.5" customHeight="1">
+      <c r="B30" s="28" t="inlineStr">
+        <is>
+          <t>Capacidad / Cobertura</t>
+        </is>
+      </c>
+      <c r="C30" s="29" t="inlineStr">
+        <is>
+          <t>Estándar: hasta 2 urnas.</t>
+        </is>
+      </c>
+      <c r="D30" s="30" t="n"/>
+      <c r="E30" s="31" t="n"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="B31" s="21" t="inlineStr">
+        <is>
+          <t>ESPECIFICACIONES TÉCNICAS</t>
+        </is>
+      </c>
+      <c r="C31" s="22" t="n"/>
+      <c r="D31" s="22" t="n"/>
+      <c r="E31" s="23" t="n"/>
+    </row>
+    <row r="32" ht="20.5" customHeight="1">
+      <c r="B32" s="24" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C32" s="25" t="inlineStr">
+        <is>
+          <t>Mármol o cristal</t>
+        </is>
+      </c>
+      <c r="D32" s="26" t="n"/>
+      <c r="E32" s="27" t="n"/>
+    </row>
+    <row r="33" ht="20.5" customHeight="1">
+      <c r="B33" s="28" t="inlineStr">
+        <is>
+          <t>Permanencia</t>
+        </is>
+      </c>
+      <c r="C33" s="29" t="inlineStr">
+        <is>
+          <t>Permanente</t>
+        </is>
+      </c>
+      <c r="D33" s="30" t="n"/>
+      <c r="E33" s="31" t="n"/>
+    </row>
+    <row r="34" ht="35" customHeight="1">
+      <c r="B34" s="24" t="inlineStr">
+        <is>
+          <t>Ubicación</t>
+        </is>
+      </c>
+      <c r="C34" s="25" t="inlineStr">
+        <is>
+          <t>Definida: se elige el nicho al contratar · A futuro: el nicho se asigna más adelante. El precio varía según fila y nivel.</t>
+        </is>
+      </c>
+      <c r="D34" s="26" t="n"/>
+      <c r="E34" s="27" t="n"/>
+    </row>
+    <row r="35" ht="35" customHeight="1">
+      <c r="B35" s="28" t="inlineStr">
+        <is>
+          <t>Servicios incluidos</t>
+        </is>
+      </c>
+      <c r="C35" s="29" t="inlineStr">
+        <is>
+          <t>• Espacio permanente en columbario de mármol o cristal
+• Ubicación definida o a futuro, según la opción contratada</t>
+        </is>
+      </c>
+      <c r="D35" s="30" t="n"/>
+      <c r="E35" s="31" t="n"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="B36" s="21" t="inlineStr">
+        <is>
+          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
+        </is>
+      </c>
+      <c r="C36" s="22" t="n"/>
+      <c r="D36" s="22" t="n"/>
+      <c r="E36" s="23" t="n"/>
+    </row>
+    <row r="37" ht="41" customHeight="1">
+      <c r="B37" s="24" t="inlineStr">
+        <is>
+          <t>Precio</t>
+        </is>
+      </c>
+      <c r="C37" s="32" t="inlineStr">
+        <is>
+          <t>Ubicación definida: US$ 2.600
+Ubicación a futuro: US$ 1.200 – US$ 1.900</t>
+        </is>
+      </c>
+      <c r="D37" s="26" t="n"/>
+      <c r="E37" s="27" t="n"/>
+    </row>
+    <row r="38" ht="41" customHeight="1">
+      <c r="B38" s="28" t="inlineStr">
+        <is>
+          <t>Precio Finados y noviembre (−15%)</t>
+        </is>
+      </c>
+      <c r="C38" s="33" t="inlineStr">
+        <is>
+          <t>Ubicación definida: US$ 2.210
+Ubicación a futuro: US$ 1.020 – US$ 1.615</t>
+        </is>
+      </c>
+      <c r="D38" s="30" t="n"/>
+      <c r="E38" s="31" t="n"/>
+    </row>
+    <row r="39" ht="20.5" customHeight="1">
+      <c r="B39" s="28" t="inlineStr">
+        <is>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C39" s="29" t="inlineStr">
+        <is>
+          <t>Solo columbario · precio según fila y nivel</t>
+        </is>
+      </c>
+      <c r="D39" s="30" t="n"/>
+      <c r="E39" s="31" t="n"/>
+    </row>
+    <row r="40" ht="20.5" customHeight="1">
+      <c r="B40" s="24" t="inlineStr">
+        <is>
+          <t>Condiciones</t>
+        </is>
+      </c>
+      <c r="C40" s="25" t="inlineStr">
+        <is>
+          <t>Pago único o financiado hasta 120 meses, con intereses.</t>
+        </is>
+      </c>
+      <c r="D40" s="26" t="n"/>
+      <c r="E40" s="27" t="n"/>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="B41" s="21" t="inlineStr">
+        <is>
+          <t>PERFIL DEL COMPRADOR</t>
+        </is>
+      </c>
+      <c r="C41" s="22" t="n"/>
+      <c r="D41" s="22" t="n"/>
+      <c r="E41" s="23" t="n"/>
+    </row>
+    <row r="42" ht="35" customHeight="1">
+      <c r="B42" s="34" t="inlineStr">
+        <is>
+          <t>Cliente objetivo</t>
+        </is>
+      </c>
+      <c r="C42" s="35" t="inlineStr">
+        <is>
+          <t>Familias que buscan un lugar permanente y elegante para las cenizas, con la cremación ya resuelta o contratada aparte.</t>
+        </is>
+      </c>
+      <c r="D42" s="36" t="n"/>
+      <c r="E42" s="37" t="n"/>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="B45" s="15" t="inlineStr">
+        <is>
+          <t>COLUMBARIO ÓNIX</t>
+        </is>
+      </c>
+      <c r="C45" s="16" t="n"/>
+      <c r="D45" s="16" t="n"/>
+      <c r="E45" s="17" t="n"/>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="B46" s="18" t="inlineStr">
+        <is>
+          <t>El Hogar de las Memorias  ·  Destino final · Columbario premium</t>
+        </is>
+      </c>
+      <c r="C46" s="19" t="n"/>
+      <c r="D46" s="19" t="n"/>
+      <c r="E46" s="20" t="n"/>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="B47" s="21" t="inlineStr">
+        <is>
+          <t>VISIÓN GENERAL</t>
+        </is>
+      </c>
+      <c r="C47" s="22" t="n"/>
+      <c r="D47" s="22" t="n"/>
+      <c r="E47" s="23" t="n"/>
+    </row>
+    <row r="48" ht="49.5" customHeight="1">
+      <c r="B48" s="24" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="C48" s="25" t="inlineStr">
+        <is>
+          <t>Columbario de ónix que combina la exclusividad de una piedra natural con un diseño elegante; sus tonalidades cálidas y apariencia luminosa crean un espacio de paz, respeto y recuerdo perdurable.</t>
+        </is>
+      </c>
+      <c r="D48" s="26" t="n"/>
+      <c r="E48" s="27" t="n"/>
+    </row>
+    <row r="49" ht="20.5" customHeight="1">
+      <c r="B49" s="28" t="inlineStr">
+        <is>
+          <t>Capacidad / Cobertura</t>
+        </is>
+      </c>
+      <c r="C49" s="29" t="inlineStr">
+        <is>
+          <t>Estándar: hasta 2 urnas · Familiar: hasta 4 urnas.</t>
+        </is>
+      </c>
+      <c r="D49" s="30" t="n"/>
+      <c r="E49" s="31" t="n"/>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="B50" s="21" t="inlineStr">
+        <is>
+          <t>ESPECIFICACIONES TÉCNICAS</t>
+        </is>
+      </c>
+      <c r="C50" s="22" t="n"/>
+      <c r="D50" s="22" t="n"/>
+      <c r="E50" s="23" t="n"/>
+    </row>
+    <row r="51" ht="20.5" customHeight="1">
+      <c r="B51" s="24" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C51" s="25" t="inlineStr">
+        <is>
+          <t>Ónix natural</t>
+        </is>
+      </c>
+      <c r="D51" s="26" t="n"/>
+      <c r="E51" s="27" t="n"/>
+    </row>
+    <row r="52" ht="20.5" customHeight="1">
+      <c r="B52" s="28" t="inlineStr">
+        <is>
+          <t>Modalidades</t>
+        </is>
+      </c>
+      <c r="C52" s="29" t="inlineStr">
+        <is>
+          <t>Estándar (2 urnas) y Familiar (4 urnas)</t>
+        </is>
+      </c>
+      <c r="D52" s="30" t="n"/>
+      <c r="E52" s="31" t="n"/>
+    </row>
+    <row r="53" ht="20.5" customHeight="1">
+      <c r="B53" s="24" t="inlineStr">
+        <is>
+          <t>Permanencia</t>
+        </is>
+      </c>
+      <c r="C53" s="25" t="inlineStr">
+        <is>
+          <t>Permanente</t>
+        </is>
+      </c>
+      <c r="D53" s="26" t="n"/>
+      <c r="E53" s="27" t="n"/>
+    </row>
+    <row r="54" ht="35" customHeight="1">
+      <c r="B54" s="28" t="inlineStr">
+        <is>
+          <t>Servicios incluidos</t>
+        </is>
+      </c>
+      <c r="C54" s="29" t="inlineStr">
+        <is>
+          <t>• Espacio permanente en columbario de ónix natural
+• Modalidad estándar o familiar</t>
+        </is>
+      </c>
+      <c r="D54" s="30" t="n"/>
+      <c r="E54" s="31" t="n"/>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="B55" s="21" t="inlineStr">
+        <is>
+          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
+        </is>
+      </c>
+      <c r="C55" s="22" t="n"/>
+      <c r="D55" s="22" t="n"/>
+      <c r="E55" s="23" t="n"/>
+    </row>
+    <row r="56" ht="41" customHeight="1">
+      <c r="B56" s="24" t="inlineStr">
+        <is>
+          <t>Precio</t>
+        </is>
+      </c>
+      <c r="C56" s="32" t="inlineStr">
+        <is>
+          <t>Estándar · ubicación definida: US$ 3.100
+Familiar · ubicación a futuro: US$ 5.000</t>
+        </is>
+      </c>
+      <c r="D56" s="26" t="n"/>
+      <c r="E56" s="27" t="n"/>
+    </row>
+    <row r="57" ht="41" customHeight="1">
+      <c r="B57" s="28" t="inlineStr">
+        <is>
+          <t>Precio Finados y noviembre (−15%)</t>
+        </is>
+      </c>
+      <c r="C57" s="33" t="inlineStr">
+        <is>
+          <t>Estándar · ubicación definida: US$ 2.635
+Familiar · ubicación a futuro: US$ 4.250</t>
+        </is>
+      </c>
+      <c r="D57" s="30" t="n"/>
+      <c r="E57" s="31" t="n"/>
+    </row>
+    <row r="58" ht="20.5" customHeight="1">
+      <c r="B58" s="28" t="inlineStr">
+        <is>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C58" s="29" t="inlineStr">
+        <is>
+          <t>Solo columbario</t>
+        </is>
+      </c>
+      <c r="D58" s="30" t="n"/>
+      <c r="E58" s="31" t="n"/>
+    </row>
+    <row r="59" ht="20.5" customHeight="1">
+      <c r="B59" s="24" t="inlineStr">
+        <is>
+          <t>Condiciones</t>
+        </is>
+      </c>
+      <c r="C59" s="25" t="inlineStr">
+        <is>
+          <t>Pago único o financiado hasta 120 meses, con intereses.</t>
+        </is>
+      </c>
+      <c r="D59" s="26" t="n"/>
+      <c r="E59" s="27" t="n"/>
+    </row>
+    <row r="60" ht="20" customHeight="1">
+      <c r="B60" s="21" t="inlineStr">
+        <is>
+          <t>PERFIL DEL COMPRADOR</t>
+        </is>
+      </c>
+      <c r="C60" s="22" t="n"/>
+      <c r="D60" s="22" t="n"/>
+      <c r="E60" s="23" t="n"/>
+    </row>
+    <row r="61" ht="35" customHeight="1">
+      <c r="B61" s="34" t="inlineStr">
+        <is>
+          <t>Cliente objetivo</t>
+        </is>
+      </c>
+      <c r="C61" s="35" t="inlineStr">
+        <is>
+          <t>Familias que buscan exclusividad y una piedra natural de alta gama para el homenaje.</t>
+        </is>
+      </c>
+      <c r="D61" s="36" t="n"/>
+      <c r="E61" s="37" t="n"/>
+    </row>
+    <row r="64" ht="30" customHeight="1">
+      <c r="B64" s="15" t="inlineStr">
+        <is>
+          <t>COLUMBARIO OBRA DE ARTE</t>
+        </is>
+      </c>
+      <c r="C64" s="16" t="n"/>
+      <c r="D64" s="16" t="n"/>
+      <c r="E64" s="17" t="n"/>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="B65" s="18" t="inlineStr">
+        <is>
+          <t>El Hogar de las Memorias  ·  Destino final · Columbario familiar exclusivo</t>
+        </is>
+      </c>
+      <c r="C65" s="19" t="n"/>
+      <c r="D65" s="19" t="n"/>
+      <c r="E65" s="20" t="n"/>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="B66" s="21" t="inlineStr">
+        <is>
+          <t>VISIÓN GENERAL</t>
+        </is>
+      </c>
+      <c r="C66" s="22" t="n"/>
+      <c r="D66" s="22" t="n"/>
+      <c r="E66" s="23" t="n"/>
+    </row>
+    <row r="67" ht="49.5" customHeight="1">
+      <c r="B67" s="24" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="C67" s="25" t="inlineStr">
+        <is>
+          <t>Una expresión única de fe, memoria y belleza: tapa de ónix con obra de arte religiosa que preserva la memoria de toda una familia en un entorno de serenidad y contemplación.</t>
+        </is>
+      </c>
+      <c r="D67" s="26" t="n"/>
+      <c r="E67" s="27" t="n"/>
+    </row>
+    <row r="68" ht="20.5" customHeight="1">
+      <c r="B68" s="28" t="inlineStr">
+        <is>
+          <t>Capacidad / Cobertura</t>
+        </is>
+      </c>
+      <c r="C68" s="29" t="inlineStr">
+        <is>
+          <t>Familiar: hasta 4 urnas.</t>
+        </is>
+      </c>
+      <c r="D68" s="30" t="n"/>
+      <c r="E68" s="31" t="n"/>
+    </row>
+    <row r="69" ht="20" customHeight="1">
+      <c r="B69" s="21" t="inlineStr">
+        <is>
+          <t>ESPECIFICACIONES TÉCNICAS</t>
+        </is>
+      </c>
+      <c r="C69" s="22" t="n"/>
+      <c r="D69" s="22" t="n"/>
+      <c r="E69" s="23" t="n"/>
+    </row>
+    <row r="70" ht="20.5" customHeight="1">
+      <c r="B70" s="24" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C70" s="25" t="inlineStr">
+        <is>
+          <t>Tapa de ónix con obra de arte religiosa</t>
+        </is>
+      </c>
+      <c r="D70" s="26" t="n"/>
+      <c r="E70" s="27" t="n"/>
+    </row>
+    <row r="71" ht="20.5" customHeight="1">
+      <c r="B71" s="28" t="inlineStr">
+        <is>
+          <t>Modalidad</t>
+        </is>
+      </c>
+      <c r="C71" s="29" t="inlineStr">
+        <is>
+          <t>Familiar (4 urnas)</t>
+        </is>
+      </c>
+      <c r="D71" s="30" t="n"/>
+      <c r="E71" s="31" t="n"/>
+    </row>
+    <row r="72" ht="20.5" customHeight="1">
+      <c r="B72" s="24" t="inlineStr">
+        <is>
+          <t>Ubicación</t>
+        </is>
+      </c>
+      <c r="C72" s="25" t="inlineStr">
+        <is>
+          <t>Definida</t>
+        </is>
+      </c>
+      <c r="D72" s="26" t="n"/>
+      <c r="E72" s="27" t="n"/>
+    </row>
+    <row r="73" ht="20.5" customHeight="1">
+      <c r="B73" s="28" t="inlineStr">
+        <is>
+          <t>Permanencia</t>
+        </is>
+      </c>
+      <c r="C73" s="29" t="inlineStr">
+        <is>
+          <t>Permanente</t>
+        </is>
+      </c>
+      <c r="D73" s="30" t="n"/>
+      <c r="E73" s="31" t="n"/>
+    </row>
+    <row r="74" ht="35" customHeight="1">
+      <c r="B74" s="24" t="inlineStr">
+        <is>
+          <t>Servicios incluidos</t>
+        </is>
+      </c>
+      <c r="C74" s="25" t="inlineStr">
+        <is>
+          <t>• Columbario familiar permanente para hasta 4 urnas
+• Tapa exclusiva de ónix con obra de arte religiosa</t>
+        </is>
+      </c>
+      <c r="D74" s="26" t="n"/>
+      <c r="E74" s="27" t="n"/>
+    </row>
+    <row r="75" ht="20" customHeight="1">
+      <c r="B75" s="21" t="inlineStr">
+        <is>
+          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
+        </is>
+      </c>
+      <c r="C75" s="22" t="n"/>
+      <c r="D75" s="22" t="n"/>
+      <c r="E75" s="23" t="n"/>
+    </row>
+    <row r="76" ht="26.5" customHeight="1">
+      <c r="B76" s="24" t="inlineStr">
+        <is>
+          <t>Precio</t>
+        </is>
+      </c>
+      <c r="C76" s="32" t="inlineStr">
+        <is>
+          <t>Familiar · ubicación definida: US$ 12.500</t>
+        </is>
+      </c>
+      <c r="D76" s="26" t="n"/>
+      <c r="E76" s="27" t="n"/>
+    </row>
+    <row r="77" ht="26.5" customHeight="1">
+      <c r="B77" s="28" t="inlineStr">
+        <is>
+          <t>Precio Finados y noviembre (−15%)</t>
+        </is>
+      </c>
+      <c r="C77" s="33" t="inlineStr">
+        <is>
+          <t>Familiar · ubicación definida: US$ 10.625</t>
+        </is>
+      </c>
+      <c r="D77" s="30" t="n"/>
+      <c r="E77" s="31" t="n"/>
+    </row>
+    <row r="78" ht="20.5" customHeight="1">
+      <c r="B78" s="28" t="inlineStr">
+        <is>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C78" s="29" t="inlineStr">
+        <is>
+          <t>Solo columbario</t>
+        </is>
+      </c>
+      <c r="D78" s="30" t="n"/>
+      <c r="E78" s="31" t="n"/>
+    </row>
+    <row r="79" ht="20.5" customHeight="1">
+      <c r="B79" s="24" t="inlineStr">
+        <is>
+          <t>Condiciones</t>
+        </is>
+      </c>
+      <c r="C79" s="25" t="inlineStr">
+        <is>
+          <t>Pago único o financiado hasta 120 meses, con intereses.</t>
+        </is>
+      </c>
+      <c r="D79" s="26" t="n"/>
+      <c r="E79" s="27" t="n"/>
+    </row>
+    <row r="80" ht="20" customHeight="1">
+      <c r="B80" s="21" t="inlineStr">
+        <is>
+          <t>PERFIL DEL COMPRADOR</t>
+        </is>
+      </c>
+      <c r="C80" s="22" t="n"/>
+      <c r="D80" s="22" t="n"/>
+      <c r="E80" s="23" t="n"/>
+    </row>
+    <row r="81" ht="20.5" customHeight="1">
+      <c r="B81" s="34" t="inlineStr">
+        <is>
+          <t>Cliente objetivo</t>
+        </is>
+      </c>
+      <c r="C81" s="35" t="inlineStr">
+        <is>
+          <t>Familias de fe que desean un legado único y de máxima exclusividad.</t>
+        </is>
+      </c>
+      <c r="D81" s="36" t="n"/>
+      <c r="E81" s="37" t="n"/>
+    </row>
+    <row r="84" ht="30" customHeight="1">
+      <c r="B84" s="15" t="inlineStr">
+        <is>
+          <t>COLUMBARIO CRISTAL · BELLA VISTA</t>
+        </is>
+      </c>
+      <c r="C84" s="16" t="n"/>
+      <c r="D84" s="16" t="n"/>
+      <c r="E84" s="17" t="n"/>
+    </row>
+    <row r="85" ht="20" customHeight="1">
+      <c r="B85" s="18" t="inlineStr">
+        <is>
+          <t>Mausoleo vertical Bella Vista  ·  Cremación + columbario</t>
+        </is>
+      </c>
+      <c r="C85" s="19" t="n"/>
+      <c r="D85" s="19" t="n"/>
+      <c r="E85" s="20" t="n"/>
+    </row>
+    <row r="86" ht="20" customHeight="1">
+      <c r="B86" s="21" t="inlineStr">
+        <is>
+          <t>VISIÓN GENERAL</t>
+        </is>
+      </c>
+      <c r="C86" s="22" t="n"/>
+      <c r="D86" s="22" t="n"/>
+      <c r="E86" s="23" t="n"/>
+    </row>
+    <row r="87" ht="49.5" customHeight="1">
+      <c r="B87" s="24" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="C87" s="25" t="inlineStr">
+        <is>
+          <t>Columbario de cristal en el mausoleo vertical Bella Vista que incluye el proceso completo de cremación: traslados, preparación, cremaciones, urnas y ceremonia de colocación.</t>
+        </is>
+      </c>
+      <c r="D87" s="26" t="n"/>
+      <c r="E87" s="27" t="n"/>
+    </row>
+    <row r="88" ht="20.5" customHeight="1">
+      <c r="B88" s="28" t="inlineStr">
+        <is>
+          <t>Capacidad / Cobertura</t>
+        </is>
+      </c>
+      <c r="C88" s="29" t="inlineStr">
+        <is>
+          <t>Estándar: 2 cremaciones y 2 urnas · Familiar: 4 cremaciones y 4 urnas.</t>
+        </is>
+      </c>
+      <c r="D88" s="30" t="n"/>
+      <c r="E88" s="31" t="n"/>
+    </row>
+    <row r="89" ht="20" customHeight="1">
+      <c r="B89" s="21" t="inlineStr">
+        <is>
+          <t>ESPECIFICACIONES TÉCNICAS</t>
+        </is>
+      </c>
+      <c r="C89" s="22" t="n"/>
+      <c r="D89" s="22" t="n"/>
+      <c r="E89" s="23" t="n"/>
+    </row>
+    <row r="90" ht="20.5" customHeight="1">
+      <c r="B90" s="24" t="inlineStr">
+        <is>
+          <t>Ubicación</t>
+        </is>
+      </c>
+      <c r="C90" s="25" t="inlineStr">
+        <is>
+          <t>Mausoleo vertical Bella Vista</t>
+        </is>
+      </c>
+      <c r="D90" s="26" t="n"/>
+      <c r="E90" s="27" t="n"/>
+    </row>
+    <row r="91" ht="20.5" customHeight="1">
+      <c r="B91" s="28" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C91" s="29" t="inlineStr">
+        <is>
+          <t>Cristal</t>
+        </is>
+      </c>
+      <c r="D91" s="30" t="n"/>
+      <c r="E91" s="31" t="n"/>
+    </row>
+    <row r="92" ht="20.5" customHeight="1">
+      <c r="B92" s="24" t="inlineStr">
+        <is>
+          <t>Medidas</t>
+        </is>
+      </c>
+      <c r="C92" s="25" t="inlineStr">
+        <is>
+          <t>30 × 30 × 30 cm</t>
+        </is>
+      </c>
+      <c r="D92" s="26" t="n"/>
+      <c r="E92" s="27" t="n"/>
+    </row>
+    <row r="93" ht="20.5" customHeight="1">
+      <c r="B93" s="28" t="inlineStr">
+        <is>
+          <t>Cremación</t>
+        </is>
+      </c>
+      <c r="C93" s="29" t="inlineStr">
+        <is>
+          <t>2 (estándar) o 4 (familiar) cremaciones, con certificado</t>
+        </is>
+      </c>
+      <c r="D93" s="30" t="n"/>
+      <c r="E93" s="31" t="n"/>
+    </row>
+    <row r="94" ht="20.5" customHeight="1">
+      <c r="B94" s="24" t="inlineStr">
+        <is>
+          <t>Preparación y resguardo</t>
+        </is>
+      </c>
+      <c r="C94" s="25" t="inlineStr">
+        <is>
+          <t>Preparación química y custodia en laboratorio hasta por 5 días</t>
+        </is>
+      </c>
+      <c r="D94" s="26" t="n"/>
+      <c r="E94" s="27" t="n"/>
+    </row>
+    <row r="95" ht="78.5" customHeight="1">
+      <c r="B95" s="28" t="inlineStr">
+        <is>
+          <t>Servicios incluidos</t>
+        </is>
+      </c>
+      <c r="C95" s="29" t="inlineStr">
+        <is>
+          <t>• Columbario de cristal permanente (estándar o familiar)
+• Traslados durante todo el proceso
+• Preparación química y resguardo hasta por 5 días
+• 2 o 4 cremaciones y 2 o 4 urnas cinerarias básicas
+• Certificado de cremación y ceremonias privadas de colocación</t>
+        </is>
+      </c>
+      <c r="D95" s="30" t="n"/>
+      <c r="E95" s="31" t="n"/>
+    </row>
+    <row r="96" ht="20" customHeight="1">
+      <c r="B96" s="21" t="inlineStr">
+        <is>
+          <t>PRECIO &amp; CONDICIONES DE PAGO</t>
+        </is>
+      </c>
+      <c r="C96" s="22" t="n"/>
+      <c r="D96" s="22" t="n"/>
+      <c r="E96" s="23" t="n"/>
+    </row>
+    <row r="97" ht="70" customHeight="1">
+      <c r="B97" s="24" t="inlineStr">
+        <is>
+          <t>Precio</t>
+        </is>
+      </c>
+      <c r="C97" s="32" t="inlineStr">
+        <is>
+          <t>Estándar · ubicación definida: US$ 1.800
+Estándar · ubicación a futuro: US$ 1.300
+Familiar · ubicación definida: US$ 2.900
+Familiar · ubicación a futuro: US$ 2.300</t>
+        </is>
+      </c>
+      <c r="D97" s="26" t="n"/>
+      <c r="E97" s="27" t="n"/>
+    </row>
+    <row r="98" ht="70" customHeight="1">
+      <c r="B98" s="28" t="inlineStr">
+        <is>
+          <t>Precio Finados y noviembre (−15%)</t>
+        </is>
+      </c>
+      <c r="C98" s="33" t="inlineStr">
+        <is>
+          <t>Estándar · ubicación definida: US$ 1.530
+Estándar · ubicación a futuro: US$ 1.105
+Familiar · ubicación definida: US$ 2.465
+Familiar · ubicación a futuro: US$ 1.955</t>
+        </is>
+      </c>
+      <c r="D98" s="30" t="n"/>
+      <c r="E98" s="31" t="n"/>
+    </row>
+    <row r="99" ht="20.5" customHeight="1">
+      <c r="B99" s="28" t="inlineStr">
+        <is>
+          <t>Base de precio</t>
+        </is>
+      </c>
+      <c r="C99" s="29" t="inlineStr">
+        <is>
+          <t>Incluye cremación · precio según modalidad y ubicación</t>
+        </is>
+      </c>
+      <c r="D99" s="30" t="n"/>
+      <c r="E99" s="31" t="n"/>
+    </row>
+    <row r="100" ht="20.5" customHeight="1">
+      <c r="B100" s="24" t="inlineStr">
+        <is>
+          <t>Condiciones</t>
+        </is>
+      </c>
+      <c r="C100" s="25" t="inlineStr">
+        <is>
+          <t>Pago único o financiado hasta 120 meses, con intereses.</t>
+        </is>
+      </c>
+      <c r="D100" s="26" t="n"/>
+      <c r="E100" s="27" t="n"/>
+    </row>
+    <row r="101" ht="20" customHeight="1">
+      <c r="B101" s="21" t="inlineStr">
+        <is>
+          <t>PERFIL DEL COMPRADOR</t>
+        </is>
+      </c>
+      <c r="C101" s="22" t="n"/>
+      <c r="D101" s="22" t="n"/>
+      <c r="E101" s="23" t="n"/>
+    </row>
+    <row r="102" ht="35" customHeight="1">
+      <c r="B102" s="34" t="inlineStr">
+        <is>
+          <t>Cliente objetivo</t>
+        </is>
+      </c>
+      <c r="C102" s="35" t="inlineStr">
+        <is>
+          <t>Familias que buscan la opción más accesible de cremación con columbario permanente, para 2 o 4 personas.</t>
+        </is>
+      </c>
+      <c r="D102" s="36" t="n"/>
+      <c r="E102" s="37" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="93">
+    <mergeCell ref="B65:E65"/>
+    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="C51:E51"/>
+    <mergeCell ref="C95:E95"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="C71:E71"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="B47:E47"/>
+    <mergeCell ref="C7:E7"/>
+    <mergeCell ref="C91:E91"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="C57:E57"/>
+    <mergeCell ref="B86:E86"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="C49:E49"/>
+    <mergeCell ref="C77:E77"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="B101:E101"/>
+    <mergeCell ref="C42:E42"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="C74:E74"/>
+    <mergeCell ref="B69:E69"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="C99:E99"/>
+    <mergeCell ref="C94:E94"/>
+    <mergeCell ref="B64:E64"/>
+    <mergeCell ref="C59:E59"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="B41:E41"/>
+    <mergeCell ref="B50:E50"/>
+    <mergeCell ref="C52:E52"/>
+    <mergeCell ref="C61:E61"/>
+    <mergeCell ref="C39:E39"/>
+    <mergeCell ref="C70:E70"/>
+    <mergeCell ref="C48:E48"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="B66:E66"/>
+    <mergeCell ref="C81:E81"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="C87:E87"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="C79:E79"/>
+    <mergeCell ref="C73:E73"/>
+    <mergeCell ref="C88:E88"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="B84:E84"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B55:E55"/>
+    <mergeCell ref="B80:E80"/>
+    <mergeCell ref="B89:E89"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="C67:E67"/>
+    <mergeCell ref="C72:E72"/>
+    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="C78:E78"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="C92:E92"/>
+    <mergeCell ref="C30:E30"/>
+    <mergeCell ref="B60:E60"/>
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C98:E98"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="C54:E54"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="C93:E93"/>
+    <mergeCell ref="C56:E56"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="C90:E90"/>
+    <mergeCell ref="B85:E85"/>
+    <mergeCell ref="C76:E76"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B75:E75"/>
+    <mergeCell ref="C8:E8"/>
+    <mergeCell ref="B46:E46"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C53:E53"/>
+    <mergeCell ref="B96:E96"/>
+    <mergeCell ref="C102:E102"/>
+    <mergeCell ref="C68:E68"/>
+    <mergeCell ref="C58:E58"/>
+    <mergeCell ref="C97:E97"/>
+    <mergeCell ref="C29:E29"/>
+    <mergeCell ref="C100:E100"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
+  <rowBreaks count="4" manualBreakCount="4">
+    <brk id="24" min="0" max="16383" man="1"/>
+    <brk id="43" min="0" max="16383" man="1"/>
+    <brk id="62" min="0" max="16383" man="1"/>
+    <brk id="82" min="0" max="16383" man="1"/>
+  </rowBreaks>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="000F2537"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>

</xml_diff>

<commit_message>
Columbarios: ubicación definida o a futuro en todas las opciones
Ónix y Obra de Arte pasan a admitir ubicación definida o a futuro,
como los demás columbarios. Salidas regeneradas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111i7vn9WWo4QxCQbucWbrF
</commit_message>
<xml_diff>
--- a/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
+++ b/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
@@ -3543,8 +3543,8 @@
       </c>
       <c r="C56" s="32" t="inlineStr">
         <is>
-          <t>Estándar · ubicación definida: US$ 3.100
-Familiar · ubicación a futuro: US$ 5.000</t>
+          <t>Estándar · ubicación definida o a futuro: US$ 3.100
+Familiar · ubicación definida o a futuro: US$ 5.000</t>
         </is>
       </c>
       <c r="D56" s="26" t="n"/>
@@ -3558,8 +3558,8 @@
       </c>
       <c r="C57" s="33" t="inlineStr">
         <is>
-          <t>Estándar · ubicación definida: US$ 2.635
-Familiar · ubicación a futuro: US$ 4.250</t>
+          <t>Estándar · ubicación definida o a futuro: US$ 2.635
+Familiar · ubicación definida o a futuro: US$ 4.250</t>
         </is>
       </c>
       <c r="D57" s="30" t="n"/>
@@ -3721,7 +3721,7 @@
       </c>
       <c r="C72" s="25" t="inlineStr">
         <is>
-          <t>Definida</t>
+          <t>Definida o a futuro</t>
         </is>
       </c>
       <c r="D72" s="26" t="n"/>
@@ -3774,7 +3774,7 @@
       </c>
       <c r="C76" s="32" t="inlineStr">
         <is>
-          <t>Familiar · ubicación definida: US$ 12.500</t>
+          <t>Familiar · ubicación definida o a futuro: US$ 12.500</t>
         </is>
       </c>
       <c r="D76" s="26" t="n"/>
@@ -3788,7 +3788,7 @@
       </c>
       <c r="C77" s="33" t="inlineStr">
         <is>
-          <t>Familiar · ubicación definida: US$ 10.625</t>
+          <t>Familiar · ubicación definida o a futuro: US$ 10.625</t>
         </is>
       </c>
       <c r="D77" s="30" t="n"/>

</xml_diff>

<commit_message>
Columbarios: Ónix estándar definida / familiar a futuro; Obra de Arte solo definida
Revierte el cambio anterior: Obra de Arte es solo familiar con ubicación
definida; Ónix estándar es ubicación definida y familiar, a futuro.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111i7vn9WWo4QxCQbucWbrF
</commit_message>
<xml_diff>
--- a/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
+++ b/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
@@ -3543,8 +3543,8 @@
       </c>
       <c r="C56" s="32" t="inlineStr">
         <is>
-          <t>Estándar · ubicación definida o a futuro: US$ 3.100
-Familiar · ubicación definida o a futuro: US$ 5.000</t>
+          <t>Estándar · ubicación definida: US$ 3.100
+Familiar · ubicación a futuro: US$ 5.000</t>
         </is>
       </c>
       <c r="D56" s="26" t="n"/>
@@ -3558,8 +3558,8 @@
       </c>
       <c r="C57" s="33" t="inlineStr">
         <is>
-          <t>Estándar · ubicación definida o a futuro: US$ 2.635
-Familiar · ubicación definida o a futuro: US$ 4.250</t>
+          <t>Estándar · ubicación definida: US$ 2.635
+Familiar · ubicación a futuro: US$ 4.250</t>
         </is>
       </c>
       <c r="D57" s="30" t="n"/>
@@ -3721,7 +3721,7 @@
       </c>
       <c r="C72" s="25" t="inlineStr">
         <is>
-          <t>Definida o a futuro</t>
+          <t>Definida</t>
         </is>
       </c>
       <c r="D72" s="26" t="n"/>
@@ -3774,7 +3774,7 @@
       </c>
       <c r="C76" s="32" t="inlineStr">
         <is>
-          <t>Familiar · ubicación definida o a futuro: US$ 12.500</t>
+          <t>Familiar · ubicación definida: US$ 12.500</t>
         </is>
       </c>
       <c r="D76" s="26" t="n"/>
@@ -3788,7 +3788,7 @@
       </c>
       <c r="C77" s="33" t="inlineStr">
         <is>
-          <t>Familiar · ubicación definida o a futuro: US$ 10.625</t>
+          <t>Familiar · ubicación definida: US$ 10.625</t>
         </is>
       </c>
       <c r="D77" s="30" t="n"/>

</xml_diff>

<commit_message>
Comisiones: Política 2026 aprobada (1 venta 8%, 2 ventas 10%, 3+ 12%)
Reemplaza la comisión única de 8% en el playbook (docx, Google Docs, pptx
horizontal y vertical), la figura de comisiones y la pestaña de comisiones
de la Ficha Técnica.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111i7vn9WWo4QxCQbucWbrF
</commit_message>
<xml_diff>
--- a/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
+++ b/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabla Gral. - Visión Comercial" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ficha Técnica Consolidada" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portafolio existente" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comisiones - uso interno" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comisiones 2026" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tabla Gral. - Visión Comercial'!$A$4:$I$10</definedName>
@@ -27,7 +27,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;US$&quot; #,##0.00"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -106,6 +106,12 @@
       <b val="1"/>
       <color rgb="000F2537"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000F2537"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="9">
@@ -275,7 +281,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -372,29 +378,41 @@
     <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="13" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="13" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
@@ -4212,357 +4230,287 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>LA AUXILIADORA · VANGRUPO  |  POLÍTICA DE COMISIONES — USO INTERNO</t>
+          <t>LA AUXILIADORA · VANGRUPO  |  POLÍTICA DE COMISIONES 2026 · CREMACIÓN</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="41" t="inlineStr">
         <is>
-          <t>PROPUESTA · pendiente de validación con el Gerente Comercial</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="36" customHeight="1">
+          <t>POLÍTICA 2026 · APROBADA · comisión según la cantidad de ventas del mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
       <c r="A4" s="42" t="inlineStr">
         <is>
+          <t>1. ESCALA POR CANTIDAD DE VENTAS EN EL MES (cualquier producto de cremación)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="43" t="inlineStr">
+        <is>
+          <t>Ventas en el mes</t>
+        </is>
+      </c>
+      <c r="B5" s="43" t="inlineStr">
+        <is>
+          <t>% comisión</t>
+        </is>
+      </c>
+      <c r="C5" s="43" t="inlineStr">
+        <is>
+          <t>Ejemplo: facturación con Solución Modular (sin IVA)</t>
+        </is>
+      </c>
+      <c r="D5" s="43" t="inlineStr">
+        <is>
+          <t>Comisión del ejemplo</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="44" t="inlineStr">
+        <is>
+          <t>1 venta</t>
+        </is>
+      </c>
+      <c r="B6" s="45" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="C6" s="46">
+        <f>1*1000*100/113</f>
+        <v/>
+      </c>
+      <c r="D6" s="47">
+        <f>B6*C6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="48" t="inlineStr">
+        <is>
+          <t>2 ventas</t>
+        </is>
+      </c>
+      <c r="B7" s="49" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C7" s="50">
+        <f>2*1000*100/113</f>
+        <v/>
+      </c>
+      <c r="D7" s="51">
+        <f>B7*C7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="44" t="inlineStr">
+        <is>
+          <t>3 ventas o más</t>
+        </is>
+      </c>
+      <c r="B8" s="45" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="C8" s="46">
+        <f>3*1000*100/113</f>
+        <v/>
+      </c>
+      <c r="D8" s="47">
+        <f>B8*C8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="42" t="inlineStr">
+        <is>
+          <t>2. CUÁNDO SE PAGA Y CUÁNDO SE DESCUENTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="43" t="inlineStr">
+        <is>
           <t>Producto</t>
         </is>
       </c>
-      <c r="B4" s="42" t="inlineStr">
-        <is>
-          <t>Precio (c/ IVA)</t>
-        </is>
-      </c>
-      <c r="C4" s="42" t="inlineStr">
-        <is>
-          <t>Precio sin IVA</t>
-        </is>
-      </c>
-      <c r="D4" s="42" t="inlineStr">
-        <is>
-          <t>% Comisión</t>
-        </is>
-      </c>
-      <c r="E4" s="42" t="inlineStr">
-        <is>
-          <t>Comisión por venta (sin IVA)</t>
-        </is>
-      </c>
-      <c r="F4" s="42" t="inlineStr">
+      <c r="B11" s="43" t="inlineStr">
         <is>
           <t>Momento de pago</t>
         </is>
       </c>
-      <c r="G4" s="42" t="inlineStr">
+      <c r="C11" s="43" t="inlineStr">
         <is>
           <t>Estorno</t>
         </is>
       </c>
-      <c r="H4" s="42" t="inlineStr">
+      <c r="D11" s="43" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="44" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="44" t="inlineStr">
         <is>
           <t>Solución Modular de Cremación</t>
         </is>
       </c>
-      <c r="B5" s="43" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C5" s="43">
-        <f>B5*100/113</f>
-        <v/>
-      </c>
-      <c r="D5" s="44" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="E5" s="45">
-        <f>C5*D5</f>
-        <v/>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="B12" s="52" t="inlineStr">
         <is>
           <t>Pago único cuando el cliente paga la 3ª cuota</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="C12" s="52" t="inlineStr">
         <is>
           <t>Si el cliente cancela antes de la 12ª cuota</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>Alternativa: comisión = 10 primeras cuotas del cliente, pagadas mes a mes, sin estorno.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="44" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Jardín de Cenizas · Individual</t>
-        </is>
-      </c>
-      <c r="B6" s="46" t="n">
-        <v>600</v>
-      </c>
-      <c r="C6" s="46">
-        <f>B6*100/113</f>
-        <v/>
-      </c>
-      <c r="D6" s="47" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="E6" s="48">
-        <f>C6*D6</f>
-        <v/>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="D12" s="52" t="inlineStr"/>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="48" t="inlineStr">
+        <is>
+          <t>Jardines de Cenizas (Individual, Familiar, Ecológico)</t>
+        </is>
+      </c>
+      <c r="B13" s="53" t="inlineStr">
         <is>
           <t>Contado: mes siguiente al pago. Financiado: proporcional a lo cobrado</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="C13" s="53" t="inlineStr">
         <is>
           <t>Cancelación en los primeros 90 días</t>
         </is>
       </c>
-      <c r="H6" s="8" t="inlineStr"/>
-    </row>
-    <row r="7" ht="44" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Jardín de Cenizas · Familiar</t>
-        </is>
-      </c>
-      <c r="B7" s="43" t="n">
-        <v>2000</v>
-      </c>
-      <c r="C7" s="43">
-        <f>B7*100/113</f>
-        <v/>
-      </c>
-      <c r="D7" s="44" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="E7" s="45">
-        <f>C7*D7</f>
-        <v/>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="D13" s="53" t="inlineStr"/>
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="44" t="inlineStr">
+        <is>
+          <t>Jardín de Mascotas</t>
+        </is>
+      </c>
+      <c r="B14" s="52" t="inlineStr">
+        <is>
+          <t>Mes siguiente al pago (pago único)</t>
+        </is>
+      </c>
+      <c r="C14" s="52" t="inlineStr">
+        <is>
+          <t>Cancelación en los primeros 90 días</t>
+        </is>
+      </c>
+      <c r="D14" s="52" t="inlineStr"/>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="48" t="inlineStr">
+        <is>
+          <t>Columbarios (portafolio existente)</t>
+        </is>
+      </c>
+      <c r="B15" s="53" t="inlineStr">
         <is>
           <t>Contado: mes siguiente al pago. Financiado: proporcional a lo cobrado</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="C15" s="53" t="inlineStr">
         <is>
           <t>Cancelación en los primeros 90 días</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr"/>
-    </row>
-    <row r="8" ht="44" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Jardín de Cenizas · Ecológico</t>
-        </is>
-      </c>
-      <c r="B8" s="46" t="n">
-        <v>750</v>
-      </c>
-      <c r="C8" s="46">
-        <f>B8*100/113</f>
-        <v/>
-      </c>
-      <c r="D8" s="47" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="E8" s="48">
-        <f>C8*D8</f>
-        <v/>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>Contado: mes siguiente al pago. Financiado: proporcional a lo cobrado</t>
-        </is>
-      </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>Cancelación en los primeros 90 días</t>
-        </is>
-      </c>
-      <c r="H8" s="8" t="inlineStr"/>
-    </row>
-    <row r="9" ht="44" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Jardín de Mascotas · solo espacio</t>
-        </is>
-      </c>
-      <c r="B9" s="43" t="n">
-        <v>400</v>
-      </c>
-      <c r="C9" s="43">
-        <f>B9*100/113</f>
-        <v/>
-      </c>
-      <c r="D9" s="44" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="E9" s="45">
-        <f>C9*D9</f>
-        <v/>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Mes siguiente al pago (pago único)</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>Cancelación en los primeros 90 días</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr"/>
-    </row>
-    <row r="10" ht="44" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>Jardín de Mascotas · jardín + cremación</t>
-        </is>
-      </c>
-      <c r="B10" s="46" t="n">
-        <v>550</v>
-      </c>
-      <c r="C10" s="46">
-        <f>B10*100/113</f>
-        <v/>
-      </c>
-      <c r="D10" s="47" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="E10" s="48">
-        <f>C10*D10</f>
-        <v/>
-      </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Mes siguiente al pago (pago único)</t>
-        </is>
-      </c>
-      <c r="G10" s="8" t="inlineStr">
-        <is>
-          <t>Cancelación en los primeros 90 días</t>
-        </is>
-      </c>
-      <c r="H10" s="8" t="inlineStr"/>
-    </row>
-    <row r="11" ht="44" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Jardín de Cenizas · Ceremonial</t>
-        </is>
-      </c>
-      <c r="B11" s="43" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-      <c r="C11" s="43" t="inlineStr"/>
-      <c r="D11" s="44" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-      <c r="E11" s="45" t="inlineStr"/>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>Próximo lanzamiento; precio a definir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="49" t="inlineStr">
-        <is>
-          <t>REGLAS GENERALES</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="50" t="inlineStr">
-        <is>
-          <t>1. Base de cálculo: valor efectivamente cobrado al cliente, sin IVA (13%).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="50" t="inlineStr">
-        <is>
-          <t>2. No generan comisión: cuotas de mantenimiento anual (US$ 15 / US$ 24).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="50" t="inlineStr">
-        <is>
-          <t>3. Bono de venta combinada: US$ 15 al vender la Solución Modular junto con cualquier jardín.</t>
+      <c r="D15" s="53" t="inlineStr">
+        <is>
+          <t>Mismo criterio de cantidad de ventas que los productos nuevos.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="50" t="inlineStr">
-        <is>
-          <t>4. Acelerador de campaña Día de los Muertos (opcional): +2 pp en Individual y Ecológico para ventas cerradas hasta el 30/11/2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="50" t="inlineStr">
-        <is>
-          <t>5. Estorno: la comisión se descuenta de los pagos siguientes al vendedor.</t>
+      <c r="A17" s="42" t="inlineStr">
+        <is>
+          <t>3. REGLAS GENERALES</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="54" t="inlineStr">
+        <is>
+          <t>1. 1 venta en el mes de cualquier producto de cremación = 8%; 2 ventas = 10%; 3 o más = 12%, sobre toda la facturación del mes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="54" t="inlineStr">
+        <is>
+          <t>2. Cada contrato vendido cuenta como 1 venta, sin distinción por grupo de producto (nuevos y columbarios).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="54" t="inlineStr">
+        <is>
+          <t>3. Base de cálculo: facturación sin IVA (13%), neta de descuentos. La comisión se paga sobre lo cobrado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="54" t="inlineStr">
+        <is>
+          <t>4. Mismo criterio para call center, contratados y freelancers. No hay bonos adicionales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="54" t="inlineStr">
+        <is>
+          <t>5. Venta compartida (call center agenda, otro vendedor cierra): 1 venta para ambos; comisión 30% / 70%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="54" t="inlineStr">
+        <is>
+          <t>6. No generan comisión ni cuentan como venta: cuotas de mantenimiento anual (US$ 15 / US$ 24).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="54" t="inlineStr">
+        <is>
+          <t>7. Estorno: la comisión se descuenta de los pagos siguientes al vendedor. Ventas anuladas no cuentan.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A18:H18"/>
-    <mergeCell ref="A15:H15"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A14:H14"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A17:H17"/>
+  <mergeCells count="12">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="A10:D10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Comisiones: nombre "Política de comisiones de los productos de cremación"
Quita las menciones a "aprobada"/"Propuesta" y renombra la pestaña de la ficha técnica a "Política de Comisiones".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111i7vn9WWo4QxCQbucWbrF
</commit_message>
<xml_diff>
--- a/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
+++ b/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabla Gral. - Visión Comercial" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ficha Técnica Consolidada" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portafolio existente" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comisiones 2026" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Política de Comisiones" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tabla Gral. - Visión Comercial'!$A$4:$I$10</definedName>
@@ -4242,14 +4242,14 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>LA AUXILIADORA · VANGRUPO  |  POLÍTICA DE COMISIONES 2026 · CREMACIÓN</t>
+          <t>LA AUXILIADORA · VANGRUPO  |  POLÍTICA DE COMISIONES DE LOS PRODUCTOS DE CREMACIÓN</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="41" t="inlineStr">
         <is>
-          <t>POLÍTICA 2026 · APROBADA · comisión según la cantidad de ventas del mes</t>
+          <t>Vigente en 2026 · comisión según la cantidad de ventas del mes (8% · 10% · 12%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ficha técnica: portafolio existente dentro de la aba consolidada
Los columbarios dejan de tener aba propia y pasan a una sección
"Portafolio existente" al final de la Ficha Técnica Consolidada,
después de la sección de lanzamientos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111i7vn9WWo4QxCQbucWbrF
</commit_message>
<xml_diff>
--- a/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
+++ b/salida/Ficha_Tecnica_Cremacion_Vangrupo.xlsx
@@ -9,14 +9,12 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabla Gral. - Visión Comercial" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ficha Técnica Consolidada" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portafolio existente" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Política de Comisiones" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Política de Comisiones" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tabla Gral. - Visión Comercial'!$A$4:$I$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Tabla Gral. - Visión Comercial'!$4:$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Ficha Técnica Consolidada'!$A$1:$F$134</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Portafolio existente'!$A$1:$F$103</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Ficha Técnica Consolidada'!$A$1:$F$241</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -27,7 +25,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;US$&quot; #,##0.00"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,6 +74,18 @@
       <i val="1"/>
       <color rgb="00C5A059"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C5A059"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -281,7 +291,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -325,22 +335,28 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -348,7 +364,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -356,13 +372,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -378,7 +394,7 @@
     <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -387,7 +403,7 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="13" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="15" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -399,7 +415,7 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="13" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="15" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1190,7 +1206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:E133"/>
+  <dimension ref="B1:E240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1211,155 +1227,169 @@
     <row r="2">
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>Portafolio de Cremación — Campaña Día de los Muertos 2026</t>
+          <t>Portafolio de Cremación — Campaña Día de los Muertos 2026 y portafolio existente</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="B4" s="15" t="inlineStr">
         <is>
+          <t>LANZAMIENTOS · FINADOS 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Solución Modular y Jardines de la Memoria · descuento de lanzamiento −20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="B7" s="17" t="inlineStr">
+        <is>
           <t>SOLUCIÓN MODULAR DE CREMACIÓN</t>
         </is>
       </c>
-      <c r="C4" s="16" t="n"/>
-      <c r="D4" s="16" t="n"/>
-      <c r="E4" s="17" t="n"/>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="B5" s="18" t="inlineStr">
+      <c r="C7" s="18" t="n"/>
+      <c r="D7" s="18" t="n"/>
+      <c r="E7" s="19" t="n"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="B8" s="20" t="inlineStr">
         <is>
           <t>Línea Cremación Modular  ·  Cremación · Módulo add-on</t>
         </is>
       </c>
-      <c r="C5" s="19" t="n"/>
-      <c r="D5" s="19" t="n"/>
-      <c r="E5" s="20" t="n"/>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="B6" s="21" t="inlineStr">
+      <c r="C8" s="21" t="n"/>
+      <c r="D8" s="21" t="n"/>
+      <c r="E8" s="22" t="n"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="B9" s="23" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C6" s="22" t="n"/>
-      <c r="D6" s="22" t="n"/>
-      <c r="E6" s="23" t="n"/>
-    </row>
-    <row r="7" ht="35" customHeight="1">
-      <c r="B7" s="24" t="inlineStr">
+      <c r="C9" s="24" t="n"/>
+      <c r="D9" s="24" t="n"/>
+      <c r="E9" s="25" t="n"/>
+    </row>
+    <row r="10" ht="35" customHeight="1">
+      <c r="B10" s="26" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C7" s="25" t="inlineStr">
+      <c r="C10" s="27" t="inlineStr">
         <is>
           <t>Módulo de cremación integrable a cualquier plan funerario vigente o nuevo de Vangrupo, sin necesidad de cambiar de plan.</t>
         </is>
       </c>
-      <c r="D7" s="26" t="n"/>
-      <c r="E7" s="27" t="n"/>
-    </row>
-    <row r="8" ht="20.5" customHeight="1">
-      <c r="B8" s="28" t="inlineStr">
+      <c r="D10" s="28" t="n"/>
+      <c r="E10" s="29" t="n"/>
+    </row>
+    <row r="11" ht="20.5" customHeight="1">
+      <c r="B11" s="30" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C8" s="29" t="inlineStr">
+      <c r="C11" s="31" t="inlineStr">
         <is>
           <t>Individual (1 titular / beneficiario por módulo).</t>
         </is>
       </c>
-      <c r="D8" s="30" t="n"/>
-      <c r="E8" s="31" t="n"/>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="B9" s="21" t="inlineStr">
+      <c r="D11" s="32" t="n"/>
+      <c r="E11" s="33" t="n"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="B12" s="23" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C9" s="22" t="n"/>
-      <c r="D9" s="22" t="n"/>
-      <c r="E9" s="23" t="n"/>
-    </row>
-    <row r="10" ht="20.5" customHeight="1">
-      <c r="B10" s="24" t="inlineStr">
+      <c r="C12" s="24" t="n"/>
+      <c r="D12" s="24" t="n"/>
+      <c r="E12" s="25" t="n"/>
+    </row>
+    <row r="13" ht="20.5" customHeight="1">
+      <c r="B13" s="26" t="inlineStr">
         <is>
           <t>Tipo de producto</t>
         </is>
       </c>
-      <c r="C10" s="25" t="inlineStr">
+      <c r="C13" s="27" t="inlineStr">
         <is>
           <t>Módulo adicional (add-on) a plan funerario</t>
         </is>
       </c>
-      <c r="D10" s="26" t="n"/>
-      <c r="E10" s="27" t="n"/>
-    </row>
-    <row r="11" ht="20.5" customHeight="1">
-      <c r="B11" s="28" t="inlineStr">
+      <c r="D13" s="28" t="n"/>
+      <c r="E13" s="29" t="n"/>
+    </row>
+    <row r="14" ht="20.5" customHeight="1">
+      <c r="B14" s="30" t="inlineStr">
         <is>
           <t>Modalidad de cremación</t>
         </is>
       </c>
-      <c r="C11" s="29" t="inlineStr">
+      <c r="C14" s="31" t="inlineStr">
         <is>
           <t>Individual</t>
         </is>
       </c>
-      <c r="D11" s="30" t="n"/>
-      <c r="E11" s="31" t="n"/>
-    </row>
-    <row r="12" ht="20.5" customHeight="1">
-      <c r="B12" s="24" t="inlineStr">
+      <c r="D14" s="32" t="n"/>
+      <c r="E14" s="33" t="n"/>
+    </row>
+    <row r="15" ht="20.5" customHeight="1">
+      <c r="B15" s="26" t="inlineStr">
         <is>
           <t>Urna</t>
         </is>
       </c>
-      <c r="C12" s="25" t="inlineStr">
+      <c r="C15" s="27" t="inlineStr">
         <is>
           <t>Cineraria, línea modular</t>
         </is>
       </c>
-      <c r="D12" s="26" t="n"/>
-      <c r="E12" s="27" t="n"/>
-    </row>
-    <row r="13" ht="20.5" customHeight="1">
-      <c r="B13" s="28" t="inlineStr">
+      <c r="D15" s="28" t="n"/>
+      <c r="E15" s="29" t="n"/>
+    </row>
+    <row r="16" ht="20.5" customHeight="1">
+      <c r="B16" s="30" t="inlineStr">
         <is>
           <t>Gestión legal</t>
         </is>
       </c>
-      <c r="C13" s="29" t="inlineStr">
+      <c r="C16" s="31" t="inlineStr">
         <is>
           <t>Trámites básicos incluidos</t>
         </is>
       </c>
-      <c r="D13" s="30" t="n"/>
-      <c r="E13" s="31" t="n"/>
-    </row>
-    <row r="14" ht="20.5" customHeight="1">
-      <c r="B14" s="24" t="inlineStr">
+      <c r="D16" s="32" t="n"/>
+      <c r="E16" s="33" t="n"/>
+    </row>
+    <row r="17" ht="20.5" customHeight="1">
+      <c r="B17" s="26" t="inlineStr">
         <is>
           <t>Columbario</t>
         </is>
       </c>
-      <c r="C14" s="25" t="inlineStr">
+      <c r="C17" s="27" t="inlineStr">
         <is>
           <t>Alquiler temporal · 12 meses incluido en Hogar de las Memorias</t>
         </is>
       </c>
-      <c r="D14" s="26" t="n"/>
-      <c r="E14" s="27" t="n"/>
-    </row>
-    <row r="15" ht="78.5" customHeight="1">
-      <c r="B15" s="28" t="inlineStr">
+      <c r="D17" s="28" t="n"/>
+      <c r="E17" s="29" t="n"/>
+    </row>
+    <row r="18" ht="78.5" customHeight="1">
+      <c r="B18" s="30" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C15" s="29" t="inlineStr">
+      <c r="C18" s="31" t="inlineStr">
         <is>
           <t>• Proceso completo de cremación individual
 • Urna cineraria de línea modular
@@ -1368,273 +1398,273 @@
 • Integración al plan funerario base (actual o nuevo)</t>
         </is>
       </c>
-      <c r="D15" s="30" t="n"/>
-      <c r="E15" s="31" t="n"/>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="B16" s="21" t="inlineStr">
+      <c r="D18" s="32" t="n"/>
+      <c r="E18" s="33" t="n"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="B19" s="23" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C16" s="22" t="n"/>
-      <c r="D16" s="22" t="n"/>
-      <c r="E16" s="23" t="n"/>
-    </row>
-    <row r="17" ht="26.5" customHeight="1">
-      <c r="B17" s="24" t="inlineStr">
+      <c r="C19" s="24" t="n"/>
+      <c r="D19" s="24" t="n"/>
+      <c r="E19" s="25" t="n"/>
+    </row>
+    <row r="20" ht="26.5" customHeight="1">
+      <c r="B20" s="26" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C17" s="32" t="inlineStr">
+      <c r="C20" s="34" t="inlineStr">
         <is>
           <t>US$ 1.000</t>
         </is>
       </c>
-      <c r="D17" s="26" t="n"/>
-      <c r="E17" s="27" t="n"/>
-    </row>
-    <row r="18" ht="26.5" customHeight="1">
-      <c r="B18" s="28" t="inlineStr">
+      <c r="D20" s="28" t="n"/>
+      <c r="E20" s="29" t="n"/>
+    </row>
+    <row r="21" ht="26.5" customHeight="1">
+      <c r="B21" s="30" t="inlineStr">
         <is>
           <t>Precio lanzamiento (−20%)</t>
         </is>
       </c>
-      <c r="C18" s="33" t="inlineStr">
+      <c r="C21" s="35" t="inlineStr">
         <is>
           <t>US$ 800</t>
         </is>
       </c>
-      <c r="D18" s="30" t="n"/>
-      <c r="E18" s="31" t="n"/>
-    </row>
-    <row r="19" ht="20.5" customHeight="1">
-      <c r="B19" s="28" t="inlineStr">
+      <c r="D21" s="32" t="n"/>
+      <c r="E21" s="33" t="n"/>
+    </row>
+    <row r="22" ht="20.5" customHeight="1">
+      <c r="B22" s="30" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C19" s="29" t="inlineStr">
+      <c r="C22" s="31" t="inlineStr">
         <is>
           <t>Por módulo individual</t>
         </is>
       </c>
-      <c r="D19" s="30" t="n"/>
-      <c r="E19" s="31" t="n"/>
-    </row>
-    <row r="20" ht="35" customHeight="1">
-      <c r="B20" s="24" t="inlineStr">
+      <c r="D22" s="32" t="n"/>
+      <c r="E22" s="33" t="n"/>
+    </row>
+    <row r="23" ht="35" customHeight="1">
+      <c r="B23" s="26" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C20" s="25" t="inlineStr">
+      <c r="C23" s="27" t="inlineStr">
         <is>
           <t>Pago en hasta 120 meses, con intereses.
 Debe estar pagado en su totalidad para el uso de la cremación y el columbario</t>
         </is>
       </c>
-      <c r="D20" s="26" t="n"/>
-      <c r="E20" s="27" t="n"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="B21" s="21" t="inlineStr">
+      <c r="D23" s="28" t="n"/>
+      <c r="E23" s="29" t="n"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="B24" s="23" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C21" s="22" t="n"/>
-      <c r="D21" s="22" t="n"/>
-      <c r="E21" s="23" t="n"/>
-    </row>
-    <row r="22" ht="35" customHeight="1">
-      <c r="B22" s="34" t="inlineStr">
+      <c r="C24" s="24" t="n"/>
+      <c r="D24" s="24" t="n"/>
+      <c r="E24" s="25" t="n"/>
+    </row>
+    <row r="25" ht="35" customHeight="1">
+      <c r="B25" s="36" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C22" s="35" t="inlineStr">
+      <c r="C25" s="37" t="inlineStr">
         <is>
           <t>Afiliados actuales y nuevos que desean incorporar la cremación a su plan con una cuota mensual mínima.</t>
         </is>
       </c>
-      <c r="D22" s="36" t="n"/>
-      <c r="E22" s="37" t="n"/>
-    </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="B25" s="15" t="inlineStr">
+      <c r="D25" s="38" t="n"/>
+      <c r="E25" s="39" t="n"/>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="B28" s="17" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · INDIVIDUAL</t>
         </is>
       </c>
-      <c r="C25" s="16" t="n"/>
-      <c r="D25" s="16" t="n"/>
-      <c r="E25" s="17" t="n"/>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="B26" s="18" t="inlineStr">
+      <c r="C28" s="18" t="n"/>
+      <c r="D28" s="18" t="n"/>
+      <c r="E28" s="19" t="n"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="B29" s="20" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Jardín 1  ·  Destino final · Inhumación individual</t>
         </is>
       </c>
-      <c r="C26" s="19" t="n"/>
-      <c r="D26" s="19" t="n"/>
-      <c r="E26" s="20" t="n"/>
-    </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="B27" s="21" t="inlineStr">
+      <c r="C29" s="21" t="n"/>
+      <c r="D29" s="21" t="n"/>
+      <c r="E29" s="22" t="n"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="B30" s="23" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C27" s="22" t="n"/>
-      <c r="D27" s="22" t="n"/>
-      <c r="E27" s="23" t="n"/>
-    </row>
-    <row r="28" ht="49.5" customHeight="1">
-      <c r="B28" s="24" t="inlineStr">
+      <c r="C30" s="24" t="n"/>
+      <c r="D30" s="24" t="n"/>
+      <c r="E30" s="25" t="n"/>
+    </row>
+    <row r="31" ht="49.5" customHeight="1">
+      <c r="B31" s="26" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C28" s="25" t="inlineStr">
+      <c r="C31" s="27" t="inlineStr">
         <is>
           <t>Inhumación de la urna de cenizas en un contenedor enterrado con tapa de granito grabada, en un jardín de plantas de sombra: un lugar físico de homenaje por 30 años desde la primera inhumación, renovable.</t>
         </is>
       </c>
-      <c r="D28" s="26" t="n"/>
-      <c r="E28" s="27" t="n"/>
-    </row>
-    <row r="29" ht="20.5" customHeight="1">
-      <c r="B29" s="28" t="inlineStr">
+      <c r="D31" s="28" t="n"/>
+      <c r="E31" s="29" t="n"/>
+    </row>
+    <row r="32" ht="20.5" customHeight="1">
+      <c r="B32" s="30" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C29" s="29" t="inlineStr">
+      <c r="C32" s="31" t="inlineStr">
         <is>
           <t>Individual (1 urna).</t>
         </is>
       </c>
-      <c r="D29" s="30" t="n"/>
-      <c r="E29" s="31" t="n"/>
-    </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="B30" s="21" t="inlineStr">
+      <c r="D32" s="32" t="n"/>
+      <c r="E32" s="33" t="n"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="B33" s="23" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C30" s="22" t="n"/>
-      <c r="D30" s="22" t="n"/>
-      <c r="E30" s="23" t="n"/>
-    </row>
-    <row r="31" ht="20.5" customHeight="1">
-      <c r="B31" s="24" t="inlineStr">
+      <c r="C33" s="24" t="n"/>
+      <c r="D33" s="24" t="n"/>
+      <c r="E33" s="25" t="n"/>
+    </row>
+    <row r="34" ht="20.5" customHeight="1">
+      <c r="B34" s="26" t="inlineStr">
         <is>
           <t>Ambiente</t>
         </is>
       </c>
-      <c r="C31" s="25" t="inlineStr">
+      <c r="C34" s="27" t="inlineStr">
         <is>
           <t>Jardín 1</t>
         </is>
       </c>
-      <c r="D31" s="26" t="n"/>
-      <c r="E31" s="27" t="n"/>
-    </row>
-    <row r="32" ht="20.5" customHeight="1">
-      <c r="B32" s="28" t="inlineStr">
+      <c r="D34" s="28" t="n"/>
+      <c r="E34" s="29" t="n"/>
+    </row>
+    <row r="35" ht="20.5" customHeight="1">
+      <c r="B35" s="30" t="inlineStr">
         <is>
           <t>Contenedor</t>
         </is>
       </c>
-      <c r="C32" s="29" t="inlineStr">
+      <c r="C35" s="31" t="inlineStr">
         <is>
           <t>Ø 32 cm × 40 cm de altura; enterrado dejando 20 cm a la vista</t>
         </is>
       </c>
-      <c r="D32" s="30" t="n"/>
-      <c r="E32" s="31" t="n"/>
-    </row>
-    <row r="33" ht="20.5" customHeight="1">
-      <c r="B33" s="24" t="inlineStr">
+      <c r="D35" s="32" t="n"/>
+      <c r="E35" s="33" t="n"/>
+    </row>
+    <row r="36" ht="20.5" customHeight="1">
+      <c r="B36" s="26" t="inlineStr">
         <is>
           <t>Identificación</t>
         </is>
       </c>
-      <c r="C33" s="25" t="inlineStr">
+      <c r="C36" s="27" t="inlineStr">
         <is>
           <t>Tapa de granito con la información del difunto</t>
         </is>
       </c>
-      <c r="D33" s="26" t="n"/>
-      <c r="E33" s="27" t="n"/>
-    </row>
-    <row r="34" ht="20.5" customHeight="1">
-      <c r="B34" s="28" t="inlineStr">
+      <c r="D36" s="28" t="n"/>
+      <c r="E36" s="29" t="n"/>
+    </row>
+    <row r="37" ht="20.5" customHeight="1">
+      <c r="B37" s="30" t="inlineStr">
         <is>
           <t>Paisajismo</t>
         </is>
       </c>
-      <c r="C34" s="29" t="inlineStr">
+      <c r="C37" s="31" t="inlineStr">
         <is>
           <t>Plantas de sombra de diferentes alturas y texturas</t>
         </is>
       </c>
-      <c r="D34" s="30" t="n"/>
-      <c r="E34" s="31" t="n"/>
-    </row>
-    <row r="35" ht="20.5" customHeight="1">
-      <c r="B35" s="24" t="inlineStr">
+      <c r="D37" s="32" t="n"/>
+      <c r="E37" s="33" t="n"/>
+    </row>
+    <row r="38" ht="20.5" customHeight="1">
+      <c r="B38" s="26" t="inlineStr">
         <is>
           <t>Acceso</t>
         </is>
       </c>
-      <c r="C35" s="25" t="inlineStr">
+      <c r="C38" s="27" t="inlineStr">
         <is>
           <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
         </is>
       </c>
-      <c r="D35" s="26" t="n"/>
-      <c r="E35" s="27" t="n"/>
-    </row>
-    <row r="36" ht="20.5" customHeight="1">
-      <c r="B36" s="28" t="inlineStr">
+      <c r="D38" s="28" t="n"/>
+      <c r="E38" s="29" t="n"/>
+    </row>
+    <row r="39" ht="20.5" customHeight="1">
+      <c r="B39" s="30" t="inlineStr">
         <is>
           <t>Permanencia</t>
         </is>
       </c>
-      <c r="C36" s="29" t="inlineStr">
+      <c r="C39" s="31" t="inlineStr">
         <is>
           <t>30 años desde la primera inhumación, renovable por igual período</t>
         </is>
       </c>
-      <c r="D36" s="30" t="n"/>
-      <c r="E36" s="31" t="n"/>
-    </row>
-    <row r="37" ht="20.5" customHeight="1">
-      <c r="B37" s="24" t="inlineStr">
+      <c r="D39" s="32" t="n"/>
+      <c r="E39" s="33" t="n"/>
+    </row>
+    <row r="40" ht="20.5" customHeight="1">
+      <c r="B40" s="26" t="inlineStr">
         <is>
           <t>Mantenimiento</t>
         </is>
       </c>
-      <c r="C37" s="25" t="inlineStr">
+      <c r="C40" s="27" t="inlineStr">
         <is>
           <t>US$ 15 anual</t>
         </is>
       </c>
-      <c r="D37" s="26" t="n"/>
-      <c r="E37" s="27" t="n"/>
-    </row>
-    <row r="38" ht="93" customHeight="1">
-      <c r="B38" s="28" t="inlineStr">
+      <c r="D40" s="28" t="n"/>
+      <c r="E40" s="29" t="n"/>
+    </row>
+    <row r="41" ht="93" customHeight="1">
+      <c r="B41" s="30" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C38" s="29" t="inlineStr">
+      <c r="C41" s="31" t="inlineStr">
         <is>
           <t>• Inhumación de la urna en contenedor individual
 • Tapa de granito con los datos del difunto
@@ -1643,258 +1673,258 @@
 • Permanencia de 30 años desde la primera inhumación, renovable por igual período</t>
         </is>
       </c>
-      <c r="D38" s="30" t="n"/>
-      <c r="E38" s="31" t="n"/>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="B39" s="21" t="inlineStr">
+      <c r="D41" s="32" t="n"/>
+      <c r="E41" s="33" t="n"/>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="B42" s="23" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C39" s="22" t="n"/>
-      <c r="D39" s="22" t="n"/>
-      <c r="E39" s="23" t="n"/>
-    </row>
-    <row r="40" ht="26.5" customHeight="1">
-      <c r="B40" s="24" t="inlineStr">
+      <c r="C42" s="24" t="n"/>
+      <c r="D42" s="24" t="n"/>
+      <c r="E42" s="25" t="n"/>
+    </row>
+    <row r="43" ht="26.5" customHeight="1">
+      <c r="B43" s="26" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C40" s="32" t="inlineStr">
+      <c r="C43" s="34" t="inlineStr">
         <is>
           <t>US$ 600</t>
         </is>
       </c>
-      <c r="D40" s="26" t="n"/>
-      <c r="E40" s="27" t="n"/>
-    </row>
-    <row r="41" ht="26.5" customHeight="1">
-      <c r="B41" s="28" t="inlineStr">
+      <c r="D43" s="28" t="n"/>
+      <c r="E43" s="29" t="n"/>
+    </row>
+    <row r="44" ht="26.5" customHeight="1">
+      <c r="B44" s="30" t="inlineStr">
         <is>
           <t>Precio lanzamiento (−20%)</t>
         </is>
       </c>
-      <c r="C41" s="33" t="inlineStr">
+      <c r="C44" s="35" t="inlineStr">
         <is>
           <t>US$ 480</t>
         </is>
       </c>
-      <c r="D41" s="30" t="n"/>
-      <c r="E41" s="31" t="n"/>
-    </row>
-    <row r="42" ht="20.5" customHeight="1">
-      <c r="B42" s="28" t="inlineStr">
+      <c r="D44" s="32" t="n"/>
+      <c r="E44" s="33" t="n"/>
+    </row>
+    <row r="45" ht="20.5" customHeight="1">
+      <c r="B45" s="30" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C42" s="29" t="inlineStr">
+      <c r="C45" s="31" t="inlineStr">
         <is>
           <t>Por espacio individual · mantenimiento US$ 15/año</t>
         </is>
       </c>
-      <c r="D42" s="30" t="n"/>
-      <c r="E42" s="31" t="n"/>
-    </row>
-    <row r="43" ht="35" customHeight="1">
-      <c r="B43" s="24" t="inlineStr">
+      <c r="D45" s="32" t="n"/>
+      <c r="E45" s="33" t="n"/>
+    </row>
+    <row r="46" ht="35" customHeight="1">
+      <c r="B46" s="26" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C43" s="25" t="inlineStr">
+      <c r="C46" s="27" t="inlineStr">
         <is>
           <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 15 anual.</t>
         </is>
       </c>
-      <c r="D43" s="26" t="n"/>
-      <c r="E43" s="27" t="n"/>
-    </row>
-    <row r="44" ht="20" customHeight="1">
-      <c r="B44" s="21" t="inlineStr">
+      <c r="D46" s="28" t="n"/>
+      <c r="E46" s="29" t="n"/>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="B47" s="23" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C44" s="22" t="n"/>
-      <c r="D44" s="22" t="n"/>
-      <c r="E44" s="23" t="n"/>
-    </row>
-    <row r="45" ht="35" customHeight="1">
-      <c r="B45" s="34" t="inlineStr">
+      <c r="C47" s="24" t="n"/>
+      <c r="D47" s="24" t="n"/>
+      <c r="E47" s="25" t="n"/>
+    </row>
+    <row r="48" ht="35" customHeight="1">
+      <c r="B48" s="36" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C45" s="35" t="inlineStr">
+      <c r="C48" s="37" t="inlineStr">
         <is>
           <t>Familias que desean un lugar propio para visitar y rendir homenaje, con una inversión moderada.</t>
         </is>
       </c>
-      <c r="D45" s="36" t="n"/>
-      <c r="E45" s="37" t="n"/>
-    </row>
-    <row r="48" ht="30" customHeight="1">
-      <c r="B48" s="15" t="inlineStr">
+      <c r="D48" s="38" t="n"/>
+      <c r="E48" s="39" t="n"/>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="B51" s="17" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · FAMILIAR</t>
         </is>
       </c>
-      <c r="C48" s="16" t="n"/>
-      <c r="D48" s="16" t="n"/>
-      <c r="E48" s="17" t="n"/>
-    </row>
-    <row r="49" ht="20" customHeight="1">
-      <c r="B49" s="18" t="inlineStr">
+      <c r="C51" s="18" t="n"/>
+      <c r="D51" s="18" t="n"/>
+      <c r="E51" s="19" t="n"/>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="B52" s="20" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Jardín 1  ·  Destino final · Inhumación familiar</t>
         </is>
       </c>
-      <c r="C49" s="19" t="n"/>
-      <c r="D49" s="19" t="n"/>
-      <c r="E49" s="20" t="n"/>
-    </row>
-    <row r="50" ht="20" customHeight="1">
-      <c r="B50" s="21" t="inlineStr">
+      <c r="C52" s="21" t="n"/>
+      <c r="D52" s="21" t="n"/>
+      <c r="E52" s="22" t="n"/>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="B53" s="23" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C50" s="22" t="n"/>
-      <c r="D50" s="22" t="n"/>
-      <c r="E50" s="23" t="n"/>
-    </row>
-    <row r="51" ht="49.5" customHeight="1">
-      <c r="B51" s="24" t="inlineStr">
+      <c r="C53" s="24" t="n"/>
+      <c r="D53" s="24" t="n"/>
+      <c r="E53" s="25" t="n"/>
+    </row>
+    <row r="54" ht="49.5" customHeight="1">
+      <c r="B54" s="26" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C51" s="25" t="inlineStr">
+      <c r="C54" s="27" t="inlineStr">
         <is>
           <t>Parcela familiar en el Jardín 1 con cuatro contenedores agrupados, cada uno con tapa de granito grabada, con permanencia de 30 años desde la primera inhumación, renovable por igual período.</t>
         </is>
       </c>
-      <c r="D51" s="26" t="n"/>
-      <c r="E51" s="27" t="n"/>
-    </row>
-    <row r="52" ht="20.5" customHeight="1">
-      <c r="B52" s="28" t="inlineStr">
+      <c r="D54" s="28" t="n"/>
+      <c r="E54" s="29" t="n"/>
+    </row>
+    <row r="55" ht="20.5" customHeight="1">
+      <c r="B55" s="30" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C52" s="29" t="inlineStr">
+      <c r="C55" s="31" t="inlineStr">
         <is>
           <t>Hasta 4 espacios (familiar).</t>
         </is>
       </c>
-      <c r="D52" s="30" t="n"/>
-      <c r="E52" s="31" t="n"/>
-    </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="B53" s="21" t="inlineStr">
+      <c r="D55" s="32" t="n"/>
+      <c r="E55" s="33" t="n"/>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="B56" s="23" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C53" s="22" t="n"/>
-      <c r="D53" s="22" t="n"/>
-      <c r="E53" s="23" t="n"/>
-    </row>
-    <row r="54" ht="20.5" customHeight="1">
-      <c r="B54" s="24" t="inlineStr">
+      <c r="C56" s="24" t="n"/>
+      <c r="D56" s="24" t="n"/>
+      <c r="E56" s="25" t="n"/>
+    </row>
+    <row r="57" ht="20.5" customHeight="1">
+      <c r="B57" s="26" t="inlineStr">
         <is>
           <t>Ambiente</t>
         </is>
       </c>
-      <c r="C54" s="25" t="inlineStr">
+      <c r="C57" s="27" t="inlineStr">
         <is>
           <t>Jardín 1</t>
         </is>
       </c>
-      <c r="D54" s="26" t="n"/>
-      <c r="E54" s="27" t="n"/>
-    </row>
-    <row r="55" ht="20.5" customHeight="1">
-      <c r="B55" s="28" t="inlineStr">
+      <c r="D57" s="28" t="n"/>
+      <c r="E57" s="29" t="n"/>
+    </row>
+    <row r="58" ht="20.5" customHeight="1">
+      <c r="B58" s="30" t="inlineStr">
         <is>
           <t>Capacidad</t>
         </is>
       </c>
-      <c r="C55" s="29" t="inlineStr">
+      <c r="C58" s="31" t="inlineStr">
         <is>
           <t>4 contenedores agrupados en losa</t>
         </is>
       </c>
-      <c r="D55" s="30" t="n"/>
-      <c r="E55" s="31" t="n"/>
-    </row>
-    <row r="56" ht="20.5" customHeight="1">
-      <c r="B56" s="24" t="inlineStr">
+      <c r="D58" s="32" t="n"/>
+      <c r="E58" s="33" t="n"/>
+    </row>
+    <row r="59" ht="20.5" customHeight="1">
+      <c r="B59" s="26" t="inlineStr">
         <is>
           <t>Identificación</t>
         </is>
       </c>
-      <c r="C56" s="25" t="inlineStr">
+      <c r="C59" s="27" t="inlineStr">
         <is>
           <t>Tapa de granito por espacio, con la información del difunto</t>
         </is>
       </c>
-      <c r="D56" s="26" t="n"/>
-      <c r="E56" s="27" t="n"/>
-    </row>
-    <row r="57" ht="20.5" customHeight="1">
-      <c r="B57" s="28" t="inlineStr">
+      <c r="D59" s="28" t="n"/>
+      <c r="E59" s="29" t="n"/>
+    </row>
+    <row r="60" ht="20.5" customHeight="1">
+      <c r="B60" s="30" t="inlineStr">
         <is>
           <t>Permanencia</t>
         </is>
       </c>
-      <c r="C57" s="29" t="inlineStr">
+      <c r="C60" s="31" t="inlineStr">
         <is>
           <t>30 años desde la primera inhumación, renovable por igual período</t>
         </is>
       </c>
-      <c r="D57" s="30" t="n"/>
-      <c r="E57" s="31" t="n"/>
-    </row>
-    <row r="58" ht="20.5" customHeight="1">
-      <c r="B58" s="24" t="inlineStr">
+      <c r="D60" s="32" t="n"/>
+      <c r="E60" s="33" t="n"/>
+    </row>
+    <row r="61" ht="20.5" customHeight="1">
+      <c r="B61" s="26" t="inlineStr">
         <is>
           <t>Acceso</t>
         </is>
       </c>
-      <c r="C58" s="25" t="inlineStr">
+      <c r="C61" s="27" t="inlineStr">
         <is>
           <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
         </is>
       </c>
-      <c r="D58" s="26" t="n"/>
-      <c r="E58" s="27" t="n"/>
-    </row>
-    <row r="59" ht="20.5" customHeight="1">
-      <c r="B59" s="28" t="inlineStr">
+      <c r="D61" s="28" t="n"/>
+      <c r="E61" s="29" t="n"/>
+    </row>
+    <row r="62" ht="20.5" customHeight="1">
+      <c r="B62" s="30" t="inlineStr">
         <is>
           <t>Mantenimiento</t>
         </is>
       </c>
-      <c r="C59" s="29" t="inlineStr">
+      <c r="C62" s="31" t="inlineStr">
         <is>
           <t>US$ 24 anual</t>
         </is>
       </c>
-      <c r="D59" s="30" t="n"/>
-      <c r="E59" s="31" t="n"/>
-    </row>
-    <row r="60" ht="64" customHeight="1">
-      <c r="B60" s="24" t="inlineStr">
+      <c r="D62" s="32" t="n"/>
+      <c r="E62" s="33" t="n"/>
+    </row>
+    <row r="63" ht="64" customHeight="1">
+      <c r="B63" s="26" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C60" s="25" t="inlineStr">
+      <c r="C63" s="27" t="inlineStr">
         <is>
           <t>• Inhumación de hasta 4 urnas
 • Tapa de granito grabada para cada espacio
@@ -1902,286 +1932,286 @@
 • Lugar de homenaje familiar por 30 años, renovable por igual período</t>
         </is>
       </c>
-      <c r="D60" s="26" t="n"/>
-      <c r="E60" s="27" t="n"/>
-    </row>
-    <row r="61" ht="20" customHeight="1">
-      <c r="B61" s="21" t="inlineStr">
+      <c r="D63" s="28" t="n"/>
+      <c r="E63" s="29" t="n"/>
+    </row>
+    <row r="64" ht="20" customHeight="1">
+      <c r="B64" s="23" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C61" s="22" t="n"/>
-      <c r="D61" s="22" t="n"/>
-      <c r="E61" s="23" t="n"/>
-    </row>
-    <row r="62" ht="26.5" customHeight="1">
-      <c r="B62" s="24" t="inlineStr">
+      <c r="C64" s="24" t="n"/>
+      <c r="D64" s="24" t="n"/>
+      <c r="E64" s="25" t="n"/>
+    </row>
+    <row r="65" ht="26.5" customHeight="1">
+      <c r="B65" s="26" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C62" s="32" t="inlineStr">
+      <c r="C65" s="34" t="inlineStr">
         <is>
           <t>US$ 2.000</t>
         </is>
       </c>
-      <c r="D62" s="26" t="n"/>
-      <c r="E62" s="27" t="n"/>
-    </row>
-    <row r="63" ht="26.5" customHeight="1">
-      <c r="B63" s="28" t="inlineStr">
+      <c r="D65" s="28" t="n"/>
+      <c r="E65" s="29" t="n"/>
+    </row>
+    <row r="66" ht="26.5" customHeight="1">
+      <c r="B66" s="30" t="inlineStr">
         <is>
           <t>Precio lanzamiento (−20%)</t>
         </is>
       </c>
-      <c r="C63" s="33" t="inlineStr">
+      <c r="C66" s="35" t="inlineStr">
         <is>
           <t>US$ 1.600</t>
         </is>
       </c>
-      <c r="D63" s="30" t="n"/>
-      <c r="E63" s="31" t="n"/>
-    </row>
-    <row r="64" ht="20.5" customHeight="1">
-      <c r="B64" s="28" t="inlineStr">
+      <c r="D66" s="32" t="n"/>
+      <c r="E66" s="33" t="n"/>
+    </row>
+    <row r="67" ht="20.5" customHeight="1">
+      <c r="B67" s="30" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C64" s="29" t="inlineStr">
+      <c r="C67" s="31" t="inlineStr">
         <is>
           <t>Por parcela familiar · hasta 4 espacios · mantenimiento US$ 24/año</t>
         </is>
       </c>
-      <c r="D64" s="30" t="n"/>
-      <c r="E64" s="31" t="n"/>
-    </row>
-    <row r="65" ht="35" customHeight="1">
-      <c r="B65" s="24" t="inlineStr">
+      <c r="D67" s="32" t="n"/>
+      <c r="E67" s="33" t="n"/>
+    </row>
+    <row r="68" ht="35" customHeight="1">
+      <c r="B68" s="26" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C65" s="25" t="inlineStr">
+      <c r="C68" s="27" t="inlineStr">
         <is>
           <t>Pago único o financiado según política comercial vigente. Cuota de mantenimiento: US$ 24 anual.</t>
         </is>
       </c>
-      <c r="D65" s="26" t="n"/>
-      <c r="E65" s="27" t="n"/>
-    </row>
-    <row r="66" ht="20" customHeight="1">
-      <c r="B66" s="21" t="inlineStr">
+      <c r="D68" s="28" t="n"/>
+      <c r="E68" s="29" t="n"/>
+    </row>
+    <row r="69" ht="20" customHeight="1">
+      <c r="B69" s="23" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C66" s="22" t="n"/>
-      <c r="D66" s="22" t="n"/>
-      <c r="E66" s="23" t="n"/>
-    </row>
-    <row r="67" ht="20.5" customHeight="1">
-      <c r="B67" s="34" t="inlineStr">
+      <c r="C69" s="24" t="n"/>
+      <c r="D69" s="24" t="n"/>
+      <c r="E69" s="25" t="n"/>
+    </row>
+    <row r="70" ht="20.5" customHeight="1">
+      <c r="B70" s="36" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C67" s="35" t="inlineStr">
+      <c r="C70" s="37" t="inlineStr">
         <is>
           <t>Familias que buscan un espacio propio para varias generaciones.</t>
         </is>
       </c>
-      <c r="D67" s="36" t="n"/>
-      <c r="E67" s="37" t="n"/>
-    </row>
-    <row r="70" ht="30" customHeight="1">
-      <c r="B70" s="15" t="inlineStr">
+      <c r="D70" s="38" t="n"/>
+      <c r="E70" s="39" t="n"/>
+    </row>
+    <row r="73" ht="30" customHeight="1">
+      <c r="B73" s="17" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · ECOLÓGICO</t>
         </is>
       </c>
-      <c r="C70" s="16" t="n"/>
-      <c r="D70" s="16" t="n"/>
-      <c r="E70" s="17" t="n"/>
-    </row>
-    <row r="71" ht="20" customHeight="1">
-      <c r="B71" s="18" t="inlineStr">
+      <c r="C73" s="18" t="n"/>
+      <c r="D73" s="18" t="n"/>
+      <c r="E73" s="19" t="n"/>
+    </row>
+    <row r="74" ht="20" customHeight="1">
+      <c r="B74" s="20" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Jardín 2  ·  Destino final · Inhumación ecológica</t>
         </is>
       </c>
-      <c r="C71" s="19" t="n"/>
-      <c r="D71" s="19" t="n"/>
-      <c r="E71" s="20" t="n"/>
-    </row>
-    <row r="72" ht="20" customHeight="1">
-      <c r="B72" s="21" t="inlineStr">
+      <c r="C74" s="21" t="n"/>
+      <c r="D74" s="21" t="n"/>
+      <c r="E74" s="22" t="n"/>
+    </row>
+    <row r="75" ht="20" customHeight="1">
+      <c r="B75" s="23" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C72" s="22" t="n"/>
-      <c r="D72" s="22" t="n"/>
-      <c r="E72" s="23" t="n"/>
-    </row>
-    <row r="73" ht="49.5" customHeight="1">
-      <c r="B73" s="24" t="inlineStr">
+      <c r="C75" s="24" t="n"/>
+      <c r="D75" s="24" t="n"/>
+      <c r="E75" s="25" t="n"/>
+    </row>
+    <row r="76" ht="49.5" customHeight="1">
+      <c r="B76" s="26" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C73" s="25" t="inlineStr">
+      <c r="C76" s="27" t="inlineStr">
         <is>
           <t>La urna biodegradable se entierra directamente en el suelo, se cubre con tierra y se descompone integrándose a la naturaleza. Jardín con agua corriente y área de esparcimiento de cenizas.</t>
         </is>
       </c>
-      <c r="D73" s="26" t="n"/>
-      <c r="E73" s="27" t="n"/>
-    </row>
-    <row r="74" ht="20.5" customHeight="1">
-      <c r="B74" s="28" t="inlineStr">
+      <c r="D76" s="28" t="n"/>
+      <c r="E76" s="29" t="n"/>
+    </row>
+    <row r="77" ht="20.5" customHeight="1">
+      <c r="B77" s="30" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C74" s="29" t="inlineStr">
+      <c r="C77" s="31" t="inlineStr">
         <is>
           <t>Individual (1 urna).</t>
         </is>
       </c>
-      <c r="D74" s="30" t="n"/>
-      <c r="E74" s="31" t="n"/>
-    </row>
-    <row r="75" ht="20" customHeight="1">
-      <c r="B75" s="21" t="inlineStr">
+      <c r="D77" s="32" t="n"/>
+      <c r="E77" s="33" t="n"/>
+    </row>
+    <row r="78" ht="20" customHeight="1">
+      <c r="B78" s="23" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C75" s="22" t="n"/>
-      <c r="D75" s="22" t="n"/>
-      <c r="E75" s="23" t="n"/>
-    </row>
-    <row r="76" ht="20.5" customHeight="1">
-      <c r="B76" s="24" t="inlineStr">
+      <c r="C78" s="24" t="n"/>
+      <c r="D78" s="24" t="n"/>
+      <c r="E78" s="25" t="n"/>
+    </row>
+    <row r="79" ht="20.5" customHeight="1">
+      <c r="B79" s="26" t="inlineStr">
         <is>
           <t>Ambientes</t>
         </is>
       </c>
-      <c r="C76" s="25" t="inlineStr">
+      <c r="C79" s="27" t="inlineStr">
         <is>
           <t>Jardín 2 · Ecológico o Bosque de las Orquídeas</t>
         </is>
       </c>
-      <c r="D76" s="26" t="n"/>
-      <c r="E76" s="27" t="n"/>
-    </row>
-    <row r="77" ht="20.5" customHeight="1">
-      <c r="B77" s="28" t="inlineStr">
+      <c r="D79" s="28" t="n"/>
+      <c r="E79" s="29" t="n"/>
+    </row>
+    <row r="80" ht="20.5" customHeight="1">
+      <c r="B80" s="30" t="inlineStr">
         <is>
           <t>Espacio por urna</t>
         </is>
       </c>
-      <c r="C77" s="29" t="inlineStr">
+      <c r="C80" s="31" t="inlineStr">
         <is>
           <t>30 × 30 cm, 40 cm de profundidad</t>
         </is>
       </c>
-      <c r="D77" s="30" t="n"/>
-      <c r="E77" s="31" t="n"/>
-    </row>
-    <row r="78" ht="20.5" customHeight="1">
-      <c r="B78" s="24" t="inlineStr">
+      <c r="D80" s="32" t="n"/>
+      <c r="E80" s="33" t="n"/>
+    </row>
+    <row r="81" ht="20.5" customHeight="1">
+      <c r="B81" s="26" t="inlineStr">
         <is>
           <t>Urna</t>
         </is>
       </c>
-      <c r="C78" s="25" t="inlineStr">
+      <c r="C81" s="27" t="inlineStr">
         <is>
           <t>Biodegradable; se integra al suelo</t>
         </is>
       </c>
-      <c r="D78" s="26" t="n"/>
-      <c r="E78" s="27" t="n"/>
-    </row>
-    <row r="79" ht="35" customHeight="1">
-      <c r="B79" s="28" t="inlineStr">
+      <c r="D81" s="28" t="n"/>
+      <c r="E81" s="29" t="n"/>
+    </row>
+    <row r="82" ht="35" customHeight="1">
+      <c r="B82" s="30" t="inlineStr">
         <is>
           <t>Identificación (Jardín 2)</t>
         </is>
       </c>
-      <c r="C79" s="29" t="inlineStr">
+      <c r="C82" s="31" t="inlineStr">
         <is>
           <t>Placa de madera de 20 cm fijada a una varilla metálica, en posición vertical y sin contacto con el suelo</t>
         </is>
       </c>
-      <c r="D79" s="30" t="n"/>
-      <c r="E79" s="31" t="n"/>
-    </row>
-    <row r="80" ht="20.5" customHeight="1">
-      <c r="B80" s="24" t="inlineStr">
+      <c r="D82" s="32" t="n"/>
+      <c r="E82" s="33" t="n"/>
+    </row>
+    <row r="83" ht="20.5" customHeight="1">
+      <c r="B83" s="26" t="inlineStr">
         <is>
           <t>Identificación (Bosque)</t>
         </is>
       </c>
-      <c r="C80" s="25" t="inlineStr">
+      <c r="C83" s="27" t="inlineStr">
         <is>
           <t>Placa de mármol de 20 × 15 cm</t>
         </is>
       </c>
-      <c r="D80" s="26" t="n"/>
-      <c r="E80" s="27" t="n"/>
-    </row>
-    <row r="81" ht="35" customHeight="1">
-      <c r="B81" s="28" t="inlineStr">
+      <c r="D83" s="28" t="n"/>
+      <c r="E83" s="29" t="n"/>
+    </row>
+    <row r="84" ht="35" customHeight="1">
+      <c r="B84" s="30" t="inlineStr">
         <is>
           <t>Permanencia</t>
         </is>
       </c>
-      <c r="C81" s="29" t="inlineStr">
+      <c r="C84" s="31" t="inlineStr">
         <is>
           <t>3 años; luego el nombre pasa a una placa memorial en el monumento y el espacio se reutiliza</t>
         </is>
       </c>
-      <c r="D81" s="30" t="n"/>
-      <c r="E81" s="31" t="n"/>
-    </row>
-    <row r="82" ht="20.5" customHeight="1">
-      <c r="B82" s="24" t="inlineStr">
+      <c r="D84" s="32" t="n"/>
+      <c r="E84" s="33" t="n"/>
+    </row>
+    <row r="85" ht="20.5" customHeight="1">
+      <c r="B85" s="26" t="inlineStr">
         <is>
           <t>Placa memorial</t>
         </is>
       </c>
-      <c r="C82" s="25" t="inlineStr">
+      <c r="C85" s="27" t="inlineStr">
         <is>
           <t>Incluida en el precio</t>
         </is>
       </c>
-      <c r="D82" s="26" t="n"/>
-      <c r="E82" s="27" t="n"/>
-    </row>
-    <row r="83" ht="20.5" customHeight="1">
-      <c r="B83" s="28" t="inlineStr">
+      <c r="D85" s="28" t="n"/>
+      <c r="E85" s="29" t="n"/>
+    </row>
+    <row r="86" ht="20.5" customHeight="1">
+      <c r="B86" s="30" t="inlineStr">
         <is>
           <t>Acceso</t>
         </is>
       </c>
-      <c r="C83" s="29" t="inlineStr">
+      <c r="C86" s="31" t="inlineStr">
         <is>
           <t>Camino de 1,2 m en gravilla con bordillo prefabricado</t>
         </is>
       </c>
-      <c r="D83" s="30" t="n"/>
-      <c r="E83" s="31" t="n"/>
-    </row>
-    <row r="84" ht="78.5" customHeight="1">
-      <c r="B84" s="24" t="inlineStr">
+      <c r="D86" s="32" t="n"/>
+      <c r="E86" s="33" t="n"/>
+    </row>
+    <row r="87" ht="78.5" customHeight="1">
+      <c r="B87" s="26" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C84" s="25" t="inlineStr">
+      <c r="C87" s="27" t="inlineStr">
         <is>
           <t>• Inhumación ecológica de la urna directamente en el suelo
 • Placa de identificación
@@ -2190,258 +2220,258 @@
 • Permanencia de 3 años; luego, placa memorial en el monumento (incluida)</t>
         </is>
       </c>
-      <c r="D84" s="26" t="n"/>
-      <c r="E84" s="27" t="n"/>
-    </row>
-    <row r="85" ht="20" customHeight="1">
-      <c r="B85" s="21" t="inlineStr">
+      <c r="D87" s="28" t="n"/>
+      <c r="E87" s="29" t="n"/>
+    </row>
+    <row r="88" ht="20" customHeight="1">
+      <c r="B88" s="23" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C85" s="22" t="n"/>
-      <c r="D85" s="22" t="n"/>
-      <c r="E85" s="23" t="n"/>
-    </row>
-    <row r="86" ht="26.5" customHeight="1">
-      <c r="B86" s="24" t="inlineStr">
+      <c r="C88" s="24" t="n"/>
+      <c r="D88" s="24" t="n"/>
+      <c r="E88" s="25" t="n"/>
+    </row>
+    <row r="89" ht="26.5" customHeight="1">
+      <c r="B89" s="26" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C86" s="32" t="inlineStr">
+      <c r="C89" s="34" t="inlineStr">
         <is>
           <t>US$ 750</t>
         </is>
       </c>
-      <c r="D86" s="26" t="n"/>
-      <c r="E86" s="27" t="n"/>
-    </row>
-    <row r="87" ht="26.5" customHeight="1">
-      <c r="B87" s="28" t="inlineStr">
+      <c r="D89" s="28" t="n"/>
+      <c r="E89" s="29" t="n"/>
+    </row>
+    <row r="90" ht="26.5" customHeight="1">
+      <c r="B90" s="30" t="inlineStr">
         <is>
           <t>Precio lanzamiento (−20%)</t>
         </is>
       </c>
-      <c r="C87" s="33" t="inlineStr">
+      <c r="C90" s="35" t="inlineStr">
         <is>
           <t>US$ 600</t>
         </is>
       </c>
-      <c r="D87" s="30" t="n"/>
-      <c r="E87" s="31" t="n"/>
-    </row>
-    <row r="88" ht="20.5" customHeight="1">
-      <c r="B88" s="28" t="inlineStr">
+      <c r="D90" s="32" t="n"/>
+      <c r="E90" s="33" t="n"/>
+    </row>
+    <row r="91" ht="20.5" customHeight="1">
+      <c r="B91" s="30" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C88" s="29" t="inlineStr">
+      <c r="C91" s="31" t="inlineStr">
         <is>
           <t>Por espacio individual · placa memorial incluida</t>
         </is>
       </c>
-      <c r="D88" s="30" t="n"/>
-      <c r="E88" s="31" t="n"/>
-    </row>
-    <row r="89" ht="35" customHeight="1">
-      <c r="B89" s="24" t="inlineStr">
+      <c r="D91" s="32" t="n"/>
+      <c r="E91" s="33" t="n"/>
+    </row>
+    <row r="92" ht="35" customHeight="1">
+      <c r="B92" s="26" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C89" s="25" t="inlineStr">
+      <c r="C92" s="27" t="inlineStr">
         <is>
           <t>Pago único o financiado según política comercial vigente. Incluye la placa memorial en el monumento al término del plazo.</t>
         </is>
       </c>
-      <c r="D89" s="26" t="n"/>
-      <c r="E89" s="27" t="n"/>
-    </row>
-    <row r="90" ht="20" customHeight="1">
-      <c r="B90" s="21" t="inlineStr">
+      <c r="D92" s="28" t="n"/>
+      <c r="E92" s="29" t="n"/>
+    </row>
+    <row r="93" ht="20" customHeight="1">
+      <c r="B93" s="23" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C90" s="22" t="n"/>
-      <c r="D90" s="22" t="n"/>
-      <c r="E90" s="23" t="n"/>
-    </row>
-    <row r="91" ht="35" customHeight="1">
-      <c r="B91" s="34" t="inlineStr">
+      <c r="C93" s="24" t="n"/>
+      <c r="D93" s="24" t="n"/>
+      <c r="E93" s="25" t="n"/>
+    </row>
+    <row r="94" ht="35" customHeight="1">
+      <c r="B94" s="36" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C91" s="35" t="inlineStr">
+      <c r="C94" s="37" t="inlineStr">
         <is>
           <t>Personas con conciencia ambiental que desean que sus cenizas vuelvan a la tierra, con un lugar identificado para visitar.</t>
         </is>
       </c>
-      <c r="D91" s="36" t="n"/>
-      <c r="E91" s="37" t="n"/>
-    </row>
-    <row r="94" ht="30" customHeight="1">
-      <c r="B94" s="15" t="inlineStr">
+      <c r="D94" s="38" t="n"/>
+      <c r="E94" s="39" t="n"/>
+    </row>
+    <row r="97" ht="30" customHeight="1">
+      <c r="B97" s="17" t="inlineStr">
         <is>
           <t>JARDÍN DE MASCOTAS</t>
         </is>
       </c>
-      <c r="C94" s="16" t="n"/>
-      <c r="D94" s="16" t="n"/>
-      <c r="E94" s="17" t="n"/>
-    </row>
-    <row r="95" ht="20" customHeight="1">
-      <c r="B95" s="18" t="inlineStr">
+      <c r="C97" s="18" t="n"/>
+      <c r="D97" s="18" t="n"/>
+      <c r="E97" s="19" t="n"/>
+    </row>
+    <row r="98" ht="20" customHeight="1">
+      <c r="B98" s="20" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Mascotas  ·  Destino final · Inhumación ecológica</t>
         </is>
       </c>
-      <c r="C95" s="19" t="n"/>
-      <c r="D95" s="19" t="n"/>
-      <c r="E95" s="20" t="n"/>
-    </row>
-    <row r="96" ht="20" customHeight="1">
-      <c r="B96" s="21" t="inlineStr">
+      <c r="C98" s="21" t="n"/>
+      <c r="D98" s="21" t="n"/>
+      <c r="E98" s="22" t="n"/>
+    </row>
+    <row r="99" ht="20" customHeight="1">
+      <c r="B99" s="23" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C96" s="22" t="n"/>
-      <c r="D96" s="22" t="n"/>
-      <c r="E96" s="23" t="n"/>
-    </row>
-    <row r="97" ht="35" customHeight="1">
-      <c r="B97" s="24" t="inlineStr">
+      <c r="C99" s="24" t="n"/>
+      <c r="D99" s="24" t="n"/>
+      <c r="E99" s="25" t="n"/>
+    </row>
+    <row r="100" ht="35" customHeight="1">
+      <c r="B100" s="26" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C97" s="25" t="inlineStr">
+      <c r="C100" s="27" t="inlineStr">
         <is>
           <t>Jardín para inhumación ecológica de cenizas de mascotas: la urna biodegradable se entierra directamente en el suelo y se identifica con una placa de madera.</t>
         </is>
       </c>
-      <c r="D97" s="26" t="n"/>
-      <c r="E97" s="27" t="n"/>
-    </row>
-    <row r="98" ht="20.5" customHeight="1">
-      <c r="B98" s="28" t="inlineStr">
+      <c r="D100" s="28" t="n"/>
+      <c r="E100" s="29" t="n"/>
+    </row>
+    <row r="101" ht="20.5" customHeight="1">
+      <c r="B101" s="30" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C98" s="29" t="inlineStr">
+      <c r="C101" s="31" t="inlineStr">
         <is>
           <t>Individual (una mascota por servicio).</t>
         </is>
       </c>
-      <c r="D98" s="30" t="n"/>
-      <c r="E98" s="31" t="n"/>
-    </row>
-    <row r="99" ht="20" customHeight="1">
-      <c r="B99" s="21" t="inlineStr">
+      <c r="D101" s="32" t="n"/>
+      <c r="E101" s="33" t="n"/>
+    </row>
+    <row r="102" ht="20" customHeight="1">
+      <c r="B102" s="23" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C99" s="22" t="n"/>
-      <c r="D99" s="22" t="n"/>
-      <c r="E99" s="23" t="n"/>
-    </row>
-    <row r="100" ht="20.5" customHeight="1">
-      <c r="B100" s="24" t="inlineStr">
+      <c r="C102" s="24" t="n"/>
+      <c r="D102" s="24" t="n"/>
+      <c r="E102" s="25" t="n"/>
+    </row>
+    <row r="103" ht="20.5" customHeight="1">
+      <c r="B103" s="26" t="inlineStr">
         <is>
           <t>Tipo de producto</t>
         </is>
       </c>
-      <c r="C100" s="25" t="inlineStr">
+      <c r="C103" s="27" t="inlineStr">
         <is>
           <t>Servicio de pago único</t>
         </is>
       </c>
-      <c r="D100" s="26" t="n"/>
-      <c r="E100" s="27" t="n"/>
-    </row>
-    <row r="101" ht="20.5" customHeight="1">
-      <c r="B101" s="28" t="inlineStr">
+      <c r="D103" s="28" t="n"/>
+      <c r="E103" s="29" t="n"/>
+    </row>
+    <row r="104" ht="20.5" customHeight="1">
+      <c r="B104" s="30" t="inlineStr">
         <is>
           <t>Espacio por urna</t>
         </is>
       </c>
-      <c r="C101" s="29" t="inlineStr">
+      <c r="C104" s="31" t="inlineStr">
         <is>
           <t>15 × 20 cm o 15 × 30 cm, según el tamaño de la urna</t>
         </is>
       </c>
-      <c r="D101" s="30" t="n"/>
-      <c r="E101" s="31" t="n"/>
-    </row>
-    <row r="102" ht="35" customHeight="1">
-      <c r="B102" s="24" t="inlineStr">
+      <c r="D104" s="32" t="n"/>
+      <c r="E104" s="33" t="n"/>
+    </row>
+    <row r="105" ht="35" customHeight="1">
+      <c r="B105" s="26" t="inlineStr">
         <is>
           <t>Urna</t>
         </is>
       </c>
-      <c r="C102" s="25" t="inlineStr">
+      <c r="C105" s="27" t="inlineStr">
         <is>
           <t>Biodegradable; se integra al suelo. Incluida solo en la opción con cremación (US$ 550); con solo espacio (US$ 400) se adquiere por separado</t>
         </is>
       </c>
-      <c r="D102" s="26" t="n"/>
-      <c r="E102" s="27" t="n"/>
-    </row>
-    <row r="103" ht="20.5" customHeight="1">
-      <c r="B103" s="28" t="inlineStr">
+      <c r="D105" s="28" t="n"/>
+      <c r="E105" s="29" t="n"/>
+    </row>
+    <row r="106" ht="20.5" customHeight="1">
+      <c r="B106" s="30" t="inlineStr">
         <is>
           <t>Identificación</t>
         </is>
       </c>
-      <c r="C103" s="29" t="inlineStr">
+      <c r="C106" s="31" t="inlineStr">
         <is>
           <t>Placa de madera de 20 cm</t>
         </is>
       </c>
-      <c r="D103" s="30" t="n"/>
-      <c r="E103" s="31" t="n"/>
-    </row>
-    <row r="104" ht="20.5" customHeight="1">
-      <c r="B104" s="24" t="inlineStr">
+      <c r="D106" s="32" t="n"/>
+      <c r="E106" s="33" t="n"/>
+    </row>
+    <row r="107" ht="20.5" customHeight="1">
+      <c r="B107" s="26" t="inlineStr">
         <is>
           <t>Permanencia</t>
         </is>
       </c>
-      <c r="C104" s="25" t="inlineStr">
+      <c r="C107" s="27" t="inlineStr">
         <is>
           <t>3 años; luego el espacio se reutiliza</t>
         </is>
       </c>
-      <c r="D104" s="26" t="n"/>
-      <c r="E104" s="27" t="n"/>
-    </row>
-    <row r="105" ht="20.5" customHeight="1">
-      <c r="B105" s="28" t="inlineStr">
+      <c r="D107" s="28" t="n"/>
+      <c r="E107" s="29" t="n"/>
+    </row>
+    <row r="108" ht="20.5" customHeight="1">
+      <c r="B108" s="30" t="inlineStr">
         <is>
           <t>Placa memorial</t>
         </is>
       </c>
-      <c r="C105" s="29" t="inlineStr">
+      <c r="C108" s="31" t="inlineStr">
         <is>
           <t>Incluida en el precio; en el monumento al término del plazo</t>
         </is>
       </c>
-      <c r="D105" s="30" t="n"/>
-      <c r="E105" s="31" t="n"/>
-    </row>
-    <row r="106" ht="64" customHeight="1">
-      <c r="B106" s="24" t="inlineStr">
+      <c r="D108" s="32" t="n"/>
+      <c r="E108" s="33" t="n"/>
+    </row>
+    <row r="109" ht="64" customHeight="1">
+      <c r="B109" s="26" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C106" s="25" t="inlineStr">
+      <c r="C109" s="27" t="inlineStr">
         <is>
           <t>• Inhumación ecológica de la urna en el jardín
 • Placa de madera de 20 cm para identificación
@@ -2449,652 +2479,497 @@
 • Cremación de la mascota y urna biodegradable (opción US$ 550)</t>
         </is>
       </c>
-      <c r="D106" s="26" t="n"/>
-      <c r="E106" s="27" t="n"/>
-    </row>
-    <row r="107" ht="20" customHeight="1">
-      <c r="B107" s="21" t="inlineStr">
+      <c r="D109" s="28" t="n"/>
+      <c r="E109" s="29" t="n"/>
+    </row>
+    <row r="110" ht="20" customHeight="1">
+      <c r="B110" s="23" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C107" s="22" t="n"/>
-      <c r="D107" s="22" t="n"/>
-      <c r="E107" s="23" t="n"/>
-    </row>
-    <row r="108" ht="26.5" customHeight="1">
-      <c r="B108" s="24" t="inlineStr">
+      <c r="C110" s="24" t="n"/>
+      <c r="D110" s="24" t="n"/>
+      <c r="E110" s="25" t="n"/>
+    </row>
+    <row r="111" ht="26.5" customHeight="1">
+      <c r="B111" s="26" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C108" s="32" t="inlineStr">
+      <c r="C111" s="34" t="inlineStr">
         <is>
           <t>US$ 400 / US$ 550</t>
         </is>
       </c>
-      <c r="D108" s="26" t="n"/>
-      <c r="E108" s="27" t="n"/>
-    </row>
-    <row r="109" ht="26.5" customHeight="1">
-      <c r="B109" s="28" t="inlineStr">
+      <c r="D111" s="28" t="n"/>
+      <c r="E111" s="29" t="n"/>
+    </row>
+    <row r="112" ht="26.5" customHeight="1">
+      <c r="B112" s="30" t="inlineStr">
         <is>
           <t>Precio lanzamiento (−20%)</t>
         </is>
       </c>
-      <c r="C109" s="33" t="inlineStr">
+      <c r="C112" s="35" t="inlineStr">
         <is>
           <t>US$ 320 / US$ 440</t>
         </is>
       </c>
-      <c r="D109" s="30" t="n"/>
-      <c r="E109" s="31" t="n"/>
-    </row>
-    <row r="110" ht="20.5" customHeight="1">
-      <c r="B110" s="28" t="inlineStr">
+      <c r="D112" s="32" t="n"/>
+      <c r="E112" s="33" t="n"/>
+    </row>
+    <row r="113" ht="20.5" customHeight="1">
+      <c r="B113" s="30" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C110" s="29" t="inlineStr">
+      <c r="C113" s="31" t="inlineStr">
         <is>
           <t>US$ 400 solo espacio (urna aparte) · US$ 550 con cremación y urna</t>
         </is>
       </c>
-      <c r="D110" s="30" t="n"/>
-      <c r="E110" s="31" t="n"/>
-    </row>
-    <row r="111" ht="49.5" customHeight="1">
-      <c r="B111" s="24" t="inlineStr">
+      <c r="D113" s="32" t="n"/>
+      <c r="E113" s="33" t="n"/>
+    </row>
+    <row r="114" ht="49.5" customHeight="1">
+      <c r="B114" s="26" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C111" s="25" t="inlineStr">
+      <c r="C114" s="27" t="inlineStr">
         <is>
           <t>Pago único; puede contratarse como adicional al plan funerario. La opción de US$ 550 incluye la cremación de la mascota y la urna biodegradable; en la opción de US$ 400 (solo espacio) la urna biodegradable se adquiere por separado.</t>
         </is>
       </c>
-      <c r="D111" s="26" t="n"/>
-      <c r="E111" s="27" t="n"/>
-    </row>
-    <row r="112" ht="20" customHeight="1">
-      <c r="B112" s="21" t="inlineStr">
+      <c r="D114" s="28" t="n"/>
+      <c r="E114" s="29" t="n"/>
+    </row>
+    <row r="115" ht="20" customHeight="1">
+      <c r="B115" s="23" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C112" s="22" t="n"/>
-      <c r="D112" s="22" t="n"/>
-      <c r="E112" s="23" t="n"/>
-    </row>
-    <row r="113" ht="20.5" customHeight="1">
-      <c r="B113" s="34" t="inlineStr">
+      <c r="C115" s="24" t="n"/>
+      <c r="D115" s="24" t="n"/>
+      <c r="E115" s="25" t="n"/>
+    </row>
+    <row r="116" ht="20.5" customHeight="1">
+      <c r="B116" s="36" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C113" s="35" t="inlineStr">
+      <c r="C116" s="37" t="inlineStr">
         <is>
           <t>Familias que consideran a su mascota parte del hogar y desean un cierre digno.</t>
         </is>
       </c>
-      <c r="D113" s="36" t="n"/>
-      <c r="E113" s="37" t="n"/>
-    </row>
-    <row r="116" ht="30" customHeight="1">
-      <c r="B116" s="15" t="inlineStr">
+      <c r="D116" s="38" t="n"/>
+      <c r="E116" s="39" t="n"/>
+    </row>
+    <row r="119" ht="30" customHeight="1">
+      <c r="B119" s="17" t="inlineStr">
         <is>
           <t>JARDÍN DE CENIZAS · CEREMONIAL</t>
         </is>
       </c>
-      <c r="C116" s="16" t="n"/>
-      <c r="D116" s="16" t="n"/>
-      <c r="E116" s="17" t="n"/>
-    </row>
-    <row r="117" ht="20" customHeight="1">
-      <c r="B117" s="18" t="inlineStr">
+      <c r="C119" s="18" t="n"/>
+      <c r="D119" s="18" t="n"/>
+      <c r="E119" s="19" t="n"/>
+    </row>
+    <row r="120" ht="20" customHeight="1">
+      <c r="B120" s="20" t="inlineStr">
         <is>
           <t>Jardines de la Memoria · Jardín 3  ·  Destino final · Inhumación con ceremonia</t>
         </is>
       </c>
-      <c r="C117" s="19" t="n"/>
-      <c r="D117" s="19" t="n"/>
-      <c r="E117" s="20" t="n"/>
-    </row>
-    <row r="118" ht="24" customHeight="1">
-      <c r="B118" s="38" t="inlineStr">
+      <c r="C120" s="21" t="n"/>
+      <c r="D120" s="21" t="n"/>
+      <c r="E120" s="22" t="n"/>
+    </row>
+    <row r="121" ht="24" customHeight="1">
+      <c r="B121" s="40" t="inlineStr">
         <is>
           <t>★  PRÓXIMO LANZAMIENTO · se lanzará en otro momento</t>
         </is>
       </c>
-      <c r="C118" s="39" t="n"/>
-      <c r="D118" s="39" t="n"/>
-      <c r="E118" s="40" t="n"/>
-    </row>
-    <row r="119" ht="20" customHeight="1">
-      <c r="B119" s="21" t="inlineStr">
+      <c r="C121" s="41" t="n"/>
+      <c r="D121" s="41" t="n"/>
+      <c r="E121" s="42" t="n"/>
+    </row>
+    <row r="122" ht="20" customHeight="1">
+      <c r="B122" s="23" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C119" s="22" t="n"/>
-      <c r="D119" s="22" t="n"/>
-      <c r="E119" s="23" t="n"/>
-    </row>
-    <row r="120" ht="35" customHeight="1">
-      <c r="B120" s="24" t="inlineStr">
+      <c r="C122" s="24" t="n"/>
+      <c r="D122" s="24" t="n"/>
+      <c r="E122" s="25" t="n"/>
+    </row>
+    <row r="123" ht="35" customHeight="1">
+      <c r="B123" s="26" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C120" s="25" t="inlineStr">
+      <c r="C123" s="27" t="inlineStr">
         <is>
           <t>Jardín para inhumación de urnas de cenizas con ceremonia de agua, con fuentes como elemento central del rito de despedida.</t>
         </is>
       </c>
-      <c r="D120" s="26" t="n"/>
-      <c r="E120" s="27" t="n"/>
-    </row>
-    <row r="121" ht="20.5" customHeight="1">
-      <c r="B121" s="28" t="inlineStr">
+      <c r="D123" s="28" t="n"/>
+      <c r="E123" s="29" t="n"/>
+    </row>
+    <row r="124" ht="20.5" customHeight="1">
+      <c r="B124" s="30" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C121" s="29" t="inlineStr">
+      <c r="C124" s="31" t="inlineStr">
         <is>
           <t>A definir.</t>
         </is>
       </c>
-      <c r="D121" s="30" t="n"/>
-      <c r="E121" s="31" t="n"/>
-    </row>
-    <row r="122" ht="20" customHeight="1">
-      <c r="B122" s="21" t="inlineStr">
+      <c r="D124" s="32" t="n"/>
+      <c r="E124" s="33" t="n"/>
+    </row>
+    <row r="125" ht="20" customHeight="1">
+      <c r="B125" s="23" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C122" s="22" t="n"/>
-      <c r="D122" s="22" t="n"/>
-      <c r="E122" s="23" t="n"/>
-    </row>
-    <row r="123" ht="20.5" customHeight="1">
-      <c r="B123" s="24" t="inlineStr">
+      <c r="C125" s="24" t="n"/>
+      <c r="D125" s="24" t="n"/>
+      <c r="E125" s="25" t="n"/>
+    </row>
+    <row r="126" ht="20.5" customHeight="1">
+      <c r="B126" s="26" t="inlineStr">
         <is>
           <t>Ambiente</t>
         </is>
       </c>
-      <c r="C123" s="25" t="inlineStr">
+      <c r="C126" s="27" t="inlineStr">
         <is>
           <t>Jardín 3</t>
         </is>
       </c>
-      <c r="D123" s="26" t="n"/>
-      <c r="E123" s="27" t="n"/>
-    </row>
-    <row r="124" ht="20.5" customHeight="1">
-      <c r="B124" s="28" t="inlineStr">
+      <c r="D126" s="28" t="n"/>
+      <c r="E126" s="29" t="n"/>
+    </row>
+    <row r="127" ht="20.5" customHeight="1">
+      <c r="B127" s="30" t="inlineStr">
         <is>
           <t>Elemento central</t>
         </is>
       </c>
-      <c r="C124" s="29" t="inlineStr">
+      <c r="C127" s="31" t="inlineStr">
         <is>
           <t>Fuente de agua para la ceremonia</t>
         </is>
       </c>
-      <c r="D124" s="30" t="n"/>
-      <c r="E124" s="31" t="n"/>
-    </row>
-    <row r="125" ht="20.5" customHeight="1">
-      <c r="B125" s="24" t="inlineStr">
+      <c r="D127" s="32" t="n"/>
+      <c r="E127" s="33" t="n"/>
+    </row>
+    <row r="128" ht="20.5" customHeight="1">
+      <c r="B128" s="26" t="inlineStr">
         <is>
           <t>Entorno</t>
         </is>
       </c>
-      <c r="C125" s="25" t="inlineStr">
+      <c r="C128" s="27" t="inlineStr">
         <is>
           <t>Barrera visual que separa el jardín del crematorio</t>
         </is>
       </c>
-      <c r="D125" s="26" t="n"/>
-      <c r="E125" s="27" t="n"/>
-    </row>
-    <row r="126" ht="35" customHeight="1">
-      <c r="B126" s="28" t="inlineStr">
+      <c r="D128" s="28" t="n"/>
+      <c r="E128" s="29" t="n"/>
+    </row>
+    <row r="129" ht="35" customHeight="1">
+      <c r="B129" s="30" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C126" s="29" t="inlineStr">
+      <c r="C129" s="31" t="inlineStr">
         <is>
           <t>• Inhumación de urnas de cenizas
 • Ceremonia con agua en fuente</t>
         </is>
       </c>
-      <c r="D126" s="30" t="n"/>
-      <c r="E126" s="31" t="n"/>
-    </row>
-    <row r="127" ht="20" customHeight="1">
-      <c r="B127" s="21" t="inlineStr">
+      <c r="D129" s="32" t="n"/>
+      <c r="E129" s="33" t="n"/>
+    </row>
+    <row r="130" ht="20" customHeight="1">
+      <c r="B130" s="23" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C127" s="22" t="n"/>
-      <c r="D127" s="22" t="n"/>
-      <c r="E127" s="23" t="n"/>
-    </row>
-    <row r="128" ht="26.5" customHeight="1">
-      <c r="B128" s="24" t="inlineStr">
+      <c r="C130" s="24" t="n"/>
+      <c r="D130" s="24" t="n"/>
+      <c r="E130" s="25" t="n"/>
+    </row>
+    <row r="131" ht="26.5" customHeight="1">
+      <c r="B131" s="26" t="inlineStr">
         <is>
           <t>Precio sugerido</t>
         </is>
       </c>
-      <c r="C128" s="32" t="inlineStr">
+      <c r="C131" s="34" t="inlineStr">
         <is>
           <t>A definir</t>
         </is>
       </c>
-      <c r="D128" s="26" t="n"/>
-      <c r="E128" s="27" t="n"/>
-    </row>
-    <row r="129" ht="26.5" customHeight="1">
-      <c r="B129" s="28" t="inlineStr">
+      <c r="D131" s="28" t="n"/>
+      <c r="E131" s="29" t="n"/>
+    </row>
+    <row r="132" ht="26.5" customHeight="1">
+      <c r="B132" s="30" t="inlineStr">
         <is>
           <t>Precio lanzamiento (−20%)</t>
         </is>
       </c>
-      <c r="C129" s="33" t="inlineStr">
+      <c r="C132" s="35" t="inlineStr">
         <is>
           <t>A definir</t>
         </is>
       </c>
-      <c r="D129" s="30" t="n"/>
-      <c r="E129" s="31" t="n"/>
-    </row>
-    <row r="130" ht="20.5" customHeight="1">
-      <c r="B130" s="28" t="inlineStr">
+      <c r="D132" s="32" t="n"/>
+      <c r="E132" s="33" t="n"/>
+    </row>
+    <row r="133" ht="20.5" customHeight="1">
+      <c r="B133" s="30" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C130" s="29" t="inlineStr">
+      <c r="C133" s="31" t="inlineStr">
         <is>
           <t>Producto en definición</t>
         </is>
       </c>
-      <c r="D130" s="30" t="n"/>
-      <c r="E130" s="31" t="n"/>
-    </row>
-    <row r="131" ht="20.5" customHeight="1">
-      <c r="B131" s="24" t="inlineStr">
+      <c r="D133" s="32" t="n"/>
+      <c r="E133" s="33" t="n"/>
+    </row>
+    <row r="134" ht="20.5" customHeight="1">
+      <c r="B134" s="26" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C131" s="25" t="inlineStr">
+      <c r="C134" s="27" t="inlineStr">
         <is>
           <t>A definir.</t>
         </is>
       </c>
-      <c r="D131" s="26" t="n"/>
-      <c r="E131" s="27" t="n"/>
-    </row>
-    <row r="132" ht="20" customHeight="1">
-      <c r="B132" s="21" t="inlineStr">
+      <c r="D134" s="28" t="n"/>
+      <c r="E134" s="29" t="n"/>
+    </row>
+    <row r="135" ht="20" customHeight="1">
+      <c r="B135" s="23" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C132" s="22" t="n"/>
-      <c r="D132" s="22" t="n"/>
-      <c r="E132" s="23" t="n"/>
-    </row>
-    <row r="133" ht="35" customHeight="1">
-      <c r="B133" s="34" t="inlineStr">
+      <c r="C135" s="24" t="n"/>
+      <c r="D135" s="24" t="n"/>
+      <c r="E135" s="25" t="n"/>
+    </row>
+    <row r="136" ht="35" customHeight="1">
+      <c r="B136" s="36" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C133" s="35" t="inlineStr">
+      <c r="C136" s="37" t="inlineStr">
         <is>
           <t>Familias que valoran un rito de despedida simbólico y un entorno contemplativo.</t>
         </is>
       </c>
-      <c r="D133" s="36" t="n"/>
-      <c r="E133" s="37" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="122">
-    <mergeCell ref="C31:E31"/>
-    <mergeCell ref="C80:E80"/>
-    <mergeCell ref="C40:E40"/>
-    <mergeCell ref="C129:E129"/>
-    <mergeCell ref="C51:E51"/>
-    <mergeCell ref="C60:E60"/>
-    <mergeCell ref="C123:E123"/>
-    <mergeCell ref="C7:E7"/>
-    <mergeCell ref="C91:E91"/>
-    <mergeCell ref="C57:E57"/>
-    <mergeCell ref="B21:E21"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="B39:E39"/>
-    <mergeCell ref="C101:E101"/>
-    <mergeCell ref="C77:E77"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="C42:E42"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="C74:E74"/>
-    <mergeCell ref="C126:E126"/>
-    <mergeCell ref="B112:E112"/>
-    <mergeCell ref="C128:E128"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="C113:E113"/>
-    <mergeCell ref="C103:E103"/>
-    <mergeCell ref="B49:E49"/>
-    <mergeCell ref="C84:E84"/>
-    <mergeCell ref="C133:E133"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="C59:E59"/>
-    <mergeCell ref="C130:E130"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="B50:E50"/>
-    <mergeCell ref="C52:E52"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="B90:E90"/>
-    <mergeCell ref="C106:E106"/>
-    <mergeCell ref="C32:E32"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="B66:E66"/>
-    <mergeCell ref="C81:E81"/>
-    <mergeCell ref="C125:E125"/>
-    <mergeCell ref="B27:E27"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="C131:E131"/>
-    <mergeCell ref="C87:E87"/>
-    <mergeCell ref="B117:E117"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="B61:E61"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="C89:E89"/>
-    <mergeCell ref="C104:E104"/>
-    <mergeCell ref="B132:E132"/>
-    <mergeCell ref="B53:E53"/>
-    <mergeCell ref="B119:E119"/>
-    <mergeCell ref="C79:E79"/>
-    <mergeCell ref="C73:E73"/>
-    <mergeCell ref="C88:E88"/>
-    <mergeCell ref="B116:E116"/>
-    <mergeCell ref="C35:E35"/>
-    <mergeCell ref="C63:E63"/>
-    <mergeCell ref="C121:E121"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="B118:E118"/>
-    <mergeCell ref="B127:E127"/>
-    <mergeCell ref="C55:E55"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B95:E95"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="C11:E11"/>
-    <mergeCell ref="B72:E72"/>
-    <mergeCell ref="C67:E67"/>
-    <mergeCell ref="C109:E109"/>
-    <mergeCell ref="B122:E122"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="B71:E71"/>
-    <mergeCell ref="C37:E37"/>
-    <mergeCell ref="C78:E78"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B107:E107"/>
-    <mergeCell ref="C62:E62"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="C98:E98"/>
-    <mergeCell ref="B44:E44"/>
-    <mergeCell ref="C64:E64"/>
-    <mergeCell ref="B99:E99"/>
-    <mergeCell ref="C54:E54"/>
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="C41:E41"/>
-    <mergeCell ref="C124:E124"/>
-    <mergeCell ref="B30:E30"/>
-    <mergeCell ref="C56:E56"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="C105:E105"/>
-    <mergeCell ref="C43:E43"/>
-    <mergeCell ref="B85:E85"/>
-    <mergeCell ref="B94:E94"/>
-    <mergeCell ref="C76:E76"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="C120:E120"/>
-    <mergeCell ref="B75:E75"/>
-    <mergeCell ref="C110:E110"/>
-    <mergeCell ref="C8:E8"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="C82:E82"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="B96:E96"/>
-    <mergeCell ref="C102:E102"/>
-    <mergeCell ref="B70:E70"/>
-    <mergeCell ref="C111:E111"/>
-    <mergeCell ref="B48:E48"/>
-    <mergeCell ref="C86:E86"/>
-    <mergeCell ref="C83:E83"/>
-    <mergeCell ref="C108:E108"/>
-    <mergeCell ref="C58:E58"/>
-    <mergeCell ref="C45:E45"/>
-    <mergeCell ref="C97:E97"/>
-    <mergeCell ref="C29:E29"/>
-    <mergeCell ref="C100:E100"/>
-    <mergeCell ref="C65:E65"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
-  <rowBreaks count="5" manualBreakCount="5">
-    <brk id="23" min="0" max="16383" man="1"/>
-    <brk id="46" min="0" max="16383" man="1"/>
-    <brk id="68" min="0" max="16383" man="1"/>
-    <brk id="92" min="0" max="16383" man="1"/>
-    <brk id="114" min="0" max="16383" man="1"/>
-  </rowBreaks>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00C5A059"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="B1:E102"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="3" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="34" customHeight="1">
-      <c r="B1" s="13" t="inlineStr">
-        <is>
-          <t>PORTAFOLIO EXISTENTE DE CREMACIÓN  ·  LA AUXILIADORA · VANGRUPO</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="B2" s="14" t="inlineStr">
+      <c r="D136" s="38" t="n"/>
+      <c r="E136" s="39" t="n"/>
+    </row>
+    <row r="139" ht="30" customHeight="1">
+      <c r="B139" s="15" t="inlineStr">
+        <is>
+          <t>PORTAFOLIO EXISTENTE · COLUMBARIOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="20" customHeight="1">
+      <c r="B140" s="16" t="inlineStr">
         <is>
           <t>Columbarios y cremación · descuento −15% en Finados y noviembre</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="B4" s="15" t="inlineStr">
+    <row r="142" ht="30" customHeight="1">
+      <c r="B142" s="17" t="inlineStr">
         <is>
           <t>COLUMBARIO SUPREMO PLUS</t>
         </is>
       </c>
-      <c r="C4" s="16" t="n"/>
-      <c r="D4" s="16" t="n"/>
-      <c r="E4" s="17" t="n"/>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="B5" s="18" t="inlineStr">
+      <c r="C142" s="18" t="n"/>
+      <c r="D142" s="18" t="n"/>
+      <c r="E142" s="19" t="n"/>
+    </row>
+    <row r="143" ht="20" customHeight="1">
+      <c r="B143" s="20" t="inlineStr">
         <is>
           <t>El Hogar de las Memorias  ·  Servicio funerario + cremación + columbario</t>
         </is>
       </c>
-      <c r="C5" s="19" t="n"/>
-      <c r="D5" s="19" t="n"/>
-      <c r="E5" s="20" t="n"/>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="B6" s="21" t="inlineStr">
+      <c r="C143" s="21" t="n"/>
+      <c r="D143" s="21" t="n"/>
+      <c r="E143" s="22" t="n"/>
+    </row>
+    <row r="144" ht="20" customHeight="1">
+      <c r="B144" s="23" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C6" s="22" t="n"/>
-      <c r="D6" s="22" t="n"/>
-      <c r="E6" s="23" t="n"/>
-    </row>
-    <row r="7" ht="49.5" customHeight="1">
-      <c r="B7" s="24" t="inlineStr">
+      <c r="C144" s="24" t="n"/>
+      <c r="D144" s="24" t="n"/>
+      <c r="E144" s="25" t="n"/>
+    </row>
+    <row r="145" ht="49.5" customHeight="1">
+      <c r="B145" s="26" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C7" s="25" t="inlineStr">
+      <c r="C145" s="27" t="inlineStr">
         <is>
           <t>Experiencia integral que combina servicio funerario y cremación, con un espacio conmemorativo para resguardar hasta dos urnas cinerarias en un entorno de respeto, acompañamiento y serenidad.</t>
         </is>
       </c>
-      <c r="D7" s="26" t="n"/>
-      <c r="E7" s="27" t="n"/>
-    </row>
-    <row r="8" ht="20.5" customHeight="1">
-      <c r="B8" s="28" t="inlineStr">
+      <c r="D145" s="28" t="n"/>
+      <c r="E145" s="29" t="n"/>
+    </row>
+    <row r="146" ht="20.5" customHeight="1">
+      <c r="B146" s="30" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C8" s="29" t="inlineStr">
+      <c r="C146" s="31" t="inlineStr">
         <is>
           <t>Hasta 2 urnas cinerarias (incluye 2 cremaciones).</t>
         </is>
       </c>
-      <c r="D8" s="30" t="n"/>
-      <c r="E8" s="31" t="n"/>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="B9" s="21" t="inlineStr">
+      <c r="D146" s="32" t="n"/>
+      <c r="E146" s="33" t="n"/>
+    </row>
+    <row r="147" ht="20" customHeight="1">
+      <c r="B147" s="23" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C9" s="22" t="n"/>
-      <c r="D9" s="22" t="n"/>
-      <c r="E9" s="23" t="n"/>
-    </row>
-    <row r="10" ht="20.5" customHeight="1">
-      <c r="B10" s="24" t="inlineStr">
+      <c r="C147" s="24" t="n"/>
+      <c r="D147" s="24" t="n"/>
+      <c r="E147" s="25" t="n"/>
+    </row>
+    <row r="148" ht="20.5" customHeight="1">
+      <c r="B148" s="26" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="C10" s="25" t="inlineStr">
+      <c r="C148" s="27" t="inlineStr">
         <is>
           <t>Cristal o mármol</t>
         </is>
       </c>
-      <c r="D10" s="26" t="n"/>
-      <c r="E10" s="27" t="n"/>
-    </row>
-    <row r="11" ht="20.5" customHeight="1">
-      <c r="B11" s="28" t="inlineStr">
+      <c r="D148" s="28" t="n"/>
+      <c r="E148" s="29" t="n"/>
+    </row>
+    <row r="149" ht="20.5" customHeight="1">
+      <c r="B149" s="30" t="inlineStr">
         <is>
           <t>Columbario</t>
         </is>
       </c>
-      <c r="C11" s="29" t="inlineStr">
+      <c r="C149" s="31" t="inlineStr">
         <is>
           <t>Estándar, espacio permanente para hasta 2 urnas</t>
         </is>
       </c>
-      <c r="D11" s="30" t="n"/>
-      <c r="E11" s="31" t="n"/>
-    </row>
-    <row r="12" ht="20.5" customHeight="1">
-      <c r="B12" s="24" t="inlineStr">
+      <c r="D149" s="32" t="n"/>
+      <c r="E149" s="33" t="n"/>
+    </row>
+    <row r="150" ht="20.5" customHeight="1">
+      <c r="B150" s="26" t="inlineStr">
         <is>
           <t>Cremación</t>
         </is>
       </c>
-      <c r="C12" s="25" t="inlineStr">
+      <c r="C150" s="27" t="inlineStr">
         <is>
           <t>2 cremaciones en crematorio propio, con certificado</t>
         </is>
       </c>
-      <c r="D12" s="26" t="n"/>
-      <c r="E12" s="27" t="n"/>
-    </row>
-    <row r="13" ht="20.5" customHeight="1">
-      <c r="B13" s="28" t="inlineStr">
+      <c r="D150" s="28" t="n"/>
+      <c r="E150" s="29" t="n"/>
+    </row>
+    <row r="151" ht="20.5" customHeight="1">
+      <c r="B151" s="30" t="inlineStr">
         <is>
           <t>Preparación y resguardo</t>
         </is>
       </c>
-      <c r="C13" s="29" t="inlineStr">
+      <c r="C151" s="31" t="inlineStr">
         <is>
           <t>Preparación química y custodia en laboratorio hasta por 5 días</t>
         </is>
       </c>
-      <c r="D13" s="30" t="n"/>
-      <c r="E13" s="31" t="n"/>
-    </row>
-    <row r="14" ht="35" customHeight="1">
-      <c r="B14" s="24" t="inlineStr">
+      <c r="D151" s="32" t="n"/>
+      <c r="E151" s="33" t="n"/>
+    </row>
+    <row r="152" ht="35" customHeight="1">
+      <c r="B152" s="26" t="inlineStr">
         <is>
           <t>Velación</t>
         </is>
       </c>
-      <c r="C14" s="25" t="inlineStr">
+      <c r="C152" s="27" t="inlineStr">
         <is>
           <t>Sala de velación 24 horas · La Auxiliadora: Capilla Maquilishuat o Básica · Capillas Memoriales: Capilla Las Camelias o Básica</t>
         </is>
       </c>
-      <c r="D14" s="26" t="n"/>
-      <c r="E14" s="27" t="n"/>
-    </row>
-    <row r="15" ht="35" customHeight="1">
-      <c r="B15" s="28" t="inlineStr">
+      <c r="D152" s="28" t="n"/>
+      <c r="E152" s="29" t="n"/>
+    </row>
+    <row r="153" ht="35" customHeight="1">
+      <c r="B153" s="30" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C15" s="29" t="inlineStr">
+      <c r="C153" s="31" t="inlineStr">
         <is>
           <t>Definida: se elige el nicho al contratar · A futuro: el nicho se asigna más adelante. El precio varía según fila y nivel.</t>
         </is>
       </c>
-      <c r="D15" s="30" t="n"/>
-      <c r="E15" s="31" t="n"/>
-    </row>
-    <row r="16" ht="122" customHeight="1">
-      <c r="B16" s="24" t="inlineStr">
+      <c r="D153" s="32" t="n"/>
+      <c r="E153" s="33" t="n"/>
+    </row>
+    <row r="154" ht="122" customHeight="1">
+      <c r="B154" s="26" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C16" s="25" t="inlineStr">
+      <c r="C154" s="27" t="inlineStr">
         <is>
           <t>• Columbario estándar de cristal o mármol para hasta 2 urnas
 • Traslados durante todo el proceso funerario
@@ -3106,909 +2981,909 @@
 • Programa Vive (acompañamiento en el duelo) y café y agua ilimitados</t>
         </is>
       </c>
-      <c r="D16" s="26" t="n"/>
-      <c r="E16" s="27" t="n"/>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="B17" s="21" t="inlineStr">
+      <c r="D154" s="28" t="n"/>
+      <c r="E154" s="29" t="n"/>
+    </row>
+    <row r="155" ht="20" customHeight="1">
+      <c r="B155" s="23" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C17" s="22" t="n"/>
-      <c r="D17" s="22" t="n"/>
-      <c r="E17" s="23" t="n"/>
-    </row>
-    <row r="18" ht="41" customHeight="1">
-      <c r="B18" s="24" t="inlineStr">
+      <c r="C155" s="24" t="n"/>
+      <c r="D155" s="24" t="n"/>
+      <c r="E155" s="25" t="n"/>
+    </row>
+    <row r="156" ht="41" customHeight="1">
+      <c r="B156" s="26" t="inlineStr">
         <is>
           <t>Precio</t>
         </is>
       </c>
-      <c r="C18" s="32" t="inlineStr">
+      <c r="C156" s="34" t="inlineStr">
         <is>
           <t>Ubicación definida: US$ 3.400 – US$ 3.900
 Ubicación a futuro: US$ 2.700 – US$ 3.200</t>
         </is>
       </c>
-      <c r="D18" s="26" t="n"/>
-      <c r="E18" s="27" t="n"/>
-    </row>
-    <row r="19" ht="41" customHeight="1">
-      <c r="B19" s="28" t="inlineStr">
+      <c r="D156" s="28" t="n"/>
+      <c r="E156" s="29" t="n"/>
+    </row>
+    <row r="157" ht="41" customHeight="1">
+      <c r="B157" s="30" t="inlineStr">
         <is>
           <t>Precio Finados y noviembre (−15%)</t>
         </is>
       </c>
-      <c r="C19" s="33" t="inlineStr">
+      <c r="C157" s="35" t="inlineStr">
         <is>
           <t>Ubicación definida: US$ 2.890 – US$ 3.315
 Ubicación a futuro: US$ 2.295 – US$ 2.720</t>
         </is>
       </c>
-      <c r="D19" s="30" t="n"/>
-      <c r="E19" s="31" t="n"/>
-    </row>
-    <row r="20" ht="20.5" customHeight="1">
-      <c r="B20" s="28" t="inlineStr">
+      <c r="D157" s="32" t="n"/>
+      <c r="E157" s="33" t="n"/>
+    </row>
+    <row r="158" ht="20.5" customHeight="1">
+      <c r="B158" s="30" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C20" s="29" t="inlineStr">
+      <c r="C158" s="31" t="inlineStr">
         <is>
           <t>Precio según fila y nivel del columbario</t>
         </is>
       </c>
-      <c r="D20" s="30" t="n"/>
-      <c r="E20" s="31" t="n"/>
-    </row>
-    <row r="21" ht="20.5" customHeight="1">
-      <c r="B21" s="24" t="inlineStr">
+      <c r="D158" s="32" t="n"/>
+      <c r="E158" s="33" t="n"/>
+    </row>
+    <row r="159" ht="20.5" customHeight="1">
+      <c r="B159" s="26" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C21" s="25" t="inlineStr">
+      <c r="C159" s="27" t="inlineStr">
         <is>
           <t>Pago único o financiado hasta 120 meses, con intereses.</t>
         </is>
       </c>
-      <c r="D21" s="26" t="n"/>
-      <c r="E21" s="27" t="n"/>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="B22" s="21" t="inlineStr">
+      <c r="D159" s="28" t="n"/>
+      <c r="E159" s="29" t="n"/>
+    </row>
+    <row r="160" ht="20" customHeight="1">
+      <c r="B160" s="23" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C22" s="22" t="n"/>
-      <c r="D22" s="22" t="n"/>
-      <c r="E22" s="23" t="n"/>
-    </row>
-    <row r="23" ht="35" customHeight="1">
-      <c r="B23" s="34" t="inlineStr">
+      <c r="C160" s="24" t="n"/>
+      <c r="D160" s="24" t="n"/>
+      <c r="E160" s="25" t="n"/>
+    </row>
+    <row r="161" ht="35" customHeight="1">
+      <c r="B161" s="36" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C23" s="35" t="inlineStr">
+      <c r="C161" s="37" t="inlineStr">
         <is>
           <t>Familias que quieren resolver en una sola compra el servicio funerario, la cremación y un lugar permanente para dos seres queridos.</t>
         </is>
       </c>
-      <c r="D23" s="36" t="n"/>
-      <c r="E23" s="37" t="n"/>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="B26" s="15" t="inlineStr">
+      <c r="D161" s="38" t="n"/>
+      <c r="E161" s="39" t="n"/>
+    </row>
+    <row r="164" ht="30" customHeight="1">
+      <c r="B164" s="17" t="inlineStr">
         <is>
           <t>COLUMBARIO MÁRMOL O CRISTAL</t>
         </is>
       </c>
-      <c r="C26" s="16" t="n"/>
-      <c r="D26" s="16" t="n"/>
-      <c r="E26" s="17" t="n"/>
-    </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="B27" s="18" t="inlineStr">
+      <c r="C164" s="18" t="n"/>
+      <c r="D164" s="18" t="n"/>
+      <c r="E164" s="19" t="n"/>
+    </row>
+    <row r="165" ht="20" customHeight="1">
+      <c r="B165" s="20" t="inlineStr">
         <is>
           <t>El Hogar de las Memorias  ·  Destino final · Columbario</t>
         </is>
       </c>
-      <c r="C27" s="19" t="n"/>
-      <c r="D27" s="19" t="n"/>
-      <c r="E27" s="20" t="n"/>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="B28" s="21" t="inlineStr">
+      <c r="C165" s="21" t="n"/>
+      <c r="D165" s="21" t="n"/>
+      <c r="E165" s="22" t="n"/>
+    </row>
+    <row r="166" ht="20" customHeight="1">
+      <c r="B166" s="23" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C28" s="22" t="n"/>
-      <c r="D28" s="22" t="n"/>
-      <c r="E28" s="23" t="n"/>
-    </row>
-    <row r="29" ht="35" customHeight="1">
-      <c r="B29" s="24" t="inlineStr">
+      <c r="C166" s="24" t="n"/>
+      <c r="D166" s="24" t="n"/>
+      <c r="E166" s="25" t="n"/>
+    </row>
+    <row r="167" ht="35" customHeight="1">
+      <c r="B167" s="26" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C29" s="25" t="inlineStr">
+      <c r="C167" s="27" t="inlineStr">
         <is>
           <t>Espacio permanente, elegante y sereno en mármol o cristal para preservar el legado de quienes más ama la familia, con un diseño atemporal.</t>
         </is>
       </c>
-      <c r="D29" s="26" t="n"/>
-      <c r="E29" s="27" t="n"/>
-    </row>
-    <row r="30" ht="20.5" customHeight="1">
-      <c r="B30" s="28" t="inlineStr">
+      <c r="D167" s="28" t="n"/>
+      <c r="E167" s="29" t="n"/>
+    </row>
+    <row r="168" ht="20.5" customHeight="1">
+      <c r="B168" s="30" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C30" s="29" t="inlineStr">
+      <c r="C168" s="31" t="inlineStr">
         <is>
           <t>Estándar: hasta 2 urnas.</t>
         </is>
       </c>
-      <c r="D30" s="30" t="n"/>
-      <c r="E30" s="31" t="n"/>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="B31" s="21" t="inlineStr">
+      <c r="D168" s="32" t="n"/>
+      <c r="E168" s="33" t="n"/>
+    </row>
+    <row r="169" ht="20" customHeight="1">
+      <c r="B169" s="23" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C31" s="22" t="n"/>
-      <c r="D31" s="22" t="n"/>
-      <c r="E31" s="23" t="n"/>
-    </row>
-    <row r="32" ht="20.5" customHeight="1">
-      <c r="B32" s="24" t="inlineStr">
+      <c r="C169" s="24" t="n"/>
+      <c r="D169" s="24" t="n"/>
+      <c r="E169" s="25" t="n"/>
+    </row>
+    <row r="170" ht="20.5" customHeight="1">
+      <c r="B170" s="26" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="C32" s="25" t="inlineStr">
+      <c r="C170" s="27" t="inlineStr">
         <is>
           <t>Mármol o cristal</t>
         </is>
       </c>
-      <c r="D32" s="26" t="n"/>
-      <c r="E32" s="27" t="n"/>
-    </row>
-    <row r="33" ht="20.5" customHeight="1">
-      <c r="B33" s="28" t="inlineStr">
+      <c r="D170" s="28" t="n"/>
+      <c r="E170" s="29" t="n"/>
+    </row>
+    <row r="171" ht="20.5" customHeight="1">
+      <c r="B171" s="30" t="inlineStr">
         <is>
           <t>Permanencia</t>
         </is>
       </c>
-      <c r="C33" s="29" t="inlineStr">
+      <c r="C171" s="31" t="inlineStr">
         <is>
           <t>Permanente</t>
         </is>
       </c>
-      <c r="D33" s="30" t="n"/>
-      <c r="E33" s="31" t="n"/>
-    </row>
-    <row r="34" ht="35" customHeight="1">
-      <c r="B34" s="24" t="inlineStr">
+      <c r="D171" s="32" t="n"/>
+      <c r="E171" s="33" t="n"/>
+    </row>
+    <row r="172" ht="35" customHeight="1">
+      <c r="B172" s="26" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C34" s="25" t="inlineStr">
+      <c r="C172" s="27" t="inlineStr">
         <is>
           <t>Definida: se elige el nicho al contratar · A futuro: el nicho se asigna más adelante. El precio varía según fila y nivel.</t>
         </is>
       </c>
-      <c r="D34" s="26" t="n"/>
-      <c r="E34" s="27" t="n"/>
-    </row>
-    <row r="35" ht="35" customHeight="1">
-      <c r="B35" s="28" t="inlineStr">
+      <c r="D172" s="28" t="n"/>
+      <c r="E172" s="29" t="n"/>
+    </row>
+    <row r="173" ht="35" customHeight="1">
+      <c r="B173" s="30" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C35" s="29" t="inlineStr">
+      <c r="C173" s="31" t="inlineStr">
         <is>
           <t>• Espacio permanente en columbario de mármol o cristal
 • Ubicación definida o a futuro, según la opción contratada</t>
         </is>
       </c>
-      <c r="D35" s="30" t="n"/>
-      <c r="E35" s="31" t="n"/>
-    </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="B36" s="21" t="inlineStr">
+      <c r="D173" s="32" t="n"/>
+      <c r="E173" s="33" t="n"/>
+    </row>
+    <row r="174" ht="20" customHeight="1">
+      <c r="B174" s="23" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C36" s="22" t="n"/>
-      <c r="D36" s="22" t="n"/>
-      <c r="E36" s="23" t="n"/>
-    </row>
-    <row r="37" ht="41" customHeight="1">
-      <c r="B37" s="24" t="inlineStr">
+      <c r="C174" s="24" t="n"/>
+      <c r="D174" s="24" t="n"/>
+      <c r="E174" s="25" t="n"/>
+    </row>
+    <row r="175" ht="41" customHeight="1">
+      <c r="B175" s="26" t="inlineStr">
         <is>
           <t>Precio</t>
         </is>
       </c>
-      <c r="C37" s="32" t="inlineStr">
+      <c r="C175" s="34" t="inlineStr">
         <is>
           <t>Ubicación definida: US$ 2.600
 Ubicación a futuro: US$ 1.200 – US$ 1.900</t>
         </is>
       </c>
-      <c r="D37" s="26" t="n"/>
-      <c r="E37" s="27" t="n"/>
-    </row>
-    <row r="38" ht="41" customHeight="1">
-      <c r="B38" s="28" t="inlineStr">
+      <c r="D175" s="28" t="n"/>
+      <c r="E175" s="29" t="n"/>
+    </row>
+    <row r="176" ht="41" customHeight="1">
+      <c r="B176" s="30" t="inlineStr">
         <is>
           <t>Precio Finados y noviembre (−15%)</t>
         </is>
       </c>
-      <c r="C38" s="33" t="inlineStr">
+      <c r="C176" s="35" t="inlineStr">
         <is>
           <t>Ubicación definida: US$ 2.210
 Ubicación a futuro: US$ 1.020 – US$ 1.615</t>
         </is>
       </c>
-      <c r="D38" s="30" t="n"/>
-      <c r="E38" s="31" t="n"/>
-    </row>
-    <row r="39" ht="20.5" customHeight="1">
-      <c r="B39" s="28" t="inlineStr">
+      <c r="D176" s="32" t="n"/>
+      <c r="E176" s="33" t="n"/>
+    </row>
+    <row r="177" ht="20.5" customHeight="1">
+      <c r="B177" s="30" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C39" s="29" t="inlineStr">
+      <c r="C177" s="31" t="inlineStr">
         <is>
           <t>Solo columbario · precio según fila y nivel</t>
         </is>
       </c>
-      <c r="D39" s="30" t="n"/>
-      <c r="E39" s="31" t="n"/>
-    </row>
-    <row r="40" ht="20.5" customHeight="1">
-      <c r="B40" s="24" t="inlineStr">
+      <c r="D177" s="32" t="n"/>
+      <c r="E177" s="33" t="n"/>
+    </row>
+    <row r="178" ht="20.5" customHeight="1">
+      <c r="B178" s="26" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C40" s="25" t="inlineStr">
+      <c r="C178" s="27" t="inlineStr">
         <is>
           <t>Pago único o financiado hasta 120 meses, con intereses.</t>
         </is>
       </c>
-      <c r="D40" s="26" t="n"/>
-      <c r="E40" s="27" t="n"/>
-    </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="B41" s="21" t="inlineStr">
+      <c r="D178" s="28" t="n"/>
+      <c r="E178" s="29" t="n"/>
+    </row>
+    <row r="179" ht="20" customHeight="1">
+      <c r="B179" s="23" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C41" s="22" t="n"/>
-      <c r="D41" s="22" t="n"/>
-      <c r="E41" s="23" t="n"/>
-    </row>
-    <row r="42" ht="35" customHeight="1">
-      <c r="B42" s="34" t="inlineStr">
+      <c r="C179" s="24" t="n"/>
+      <c r="D179" s="24" t="n"/>
+      <c r="E179" s="25" t="n"/>
+    </row>
+    <row r="180" ht="35" customHeight="1">
+      <c r="B180" s="36" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C42" s="35" t="inlineStr">
+      <c r="C180" s="37" t="inlineStr">
         <is>
           <t>Familias que buscan un lugar permanente y elegante para las cenizas, con la cremación ya resuelta o contratada aparte.</t>
         </is>
       </c>
-      <c r="D42" s="36" t="n"/>
-      <c r="E42" s="37" t="n"/>
-    </row>
-    <row r="45" ht="30" customHeight="1">
-      <c r="B45" s="15" t="inlineStr">
+      <c r="D180" s="38" t="n"/>
+      <c r="E180" s="39" t="n"/>
+    </row>
+    <row r="183" ht="30" customHeight="1">
+      <c r="B183" s="17" t="inlineStr">
         <is>
           <t>COLUMBARIO ÓNIX</t>
         </is>
       </c>
-      <c r="C45" s="16" t="n"/>
-      <c r="D45" s="16" t="n"/>
-      <c r="E45" s="17" t="n"/>
-    </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="B46" s="18" t="inlineStr">
+      <c r="C183" s="18" t="n"/>
+      <c r="D183" s="18" t="n"/>
+      <c r="E183" s="19" t="n"/>
+    </row>
+    <row r="184" ht="20" customHeight="1">
+      <c r="B184" s="20" t="inlineStr">
         <is>
           <t>El Hogar de las Memorias  ·  Destino final · Columbario premium</t>
         </is>
       </c>
-      <c r="C46" s="19" t="n"/>
-      <c r="D46" s="19" t="n"/>
-      <c r="E46" s="20" t="n"/>
-    </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="B47" s="21" t="inlineStr">
+      <c r="C184" s="21" t="n"/>
+      <c r="D184" s="21" t="n"/>
+      <c r="E184" s="22" t="n"/>
+    </row>
+    <row r="185" ht="20" customHeight="1">
+      <c r="B185" s="23" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C47" s="22" t="n"/>
-      <c r="D47" s="22" t="n"/>
-      <c r="E47" s="23" t="n"/>
-    </row>
-    <row r="48" ht="49.5" customHeight="1">
-      <c r="B48" s="24" t="inlineStr">
+      <c r="C185" s="24" t="n"/>
+      <c r="D185" s="24" t="n"/>
+      <c r="E185" s="25" t="n"/>
+    </row>
+    <row r="186" ht="49.5" customHeight="1">
+      <c r="B186" s="26" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C48" s="25" t="inlineStr">
+      <c r="C186" s="27" t="inlineStr">
         <is>
           <t>Columbario de ónix que combina la exclusividad de una piedra natural con un diseño elegante; sus tonalidades cálidas y apariencia luminosa crean un espacio de paz, respeto y recuerdo perdurable.</t>
         </is>
       </c>
-      <c r="D48" s="26" t="n"/>
-      <c r="E48" s="27" t="n"/>
-    </row>
-    <row r="49" ht="20.5" customHeight="1">
-      <c r="B49" s="28" t="inlineStr">
+      <c r="D186" s="28" t="n"/>
+      <c r="E186" s="29" t="n"/>
+    </row>
+    <row r="187" ht="20.5" customHeight="1">
+      <c r="B187" s="30" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C49" s="29" t="inlineStr">
+      <c r="C187" s="31" t="inlineStr">
         <is>
           <t>Estándar: hasta 2 urnas · Familiar: hasta 4 urnas.</t>
         </is>
       </c>
-      <c r="D49" s="30" t="n"/>
-      <c r="E49" s="31" t="n"/>
-    </row>
-    <row r="50" ht="20" customHeight="1">
-      <c r="B50" s="21" t="inlineStr">
+      <c r="D187" s="32" t="n"/>
+      <c r="E187" s="33" t="n"/>
+    </row>
+    <row r="188" ht="20" customHeight="1">
+      <c r="B188" s="23" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C50" s="22" t="n"/>
-      <c r="D50" s="22" t="n"/>
-      <c r="E50" s="23" t="n"/>
-    </row>
-    <row r="51" ht="20.5" customHeight="1">
-      <c r="B51" s="24" t="inlineStr">
+      <c r="C188" s="24" t="n"/>
+      <c r="D188" s="24" t="n"/>
+      <c r="E188" s="25" t="n"/>
+    </row>
+    <row r="189" ht="20.5" customHeight="1">
+      <c r="B189" s="26" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="C51" s="25" t="inlineStr">
+      <c r="C189" s="27" t="inlineStr">
         <is>
           <t>Ónix natural</t>
         </is>
       </c>
-      <c r="D51" s="26" t="n"/>
-      <c r="E51" s="27" t="n"/>
-    </row>
-    <row r="52" ht="20.5" customHeight="1">
-      <c r="B52" s="28" t="inlineStr">
+      <c r="D189" s="28" t="n"/>
+      <c r="E189" s="29" t="n"/>
+    </row>
+    <row r="190" ht="20.5" customHeight="1">
+      <c r="B190" s="30" t="inlineStr">
         <is>
           <t>Modalidades</t>
         </is>
       </c>
-      <c r="C52" s="29" t="inlineStr">
+      <c r="C190" s="31" t="inlineStr">
         <is>
           <t>Estándar (2 urnas) y Familiar (4 urnas)</t>
         </is>
       </c>
-      <c r="D52" s="30" t="n"/>
-      <c r="E52" s="31" t="n"/>
-    </row>
-    <row r="53" ht="20.5" customHeight="1">
-      <c r="B53" s="24" t="inlineStr">
+      <c r="D190" s="32" t="n"/>
+      <c r="E190" s="33" t="n"/>
+    </row>
+    <row r="191" ht="20.5" customHeight="1">
+      <c r="B191" s="26" t="inlineStr">
         <is>
           <t>Permanencia</t>
         </is>
       </c>
-      <c r="C53" s="25" t="inlineStr">
+      <c r="C191" s="27" t="inlineStr">
         <is>
           <t>Permanente</t>
         </is>
       </c>
-      <c r="D53" s="26" t="n"/>
-      <c r="E53" s="27" t="n"/>
-    </row>
-    <row r="54" ht="35" customHeight="1">
-      <c r="B54" s="28" t="inlineStr">
+      <c r="D191" s="28" t="n"/>
+      <c r="E191" s="29" t="n"/>
+    </row>
+    <row r="192" ht="35" customHeight="1">
+      <c r="B192" s="30" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C54" s="29" t="inlineStr">
+      <c r="C192" s="31" t="inlineStr">
         <is>
           <t>• Espacio permanente en columbario de ónix natural
 • Modalidad estándar o familiar</t>
         </is>
       </c>
-      <c r="D54" s="30" t="n"/>
-      <c r="E54" s="31" t="n"/>
-    </row>
-    <row r="55" ht="20" customHeight="1">
-      <c r="B55" s="21" t="inlineStr">
+      <c r="D192" s="32" t="n"/>
+      <c r="E192" s="33" t="n"/>
+    </row>
+    <row r="193" ht="20" customHeight="1">
+      <c r="B193" s="23" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C55" s="22" t="n"/>
-      <c r="D55" s="22" t="n"/>
-      <c r="E55" s="23" t="n"/>
-    </row>
-    <row r="56" ht="41" customHeight="1">
-      <c r="B56" s="24" t="inlineStr">
+      <c r="C193" s="24" t="n"/>
+      <c r="D193" s="24" t="n"/>
+      <c r="E193" s="25" t="n"/>
+    </row>
+    <row r="194" ht="41" customHeight="1">
+      <c r="B194" s="26" t="inlineStr">
         <is>
           <t>Precio</t>
         </is>
       </c>
-      <c r="C56" s="32" t="inlineStr">
+      <c r="C194" s="34" t="inlineStr">
         <is>
           <t>Estándar · ubicación definida: US$ 3.100
 Familiar · ubicación a futuro: US$ 5.000</t>
         </is>
       </c>
-      <c r="D56" s="26" t="n"/>
-      <c r="E56" s="27" t="n"/>
-    </row>
-    <row r="57" ht="41" customHeight="1">
-      <c r="B57" s="28" t="inlineStr">
+      <c r="D194" s="28" t="n"/>
+      <c r="E194" s="29" t="n"/>
+    </row>
+    <row r="195" ht="41" customHeight="1">
+      <c r="B195" s="30" t="inlineStr">
         <is>
           <t>Precio Finados y noviembre (−15%)</t>
         </is>
       </c>
-      <c r="C57" s="33" t="inlineStr">
+      <c r="C195" s="35" t="inlineStr">
         <is>
           <t>Estándar · ubicación definida: US$ 2.635
 Familiar · ubicación a futuro: US$ 4.250</t>
         </is>
       </c>
-      <c r="D57" s="30" t="n"/>
-      <c r="E57" s="31" t="n"/>
-    </row>
-    <row r="58" ht="20.5" customHeight="1">
-      <c r="B58" s="28" t="inlineStr">
+      <c r="D195" s="32" t="n"/>
+      <c r="E195" s="33" t="n"/>
+    </row>
+    <row r="196" ht="20.5" customHeight="1">
+      <c r="B196" s="30" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C58" s="29" t="inlineStr">
+      <c r="C196" s="31" t="inlineStr">
         <is>
           <t>Solo columbario</t>
         </is>
       </c>
-      <c r="D58" s="30" t="n"/>
-      <c r="E58" s="31" t="n"/>
-    </row>
-    <row r="59" ht="20.5" customHeight="1">
-      <c r="B59" s="24" t="inlineStr">
+      <c r="D196" s="32" t="n"/>
+      <c r="E196" s="33" t="n"/>
+    </row>
+    <row r="197" ht="20.5" customHeight="1">
+      <c r="B197" s="26" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C59" s="25" t="inlineStr">
+      <c r="C197" s="27" t="inlineStr">
         <is>
           <t>Pago único o financiado hasta 120 meses, con intereses.</t>
         </is>
       </c>
-      <c r="D59" s="26" t="n"/>
-      <c r="E59" s="27" t="n"/>
-    </row>
-    <row r="60" ht="20" customHeight="1">
-      <c r="B60" s="21" t="inlineStr">
+      <c r="D197" s="28" t="n"/>
+      <c r="E197" s="29" t="n"/>
+    </row>
+    <row r="198" ht="20" customHeight="1">
+      <c r="B198" s="23" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C60" s="22" t="n"/>
-      <c r="D60" s="22" t="n"/>
-      <c r="E60" s="23" t="n"/>
-    </row>
-    <row r="61" ht="35" customHeight="1">
-      <c r="B61" s="34" t="inlineStr">
+      <c r="C198" s="24" t="n"/>
+      <c r="D198" s="24" t="n"/>
+      <c r="E198" s="25" t="n"/>
+    </row>
+    <row r="199" ht="35" customHeight="1">
+      <c r="B199" s="36" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C61" s="35" t="inlineStr">
+      <c r="C199" s="37" t="inlineStr">
         <is>
           <t>Familias que buscan exclusividad y una piedra natural de alta gama para el homenaje.</t>
         </is>
       </c>
-      <c r="D61" s="36" t="n"/>
-      <c r="E61" s="37" t="n"/>
-    </row>
-    <row r="64" ht="30" customHeight="1">
-      <c r="B64" s="15" t="inlineStr">
+      <c r="D199" s="38" t="n"/>
+      <c r="E199" s="39" t="n"/>
+    </row>
+    <row r="202" ht="30" customHeight="1">
+      <c r="B202" s="17" t="inlineStr">
         <is>
           <t>COLUMBARIO OBRA DE ARTE</t>
         </is>
       </c>
-      <c r="C64" s="16" t="n"/>
-      <c r="D64" s="16" t="n"/>
-      <c r="E64" s="17" t="n"/>
-    </row>
-    <row r="65" ht="20" customHeight="1">
-      <c r="B65" s="18" t="inlineStr">
+      <c r="C202" s="18" t="n"/>
+      <c r="D202" s="18" t="n"/>
+      <c r="E202" s="19" t="n"/>
+    </row>
+    <row r="203" ht="20" customHeight="1">
+      <c r="B203" s="20" t="inlineStr">
         <is>
           <t>El Hogar de las Memorias  ·  Destino final · Columbario familiar exclusivo</t>
         </is>
       </c>
-      <c r="C65" s="19" t="n"/>
-      <c r="D65" s="19" t="n"/>
-      <c r="E65" s="20" t="n"/>
-    </row>
-    <row r="66" ht="20" customHeight="1">
-      <c r="B66" s="21" t="inlineStr">
+      <c r="C203" s="21" t="n"/>
+      <c r="D203" s="21" t="n"/>
+      <c r="E203" s="22" t="n"/>
+    </row>
+    <row r="204" ht="20" customHeight="1">
+      <c r="B204" s="23" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C66" s="22" t="n"/>
-      <c r="D66" s="22" t="n"/>
-      <c r="E66" s="23" t="n"/>
-    </row>
-    <row r="67" ht="49.5" customHeight="1">
-      <c r="B67" s="24" t="inlineStr">
+      <c r="C204" s="24" t="n"/>
+      <c r="D204" s="24" t="n"/>
+      <c r="E204" s="25" t="n"/>
+    </row>
+    <row r="205" ht="49.5" customHeight="1">
+      <c r="B205" s="26" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C67" s="25" t="inlineStr">
+      <c r="C205" s="27" t="inlineStr">
         <is>
           <t>Una expresión única de fe, memoria y belleza: tapa de ónix con obra de arte religiosa que preserva la memoria de toda una familia en un entorno de serenidad y contemplación.</t>
         </is>
       </c>
-      <c r="D67" s="26" t="n"/>
-      <c r="E67" s="27" t="n"/>
-    </row>
-    <row r="68" ht="20.5" customHeight="1">
-      <c r="B68" s="28" t="inlineStr">
+      <c r="D205" s="28" t="n"/>
+      <c r="E205" s="29" t="n"/>
+    </row>
+    <row r="206" ht="20.5" customHeight="1">
+      <c r="B206" s="30" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C68" s="29" t="inlineStr">
+      <c r="C206" s="31" t="inlineStr">
         <is>
           <t>Familiar: hasta 4 urnas.</t>
         </is>
       </c>
-      <c r="D68" s="30" t="n"/>
-      <c r="E68" s="31" t="n"/>
-    </row>
-    <row r="69" ht="20" customHeight="1">
-      <c r="B69" s="21" t="inlineStr">
+      <c r="D206" s="32" t="n"/>
+      <c r="E206" s="33" t="n"/>
+    </row>
+    <row r="207" ht="20" customHeight="1">
+      <c r="B207" s="23" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C69" s="22" t="n"/>
-      <c r="D69" s="22" t="n"/>
-      <c r="E69" s="23" t="n"/>
-    </row>
-    <row r="70" ht="20.5" customHeight="1">
-      <c r="B70" s="24" t="inlineStr">
+      <c r="C207" s="24" t="n"/>
+      <c r="D207" s="24" t="n"/>
+      <c r="E207" s="25" t="n"/>
+    </row>
+    <row r="208" ht="20.5" customHeight="1">
+      <c r="B208" s="26" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="C70" s="25" t="inlineStr">
+      <c r="C208" s="27" t="inlineStr">
         <is>
           <t>Tapa de ónix con obra de arte religiosa</t>
         </is>
       </c>
-      <c r="D70" s="26" t="n"/>
-      <c r="E70" s="27" t="n"/>
-    </row>
-    <row r="71" ht="20.5" customHeight="1">
-      <c r="B71" s="28" t="inlineStr">
+      <c r="D208" s="28" t="n"/>
+      <c r="E208" s="29" t="n"/>
+    </row>
+    <row r="209" ht="20.5" customHeight="1">
+      <c r="B209" s="30" t="inlineStr">
         <is>
           <t>Modalidad</t>
         </is>
       </c>
-      <c r="C71" s="29" t="inlineStr">
+      <c r="C209" s="31" t="inlineStr">
         <is>
           <t>Familiar (4 urnas)</t>
         </is>
       </c>
-      <c r="D71" s="30" t="n"/>
-      <c r="E71" s="31" t="n"/>
-    </row>
-    <row r="72" ht="20.5" customHeight="1">
-      <c r="B72" s="24" t="inlineStr">
+      <c r="D209" s="32" t="n"/>
+      <c r="E209" s="33" t="n"/>
+    </row>
+    <row r="210" ht="20.5" customHeight="1">
+      <c r="B210" s="26" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C72" s="25" t="inlineStr">
+      <c r="C210" s="27" t="inlineStr">
         <is>
           <t>Definida</t>
         </is>
       </c>
-      <c r="D72" s="26" t="n"/>
-      <c r="E72" s="27" t="n"/>
-    </row>
-    <row r="73" ht="20.5" customHeight="1">
-      <c r="B73" s="28" t="inlineStr">
+      <c r="D210" s="28" t="n"/>
+      <c r="E210" s="29" t="n"/>
+    </row>
+    <row r="211" ht="20.5" customHeight="1">
+      <c r="B211" s="30" t="inlineStr">
         <is>
           <t>Permanencia</t>
         </is>
       </c>
-      <c r="C73" s="29" t="inlineStr">
+      <c r="C211" s="31" t="inlineStr">
         <is>
           <t>Permanente</t>
         </is>
       </c>
-      <c r="D73" s="30" t="n"/>
-      <c r="E73" s="31" t="n"/>
-    </row>
-    <row r="74" ht="35" customHeight="1">
-      <c r="B74" s="24" t="inlineStr">
+      <c r="D211" s="32" t="n"/>
+      <c r="E211" s="33" t="n"/>
+    </row>
+    <row r="212" ht="35" customHeight="1">
+      <c r="B212" s="26" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C74" s="25" t="inlineStr">
+      <c r="C212" s="27" t="inlineStr">
         <is>
           <t>• Columbario familiar permanente para hasta 4 urnas
 • Tapa exclusiva de ónix con obra de arte religiosa</t>
         </is>
       </c>
-      <c r="D74" s="26" t="n"/>
-      <c r="E74" s="27" t="n"/>
-    </row>
-    <row r="75" ht="20" customHeight="1">
-      <c r="B75" s="21" t="inlineStr">
+      <c r="D212" s="28" t="n"/>
+      <c r="E212" s="29" t="n"/>
+    </row>
+    <row r="213" ht="20" customHeight="1">
+      <c r="B213" s="23" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C75" s="22" t="n"/>
-      <c r="D75" s="22" t="n"/>
-      <c r="E75" s="23" t="n"/>
-    </row>
-    <row r="76" ht="26.5" customHeight="1">
-      <c r="B76" s="24" t="inlineStr">
+      <c r="C213" s="24" t="n"/>
+      <c r="D213" s="24" t="n"/>
+      <c r="E213" s="25" t="n"/>
+    </row>
+    <row r="214" ht="26.5" customHeight="1">
+      <c r="B214" s="26" t="inlineStr">
         <is>
           <t>Precio</t>
         </is>
       </c>
-      <c r="C76" s="32" t="inlineStr">
+      <c r="C214" s="34" t="inlineStr">
         <is>
           <t>Familiar · ubicación definida: US$ 12.500</t>
         </is>
       </c>
-      <c r="D76" s="26" t="n"/>
-      <c r="E76" s="27" t="n"/>
-    </row>
-    <row r="77" ht="26.5" customHeight="1">
-      <c r="B77" s="28" t="inlineStr">
+      <c r="D214" s="28" t="n"/>
+      <c r="E214" s="29" t="n"/>
+    </row>
+    <row r="215" ht="26.5" customHeight="1">
+      <c r="B215" s="30" t="inlineStr">
         <is>
           <t>Precio Finados y noviembre (−15%)</t>
         </is>
       </c>
-      <c r="C77" s="33" t="inlineStr">
+      <c r="C215" s="35" t="inlineStr">
         <is>
           <t>Familiar · ubicación definida: US$ 10.625</t>
         </is>
       </c>
-      <c r="D77" s="30" t="n"/>
-      <c r="E77" s="31" t="n"/>
-    </row>
-    <row r="78" ht="20.5" customHeight="1">
-      <c r="B78" s="28" t="inlineStr">
+      <c r="D215" s="32" t="n"/>
+      <c r="E215" s="33" t="n"/>
+    </row>
+    <row r="216" ht="20.5" customHeight="1">
+      <c r="B216" s="30" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C78" s="29" t="inlineStr">
+      <c r="C216" s="31" t="inlineStr">
         <is>
           <t>Solo columbario</t>
         </is>
       </c>
-      <c r="D78" s="30" t="n"/>
-      <c r="E78" s="31" t="n"/>
-    </row>
-    <row r="79" ht="20.5" customHeight="1">
-      <c r="B79" s="24" t="inlineStr">
+      <c r="D216" s="32" t="n"/>
+      <c r="E216" s="33" t="n"/>
+    </row>
+    <row r="217" ht="20.5" customHeight="1">
+      <c r="B217" s="26" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C79" s="25" t="inlineStr">
+      <c r="C217" s="27" t="inlineStr">
         <is>
           <t>Pago único o financiado hasta 120 meses, con intereses.</t>
         </is>
       </c>
-      <c r="D79" s="26" t="n"/>
-      <c r="E79" s="27" t="n"/>
-    </row>
-    <row r="80" ht="20" customHeight="1">
-      <c r="B80" s="21" t="inlineStr">
+      <c r="D217" s="28" t="n"/>
+      <c r="E217" s="29" t="n"/>
+    </row>
+    <row r="218" ht="20" customHeight="1">
+      <c r="B218" s="23" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C80" s="22" t="n"/>
-      <c r="D80" s="22" t="n"/>
-      <c r="E80" s="23" t="n"/>
-    </row>
-    <row r="81" ht="20.5" customHeight="1">
-      <c r="B81" s="34" t="inlineStr">
+      <c r="C218" s="24" t="n"/>
+      <c r="D218" s="24" t="n"/>
+      <c r="E218" s="25" t="n"/>
+    </row>
+    <row r="219" ht="20.5" customHeight="1">
+      <c r="B219" s="36" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C81" s="35" t="inlineStr">
+      <c r="C219" s="37" t="inlineStr">
         <is>
           <t>Familias de fe que desean un legado único y de máxima exclusividad.</t>
         </is>
       </c>
-      <c r="D81" s="36" t="n"/>
-      <c r="E81" s="37" t="n"/>
-    </row>
-    <row r="84" ht="30" customHeight="1">
-      <c r="B84" s="15" t="inlineStr">
+      <c r="D219" s="38" t="n"/>
+      <c r="E219" s="39" t="n"/>
+    </row>
+    <row r="222" ht="30" customHeight="1">
+      <c r="B222" s="17" t="inlineStr">
         <is>
           <t>COLUMBARIO CRISTAL · BELLA VISTA</t>
         </is>
       </c>
-      <c r="C84" s="16" t="n"/>
-      <c r="D84" s="16" t="n"/>
-      <c r="E84" s="17" t="n"/>
-    </row>
-    <row r="85" ht="20" customHeight="1">
-      <c r="B85" s="18" t="inlineStr">
+      <c r="C222" s="18" t="n"/>
+      <c r="D222" s="18" t="n"/>
+      <c r="E222" s="19" t="n"/>
+    </row>
+    <row r="223" ht="20" customHeight="1">
+      <c r="B223" s="20" t="inlineStr">
         <is>
           <t>Mausoleo vertical Bella Vista  ·  Cremación + columbario</t>
         </is>
       </c>
-      <c r="C85" s="19" t="n"/>
-      <c r="D85" s="19" t="n"/>
-      <c r="E85" s="20" t="n"/>
-    </row>
-    <row r="86" ht="20" customHeight="1">
-      <c r="B86" s="21" t="inlineStr">
+      <c r="C223" s="21" t="n"/>
+      <c r="D223" s="21" t="n"/>
+      <c r="E223" s="22" t="n"/>
+    </row>
+    <row r="224" ht="20" customHeight="1">
+      <c r="B224" s="23" t="inlineStr">
         <is>
           <t>VISIÓN GENERAL</t>
         </is>
       </c>
-      <c r="C86" s="22" t="n"/>
-      <c r="D86" s="22" t="n"/>
-      <c r="E86" s="23" t="n"/>
-    </row>
-    <row r="87" ht="49.5" customHeight="1">
-      <c r="B87" s="24" t="inlineStr">
+      <c r="C224" s="24" t="n"/>
+      <c r="D224" s="24" t="n"/>
+      <c r="E224" s="25" t="n"/>
+    </row>
+    <row r="225" ht="49.5" customHeight="1">
+      <c r="B225" s="26" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C87" s="25" t="inlineStr">
+      <c r="C225" s="27" t="inlineStr">
         <is>
           <t>Columbario de cristal en el mausoleo vertical Bella Vista que incluye el proceso completo de cremación: traslados, preparación, cremaciones, urnas y ceremonia de colocación.</t>
         </is>
       </c>
-      <c r="D87" s="26" t="n"/>
-      <c r="E87" s="27" t="n"/>
-    </row>
-    <row r="88" ht="20.5" customHeight="1">
-      <c r="B88" s="28" t="inlineStr">
+      <c r="D225" s="28" t="n"/>
+      <c r="E225" s="29" t="n"/>
+    </row>
+    <row r="226" ht="20.5" customHeight="1">
+      <c r="B226" s="30" t="inlineStr">
         <is>
           <t>Capacidad / Cobertura</t>
         </is>
       </c>
-      <c r="C88" s="29" t="inlineStr">
+      <c r="C226" s="31" t="inlineStr">
         <is>
           <t>Estándar: 2 cremaciones y 2 urnas · Familiar: 4 cremaciones y 4 urnas.</t>
         </is>
       </c>
-      <c r="D88" s="30" t="n"/>
-      <c r="E88" s="31" t="n"/>
-    </row>
-    <row r="89" ht="20" customHeight="1">
-      <c r="B89" s="21" t="inlineStr">
+      <c r="D226" s="32" t="n"/>
+      <c r="E226" s="33" t="n"/>
+    </row>
+    <row r="227" ht="20" customHeight="1">
+      <c r="B227" s="23" t="inlineStr">
         <is>
           <t>ESPECIFICACIONES TÉCNICAS</t>
         </is>
       </c>
-      <c r="C89" s="22" t="n"/>
-      <c r="D89" s="22" t="n"/>
-      <c r="E89" s="23" t="n"/>
-    </row>
-    <row r="90" ht="20.5" customHeight="1">
-      <c r="B90" s="24" t="inlineStr">
+      <c r="C227" s="24" t="n"/>
+      <c r="D227" s="24" t="n"/>
+      <c r="E227" s="25" t="n"/>
+    </row>
+    <row r="228" ht="20.5" customHeight="1">
+      <c r="B228" s="26" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C90" s="25" t="inlineStr">
+      <c r="C228" s="27" t="inlineStr">
         <is>
           <t>Mausoleo vertical Bella Vista</t>
         </is>
       </c>
-      <c r="D90" s="26" t="n"/>
-      <c r="E90" s="27" t="n"/>
-    </row>
-    <row r="91" ht="20.5" customHeight="1">
-      <c r="B91" s="28" t="inlineStr">
+      <c r="D228" s="28" t="n"/>
+      <c r="E228" s="29" t="n"/>
+    </row>
+    <row r="229" ht="20.5" customHeight="1">
+      <c r="B229" s="30" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="C91" s="29" t="inlineStr">
+      <c r="C229" s="31" t="inlineStr">
         <is>
           <t>Cristal</t>
         </is>
       </c>
-      <c r="D91" s="30" t="n"/>
-      <c r="E91" s="31" t="n"/>
-    </row>
-    <row r="92" ht="20.5" customHeight="1">
-      <c r="B92" s="24" t="inlineStr">
+      <c r="D229" s="32" t="n"/>
+      <c r="E229" s="33" t="n"/>
+    </row>
+    <row r="230" ht="20.5" customHeight="1">
+      <c r="B230" s="26" t="inlineStr">
         <is>
           <t>Medidas</t>
         </is>
       </c>
-      <c r="C92" s="25" t="inlineStr">
+      <c r="C230" s="27" t="inlineStr">
         <is>
           <t>30 × 30 × 30 cm</t>
         </is>
       </c>
-      <c r="D92" s="26" t="n"/>
-      <c r="E92" s="27" t="n"/>
-    </row>
-    <row r="93" ht="20.5" customHeight="1">
-      <c r="B93" s="28" t="inlineStr">
+      <c r="D230" s="28" t="n"/>
+      <c r="E230" s="29" t="n"/>
+    </row>
+    <row r="231" ht="20.5" customHeight="1">
+      <c r="B231" s="30" t="inlineStr">
         <is>
           <t>Cremación</t>
         </is>
       </c>
-      <c r="C93" s="29" t="inlineStr">
+      <c r="C231" s="31" t="inlineStr">
         <is>
           <t>2 (estándar) o 4 (familiar) cremaciones, con certificado</t>
         </is>
       </c>
-      <c r="D93" s="30" t="n"/>
-      <c r="E93" s="31" t="n"/>
-    </row>
-    <row r="94" ht="20.5" customHeight="1">
-      <c r="B94" s="24" t="inlineStr">
+      <c r="D231" s="32" t="n"/>
+      <c r="E231" s="33" t="n"/>
+    </row>
+    <row r="232" ht="20.5" customHeight="1">
+      <c r="B232" s="26" t="inlineStr">
         <is>
           <t>Preparación y resguardo</t>
         </is>
       </c>
-      <c r="C94" s="25" t="inlineStr">
+      <c r="C232" s="27" t="inlineStr">
         <is>
           <t>Preparación química y custodia en laboratorio hasta por 5 días</t>
         </is>
       </c>
-      <c r="D94" s="26" t="n"/>
-      <c r="E94" s="27" t="n"/>
-    </row>
-    <row r="95" ht="78.5" customHeight="1">
-      <c r="B95" s="28" t="inlineStr">
+      <c r="D232" s="28" t="n"/>
+      <c r="E232" s="29" t="n"/>
+    </row>
+    <row r="233" ht="78.5" customHeight="1">
+      <c r="B233" s="30" t="inlineStr">
         <is>
           <t>Servicios incluidos</t>
         </is>
       </c>
-      <c r="C95" s="29" t="inlineStr">
+      <c r="C233" s="31" t="inlineStr">
         <is>
           <t>• Columbario de cristal permanente (estándar o familiar)
 • Traslados durante todo el proceso
@@ -4017,26 +3892,26 @@
 • Certificado de cremación y ceremonias privadas de colocación</t>
         </is>
       </c>
-      <c r="D95" s="30" t="n"/>
-      <c r="E95" s="31" t="n"/>
-    </row>
-    <row r="96" ht="20" customHeight="1">
-      <c r="B96" s="21" t="inlineStr">
+      <c r="D233" s="32" t="n"/>
+      <c r="E233" s="33" t="n"/>
+    </row>
+    <row r="234" ht="20" customHeight="1">
+      <c r="B234" s="23" t="inlineStr">
         <is>
           <t>PRECIO &amp; CONDICIONES DE PAGO</t>
         </is>
       </c>
-      <c r="C96" s="22" t="n"/>
-      <c r="D96" s="22" t="n"/>
-      <c r="E96" s="23" t="n"/>
-    </row>
-    <row r="97" ht="70" customHeight="1">
-      <c r="B97" s="24" t="inlineStr">
+      <c r="C234" s="24" t="n"/>
+      <c r="D234" s="24" t="n"/>
+      <c r="E234" s="25" t="n"/>
+    </row>
+    <row r="235" ht="70" customHeight="1">
+      <c r="B235" s="26" t="inlineStr">
         <is>
           <t>Precio</t>
         </is>
       </c>
-      <c r="C97" s="32" t="inlineStr">
+      <c r="C235" s="34" t="inlineStr">
         <is>
           <t>Estándar · ubicación definida: US$ 1.800
 Estándar · ubicación a futuro: US$ 1.300
@@ -4044,16 +3919,16 @@
 Familiar · ubicación a futuro: US$ 2.300</t>
         </is>
       </c>
-      <c r="D97" s="26" t="n"/>
-      <c r="E97" s="27" t="n"/>
-    </row>
-    <row r="98" ht="70" customHeight="1">
-      <c r="B98" s="28" t="inlineStr">
+      <c r="D235" s="28" t="n"/>
+      <c r="E235" s="29" t="n"/>
+    </row>
+    <row r="236" ht="70" customHeight="1">
+      <c r="B236" s="30" t="inlineStr">
         <is>
           <t>Precio Finados y noviembre (−15%)</t>
         </is>
       </c>
-      <c r="C98" s="33" t="inlineStr">
+      <c r="C236" s="35" t="inlineStr">
         <is>
           <t>Estándar · ubicación definida: US$ 1.530
 Estándar · ubicación a futuro: US$ 1.105
@@ -4061,169 +3936,299 @@
 Familiar · ubicación a futuro: US$ 1.955</t>
         </is>
       </c>
-      <c r="D98" s="30" t="n"/>
-      <c r="E98" s="31" t="n"/>
-    </row>
-    <row r="99" ht="20.5" customHeight="1">
-      <c r="B99" s="28" t="inlineStr">
+      <c r="D236" s="32" t="n"/>
+      <c r="E236" s="33" t="n"/>
+    </row>
+    <row r="237" ht="20.5" customHeight="1">
+      <c r="B237" s="30" t="inlineStr">
         <is>
           <t>Base de precio</t>
         </is>
       </c>
-      <c r="C99" s="29" t="inlineStr">
+      <c r="C237" s="31" t="inlineStr">
         <is>
           <t>Incluye cremación · precio según modalidad y ubicación</t>
         </is>
       </c>
-      <c r="D99" s="30" t="n"/>
-      <c r="E99" s="31" t="n"/>
-    </row>
-    <row r="100" ht="20.5" customHeight="1">
-      <c r="B100" s="24" t="inlineStr">
+      <c r="D237" s="32" t="n"/>
+      <c r="E237" s="33" t="n"/>
+    </row>
+    <row r="238" ht="20.5" customHeight="1">
+      <c r="B238" s="26" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
-      <c r="C100" s="25" t="inlineStr">
+      <c r="C238" s="27" t="inlineStr">
         <is>
           <t>Pago único o financiado hasta 120 meses, con intereses.</t>
         </is>
       </c>
-      <c r="D100" s="26" t="n"/>
-      <c r="E100" s="27" t="n"/>
-    </row>
-    <row r="101" ht="20" customHeight="1">
-      <c r="B101" s="21" t="inlineStr">
+      <c r="D238" s="28" t="n"/>
+      <c r="E238" s="29" t="n"/>
+    </row>
+    <row r="239" ht="20" customHeight="1">
+      <c r="B239" s="23" t="inlineStr">
         <is>
           <t>PERFIL DEL COMPRADOR</t>
         </is>
       </c>
-      <c r="C101" s="22" t="n"/>
-      <c r="D101" s="22" t="n"/>
-      <c r="E101" s="23" t="n"/>
-    </row>
-    <row r="102" ht="35" customHeight="1">
-      <c r="B102" s="34" t="inlineStr">
+      <c r="C239" s="24" t="n"/>
+      <c r="D239" s="24" t="n"/>
+      <c r="E239" s="25" t="n"/>
+    </row>
+    <row r="240" ht="35" customHeight="1">
+      <c r="B240" s="36" t="inlineStr">
         <is>
           <t>Cliente objetivo</t>
         </is>
       </c>
-      <c r="C102" s="35" t="inlineStr">
+      <c r="C240" s="37" t="inlineStr">
         <is>
           <t>Familias que buscan la opción más accesible de cremación con columbario permanente, para 2 o 4 personas.</t>
         </is>
       </c>
-      <c r="D102" s="36" t="n"/>
-      <c r="E102" s="37" t="n"/>
+      <c r="D240" s="38" t="n"/>
+      <c r="E240" s="39" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="93">
-    <mergeCell ref="B65:E65"/>
+  <mergeCells count="217">
+    <mergeCell ref="C44:E44"/>
+    <mergeCell ref="C31:E31"/>
+    <mergeCell ref="B74:E74"/>
+    <mergeCell ref="C80:E80"/>
     <mergeCell ref="C40:E40"/>
+    <mergeCell ref="C129:E129"/>
+    <mergeCell ref="B139:E139"/>
     <mergeCell ref="C21:E21"/>
-    <mergeCell ref="B36:E36"/>
-    <mergeCell ref="C51:E51"/>
-    <mergeCell ref="C95:E95"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="C71:E71"/>
+    <mergeCell ref="C192:E192"/>
+    <mergeCell ref="B207:E207"/>
+    <mergeCell ref="C60:E60"/>
+    <mergeCell ref="B110:E110"/>
+    <mergeCell ref="B203:E203"/>
+    <mergeCell ref="C123:E123"/>
     <mergeCell ref="C23:E23"/>
+    <mergeCell ref="C194:E194"/>
+    <mergeCell ref="C228:E228"/>
+    <mergeCell ref="B165:E165"/>
     <mergeCell ref="B47:E47"/>
-    <mergeCell ref="C7:E7"/>
     <mergeCell ref="C91:E91"/>
-    <mergeCell ref="B22:E22"/>
-    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="B115:E115"/>
+    <mergeCell ref="B155:E155"/>
+    <mergeCell ref="B93:E93"/>
+    <mergeCell ref="B193:E193"/>
+    <mergeCell ref="B102:E102"/>
     <mergeCell ref="C57:E57"/>
-    <mergeCell ref="B86:E86"/>
+    <mergeCell ref="B12:E12"/>
     <mergeCell ref="C18:E18"/>
-    <mergeCell ref="C49:E49"/>
+    <mergeCell ref="C101:E101"/>
+    <mergeCell ref="C229:E229"/>
     <mergeCell ref="C77:E77"/>
     <mergeCell ref="C34:E34"/>
-    <mergeCell ref="B101:E101"/>
-    <mergeCell ref="C42:E42"/>
+    <mergeCell ref="C157:E157"/>
+    <mergeCell ref="C151:E151"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="C74:E74"/>
+    <mergeCell ref="C126:E126"/>
     <mergeCell ref="B69:E69"/>
+    <mergeCell ref="B78:E78"/>
+    <mergeCell ref="C206:E206"/>
+    <mergeCell ref="C215:E215"/>
+    <mergeCell ref="C128:E128"/>
     <mergeCell ref="C20:E20"/>
-    <mergeCell ref="C99:E99"/>
+    <mergeCell ref="C113:E113"/>
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="C103:E103"/>
+    <mergeCell ref="C85:E85"/>
+    <mergeCell ref="C196:E196"/>
+    <mergeCell ref="C112:E112"/>
+    <mergeCell ref="C168:E168"/>
     <mergeCell ref="C94:E94"/>
+    <mergeCell ref="C205:E205"/>
+    <mergeCell ref="C180:E180"/>
+    <mergeCell ref="C84:E84"/>
+    <mergeCell ref="C133:E133"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="C127:E127"/>
     <mergeCell ref="B64:E64"/>
+    <mergeCell ref="C167:E167"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="C176:E176"/>
+    <mergeCell ref="B183:E183"/>
+    <mergeCell ref="C114:E114"/>
+    <mergeCell ref="B51:E51"/>
+    <mergeCell ref="B164:E164"/>
     <mergeCell ref="C59:E59"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="B41:E41"/>
-    <mergeCell ref="B50:E50"/>
-    <mergeCell ref="C52:E52"/>
+    <mergeCell ref="C232:E232"/>
+    <mergeCell ref="B222:E222"/>
+    <mergeCell ref="C46:E46"/>
+    <mergeCell ref="C178:E178"/>
     <mergeCell ref="C61:E61"/>
     <mergeCell ref="C39:E39"/>
     <mergeCell ref="C70:E70"/>
+    <mergeCell ref="C159:E159"/>
     <mergeCell ref="C48:E48"/>
+    <mergeCell ref="C153:E153"/>
+    <mergeCell ref="C219:E219"/>
+    <mergeCell ref="C233:E233"/>
+    <mergeCell ref="C106:E106"/>
     <mergeCell ref="C32:E32"/>
     <mergeCell ref="C38:E38"/>
-    <mergeCell ref="B66:E66"/>
     <mergeCell ref="C81:E81"/>
-    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="C209:E209"/>
+    <mergeCell ref="B140:E140"/>
+    <mergeCell ref="C161:E161"/>
+    <mergeCell ref="C217:E217"/>
+    <mergeCell ref="B223:E223"/>
     <mergeCell ref="C13:E13"/>
+    <mergeCell ref="C170:E170"/>
+    <mergeCell ref="C131:E131"/>
     <mergeCell ref="C87:E87"/>
+    <mergeCell ref="B130:E130"/>
+    <mergeCell ref="C145:E145"/>
+    <mergeCell ref="C154:E154"/>
     <mergeCell ref="C15:E15"/>
-    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="C195:E195"/>
+    <mergeCell ref="B179:E179"/>
+    <mergeCell ref="C89:E89"/>
+    <mergeCell ref="C104:E104"/>
+    <mergeCell ref="C116:E116"/>
+    <mergeCell ref="B53:E53"/>
+    <mergeCell ref="C156:E156"/>
+    <mergeCell ref="B166:E166"/>
+    <mergeCell ref="B119:E119"/>
+    <mergeCell ref="C187:E187"/>
     <mergeCell ref="C79:E79"/>
-    <mergeCell ref="C73:E73"/>
-    <mergeCell ref="C88:E88"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="C197:E197"/>
+    <mergeCell ref="C231:E231"/>
     <mergeCell ref="C35:E35"/>
-    <mergeCell ref="B84:E84"/>
+    <mergeCell ref="B174:E174"/>
+    <mergeCell ref="C63:E63"/>
+    <mergeCell ref="C10:E10"/>
     <mergeCell ref="C16:E16"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B55:E55"/>
-    <mergeCell ref="B80:E80"/>
-    <mergeCell ref="B89:E89"/>
+    <mergeCell ref="C212:E212"/>
+    <mergeCell ref="C230:E230"/>
+    <mergeCell ref="C173:E173"/>
+    <mergeCell ref="C55:E55"/>
+    <mergeCell ref="C236:E236"/>
+    <mergeCell ref="C214:E214"/>
+    <mergeCell ref="B142:E142"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B160:E160"/>
+    <mergeCell ref="B169:E169"/>
+    <mergeCell ref="C36:E36"/>
     <mergeCell ref="C11:E11"/>
+    <mergeCell ref="B144:E144"/>
+    <mergeCell ref="B97:E97"/>
+    <mergeCell ref="B224:E224"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="C150:E150"/>
+    <mergeCell ref="B185:E185"/>
+    <mergeCell ref="C158:E158"/>
     <mergeCell ref="C67:E67"/>
-    <mergeCell ref="C72:E72"/>
+    <mergeCell ref="B121:E121"/>
+    <mergeCell ref="C190:E190"/>
+    <mergeCell ref="C109:E109"/>
+    <mergeCell ref="B122:E122"/>
+    <mergeCell ref="B56:E56"/>
+    <mergeCell ref="B184:E184"/>
+    <mergeCell ref="C199:E199"/>
     <mergeCell ref="C37:E37"/>
-    <mergeCell ref="C78:E78"/>
+    <mergeCell ref="C208:E208"/>
+    <mergeCell ref="C186:E186"/>
+    <mergeCell ref="B52:E52"/>
+    <mergeCell ref="C136:E136"/>
+    <mergeCell ref="B120:E120"/>
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="C92:E92"/>
-    <mergeCell ref="C30:E30"/>
-    <mergeCell ref="B60:E60"/>
-    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="B42:E42"/>
+    <mergeCell ref="C235:E235"/>
+    <mergeCell ref="C210:E210"/>
+    <mergeCell ref="C62:E62"/>
     <mergeCell ref="C14:E14"/>
-    <mergeCell ref="C98:E98"/>
+    <mergeCell ref="C191:E191"/>
+    <mergeCell ref="C225:E225"/>
+    <mergeCell ref="C107:E107"/>
+    <mergeCell ref="C172:E172"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="B234:E234"/>
     <mergeCell ref="B28:E28"/>
+    <mergeCell ref="C171:E171"/>
+    <mergeCell ref="B99:E99"/>
     <mergeCell ref="C54:E54"/>
     <mergeCell ref="B9:E9"/>
-    <mergeCell ref="C93:E93"/>
-    <mergeCell ref="C56:E56"/>
+    <mergeCell ref="C177:E177"/>
+    <mergeCell ref="C41:E41"/>
+    <mergeCell ref="C134:E134"/>
+    <mergeCell ref="C146:E146"/>
+    <mergeCell ref="C124:E124"/>
+    <mergeCell ref="B143:E143"/>
+    <mergeCell ref="C211:E211"/>
+    <mergeCell ref="C226:E226"/>
+    <mergeCell ref="B239:E239"/>
+    <mergeCell ref="B30:E30"/>
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="C90:E90"/>
-    <mergeCell ref="B85:E85"/>
+    <mergeCell ref="C105:E105"/>
+    <mergeCell ref="C148:E148"/>
+    <mergeCell ref="C43:E43"/>
+    <mergeCell ref="B204:E204"/>
+    <mergeCell ref="B198:E198"/>
+    <mergeCell ref="B213:E213"/>
+    <mergeCell ref="B188:E188"/>
     <mergeCell ref="C76:E76"/>
     <mergeCell ref="B4:E4"/>
+    <mergeCell ref="C132:E132"/>
     <mergeCell ref="B75:E75"/>
-    <mergeCell ref="C8:E8"/>
-    <mergeCell ref="B46:E46"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="C53:E53"/>
-    <mergeCell ref="B96:E96"/>
-    <mergeCell ref="C102:E102"/>
+    <mergeCell ref="B135:E135"/>
+    <mergeCell ref="B218:E218"/>
+    <mergeCell ref="B227:E227"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="C82:E82"/>
+    <mergeCell ref="B125:E125"/>
+    <mergeCell ref="B202:E202"/>
+    <mergeCell ref="C149:E149"/>
+    <mergeCell ref="C240:E240"/>
+    <mergeCell ref="C66:E66"/>
+    <mergeCell ref="C237:E237"/>
+    <mergeCell ref="C189:E189"/>
+    <mergeCell ref="C111:E111"/>
+    <mergeCell ref="C86:E86"/>
     <mergeCell ref="C68:E68"/>
+    <mergeCell ref="C83:E83"/>
+    <mergeCell ref="C238:E238"/>
+    <mergeCell ref="C108:E108"/>
+    <mergeCell ref="B98:E98"/>
+    <mergeCell ref="C175:E175"/>
     <mergeCell ref="C58:E58"/>
-    <mergeCell ref="C97:E97"/>
-    <mergeCell ref="C29:E29"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="B73:E73"/>
+    <mergeCell ref="C45:E45"/>
+    <mergeCell ref="B88:E88"/>
+    <mergeCell ref="C216:E216"/>
+    <mergeCell ref="B147:E147"/>
     <mergeCell ref="C100:E100"/>
+    <mergeCell ref="C152:E152"/>
+    <mergeCell ref="C65:E65"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
-  <rowBreaks count="4" manualBreakCount="4">
-    <brk id="24" min="0" max="16383" man="1"/>
-    <brk id="43" min="0" max="16383" man="1"/>
-    <brk id="62" min="0" max="16383" man="1"/>
-    <brk id="82" min="0" max="16383" man="1"/>
+  <rowBreaks count="10" manualBreakCount="10">
+    <brk id="26" min="0" max="16383" man="1"/>
+    <brk id="49" min="0" max="16383" man="1"/>
+    <brk id="71" min="0" max="16383" man="1"/>
+    <brk id="95" min="0" max="16383" man="1"/>
+    <brk id="117" min="0" max="16383" man="1"/>
+    <brk id="137" min="0" max="16383" man="1"/>
+    <brk id="162" min="0" max="16383" man="1"/>
+    <brk id="181" min="0" max="16383" man="1"/>
+    <brk id="200" min="0" max="16383" man="1"/>
+    <brk id="220" min="0" max="16383" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="000F2537"/>
@@ -4247,251 +4252,251 @@
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="41" t="inlineStr">
+      <c r="A2" s="43" t="inlineStr">
         <is>
           <t>Vigente en 2026 · comisión según la cantidad de ventas del mes (8% · 10% · 12%)</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="42" t="inlineStr">
+      <c r="A4" s="44" t="inlineStr">
         <is>
           <t>1. ESCALA POR CANTIDAD DE VENTAS EN EL MES (cualquier producto de cremación)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="43" t="inlineStr">
+      <c r="A5" s="45" t="inlineStr">
         <is>
           <t>Ventas en el mes</t>
         </is>
       </c>
-      <c r="B5" s="43" t="inlineStr">
+      <c r="B5" s="45" t="inlineStr">
         <is>
           <t>% comisión</t>
         </is>
       </c>
-      <c r="C5" s="43" t="inlineStr">
+      <c r="C5" s="45" t="inlineStr">
         <is>
           <t>Ejemplo: facturación con Solución Modular (sin IVA)</t>
         </is>
       </c>
-      <c r="D5" s="43" t="inlineStr">
+      <c r="D5" s="45" t="inlineStr">
         <is>
           <t>Comisión del ejemplo</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="44" t="inlineStr">
+      <c r="A6" s="46" t="inlineStr">
         <is>
           <t>1 venta</t>
         </is>
       </c>
-      <c r="B6" s="45" t="n">
+      <c r="B6" s="47" t="n">
         <v>0.08</v>
       </c>
-      <c r="C6" s="46">
+      <c r="C6" s="48">
         <f>1*1000*100/113</f>
         <v/>
       </c>
-      <c r="D6" s="47">
+      <c r="D6" s="49">
         <f>B6*C6</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="48" t="inlineStr">
+      <c r="A7" s="50" t="inlineStr">
         <is>
           <t>2 ventas</t>
         </is>
       </c>
-      <c r="B7" s="49" t="n">
+      <c r="B7" s="51" t="n">
         <v>0.1</v>
       </c>
-      <c r="C7" s="50">
+      <c r="C7" s="52">
         <f>2*1000*100/113</f>
         <v/>
       </c>
-      <c r="D7" s="51">
+      <c r="D7" s="53">
         <f>B7*C7</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="44" t="inlineStr">
+      <c r="A8" s="46" t="inlineStr">
         <is>
           <t>3 ventas o más</t>
         </is>
       </c>
-      <c r="B8" s="45" t="n">
+      <c r="B8" s="47" t="n">
         <v>0.12</v>
       </c>
-      <c r="C8" s="46">
+      <c r="C8" s="48">
         <f>3*1000*100/113</f>
         <v/>
       </c>
-      <c r="D8" s="47">
+      <c r="D8" s="49">
         <f>B8*C8</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="42" t="inlineStr">
+      <c r="A10" s="44" t="inlineStr">
         <is>
           <t>2. CUÁNDO SE PAGA Y CUÁNDO SE DESCUENTA</t>
         </is>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="43" t="inlineStr">
+      <c r="A11" s="45" t="inlineStr">
         <is>
           <t>Producto</t>
         </is>
       </c>
-      <c r="B11" s="43" t="inlineStr">
+      <c r="B11" s="45" t="inlineStr">
         <is>
           <t>Momento de pago</t>
         </is>
       </c>
-      <c r="C11" s="43" t="inlineStr">
+      <c r="C11" s="45" t="inlineStr">
         <is>
           <t>Estorno</t>
         </is>
       </c>
-      <c r="D11" s="43" t="inlineStr">
+      <c r="D11" s="45" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
       </c>
     </row>
     <row r="12" ht="36" customHeight="1">
-      <c r="A12" s="44" t="inlineStr">
+      <c r="A12" s="46" t="inlineStr">
         <is>
           <t>Solución Modular de Cremación</t>
         </is>
       </c>
-      <c r="B12" s="52" t="inlineStr">
+      <c r="B12" s="54" t="inlineStr">
         <is>
           <t>Pago único cuando el cliente paga la 3ª cuota</t>
         </is>
       </c>
-      <c r="C12" s="52" t="inlineStr">
+      <c r="C12" s="54" t="inlineStr">
         <is>
           <t>Si el cliente cancela antes de la 12ª cuota</t>
         </is>
       </c>
-      <c r="D12" s="52" t="inlineStr"/>
+      <c r="D12" s="54" t="inlineStr"/>
     </row>
     <row r="13" ht="36" customHeight="1">
-      <c r="A13" s="48" t="inlineStr">
+      <c r="A13" s="50" t="inlineStr">
         <is>
           <t>Jardines de Cenizas (Individual, Familiar, Ecológico)</t>
         </is>
       </c>
-      <c r="B13" s="53" t="inlineStr">
+      <c r="B13" s="55" t="inlineStr">
         <is>
           <t>Contado: mes siguiente al pago. Financiado: proporcional a lo cobrado</t>
         </is>
       </c>
-      <c r="C13" s="53" t="inlineStr">
+      <c r="C13" s="55" t="inlineStr">
         <is>
           <t>Cancelación en los primeros 90 días</t>
         </is>
       </c>
-      <c r="D13" s="53" t="inlineStr"/>
+      <c r="D13" s="55" t="inlineStr"/>
     </row>
     <row r="14" ht="36" customHeight="1">
-      <c r="A14" s="44" t="inlineStr">
+      <c r="A14" s="46" t="inlineStr">
         <is>
           <t>Jardín de Mascotas</t>
         </is>
       </c>
-      <c r="B14" s="52" t="inlineStr">
+      <c r="B14" s="54" t="inlineStr">
         <is>
           <t>Mes siguiente al pago (pago único)</t>
         </is>
       </c>
-      <c r="C14" s="52" t="inlineStr">
+      <c r="C14" s="54" t="inlineStr">
         <is>
           <t>Cancelación en los primeros 90 días</t>
         </is>
       </c>
-      <c r="D14" s="52" t="inlineStr"/>
+      <c r="D14" s="54" t="inlineStr"/>
     </row>
     <row r="15" ht="36" customHeight="1">
-      <c r="A15" s="48" t="inlineStr">
+      <c r="A15" s="50" t="inlineStr">
         <is>
           <t>Columbarios (portafolio existente)</t>
         </is>
       </c>
-      <c r="B15" s="53" t="inlineStr">
+      <c r="B15" s="55" t="inlineStr">
         <is>
           <t>Contado: mes siguiente al pago. Financiado: proporcional a lo cobrado</t>
         </is>
       </c>
-      <c r="C15" s="53" t="inlineStr">
+      <c r="C15" s="55" t="inlineStr">
         <is>
           <t>Cancelación en los primeros 90 días</t>
         </is>
       </c>
-      <c r="D15" s="53" t="inlineStr">
+      <c r="D15" s="55" t="inlineStr">
         <is>
           <t>Mismo criterio de cantidad de ventas que los productos nuevos.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="42" t="inlineStr">
+      <c r="A17" s="44" t="inlineStr">
         <is>
           <t>3. REGLAS GENERALES</t>
         </is>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="54" t="inlineStr">
+      <c r="A18" s="56" t="inlineStr">
         <is>
           <t>1. 1 venta en el mes de cualquier producto de cremación = 8%; 2 ventas = 10%; 3 o más = 12%, sobre toda la facturación del mes.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="54" t="inlineStr">
+      <c r="A19" s="56" t="inlineStr">
         <is>
           <t>2. Cada contrato vendido cuenta como 1 venta, sin distinción por grupo de producto (nuevos y columbarios).</t>
         </is>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="54" t="inlineStr">
+      <c r="A20" s="56" t="inlineStr">
         <is>
           <t>3. Base de cálculo: facturación sin IVA (13%), neta de descuentos. La comisión se paga sobre lo cobrado.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="54" t="inlineStr">
+      <c r="A21" s="56" t="inlineStr">
         <is>
           <t>4. Mismo criterio para call center, contratados y freelancers. No hay bonos adicionales.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="54" t="inlineStr">
+      <c r="A22" s="56" t="inlineStr">
         <is>
           <t>5. Venta compartida (call center agenda, otro vendedor cierra): 1 venta para ambos; comisión 30% / 70%.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="54" t="inlineStr">
+      <c r="A23" s="56" t="inlineStr">
         <is>
           <t>6. No generan comisión ni cuentan como venta: cuotas de mantenimiento anual (US$ 15 / US$ 24).</t>
         </is>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="54" t="inlineStr">
+      <c r="A24" s="56" t="inlineStr">
         <is>
           <t>7. Estorno: la comisión se descuenta de los pagos siguientes al vendedor. Ventas anuladas no cuentan.</t>
         </is>

</xml_diff>